<commit_message>
Atualização automática: tpjl (14/09/2026 13:57)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10597,7 +10597,7 @@
         <v>590</v>
       </c>
       <c r="M8" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N8" t="s">
         <v>596</v>
@@ -10682,7 +10682,7 @@
         <v>592</v>
       </c>
       <c r="M10" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N10" t="s">
         <v>596</v>
@@ -10726,7 +10726,7 @@
         <v>592</v>
       </c>
       <c r="M11" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N11" t="s">
         <v>596</v>
@@ -10893,7 +10893,7 @@
         <v>590</v>
       </c>
       <c r="M15" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N15" t="s">
         <v>596</v>
@@ -10937,7 +10937,7 @@
         <v>592</v>
       </c>
       <c r="M16" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N16" t="s">
         <v>596</v>
@@ -10981,7 +10981,7 @@
         <v>590</v>
       </c>
       <c r="M17" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N17" t="s">
         <v>596</v>
@@ -11025,7 +11025,7 @@
         <v>592</v>
       </c>
       <c r="M18" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N18" t="s">
         <v>596</v>
@@ -11069,7 +11069,7 @@
         <v>592</v>
       </c>
       <c r="M19" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N19" t="s">
         <v>596</v>
@@ -11113,7 +11113,7 @@
         <v>592</v>
       </c>
       <c r="M20" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N20" t="s">
         <v>596</v>
@@ -11157,7 +11157,7 @@
         <v>592</v>
       </c>
       <c r="M21" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N21" t="s">
         <v>596</v>
@@ -11324,7 +11324,7 @@
         <v>592</v>
       </c>
       <c r="M25" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N25" t="s">
         <v>596</v>
@@ -11409,7 +11409,7 @@
         <v>590</v>
       </c>
       <c r="M27" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N27" t="s">
         <v>596</v>
@@ -11453,7 +11453,7 @@
         <v>592</v>
       </c>
       <c r="M28" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N28" t="s">
         <v>596</v>
@@ -11497,7 +11497,7 @@
         <v>593</v>
       </c>
       <c r="M29" s="1">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="N29" t="s">
         <v>596</v>
@@ -11541,7 +11541,7 @@
         <v>592</v>
       </c>
       <c r="M30" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N30" t="s">
         <v>596</v>
@@ -11585,7 +11585,7 @@
         <v>593</v>
       </c>
       <c r="M31" s="1">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="N31" t="s">
         <v>596</v>
@@ -11629,7 +11629,7 @@
         <v>590</v>
       </c>
       <c r="M32" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N32" t="s">
         <v>596</v>
@@ -11673,7 +11673,7 @@
         <v>590</v>
       </c>
       <c r="M33" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N33" t="s">
         <v>596</v>
@@ -11717,7 +11717,7 @@
         <v>590</v>
       </c>
       <c r="M34" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N34" t="s">
         <v>596</v>
@@ -11761,7 +11761,7 @@
         <v>590</v>
       </c>
       <c r="M35" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N35" t="s">
         <v>596</v>
@@ -11805,7 +11805,7 @@
         <v>590</v>
       </c>
       <c r="M36" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N36" t="s">
         <v>596</v>
@@ -11849,7 +11849,7 @@
         <v>590</v>
       </c>
       <c r="M37" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N37" t="s">
         <v>596</v>
@@ -11893,7 +11893,7 @@
         <v>590</v>
       </c>
       <c r="M38" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N38" t="s">
         <v>596</v>
@@ -11978,7 +11978,7 @@
         <v>590</v>
       </c>
       <c r="M40" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N40" t="s">
         <v>596</v>
@@ -12022,7 +12022,7 @@
         <v>592</v>
       </c>
       <c r="M41" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N41" t="s">
         <v>596</v>
@@ -12066,7 +12066,7 @@
         <v>590</v>
       </c>
       <c r="M42" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N42" t="s">
         <v>596</v>
@@ -12110,7 +12110,7 @@
         <v>592</v>
       </c>
       <c r="M43" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N43" t="s">
         <v>596</v>
@@ -12154,7 +12154,7 @@
         <v>592</v>
       </c>
       <c r="M44" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N44" t="s">
         <v>596</v>
@@ -12198,7 +12198,7 @@
         <v>592</v>
       </c>
       <c r="M45" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N45" t="s">
         <v>596</v>
@@ -12242,7 +12242,7 @@
         <v>590</v>
       </c>
       <c r="M46" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N46" t="s">
         <v>596</v>
@@ -12286,7 +12286,7 @@
         <v>590</v>
       </c>
       <c r="M47" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N47" t="s">
         <v>596</v>
@@ -12330,7 +12330,7 @@
         <v>592</v>
       </c>
       <c r="M48" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N48" t="s">
         <v>596</v>
@@ -12374,7 +12374,7 @@
         <v>593</v>
       </c>
       <c r="M49" s="1">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="N49" t="s">
         <v>596</v>
@@ -12418,7 +12418,7 @@
         <v>593</v>
       </c>
       <c r="M50" s="1">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="N50" t="s">
         <v>596</v>
@@ -12462,7 +12462,7 @@
         <v>592</v>
       </c>
       <c r="M51" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N51" t="s">
         <v>596</v>
@@ -12506,7 +12506,7 @@
         <v>592</v>
       </c>
       <c r="M52" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N52" t="s">
         <v>596</v>
@@ -12550,7 +12550,7 @@
         <v>592</v>
       </c>
       <c r="M53" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N53" t="s">
         <v>596</v>
@@ -12594,7 +12594,7 @@
         <v>592</v>
       </c>
       <c r="M54" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N54" t="s">
         <v>596</v>
@@ -12638,7 +12638,7 @@
         <v>592</v>
       </c>
       <c r="M55" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N55" t="s">
         <v>596</v>
@@ -12682,7 +12682,7 @@
         <v>593</v>
       </c>
       <c r="M56" s="1">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="N56" t="s">
         <v>596</v>
@@ -12726,7 +12726,7 @@
         <v>593</v>
       </c>
       <c r="M57" s="1">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="N57" t="s">
         <v>596</v>
@@ -12770,7 +12770,7 @@
         <v>593</v>
       </c>
       <c r="M58" s="1">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="N58" t="s">
         <v>596</v>
@@ -12814,7 +12814,7 @@
         <v>592</v>
       </c>
       <c r="M59" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N59" t="s">
         <v>596</v>
@@ -12858,7 +12858,7 @@
         <v>593</v>
       </c>
       <c r="M60" s="1">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="N60" t="s">
         <v>596</v>
@@ -12902,7 +12902,7 @@
         <v>593</v>
       </c>
       <c r="M61" s="1">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="N61" t="s">
         <v>596</v>
@@ -12946,7 +12946,7 @@
         <v>592</v>
       </c>
       <c r="M62" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N62" t="s">
         <v>596</v>
@@ -12990,7 +12990,7 @@
         <v>592</v>
       </c>
       <c r="M63" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N63" t="s">
         <v>596</v>
@@ -13034,7 +13034,7 @@
         <v>592</v>
       </c>
       <c r="M64" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N64" t="s">
         <v>596</v>
@@ -13078,7 +13078,7 @@
         <v>592</v>
       </c>
       <c r="M65" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N65" t="s">
         <v>596</v>
@@ -13122,7 +13122,7 @@
         <v>592</v>
       </c>
       <c r="M66" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N66" t="s">
         <v>596</v>
@@ -13166,7 +13166,7 @@
         <v>592</v>
       </c>
       <c r="M67" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N67" t="s">
         <v>596</v>
@@ -13210,7 +13210,7 @@
         <v>592</v>
       </c>
       <c r="M68" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N68" t="s">
         <v>596</v>
@@ -13254,7 +13254,7 @@
         <v>592</v>
       </c>
       <c r="M69" s="1">
-        <v>46351</v>
+        <v>46354</v>
       </c>
       <c r="N69" t="s">
         <v>596</v>
@@ -13339,7 +13339,7 @@
         <v>595</v>
       </c>
       <c r="M71" s="1">
-        <v>46366</v>
+        <v>46369</v>
       </c>
       <c r="N71" t="s">
         <v>596</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (15/09/2026 08:56)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,8 +1815,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1832,7 +1840,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1840,12 +1848,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2145,55 +2171,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2237,7 +2263,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2281,7 +2307,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2325,7 +2351,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2451,7 +2477,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2495,7 +2521,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2539,7 +2565,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2586,7 +2612,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2709,7 +2735,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2753,7 +2779,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2797,7 +2823,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2888,7 +2914,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2932,7 +2958,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3058,7 +3084,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3102,7 +3128,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3187,7 +3213,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3234,7 +3260,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3281,7 +3307,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3325,7 +3351,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3369,7 +3395,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3454,7 +3480,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3539,7 +3565,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3586,7 +3612,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3630,7 +3656,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3674,7 +3700,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3759,7 +3785,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3803,7 +3829,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3847,7 +3873,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3932,7 +3958,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3976,7 +4002,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4020,7 +4046,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4064,7 +4090,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4231,7 +4257,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4275,7 +4301,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4319,7 +4345,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4363,7 +4389,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4410,7 +4436,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4454,7 +4480,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4536,7 +4562,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4580,7 +4606,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4668,7 +4694,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4712,7 +4738,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4759,7 +4785,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4803,7 +4829,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4847,7 +4873,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4891,7 +4917,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4935,7 +4961,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4982,7 +5008,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5026,7 +5052,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5073,7 +5099,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5117,7 +5143,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5164,7 +5190,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5252,7 +5278,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5296,7 +5322,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5340,7 +5366,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5384,7 +5410,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5428,7 +5454,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5472,7 +5498,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5557,7 +5583,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5601,7 +5627,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5645,7 +5671,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5689,7 +5715,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5733,7 +5759,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5777,7 +5803,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5821,7 +5847,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5865,7 +5891,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5912,7 +5938,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5956,7 +5982,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6000,7 +6026,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6044,7 +6070,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6088,7 +6114,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6132,7 +6158,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6176,7 +6202,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6220,7 +6246,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6264,7 +6290,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6352,7 +6378,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6396,7 +6422,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6566,7 +6592,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6610,7 +6636,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6654,7 +6680,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6736,7 +6762,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6780,7 +6806,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6827,7 +6853,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6871,7 +6897,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6997,7 +7023,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7041,7 +7067,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7126,7 +7152,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7170,7 +7196,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7214,7 +7240,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7258,7 +7284,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7302,7 +7328,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7346,7 +7372,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7390,7 +7416,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7434,7 +7460,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7519,7 +7545,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7686,7 +7712,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7730,7 +7756,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7774,7 +7800,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7818,7 +7844,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7862,7 +7888,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7906,7 +7932,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7950,7 +7976,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8035,7 +8061,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8079,7 +8105,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8164,7 +8190,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8290,7 +8316,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8334,7 +8360,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8419,7 +8445,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8463,7 +8489,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8507,7 +8533,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8551,7 +8577,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8595,7 +8621,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8639,7 +8665,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8683,7 +8709,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8727,7 +8753,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8812,7 +8838,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8979,7 +9005,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9023,7 +9049,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9067,7 +9093,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9111,7 +9137,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9196,7 +9222,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9240,7 +9266,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9284,7 +9310,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9328,7 +9354,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9372,7 +9398,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9416,7 +9442,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9460,7 +9486,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9504,7 +9530,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9548,7 +9574,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9592,7 +9618,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9636,7 +9662,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9680,7 +9706,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9724,7 +9750,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9768,7 +9794,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9812,7 +9838,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9856,7 +9882,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9900,7 +9926,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9944,7 +9970,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9988,7 +10014,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10032,7 +10058,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10076,7 +10102,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10161,7 +10187,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10246,7 +10272,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10261,55 +10287,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10596,8 +10622,8 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="1">
-        <v>46289</v>
+      <c r="M8" s="2">
+        <v>46290</v>
       </c>
       <c r="N8" t="s">
         <v>596</v>
@@ -10681,8 +10707,8 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="1">
-        <v>46354</v>
+      <c r="M10" s="2">
+        <v>46355</v>
       </c>
       <c r="N10" t="s">
         <v>596</v>
@@ -10725,8 +10751,8 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="1">
-        <v>46354</v>
+      <c r="M11" s="2">
+        <v>46355</v>
       </c>
       <c r="N11" t="s">
         <v>596</v>
@@ -10892,8 +10918,8 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="1">
-        <v>46289</v>
+      <c r="M15" s="2">
+        <v>46290</v>
       </c>
       <c r="N15" t="s">
         <v>596</v>
@@ -10936,8 +10962,8 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="1">
-        <v>46354</v>
+      <c r="M16" s="2">
+        <v>46355</v>
       </c>
       <c r="N16" t="s">
         <v>596</v>
@@ -10980,8 +11006,8 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="1">
-        <v>46289</v>
+      <c r="M17" s="2">
+        <v>46290</v>
       </c>
       <c r="N17" t="s">
         <v>596</v>
@@ -11024,8 +11050,8 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="1">
-        <v>46354</v>
+      <c r="M18" s="2">
+        <v>46355</v>
       </c>
       <c r="N18" t="s">
         <v>596</v>
@@ -11068,8 +11094,8 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="1">
-        <v>46354</v>
+      <c r="M19" s="2">
+        <v>46355</v>
       </c>
       <c r="N19" t="s">
         <v>596</v>
@@ -11112,8 +11138,8 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="1">
-        <v>46354</v>
+      <c r="M20" s="2">
+        <v>46355</v>
       </c>
       <c r="N20" t="s">
         <v>596</v>
@@ -11156,8 +11182,8 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="1">
-        <v>46354</v>
+      <c r="M21" s="2">
+        <v>46355</v>
       </c>
       <c r="N21" t="s">
         <v>596</v>
@@ -11323,8 +11349,8 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="1">
-        <v>46354</v>
+      <c r="M25" s="2">
+        <v>46355</v>
       </c>
       <c r="N25" t="s">
         <v>596</v>
@@ -11408,8 +11434,8 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="1">
-        <v>46289</v>
+      <c r="M27" s="2">
+        <v>46290</v>
       </c>
       <c r="N27" t="s">
         <v>596</v>
@@ -11452,8 +11478,8 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="1">
-        <v>46354</v>
+      <c r="M28" s="2">
+        <v>46355</v>
       </c>
       <c r="N28" t="s">
         <v>596</v>
@@ -11496,8 +11522,8 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="1">
-        <v>46309</v>
+      <c r="M29" s="2">
+        <v>46310</v>
       </c>
       <c r="N29" t="s">
         <v>596</v>
@@ -11540,8 +11566,8 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="1">
-        <v>46354</v>
+      <c r="M30" s="2">
+        <v>46355</v>
       </c>
       <c r="N30" t="s">
         <v>596</v>
@@ -11584,8 +11610,8 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="1">
-        <v>46309</v>
+      <c r="M31" s="2">
+        <v>46310</v>
       </c>
       <c r="N31" t="s">
         <v>596</v>
@@ -11628,8 +11654,8 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="1">
-        <v>46289</v>
+      <c r="M32" s="2">
+        <v>46290</v>
       </c>
       <c r="N32" t="s">
         <v>596</v>
@@ -11672,8 +11698,8 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="1">
-        <v>46289</v>
+      <c r="M33" s="2">
+        <v>46290</v>
       </c>
       <c r="N33" t="s">
         <v>596</v>
@@ -11716,8 +11742,8 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="1">
-        <v>46289</v>
+      <c r="M34" s="2">
+        <v>46290</v>
       </c>
       <c r="N34" t="s">
         <v>596</v>
@@ -11760,8 +11786,8 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="1">
-        <v>46289</v>
+      <c r="M35" s="2">
+        <v>46290</v>
       </c>
       <c r="N35" t="s">
         <v>596</v>
@@ -11804,8 +11830,8 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="1">
-        <v>46289</v>
+      <c r="M36" s="2">
+        <v>46290</v>
       </c>
       <c r="N36" t="s">
         <v>596</v>
@@ -11848,8 +11874,8 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="1">
-        <v>46289</v>
+      <c r="M37" s="2">
+        <v>46290</v>
       </c>
       <c r="N37" t="s">
         <v>596</v>
@@ -11892,8 +11918,8 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="1">
-        <v>46289</v>
+      <c r="M38" s="2">
+        <v>46290</v>
       </c>
       <c r="N38" t="s">
         <v>596</v>
@@ -11977,8 +12003,8 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="1">
-        <v>46289</v>
+      <c r="M40" s="2">
+        <v>46290</v>
       </c>
       <c r="N40" t="s">
         <v>596</v>
@@ -12021,8 +12047,8 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="1">
-        <v>46354</v>
+      <c r="M41" s="2">
+        <v>46355</v>
       </c>
       <c r="N41" t="s">
         <v>596</v>
@@ -12065,8 +12091,8 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="1">
-        <v>46289</v>
+      <c r="M42" s="2">
+        <v>46290</v>
       </c>
       <c r="N42" t="s">
         <v>596</v>
@@ -12109,8 +12135,8 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="1">
-        <v>46354</v>
+      <c r="M43" s="2">
+        <v>46355</v>
       </c>
       <c r="N43" t="s">
         <v>596</v>
@@ -12153,8 +12179,8 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="1">
-        <v>46354</v>
+      <c r="M44" s="2">
+        <v>46355</v>
       </c>
       <c r="N44" t="s">
         <v>596</v>
@@ -12197,8 +12223,8 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="1">
-        <v>46354</v>
+      <c r="M45" s="2">
+        <v>46355</v>
       </c>
       <c r="N45" t="s">
         <v>596</v>
@@ -12241,8 +12267,8 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="1">
-        <v>46289</v>
+      <c r="M46" s="2">
+        <v>46290</v>
       </c>
       <c r="N46" t="s">
         <v>596</v>
@@ -12285,8 +12311,8 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="1">
-        <v>46289</v>
+      <c r="M47" s="2">
+        <v>46290</v>
       </c>
       <c r="N47" t="s">
         <v>596</v>
@@ -12329,8 +12355,8 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="1">
-        <v>46354</v>
+      <c r="M48" s="2">
+        <v>46355</v>
       </c>
       <c r="N48" t="s">
         <v>596</v>
@@ -12373,8 +12399,8 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="1">
-        <v>46309</v>
+      <c r="M49" s="2">
+        <v>46310</v>
       </c>
       <c r="N49" t="s">
         <v>596</v>
@@ -12417,8 +12443,8 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="1">
-        <v>46309</v>
+      <c r="M50" s="2">
+        <v>46310</v>
       </c>
       <c r="N50" t="s">
         <v>596</v>
@@ -12461,8 +12487,8 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="1">
-        <v>46354</v>
+      <c r="M51" s="2">
+        <v>46355</v>
       </c>
       <c r="N51" t="s">
         <v>596</v>
@@ -12505,8 +12531,8 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="1">
-        <v>46354</v>
+      <c r="M52" s="2">
+        <v>46355</v>
       </c>
       <c r="N52" t="s">
         <v>596</v>
@@ -12549,8 +12575,8 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="1">
-        <v>46354</v>
+      <c r="M53" s="2">
+        <v>46355</v>
       </c>
       <c r="N53" t="s">
         <v>596</v>
@@ -12593,8 +12619,8 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="1">
-        <v>46354</v>
+      <c r="M54" s="2">
+        <v>46355</v>
       </c>
       <c r="N54" t="s">
         <v>596</v>
@@ -12637,8 +12663,8 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="1">
-        <v>46354</v>
+      <c r="M55" s="2">
+        <v>46355</v>
       </c>
       <c r="N55" t="s">
         <v>596</v>
@@ -12681,8 +12707,8 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="1">
-        <v>46309</v>
+      <c r="M56" s="2">
+        <v>46310</v>
       </c>
       <c r="N56" t="s">
         <v>596</v>
@@ -12725,8 +12751,8 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="1">
-        <v>46309</v>
+      <c r="M57" s="2">
+        <v>46310</v>
       </c>
       <c r="N57" t="s">
         <v>596</v>
@@ -12769,8 +12795,8 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="1">
-        <v>46309</v>
+      <c r="M58" s="2">
+        <v>46310</v>
       </c>
       <c r="N58" t="s">
         <v>596</v>
@@ -12813,8 +12839,8 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="1">
-        <v>46354</v>
+      <c r="M59" s="2">
+        <v>46355</v>
       </c>
       <c r="N59" t="s">
         <v>596</v>
@@ -12857,8 +12883,8 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="1">
-        <v>46309</v>
+      <c r="M60" s="2">
+        <v>46310</v>
       </c>
       <c r="N60" t="s">
         <v>596</v>
@@ -12901,8 +12927,8 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="1">
-        <v>46309</v>
+      <c r="M61" s="2">
+        <v>46310</v>
       </c>
       <c r="N61" t="s">
         <v>596</v>
@@ -12945,8 +12971,8 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="1">
-        <v>46354</v>
+      <c r="M62" s="2">
+        <v>46355</v>
       </c>
       <c r="N62" t="s">
         <v>596</v>
@@ -12989,8 +13015,8 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="1">
-        <v>46354</v>
+      <c r="M63" s="2">
+        <v>46355</v>
       </c>
       <c r="N63" t="s">
         <v>596</v>
@@ -13033,8 +13059,8 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="1">
-        <v>46354</v>
+      <c r="M64" s="2">
+        <v>46355</v>
       </c>
       <c r="N64" t="s">
         <v>596</v>
@@ -13077,8 +13103,8 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="1">
-        <v>46354</v>
+      <c r="M65" s="2">
+        <v>46355</v>
       </c>
       <c r="N65" t="s">
         <v>596</v>
@@ -13121,8 +13147,8 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="1">
-        <v>46354</v>
+      <c r="M66" s="2">
+        <v>46355</v>
       </c>
       <c r="N66" t="s">
         <v>596</v>
@@ -13165,8 +13191,8 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="1">
-        <v>46354</v>
+      <c r="M67" s="2">
+        <v>46355</v>
       </c>
       <c r="N67" t="s">
         <v>596</v>
@@ -13209,8 +13235,8 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="1">
-        <v>46354</v>
+      <c r="M68" s="2">
+        <v>46355</v>
       </c>
       <c r="N68" t="s">
         <v>596</v>
@@ -13253,8 +13279,8 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="1">
-        <v>46354</v>
+      <c r="M69" s="2">
+        <v>46355</v>
       </c>
       <c r="N69" t="s">
         <v>596</v>
@@ -13338,8 +13364,8 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="1">
-        <v>46369</v>
+      <c r="M71" s="2">
+        <v>46370</v>
       </c>
       <c r="N71" t="s">
         <v>596</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (15/09/2026 12:33)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,16 +1815,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1840,7 +1832,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1848,30 +1840,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2171,55 +2145,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2263,7 +2237,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2307,7 +2281,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2351,7 +2325,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2477,7 +2451,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2521,7 +2495,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2565,7 +2539,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2612,7 +2586,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2735,7 +2709,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2779,7 +2753,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2823,7 +2797,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2914,7 +2888,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2958,7 +2932,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3084,7 +3058,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3128,7 +3102,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3213,7 +3187,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3260,7 +3234,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3307,7 +3281,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3351,7 +3325,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3395,7 +3369,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3480,7 +3454,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3565,7 +3539,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3612,7 +3586,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3656,7 +3630,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3700,7 +3674,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3785,7 +3759,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3829,7 +3803,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3873,7 +3847,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3958,7 +3932,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4002,7 +3976,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4046,7 +4020,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4090,7 +4064,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4257,7 +4231,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4301,7 +4275,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4345,7 +4319,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4389,7 +4363,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4436,7 +4410,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4480,7 +4454,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4562,7 +4536,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4606,7 +4580,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4694,7 +4668,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4738,7 +4712,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4785,7 +4759,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4829,7 +4803,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4873,7 +4847,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4917,7 +4891,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4961,7 +4935,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5008,7 +4982,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5052,7 +5026,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5099,7 +5073,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5143,7 +5117,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5190,7 +5164,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5278,7 +5252,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5322,7 +5296,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5366,7 +5340,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5410,7 +5384,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5454,7 +5428,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5498,7 +5472,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5583,7 +5557,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5627,7 +5601,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5671,7 +5645,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5715,7 +5689,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5759,7 +5733,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5803,7 +5777,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5847,7 +5821,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5891,7 +5865,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5938,7 +5912,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5982,7 +5956,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6026,7 +6000,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6070,7 +6044,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6114,7 +6088,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6158,7 +6132,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6202,7 +6176,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6246,7 +6220,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6290,7 +6264,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6378,7 +6352,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6422,7 +6396,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6592,7 +6566,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6636,7 +6610,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6680,7 +6654,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6762,7 +6736,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6806,7 +6780,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6853,7 +6827,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6897,7 +6871,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7023,7 +6997,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7067,7 +7041,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7152,7 +7126,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7196,7 +7170,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7240,7 +7214,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7284,7 +7258,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7328,7 +7302,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7372,7 +7346,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7416,7 +7390,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7460,7 +7434,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7545,7 +7519,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7712,7 +7686,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7756,7 +7730,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7800,7 +7774,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7844,7 +7818,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7888,7 +7862,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7932,7 +7906,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7976,7 +7950,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8061,7 +8035,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8105,7 +8079,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8190,7 +8164,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8316,7 +8290,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8360,7 +8334,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8445,7 +8419,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8489,7 +8463,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8533,7 +8507,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8577,7 +8551,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8621,7 +8595,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8665,7 +8639,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8709,7 +8683,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8753,7 +8727,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8838,7 +8812,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9005,7 +8979,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9049,7 +9023,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9093,7 +9067,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9137,7 +9111,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9222,7 +9196,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9266,7 +9240,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9310,7 +9284,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9354,7 +9328,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9398,7 +9372,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9442,7 +9416,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9486,7 +9460,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9530,7 +9504,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9574,7 +9548,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9618,7 +9592,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9662,7 +9636,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9706,7 +9680,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9750,7 +9724,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9794,7 +9768,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9838,7 +9812,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9882,7 +9856,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9926,7 +9900,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9970,7 +9944,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10014,7 +9988,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10058,7 +10032,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10102,7 +10076,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10187,7 +10161,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10272,7 +10246,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10287,55 +10261,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10622,7 +10596,7 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="1">
         <v>46290</v>
       </c>
       <c r="N8" t="s">
@@ -10707,7 +10681,7 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46355</v>
       </c>
       <c r="N10" t="s">
@@ -10751,7 +10725,7 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46355</v>
       </c>
       <c r="N11" t="s">
@@ -10918,7 +10892,7 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="1">
         <v>46290</v>
       </c>
       <c r="N15" t="s">
@@ -10962,7 +10936,7 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46355</v>
       </c>
       <c r="N16" t="s">
@@ -11006,7 +10980,7 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>46290</v>
       </c>
       <c r="N17" t="s">
@@ -11050,7 +11024,7 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46355</v>
       </c>
       <c r="N18" t="s">
@@ -11094,7 +11068,7 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46355</v>
       </c>
       <c r="N19" t="s">
@@ -11138,7 +11112,7 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46355</v>
       </c>
       <c r="N20" t="s">
@@ -11182,7 +11156,7 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46355</v>
       </c>
       <c r="N21" t="s">
@@ -11349,7 +11323,7 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46355</v>
       </c>
       <c r="N25" t="s">
@@ -11434,7 +11408,7 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="1">
         <v>46290</v>
       </c>
       <c r="N27" t="s">
@@ -11478,7 +11452,7 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46355</v>
       </c>
       <c r="N28" t="s">
@@ -11522,7 +11496,7 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46310</v>
       </c>
       <c r="N29" t="s">
@@ -11566,7 +11540,7 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46355</v>
       </c>
       <c r="N30" t="s">
@@ -11610,7 +11584,7 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46310</v>
       </c>
       <c r="N31" t="s">
@@ -11654,7 +11628,7 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="2">
+      <c r="M32" s="1">
         <v>46290</v>
       </c>
       <c r="N32" t="s">
@@ -11698,7 +11672,7 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="2">
+      <c r="M33" s="1">
         <v>46290</v>
       </c>
       <c r="N33" t="s">
@@ -11742,7 +11716,7 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="2">
+      <c r="M34" s="1">
         <v>46290</v>
       </c>
       <c r="N34" t="s">
@@ -11786,7 +11760,7 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="2">
+      <c r="M35" s="1">
         <v>46290</v>
       </c>
       <c r="N35" t="s">
@@ -11830,7 +11804,7 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="2">
+      <c r="M36" s="1">
         <v>46290</v>
       </c>
       <c r="N36" t="s">
@@ -11874,7 +11848,7 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="2">
+      <c r="M37" s="1">
         <v>46290</v>
       </c>
       <c r="N37" t="s">
@@ -11918,7 +11892,7 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="2">
+      <c r="M38" s="1">
         <v>46290</v>
       </c>
       <c r="N38" t="s">
@@ -12003,7 +11977,7 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="2">
+      <c r="M40" s="1">
         <v>46290</v>
       </c>
       <c r="N40" t="s">
@@ -12047,7 +12021,7 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46355</v>
       </c>
       <c r="N41" t="s">
@@ -12091,7 +12065,7 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M42" s="1">
         <v>46290</v>
       </c>
       <c r="N42" t="s">
@@ -12135,7 +12109,7 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46355</v>
       </c>
       <c r="N43" t="s">
@@ -12179,7 +12153,7 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46355</v>
       </c>
       <c r="N44" t="s">
@@ -12223,7 +12197,7 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46355</v>
       </c>
       <c r="N45" t="s">
@@ -12267,7 +12241,7 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="2">
+      <c r="M46" s="1">
         <v>46290</v>
       </c>
       <c r="N46" t="s">
@@ -12311,7 +12285,7 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46290</v>
       </c>
       <c r="N47" t="s">
@@ -12355,7 +12329,7 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46355</v>
       </c>
       <c r="N48" t="s">
@@ -12399,7 +12373,7 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46310</v>
       </c>
       <c r="N49" t="s">
@@ -12443,7 +12417,7 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46310</v>
       </c>
       <c r="N50" t="s">
@@ -12487,7 +12461,7 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46355</v>
       </c>
       <c r="N51" t="s">
@@ -12531,7 +12505,7 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46355</v>
       </c>
       <c r="N52" t="s">
@@ -12575,7 +12549,7 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46355</v>
       </c>
       <c r="N53" t="s">
@@ -12619,7 +12593,7 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46355</v>
       </c>
       <c r="N54" t="s">
@@ -12663,7 +12637,7 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46355</v>
       </c>
       <c r="N55" t="s">
@@ -12707,7 +12681,7 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46310</v>
       </c>
       <c r="N56" t="s">
@@ -12751,7 +12725,7 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46310</v>
       </c>
       <c r="N57" t="s">
@@ -12795,7 +12769,7 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46310</v>
       </c>
       <c r="N58" t="s">
@@ -12839,7 +12813,7 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46355</v>
       </c>
       <c r="N59" t="s">
@@ -12883,7 +12857,7 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46310</v>
       </c>
       <c r="N60" t="s">
@@ -12927,7 +12901,7 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46310</v>
       </c>
       <c r="N61" t="s">
@@ -12971,7 +12945,7 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46355</v>
       </c>
       <c r="N62" t="s">
@@ -13015,7 +12989,7 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46355</v>
       </c>
       <c r="N63" t="s">
@@ -13059,7 +13033,7 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46355</v>
       </c>
       <c r="N64" t="s">
@@ -13103,7 +13077,7 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="1">
         <v>46355</v>
       </c>
       <c r="N65" t="s">
@@ -13147,7 +13121,7 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="1">
         <v>46355</v>
       </c>
       <c r="N66" t="s">
@@ -13191,7 +13165,7 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="2">
+      <c r="M67" s="1">
         <v>46355</v>
       </c>
       <c r="N67" t="s">
@@ -13235,7 +13209,7 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="2">
+      <c r="M68" s="1">
         <v>46355</v>
       </c>
       <c r="N68" t="s">
@@ -13279,7 +13253,7 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="2">
+      <c r="M69" s="1">
         <v>46355</v>
       </c>
       <c r="N69" t="s">
@@ -13364,7 +13338,7 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="2">
+      <c r="M71" s="1">
         <v>46370</v>
       </c>
       <c r="N71" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (15/09/2026 14:02)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,8 +1815,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1832,7 +1840,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1840,12 +1848,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2145,55 +2171,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2237,7 +2263,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2281,7 +2307,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2325,7 +2351,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2451,7 +2477,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2495,7 +2521,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2539,7 +2565,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2586,7 +2612,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2709,7 +2735,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2753,7 +2779,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2797,7 +2823,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2888,7 +2914,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2932,7 +2958,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3058,7 +3084,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3102,7 +3128,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3187,7 +3213,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3234,7 +3260,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3281,7 +3307,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3325,7 +3351,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3369,7 +3395,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3454,7 +3480,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3539,7 +3565,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3586,7 +3612,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3630,7 +3656,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3674,7 +3700,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3759,7 +3785,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3803,7 +3829,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3847,7 +3873,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3932,7 +3958,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3976,7 +4002,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4020,7 +4046,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4064,7 +4090,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4231,7 +4257,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4275,7 +4301,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4319,7 +4345,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4363,7 +4389,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4410,7 +4436,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4454,7 +4480,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4536,7 +4562,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4580,7 +4606,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4668,7 +4694,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4712,7 +4738,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4759,7 +4785,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4803,7 +4829,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4847,7 +4873,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4891,7 +4917,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4935,7 +4961,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4982,7 +5008,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5026,7 +5052,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5073,7 +5099,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5117,7 +5143,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5164,7 +5190,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5252,7 +5278,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5296,7 +5322,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5340,7 +5366,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5384,7 +5410,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5428,7 +5454,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5472,7 +5498,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5557,7 +5583,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5601,7 +5627,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5645,7 +5671,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5689,7 +5715,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5733,7 +5759,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5777,7 +5803,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5821,7 +5847,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5865,7 +5891,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5912,7 +5938,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5956,7 +5982,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6000,7 +6026,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6044,7 +6070,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6088,7 +6114,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6132,7 +6158,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6176,7 +6202,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6220,7 +6246,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6264,7 +6290,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6352,7 +6378,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6396,7 +6422,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6566,7 +6592,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6610,7 +6636,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6654,7 +6680,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6736,7 +6762,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6780,7 +6806,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6827,7 +6853,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6871,7 +6897,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6997,7 +7023,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7041,7 +7067,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7126,7 +7152,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7170,7 +7196,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7214,7 +7240,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7258,7 +7284,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7302,7 +7328,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7346,7 +7372,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7390,7 +7416,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7434,7 +7460,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7519,7 +7545,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7686,7 +7712,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7730,7 +7756,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7774,7 +7800,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7818,7 +7844,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7862,7 +7888,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7906,7 +7932,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7950,7 +7976,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8035,7 +8061,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8079,7 +8105,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8164,7 +8190,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8290,7 +8316,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8334,7 +8360,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8419,7 +8445,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8463,7 +8489,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8507,7 +8533,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8551,7 +8577,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8595,7 +8621,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8639,7 +8665,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8683,7 +8709,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8727,7 +8753,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8812,7 +8838,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8979,7 +9005,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9023,7 +9049,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9067,7 +9093,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9111,7 +9137,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9196,7 +9222,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9240,7 +9266,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9284,7 +9310,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9328,7 +9354,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9372,7 +9398,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9416,7 +9442,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9460,7 +9486,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9504,7 +9530,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9548,7 +9574,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9592,7 +9618,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9636,7 +9662,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9680,7 +9706,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9724,7 +9750,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9768,7 +9794,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9812,7 +9838,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9856,7 +9882,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9900,7 +9926,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9944,7 +9970,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9988,7 +10014,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10032,7 +10058,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10076,7 +10102,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10161,7 +10187,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10246,7 +10272,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10261,55 +10287,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10596,7 +10622,7 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="2">
         <v>46290</v>
       </c>
       <c r="N8" t="s">
@@ -10681,7 +10707,7 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46355</v>
       </c>
       <c r="N10" t="s">
@@ -10725,7 +10751,7 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46355</v>
       </c>
       <c r="N11" t="s">
@@ -10892,7 +10918,7 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="2">
         <v>46290</v>
       </c>
       <c r="N15" t="s">
@@ -10936,7 +10962,7 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46355</v>
       </c>
       <c r="N16" t="s">
@@ -10980,7 +11006,7 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M17" s="2">
         <v>46290</v>
       </c>
       <c r="N17" t="s">
@@ -11024,7 +11050,7 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>46355</v>
       </c>
       <c r="N18" t="s">
@@ -11068,7 +11094,7 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46355</v>
       </c>
       <c r="N19" t="s">
@@ -11112,7 +11138,7 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46355</v>
       </c>
       <c r="N20" t="s">
@@ -11156,7 +11182,7 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46355</v>
       </c>
       <c r="N21" t="s">
@@ -11323,7 +11349,7 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46355</v>
       </c>
       <c r="N25" t="s">
@@ -11408,7 +11434,7 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="1">
+      <c r="M27" s="2">
         <v>46290</v>
       </c>
       <c r="N27" t="s">
@@ -11452,7 +11478,7 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46355</v>
       </c>
       <c r="N28" t="s">
@@ -11496,7 +11522,7 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="2">
         <v>46310</v>
       </c>
       <c r="N29" t="s">
@@ -11540,7 +11566,7 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46355</v>
       </c>
       <c r="N30" t="s">
@@ -11584,7 +11610,7 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="2">
         <v>46310</v>
       </c>
       <c r="N31" t="s">
@@ -11628,7 +11654,7 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="1">
+      <c r="M32" s="2">
         <v>46290</v>
       </c>
       <c r="N32" t="s">
@@ -11672,7 +11698,7 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="1">
+      <c r="M33" s="2">
         <v>46290</v>
       </c>
       <c r="N33" t="s">
@@ -11716,7 +11742,7 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="1">
+      <c r="M34" s="2">
         <v>46290</v>
       </c>
       <c r="N34" t="s">
@@ -11760,7 +11786,7 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="1">
+      <c r="M35" s="2">
         <v>46290</v>
       </c>
       <c r="N35" t="s">
@@ -11804,7 +11830,7 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="1">
+      <c r="M36" s="2">
         <v>46290</v>
       </c>
       <c r="N36" t="s">
@@ -11848,7 +11874,7 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="1">
+      <c r="M37" s="2">
         <v>46290</v>
       </c>
       <c r="N37" t="s">
@@ -11892,7 +11918,7 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="1">
+      <c r="M38" s="2">
         <v>46290</v>
       </c>
       <c r="N38" t="s">
@@ -11977,7 +12003,7 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="1">
+      <c r="M40" s="2">
         <v>46290</v>
       </c>
       <c r="N40" t="s">
@@ -12021,7 +12047,7 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46355</v>
       </c>
       <c r="N41" t="s">
@@ -12065,7 +12091,7 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="1">
+      <c r="M42" s="2">
         <v>46290</v>
       </c>
       <c r="N42" t="s">
@@ -12109,7 +12135,7 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46355</v>
       </c>
       <c r="N43" t="s">
@@ -12153,7 +12179,7 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46355</v>
       </c>
       <c r="N44" t="s">
@@ -12197,7 +12223,7 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46355</v>
       </c>
       <c r="N45" t="s">
@@ -12241,7 +12267,7 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="1">
+      <c r="M46" s="2">
         <v>46290</v>
       </c>
       <c r="N46" t="s">
@@ -12285,7 +12311,7 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="1">
+      <c r="M47" s="2">
         <v>46290</v>
       </c>
       <c r="N47" t="s">
@@ -12329,7 +12355,7 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46355</v>
       </c>
       <c r="N48" t="s">
@@ -12373,7 +12399,7 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46310</v>
       </c>
       <c r="N49" t="s">
@@ -12417,7 +12443,7 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46310</v>
       </c>
       <c r="N50" t="s">
@@ -12461,7 +12487,7 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46355</v>
       </c>
       <c r="N51" t="s">
@@ -12505,7 +12531,7 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46355</v>
       </c>
       <c r="N52" t="s">
@@ -12549,7 +12575,7 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46355</v>
       </c>
       <c r="N53" t="s">
@@ -12593,7 +12619,7 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46355</v>
       </c>
       <c r="N54" t="s">
@@ -12637,7 +12663,7 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46355</v>
       </c>
       <c r="N55" t="s">
@@ -12681,7 +12707,7 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="1">
+      <c r="M56" s="2">
         <v>46310</v>
       </c>
       <c r="N56" t="s">
@@ -12725,7 +12751,7 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="1">
+      <c r="M57" s="2">
         <v>46310</v>
       </c>
       <c r="N57" t="s">
@@ -12769,7 +12795,7 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="1">
+      <c r="M58" s="2">
         <v>46310</v>
       </c>
       <c r="N58" t="s">
@@ -12813,7 +12839,7 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46355</v>
       </c>
       <c r="N59" t="s">
@@ -12857,7 +12883,7 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="1">
+      <c r="M60" s="2">
         <v>46310</v>
       </c>
       <c r="N60" t="s">
@@ -12901,7 +12927,7 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="1">
+      <c r="M61" s="2">
         <v>46310</v>
       </c>
       <c r="N61" t="s">
@@ -12945,7 +12971,7 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46355</v>
       </c>
       <c r="N62" t="s">
@@ -12989,7 +13015,7 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46355</v>
       </c>
       <c r="N63" t="s">
@@ -13033,7 +13059,7 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46355</v>
       </c>
       <c r="N64" t="s">
@@ -13077,7 +13103,7 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="1">
+      <c r="M65" s="2">
         <v>46355</v>
       </c>
       <c r="N65" t="s">
@@ -13121,7 +13147,7 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="1">
+      <c r="M66" s="2">
         <v>46355</v>
       </c>
       <c r="N66" t="s">
@@ -13165,7 +13191,7 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="1">
+      <c r="M67" s="2">
         <v>46355</v>
       </c>
       <c r="N67" t="s">
@@ -13209,7 +13235,7 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="1">
+      <c r="M68" s="2">
         <v>46355</v>
       </c>
       <c r="N68" t="s">
@@ -13253,7 +13279,7 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="1">
+      <c r="M69" s="2">
         <v>46355</v>
       </c>
       <c r="N69" t="s">
@@ -13338,7 +13364,7 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="1">
+      <c r="M71" s="2">
         <v>46370</v>
       </c>
       <c r="N71" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (16/09/2026 12:25)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,16 +1815,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1840,7 +1832,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1848,30 +1840,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2171,55 +2145,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2263,7 +2237,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2307,7 +2281,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2351,7 +2325,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2477,7 +2451,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2521,7 +2495,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2565,7 +2539,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2612,7 +2586,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2735,7 +2709,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2779,7 +2753,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2823,7 +2797,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2914,7 +2888,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2958,7 +2932,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3084,7 +3058,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3128,7 +3102,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3213,7 +3187,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3260,7 +3234,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3307,7 +3281,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3351,7 +3325,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3395,7 +3369,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3480,7 +3454,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3565,7 +3539,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3612,7 +3586,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3656,7 +3630,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3700,7 +3674,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3785,7 +3759,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3829,7 +3803,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3873,7 +3847,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3958,7 +3932,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4002,7 +3976,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4046,7 +4020,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4090,7 +4064,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4257,7 +4231,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4301,7 +4275,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4345,7 +4319,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4389,7 +4363,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4436,7 +4410,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4480,7 +4454,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4562,7 +4536,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4606,7 +4580,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4694,7 +4668,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4738,7 +4712,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4785,7 +4759,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4829,7 +4803,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4873,7 +4847,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4917,7 +4891,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4961,7 +4935,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5008,7 +4982,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5052,7 +5026,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5099,7 +5073,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5143,7 +5117,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5190,7 +5164,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5278,7 +5252,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5322,7 +5296,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5366,7 +5340,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5410,7 +5384,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5454,7 +5428,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5498,7 +5472,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5583,7 +5557,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5627,7 +5601,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5671,7 +5645,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5715,7 +5689,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5759,7 +5733,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5803,7 +5777,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5847,7 +5821,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5891,7 +5865,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5938,7 +5912,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5982,7 +5956,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6026,7 +6000,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6070,7 +6044,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6114,7 +6088,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6158,7 +6132,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6202,7 +6176,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6246,7 +6220,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6290,7 +6264,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6378,7 +6352,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6422,7 +6396,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6592,7 +6566,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6636,7 +6610,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6680,7 +6654,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6762,7 +6736,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6806,7 +6780,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6853,7 +6827,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6897,7 +6871,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7023,7 +6997,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7067,7 +7041,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7152,7 +7126,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7196,7 +7170,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7240,7 +7214,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7284,7 +7258,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7328,7 +7302,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7372,7 +7346,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7416,7 +7390,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7460,7 +7434,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7545,7 +7519,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7712,7 +7686,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7756,7 +7730,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7800,7 +7774,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7844,7 +7818,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7888,7 +7862,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7932,7 +7906,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7976,7 +7950,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8061,7 +8035,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8105,7 +8079,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8190,7 +8164,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8316,7 +8290,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8360,7 +8334,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8445,7 +8419,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8489,7 +8463,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8533,7 +8507,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8577,7 +8551,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8621,7 +8595,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8665,7 +8639,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8709,7 +8683,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8753,7 +8727,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8838,7 +8812,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9005,7 +8979,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9049,7 +9023,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9093,7 +9067,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9137,7 +9111,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9222,7 +9196,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9266,7 +9240,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9310,7 +9284,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9354,7 +9328,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9398,7 +9372,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9442,7 +9416,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9486,7 +9460,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9530,7 +9504,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9574,7 +9548,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9618,7 +9592,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9662,7 +9636,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9706,7 +9680,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9750,7 +9724,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9794,7 +9768,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9838,7 +9812,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9882,7 +9856,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9926,7 +9900,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9970,7 +9944,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10014,7 +9988,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10058,7 +10032,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10102,7 +10076,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10187,7 +10161,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10272,7 +10246,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10287,55 +10261,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10622,8 +10596,8 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="2">
-        <v>46290</v>
+      <c r="M8" s="1">
+        <v>46291</v>
       </c>
       <c r="N8" t="s">
         <v>596</v>
@@ -10707,8 +10681,8 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="2">
-        <v>46355</v>
+      <c r="M10" s="1">
+        <v>46356</v>
       </c>
       <c r="N10" t="s">
         <v>596</v>
@@ -10751,8 +10725,8 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="2">
-        <v>46355</v>
+      <c r="M11" s="1">
+        <v>46356</v>
       </c>
       <c r="N11" t="s">
         <v>596</v>
@@ -10918,8 +10892,8 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="2">
-        <v>46290</v>
+      <c r="M15" s="1">
+        <v>46291</v>
       </c>
       <c r="N15" t="s">
         <v>596</v>
@@ -10962,8 +10936,8 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="2">
-        <v>46355</v>
+      <c r="M16" s="1">
+        <v>46356</v>
       </c>
       <c r="N16" t="s">
         <v>596</v>
@@ -11006,8 +10980,8 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="2">
-        <v>46290</v>
+      <c r="M17" s="1">
+        <v>46291</v>
       </c>
       <c r="N17" t="s">
         <v>596</v>
@@ -11050,8 +11024,8 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="2">
-        <v>46355</v>
+      <c r="M18" s="1">
+        <v>46356</v>
       </c>
       <c r="N18" t="s">
         <v>596</v>
@@ -11094,8 +11068,8 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="2">
-        <v>46355</v>
+      <c r="M19" s="1">
+        <v>46356</v>
       </c>
       <c r="N19" t="s">
         <v>596</v>
@@ -11138,8 +11112,8 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="2">
-        <v>46355</v>
+      <c r="M20" s="1">
+        <v>46356</v>
       </c>
       <c r="N20" t="s">
         <v>596</v>
@@ -11182,8 +11156,8 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="2">
-        <v>46355</v>
+      <c r="M21" s="1">
+        <v>46356</v>
       </c>
       <c r="N21" t="s">
         <v>596</v>
@@ -11349,8 +11323,8 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="2">
-        <v>46355</v>
+      <c r="M25" s="1">
+        <v>46356</v>
       </c>
       <c r="N25" t="s">
         <v>596</v>
@@ -11434,8 +11408,8 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="2">
-        <v>46290</v>
+      <c r="M27" s="1">
+        <v>46291</v>
       </c>
       <c r="N27" t="s">
         <v>596</v>
@@ -11478,8 +11452,8 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="2">
-        <v>46355</v>
+      <c r="M28" s="1">
+        <v>46356</v>
       </c>
       <c r="N28" t="s">
         <v>596</v>
@@ -11522,8 +11496,8 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="2">
-        <v>46310</v>
+      <c r="M29" s="1">
+        <v>46311</v>
       </c>
       <c r="N29" t="s">
         <v>596</v>
@@ -11566,8 +11540,8 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="2">
-        <v>46355</v>
+      <c r="M30" s="1">
+        <v>46356</v>
       </c>
       <c r="N30" t="s">
         <v>596</v>
@@ -11610,8 +11584,8 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="2">
-        <v>46310</v>
+      <c r="M31" s="1">
+        <v>46311</v>
       </c>
       <c r="N31" t="s">
         <v>596</v>
@@ -11654,8 +11628,8 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="2">
-        <v>46290</v>
+      <c r="M32" s="1">
+        <v>46291</v>
       </c>
       <c r="N32" t="s">
         <v>596</v>
@@ -11698,8 +11672,8 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="2">
-        <v>46290</v>
+      <c r="M33" s="1">
+        <v>46291</v>
       </c>
       <c r="N33" t="s">
         <v>596</v>
@@ -11742,8 +11716,8 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="2">
-        <v>46290</v>
+      <c r="M34" s="1">
+        <v>46291</v>
       </c>
       <c r="N34" t="s">
         <v>596</v>
@@ -11786,8 +11760,8 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="2">
-        <v>46290</v>
+      <c r="M35" s="1">
+        <v>46291</v>
       </c>
       <c r="N35" t="s">
         <v>596</v>
@@ -11830,8 +11804,8 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="2">
-        <v>46290</v>
+      <c r="M36" s="1">
+        <v>46291</v>
       </c>
       <c r="N36" t="s">
         <v>596</v>
@@ -11874,8 +11848,8 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="2">
-        <v>46290</v>
+      <c r="M37" s="1">
+        <v>46291</v>
       </c>
       <c r="N37" t="s">
         <v>596</v>
@@ -11918,8 +11892,8 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="2">
-        <v>46290</v>
+      <c r="M38" s="1">
+        <v>46291</v>
       </c>
       <c r="N38" t="s">
         <v>596</v>
@@ -12003,8 +11977,8 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="2">
-        <v>46290</v>
+      <c r="M40" s="1">
+        <v>46291</v>
       </c>
       <c r="N40" t="s">
         <v>596</v>
@@ -12047,8 +12021,8 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="2">
-        <v>46355</v>
+      <c r="M41" s="1">
+        <v>46356</v>
       </c>
       <c r="N41" t="s">
         <v>596</v>
@@ -12091,8 +12065,8 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="2">
-        <v>46290</v>
+      <c r="M42" s="1">
+        <v>46291</v>
       </c>
       <c r="N42" t="s">
         <v>596</v>
@@ -12135,8 +12109,8 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="2">
-        <v>46355</v>
+      <c r="M43" s="1">
+        <v>46356</v>
       </c>
       <c r="N43" t="s">
         <v>596</v>
@@ -12179,8 +12153,8 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="2">
-        <v>46355</v>
+      <c r="M44" s="1">
+        <v>46356</v>
       </c>
       <c r="N44" t="s">
         <v>596</v>
@@ -12223,8 +12197,8 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="2">
-        <v>46355</v>
+      <c r="M45" s="1">
+        <v>46356</v>
       </c>
       <c r="N45" t="s">
         <v>596</v>
@@ -12267,8 +12241,8 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="2">
-        <v>46290</v>
+      <c r="M46" s="1">
+        <v>46291</v>
       </c>
       <c r="N46" t="s">
         <v>596</v>
@@ -12311,8 +12285,8 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="2">
-        <v>46290</v>
+      <c r="M47" s="1">
+        <v>46291</v>
       </c>
       <c r="N47" t="s">
         <v>596</v>
@@ -12355,8 +12329,8 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="2">
-        <v>46355</v>
+      <c r="M48" s="1">
+        <v>46356</v>
       </c>
       <c r="N48" t="s">
         <v>596</v>
@@ -12399,8 +12373,8 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="2">
-        <v>46310</v>
+      <c r="M49" s="1">
+        <v>46311</v>
       </c>
       <c r="N49" t="s">
         <v>596</v>
@@ -12443,8 +12417,8 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="2">
-        <v>46310</v>
+      <c r="M50" s="1">
+        <v>46311</v>
       </c>
       <c r="N50" t="s">
         <v>596</v>
@@ -12487,8 +12461,8 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="2">
-        <v>46355</v>
+      <c r="M51" s="1">
+        <v>46356</v>
       </c>
       <c r="N51" t="s">
         <v>596</v>
@@ -12531,8 +12505,8 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="2">
-        <v>46355</v>
+      <c r="M52" s="1">
+        <v>46356</v>
       </c>
       <c r="N52" t="s">
         <v>596</v>
@@ -12575,8 +12549,8 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="2">
-        <v>46355</v>
+      <c r="M53" s="1">
+        <v>46356</v>
       </c>
       <c r="N53" t="s">
         <v>596</v>
@@ -12619,8 +12593,8 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="2">
-        <v>46355</v>
+      <c r="M54" s="1">
+        <v>46356</v>
       </c>
       <c r="N54" t="s">
         <v>596</v>
@@ -12663,8 +12637,8 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="2">
-        <v>46355</v>
+      <c r="M55" s="1">
+        <v>46356</v>
       </c>
       <c r="N55" t="s">
         <v>596</v>
@@ -12707,8 +12681,8 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="2">
-        <v>46310</v>
+      <c r="M56" s="1">
+        <v>46311</v>
       </c>
       <c r="N56" t="s">
         <v>596</v>
@@ -12751,8 +12725,8 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="2">
-        <v>46310</v>
+      <c r="M57" s="1">
+        <v>46311</v>
       </c>
       <c r="N57" t="s">
         <v>596</v>
@@ -12795,8 +12769,8 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="2">
-        <v>46310</v>
+      <c r="M58" s="1">
+        <v>46311</v>
       </c>
       <c r="N58" t="s">
         <v>596</v>
@@ -12839,8 +12813,8 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="2">
-        <v>46355</v>
+      <c r="M59" s="1">
+        <v>46356</v>
       </c>
       <c r="N59" t="s">
         <v>596</v>
@@ -12883,8 +12857,8 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="2">
-        <v>46310</v>
+      <c r="M60" s="1">
+        <v>46311</v>
       </c>
       <c r="N60" t="s">
         <v>596</v>
@@ -12927,8 +12901,8 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="2">
-        <v>46310</v>
+      <c r="M61" s="1">
+        <v>46311</v>
       </c>
       <c r="N61" t="s">
         <v>596</v>
@@ -12971,8 +12945,8 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="2">
-        <v>46355</v>
+      <c r="M62" s="1">
+        <v>46356</v>
       </c>
       <c r="N62" t="s">
         <v>596</v>
@@ -13015,8 +12989,8 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="2">
-        <v>46355</v>
+      <c r="M63" s="1">
+        <v>46356</v>
       </c>
       <c r="N63" t="s">
         <v>596</v>
@@ -13059,8 +13033,8 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="2">
-        <v>46355</v>
+      <c r="M64" s="1">
+        <v>46356</v>
       </c>
       <c r="N64" t="s">
         <v>596</v>
@@ -13103,8 +13077,8 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="2">
-        <v>46355</v>
+      <c r="M65" s="1">
+        <v>46356</v>
       </c>
       <c r="N65" t="s">
         <v>596</v>
@@ -13147,8 +13121,8 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="2">
-        <v>46355</v>
+      <c r="M66" s="1">
+        <v>46356</v>
       </c>
       <c r="N66" t="s">
         <v>596</v>
@@ -13191,8 +13165,8 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="2">
-        <v>46355</v>
+      <c r="M67" s="1">
+        <v>46356</v>
       </c>
       <c r="N67" t="s">
         <v>596</v>
@@ -13235,8 +13209,8 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="2">
-        <v>46355</v>
+      <c r="M68" s="1">
+        <v>46356</v>
       </c>
       <c r="N68" t="s">
         <v>596</v>
@@ -13279,8 +13253,8 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="2">
-        <v>46355</v>
+      <c r="M69" s="1">
+        <v>46356</v>
       </c>
       <c r="N69" t="s">
         <v>596</v>
@@ -13364,8 +13338,8 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="2">
-        <v>46370</v>
+      <c r="M71" s="1">
+        <v>46371</v>
       </c>
       <c r="N71" t="s">
         <v>596</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (16/09/2026 12:42)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,8 +1815,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1832,7 +1840,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1840,12 +1848,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2145,55 +2171,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2237,7 +2263,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2281,7 +2307,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2325,7 +2351,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2451,7 +2477,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2495,7 +2521,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2539,7 +2565,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2586,7 +2612,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2709,7 +2735,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2753,7 +2779,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2797,7 +2823,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2888,7 +2914,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2932,7 +2958,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3058,7 +3084,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3102,7 +3128,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3187,7 +3213,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3234,7 +3260,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3281,7 +3307,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3325,7 +3351,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3369,7 +3395,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3454,7 +3480,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3539,7 +3565,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3586,7 +3612,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3630,7 +3656,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3674,7 +3700,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3759,7 +3785,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3803,7 +3829,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3847,7 +3873,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3932,7 +3958,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3976,7 +4002,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4020,7 +4046,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4064,7 +4090,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4231,7 +4257,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4275,7 +4301,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4319,7 +4345,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4363,7 +4389,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4410,7 +4436,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4454,7 +4480,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4536,7 +4562,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4580,7 +4606,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4668,7 +4694,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4712,7 +4738,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4759,7 +4785,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4803,7 +4829,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4847,7 +4873,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4891,7 +4917,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4935,7 +4961,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4982,7 +5008,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5026,7 +5052,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5073,7 +5099,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5117,7 +5143,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5164,7 +5190,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5252,7 +5278,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5296,7 +5322,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5340,7 +5366,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5384,7 +5410,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5428,7 +5454,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5472,7 +5498,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5557,7 +5583,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5601,7 +5627,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5645,7 +5671,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5689,7 +5715,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5733,7 +5759,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5777,7 +5803,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5821,7 +5847,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5865,7 +5891,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5912,7 +5938,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5956,7 +5982,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6000,7 +6026,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6044,7 +6070,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6088,7 +6114,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6132,7 +6158,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6176,7 +6202,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6220,7 +6246,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6264,7 +6290,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6352,7 +6378,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6396,7 +6422,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6566,7 +6592,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6610,7 +6636,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6654,7 +6680,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6736,7 +6762,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6780,7 +6806,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6827,7 +6853,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6871,7 +6897,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6997,7 +7023,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7041,7 +7067,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7126,7 +7152,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7170,7 +7196,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7214,7 +7240,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7258,7 +7284,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7302,7 +7328,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7346,7 +7372,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7390,7 +7416,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7434,7 +7460,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7519,7 +7545,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7686,7 +7712,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7730,7 +7756,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7774,7 +7800,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7818,7 +7844,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7862,7 +7888,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7906,7 +7932,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7950,7 +7976,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8035,7 +8061,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8079,7 +8105,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8164,7 +8190,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8290,7 +8316,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8334,7 +8360,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8419,7 +8445,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8463,7 +8489,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8507,7 +8533,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8551,7 +8577,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8595,7 +8621,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8639,7 +8665,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8683,7 +8709,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8727,7 +8753,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8812,7 +8838,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8979,7 +9005,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9023,7 +9049,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9067,7 +9093,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9111,7 +9137,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9196,7 +9222,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9240,7 +9266,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9284,7 +9310,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9328,7 +9354,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9372,7 +9398,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9416,7 +9442,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9460,7 +9486,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9504,7 +9530,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9548,7 +9574,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9592,7 +9618,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9636,7 +9662,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9680,7 +9706,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9724,7 +9750,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9768,7 +9794,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9812,7 +9838,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9856,7 +9882,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9900,7 +9926,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9944,7 +9970,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9988,7 +10014,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10032,7 +10058,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10076,7 +10102,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10161,7 +10187,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10246,7 +10272,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10261,55 +10287,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10596,7 +10622,7 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="2">
         <v>46291</v>
       </c>
       <c r="N8" t="s">
@@ -10681,7 +10707,7 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46356</v>
       </c>
       <c r="N10" t="s">
@@ -10725,7 +10751,7 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46356</v>
       </c>
       <c r="N11" t="s">
@@ -10892,7 +10918,7 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="2">
         <v>46291</v>
       </c>
       <c r="N15" t="s">
@@ -10936,7 +10962,7 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46356</v>
       </c>
       <c r="N16" t="s">
@@ -10980,7 +11006,7 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M17" s="2">
         <v>46291</v>
       </c>
       <c r="N17" t="s">
@@ -11024,7 +11050,7 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>46356</v>
       </c>
       <c r="N18" t="s">
@@ -11068,7 +11094,7 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46356</v>
       </c>
       <c r="N19" t="s">
@@ -11112,7 +11138,7 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46356</v>
       </c>
       <c r="N20" t="s">
@@ -11156,7 +11182,7 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46356</v>
       </c>
       <c r="N21" t="s">
@@ -11323,7 +11349,7 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46356</v>
       </c>
       <c r="N25" t="s">
@@ -11408,7 +11434,7 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="1">
+      <c r="M27" s="2">
         <v>46291</v>
       </c>
       <c r="N27" t="s">
@@ -11452,7 +11478,7 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46356</v>
       </c>
       <c r="N28" t="s">
@@ -11496,7 +11522,7 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="2">
         <v>46311</v>
       </c>
       <c r="N29" t="s">
@@ -11540,7 +11566,7 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46356</v>
       </c>
       <c r="N30" t="s">
@@ -11584,7 +11610,7 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="2">
         <v>46311</v>
       </c>
       <c r="N31" t="s">
@@ -11628,7 +11654,7 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="1">
+      <c r="M32" s="2">
         <v>46291</v>
       </c>
       <c r="N32" t="s">
@@ -11672,7 +11698,7 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="1">
+      <c r="M33" s="2">
         <v>46291</v>
       </c>
       <c r="N33" t="s">
@@ -11716,7 +11742,7 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="1">
+      <c r="M34" s="2">
         <v>46291</v>
       </c>
       <c r="N34" t="s">
@@ -11760,7 +11786,7 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="1">
+      <c r="M35" s="2">
         <v>46291</v>
       </c>
       <c r="N35" t="s">
@@ -11804,7 +11830,7 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="1">
+      <c r="M36" s="2">
         <v>46291</v>
       </c>
       <c r="N36" t="s">
@@ -11848,7 +11874,7 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="1">
+      <c r="M37" s="2">
         <v>46291</v>
       </c>
       <c r="N37" t="s">
@@ -11892,7 +11918,7 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="1">
+      <c r="M38" s="2">
         <v>46291</v>
       </c>
       <c r="N38" t="s">
@@ -11977,7 +12003,7 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="1">
+      <c r="M40" s="2">
         <v>46291</v>
       </c>
       <c r="N40" t="s">
@@ -12021,7 +12047,7 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46356</v>
       </c>
       <c r="N41" t="s">
@@ -12065,7 +12091,7 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="1">
+      <c r="M42" s="2">
         <v>46291</v>
       </c>
       <c r="N42" t="s">
@@ -12109,7 +12135,7 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46356</v>
       </c>
       <c r="N43" t="s">
@@ -12153,7 +12179,7 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46356</v>
       </c>
       <c r="N44" t="s">
@@ -12197,7 +12223,7 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46356</v>
       </c>
       <c r="N45" t="s">
@@ -12241,7 +12267,7 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="1">
+      <c r="M46" s="2">
         <v>46291</v>
       </c>
       <c r="N46" t="s">
@@ -12285,7 +12311,7 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="1">
+      <c r="M47" s="2">
         <v>46291</v>
       </c>
       <c r="N47" t="s">
@@ -12329,7 +12355,7 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46356</v>
       </c>
       <c r="N48" t="s">
@@ -12373,7 +12399,7 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46311</v>
       </c>
       <c r="N49" t="s">
@@ -12417,7 +12443,7 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46311</v>
       </c>
       <c r="N50" t="s">
@@ -12461,7 +12487,7 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46356</v>
       </c>
       <c r="N51" t="s">
@@ -12505,7 +12531,7 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46356</v>
       </c>
       <c r="N52" t="s">
@@ -12549,7 +12575,7 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46356</v>
       </c>
       <c r="N53" t="s">
@@ -12593,7 +12619,7 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46356</v>
       </c>
       <c r="N54" t="s">
@@ -12637,7 +12663,7 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46356</v>
       </c>
       <c r="N55" t="s">
@@ -12681,7 +12707,7 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="1">
+      <c r="M56" s="2">
         <v>46311</v>
       </c>
       <c r="N56" t="s">
@@ -12725,7 +12751,7 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="1">
+      <c r="M57" s="2">
         <v>46311</v>
       </c>
       <c r="N57" t="s">
@@ -12769,7 +12795,7 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="1">
+      <c r="M58" s="2">
         <v>46311</v>
       </c>
       <c r="N58" t="s">
@@ -12813,7 +12839,7 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46356</v>
       </c>
       <c r="N59" t="s">
@@ -12857,7 +12883,7 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="1">
+      <c r="M60" s="2">
         <v>46311</v>
       </c>
       <c r="N60" t="s">
@@ -12901,7 +12927,7 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="1">
+      <c r="M61" s="2">
         <v>46311</v>
       </c>
       <c r="N61" t="s">
@@ -12945,7 +12971,7 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46356</v>
       </c>
       <c r="N62" t="s">
@@ -12989,7 +13015,7 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46356</v>
       </c>
       <c r="N63" t="s">
@@ -13033,7 +13059,7 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46356</v>
       </c>
       <c r="N64" t="s">
@@ -13077,7 +13103,7 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="1">
+      <c r="M65" s="2">
         <v>46356</v>
       </c>
       <c r="N65" t="s">
@@ -13121,7 +13147,7 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="1">
+      <c r="M66" s="2">
         <v>46356</v>
       </c>
       <c r="N66" t="s">
@@ -13165,7 +13191,7 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="1">
+      <c r="M67" s="2">
         <v>46356</v>
       </c>
       <c r="N67" t="s">
@@ -13209,7 +13235,7 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="1">
+      <c r="M68" s="2">
         <v>46356</v>
       </c>
       <c r="N68" t="s">
@@ -13253,7 +13279,7 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="1">
+      <c r="M69" s="2">
         <v>46356</v>
       </c>
       <c r="N69" t="s">
@@ -13338,7 +13364,7 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="1">
+      <c r="M71" s="2">
         <v>46371</v>
       </c>
       <c r="N71" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (17/09/2026 12:33)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,16 +1815,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1840,7 +1832,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1848,30 +1840,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2171,55 +2145,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2263,7 +2237,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2307,7 +2281,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2351,7 +2325,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2477,7 +2451,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2521,7 +2495,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2565,7 +2539,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2612,7 +2586,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2735,7 +2709,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2779,7 +2753,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2823,7 +2797,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2914,7 +2888,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2958,7 +2932,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3084,7 +3058,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3128,7 +3102,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3213,7 +3187,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3260,7 +3234,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3307,7 +3281,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3351,7 +3325,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3395,7 +3369,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3480,7 +3454,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3565,7 +3539,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3612,7 +3586,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3656,7 +3630,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3700,7 +3674,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3785,7 +3759,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3829,7 +3803,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3873,7 +3847,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3958,7 +3932,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4002,7 +3976,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4046,7 +4020,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4090,7 +4064,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4257,7 +4231,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4301,7 +4275,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4345,7 +4319,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4389,7 +4363,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4436,7 +4410,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4480,7 +4454,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4562,7 +4536,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4606,7 +4580,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4694,7 +4668,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4738,7 +4712,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4785,7 +4759,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4829,7 +4803,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4873,7 +4847,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4917,7 +4891,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4961,7 +4935,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5008,7 +4982,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5052,7 +5026,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5099,7 +5073,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5143,7 +5117,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5190,7 +5164,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5278,7 +5252,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5322,7 +5296,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5366,7 +5340,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5410,7 +5384,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5454,7 +5428,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5498,7 +5472,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5583,7 +5557,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5627,7 +5601,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5671,7 +5645,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5715,7 +5689,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5759,7 +5733,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5803,7 +5777,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5847,7 +5821,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5891,7 +5865,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5938,7 +5912,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5982,7 +5956,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6026,7 +6000,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6070,7 +6044,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6114,7 +6088,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6158,7 +6132,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6202,7 +6176,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6246,7 +6220,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6290,7 +6264,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6378,7 +6352,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6422,7 +6396,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6592,7 +6566,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6636,7 +6610,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6680,7 +6654,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6762,7 +6736,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6806,7 +6780,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6853,7 +6827,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6897,7 +6871,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7023,7 +6997,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7067,7 +7041,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7152,7 +7126,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7196,7 +7170,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7240,7 +7214,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7284,7 +7258,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7328,7 +7302,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7372,7 +7346,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7416,7 +7390,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7460,7 +7434,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7545,7 +7519,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7712,7 +7686,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7756,7 +7730,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7800,7 +7774,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7844,7 +7818,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7888,7 +7862,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7932,7 +7906,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7976,7 +7950,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8061,7 +8035,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8105,7 +8079,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8190,7 +8164,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8316,7 +8290,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8360,7 +8334,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8445,7 +8419,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8489,7 +8463,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8533,7 +8507,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8577,7 +8551,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8621,7 +8595,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8665,7 +8639,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8709,7 +8683,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8753,7 +8727,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8838,7 +8812,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9005,7 +8979,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9049,7 +9023,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9093,7 +9067,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9137,7 +9111,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9222,7 +9196,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9266,7 +9240,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9310,7 +9284,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9354,7 +9328,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9398,7 +9372,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9442,7 +9416,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9486,7 +9460,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9530,7 +9504,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9574,7 +9548,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9618,7 +9592,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9662,7 +9636,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9706,7 +9680,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9750,7 +9724,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9794,7 +9768,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9838,7 +9812,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9882,7 +9856,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9926,7 +9900,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9970,7 +9944,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10014,7 +9988,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10058,7 +10032,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10102,7 +10076,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10187,7 +10161,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10272,7 +10246,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10287,55 +10261,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10622,8 +10596,8 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="2">
-        <v>46291</v>
+      <c r="M8" s="1">
+        <v>46292</v>
       </c>
       <c r="N8" t="s">
         <v>596</v>
@@ -10707,8 +10681,8 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="2">
-        <v>46356</v>
+      <c r="M10" s="1">
+        <v>46357</v>
       </c>
       <c r="N10" t="s">
         <v>596</v>
@@ -10751,8 +10725,8 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="2">
-        <v>46356</v>
+      <c r="M11" s="1">
+        <v>46357</v>
       </c>
       <c r="N11" t="s">
         <v>596</v>
@@ -10918,8 +10892,8 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="2">
-        <v>46291</v>
+      <c r="M15" s="1">
+        <v>46292</v>
       </c>
       <c r="N15" t="s">
         <v>596</v>
@@ -10962,8 +10936,8 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="2">
-        <v>46356</v>
+      <c r="M16" s="1">
+        <v>46357</v>
       </c>
       <c r="N16" t="s">
         <v>596</v>
@@ -11006,8 +10980,8 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="2">
-        <v>46291</v>
+      <c r="M17" s="1">
+        <v>46292</v>
       </c>
       <c r="N17" t="s">
         <v>596</v>
@@ -11050,8 +11024,8 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="2">
-        <v>46356</v>
+      <c r="M18" s="1">
+        <v>46357</v>
       </c>
       <c r="N18" t="s">
         <v>596</v>
@@ -11094,8 +11068,8 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="2">
-        <v>46356</v>
+      <c r="M19" s="1">
+        <v>46357</v>
       </c>
       <c r="N19" t="s">
         <v>596</v>
@@ -11138,8 +11112,8 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="2">
-        <v>46356</v>
+      <c r="M20" s="1">
+        <v>46357</v>
       </c>
       <c r="N20" t="s">
         <v>596</v>
@@ -11182,8 +11156,8 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="2">
-        <v>46356</v>
+      <c r="M21" s="1">
+        <v>46357</v>
       </c>
       <c r="N21" t="s">
         <v>596</v>
@@ -11349,8 +11323,8 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="2">
-        <v>46356</v>
+      <c r="M25" s="1">
+        <v>46357</v>
       </c>
       <c r="N25" t="s">
         <v>596</v>
@@ -11434,8 +11408,8 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="2">
-        <v>46291</v>
+      <c r="M27" s="1">
+        <v>46292</v>
       </c>
       <c r="N27" t="s">
         <v>596</v>
@@ -11478,8 +11452,8 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="2">
-        <v>46356</v>
+      <c r="M28" s="1">
+        <v>46357</v>
       </c>
       <c r="N28" t="s">
         <v>596</v>
@@ -11522,8 +11496,8 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="2">
-        <v>46311</v>
+      <c r="M29" s="1">
+        <v>46312</v>
       </c>
       <c r="N29" t="s">
         <v>596</v>
@@ -11566,8 +11540,8 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="2">
-        <v>46356</v>
+      <c r="M30" s="1">
+        <v>46357</v>
       </c>
       <c r="N30" t="s">
         <v>596</v>
@@ -11610,8 +11584,8 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="2">
-        <v>46311</v>
+      <c r="M31" s="1">
+        <v>46312</v>
       </c>
       <c r="N31" t="s">
         <v>596</v>
@@ -11654,8 +11628,8 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="2">
-        <v>46291</v>
+      <c r="M32" s="1">
+        <v>46292</v>
       </c>
       <c r="N32" t="s">
         <v>596</v>
@@ -11698,8 +11672,8 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="2">
-        <v>46291</v>
+      <c r="M33" s="1">
+        <v>46292</v>
       </c>
       <c r="N33" t="s">
         <v>596</v>
@@ -11742,8 +11716,8 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="2">
-        <v>46291</v>
+      <c r="M34" s="1">
+        <v>46292</v>
       </c>
       <c r="N34" t="s">
         <v>596</v>
@@ -11786,8 +11760,8 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="2">
-        <v>46291</v>
+      <c r="M35" s="1">
+        <v>46292</v>
       </c>
       <c r="N35" t="s">
         <v>596</v>
@@ -11830,8 +11804,8 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="2">
-        <v>46291</v>
+      <c r="M36" s="1">
+        <v>46292</v>
       </c>
       <c r="N36" t="s">
         <v>596</v>
@@ -11874,8 +11848,8 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="2">
-        <v>46291</v>
+      <c r="M37" s="1">
+        <v>46292</v>
       </c>
       <c r="N37" t="s">
         <v>596</v>
@@ -11918,8 +11892,8 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="2">
-        <v>46291</v>
+      <c r="M38" s="1">
+        <v>46292</v>
       </c>
       <c r="N38" t="s">
         <v>596</v>
@@ -12003,8 +11977,8 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="2">
-        <v>46291</v>
+      <c r="M40" s="1">
+        <v>46292</v>
       </c>
       <c r="N40" t="s">
         <v>596</v>
@@ -12047,8 +12021,8 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="2">
-        <v>46356</v>
+      <c r="M41" s="1">
+        <v>46357</v>
       </c>
       <c r="N41" t="s">
         <v>596</v>
@@ -12091,8 +12065,8 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="2">
-        <v>46291</v>
+      <c r="M42" s="1">
+        <v>46292</v>
       </c>
       <c r="N42" t="s">
         <v>596</v>
@@ -12135,8 +12109,8 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="2">
-        <v>46356</v>
+      <c r="M43" s="1">
+        <v>46357</v>
       </c>
       <c r="N43" t="s">
         <v>596</v>
@@ -12179,8 +12153,8 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="2">
-        <v>46356</v>
+      <c r="M44" s="1">
+        <v>46357</v>
       </c>
       <c r="N44" t="s">
         <v>596</v>
@@ -12223,8 +12197,8 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="2">
-        <v>46356</v>
+      <c r="M45" s="1">
+        <v>46357</v>
       </c>
       <c r="N45" t="s">
         <v>596</v>
@@ -12267,8 +12241,8 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="2">
-        <v>46291</v>
+      <c r="M46" s="1">
+        <v>46292</v>
       </c>
       <c r="N46" t="s">
         <v>596</v>
@@ -12311,8 +12285,8 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="2">
-        <v>46291</v>
+      <c r="M47" s="1">
+        <v>46292</v>
       </c>
       <c r="N47" t="s">
         <v>596</v>
@@ -12355,8 +12329,8 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="2">
-        <v>46356</v>
+      <c r="M48" s="1">
+        <v>46357</v>
       </c>
       <c r="N48" t="s">
         <v>596</v>
@@ -12399,8 +12373,8 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="2">
-        <v>46311</v>
+      <c r="M49" s="1">
+        <v>46312</v>
       </c>
       <c r="N49" t="s">
         <v>596</v>
@@ -12443,8 +12417,8 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="2">
-        <v>46311</v>
+      <c r="M50" s="1">
+        <v>46312</v>
       </c>
       <c r="N50" t="s">
         <v>596</v>
@@ -12487,8 +12461,8 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="2">
-        <v>46356</v>
+      <c r="M51" s="1">
+        <v>46357</v>
       </c>
       <c r="N51" t="s">
         <v>596</v>
@@ -12531,8 +12505,8 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="2">
-        <v>46356</v>
+      <c r="M52" s="1">
+        <v>46357</v>
       </c>
       <c r="N52" t="s">
         <v>596</v>
@@ -12575,8 +12549,8 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="2">
-        <v>46356</v>
+      <c r="M53" s="1">
+        <v>46357</v>
       </c>
       <c r="N53" t="s">
         <v>596</v>
@@ -12619,8 +12593,8 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="2">
-        <v>46356</v>
+      <c r="M54" s="1">
+        <v>46357</v>
       </c>
       <c r="N54" t="s">
         <v>596</v>
@@ -12663,8 +12637,8 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="2">
-        <v>46356</v>
+      <c r="M55" s="1">
+        <v>46357</v>
       </c>
       <c r="N55" t="s">
         <v>596</v>
@@ -12707,8 +12681,8 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="2">
-        <v>46311</v>
+      <c r="M56" s="1">
+        <v>46312</v>
       </c>
       <c r="N56" t="s">
         <v>596</v>
@@ -12751,8 +12725,8 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="2">
-        <v>46311</v>
+      <c r="M57" s="1">
+        <v>46312</v>
       </c>
       <c r="N57" t="s">
         <v>596</v>
@@ -12795,8 +12769,8 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="2">
-        <v>46311</v>
+      <c r="M58" s="1">
+        <v>46312</v>
       </c>
       <c r="N58" t="s">
         <v>596</v>
@@ -12839,8 +12813,8 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="2">
-        <v>46356</v>
+      <c r="M59" s="1">
+        <v>46357</v>
       </c>
       <c r="N59" t="s">
         <v>596</v>
@@ -12883,8 +12857,8 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="2">
-        <v>46311</v>
+      <c r="M60" s="1">
+        <v>46312</v>
       </c>
       <c r="N60" t="s">
         <v>596</v>
@@ -12927,8 +12901,8 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="2">
-        <v>46311</v>
+      <c r="M61" s="1">
+        <v>46312</v>
       </c>
       <c r="N61" t="s">
         <v>596</v>
@@ -12971,8 +12945,8 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="2">
-        <v>46356</v>
+      <c r="M62" s="1">
+        <v>46357</v>
       </c>
       <c r="N62" t="s">
         <v>596</v>
@@ -13015,8 +12989,8 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="2">
-        <v>46356</v>
+      <c r="M63" s="1">
+        <v>46357</v>
       </c>
       <c r="N63" t="s">
         <v>596</v>
@@ -13059,8 +13033,8 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="2">
-        <v>46356</v>
+      <c r="M64" s="1">
+        <v>46357</v>
       </c>
       <c r="N64" t="s">
         <v>596</v>
@@ -13103,8 +13077,8 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="2">
-        <v>46356</v>
+      <c r="M65" s="1">
+        <v>46357</v>
       </c>
       <c r="N65" t="s">
         <v>596</v>
@@ -13147,8 +13121,8 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="2">
-        <v>46356</v>
+      <c r="M66" s="1">
+        <v>46357</v>
       </c>
       <c r="N66" t="s">
         <v>596</v>
@@ -13191,8 +13165,8 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="2">
-        <v>46356</v>
+      <c r="M67" s="1">
+        <v>46357</v>
       </c>
       <c r="N67" t="s">
         <v>596</v>
@@ -13235,8 +13209,8 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="2">
-        <v>46356</v>
+      <c r="M68" s="1">
+        <v>46357</v>
       </c>
       <c r="N68" t="s">
         <v>596</v>
@@ -13279,8 +13253,8 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="2">
-        <v>46356</v>
+      <c r="M69" s="1">
+        <v>46357</v>
       </c>
       <c r="N69" t="s">
         <v>596</v>
@@ -13364,8 +13338,8 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="2">
-        <v>46371</v>
+      <c r="M71" s="1">
+        <v>46372</v>
       </c>
       <c r="N71" t="s">
         <v>596</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (17/09/2026 12:59)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,8 +1815,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1832,7 +1840,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1840,12 +1848,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2145,55 +2171,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2237,7 +2263,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2281,7 +2307,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2325,7 +2351,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2451,7 +2477,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2495,7 +2521,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2539,7 +2565,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2586,7 +2612,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2709,7 +2735,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2753,7 +2779,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2797,7 +2823,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2888,7 +2914,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2932,7 +2958,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3058,7 +3084,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3102,7 +3128,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3187,7 +3213,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3234,7 +3260,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3281,7 +3307,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3325,7 +3351,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3369,7 +3395,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3454,7 +3480,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3539,7 +3565,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3586,7 +3612,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3630,7 +3656,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3674,7 +3700,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3759,7 +3785,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3803,7 +3829,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3847,7 +3873,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3932,7 +3958,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3976,7 +4002,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4020,7 +4046,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4064,7 +4090,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4231,7 +4257,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4275,7 +4301,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4319,7 +4345,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4363,7 +4389,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4410,7 +4436,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4454,7 +4480,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4536,7 +4562,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4580,7 +4606,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4668,7 +4694,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4712,7 +4738,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4759,7 +4785,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4803,7 +4829,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4847,7 +4873,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4891,7 +4917,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4935,7 +4961,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4982,7 +5008,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5026,7 +5052,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5073,7 +5099,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5117,7 +5143,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5164,7 +5190,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5252,7 +5278,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5296,7 +5322,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5340,7 +5366,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5384,7 +5410,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5428,7 +5454,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5472,7 +5498,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5557,7 +5583,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5601,7 +5627,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5645,7 +5671,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5689,7 +5715,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5733,7 +5759,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5777,7 +5803,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5821,7 +5847,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5865,7 +5891,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5912,7 +5938,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5956,7 +5982,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6000,7 +6026,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6044,7 +6070,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6088,7 +6114,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6132,7 +6158,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6176,7 +6202,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6220,7 +6246,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6264,7 +6290,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6352,7 +6378,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6396,7 +6422,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6566,7 +6592,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6610,7 +6636,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6654,7 +6680,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6736,7 +6762,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6780,7 +6806,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6827,7 +6853,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6871,7 +6897,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6997,7 +7023,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7041,7 +7067,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7126,7 +7152,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7170,7 +7196,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7214,7 +7240,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7258,7 +7284,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7302,7 +7328,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7346,7 +7372,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7390,7 +7416,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7434,7 +7460,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7519,7 +7545,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7686,7 +7712,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7730,7 +7756,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7774,7 +7800,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7818,7 +7844,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7862,7 +7888,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7906,7 +7932,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7950,7 +7976,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8035,7 +8061,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8079,7 +8105,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8164,7 +8190,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8290,7 +8316,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8334,7 +8360,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8419,7 +8445,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8463,7 +8489,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8507,7 +8533,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8551,7 +8577,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8595,7 +8621,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8639,7 +8665,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8683,7 +8709,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8727,7 +8753,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8812,7 +8838,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8979,7 +9005,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9023,7 +9049,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9067,7 +9093,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9111,7 +9137,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9196,7 +9222,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9240,7 +9266,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9284,7 +9310,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9328,7 +9354,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9372,7 +9398,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9416,7 +9442,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9460,7 +9486,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9504,7 +9530,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9548,7 +9574,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9592,7 +9618,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9636,7 +9662,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9680,7 +9706,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9724,7 +9750,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9768,7 +9794,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9812,7 +9838,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9856,7 +9882,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9900,7 +9926,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9944,7 +9970,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9988,7 +10014,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10032,7 +10058,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10076,7 +10102,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10161,7 +10187,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10246,7 +10272,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10261,55 +10287,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10596,7 +10622,7 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="2">
         <v>46292</v>
       </c>
       <c r="N8" t="s">
@@ -10681,7 +10707,7 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46357</v>
       </c>
       <c r="N10" t="s">
@@ -10725,7 +10751,7 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46357</v>
       </c>
       <c r="N11" t="s">
@@ -10892,7 +10918,7 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="2">
         <v>46292</v>
       </c>
       <c r="N15" t="s">
@@ -10936,7 +10962,7 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46357</v>
       </c>
       <c r="N16" t="s">
@@ -10980,7 +11006,7 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M17" s="2">
         <v>46292</v>
       </c>
       <c r="N17" t="s">
@@ -11024,7 +11050,7 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>46357</v>
       </c>
       <c r="N18" t="s">
@@ -11068,7 +11094,7 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46357</v>
       </c>
       <c r="N19" t="s">
@@ -11112,7 +11138,7 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46357</v>
       </c>
       <c r="N20" t="s">
@@ -11156,7 +11182,7 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46357</v>
       </c>
       <c r="N21" t="s">
@@ -11323,7 +11349,7 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46357</v>
       </c>
       <c r="N25" t="s">
@@ -11408,7 +11434,7 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="1">
+      <c r="M27" s="2">
         <v>46292</v>
       </c>
       <c r="N27" t="s">
@@ -11452,7 +11478,7 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46357</v>
       </c>
       <c r="N28" t="s">
@@ -11496,7 +11522,7 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="2">
         <v>46312</v>
       </c>
       <c r="N29" t="s">
@@ -11540,7 +11566,7 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46357</v>
       </c>
       <c r="N30" t="s">
@@ -11584,7 +11610,7 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="2">
         <v>46312</v>
       </c>
       <c r="N31" t="s">
@@ -11628,7 +11654,7 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="1">
+      <c r="M32" s="2">
         <v>46292</v>
       </c>
       <c r="N32" t="s">
@@ -11672,7 +11698,7 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="1">
+      <c r="M33" s="2">
         <v>46292</v>
       </c>
       <c r="N33" t="s">
@@ -11716,7 +11742,7 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="1">
+      <c r="M34" s="2">
         <v>46292</v>
       </c>
       <c r="N34" t="s">
@@ -11760,7 +11786,7 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="1">
+      <c r="M35" s="2">
         <v>46292</v>
       </c>
       <c r="N35" t="s">
@@ -11804,7 +11830,7 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="1">
+      <c r="M36" s="2">
         <v>46292</v>
       </c>
       <c r="N36" t="s">
@@ -11848,7 +11874,7 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="1">
+      <c r="M37" s="2">
         <v>46292</v>
       </c>
       <c r="N37" t="s">
@@ -11892,7 +11918,7 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="1">
+      <c r="M38" s="2">
         <v>46292</v>
       </c>
       <c r="N38" t="s">
@@ -11977,7 +12003,7 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="1">
+      <c r="M40" s="2">
         <v>46292</v>
       </c>
       <c r="N40" t="s">
@@ -12021,7 +12047,7 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46357</v>
       </c>
       <c r="N41" t="s">
@@ -12065,7 +12091,7 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="1">
+      <c r="M42" s="2">
         <v>46292</v>
       </c>
       <c r="N42" t="s">
@@ -12109,7 +12135,7 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46357</v>
       </c>
       <c r="N43" t="s">
@@ -12153,7 +12179,7 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46357</v>
       </c>
       <c r="N44" t="s">
@@ -12197,7 +12223,7 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46357</v>
       </c>
       <c r="N45" t="s">
@@ -12241,7 +12267,7 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="1">
+      <c r="M46" s="2">
         <v>46292</v>
       </c>
       <c r="N46" t="s">
@@ -12285,7 +12311,7 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="1">
+      <c r="M47" s="2">
         <v>46292</v>
       </c>
       <c r="N47" t="s">
@@ -12329,7 +12355,7 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46357</v>
       </c>
       <c r="N48" t="s">
@@ -12373,7 +12399,7 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46312</v>
       </c>
       <c r="N49" t="s">
@@ -12417,7 +12443,7 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46312</v>
       </c>
       <c r="N50" t="s">
@@ -12461,7 +12487,7 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46357</v>
       </c>
       <c r="N51" t="s">
@@ -12505,7 +12531,7 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46357</v>
       </c>
       <c r="N52" t="s">
@@ -12549,7 +12575,7 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46357</v>
       </c>
       <c r="N53" t="s">
@@ -12593,7 +12619,7 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46357</v>
       </c>
       <c r="N54" t="s">
@@ -12637,7 +12663,7 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46357</v>
       </c>
       <c r="N55" t="s">
@@ -12681,7 +12707,7 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="1">
+      <c r="M56" s="2">
         <v>46312</v>
       </c>
       <c r="N56" t="s">
@@ -12725,7 +12751,7 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="1">
+      <c r="M57" s="2">
         <v>46312</v>
       </c>
       <c r="N57" t="s">
@@ -12769,7 +12795,7 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="1">
+      <c r="M58" s="2">
         <v>46312</v>
       </c>
       <c r="N58" t="s">
@@ -12813,7 +12839,7 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46357</v>
       </c>
       <c r="N59" t="s">
@@ -12857,7 +12883,7 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="1">
+      <c r="M60" s="2">
         <v>46312</v>
       </c>
       <c r="N60" t="s">
@@ -12901,7 +12927,7 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="1">
+      <c r="M61" s="2">
         <v>46312</v>
       </c>
       <c r="N61" t="s">
@@ -12945,7 +12971,7 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46357</v>
       </c>
       <c r="N62" t="s">
@@ -12989,7 +13015,7 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46357</v>
       </c>
       <c r="N63" t="s">
@@ -13033,7 +13059,7 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46357</v>
       </c>
       <c r="N64" t="s">
@@ -13077,7 +13103,7 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="1">
+      <c r="M65" s="2">
         <v>46357</v>
       </c>
       <c r="N65" t="s">
@@ -13121,7 +13147,7 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="1">
+      <c r="M66" s="2">
         <v>46357</v>
       </c>
       <c r="N66" t="s">
@@ -13165,7 +13191,7 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="1">
+      <c r="M67" s="2">
         <v>46357</v>
       </c>
       <c r="N67" t="s">
@@ -13209,7 +13235,7 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="1">
+      <c r="M68" s="2">
         <v>46357</v>
       </c>
       <c r="N68" t="s">
@@ -13253,7 +13279,7 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="1">
+      <c r="M69" s="2">
         <v>46357</v>
       </c>
       <c r="N69" t="s">
@@ -13338,7 +13364,7 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="1">
+      <c r="M71" s="2">
         <v>46372</v>
       </c>
       <c r="N71" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (18/09/2026 11:56)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,16 +1815,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1840,7 +1832,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1848,30 +1840,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2171,55 +2145,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2263,7 +2237,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2307,7 +2281,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2351,7 +2325,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2477,7 +2451,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2521,7 +2495,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2565,7 +2539,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2612,7 +2586,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2735,7 +2709,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2779,7 +2753,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2823,7 +2797,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2914,7 +2888,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2958,7 +2932,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3084,7 +3058,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3128,7 +3102,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3213,7 +3187,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3260,7 +3234,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3307,7 +3281,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3351,7 +3325,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3395,7 +3369,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3480,7 +3454,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3565,7 +3539,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3612,7 +3586,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3656,7 +3630,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3700,7 +3674,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3785,7 +3759,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3829,7 +3803,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3873,7 +3847,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3958,7 +3932,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4002,7 +3976,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4046,7 +4020,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4090,7 +4064,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4257,7 +4231,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4301,7 +4275,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4345,7 +4319,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4389,7 +4363,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4436,7 +4410,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4480,7 +4454,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4562,7 +4536,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4606,7 +4580,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4694,7 +4668,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4738,7 +4712,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4785,7 +4759,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4829,7 +4803,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4873,7 +4847,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4917,7 +4891,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4961,7 +4935,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5008,7 +4982,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5052,7 +5026,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5099,7 +5073,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5143,7 +5117,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5190,7 +5164,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5278,7 +5252,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5322,7 +5296,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5366,7 +5340,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5410,7 +5384,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5454,7 +5428,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5498,7 +5472,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5583,7 +5557,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5627,7 +5601,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5671,7 +5645,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5715,7 +5689,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5759,7 +5733,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5803,7 +5777,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5847,7 +5821,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5891,7 +5865,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5938,7 +5912,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5982,7 +5956,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6026,7 +6000,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6070,7 +6044,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6114,7 +6088,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6158,7 +6132,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6202,7 +6176,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6246,7 +6220,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6290,7 +6264,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6378,7 +6352,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6422,7 +6396,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6592,7 +6566,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6636,7 +6610,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6680,7 +6654,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6762,7 +6736,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6806,7 +6780,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6853,7 +6827,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6897,7 +6871,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7023,7 +6997,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7067,7 +7041,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7152,7 +7126,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7196,7 +7170,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7240,7 +7214,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7284,7 +7258,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7328,7 +7302,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7372,7 +7346,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7416,7 +7390,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7460,7 +7434,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7545,7 +7519,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7712,7 +7686,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7756,7 +7730,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7800,7 +7774,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7844,7 +7818,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7888,7 +7862,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7932,7 +7906,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7976,7 +7950,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8061,7 +8035,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8105,7 +8079,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8190,7 +8164,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8316,7 +8290,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8360,7 +8334,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8445,7 +8419,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8489,7 +8463,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8533,7 +8507,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8577,7 +8551,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8621,7 +8595,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8665,7 +8639,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8709,7 +8683,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8753,7 +8727,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8838,7 +8812,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9005,7 +8979,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9049,7 +9023,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9093,7 +9067,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9137,7 +9111,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9222,7 +9196,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9266,7 +9240,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9310,7 +9284,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9354,7 +9328,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9398,7 +9372,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9442,7 +9416,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9486,7 +9460,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9530,7 +9504,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9574,7 +9548,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9618,7 +9592,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9662,7 +9636,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9706,7 +9680,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9750,7 +9724,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9794,7 +9768,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9838,7 +9812,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9882,7 +9856,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9926,7 +9900,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9970,7 +9944,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10014,7 +9988,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10058,7 +10032,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10102,7 +10076,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10187,7 +10161,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10272,7 +10246,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10287,55 +10261,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10622,8 +10596,8 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="2">
-        <v>46292</v>
+      <c r="M8" s="1">
+        <v>46293</v>
       </c>
       <c r="N8" t="s">
         <v>596</v>
@@ -10707,8 +10681,8 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="2">
-        <v>46357</v>
+      <c r="M10" s="1">
+        <v>46358</v>
       </c>
       <c r="N10" t="s">
         <v>596</v>
@@ -10751,8 +10725,8 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="2">
-        <v>46357</v>
+      <c r="M11" s="1">
+        <v>46358</v>
       </c>
       <c r="N11" t="s">
         <v>596</v>
@@ -10918,8 +10892,8 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="2">
-        <v>46292</v>
+      <c r="M15" s="1">
+        <v>46293</v>
       </c>
       <c r="N15" t="s">
         <v>596</v>
@@ -10962,8 +10936,8 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="2">
-        <v>46357</v>
+      <c r="M16" s="1">
+        <v>46358</v>
       </c>
       <c r="N16" t="s">
         <v>596</v>
@@ -11006,8 +10980,8 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="2">
-        <v>46292</v>
+      <c r="M17" s="1">
+        <v>46293</v>
       </c>
       <c r="N17" t="s">
         <v>596</v>
@@ -11050,8 +11024,8 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="2">
-        <v>46357</v>
+      <c r="M18" s="1">
+        <v>46358</v>
       </c>
       <c r="N18" t="s">
         <v>596</v>
@@ -11094,8 +11068,8 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="2">
-        <v>46357</v>
+      <c r="M19" s="1">
+        <v>46358</v>
       </c>
       <c r="N19" t="s">
         <v>596</v>
@@ -11138,8 +11112,8 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="2">
-        <v>46357</v>
+      <c r="M20" s="1">
+        <v>46358</v>
       </c>
       <c r="N20" t="s">
         <v>596</v>
@@ -11182,8 +11156,8 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="2">
-        <v>46357</v>
+      <c r="M21" s="1">
+        <v>46358</v>
       </c>
       <c r="N21" t="s">
         <v>596</v>
@@ -11349,8 +11323,8 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="2">
-        <v>46357</v>
+      <c r="M25" s="1">
+        <v>46358</v>
       </c>
       <c r="N25" t="s">
         <v>596</v>
@@ -11434,8 +11408,8 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="2">
-        <v>46292</v>
+      <c r="M27" s="1">
+        <v>46293</v>
       </c>
       <c r="N27" t="s">
         <v>596</v>
@@ -11478,8 +11452,8 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="2">
-        <v>46357</v>
+      <c r="M28" s="1">
+        <v>46358</v>
       </c>
       <c r="N28" t="s">
         <v>596</v>
@@ -11522,8 +11496,8 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="2">
-        <v>46312</v>
+      <c r="M29" s="1">
+        <v>46313</v>
       </c>
       <c r="N29" t="s">
         <v>596</v>
@@ -11566,8 +11540,8 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="2">
-        <v>46357</v>
+      <c r="M30" s="1">
+        <v>46358</v>
       </c>
       <c r="N30" t="s">
         <v>596</v>
@@ -11610,8 +11584,8 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="2">
-        <v>46312</v>
+      <c r="M31" s="1">
+        <v>46313</v>
       </c>
       <c r="N31" t="s">
         <v>596</v>
@@ -11654,8 +11628,8 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="2">
-        <v>46292</v>
+      <c r="M32" s="1">
+        <v>46293</v>
       </c>
       <c r="N32" t="s">
         <v>596</v>
@@ -11698,8 +11672,8 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="2">
-        <v>46292</v>
+      <c r="M33" s="1">
+        <v>46293</v>
       </c>
       <c r="N33" t="s">
         <v>596</v>
@@ -11742,8 +11716,8 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="2">
-        <v>46292</v>
+      <c r="M34" s="1">
+        <v>46293</v>
       </c>
       <c r="N34" t="s">
         <v>596</v>
@@ -11786,8 +11760,8 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="2">
-        <v>46292</v>
+      <c r="M35" s="1">
+        <v>46293</v>
       </c>
       <c r="N35" t="s">
         <v>596</v>
@@ -11830,8 +11804,8 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="2">
-        <v>46292</v>
+      <c r="M36" s="1">
+        <v>46293</v>
       </c>
       <c r="N36" t="s">
         <v>596</v>
@@ -11874,8 +11848,8 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="2">
-        <v>46292</v>
+      <c r="M37" s="1">
+        <v>46293</v>
       </c>
       <c r="N37" t="s">
         <v>596</v>
@@ -11918,8 +11892,8 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="2">
-        <v>46292</v>
+      <c r="M38" s="1">
+        <v>46293</v>
       </c>
       <c r="N38" t="s">
         <v>596</v>
@@ -12003,8 +11977,8 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="2">
-        <v>46292</v>
+      <c r="M40" s="1">
+        <v>46293</v>
       </c>
       <c r="N40" t="s">
         <v>596</v>
@@ -12047,8 +12021,8 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="2">
-        <v>46357</v>
+      <c r="M41" s="1">
+        <v>46358</v>
       </c>
       <c r="N41" t="s">
         <v>596</v>
@@ -12091,8 +12065,8 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="2">
-        <v>46292</v>
+      <c r="M42" s="1">
+        <v>46293</v>
       </c>
       <c r="N42" t="s">
         <v>596</v>
@@ -12135,8 +12109,8 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="2">
-        <v>46357</v>
+      <c r="M43" s="1">
+        <v>46358</v>
       </c>
       <c r="N43" t="s">
         <v>596</v>
@@ -12179,8 +12153,8 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="2">
-        <v>46357</v>
+      <c r="M44" s="1">
+        <v>46358</v>
       </c>
       <c r="N44" t="s">
         <v>596</v>
@@ -12223,8 +12197,8 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="2">
-        <v>46357</v>
+      <c r="M45" s="1">
+        <v>46358</v>
       </c>
       <c r="N45" t="s">
         <v>596</v>
@@ -12267,8 +12241,8 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="2">
-        <v>46292</v>
+      <c r="M46" s="1">
+        <v>46293</v>
       </c>
       <c r="N46" t="s">
         <v>596</v>
@@ -12311,8 +12285,8 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="2">
-        <v>46292</v>
+      <c r="M47" s="1">
+        <v>46293</v>
       </c>
       <c r="N47" t="s">
         <v>596</v>
@@ -12355,8 +12329,8 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="2">
-        <v>46357</v>
+      <c r="M48" s="1">
+        <v>46358</v>
       </c>
       <c r="N48" t="s">
         <v>596</v>
@@ -12399,8 +12373,8 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="2">
-        <v>46312</v>
+      <c r="M49" s="1">
+        <v>46313</v>
       </c>
       <c r="N49" t="s">
         <v>596</v>
@@ -12443,8 +12417,8 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="2">
-        <v>46312</v>
+      <c r="M50" s="1">
+        <v>46313</v>
       </c>
       <c r="N50" t="s">
         <v>596</v>
@@ -12487,8 +12461,8 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="2">
-        <v>46357</v>
+      <c r="M51" s="1">
+        <v>46358</v>
       </c>
       <c r="N51" t="s">
         <v>596</v>
@@ -12531,8 +12505,8 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="2">
-        <v>46357</v>
+      <c r="M52" s="1">
+        <v>46358</v>
       </c>
       <c r="N52" t="s">
         <v>596</v>
@@ -12575,8 +12549,8 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="2">
-        <v>46357</v>
+      <c r="M53" s="1">
+        <v>46358</v>
       </c>
       <c r="N53" t="s">
         <v>596</v>
@@ -12619,8 +12593,8 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="2">
-        <v>46357</v>
+      <c r="M54" s="1">
+        <v>46358</v>
       </c>
       <c r="N54" t="s">
         <v>596</v>
@@ -12663,8 +12637,8 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="2">
-        <v>46357</v>
+      <c r="M55" s="1">
+        <v>46358</v>
       </c>
       <c r="N55" t="s">
         <v>596</v>
@@ -12707,8 +12681,8 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="2">
-        <v>46312</v>
+      <c r="M56" s="1">
+        <v>46313</v>
       </c>
       <c r="N56" t="s">
         <v>596</v>
@@ -12751,8 +12725,8 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="2">
-        <v>46312</v>
+      <c r="M57" s="1">
+        <v>46313</v>
       </c>
       <c r="N57" t="s">
         <v>596</v>
@@ -12795,8 +12769,8 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="2">
-        <v>46312</v>
+      <c r="M58" s="1">
+        <v>46313</v>
       </c>
       <c r="N58" t="s">
         <v>596</v>
@@ -12839,8 +12813,8 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="2">
-        <v>46357</v>
+      <c r="M59" s="1">
+        <v>46358</v>
       </c>
       <c r="N59" t="s">
         <v>596</v>
@@ -12883,8 +12857,8 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="2">
-        <v>46312</v>
+      <c r="M60" s="1">
+        <v>46313</v>
       </c>
       <c r="N60" t="s">
         <v>596</v>
@@ -12927,8 +12901,8 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="2">
-        <v>46312</v>
+      <c r="M61" s="1">
+        <v>46313</v>
       </c>
       <c r="N61" t="s">
         <v>596</v>
@@ -12971,8 +12945,8 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="2">
-        <v>46357</v>
+      <c r="M62" s="1">
+        <v>46358</v>
       </c>
       <c r="N62" t="s">
         <v>596</v>
@@ -13015,8 +12989,8 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="2">
-        <v>46357</v>
+      <c r="M63" s="1">
+        <v>46358</v>
       </c>
       <c r="N63" t="s">
         <v>596</v>
@@ -13059,8 +13033,8 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="2">
-        <v>46357</v>
+      <c r="M64" s="1">
+        <v>46358</v>
       </c>
       <c r="N64" t="s">
         <v>596</v>
@@ -13103,8 +13077,8 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="2">
-        <v>46357</v>
+      <c r="M65" s="1">
+        <v>46358</v>
       </c>
       <c r="N65" t="s">
         <v>596</v>
@@ -13147,8 +13121,8 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="2">
-        <v>46357</v>
+      <c r="M66" s="1">
+        <v>46358</v>
       </c>
       <c r="N66" t="s">
         <v>596</v>
@@ -13191,8 +13165,8 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="2">
-        <v>46357</v>
+      <c r="M67" s="1">
+        <v>46358</v>
       </c>
       <c r="N67" t="s">
         <v>596</v>
@@ -13235,8 +13209,8 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="2">
-        <v>46357</v>
+      <c r="M68" s="1">
+        <v>46358</v>
       </c>
       <c r="N68" t="s">
         <v>596</v>
@@ -13279,8 +13253,8 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="2">
-        <v>46357</v>
+      <c r="M69" s="1">
+        <v>46358</v>
       </c>
       <c r="N69" t="s">
         <v>596</v>
@@ -13364,8 +13338,8 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="2">
-        <v>46372</v>
+      <c r="M71" s="1">
+        <v>46373</v>
       </c>
       <c r="N71" t="s">
         <v>596</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (18/09/2026 16:37)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,8 +1815,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1832,7 +1840,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1840,12 +1848,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2145,55 +2171,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2237,7 +2263,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2281,7 +2307,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2325,7 +2351,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2451,7 +2477,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2495,7 +2521,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2539,7 +2565,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2586,7 +2612,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2709,7 +2735,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2753,7 +2779,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2797,7 +2823,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2888,7 +2914,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2932,7 +2958,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3058,7 +3084,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3102,7 +3128,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3187,7 +3213,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3234,7 +3260,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3281,7 +3307,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3325,7 +3351,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3369,7 +3395,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3454,7 +3480,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3539,7 +3565,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3586,7 +3612,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3630,7 +3656,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3674,7 +3700,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3759,7 +3785,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3803,7 +3829,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3847,7 +3873,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3932,7 +3958,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3976,7 +4002,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4020,7 +4046,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4064,7 +4090,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4231,7 +4257,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4275,7 +4301,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4319,7 +4345,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4363,7 +4389,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4410,7 +4436,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4454,7 +4480,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4536,7 +4562,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4580,7 +4606,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4668,7 +4694,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4712,7 +4738,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4759,7 +4785,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4803,7 +4829,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4847,7 +4873,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4891,7 +4917,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4935,7 +4961,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4982,7 +5008,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5026,7 +5052,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5073,7 +5099,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5117,7 +5143,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5164,7 +5190,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5252,7 +5278,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5296,7 +5322,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5340,7 +5366,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5384,7 +5410,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5428,7 +5454,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5472,7 +5498,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5557,7 +5583,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5601,7 +5627,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5645,7 +5671,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5689,7 +5715,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5733,7 +5759,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5777,7 +5803,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5821,7 +5847,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5865,7 +5891,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5912,7 +5938,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5956,7 +5982,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6000,7 +6026,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6044,7 +6070,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6088,7 +6114,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6132,7 +6158,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6176,7 +6202,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6220,7 +6246,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6264,7 +6290,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6352,7 +6378,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6396,7 +6422,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6566,7 +6592,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6610,7 +6636,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6654,7 +6680,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6736,7 +6762,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6780,7 +6806,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6827,7 +6853,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6871,7 +6897,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6997,7 +7023,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7041,7 +7067,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7126,7 +7152,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7170,7 +7196,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7214,7 +7240,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7258,7 +7284,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7302,7 +7328,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7346,7 +7372,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7390,7 +7416,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7434,7 +7460,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7519,7 +7545,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7686,7 +7712,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7730,7 +7756,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7774,7 +7800,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7818,7 +7844,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7862,7 +7888,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7906,7 +7932,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7950,7 +7976,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8035,7 +8061,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8079,7 +8105,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8164,7 +8190,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8290,7 +8316,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8334,7 +8360,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8419,7 +8445,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8463,7 +8489,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8507,7 +8533,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8551,7 +8577,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8595,7 +8621,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8639,7 +8665,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8683,7 +8709,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8727,7 +8753,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8812,7 +8838,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8979,7 +9005,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9023,7 +9049,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9067,7 +9093,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9111,7 +9137,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9196,7 +9222,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9240,7 +9266,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9284,7 +9310,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9328,7 +9354,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9372,7 +9398,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9416,7 +9442,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9460,7 +9486,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9504,7 +9530,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9548,7 +9574,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9592,7 +9618,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9636,7 +9662,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9680,7 +9706,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9724,7 +9750,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9768,7 +9794,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9812,7 +9838,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9856,7 +9882,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9900,7 +9926,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9944,7 +9970,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9988,7 +10014,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10032,7 +10058,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10076,7 +10102,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10161,7 +10187,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10246,7 +10272,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10261,55 +10287,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10596,7 +10622,7 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="2">
         <v>46293</v>
       </c>
       <c r="N8" t="s">
@@ -10681,7 +10707,7 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46358</v>
       </c>
       <c r="N10" t="s">
@@ -10725,7 +10751,7 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46358</v>
       </c>
       <c r="N11" t="s">
@@ -10892,7 +10918,7 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="2">
         <v>46293</v>
       </c>
       <c r="N15" t="s">
@@ -10936,7 +10962,7 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46358</v>
       </c>
       <c r="N16" t="s">
@@ -10980,7 +11006,7 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M17" s="2">
         <v>46293</v>
       </c>
       <c r="N17" t="s">
@@ -11024,7 +11050,7 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>46358</v>
       </c>
       <c r="N18" t="s">
@@ -11068,7 +11094,7 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46358</v>
       </c>
       <c r="N19" t="s">
@@ -11112,7 +11138,7 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46358</v>
       </c>
       <c r="N20" t="s">
@@ -11156,7 +11182,7 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46358</v>
       </c>
       <c r="N21" t="s">
@@ -11323,7 +11349,7 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46358</v>
       </c>
       <c r="N25" t="s">
@@ -11408,7 +11434,7 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="1">
+      <c r="M27" s="2">
         <v>46293</v>
       </c>
       <c r="N27" t="s">
@@ -11452,7 +11478,7 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46358</v>
       </c>
       <c r="N28" t="s">
@@ -11496,7 +11522,7 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="2">
         <v>46313</v>
       </c>
       <c r="N29" t="s">
@@ -11540,7 +11566,7 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46358</v>
       </c>
       <c r="N30" t="s">
@@ -11584,7 +11610,7 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="2">
         <v>46313</v>
       </c>
       <c r="N31" t="s">
@@ -11628,7 +11654,7 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="1">
+      <c r="M32" s="2">
         <v>46293</v>
       </c>
       <c r="N32" t="s">
@@ -11672,7 +11698,7 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="1">
+      <c r="M33" s="2">
         <v>46293</v>
       </c>
       <c r="N33" t="s">
@@ -11716,7 +11742,7 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="1">
+      <c r="M34" s="2">
         <v>46293</v>
       </c>
       <c r="N34" t="s">
@@ -11760,7 +11786,7 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="1">
+      <c r="M35" s="2">
         <v>46293</v>
       </c>
       <c r="N35" t="s">
@@ -11804,7 +11830,7 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="1">
+      <c r="M36" s="2">
         <v>46293</v>
       </c>
       <c r="N36" t="s">
@@ -11848,7 +11874,7 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="1">
+      <c r="M37" s="2">
         <v>46293</v>
       </c>
       <c r="N37" t="s">
@@ -11892,7 +11918,7 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="1">
+      <c r="M38" s="2">
         <v>46293</v>
       </c>
       <c r="N38" t="s">
@@ -11977,7 +12003,7 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="1">
+      <c r="M40" s="2">
         <v>46293</v>
       </c>
       <c r="N40" t="s">
@@ -12021,7 +12047,7 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46358</v>
       </c>
       <c r="N41" t="s">
@@ -12065,7 +12091,7 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="1">
+      <c r="M42" s="2">
         <v>46293</v>
       </c>
       <c r="N42" t="s">
@@ -12109,7 +12135,7 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46358</v>
       </c>
       <c r="N43" t="s">
@@ -12153,7 +12179,7 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46358</v>
       </c>
       <c r="N44" t="s">
@@ -12197,7 +12223,7 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46358</v>
       </c>
       <c r="N45" t="s">
@@ -12241,7 +12267,7 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="1">
+      <c r="M46" s="2">
         <v>46293</v>
       </c>
       <c r="N46" t="s">
@@ -12285,7 +12311,7 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="1">
+      <c r="M47" s="2">
         <v>46293</v>
       </c>
       <c r="N47" t="s">
@@ -12329,7 +12355,7 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46358</v>
       </c>
       <c r="N48" t="s">
@@ -12373,7 +12399,7 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46313</v>
       </c>
       <c r="N49" t="s">
@@ -12417,7 +12443,7 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46313</v>
       </c>
       <c r="N50" t="s">
@@ -12461,7 +12487,7 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46358</v>
       </c>
       <c r="N51" t="s">
@@ -12505,7 +12531,7 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46358</v>
       </c>
       <c r="N52" t="s">
@@ -12549,7 +12575,7 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46358</v>
       </c>
       <c r="N53" t="s">
@@ -12593,7 +12619,7 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46358</v>
       </c>
       <c r="N54" t="s">
@@ -12637,7 +12663,7 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46358</v>
       </c>
       <c r="N55" t="s">
@@ -12681,7 +12707,7 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="1">
+      <c r="M56" s="2">
         <v>46313</v>
       </c>
       <c r="N56" t="s">
@@ -12725,7 +12751,7 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="1">
+      <c r="M57" s="2">
         <v>46313</v>
       </c>
       <c r="N57" t="s">
@@ -12769,7 +12795,7 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="1">
+      <c r="M58" s="2">
         <v>46313</v>
       </c>
       <c r="N58" t="s">
@@ -12813,7 +12839,7 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46358</v>
       </c>
       <c r="N59" t="s">
@@ -12857,7 +12883,7 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="1">
+      <c r="M60" s="2">
         <v>46313</v>
       </c>
       <c r="N60" t="s">
@@ -12901,7 +12927,7 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="1">
+      <c r="M61" s="2">
         <v>46313</v>
       </c>
       <c r="N61" t="s">
@@ -12945,7 +12971,7 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46358</v>
       </c>
       <c r="N62" t="s">
@@ -12989,7 +13015,7 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46358</v>
       </c>
       <c r="N63" t="s">
@@ -13033,7 +13059,7 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46358</v>
       </c>
       <c r="N64" t="s">
@@ -13077,7 +13103,7 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="1">
+      <c r="M65" s="2">
         <v>46358</v>
       </c>
       <c r="N65" t="s">
@@ -13121,7 +13147,7 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="1">
+      <c r="M66" s="2">
         <v>46358</v>
       </c>
       <c r="N66" t="s">
@@ -13165,7 +13191,7 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="1">
+      <c r="M67" s="2">
         <v>46358</v>
       </c>
       <c r="N67" t="s">
@@ -13209,7 +13235,7 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="1">
+      <c r="M68" s="2">
         <v>46358</v>
       </c>
       <c r="N68" t="s">
@@ -13253,7 +13279,7 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="1">
+      <c r="M69" s="2">
         <v>46358</v>
       </c>
       <c r="N69" t="s">
@@ -13338,7 +13364,7 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="1">
+      <c r="M71" s="2">
         <v>46373</v>
       </c>
       <c r="N71" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (21/09/2026 14:00)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,16 +1815,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1840,7 +1832,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1848,30 +1840,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2171,55 +2145,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2263,7 +2237,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2307,7 +2281,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2351,7 +2325,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2477,7 +2451,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2521,7 +2495,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2565,7 +2539,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2612,7 +2586,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2735,7 +2709,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2779,7 +2753,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2823,7 +2797,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2914,7 +2888,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2958,7 +2932,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3084,7 +3058,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3128,7 +3102,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3213,7 +3187,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3260,7 +3234,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3307,7 +3281,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3351,7 +3325,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3395,7 +3369,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3480,7 +3454,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3565,7 +3539,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3612,7 +3586,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3656,7 +3630,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3700,7 +3674,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3785,7 +3759,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3829,7 +3803,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3873,7 +3847,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3958,7 +3932,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4002,7 +3976,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4046,7 +4020,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4090,7 +4064,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4257,7 +4231,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4301,7 +4275,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4345,7 +4319,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4389,7 +4363,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4436,7 +4410,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4480,7 +4454,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4562,7 +4536,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4606,7 +4580,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4694,7 +4668,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4738,7 +4712,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4785,7 +4759,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4829,7 +4803,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4873,7 +4847,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4917,7 +4891,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4961,7 +4935,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5008,7 +4982,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5052,7 +5026,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5099,7 +5073,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5143,7 +5117,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5190,7 +5164,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5278,7 +5252,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5322,7 +5296,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5366,7 +5340,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5410,7 +5384,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5454,7 +5428,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5498,7 +5472,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5583,7 +5557,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5627,7 +5601,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5671,7 +5645,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5715,7 +5689,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5759,7 +5733,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5803,7 +5777,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5847,7 +5821,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5891,7 +5865,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5938,7 +5912,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5982,7 +5956,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6026,7 +6000,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6070,7 +6044,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6114,7 +6088,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6158,7 +6132,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6202,7 +6176,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6246,7 +6220,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6290,7 +6264,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6378,7 +6352,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6422,7 +6396,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6592,7 +6566,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6636,7 +6610,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6680,7 +6654,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6762,7 +6736,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6806,7 +6780,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6853,7 +6827,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6897,7 +6871,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7023,7 +6997,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7067,7 +7041,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7152,7 +7126,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7196,7 +7170,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7240,7 +7214,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7284,7 +7258,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7328,7 +7302,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7372,7 +7346,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7416,7 +7390,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7460,7 +7434,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7545,7 +7519,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7712,7 +7686,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7756,7 +7730,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7800,7 +7774,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7844,7 +7818,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7888,7 +7862,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7932,7 +7906,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7976,7 +7950,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8061,7 +8035,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8105,7 +8079,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8190,7 +8164,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8316,7 +8290,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8360,7 +8334,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8445,7 +8419,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8489,7 +8463,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8533,7 +8507,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8577,7 +8551,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8621,7 +8595,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8665,7 +8639,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8709,7 +8683,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8753,7 +8727,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8838,7 +8812,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9005,7 +8979,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9049,7 +9023,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9093,7 +9067,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9137,7 +9111,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9222,7 +9196,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9266,7 +9240,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9310,7 +9284,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9354,7 +9328,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9398,7 +9372,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9442,7 +9416,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9486,7 +9460,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9530,7 +9504,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9574,7 +9548,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9618,7 +9592,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9662,7 +9636,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9706,7 +9680,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9750,7 +9724,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9794,7 +9768,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9838,7 +9812,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9882,7 +9856,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9926,7 +9900,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9970,7 +9944,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10014,7 +9988,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10058,7 +10032,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10102,7 +10076,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10187,7 +10161,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10272,7 +10246,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10287,55 +10261,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10622,8 +10596,8 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="2">
-        <v>46293</v>
+      <c r="M8" s="1">
+        <v>46296</v>
       </c>
       <c r="N8" t="s">
         <v>596</v>
@@ -10707,8 +10681,8 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="2">
-        <v>46358</v>
+      <c r="M10" s="1">
+        <v>46361</v>
       </c>
       <c r="N10" t="s">
         <v>596</v>
@@ -10751,8 +10725,8 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="2">
-        <v>46358</v>
+      <c r="M11" s="1">
+        <v>46361</v>
       </c>
       <c r="N11" t="s">
         <v>596</v>
@@ -10918,8 +10892,8 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="2">
-        <v>46293</v>
+      <c r="M15" s="1">
+        <v>46296</v>
       </c>
       <c r="N15" t="s">
         <v>596</v>
@@ -10962,8 +10936,8 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="2">
-        <v>46358</v>
+      <c r="M16" s="1">
+        <v>46361</v>
       </c>
       <c r="N16" t="s">
         <v>596</v>
@@ -11006,8 +10980,8 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="2">
-        <v>46293</v>
+      <c r="M17" s="1">
+        <v>46296</v>
       </c>
       <c r="N17" t="s">
         <v>596</v>
@@ -11050,8 +11024,8 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="2">
-        <v>46358</v>
+      <c r="M18" s="1">
+        <v>46361</v>
       </c>
       <c r="N18" t="s">
         <v>596</v>
@@ -11094,8 +11068,8 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="2">
-        <v>46358</v>
+      <c r="M19" s="1">
+        <v>46361</v>
       </c>
       <c r="N19" t="s">
         <v>596</v>
@@ -11138,8 +11112,8 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="2">
-        <v>46358</v>
+      <c r="M20" s="1">
+        <v>46361</v>
       </c>
       <c r="N20" t="s">
         <v>596</v>
@@ -11182,8 +11156,8 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="2">
-        <v>46358</v>
+      <c r="M21" s="1">
+        <v>46361</v>
       </c>
       <c r="N21" t="s">
         <v>596</v>
@@ -11349,8 +11323,8 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="2">
-        <v>46358</v>
+      <c r="M25" s="1">
+        <v>46361</v>
       </c>
       <c r="N25" t="s">
         <v>596</v>
@@ -11434,8 +11408,8 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="2">
-        <v>46293</v>
+      <c r="M27" s="1">
+        <v>46296</v>
       </c>
       <c r="N27" t="s">
         <v>596</v>
@@ -11478,8 +11452,8 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="2">
-        <v>46358</v>
+      <c r="M28" s="1">
+        <v>46361</v>
       </c>
       <c r="N28" t="s">
         <v>596</v>
@@ -11522,8 +11496,8 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="2">
-        <v>46313</v>
+      <c r="M29" s="1">
+        <v>46316</v>
       </c>
       <c r="N29" t="s">
         <v>596</v>
@@ -11566,8 +11540,8 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="2">
-        <v>46358</v>
+      <c r="M30" s="1">
+        <v>46361</v>
       </c>
       <c r="N30" t="s">
         <v>596</v>
@@ -11610,8 +11584,8 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="2">
-        <v>46313</v>
+      <c r="M31" s="1">
+        <v>46316</v>
       </c>
       <c r="N31" t="s">
         <v>596</v>
@@ -11654,8 +11628,8 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="2">
-        <v>46293</v>
+      <c r="M32" s="1">
+        <v>46296</v>
       </c>
       <c r="N32" t="s">
         <v>596</v>
@@ -11698,8 +11672,8 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="2">
-        <v>46293</v>
+      <c r="M33" s="1">
+        <v>46296</v>
       </c>
       <c r="N33" t="s">
         <v>596</v>
@@ -11742,8 +11716,8 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="2">
-        <v>46293</v>
+      <c r="M34" s="1">
+        <v>46296</v>
       </c>
       <c r="N34" t="s">
         <v>596</v>
@@ -11786,8 +11760,8 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="2">
-        <v>46293</v>
+      <c r="M35" s="1">
+        <v>46296</v>
       </c>
       <c r="N35" t="s">
         <v>596</v>
@@ -11830,8 +11804,8 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="2">
-        <v>46293</v>
+      <c r="M36" s="1">
+        <v>46296</v>
       </c>
       <c r="N36" t="s">
         <v>596</v>
@@ -11874,8 +11848,8 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="2">
-        <v>46293</v>
+      <c r="M37" s="1">
+        <v>46296</v>
       </c>
       <c r="N37" t="s">
         <v>596</v>
@@ -11918,8 +11892,8 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="2">
-        <v>46293</v>
+      <c r="M38" s="1">
+        <v>46296</v>
       </c>
       <c r="N38" t="s">
         <v>596</v>
@@ -12003,8 +11977,8 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="2">
-        <v>46293</v>
+      <c r="M40" s="1">
+        <v>46296</v>
       </c>
       <c r="N40" t="s">
         <v>596</v>
@@ -12047,8 +12021,8 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="2">
-        <v>46358</v>
+      <c r="M41" s="1">
+        <v>46361</v>
       </c>
       <c r="N41" t="s">
         <v>596</v>
@@ -12091,8 +12065,8 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="2">
-        <v>46293</v>
+      <c r="M42" s="1">
+        <v>46296</v>
       </c>
       <c r="N42" t="s">
         <v>596</v>
@@ -12135,8 +12109,8 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="2">
-        <v>46358</v>
+      <c r="M43" s="1">
+        <v>46361</v>
       </c>
       <c r="N43" t="s">
         <v>596</v>
@@ -12179,8 +12153,8 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="2">
-        <v>46358</v>
+      <c r="M44" s="1">
+        <v>46361</v>
       </c>
       <c r="N44" t="s">
         <v>596</v>
@@ -12223,8 +12197,8 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="2">
-        <v>46358</v>
+      <c r="M45" s="1">
+        <v>46361</v>
       </c>
       <c r="N45" t="s">
         <v>596</v>
@@ -12267,8 +12241,8 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="2">
-        <v>46293</v>
+      <c r="M46" s="1">
+        <v>46296</v>
       </c>
       <c r="N46" t="s">
         <v>596</v>
@@ -12311,8 +12285,8 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="2">
-        <v>46293</v>
+      <c r="M47" s="1">
+        <v>46296</v>
       </c>
       <c r="N47" t="s">
         <v>596</v>
@@ -12355,8 +12329,8 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="2">
-        <v>46358</v>
+      <c r="M48" s="1">
+        <v>46361</v>
       </c>
       <c r="N48" t="s">
         <v>596</v>
@@ -12399,8 +12373,8 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="2">
-        <v>46313</v>
+      <c r="M49" s="1">
+        <v>46316</v>
       </c>
       <c r="N49" t="s">
         <v>596</v>
@@ -12443,8 +12417,8 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="2">
-        <v>46313</v>
+      <c r="M50" s="1">
+        <v>46316</v>
       </c>
       <c r="N50" t="s">
         <v>596</v>
@@ -12487,8 +12461,8 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="2">
-        <v>46358</v>
+      <c r="M51" s="1">
+        <v>46361</v>
       </c>
       <c r="N51" t="s">
         <v>596</v>
@@ -12531,8 +12505,8 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="2">
-        <v>46358</v>
+      <c r="M52" s="1">
+        <v>46361</v>
       </c>
       <c r="N52" t="s">
         <v>596</v>
@@ -12575,8 +12549,8 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="2">
-        <v>46358</v>
+      <c r="M53" s="1">
+        <v>46361</v>
       </c>
       <c r="N53" t="s">
         <v>596</v>
@@ -12619,8 +12593,8 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="2">
-        <v>46358</v>
+      <c r="M54" s="1">
+        <v>46361</v>
       </c>
       <c r="N54" t="s">
         <v>596</v>
@@ -12663,8 +12637,8 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="2">
-        <v>46358</v>
+      <c r="M55" s="1">
+        <v>46361</v>
       </c>
       <c r="N55" t="s">
         <v>596</v>
@@ -12707,8 +12681,8 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="2">
-        <v>46313</v>
+      <c r="M56" s="1">
+        <v>46316</v>
       </c>
       <c r="N56" t="s">
         <v>596</v>
@@ -12751,8 +12725,8 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="2">
-        <v>46313</v>
+      <c r="M57" s="1">
+        <v>46316</v>
       </c>
       <c r="N57" t="s">
         <v>596</v>
@@ -12795,8 +12769,8 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="2">
-        <v>46313</v>
+      <c r="M58" s="1">
+        <v>46316</v>
       </c>
       <c r="N58" t="s">
         <v>596</v>
@@ -12839,8 +12813,8 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="2">
-        <v>46358</v>
+      <c r="M59" s="1">
+        <v>46361</v>
       </c>
       <c r="N59" t="s">
         <v>596</v>
@@ -12883,8 +12857,8 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="2">
-        <v>46313</v>
+      <c r="M60" s="1">
+        <v>46316</v>
       </c>
       <c r="N60" t="s">
         <v>596</v>
@@ -12927,8 +12901,8 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="2">
-        <v>46313</v>
+      <c r="M61" s="1">
+        <v>46316</v>
       </c>
       <c r="N61" t="s">
         <v>596</v>
@@ -12971,8 +12945,8 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="2">
-        <v>46358</v>
+      <c r="M62" s="1">
+        <v>46361</v>
       </c>
       <c r="N62" t="s">
         <v>596</v>
@@ -13015,8 +12989,8 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="2">
-        <v>46358</v>
+      <c r="M63" s="1">
+        <v>46361</v>
       </c>
       <c r="N63" t="s">
         <v>596</v>
@@ -13059,8 +13033,8 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="2">
-        <v>46358</v>
+      <c r="M64" s="1">
+        <v>46361</v>
       </c>
       <c r="N64" t="s">
         <v>596</v>
@@ -13103,8 +13077,8 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="2">
-        <v>46358</v>
+      <c r="M65" s="1">
+        <v>46361</v>
       </c>
       <c r="N65" t="s">
         <v>596</v>
@@ -13147,8 +13121,8 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="2">
-        <v>46358</v>
+      <c r="M66" s="1">
+        <v>46361</v>
       </c>
       <c r="N66" t="s">
         <v>596</v>
@@ -13191,8 +13165,8 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="2">
-        <v>46358</v>
+      <c r="M67" s="1">
+        <v>46361</v>
       </c>
       <c r="N67" t="s">
         <v>596</v>
@@ -13235,8 +13209,8 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="2">
-        <v>46358</v>
+      <c r="M68" s="1">
+        <v>46361</v>
       </c>
       <c r="N68" t="s">
         <v>596</v>
@@ -13279,8 +13253,8 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="2">
-        <v>46358</v>
+      <c r="M69" s="1">
+        <v>46361</v>
       </c>
       <c r="N69" t="s">
         <v>596</v>
@@ -13364,8 +13338,8 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="2">
-        <v>46373</v>
+      <c r="M71" s="1">
+        <v>46376</v>
       </c>
       <c r="N71" t="s">
         <v>596</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (21/09/2026 14:31)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,8 +1815,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1832,7 +1840,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1840,12 +1848,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2145,55 +2171,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2237,7 +2263,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2281,7 +2307,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2325,7 +2351,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2451,7 +2477,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2495,7 +2521,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2539,7 +2565,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2586,7 +2612,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2709,7 +2735,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2753,7 +2779,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2797,7 +2823,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2888,7 +2914,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2932,7 +2958,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3058,7 +3084,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3102,7 +3128,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3187,7 +3213,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3234,7 +3260,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3281,7 +3307,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3325,7 +3351,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3369,7 +3395,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3454,7 +3480,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3539,7 +3565,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3586,7 +3612,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3630,7 +3656,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3674,7 +3700,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3759,7 +3785,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3803,7 +3829,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3847,7 +3873,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3932,7 +3958,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3976,7 +4002,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4020,7 +4046,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4064,7 +4090,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4231,7 +4257,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4275,7 +4301,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4319,7 +4345,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4363,7 +4389,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4410,7 +4436,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4454,7 +4480,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4536,7 +4562,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4580,7 +4606,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4668,7 +4694,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4712,7 +4738,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4759,7 +4785,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4803,7 +4829,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4847,7 +4873,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4891,7 +4917,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4935,7 +4961,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4982,7 +5008,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5026,7 +5052,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5073,7 +5099,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5117,7 +5143,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5164,7 +5190,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5252,7 +5278,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5296,7 +5322,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5340,7 +5366,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5384,7 +5410,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5428,7 +5454,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5472,7 +5498,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5557,7 +5583,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5601,7 +5627,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5645,7 +5671,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5689,7 +5715,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5733,7 +5759,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5777,7 +5803,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5821,7 +5847,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5865,7 +5891,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5912,7 +5938,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5956,7 +5982,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6000,7 +6026,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6044,7 +6070,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6088,7 +6114,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6132,7 +6158,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6176,7 +6202,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6220,7 +6246,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6264,7 +6290,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6352,7 +6378,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6396,7 +6422,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6566,7 +6592,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6610,7 +6636,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6654,7 +6680,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6736,7 +6762,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6780,7 +6806,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6827,7 +6853,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6871,7 +6897,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6997,7 +7023,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7041,7 +7067,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7126,7 +7152,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7170,7 +7196,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7214,7 +7240,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7258,7 +7284,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7302,7 +7328,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7346,7 +7372,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7390,7 +7416,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7434,7 +7460,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7519,7 +7545,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7686,7 +7712,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7730,7 +7756,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7774,7 +7800,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7818,7 +7844,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7862,7 +7888,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7906,7 +7932,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7950,7 +7976,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8035,7 +8061,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8079,7 +8105,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8164,7 +8190,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8290,7 +8316,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8334,7 +8360,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8419,7 +8445,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8463,7 +8489,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8507,7 +8533,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8551,7 +8577,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8595,7 +8621,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8639,7 +8665,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8683,7 +8709,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8727,7 +8753,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8812,7 +8838,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8979,7 +9005,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9023,7 +9049,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9067,7 +9093,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9111,7 +9137,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9196,7 +9222,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9240,7 +9266,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9284,7 +9310,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9328,7 +9354,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9372,7 +9398,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9416,7 +9442,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9460,7 +9486,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9504,7 +9530,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9548,7 +9574,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9592,7 +9618,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9636,7 +9662,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9680,7 +9706,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9724,7 +9750,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9768,7 +9794,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9812,7 +9838,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9856,7 +9882,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9900,7 +9926,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9944,7 +9970,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9988,7 +10014,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10032,7 +10058,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10076,7 +10102,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10161,7 +10187,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10246,7 +10272,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10261,55 +10287,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10596,7 +10622,7 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="2">
         <v>46296</v>
       </c>
       <c r="N8" t="s">
@@ -10681,7 +10707,7 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46361</v>
       </c>
       <c r="N10" t="s">
@@ -10725,7 +10751,7 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46361</v>
       </c>
       <c r="N11" t="s">
@@ -10892,7 +10918,7 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="2">
         <v>46296</v>
       </c>
       <c r="N15" t="s">
@@ -10936,7 +10962,7 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46361</v>
       </c>
       <c r="N16" t="s">
@@ -10980,7 +11006,7 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M17" s="2">
         <v>46296</v>
       </c>
       <c r="N17" t="s">
@@ -11024,7 +11050,7 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>46361</v>
       </c>
       <c r="N18" t="s">
@@ -11068,7 +11094,7 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46361</v>
       </c>
       <c r="N19" t="s">
@@ -11112,7 +11138,7 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46361</v>
       </c>
       <c r="N20" t="s">
@@ -11156,7 +11182,7 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46361</v>
       </c>
       <c r="N21" t="s">
@@ -11323,7 +11349,7 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46361</v>
       </c>
       <c r="N25" t="s">
@@ -11408,7 +11434,7 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="1">
+      <c r="M27" s="2">
         <v>46296</v>
       </c>
       <c r="N27" t="s">
@@ -11452,7 +11478,7 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46361</v>
       </c>
       <c r="N28" t="s">
@@ -11496,7 +11522,7 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="2">
         <v>46316</v>
       </c>
       <c r="N29" t="s">
@@ -11540,7 +11566,7 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46361</v>
       </c>
       <c r="N30" t="s">
@@ -11584,7 +11610,7 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="2">
         <v>46316</v>
       </c>
       <c r="N31" t="s">
@@ -11628,7 +11654,7 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="1">
+      <c r="M32" s="2">
         <v>46296</v>
       </c>
       <c r="N32" t="s">
@@ -11672,7 +11698,7 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="1">
+      <c r="M33" s="2">
         <v>46296</v>
       </c>
       <c r="N33" t="s">
@@ -11716,7 +11742,7 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="1">
+      <c r="M34" s="2">
         <v>46296</v>
       </c>
       <c r="N34" t="s">
@@ -11760,7 +11786,7 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="1">
+      <c r="M35" s="2">
         <v>46296</v>
       </c>
       <c r="N35" t="s">
@@ -11804,7 +11830,7 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="1">
+      <c r="M36" s="2">
         <v>46296</v>
       </c>
       <c r="N36" t="s">
@@ -11848,7 +11874,7 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="1">
+      <c r="M37" s="2">
         <v>46296</v>
       </c>
       <c r="N37" t="s">
@@ -11892,7 +11918,7 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="1">
+      <c r="M38" s="2">
         <v>46296</v>
       </c>
       <c r="N38" t="s">
@@ -11977,7 +12003,7 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="1">
+      <c r="M40" s="2">
         <v>46296</v>
       </c>
       <c r="N40" t="s">
@@ -12021,7 +12047,7 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46361</v>
       </c>
       <c r="N41" t="s">
@@ -12065,7 +12091,7 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="1">
+      <c r="M42" s="2">
         <v>46296</v>
       </c>
       <c r="N42" t="s">
@@ -12109,7 +12135,7 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46361</v>
       </c>
       <c r="N43" t="s">
@@ -12153,7 +12179,7 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46361</v>
       </c>
       <c r="N44" t="s">
@@ -12197,7 +12223,7 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46361</v>
       </c>
       <c r="N45" t="s">
@@ -12241,7 +12267,7 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="1">
+      <c r="M46" s="2">
         <v>46296</v>
       </c>
       <c r="N46" t="s">
@@ -12285,7 +12311,7 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="1">
+      <c r="M47" s="2">
         <v>46296</v>
       </c>
       <c r="N47" t="s">
@@ -12329,7 +12355,7 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46361</v>
       </c>
       <c r="N48" t="s">
@@ -12373,7 +12399,7 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46316</v>
       </c>
       <c r="N49" t="s">
@@ -12417,7 +12443,7 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46316</v>
       </c>
       <c r="N50" t="s">
@@ -12461,7 +12487,7 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46361</v>
       </c>
       <c r="N51" t="s">
@@ -12505,7 +12531,7 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46361</v>
       </c>
       <c r="N52" t="s">
@@ -12549,7 +12575,7 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46361</v>
       </c>
       <c r="N53" t="s">
@@ -12593,7 +12619,7 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46361</v>
       </c>
       <c r="N54" t="s">
@@ -12637,7 +12663,7 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46361</v>
       </c>
       <c r="N55" t="s">
@@ -12681,7 +12707,7 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="1">
+      <c r="M56" s="2">
         <v>46316</v>
       </c>
       <c r="N56" t="s">
@@ -12725,7 +12751,7 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="1">
+      <c r="M57" s="2">
         <v>46316</v>
       </c>
       <c r="N57" t="s">
@@ -12769,7 +12795,7 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="1">
+      <c r="M58" s="2">
         <v>46316</v>
       </c>
       <c r="N58" t="s">
@@ -12813,7 +12839,7 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46361</v>
       </c>
       <c r="N59" t="s">
@@ -12857,7 +12883,7 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="1">
+      <c r="M60" s="2">
         <v>46316</v>
       </c>
       <c r="N60" t="s">
@@ -12901,7 +12927,7 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="1">
+      <c r="M61" s="2">
         <v>46316</v>
       </c>
       <c r="N61" t="s">
@@ -12945,7 +12971,7 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46361</v>
       </c>
       <c r="N62" t="s">
@@ -12989,7 +13015,7 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46361</v>
       </c>
       <c r="N63" t="s">
@@ -13033,7 +13059,7 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46361</v>
       </c>
       <c r="N64" t="s">
@@ -13077,7 +13103,7 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="1">
+      <c r="M65" s="2">
         <v>46361</v>
       </c>
       <c r="N65" t="s">
@@ -13121,7 +13147,7 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="1">
+      <c r="M66" s="2">
         <v>46361</v>
       </c>
       <c r="N66" t="s">
@@ -13165,7 +13191,7 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="1">
+      <c r="M67" s="2">
         <v>46361</v>
       </c>
       <c r="N67" t="s">
@@ -13209,7 +13235,7 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="1">
+      <c r="M68" s="2">
         <v>46361</v>
       </c>
       <c r="N68" t="s">
@@ -13253,7 +13279,7 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="1">
+      <c r="M69" s="2">
         <v>46361</v>
       </c>
       <c r="N69" t="s">
@@ -13338,7 +13364,7 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="1">
+      <c r="M71" s="2">
         <v>46376</v>
       </c>
       <c r="N71" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (22/09/2026 12:31)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1815,16 +1815,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1840,7 +1832,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1848,30 +1840,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2171,55 +2145,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2263,7 +2237,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2307,7 +2281,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2351,7 +2325,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2477,7 +2451,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2521,7 +2495,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2565,7 +2539,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2612,7 +2586,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2735,7 +2709,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2779,7 +2753,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2823,7 +2797,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2914,7 +2888,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2958,7 +2932,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3084,7 +3058,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3128,7 +3102,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3213,7 +3187,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3260,7 +3234,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3307,7 +3281,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3351,7 +3325,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3395,7 +3369,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3480,7 +3454,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3565,7 +3539,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3612,7 +3586,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3656,7 +3630,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3700,7 +3674,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3785,7 +3759,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3829,7 +3803,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3873,7 +3847,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3958,7 +3932,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4002,7 +3976,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4046,7 +4020,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4090,7 +4064,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4257,7 +4231,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4301,7 +4275,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4345,7 +4319,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4389,7 +4363,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4436,7 +4410,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4480,7 +4454,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4562,7 +4536,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4606,7 +4580,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4694,7 +4668,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4738,7 +4712,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4785,7 +4759,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4829,7 +4803,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4873,7 +4847,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4917,7 +4891,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4961,7 +4935,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5008,7 +4982,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5052,7 +5026,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5099,7 +5073,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5143,7 +5117,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5190,7 +5164,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5278,7 +5252,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5322,7 +5296,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5366,7 +5340,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5410,7 +5384,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5454,7 +5428,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5498,7 +5472,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5583,7 +5557,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5627,7 +5601,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5671,7 +5645,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5715,7 +5689,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5759,7 +5733,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5803,7 +5777,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5847,7 +5821,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5891,7 +5865,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5938,7 +5912,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5982,7 +5956,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6026,7 +6000,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6070,7 +6044,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6114,7 +6088,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6158,7 +6132,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6202,7 +6176,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6246,7 +6220,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6290,7 +6264,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6378,7 +6352,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6422,7 +6396,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6592,7 +6566,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6636,7 +6610,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6680,7 +6654,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6762,7 +6736,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6806,7 +6780,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6853,7 +6827,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6897,7 +6871,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7023,7 +6997,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7067,7 +7041,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7152,7 +7126,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7196,7 +7170,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7240,7 +7214,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7284,7 +7258,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7328,7 +7302,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7372,7 +7346,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7416,7 +7390,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7460,7 +7434,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7545,7 +7519,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7712,7 +7686,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7756,7 +7730,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7800,7 +7774,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7844,7 +7818,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7888,7 +7862,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7932,7 +7906,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7976,7 +7950,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8061,7 +8035,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8105,7 +8079,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8190,7 +8164,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8316,7 +8290,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8360,7 +8334,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8445,7 +8419,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8489,7 +8463,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8533,7 +8507,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8577,7 +8551,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8621,7 +8595,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8665,7 +8639,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8709,7 +8683,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8753,7 +8727,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8838,7 +8812,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9005,7 +8979,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9049,7 +9023,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9093,7 +9067,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9137,7 +9111,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9222,7 +9196,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9266,7 +9240,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9310,7 +9284,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9354,7 +9328,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9398,7 +9372,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9442,7 +9416,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9486,7 +9460,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9530,7 +9504,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9574,7 +9548,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9618,7 +9592,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9662,7 +9636,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9706,7 +9680,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9750,7 +9724,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9794,7 +9768,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9838,7 +9812,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9882,7 +9856,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9926,7 +9900,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9970,7 +9944,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10014,7 +9988,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10058,7 +10032,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10102,7 +10076,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10187,7 +10161,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10272,7 +10246,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10287,55 +10261,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10622,8 +10596,8 @@
       <c r="L8" t="s">
         <v>590</v>
       </c>
-      <c r="M8" s="2">
-        <v>46296</v>
+      <c r="M8" s="1">
+        <v>46297</v>
       </c>
       <c r="N8" t="s">
         <v>596</v>
@@ -10707,8 +10681,8 @@
       <c r="L10" t="s">
         <v>592</v>
       </c>
-      <c r="M10" s="2">
-        <v>46361</v>
+      <c r="M10" s="1">
+        <v>46362</v>
       </c>
       <c r="N10" t="s">
         <v>596</v>
@@ -10751,8 +10725,8 @@
       <c r="L11" t="s">
         <v>592</v>
       </c>
-      <c r="M11" s="2">
-        <v>46361</v>
+      <c r="M11" s="1">
+        <v>46362</v>
       </c>
       <c r="N11" t="s">
         <v>596</v>
@@ -10918,8 +10892,8 @@
       <c r="L15" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="2">
-        <v>46296</v>
+      <c r="M15" s="1">
+        <v>46297</v>
       </c>
       <c r="N15" t="s">
         <v>596</v>
@@ -10962,8 +10936,8 @@
       <c r="L16" t="s">
         <v>592</v>
       </c>
-      <c r="M16" s="2">
-        <v>46361</v>
+      <c r="M16" s="1">
+        <v>46362</v>
       </c>
       <c r="N16" t="s">
         <v>596</v>
@@ -11006,8 +10980,8 @@
       <c r="L17" t="s">
         <v>590</v>
       </c>
-      <c r="M17" s="2">
-        <v>46296</v>
+      <c r="M17" s="1">
+        <v>46297</v>
       </c>
       <c r="N17" t="s">
         <v>596</v>
@@ -11050,8 +11024,8 @@
       <c r="L18" t="s">
         <v>592</v>
       </c>
-      <c r="M18" s="2">
-        <v>46361</v>
+      <c r="M18" s="1">
+        <v>46362</v>
       </c>
       <c r="N18" t="s">
         <v>596</v>
@@ -11094,8 +11068,8 @@
       <c r="L19" t="s">
         <v>592</v>
       </c>
-      <c r="M19" s="2">
-        <v>46361</v>
+      <c r="M19" s="1">
+        <v>46362</v>
       </c>
       <c r="N19" t="s">
         <v>596</v>
@@ -11138,8 +11112,8 @@
       <c r="L20" t="s">
         <v>592</v>
       </c>
-      <c r="M20" s="2">
-        <v>46361</v>
+      <c r="M20" s="1">
+        <v>46362</v>
       </c>
       <c r="N20" t="s">
         <v>596</v>
@@ -11182,8 +11156,8 @@
       <c r="L21" t="s">
         <v>592</v>
       </c>
-      <c r="M21" s="2">
-        <v>46361</v>
+      <c r="M21" s="1">
+        <v>46362</v>
       </c>
       <c r="N21" t="s">
         <v>596</v>
@@ -11349,8 +11323,8 @@
       <c r="L25" t="s">
         <v>592</v>
       </c>
-      <c r="M25" s="2">
-        <v>46361</v>
+      <c r="M25" s="1">
+        <v>46362</v>
       </c>
       <c r="N25" t="s">
         <v>596</v>
@@ -11434,8 +11408,8 @@
       <c r="L27" t="s">
         <v>590</v>
       </c>
-      <c r="M27" s="2">
-        <v>46296</v>
+      <c r="M27" s="1">
+        <v>46297</v>
       </c>
       <c r="N27" t="s">
         <v>596</v>
@@ -11478,8 +11452,8 @@
       <c r="L28" t="s">
         <v>592</v>
       </c>
-      <c r="M28" s="2">
-        <v>46361</v>
+      <c r="M28" s="1">
+        <v>46362</v>
       </c>
       <c r="N28" t="s">
         <v>596</v>
@@ -11522,8 +11496,8 @@
       <c r="L29" t="s">
         <v>593</v>
       </c>
-      <c r="M29" s="2">
-        <v>46316</v>
+      <c r="M29" s="1">
+        <v>46317</v>
       </c>
       <c r="N29" t="s">
         <v>596</v>
@@ -11566,8 +11540,8 @@
       <c r="L30" t="s">
         <v>592</v>
       </c>
-      <c r="M30" s="2">
-        <v>46361</v>
+      <c r="M30" s="1">
+        <v>46362</v>
       </c>
       <c r="N30" t="s">
         <v>596</v>
@@ -11610,8 +11584,8 @@
       <c r="L31" t="s">
         <v>593</v>
       </c>
-      <c r="M31" s="2">
-        <v>46316</v>
+      <c r="M31" s="1">
+        <v>46317</v>
       </c>
       <c r="N31" t="s">
         <v>596</v>
@@ -11654,8 +11628,8 @@
       <c r="L32" t="s">
         <v>590</v>
       </c>
-      <c r="M32" s="2">
-        <v>46296</v>
+      <c r="M32" s="1">
+        <v>46297</v>
       </c>
       <c r="N32" t="s">
         <v>596</v>
@@ -11698,8 +11672,8 @@
       <c r="L33" t="s">
         <v>590</v>
       </c>
-      <c r="M33" s="2">
-        <v>46296</v>
+      <c r="M33" s="1">
+        <v>46297</v>
       </c>
       <c r="N33" t="s">
         <v>596</v>
@@ -11742,8 +11716,8 @@
       <c r="L34" t="s">
         <v>590</v>
       </c>
-      <c r="M34" s="2">
-        <v>46296</v>
+      <c r="M34" s="1">
+        <v>46297</v>
       </c>
       <c r="N34" t="s">
         <v>596</v>
@@ -11786,8 +11760,8 @@
       <c r="L35" t="s">
         <v>590</v>
       </c>
-      <c r="M35" s="2">
-        <v>46296</v>
+      <c r="M35" s="1">
+        <v>46297</v>
       </c>
       <c r="N35" t="s">
         <v>596</v>
@@ -11830,8 +11804,8 @@
       <c r="L36" t="s">
         <v>590</v>
       </c>
-      <c r="M36" s="2">
-        <v>46296</v>
+      <c r="M36" s="1">
+        <v>46297</v>
       </c>
       <c r="N36" t="s">
         <v>596</v>
@@ -11874,8 +11848,8 @@
       <c r="L37" t="s">
         <v>590</v>
       </c>
-      <c r="M37" s="2">
-        <v>46296</v>
+      <c r="M37" s="1">
+        <v>46297</v>
       </c>
       <c r="N37" t="s">
         <v>596</v>
@@ -11918,8 +11892,8 @@
       <c r="L38" t="s">
         <v>590</v>
       </c>
-      <c r="M38" s="2">
-        <v>46296</v>
+      <c r="M38" s="1">
+        <v>46297</v>
       </c>
       <c r="N38" t="s">
         <v>596</v>
@@ -12003,8 +11977,8 @@
       <c r="L40" t="s">
         <v>590</v>
       </c>
-      <c r="M40" s="2">
-        <v>46296</v>
+      <c r="M40" s="1">
+        <v>46297</v>
       </c>
       <c r="N40" t="s">
         <v>596</v>
@@ -12047,8 +12021,8 @@
       <c r="L41" t="s">
         <v>592</v>
       </c>
-      <c r="M41" s="2">
-        <v>46361</v>
+      <c r="M41" s="1">
+        <v>46362</v>
       </c>
       <c r="N41" t="s">
         <v>596</v>
@@ -12091,8 +12065,8 @@
       <c r="L42" t="s">
         <v>590</v>
       </c>
-      <c r="M42" s="2">
-        <v>46296</v>
+      <c r="M42" s="1">
+        <v>46297</v>
       </c>
       <c r="N42" t="s">
         <v>596</v>
@@ -12135,8 +12109,8 @@
       <c r="L43" t="s">
         <v>592</v>
       </c>
-      <c r="M43" s="2">
-        <v>46361</v>
+      <c r="M43" s="1">
+        <v>46362</v>
       </c>
       <c r="N43" t="s">
         <v>596</v>
@@ -12179,8 +12153,8 @@
       <c r="L44" t="s">
         <v>592</v>
       </c>
-      <c r="M44" s="2">
-        <v>46361</v>
+      <c r="M44" s="1">
+        <v>46362</v>
       </c>
       <c r="N44" t="s">
         <v>596</v>
@@ -12223,8 +12197,8 @@
       <c r="L45" t="s">
         <v>592</v>
       </c>
-      <c r="M45" s="2">
-        <v>46361</v>
+      <c r="M45" s="1">
+        <v>46362</v>
       </c>
       <c r="N45" t="s">
         <v>596</v>
@@ -12267,8 +12241,8 @@
       <c r="L46" t="s">
         <v>590</v>
       </c>
-      <c r="M46" s="2">
-        <v>46296</v>
+      <c r="M46" s="1">
+        <v>46297</v>
       </c>
       <c r="N46" t="s">
         <v>596</v>
@@ -12311,8 +12285,8 @@
       <c r="L47" t="s">
         <v>590</v>
       </c>
-      <c r="M47" s="2">
-        <v>46296</v>
+      <c r="M47" s="1">
+        <v>46297</v>
       </c>
       <c r="N47" t="s">
         <v>596</v>
@@ -12355,8 +12329,8 @@
       <c r="L48" t="s">
         <v>592</v>
       </c>
-      <c r="M48" s="2">
-        <v>46361</v>
+      <c r="M48" s="1">
+        <v>46362</v>
       </c>
       <c r="N48" t="s">
         <v>596</v>
@@ -12399,8 +12373,8 @@
       <c r="L49" t="s">
         <v>593</v>
       </c>
-      <c r="M49" s="2">
-        <v>46316</v>
+      <c r="M49" s="1">
+        <v>46317</v>
       </c>
       <c r="N49" t="s">
         <v>596</v>
@@ -12443,8 +12417,8 @@
       <c r="L50" t="s">
         <v>593</v>
       </c>
-      <c r="M50" s="2">
-        <v>46316</v>
+      <c r="M50" s="1">
+        <v>46317</v>
       </c>
       <c r="N50" t="s">
         <v>596</v>
@@ -12487,8 +12461,8 @@
       <c r="L51" t="s">
         <v>592</v>
       </c>
-      <c r="M51" s="2">
-        <v>46361</v>
+      <c r="M51" s="1">
+        <v>46362</v>
       </c>
       <c r="N51" t="s">
         <v>596</v>
@@ -12531,8 +12505,8 @@
       <c r="L52" t="s">
         <v>592</v>
       </c>
-      <c r="M52" s="2">
-        <v>46361</v>
+      <c r="M52" s="1">
+        <v>46362</v>
       </c>
       <c r="N52" t="s">
         <v>596</v>
@@ -12575,8 +12549,8 @@
       <c r="L53" t="s">
         <v>592</v>
       </c>
-      <c r="M53" s="2">
-        <v>46361</v>
+      <c r="M53" s="1">
+        <v>46362</v>
       </c>
       <c r="N53" t="s">
         <v>596</v>
@@ -12619,8 +12593,8 @@
       <c r="L54" t="s">
         <v>592</v>
       </c>
-      <c r="M54" s="2">
-        <v>46361</v>
+      <c r="M54" s="1">
+        <v>46362</v>
       </c>
       <c r="N54" t="s">
         <v>596</v>
@@ -12663,8 +12637,8 @@
       <c r="L55" t="s">
         <v>592</v>
       </c>
-      <c r="M55" s="2">
-        <v>46361</v>
+      <c r="M55" s="1">
+        <v>46362</v>
       </c>
       <c r="N55" t="s">
         <v>596</v>
@@ -12707,8 +12681,8 @@
       <c r="L56" t="s">
         <v>593</v>
       </c>
-      <c r="M56" s="2">
-        <v>46316</v>
+      <c r="M56" s="1">
+        <v>46317</v>
       </c>
       <c r="N56" t="s">
         <v>596</v>
@@ -12751,8 +12725,8 @@
       <c r="L57" t="s">
         <v>593</v>
       </c>
-      <c r="M57" s="2">
-        <v>46316</v>
+      <c r="M57" s="1">
+        <v>46317</v>
       </c>
       <c r="N57" t="s">
         <v>596</v>
@@ -12795,8 +12769,8 @@
       <c r="L58" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="2">
-        <v>46316</v>
+      <c r="M58" s="1">
+        <v>46317</v>
       </c>
       <c r="N58" t="s">
         <v>596</v>
@@ -12839,8 +12813,8 @@
       <c r="L59" t="s">
         <v>592</v>
       </c>
-      <c r="M59" s="2">
-        <v>46361</v>
+      <c r="M59" s="1">
+        <v>46362</v>
       </c>
       <c r="N59" t="s">
         <v>596</v>
@@ -12883,8 +12857,8 @@
       <c r="L60" t="s">
         <v>593</v>
       </c>
-      <c r="M60" s="2">
-        <v>46316</v>
+      <c r="M60" s="1">
+        <v>46317</v>
       </c>
       <c r="N60" t="s">
         <v>596</v>
@@ -12927,8 +12901,8 @@
       <c r="L61" t="s">
         <v>593</v>
       </c>
-      <c r="M61" s="2">
-        <v>46316</v>
+      <c r="M61" s="1">
+        <v>46317</v>
       </c>
       <c r="N61" t="s">
         <v>596</v>
@@ -12971,8 +12945,8 @@
       <c r="L62" t="s">
         <v>592</v>
       </c>
-      <c r="M62" s="2">
-        <v>46361</v>
+      <c r="M62" s="1">
+        <v>46362</v>
       </c>
       <c r="N62" t="s">
         <v>596</v>
@@ -13015,8 +12989,8 @@
       <c r="L63" t="s">
         <v>592</v>
       </c>
-      <c r="M63" s="2">
-        <v>46361</v>
+      <c r="M63" s="1">
+        <v>46362</v>
       </c>
       <c r="N63" t="s">
         <v>596</v>
@@ -13059,8 +13033,8 @@
       <c r="L64" t="s">
         <v>592</v>
       </c>
-      <c r="M64" s="2">
-        <v>46361</v>
+      <c r="M64" s="1">
+        <v>46362</v>
       </c>
       <c r="N64" t="s">
         <v>596</v>
@@ -13103,8 +13077,8 @@
       <c r="L65" t="s">
         <v>592</v>
       </c>
-      <c r="M65" s="2">
-        <v>46361</v>
+      <c r="M65" s="1">
+        <v>46362</v>
       </c>
       <c r="N65" t="s">
         <v>596</v>
@@ -13147,8 +13121,8 @@
       <c r="L66" t="s">
         <v>592</v>
       </c>
-      <c r="M66" s="2">
-        <v>46361</v>
+      <c r="M66" s="1">
+        <v>46362</v>
       </c>
       <c r="N66" t="s">
         <v>596</v>
@@ -13191,8 +13165,8 @@
       <c r="L67" t="s">
         <v>592</v>
       </c>
-      <c r="M67" s="2">
-        <v>46361</v>
+      <c r="M67" s="1">
+        <v>46362</v>
       </c>
       <c r="N67" t="s">
         <v>596</v>
@@ -13235,8 +13209,8 @@
       <c r="L68" t="s">
         <v>592</v>
       </c>
-      <c r="M68" s="2">
-        <v>46361</v>
+      <c r="M68" s="1">
+        <v>46362</v>
       </c>
       <c r="N68" t="s">
         <v>596</v>
@@ -13279,8 +13253,8 @@
       <c r="L69" t="s">
         <v>592</v>
       </c>
-      <c r="M69" s="2">
-        <v>46361</v>
+      <c r="M69" s="1">
+        <v>46362</v>
       </c>
       <c r="N69" t="s">
         <v>596</v>
@@ -13364,8 +13338,8 @@
       <c r="L71" t="s">
         <v>595</v>
       </c>
-      <c r="M71" s="2">
-        <v>46376</v>
+      <c r="M71" s="1">
+        <v>46377</v>
       </c>
       <c r="N71" t="s">
         <v>596</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (23/09/2026 12:27)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2073,16 +2073,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2098,7 +2090,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2106,30 +2098,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2429,55 +2403,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2521,7 +2495,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2565,7 +2539,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2609,7 +2583,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2735,7 +2709,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2779,7 +2753,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2823,7 +2797,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2870,7 +2844,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2993,7 +2967,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -3037,7 +3011,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3081,7 +3055,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3125,7 +3099,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3172,7 +3146,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3216,7 +3190,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3342,7 +3316,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3386,7 +3360,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3471,7 +3445,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3518,7 +3492,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3565,7 +3539,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3609,7 +3583,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3653,7 +3627,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3738,7 +3712,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3823,7 +3797,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3870,7 +3844,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3914,7 +3888,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3958,7 +3932,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4043,7 +4017,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4087,7 +4061,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4131,7 +4105,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4216,7 +4190,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4260,7 +4234,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4304,7 +4278,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4348,7 +4322,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4515,7 +4489,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4559,7 +4533,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4603,7 +4577,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4647,7 +4621,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4694,7 +4668,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4738,7 +4712,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4820,7 +4794,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4864,7 +4838,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4952,7 +4926,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4996,7 +4970,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5043,7 +5017,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5087,7 +5061,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -5131,7 +5105,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5175,7 +5149,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5219,7 +5193,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5266,7 +5240,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5310,7 +5284,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5357,7 +5331,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5401,7 +5375,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5448,7 +5422,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5536,7 +5510,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5580,7 +5554,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5624,7 +5598,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5668,7 +5642,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5712,7 +5686,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5756,7 +5730,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5841,7 +5815,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5885,7 +5859,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5929,7 +5903,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5973,7 +5947,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -6017,7 +5991,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -6061,7 +6035,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6105,7 +6079,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6149,7 +6123,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6196,7 +6170,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6240,7 +6214,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6284,7 +6258,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6328,7 +6302,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6372,7 +6346,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6416,7 +6390,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6460,7 +6434,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6504,7 +6478,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6636,7 +6610,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6680,7 +6654,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6806,7 +6780,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6850,7 +6824,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6894,7 +6868,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6938,7 +6912,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7020,7 +6994,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7064,7 +7038,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7111,7 +7085,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7155,7 +7129,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7281,7 +7255,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7325,7 +7299,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7410,7 +7384,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7454,7 +7428,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7498,7 +7472,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7542,7 +7516,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7586,7 +7560,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7630,7 +7604,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7674,7 +7648,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7718,7 +7692,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7803,7 +7777,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7970,7 +7944,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8014,7 +7988,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8058,7 +8032,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8102,7 +8076,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8146,7 +8120,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8190,7 +8164,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8234,7 +8208,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8319,7 +8293,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8363,7 +8337,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8448,7 +8422,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8574,7 +8548,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8618,7 +8592,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8703,7 +8677,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8747,7 +8721,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8791,7 +8765,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8835,7 +8809,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8879,7 +8853,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8923,7 +8897,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8967,7 +8941,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9011,7 +8985,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9096,7 +9070,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9263,7 +9237,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9307,7 +9281,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9351,7 +9325,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9395,7 +9369,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9480,7 +9454,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9524,7 +9498,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9568,7 +9542,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9612,7 +9586,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9656,7 +9630,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9700,7 +9674,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9744,7 +9718,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9788,7 +9762,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9832,7 +9806,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9876,7 +9850,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9920,7 +9894,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9964,7 +9938,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10008,7 +9982,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10052,7 +10026,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -10096,7 +10070,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10140,7 +10114,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10184,7 +10158,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10228,7 +10202,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10272,7 +10246,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10316,7 +10290,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10360,7 +10334,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10445,7 +10419,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10530,7 +10504,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10545,55 +10519,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10962,7 +10936,7 @@
       <c r="L10" t="s">
         <v>677</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46378</v>
       </c>
       <c r="N10" t="s">
@@ -11006,7 +10980,7 @@
       <c r="L11" t="s">
         <v>677</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46378</v>
       </c>
       <c r="N11" t="s">
@@ -11214,7 +11188,7 @@
       <c r="L16" t="s">
         <v>677</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46378</v>
       </c>
       <c r="N16" t="s">
@@ -11299,7 +11273,7 @@
       <c r="L18" t="s">
         <v>677</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46378</v>
       </c>
       <c r="N18" t="s">
@@ -11343,7 +11317,7 @@
       <c r="L19" t="s">
         <v>680</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46363</v>
       </c>
       <c r="N19" t="s">
@@ -11387,7 +11361,7 @@
       <c r="L20" t="s">
         <v>677</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46378</v>
       </c>
       <c r="N20" t="s">
@@ -11431,7 +11405,7 @@
       <c r="L21" t="s">
         <v>680</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46363</v>
       </c>
       <c r="N21" t="s">
@@ -11598,7 +11572,7 @@
       <c r="L25" t="s">
         <v>680</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46363</v>
       </c>
       <c r="N25" t="s">
@@ -11724,7 +11698,7 @@
       <c r="L28" t="s">
         <v>680</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46363</v>
       </c>
       <c r="N28" t="s">
@@ -11768,7 +11742,7 @@
       <c r="L29" t="s">
         <v>679</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46318</v>
       </c>
       <c r="N29" t="s">
@@ -11812,7 +11786,7 @@
       <c r="L30" t="s">
         <v>680</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46363</v>
       </c>
       <c r="N30" t="s">
@@ -11856,7 +11830,7 @@
       <c r="L31" t="s">
         <v>679</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46318</v>
       </c>
       <c r="N31" t="s">
@@ -12269,7 +12243,7 @@
       <c r="L41" t="s">
         <v>680</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46363</v>
       </c>
       <c r="N41" t="s">
@@ -12354,7 +12328,7 @@
       <c r="L43" t="s">
         <v>680</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46363</v>
       </c>
       <c r="N43" t="s">
@@ -12398,7 +12372,7 @@
       <c r="L44" t="s">
         <v>680</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46363</v>
       </c>
       <c r="N44" t="s">
@@ -12442,7 +12416,7 @@
       <c r="L45" t="s">
         <v>680</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46363</v>
       </c>
       <c r="N45" t="s">
@@ -12568,7 +12542,7 @@
       <c r="L48" t="s">
         <v>680</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46363</v>
       </c>
       <c r="N48" t="s">
@@ -12612,7 +12586,7 @@
       <c r="L49" t="s">
         <v>679</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46318</v>
       </c>
       <c r="N49" t="s">
@@ -12656,7 +12630,7 @@
       <c r="L50" t="s">
         <v>679</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46318</v>
       </c>
       <c r="N50" t="s">
@@ -12700,7 +12674,7 @@
       <c r="L51" t="s">
         <v>680</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46363</v>
       </c>
       <c r="N51" t="s">
@@ -12744,7 +12718,7 @@
       <c r="L52" t="s">
         <v>680</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46363</v>
       </c>
       <c r="N52" t="s">
@@ -12788,7 +12762,7 @@
       <c r="L53" t="s">
         <v>680</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46363</v>
       </c>
       <c r="N53" t="s">
@@ -12832,7 +12806,7 @@
       <c r="L54" t="s">
         <v>680</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46363</v>
       </c>
       <c r="N54" t="s">
@@ -12876,7 +12850,7 @@
       <c r="L55" t="s">
         <v>680</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46363</v>
       </c>
       <c r="N55" t="s">
@@ -12920,7 +12894,7 @@
       <c r="L56" t="s">
         <v>679</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46318</v>
       </c>
       <c r="N56" t="s">
@@ -12964,7 +12938,7 @@
       <c r="L57" t="s">
         <v>679</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46318</v>
       </c>
       <c r="N57" t="s">
@@ -13008,7 +12982,7 @@
       <c r="L58" t="s">
         <v>679</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46318</v>
       </c>
       <c r="N58" t="s">
@@ -13052,7 +13026,7 @@
       <c r="L59" t="s">
         <v>680</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46363</v>
       </c>
       <c r="N59" t="s">
@@ -13096,7 +13070,7 @@
       <c r="L60" t="s">
         <v>679</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46318</v>
       </c>
       <c r="N60" t="s">
@@ -13140,7 +13114,7 @@
       <c r="L61" t="s">
         <v>679</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46318</v>
       </c>
       <c r="N61" t="s">
@@ -13184,7 +13158,7 @@
       <c r="L62" t="s">
         <v>680</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46363</v>
       </c>
       <c r="N62" t="s">
@@ -13228,7 +13202,7 @@
       <c r="L63" t="s">
         <v>680</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46363</v>
       </c>
       <c r="N63" t="s">
@@ -13272,7 +13246,7 @@
       <c r="L64" t="s">
         <v>680</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46363</v>
       </c>
       <c r="N64" t="s">
@@ -13316,7 +13290,7 @@
       <c r="L65" t="s">
         <v>680</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="1">
         <v>46363</v>
       </c>
       <c r="N65" t="s">
@@ -13360,7 +13334,7 @@
       <c r="L66" t="s">
         <v>680</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="1">
         <v>46363</v>
       </c>
       <c r="N66" t="s">
@@ -13404,7 +13378,7 @@
       <c r="L67" t="s">
         <v>680</v>
       </c>
-      <c r="M67" s="2">
+      <c r="M67" s="1">
         <v>46363</v>
       </c>
       <c r="N67" t="s">
@@ -13448,7 +13422,7 @@
       <c r="L68" t="s">
         <v>680</v>
       </c>
-      <c r="M68" s="2">
+      <c r="M68" s="1">
         <v>46363</v>
       </c>
       <c r="N68" t="s">
@@ -13492,7 +13466,7 @@
       <c r="L69" t="s">
         <v>680</v>
       </c>
-      <c r="M69" s="2">
+      <c r="M69" s="1">
         <v>46363</v>
       </c>
       <c r="N69" t="s">
@@ -13536,7 +13510,7 @@
       <c r="L70" t="s">
         <v>680</v>
       </c>
-      <c r="M70" s="2">
+      <c r="M70" s="1">
         <v>46363</v>
       </c>
       <c r="N70" t="s">
@@ -13580,7 +13554,7 @@
       <c r="L71" t="s">
         <v>680</v>
       </c>
-      <c r="M71" s="2">
+      <c r="M71" s="1">
         <v>46363</v>
       </c>
       <c r="N71" t="s">
@@ -13624,7 +13598,7 @@
       <c r="L72" t="s">
         <v>680</v>
       </c>
-      <c r="M72" s="2">
+      <c r="M72" s="1">
         <v>46363</v>
       </c>
       <c r="N72" t="s">
@@ -13668,7 +13642,7 @@
       <c r="L73" t="s">
         <v>677</v>
       </c>
-      <c r="M73" s="2">
+      <c r="M73" s="1">
         <v>46378</v>
       </c>
       <c r="N73" t="s">
@@ -13712,7 +13686,7 @@
       <c r="L74" t="s">
         <v>680</v>
       </c>
-      <c r="M74" s="2">
+      <c r="M74" s="1">
         <v>46363</v>
       </c>
       <c r="N74" t="s">
@@ -13756,7 +13730,7 @@
       <c r="L75" t="s">
         <v>680</v>
       </c>
-      <c r="M75" s="2">
+      <c r="M75" s="1">
         <v>46363</v>
       </c>
       <c r="N75" t="s">
@@ -13841,7 +13815,7 @@
       <c r="L77" t="s">
         <v>677</v>
       </c>
-      <c r="M77" s="2">
+      <c r="M77" s="1">
         <v>46378</v>
       </c>
       <c r="N77" t="s">
@@ -13885,7 +13859,7 @@
       <c r="L78" t="s">
         <v>680</v>
       </c>
-      <c r="M78" s="2">
+      <c r="M78" s="1">
         <v>46363</v>
       </c>
       <c r="N78" t="s">
@@ -13929,7 +13903,7 @@
       <c r="L79" t="s">
         <v>680</v>
       </c>
-      <c r="M79" s="2">
+      <c r="M79" s="1">
         <v>46363</v>
       </c>
       <c r="N79" t="s">
@@ -13973,7 +13947,7 @@
       <c r="L80" t="s">
         <v>677</v>
       </c>
-      <c r="M80" s="2">
+      <c r="M80" s="1">
         <v>46378</v>
       </c>
       <c r="N80" t="s">
@@ -14017,7 +13991,7 @@
       <c r="L81" t="s">
         <v>677</v>
       </c>
-      <c r="M81" s="2">
+      <c r="M81" s="1">
         <v>46378</v>
       </c>
       <c r="N81" t="s">
@@ -14061,7 +14035,7 @@
       <c r="L82" t="s">
         <v>677</v>
       </c>
-      <c r="M82" s="2">
+      <c r="M82" s="1">
         <v>46378</v>
       </c>
       <c r="N82" t="s">
@@ -14105,7 +14079,7 @@
       <c r="L83" t="s">
         <v>677</v>
       </c>
-      <c r="M83" s="2">
+      <c r="M83" s="1">
         <v>46378</v>
       </c>
       <c r="N83" t="s">
@@ -14149,7 +14123,7 @@
       <c r="L84" t="s">
         <v>677</v>
       </c>
-      <c r="M84" s="2">
+      <c r="M84" s="1">
         <v>46378</v>
       </c>
       <c r="N84" t="s">
@@ -14193,7 +14167,7 @@
       <c r="L85" t="s">
         <v>680</v>
       </c>
-      <c r="M85" s="2">
+      <c r="M85" s="1">
         <v>46363</v>
       </c>
       <c r="N85" t="s">
@@ -14237,7 +14211,7 @@
       <c r="L86" t="s">
         <v>680</v>
       </c>
-      <c r="M86" s="2">
+      <c r="M86" s="1">
         <v>46363</v>
       </c>
       <c r="N86" t="s">
@@ -14281,7 +14255,7 @@
       <c r="L87" t="s">
         <v>680</v>
       </c>
-      <c r="M87" s="2">
+      <c r="M87" s="1">
         <v>46363</v>
       </c>
       <c r="N87" t="s">
@@ -14325,7 +14299,7 @@
       <c r="L88" t="s">
         <v>680</v>
       </c>
-      <c r="M88" s="2">
+      <c r="M88" s="1">
         <v>46363</v>
       </c>
       <c r="N88" t="s">
@@ -14369,7 +14343,7 @@
       <c r="L89" t="s">
         <v>680</v>
       </c>
-      <c r="M89" s="2">
+      <c r="M89" s="1">
         <v>46363</v>
       </c>
       <c r="N89" t="s">
@@ -14413,7 +14387,7 @@
       <c r="L90" t="s">
         <v>680</v>
       </c>
-      <c r="M90" s="2">
+      <c r="M90" s="1">
         <v>46363</v>
       </c>
       <c r="N90" t="s">
@@ -14457,7 +14431,7 @@
       <c r="L91" t="s">
         <v>680</v>
       </c>
-      <c r="M91" s="2">
+      <c r="M91" s="1">
         <v>46363</v>
       </c>
       <c r="N91" t="s">
@@ -14501,7 +14475,7 @@
       <c r="L92" t="s">
         <v>680</v>
       </c>
-      <c r="M92" s="2">
+      <c r="M92" s="1">
         <v>46363</v>
       </c>
       <c r="N92" t="s">
@@ -14545,7 +14519,7 @@
       <c r="L93" t="s">
         <v>680</v>
       </c>
-      <c r="M93" s="2">
+      <c r="M93" s="1">
         <v>46363</v>
       </c>
       <c r="N93" t="s">
@@ -14589,7 +14563,7 @@
       <c r="L94" t="s">
         <v>680</v>
       </c>
-      <c r="M94" s="2">
+      <c r="M94" s="1">
         <v>46363</v>
       </c>
       <c r="N94" t="s">
@@ -14633,7 +14607,7 @@
       <c r="L95" t="s">
         <v>680</v>
       </c>
-      <c r="M95" s="2">
+      <c r="M95" s="1">
         <v>46363</v>
       </c>
       <c r="N95" t="s">
@@ -14677,7 +14651,7 @@
       <c r="L96" t="s">
         <v>680</v>
       </c>
-      <c r="M96" s="2">
+      <c r="M96" s="1">
         <v>46363</v>
       </c>
       <c r="N96" t="s">
@@ -14721,7 +14695,7 @@
       <c r="L97" t="s">
         <v>680</v>
       </c>
-      <c r="M97" s="2">
+      <c r="M97" s="1">
         <v>46363</v>
       </c>
       <c r="N97" t="s">
@@ -14765,7 +14739,7 @@
       <c r="L98" t="s">
         <v>680</v>
       </c>
-      <c r="M98" s="2">
+      <c r="M98" s="1">
         <v>46363</v>
       </c>
       <c r="N98" t="s">
@@ -14809,7 +14783,7 @@
       <c r="L99" t="s">
         <v>680</v>
       </c>
-      <c r="M99" s="2">
+      <c r="M99" s="1">
         <v>46363</v>
       </c>
       <c r="N99" t="s">
@@ -14853,7 +14827,7 @@
       <c r="L100" t="s">
         <v>680</v>
       </c>
-      <c r="M100" s="2">
+      <c r="M100" s="1">
         <v>46363</v>
       </c>
       <c r="N100" t="s">
@@ -14897,7 +14871,7 @@
       <c r="L101" t="s">
         <v>680</v>
       </c>
-      <c r="M101" s="2">
+      <c r="M101" s="1">
         <v>46363</v>
       </c>
       <c r="N101" t="s">
@@ -14941,7 +14915,7 @@
       <c r="L102" t="s">
         <v>680</v>
       </c>
-      <c r="M102" s="2">
+      <c r="M102" s="1">
         <v>46363</v>
       </c>
       <c r="N102" t="s">
@@ -14985,7 +14959,7 @@
       <c r="L103" t="s">
         <v>680</v>
       </c>
-      <c r="M103" s="2">
+      <c r="M103" s="1">
         <v>46363</v>
       </c>
       <c r="N103" t="s">
@@ -15029,7 +15003,7 @@
       <c r="L104" t="s">
         <v>680</v>
       </c>
-      <c r="M104" s="2">
+      <c r="M104" s="1">
         <v>46363</v>
       </c>
       <c r="N104" t="s">
@@ -15073,7 +15047,7 @@
       <c r="L105" t="s">
         <v>680</v>
       </c>
-      <c r="M105" s="2">
+      <c r="M105" s="1">
         <v>46363</v>
       </c>
       <c r="N105" t="s">
@@ -15117,7 +15091,7 @@
       <c r="L106" t="s">
         <v>680</v>
       </c>
-      <c r="M106" s="2">
+      <c r="M106" s="1">
         <v>46363</v>
       </c>
       <c r="N106" t="s">
@@ -15161,7 +15135,7 @@
       <c r="L107" t="s">
         <v>680</v>
       </c>
-      <c r="M107" s="2">
+      <c r="M107" s="1">
         <v>46363</v>
       </c>
       <c r="N107" t="s">
@@ -15205,7 +15179,7 @@
       <c r="L108" t="s">
         <v>680</v>
       </c>
-      <c r="M108" s="2">
+      <c r="M108" s="1">
         <v>46363</v>
       </c>
       <c r="N108" t="s">
@@ -15249,7 +15223,7 @@
       <c r="L109" t="s">
         <v>680</v>
       </c>
-      <c r="M109" s="2">
+      <c r="M109" s="1">
         <v>46363</v>
       </c>
       <c r="N109" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (24/09/2026 12:49)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10937,7 +10937,7 @@
         <v>677</v>
       </c>
       <c r="M10" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N10" t="s">
         <v>682</v>
@@ -10981,7 +10981,7 @@
         <v>677</v>
       </c>
       <c r="M11" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N11" t="s">
         <v>682</v>
@@ -11189,7 +11189,7 @@
         <v>677</v>
       </c>
       <c r="M16" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N16" t="s">
         <v>682</v>
@@ -11274,7 +11274,7 @@
         <v>677</v>
       </c>
       <c r="M18" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N18" t="s">
         <v>682</v>
@@ -11318,7 +11318,7 @@
         <v>680</v>
       </c>
       <c r="M19" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N19" t="s">
         <v>682</v>
@@ -11362,7 +11362,7 @@
         <v>677</v>
       </c>
       <c r="M20" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N20" t="s">
         <v>682</v>
@@ -11406,7 +11406,7 @@
         <v>680</v>
       </c>
       <c r="M21" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N21" t="s">
         <v>682</v>
@@ -11573,7 +11573,7 @@
         <v>680</v>
       </c>
       <c r="M25" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N25" t="s">
         <v>682</v>
@@ -11699,7 +11699,7 @@
         <v>680</v>
       </c>
       <c r="M28" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N28" t="s">
         <v>682</v>
@@ -11743,7 +11743,7 @@
         <v>679</v>
       </c>
       <c r="M29" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N29" t="s">
         <v>682</v>
@@ -11787,7 +11787,7 @@
         <v>680</v>
       </c>
       <c r="M30" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N30" t="s">
         <v>682</v>
@@ -11831,7 +11831,7 @@
         <v>679</v>
       </c>
       <c r="M31" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N31" t="s">
         <v>682</v>
@@ -12244,7 +12244,7 @@
         <v>680</v>
       </c>
       <c r="M41" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N41" t="s">
         <v>682</v>
@@ -12329,7 +12329,7 @@
         <v>680</v>
       </c>
       <c r="M43" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N43" t="s">
         <v>682</v>
@@ -12373,7 +12373,7 @@
         <v>680</v>
       </c>
       <c r="M44" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N44" t="s">
         <v>682</v>
@@ -12417,7 +12417,7 @@
         <v>680</v>
       </c>
       <c r="M45" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N45" t="s">
         <v>682</v>
@@ -12543,7 +12543,7 @@
         <v>680</v>
       </c>
       <c r="M48" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N48" t="s">
         <v>682</v>
@@ -12587,7 +12587,7 @@
         <v>679</v>
       </c>
       <c r="M49" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N49" t="s">
         <v>682</v>
@@ -12631,7 +12631,7 @@
         <v>679</v>
       </c>
       <c r="M50" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N50" t="s">
         <v>682</v>
@@ -12675,7 +12675,7 @@
         <v>680</v>
       </c>
       <c r="M51" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N51" t="s">
         <v>682</v>
@@ -12719,7 +12719,7 @@
         <v>680</v>
       </c>
       <c r="M52" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N52" t="s">
         <v>682</v>
@@ -12763,7 +12763,7 @@
         <v>680</v>
       </c>
       <c r="M53" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N53" t="s">
         <v>682</v>
@@ -12807,7 +12807,7 @@
         <v>680</v>
       </c>
       <c r="M54" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N54" t="s">
         <v>682</v>
@@ -12851,7 +12851,7 @@
         <v>680</v>
       </c>
       <c r="M55" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N55" t="s">
         <v>682</v>
@@ -12895,7 +12895,7 @@
         <v>679</v>
       </c>
       <c r="M56" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N56" t="s">
         <v>682</v>
@@ -12939,7 +12939,7 @@
         <v>679</v>
       </c>
       <c r="M57" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N57" t="s">
         <v>682</v>
@@ -12983,7 +12983,7 @@
         <v>679</v>
       </c>
       <c r="M58" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N58" t="s">
         <v>682</v>
@@ -13027,7 +13027,7 @@
         <v>680</v>
       </c>
       <c r="M59" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N59" t="s">
         <v>682</v>
@@ -13071,7 +13071,7 @@
         <v>679</v>
       </c>
       <c r="M60" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N60" t="s">
         <v>682</v>
@@ -13115,7 +13115,7 @@
         <v>679</v>
       </c>
       <c r="M61" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N61" t="s">
         <v>682</v>
@@ -13159,7 +13159,7 @@
         <v>680</v>
       </c>
       <c r="M62" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N62" t="s">
         <v>682</v>
@@ -13203,7 +13203,7 @@
         <v>680</v>
       </c>
       <c r="M63" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N63" t="s">
         <v>682</v>
@@ -13247,7 +13247,7 @@
         <v>680</v>
       </c>
       <c r="M64" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N64" t="s">
         <v>682</v>
@@ -13291,7 +13291,7 @@
         <v>680</v>
       </c>
       <c r="M65" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N65" t="s">
         <v>682</v>
@@ -13335,7 +13335,7 @@
         <v>680</v>
       </c>
       <c r="M66" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N66" t="s">
         <v>682</v>
@@ -13379,7 +13379,7 @@
         <v>680</v>
       </c>
       <c r="M67" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N67" t="s">
         <v>682</v>
@@ -13423,7 +13423,7 @@
         <v>680</v>
       </c>
       <c r="M68" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N68" t="s">
         <v>682</v>
@@ -13467,7 +13467,7 @@
         <v>680</v>
       </c>
       <c r="M69" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N69" t="s">
         <v>682</v>
@@ -13511,7 +13511,7 @@
         <v>680</v>
       </c>
       <c r="M70" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N70" t="s">
         <v>682</v>
@@ -13555,7 +13555,7 @@
         <v>680</v>
       </c>
       <c r="M71" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N71" t="s">
         <v>682</v>
@@ -13599,7 +13599,7 @@
         <v>680</v>
       </c>
       <c r="M72" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N72" t="s">
         <v>682</v>
@@ -13643,7 +13643,7 @@
         <v>677</v>
       </c>
       <c r="M73" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N73" t="s">
         <v>682</v>
@@ -13687,7 +13687,7 @@
         <v>680</v>
       </c>
       <c r="M74" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N74" t="s">
         <v>682</v>
@@ -13731,7 +13731,7 @@
         <v>680</v>
       </c>
       <c r="M75" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N75" t="s">
         <v>682</v>
@@ -13816,7 +13816,7 @@
         <v>677</v>
       </c>
       <c r="M77" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N77" t="s">
         <v>682</v>
@@ -13860,7 +13860,7 @@
         <v>680</v>
       </c>
       <c r="M78" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N78" t="s">
         <v>682</v>
@@ -13904,7 +13904,7 @@
         <v>680</v>
       </c>
       <c r="M79" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N79" t="s">
         <v>682</v>
@@ -13948,7 +13948,7 @@
         <v>677</v>
       </c>
       <c r="M80" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N80" t="s">
         <v>682</v>
@@ -13992,7 +13992,7 @@
         <v>677</v>
       </c>
       <c r="M81" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N81" t="s">
         <v>682</v>
@@ -14036,7 +14036,7 @@
         <v>677</v>
       </c>
       <c r="M82" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N82" t="s">
         <v>682</v>
@@ -14080,7 +14080,7 @@
         <v>677</v>
       </c>
       <c r="M83" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N83" t="s">
         <v>682</v>
@@ -14124,7 +14124,7 @@
         <v>677</v>
       </c>
       <c r="M84" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N84" t="s">
         <v>682</v>
@@ -14168,7 +14168,7 @@
         <v>680</v>
       </c>
       <c r="M85" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N85" t="s">
         <v>682</v>
@@ -14212,7 +14212,7 @@
         <v>680</v>
       </c>
       <c r="M86" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N86" t="s">
         <v>682</v>
@@ -14256,7 +14256,7 @@
         <v>680</v>
       </c>
       <c r="M87" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N87" t="s">
         <v>682</v>
@@ -14300,7 +14300,7 @@
         <v>680</v>
       </c>
       <c r="M88" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N88" t="s">
         <v>682</v>
@@ -14344,7 +14344,7 @@
         <v>680</v>
       </c>
       <c r="M89" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N89" t="s">
         <v>682</v>
@@ -14388,7 +14388,7 @@
         <v>680</v>
       </c>
       <c r="M90" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N90" t="s">
         <v>682</v>
@@ -14432,7 +14432,7 @@
         <v>680</v>
       </c>
       <c r="M91" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N91" t="s">
         <v>682</v>
@@ -14476,7 +14476,7 @@
         <v>680</v>
       </c>
       <c r="M92" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N92" t="s">
         <v>682</v>
@@ -14520,7 +14520,7 @@
         <v>680</v>
       </c>
       <c r="M93" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N93" t="s">
         <v>682</v>
@@ -14564,7 +14564,7 @@
         <v>680</v>
       </c>
       <c r="M94" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N94" t="s">
         <v>682</v>
@@ -14608,7 +14608,7 @@
         <v>680</v>
       </c>
       <c r="M95" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N95" t="s">
         <v>682</v>
@@ -14652,7 +14652,7 @@
         <v>680</v>
       </c>
       <c r="M96" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N96" t="s">
         <v>682</v>
@@ -14696,7 +14696,7 @@
         <v>680</v>
       </c>
       <c r="M97" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N97" t="s">
         <v>682</v>
@@ -14740,7 +14740,7 @@
         <v>680</v>
       </c>
       <c r="M98" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N98" t="s">
         <v>682</v>
@@ -14784,7 +14784,7 @@
         <v>680</v>
       </c>
       <c r="M99" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N99" t="s">
         <v>682</v>
@@ -14828,7 +14828,7 @@
         <v>680</v>
       </c>
       <c r="M100" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N100" t="s">
         <v>682</v>
@@ -14872,7 +14872,7 @@
         <v>680</v>
       </c>
       <c r="M101" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N101" t="s">
         <v>682</v>
@@ -14916,7 +14916,7 @@
         <v>680</v>
       </c>
       <c r="M102" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N102" t="s">
         <v>682</v>
@@ -14960,7 +14960,7 @@
         <v>680</v>
       </c>
       <c r="M103" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N103" t="s">
         <v>682</v>
@@ -15004,7 +15004,7 @@
         <v>680</v>
       </c>
       <c r="M104" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N104" t="s">
         <v>682</v>
@@ -15048,7 +15048,7 @@
         <v>680</v>
       </c>
       <c r="M105" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N105" t="s">
         <v>682</v>
@@ -15092,7 +15092,7 @@
         <v>680</v>
       </c>
       <c r="M106" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N106" t="s">
         <v>682</v>
@@ -15136,7 +15136,7 @@
         <v>680</v>
       </c>
       <c r="M107" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N107" t="s">
         <v>682</v>
@@ -15180,7 +15180,7 @@
         <v>680</v>
       </c>
       <c r="M108" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N108" t="s">
         <v>682</v>
@@ -15224,7 +15224,7 @@
         <v>680</v>
       </c>
       <c r="M109" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N109" t="s">
         <v>682</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (25/09/2026 12:50)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10937,7 +10937,7 @@
         <v>677</v>
       </c>
       <c r="M10" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N10" t="s">
         <v>682</v>
@@ -10981,7 +10981,7 @@
         <v>677</v>
       </c>
       <c r="M11" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N11" t="s">
         <v>682</v>
@@ -11189,7 +11189,7 @@
         <v>677</v>
       </c>
       <c r="M16" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N16" t="s">
         <v>682</v>
@@ -11274,7 +11274,7 @@
         <v>677</v>
       </c>
       <c r="M18" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N18" t="s">
         <v>682</v>
@@ -11318,7 +11318,7 @@
         <v>680</v>
       </c>
       <c r="M19" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N19" t="s">
         <v>682</v>
@@ -11362,7 +11362,7 @@
         <v>677</v>
       </c>
       <c r="M20" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N20" t="s">
         <v>682</v>
@@ -11406,7 +11406,7 @@
         <v>680</v>
       </c>
       <c r="M21" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N21" t="s">
         <v>682</v>
@@ -11573,7 +11573,7 @@
         <v>680</v>
       </c>
       <c r="M25" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N25" t="s">
         <v>682</v>
@@ -11699,7 +11699,7 @@
         <v>680</v>
       </c>
       <c r="M28" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N28" t="s">
         <v>682</v>
@@ -11743,7 +11743,7 @@
         <v>679</v>
       </c>
       <c r="M29" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N29" t="s">
         <v>682</v>
@@ -11787,7 +11787,7 @@
         <v>680</v>
       </c>
       <c r="M30" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N30" t="s">
         <v>682</v>
@@ -11831,7 +11831,7 @@
         <v>679</v>
       </c>
       <c r="M31" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N31" t="s">
         <v>682</v>
@@ -12244,7 +12244,7 @@
         <v>680</v>
       </c>
       <c r="M41" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N41" t="s">
         <v>682</v>
@@ -12329,7 +12329,7 @@
         <v>680</v>
       </c>
       <c r="M43" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N43" t="s">
         <v>682</v>
@@ -12373,7 +12373,7 @@
         <v>680</v>
       </c>
       <c r="M44" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N44" t="s">
         <v>682</v>
@@ -12417,7 +12417,7 @@
         <v>680</v>
       </c>
       <c r="M45" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N45" t="s">
         <v>682</v>
@@ -12543,7 +12543,7 @@
         <v>680</v>
       </c>
       <c r="M48" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N48" t="s">
         <v>682</v>
@@ -12587,7 +12587,7 @@
         <v>679</v>
       </c>
       <c r="M49" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N49" t="s">
         <v>682</v>
@@ -12631,7 +12631,7 @@
         <v>679</v>
       </c>
       <c r="M50" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N50" t="s">
         <v>682</v>
@@ -12675,7 +12675,7 @@
         <v>680</v>
       </c>
       <c r="M51" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N51" t="s">
         <v>682</v>
@@ -12719,7 +12719,7 @@
         <v>680</v>
       </c>
       <c r="M52" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N52" t="s">
         <v>682</v>
@@ -12763,7 +12763,7 @@
         <v>680</v>
       </c>
       <c r="M53" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N53" t="s">
         <v>682</v>
@@ -12807,7 +12807,7 @@
         <v>680</v>
       </c>
       <c r="M54" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N54" t="s">
         <v>682</v>
@@ -12851,7 +12851,7 @@
         <v>680</v>
       </c>
       <c r="M55" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N55" t="s">
         <v>682</v>
@@ -12895,7 +12895,7 @@
         <v>679</v>
       </c>
       <c r="M56" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N56" t="s">
         <v>682</v>
@@ -12939,7 +12939,7 @@
         <v>679</v>
       </c>
       <c r="M57" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N57" t="s">
         <v>682</v>
@@ -12983,7 +12983,7 @@
         <v>679</v>
       </c>
       <c r="M58" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N58" t="s">
         <v>682</v>
@@ -13027,7 +13027,7 @@
         <v>680</v>
       </c>
       <c r="M59" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N59" t="s">
         <v>682</v>
@@ -13071,7 +13071,7 @@
         <v>679</v>
       </c>
       <c r="M60" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N60" t="s">
         <v>682</v>
@@ -13115,7 +13115,7 @@
         <v>679</v>
       </c>
       <c r="M61" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N61" t="s">
         <v>682</v>
@@ -13159,7 +13159,7 @@
         <v>680</v>
       </c>
       <c r="M62" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N62" t="s">
         <v>682</v>
@@ -13203,7 +13203,7 @@
         <v>680</v>
       </c>
       <c r="M63" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N63" t="s">
         <v>682</v>
@@ -13247,7 +13247,7 @@
         <v>680</v>
       </c>
       <c r="M64" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N64" t="s">
         <v>682</v>
@@ -13291,7 +13291,7 @@
         <v>680</v>
       </c>
       <c r="M65" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N65" t="s">
         <v>682</v>
@@ -13335,7 +13335,7 @@
         <v>680</v>
       </c>
       <c r="M66" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N66" t="s">
         <v>682</v>
@@ -13379,7 +13379,7 @@
         <v>680</v>
       </c>
       <c r="M67" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N67" t="s">
         <v>682</v>
@@ -13423,7 +13423,7 @@
         <v>680</v>
       </c>
       <c r="M68" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N68" t="s">
         <v>682</v>
@@ -13467,7 +13467,7 @@
         <v>680</v>
       </c>
       <c r="M69" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N69" t="s">
         <v>682</v>
@@ -13511,7 +13511,7 @@
         <v>680</v>
       </c>
       <c r="M70" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N70" t="s">
         <v>682</v>
@@ -13555,7 +13555,7 @@
         <v>680</v>
       </c>
       <c r="M71" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N71" t="s">
         <v>682</v>
@@ -13599,7 +13599,7 @@
         <v>680</v>
       </c>
       <c r="M72" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N72" t="s">
         <v>682</v>
@@ -13643,7 +13643,7 @@
         <v>677</v>
       </c>
       <c r="M73" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N73" t="s">
         <v>682</v>
@@ -13687,7 +13687,7 @@
         <v>680</v>
       </c>
       <c r="M74" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N74" t="s">
         <v>682</v>
@@ -13731,7 +13731,7 @@
         <v>680</v>
       </c>
       <c r="M75" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N75" t="s">
         <v>682</v>
@@ -13816,7 +13816,7 @@
         <v>677</v>
       </c>
       <c r="M77" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N77" t="s">
         <v>682</v>
@@ -13860,7 +13860,7 @@
         <v>680</v>
       </c>
       <c r="M78" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N78" t="s">
         <v>682</v>
@@ -13904,7 +13904,7 @@
         <v>680</v>
       </c>
       <c r="M79" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N79" t="s">
         <v>682</v>
@@ -13948,7 +13948,7 @@
         <v>677</v>
       </c>
       <c r="M80" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N80" t="s">
         <v>682</v>
@@ -13992,7 +13992,7 @@
         <v>677</v>
       </c>
       <c r="M81" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N81" t="s">
         <v>682</v>
@@ -14036,7 +14036,7 @@
         <v>677</v>
       </c>
       <c r="M82" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N82" t="s">
         <v>682</v>
@@ -14080,7 +14080,7 @@
         <v>677</v>
       </c>
       <c r="M83" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N83" t="s">
         <v>682</v>
@@ -14124,7 +14124,7 @@
         <v>677</v>
       </c>
       <c r="M84" s="1">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="N84" t="s">
         <v>682</v>
@@ -14168,7 +14168,7 @@
         <v>680</v>
       </c>
       <c r="M85" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N85" t="s">
         <v>682</v>
@@ -14212,7 +14212,7 @@
         <v>680</v>
       </c>
       <c r="M86" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N86" t="s">
         <v>682</v>
@@ -14256,7 +14256,7 @@
         <v>680</v>
       </c>
       <c r="M87" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N87" t="s">
         <v>682</v>
@@ -14300,7 +14300,7 @@
         <v>680</v>
       </c>
       <c r="M88" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N88" t="s">
         <v>682</v>
@@ -14344,7 +14344,7 @@
         <v>680</v>
       </c>
       <c r="M89" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N89" t="s">
         <v>682</v>
@@ -14388,7 +14388,7 @@
         <v>680</v>
       </c>
       <c r="M90" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N90" t="s">
         <v>682</v>
@@ -14432,7 +14432,7 @@
         <v>680</v>
       </c>
       <c r="M91" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N91" t="s">
         <v>682</v>
@@ -14476,7 +14476,7 @@
         <v>680</v>
       </c>
       <c r="M92" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N92" t="s">
         <v>682</v>
@@ -14520,7 +14520,7 @@
         <v>680</v>
       </c>
       <c r="M93" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N93" t="s">
         <v>682</v>
@@ -14564,7 +14564,7 @@
         <v>680</v>
       </c>
       <c r="M94" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N94" t="s">
         <v>682</v>
@@ -14608,7 +14608,7 @@
         <v>680</v>
       </c>
       <c r="M95" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N95" t="s">
         <v>682</v>
@@ -14652,7 +14652,7 @@
         <v>680</v>
       </c>
       <c r="M96" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N96" t="s">
         <v>682</v>
@@ -14696,7 +14696,7 @@
         <v>680</v>
       </c>
       <c r="M97" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N97" t="s">
         <v>682</v>
@@ -14740,7 +14740,7 @@
         <v>680</v>
       </c>
       <c r="M98" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N98" t="s">
         <v>682</v>
@@ -14784,7 +14784,7 @@
         <v>680</v>
       </c>
       <c r="M99" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N99" t="s">
         <v>682</v>
@@ -14828,7 +14828,7 @@
         <v>680</v>
       </c>
       <c r="M100" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N100" t="s">
         <v>682</v>
@@ -14872,7 +14872,7 @@
         <v>680</v>
       </c>
       <c r="M101" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N101" t="s">
         <v>682</v>
@@ -14916,7 +14916,7 @@
         <v>680</v>
       </c>
       <c r="M102" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N102" t="s">
         <v>682</v>
@@ -14960,7 +14960,7 @@
         <v>680</v>
       </c>
       <c r="M103" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N103" t="s">
         <v>682</v>
@@ -15004,7 +15004,7 @@
         <v>680</v>
       </c>
       <c r="M104" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N104" t="s">
         <v>682</v>
@@ -15048,7 +15048,7 @@
         <v>680</v>
       </c>
       <c r="M105" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N105" t="s">
         <v>682</v>
@@ -15092,7 +15092,7 @@
         <v>680</v>
       </c>
       <c r="M106" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N106" t="s">
         <v>682</v>
@@ -15136,7 +15136,7 @@
         <v>680</v>
       </c>
       <c r="M107" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N107" t="s">
         <v>682</v>
@@ -15180,7 +15180,7 @@
         <v>680</v>
       </c>
       <c r="M108" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N108" t="s">
         <v>682</v>
@@ -15224,7 +15224,7 @@
         <v>680</v>
       </c>
       <c r="M109" s="1">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="N109" t="s">
         <v>682</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (28/09/2026 13:07)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2073,8 +2073,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2090,7 +2098,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2098,12 +2106,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2403,55 +2429,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2495,7 +2521,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2539,7 +2565,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2583,7 +2609,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2709,7 +2735,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2753,7 +2779,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2797,7 +2823,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2844,7 +2870,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2967,7 +2993,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -3011,7 +3037,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3055,7 +3081,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3099,7 +3125,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3146,7 +3172,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3190,7 +3216,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3316,7 +3342,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3360,7 +3386,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3445,7 +3471,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3492,7 +3518,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3539,7 +3565,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3583,7 +3609,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3627,7 +3653,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3712,7 +3738,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3797,7 +3823,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3844,7 +3870,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3888,7 +3914,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3932,7 +3958,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4017,7 +4043,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4061,7 +4087,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4105,7 +4131,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4190,7 +4216,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4234,7 +4260,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4278,7 +4304,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4322,7 +4348,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4489,7 +4515,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4533,7 +4559,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4577,7 +4603,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4621,7 +4647,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4668,7 +4694,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4712,7 +4738,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4794,7 +4820,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4838,7 +4864,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4926,7 +4952,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4970,7 +4996,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5017,7 +5043,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5061,7 +5087,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -5105,7 +5131,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5149,7 +5175,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5193,7 +5219,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5240,7 +5266,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5284,7 +5310,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5331,7 +5357,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5375,7 +5401,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5422,7 +5448,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5510,7 +5536,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5554,7 +5580,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5598,7 +5624,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5642,7 +5668,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5686,7 +5712,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5730,7 +5756,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5815,7 +5841,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5859,7 +5885,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5903,7 +5929,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5947,7 +5973,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5991,7 +6017,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -6035,7 +6061,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6079,7 +6105,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6123,7 +6149,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6170,7 +6196,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6214,7 +6240,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6258,7 +6284,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6302,7 +6328,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6346,7 +6372,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6390,7 +6416,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6434,7 +6460,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6478,7 +6504,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6610,7 +6636,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6654,7 +6680,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6780,7 +6806,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6824,7 +6850,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6868,7 +6894,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6912,7 +6938,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6994,7 +7020,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7038,7 +7064,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7085,7 +7111,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7129,7 +7155,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7255,7 +7281,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7299,7 +7325,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7384,7 +7410,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7428,7 +7454,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7472,7 +7498,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7516,7 +7542,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7560,7 +7586,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7604,7 +7630,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7648,7 +7674,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7692,7 +7718,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7777,7 +7803,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7944,7 +7970,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7988,7 +8014,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8032,7 +8058,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8076,7 +8102,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8120,7 +8146,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8164,7 +8190,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8208,7 +8234,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8293,7 +8319,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8337,7 +8363,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8422,7 +8448,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8548,7 +8574,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8592,7 +8618,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8677,7 +8703,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8721,7 +8747,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8765,7 +8791,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8809,7 +8835,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8853,7 +8879,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8897,7 +8923,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8941,7 +8967,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8985,7 +9011,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9070,7 +9096,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9237,7 +9263,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9281,7 +9307,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9325,7 +9351,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9369,7 +9395,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9454,7 +9480,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9498,7 +9524,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9542,7 +9568,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9586,7 +9612,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9630,7 +9656,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9674,7 +9700,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9718,7 +9744,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9762,7 +9788,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9806,7 +9832,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9850,7 +9876,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9894,7 +9920,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9938,7 +9964,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9982,7 +10008,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10026,7 +10052,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -10070,7 +10096,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10114,7 +10140,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10158,7 +10184,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10202,7 +10228,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10246,7 +10272,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10290,7 +10316,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10334,7 +10360,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10419,7 +10445,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10504,7 +10530,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10519,55 +10545,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10936,8 +10962,8 @@
       <c r="L10" t="s">
         <v>677</v>
       </c>
-      <c r="M10" s="1">
-        <v>46380</v>
+      <c r="M10" s="2">
+        <v>46383</v>
       </c>
       <c r="N10" t="s">
         <v>682</v>
@@ -10980,8 +11006,8 @@
       <c r="L11" t="s">
         <v>677</v>
       </c>
-      <c r="M11" s="1">
-        <v>46380</v>
+      <c r="M11" s="2">
+        <v>46383</v>
       </c>
       <c r="N11" t="s">
         <v>682</v>
@@ -11188,8 +11214,8 @@
       <c r="L16" t="s">
         <v>677</v>
       </c>
-      <c r="M16" s="1">
-        <v>46380</v>
+      <c r="M16" s="2">
+        <v>46383</v>
       </c>
       <c r="N16" t="s">
         <v>682</v>
@@ -11273,8 +11299,8 @@
       <c r="L18" t="s">
         <v>677</v>
       </c>
-      <c r="M18" s="1">
-        <v>46380</v>
+      <c r="M18" s="2">
+        <v>46383</v>
       </c>
       <c r="N18" t="s">
         <v>682</v>
@@ -11317,8 +11343,8 @@
       <c r="L19" t="s">
         <v>680</v>
       </c>
-      <c r="M19" s="1">
-        <v>46365</v>
+      <c r="M19" s="2">
+        <v>46368</v>
       </c>
       <c r="N19" t="s">
         <v>682</v>
@@ -11361,8 +11387,8 @@
       <c r="L20" t="s">
         <v>677</v>
       </c>
-      <c r="M20" s="1">
-        <v>46380</v>
+      <c r="M20" s="2">
+        <v>46383</v>
       </c>
       <c r="N20" t="s">
         <v>682</v>
@@ -11405,8 +11431,8 @@
       <c r="L21" t="s">
         <v>680</v>
       </c>
-      <c r="M21" s="1">
-        <v>46365</v>
+      <c r="M21" s="2">
+        <v>46368</v>
       </c>
       <c r="N21" t="s">
         <v>682</v>
@@ -11572,8 +11598,8 @@
       <c r="L25" t="s">
         <v>680</v>
       </c>
-      <c r="M25" s="1">
-        <v>46365</v>
+      <c r="M25" s="2">
+        <v>46368</v>
       </c>
       <c r="N25" t="s">
         <v>682</v>
@@ -11698,8 +11724,8 @@
       <c r="L28" t="s">
         <v>680</v>
       </c>
-      <c r="M28" s="1">
-        <v>46365</v>
+      <c r="M28" s="2">
+        <v>46368</v>
       </c>
       <c r="N28" t="s">
         <v>682</v>
@@ -11742,8 +11768,8 @@
       <c r="L29" t="s">
         <v>679</v>
       </c>
-      <c r="M29" s="1">
-        <v>46320</v>
+      <c r="M29" s="2">
+        <v>46323</v>
       </c>
       <c r="N29" t="s">
         <v>682</v>
@@ -11786,8 +11812,8 @@
       <c r="L30" t="s">
         <v>680</v>
       </c>
-      <c r="M30" s="1">
-        <v>46365</v>
+      <c r="M30" s="2">
+        <v>46368</v>
       </c>
       <c r="N30" t="s">
         <v>682</v>
@@ -11830,8 +11856,8 @@
       <c r="L31" t="s">
         <v>679</v>
       </c>
-      <c r="M31" s="1">
-        <v>46320</v>
+      <c r="M31" s="2">
+        <v>46323</v>
       </c>
       <c r="N31" t="s">
         <v>682</v>
@@ -12243,8 +12269,8 @@
       <c r="L41" t="s">
         <v>680</v>
       </c>
-      <c r="M41" s="1">
-        <v>46365</v>
+      <c r="M41" s="2">
+        <v>46368</v>
       </c>
       <c r="N41" t="s">
         <v>682</v>
@@ -12328,8 +12354,8 @@
       <c r="L43" t="s">
         <v>680</v>
       </c>
-      <c r="M43" s="1">
-        <v>46365</v>
+      <c r="M43" s="2">
+        <v>46368</v>
       </c>
       <c r="N43" t="s">
         <v>682</v>
@@ -12372,8 +12398,8 @@
       <c r="L44" t="s">
         <v>680</v>
       </c>
-      <c r="M44" s="1">
-        <v>46365</v>
+      <c r="M44" s="2">
+        <v>46368</v>
       </c>
       <c r="N44" t="s">
         <v>682</v>
@@ -12416,8 +12442,8 @@
       <c r="L45" t="s">
         <v>680</v>
       </c>
-      <c r="M45" s="1">
-        <v>46365</v>
+      <c r="M45" s="2">
+        <v>46368</v>
       </c>
       <c r="N45" t="s">
         <v>682</v>
@@ -12542,8 +12568,8 @@
       <c r="L48" t="s">
         <v>680</v>
       </c>
-      <c r="M48" s="1">
-        <v>46365</v>
+      <c r="M48" s="2">
+        <v>46368</v>
       </c>
       <c r="N48" t="s">
         <v>682</v>
@@ -12586,8 +12612,8 @@
       <c r="L49" t="s">
         <v>679</v>
       </c>
-      <c r="M49" s="1">
-        <v>46320</v>
+      <c r="M49" s="2">
+        <v>46323</v>
       </c>
       <c r="N49" t="s">
         <v>682</v>
@@ -12630,8 +12656,8 @@
       <c r="L50" t="s">
         <v>679</v>
       </c>
-      <c r="M50" s="1">
-        <v>46320</v>
+      <c r="M50" s="2">
+        <v>46323</v>
       </c>
       <c r="N50" t="s">
         <v>682</v>
@@ -12674,8 +12700,8 @@
       <c r="L51" t="s">
         <v>680</v>
       </c>
-      <c r="M51" s="1">
-        <v>46365</v>
+      <c r="M51" s="2">
+        <v>46368</v>
       </c>
       <c r="N51" t="s">
         <v>682</v>
@@ -12718,8 +12744,8 @@
       <c r="L52" t="s">
         <v>680</v>
       </c>
-      <c r="M52" s="1">
-        <v>46365</v>
+      <c r="M52" s="2">
+        <v>46368</v>
       </c>
       <c r="N52" t="s">
         <v>682</v>
@@ -12762,8 +12788,8 @@
       <c r="L53" t="s">
         <v>680</v>
       </c>
-      <c r="M53" s="1">
-        <v>46365</v>
+      <c r="M53" s="2">
+        <v>46368</v>
       </c>
       <c r="N53" t="s">
         <v>682</v>
@@ -12806,8 +12832,8 @@
       <c r="L54" t="s">
         <v>680</v>
       </c>
-      <c r="M54" s="1">
-        <v>46365</v>
+      <c r="M54" s="2">
+        <v>46368</v>
       </c>
       <c r="N54" t="s">
         <v>682</v>
@@ -12850,8 +12876,8 @@
       <c r="L55" t="s">
         <v>680</v>
       </c>
-      <c r="M55" s="1">
-        <v>46365</v>
+      <c r="M55" s="2">
+        <v>46368</v>
       </c>
       <c r="N55" t="s">
         <v>682</v>
@@ -12894,8 +12920,8 @@
       <c r="L56" t="s">
         <v>679</v>
       </c>
-      <c r="M56" s="1">
-        <v>46320</v>
+      <c r="M56" s="2">
+        <v>46323</v>
       </c>
       <c r="N56" t="s">
         <v>682</v>
@@ -12938,8 +12964,8 @@
       <c r="L57" t="s">
         <v>679</v>
       </c>
-      <c r="M57" s="1">
-        <v>46320</v>
+      <c r="M57" s="2">
+        <v>46323</v>
       </c>
       <c r="N57" t="s">
         <v>682</v>
@@ -12982,8 +13008,8 @@
       <c r="L58" t="s">
         <v>679</v>
       </c>
-      <c r="M58" s="1">
-        <v>46320</v>
+      <c r="M58" s="2">
+        <v>46323</v>
       </c>
       <c r="N58" t="s">
         <v>682</v>
@@ -13026,8 +13052,8 @@
       <c r="L59" t="s">
         <v>680</v>
       </c>
-      <c r="M59" s="1">
-        <v>46365</v>
+      <c r="M59" s="2">
+        <v>46368</v>
       </c>
       <c r="N59" t="s">
         <v>682</v>
@@ -13070,8 +13096,8 @@
       <c r="L60" t="s">
         <v>679</v>
       </c>
-      <c r="M60" s="1">
-        <v>46320</v>
+      <c r="M60" s="2">
+        <v>46323</v>
       </c>
       <c r="N60" t="s">
         <v>682</v>
@@ -13114,8 +13140,8 @@
       <c r="L61" t="s">
         <v>679</v>
       </c>
-      <c r="M61" s="1">
-        <v>46320</v>
+      <c r="M61" s="2">
+        <v>46323</v>
       </c>
       <c r="N61" t="s">
         <v>682</v>
@@ -13158,8 +13184,8 @@
       <c r="L62" t="s">
         <v>680</v>
       </c>
-      <c r="M62" s="1">
-        <v>46365</v>
+      <c r="M62" s="2">
+        <v>46368</v>
       </c>
       <c r="N62" t="s">
         <v>682</v>
@@ -13202,8 +13228,8 @@
       <c r="L63" t="s">
         <v>680</v>
       </c>
-      <c r="M63" s="1">
-        <v>46365</v>
+      <c r="M63" s="2">
+        <v>46368</v>
       </c>
       <c r="N63" t="s">
         <v>682</v>
@@ -13246,8 +13272,8 @@
       <c r="L64" t="s">
         <v>680</v>
       </c>
-      <c r="M64" s="1">
-        <v>46365</v>
+      <c r="M64" s="2">
+        <v>46368</v>
       </c>
       <c r="N64" t="s">
         <v>682</v>
@@ -13290,8 +13316,8 @@
       <c r="L65" t="s">
         <v>680</v>
       </c>
-      <c r="M65" s="1">
-        <v>46365</v>
+      <c r="M65" s="2">
+        <v>46368</v>
       </c>
       <c r="N65" t="s">
         <v>682</v>
@@ -13334,8 +13360,8 @@
       <c r="L66" t="s">
         <v>680</v>
       </c>
-      <c r="M66" s="1">
-        <v>46365</v>
+      <c r="M66" s="2">
+        <v>46368</v>
       </c>
       <c r="N66" t="s">
         <v>682</v>
@@ -13378,8 +13404,8 @@
       <c r="L67" t="s">
         <v>680</v>
       </c>
-      <c r="M67" s="1">
-        <v>46365</v>
+      <c r="M67" s="2">
+        <v>46368</v>
       </c>
       <c r="N67" t="s">
         <v>682</v>
@@ -13422,8 +13448,8 @@
       <c r="L68" t="s">
         <v>680</v>
       </c>
-      <c r="M68" s="1">
-        <v>46365</v>
+      <c r="M68" s="2">
+        <v>46368</v>
       </c>
       <c r="N68" t="s">
         <v>682</v>
@@ -13466,8 +13492,8 @@
       <c r="L69" t="s">
         <v>680</v>
       </c>
-      <c r="M69" s="1">
-        <v>46365</v>
+      <c r="M69" s="2">
+        <v>46368</v>
       </c>
       <c r="N69" t="s">
         <v>682</v>
@@ -13510,8 +13536,8 @@
       <c r="L70" t="s">
         <v>680</v>
       </c>
-      <c r="M70" s="1">
-        <v>46365</v>
+      <c r="M70" s="2">
+        <v>46368</v>
       </c>
       <c r="N70" t="s">
         <v>682</v>
@@ -13554,8 +13580,8 @@
       <c r="L71" t="s">
         <v>680</v>
       </c>
-      <c r="M71" s="1">
-        <v>46365</v>
+      <c r="M71" s="2">
+        <v>46368</v>
       </c>
       <c r="N71" t="s">
         <v>682</v>
@@ -13598,8 +13624,8 @@
       <c r="L72" t="s">
         <v>680</v>
       </c>
-      <c r="M72" s="1">
-        <v>46365</v>
+      <c r="M72" s="2">
+        <v>46368</v>
       </c>
       <c r="N72" t="s">
         <v>682</v>
@@ -13642,8 +13668,8 @@
       <c r="L73" t="s">
         <v>677</v>
       </c>
-      <c r="M73" s="1">
-        <v>46380</v>
+      <c r="M73" s="2">
+        <v>46383</v>
       </c>
       <c r="N73" t="s">
         <v>682</v>
@@ -13686,8 +13712,8 @@
       <c r="L74" t="s">
         <v>680</v>
       </c>
-      <c r="M74" s="1">
-        <v>46365</v>
+      <c r="M74" s="2">
+        <v>46368</v>
       </c>
       <c r="N74" t="s">
         <v>682</v>
@@ -13730,8 +13756,8 @@
       <c r="L75" t="s">
         <v>680</v>
       </c>
-      <c r="M75" s="1">
-        <v>46365</v>
+      <c r="M75" s="2">
+        <v>46368</v>
       </c>
       <c r="N75" t="s">
         <v>682</v>
@@ -13815,8 +13841,8 @@
       <c r="L77" t="s">
         <v>677</v>
       </c>
-      <c r="M77" s="1">
-        <v>46380</v>
+      <c r="M77" s="2">
+        <v>46383</v>
       </c>
       <c r="N77" t="s">
         <v>682</v>
@@ -13859,8 +13885,8 @@
       <c r="L78" t="s">
         <v>680</v>
       </c>
-      <c r="M78" s="1">
-        <v>46365</v>
+      <c r="M78" s="2">
+        <v>46368</v>
       </c>
       <c r="N78" t="s">
         <v>682</v>
@@ -13903,8 +13929,8 @@
       <c r="L79" t="s">
         <v>680</v>
       </c>
-      <c r="M79" s="1">
-        <v>46365</v>
+      <c r="M79" s="2">
+        <v>46368</v>
       </c>
       <c r="N79" t="s">
         <v>682</v>
@@ -13947,8 +13973,8 @@
       <c r="L80" t="s">
         <v>677</v>
       </c>
-      <c r="M80" s="1">
-        <v>46380</v>
+      <c r="M80" s="2">
+        <v>46383</v>
       </c>
       <c r="N80" t="s">
         <v>682</v>
@@ -13991,8 +14017,8 @@
       <c r="L81" t="s">
         <v>677</v>
       </c>
-      <c r="M81" s="1">
-        <v>46380</v>
+      <c r="M81" s="2">
+        <v>46383</v>
       </c>
       <c r="N81" t="s">
         <v>682</v>
@@ -14035,8 +14061,8 @@
       <c r="L82" t="s">
         <v>677</v>
       </c>
-      <c r="M82" s="1">
-        <v>46380</v>
+      <c r="M82" s="2">
+        <v>46383</v>
       </c>
       <c r="N82" t="s">
         <v>682</v>
@@ -14079,8 +14105,8 @@
       <c r="L83" t="s">
         <v>677</v>
       </c>
-      <c r="M83" s="1">
-        <v>46380</v>
+      <c r="M83" s="2">
+        <v>46383</v>
       </c>
       <c r="N83" t="s">
         <v>682</v>
@@ -14123,8 +14149,8 @@
       <c r="L84" t="s">
         <v>677</v>
       </c>
-      <c r="M84" s="1">
-        <v>46380</v>
+      <c r="M84" s="2">
+        <v>46383</v>
       </c>
       <c r="N84" t="s">
         <v>682</v>
@@ -14167,8 +14193,8 @@
       <c r="L85" t="s">
         <v>680</v>
       </c>
-      <c r="M85" s="1">
-        <v>46365</v>
+      <c r="M85" s="2">
+        <v>46368</v>
       </c>
       <c r="N85" t="s">
         <v>682</v>
@@ -14211,8 +14237,8 @@
       <c r="L86" t="s">
         <v>680</v>
       </c>
-      <c r="M86" s="1">
-        <v>46365</v>
+      <c r="M86" s="2">
+        <v>46368</v>
       </c>
       <c r="N86" t="s">
         <v>682</v>
@@ -14255,8 +14281,8 @@
       <c r="L87" t="s">
         <v>680</v>
       </c>
-      <c r="M87" s="1">
-        <v>46365</v>
+      <c r="M87" s="2">
+        <v>46368</v>
       </c>
       <c r="N87" t="s">
         <v>682</v>
@@ -14299,8 +14325,8 @@
       <c r="L88" t="s">
         <v>680</v>
       </c>
-      <c r="M88" s="1">
-        <v>46365</v>
+      <c r="M88" s="2">
+        <v>46368</v>
       </c>
       <c r="N88" t="s">
         <v>682</v>
@@ -14343,8 +14369,8 @@
       <c r="L89" t="s">
         <v>680</v>
       </c>
-      <c r="M89" s="1">
-        <v>46365</v>
+      <c r="M89" s="2">
+        <v>46368</v>
       </c>
       <c r="N89" t="s">
         <v>682</v>
@@ -14387,8 +14413,8 @@
       <c r="L90" t="s">
         <v>680</v>
       </c>
-      <c r="M90" s="1">
-        <v>46365</v>
+      <c r="M90" s="2">
+        <v>46368</v>
       </c>
       <c r="N90" t="s">
         <v>682</v>
@@ -14431,8 +14457,8 @@
       <c r="L91" t="s">
         <v>680</v>
       </c>
-      <c r="M91" s="1">
-        <v>46365</v>
+      <c r="M91" s="2">
+        <v>46368</v>
       </c>
       <c r="N91" t="s">
         <v>682</v>
@@ -14475,8 +14501,8 @@
       <c r="L92" t="s">
         <v>680</v>
       </c>
-      <c r="M92" s="1">
-        <v>46365</v>
+      <c r="M92" s="2">
+        <v>46368</v>
       </c>
       <c r="N92" t="s">
         <v>682</v>
@@ -14519,8 +14545,8 @@
       <c r="L93" t="s">
         <v>680</v>
       </c>
-      <c r="M93" s="1">
-        <v>46365</v>
+      <c r="M93" s="2">
+        <v>46368</v>
       </c>
       <c r="N93" t="s">
         <v>682</v>
@@ -14563,8 +14589,8 @@
       <c r="L94" t="s">
         <v>680</v>
       </c>
-      <c r="M94" s="1">
-        <v>46365</v>
+      <c r="M94" s="2">
+        <v>46368</v>
       </c>
       <c r="N94" t="s">
         <v>682</v>
@@ -14607,8 +14633,8 @@
       <c r="L95" t="s">
         <v>680</v>
       </c>
-      <c r="M95" s="1">
-        <v>46365</v>
+      <c r="M95" s="2">
+        <v>46368</v>
       </c>
       <c r="N95" t="s">
         <v>682</v>
@@ -14651,8 +14677,8 @@
       <c r="L96" t="s">
         <v>680</v>
       </c>
-      <c r="M96" s="1">
-        <v>46365</v>
+      <c r="M96" s="2">
+        <v>46368</v>
       </c>
       <c r="N96" t="s">
         <v>682</v>
@@ -14695,8 +14721,8 @@
       <c r="L97" t="s">
         <v>680</v>
       </c>
-      <c r="M97" s="1">
-        <v>46365</v>
+      <c r="M97" s="2">
+        <v>46368</v>
       </c>
       <c r="N97" t="s">
         <v>682</v>
@@ -14739,8 +14765,8 @@
       <c r="L98" t="s">
         <v>680</v>
       </c>
-      <c r="M98" s="1">
-        <v>46365</v>
+      <c r="M98" s="2">
+        <v>46368</v>
       </c>
       <c r="N98" t="s">
         <v>682</v>
@@ -14783,8 +14809,8 @@
       <c r="L99" t="s">
         <v>680</v>
       </c>
-      <c r="M99" s="1">
-        <v>46365</v>
+      <c r="M99" s="2">
+        <v>46368</v>
       </c>
       <c r="N99" t="s">
         <v>682</v>
@@ -14827,8 +14853,8 @@
       <c r="L100" t="s">
         <v>680</v>
       </c>
-      <c r="M100" s="1">
-        <v>46365</v>
+      <c r="M100" s="2">
+        <v>46368</v>
       </c>
       <c r="N100" t="s">
         <v>682</v>
@@ -14871,8 +14897,8 @@
       <c r="L101" t="s">
         <v>680</v>
       </c>
-      <c r="M101" s="1">
-        <v>46365</v>
+      <c r="M101" s="2">
+        <v>46368</v>
       </c>
       <c r="N101" t="s">
         <v>682</v>
@@ -14915,8 +14941,8 @@
       <c r="L102" t="s">
         <v>680</v>
       </c>
-      <c r="M102" s="1">
-        <v>46365</v>
+      <c r="M102" s="2">
+        <v>46368</v>
       </c>
       <c r="N102" t="s">
         <v>682</v>
@@ -14959,8 +14985,8 @@
       <c r="L103" t="s">
         <v>680</v>
       </c>
-      <c r="M103" s="1">
-        <v>46365</v>
+      <c r="M103" s="2">
+        <v>46368</v>
       </c>
       <c r="N103" t="s">
         <v>682</v>
@@ -15003,8 +15029,8 @@
       <c r="L104" t="s">
         <v>680</v>
       </c>
-      <c r="M104" s="1">
-        <v>46365</v>
+      <c r="M104" s="2">
+        <v>46368</v>
       </c>
       <c r="N104" t="s">
         <v>682</v>
@@ -15047,8 +15073,8 @@
       <c r="L105" t="s">
         <v>680</v>
       </c>
-      <c r="M105" s="1">
-        <v>46365</v>
+      <c r="M105" s="2">
+        <v>46368</v>
       </c>
       <c r="N105" t="s">
         <v>682</v>
@@ -15091,8 +15117,8 @@
       <c r="L106" t="s">
         <v>680</v>
       </c>
-      <c r="M106" s="1">
-        <v>46365</v>
+      <c r="M106" s="2">
+        <v>46368</v>
       </c>
       <c r="N106" t="s">
         <v>682</v>
@@ -15135,8 +15161,8 @@
       <c r="L107" t="s">
         <v>680</v>
       </c>
-      <c r="M107" s="1">
-        <v>46365</v>
+      <c r="M107" s="2">
+        <v>46368</v>
       </c>
       <c r="N107" t="s">
         <v>682</v>
@@ -15179,8 +15205,8 @@
       <c r="L108" t="s">
         <v>680</v>
       </c>
-      <c r="M108" s="1">
-        <v>46365</v>
+      <c r="M108" s="2">
+        <v>46368</v>
       </c>
       <c r="N108" t="s">
         <v>682</v>
@@ -15223,8 +15249,8 @@
       <c r="L109" t="s">
         <v>680</v>
       </c>
-      <c r="M109" s="1">
-        <v>46365</v>
+      <c r="M109" s="2">
+        <v>46368</v>
       </c>
       <c r="N109" t="s">
         <v>682</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (28/09/2026 15:35)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2073,16 +2073,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2098,7 +2090,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2106,30 +2098,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2429,55 +2403,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2521,7 +2495,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2565,7 +2539,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2609,7 +2583,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2735,7 +2709,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2779,7 +2753,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2823,7 +2797,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2870,7 +2844,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2993,7 +2967,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -3037,7 +3011,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3081,7 +3055,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3125,7 +3099,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3172,7 +3146,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3216,7 +3190,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3342,7 +3316,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3386,7 +3360,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3471,7 +3445,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3518,7 +3492,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3565,7 +3539,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3609,7 +3583,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3653,7 +3627,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3738,7 +3712,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3823,7 +3797,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3870,7 +3844,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3914,7 +3888,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3958,7 +3932,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4043,7 +4017,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4087,7 +4061,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4131,7 +4105,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4216,7 +4190,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4260,7 +4234,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4304,7 +4278,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4348,7 +4322,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4515,7 +4489,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4559,7 +4533,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4603,7 +4577,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4647,7 +4621,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4694,7 +4668,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4738,7 +4712,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4820,7 +4794,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4864,7 +4838,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4952,7 +4926,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4996,7 +4970,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5043,7 +5017,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5087,7 +5061,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -5131,7 +5105,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5175,7 +5149,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5219,7 +5193,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5266,7 +5240,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5310,7 +5284,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5357,7 +5331,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5401,7 +5375,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5448,7 +5422,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5536,7 +5510,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5580,7 +5554,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5624,7 +5598,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5668,7 +5642,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5712,7 +5686,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5756,7 +5730,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5841,7 +5815,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5885,7 +5859,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5929,7 +5903,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5973,7 +5947,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -6017,7 +5991,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -6061,7 +6035,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6105,7 +6079,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6149,7 +6123,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6196,7 +6170,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6240,7 +6214,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6284,7 +6258,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6328,7 +6302,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6372,7 +6346,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6416,7 +6390,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6460,7 +6434,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6504,7 +6478,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6636,7 +6610,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6680,7 +6654,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6806,7 +6780,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6850,7 +6824,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6894,7 +6868,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6938,7 +6912,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7020,7 +6994,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7064,7 +7038,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7111,7 +7085,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7155,7 +7129,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7281,7 +7255,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7325,7 +7299,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7410,7 +7384,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7454,7 +7428,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7498,7 +7472,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7542,7 +7516,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7586,7 +7560,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7630,7 +7604,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7674,7 +7648,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7718,7 +7692,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7803,7 +7777,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7970,7 +7944,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8014,7 +7988,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8058,7 +8032,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8102,7 +8076,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8146,7 +8120,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8190,7 +8164,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8234,7 +8208,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8319,7 +8293,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8363,7 +8337,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8448,7 +8422,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8574,7 +8548,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8618,7 +8592,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8703,7 +8677,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8747,7 +8721,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8791,7 +8765,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8835,7 +8809,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8879,7 +8853,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8923,7 +8897,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8967,7 +8941,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9011,7 +8985,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9096,7 +9070,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9263,7 +9237,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9307,7 +9281,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9351,7 +9325,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9395,7 +9369,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9480,7 +9454,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9524,7 +9498,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9568,7 +9542,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9612,7 +9586,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9656,7 +9630,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9700,7 +9674,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9744,7 +9718,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9788,7 +9762,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9832,7 +9806,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9876,7 +9850,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9920,7 +9894,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9964,7 +9938,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10008,7 +9982,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10052,7 +10026,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -10096,7 +10070,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10140,7 +10114,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10184,7 +10158,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10228,7 +10202,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10272,7 +10246,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10316,7 +10290,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10360,7 +10334,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10445,7 +10419,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10530,7 +10504,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10545,55 +10519,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10962,7 +10936,7 @@
       <c r="L10" t="s">
         <v>677</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46383</v>
       </c>
       <c r="N10" t="s">
@@ -11006,7 +10980,7 @@
       <c r="L11" t="s">
         <v>677</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46383</v>
       </c>
       <c r="N11" t="s">
@@ -11214,7 +11188,7 @@
       <c r="L16" t="s">
         <v>677</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46383</v>
       </c>
       <c r="N16" t="s">
@@ -11299,7 +11273,7 @@
       <c r="L18" t="s">
         <v>677</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46383</v>
       </c>
       <c r="N18" t="s">
@@ -11343,7 +11317,7 @@
       <c r="L19" t="s">
         <v>680</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46368</v>
       </c>
       <c r="N19" t="s">
@@ -11387,7 +11361,7 @@
       <c r="L20" t="s">
         <v>677</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46383</v>
       </c>
       <c r="N20" t="s">
@@ -11431,7 +11405,7 @@
       <c r="L21" t="s">
         <v>680</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46368</v>
       </c>
       <c r="N21" t="s">
@@ -11598,7 +11572,7 @@
       <c r="L25" t="s">
         <v>680</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46368</v>
       </c>
       <c r="N25" t="s">
@@ -11724,7 +11698,7 @@
       <c r="L28" t="s">
         <v>680</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46368</v>
       </c>
       <c r="N28" t="s">
@@ -11768,7 +11742,7 @@
       <c r="L29" t="s">
         <v>679</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46323</v>
       </c>
       <c r="N29" t="s">
@@ -11812,7 +11786,7 @@
       <c r="L30" t="s">
         <v>680</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46368</v>
       </c>
       <c r="N30" t="s">
@@ -11856,7 +11830,7 @@
       <c r="L31" t="s">
         <v>679</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46323</v>
       </c>
       <c r="N31" t="s">
@@ -12269,7 +12243,7 @@
       <c r="L41" t="s">
         <v>680</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46368</v>
       </c>
       <c r="N41" t="s">
@@ -12354,7 +12328,7 @@
       <c r="L43" t="s">
         <v>680</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46368</v>
       </c>
       <c r="N43" t="s">
@@ -12398,7 +12372,7 @@
       <c r="L44" t="s">
         <v>680</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46368</v>
       </c>
       <c r="N44" t="s">
@@ -12442,7 +12416,7 @@
       <c r="L45" t="s">
         <v>680</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46368</v>
       </c>
       <c r="N45" t="s">
@@ -12568,7 +12542,7 @@
       <c r="L48" t="s">
         <v>680</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46368</v>
       </c>
       <c r="N48" t="s">
@@ -12612,7 +12586,7 @@
       <c r="L49" t="s">
         <v>679</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46323</v>
       </c>
       <c r="N49" t="s">
@@ -12656,7 +12630,7 @@
       <c r="L50" t="s">
         <v>679</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46323</v>
       </c>
       <c r="N50" t="s">
@@ -12700,7 +12674,7 @@
       <c r="L51" t="s">
         <v>680</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46368</v>
       </c>
       <c r="N51" t="s">
@@ -12744,7 +12718,7 @@
       <c r="L52" t="s">
         <v>680</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46368</v>
       </c>
       <c r="N52" t="s">
@@ -12788,7 +12762,7 @@
       <c r="L53" t="s">
         <v>680</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46368</v>
       </c>
       <c r="N53" t="s">
@@ -12832,7 +12806,7 @@
       <c r="L54" t="s">
         <v>680</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46368</v>
       </c>
       <c r="N54" t="s">
@@ -12876,7 +12850,7 @@
       <c r="L55" t="s">
         <v>680</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46368</v>
       </c>
       <c r="N55" t="s">
@@ -12920,7 +12894,7 @@
       <c r="L56" t="s">
         <v>679</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46323</v>
       </c>
       <c r="N56" t="s">
@@ -12964,7 +12938,7 @@
       <c r="L57" t="s">
         <v>679</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46323</v>
       </c>
       <c r="N57" t="s">
@@ -13008,7 +12982,7 @@
       <c r="L58" t="s">
         <v>679</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46323</v>
       </c>
       <c r="N58" t="s">
@@ -13052,7 +13026,7 @@
       <c r="L59" t="s">
         <v>680</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46368</v>
       </c>
       <c r="N59" t="s">
@@ -13096,7 +13070,7 @@
       <c r="L60" t="s">
         <v>679</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46323</v>
       </c>
       <c r="N60" t="s">
@@ -13140,7 +13114,7 @@
       <c r="L61" t="s">
         <v>679</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46323</v>
       </c>
       <c r="N61" t="s">
@@ -13184,7 +13158,7 @@
       <c r="L62" t="s">
         <v>680</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46368</v>
       </c>
       <c r="N62" t="s">
@@ -13228,7 +13202,7 @@
       <c r="L63" t="s">
         <v>680</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46368</v>
       </c>
       <c r="N63" t="s">
@@ -13272,7 +13246,7 @@
       <c r="L64" t="s">
         <v>680</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46368</v>
       </c>
       <c r="N64" t="s">
@@ -13316,7 +13290,7 @@
       <c r="L65" t="s">
         <v>680</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="1">
         <v>46368</v>
       </c>
       <c r="N65" t="s">
@@ -13360,7 +13334,7 @@
       <c r="L66" t="s">
         <v>680</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="1">
         <v>46368</v>
       </c>
       <c r="N66" t="s">
@@ -13404,7 +13378,7 @@
       <c r="L67" t="s">
         <v>680</v>
       </c>
-      <c r="M67" s="2">
+      <c r="M67" s="1">
         <v>46368</v>
       </c>
       <c r="N67" t="s">
@@ -13448,7 +13422,7 @@
       <c r="L68" t="s">
         <v>680</v>
       </c>
-      <c r="M68" s="2">
+      <c r="M68" s="1">
         <v>46368</v>
       </c>
       <c r="N68" t="s">
@@ -13492,7 +13466,7 @@
       <c r="L69" t="s">
         <v>680</v>
       </c>
-      <c r="M69" s="2">
+      <c r="M69" s="1">
         <v>46368</v>
       </c>
       <c r="N69" t="s">
@@ -13536,7 +13510,7 @@
       <c r="L70" t="s">
         <v>680</v>
       </c>
-      <c r="M70" s="2">
+      <c r="M70" s="1">
         <v>46368</v>
       </c>
       <c r="N70" t="s">
@@ -13580,7 +13554,7 @@
       <c r="L71" t="s">
         <v>680</v>
       </c>
-      <c r="M71" s="2">
+      <c r="M71" s="1">
         <v>46368</v>
       </c>
       <c r="N71" t="s">
@@ -13624,7 +13598,7 @@
       <c r="L72" t="s">
         <v>680</v>
       </c>
-      <c r="M72" s="2">
+      <c r="M72" s="1">
         <v>46368</v>
       </c>
       <c r="N72" t="s">
@@ -13668,7 +13642,7 @@
       <c r="L73" t="s">
         <v>677</v>
       </c>
-      <c r="M73" s="2">
+      <c r="M73" s="1">
         <v>46383</v>
       </c>
       <c r="N73" t="s">
@@ -13712,7 +13686,7 @@
       <c r="L74" t="s">
         <v>680</v>
       </c>
-      <c r="M74" s="2">
+      <c r="M74" s="1">
         <v>46368</v>
       </c>
       <c r="N74" t="s">
@@ -13756,7 +13730,7 @@
       <c r="L75" t="s">
         <v>680</v>
       </c>
-      <c r="M75" s="2">
+      <c r="M75" s="1">
         <v>46368</v>
       </c>
       <c r="N75" t="s">
@@ -13841,7 +13815,7 @@
       <c r="L77" t="s">
         <v>677</v>
       </c>
-      <c r="M77" s="2">
+      <c r="M77" s="1">
         <v>46383</v>
       </c>
       <c r="N77" t="s">
@@ -13885,7 +13859,7 @@
       <c r="L78" t="s">
         <v>680</v>
       </c>
-      <c r="M78" s="2">
+      <c r="M78" s="1">
         <v>46368</v>
       </c>
       <c r="N78" t="s">
@@ -13929,7 +13903,7 @@
       <c r="L79" t="s">
         <v>680</v>
       </c>
-      <c r="M79" s="2">
+      <c r="M79" s="1">
         <v>46368</v>
       </c>
       <c r="N79" t="s">
@@ -13973,7 +13947,7 @@
       <c r="L80" t="s">
         <v>677</v>
       </c>
-      <c r="M80" s="2">
+      <c r="M80" s="1">
         <v>46383</v>
       </c>
       <c r="N80" t="s">
@@ -14017,7 +13991,7 @@
       <c r="L81" t="s">
         <v>677</v>
       </c>
-      <c r="M81" s="2">
+      <c r="M81" s="1">
         <v>46383</v>
       </c>
       <c r="N81" t="s">
@@ -14061,7 +14035,7 @@
       <c r="L82" t="s">
         <v>677</v>
       </c>
-      <c r="M82" s="2">
+      <c r="M82" s="1">
         <v>46383</v>
       </c>
       <c r="N82" t="s">
@@ -14105,7 +14079,7 @@
       <c r="L83" t="s">
         <v>677</v>
       </c>
-      <c r="M83" s="2">
+      <c r="M83" s="1">
         <v>46383</v>
       </c>
       <c r="N83" t="s">
@@ -14149,7 +14123,7 @@
       <c r="L84" t="s">
         <v>677</v>
       </c>
-      <c r="M84" s="2">
+      <c r="M84" s="1">
         <v>46383</v>
       </c>
       <c r="N84" t="s">
@@ -14193,7 +14167,7 @@
       <c r="L85" t="s">
         <v>680</v>
       </c>
-      <c r="M85" s="2">
+      <c r="M85" s="1">
         <v>46368</v>
       </c>
       <c r="N85" t="s">
@@ -14237,7 +14211,7 @@
       <c r="L86" t="s">
         <v>680</v>
       </c>
-      <c r="M86" s="2">
+      <c r="M86" s="1">
         <v>46368</v>
       </c>
       <c r="N86" t="s">
@@ -14281,7 +14255,7 @@
       <c r="L87" t="s">
         <v>680</v>
       </c>
-      <c r="M87" s="2">
+      <c r="M87" s="1">
         <v>46368</v>
       </c>
       <c r="N87" t="s">
@@ -14325,7 +14299,7 @@
       <c r="L88" t="s">
         <v>680</v>
       </c>
-      <c r="M88" s="2">
+      <c r="M88" s="1">
         <v>46368</v>
       </c>
       <c r="N88" t="s">
@@ -14369,7 +14343,7 @@
       <c r="L89" t="s">
         <v>680</v>
       </c>
-      <c r="M89" s="2">
+      <c r="M89" s="1">
         <v>46368</v>
       </c>
       <c r="N89" t="s">
@@ -14413,7 +14387,7 @@
       <c r="L90" t="s">
         <v>680</v>
       </c>
-      <c r="M90" s="2">
+      <c r="M90" s="1">
         <v>46368</v>
       </c>
       <c r="N90" t="s">
@@ -14457,7 +14431,7 @@
       <c r="L91" t="s">
         <v>680</v>
       </c>
-      <c r="M91" s="2">
+      <c r="M91" s="1">
         <v>46368</v>
       </c>
       <c r="N91" t="s">
@@ -14501,7 +14475,7 @@
       <c r="L92" t="s">
         <v>680</v>
       </c>
-      <c r="M92" s="2">
+      <c r="M92" s="1">
         <v>46368</v>
       </c>
       <c r="N92" t="s">
@@ -14545,7 +14519,7 @@
       <c r="L93" t="s">
         <v>680</v>
       </c>
-      <c r="M93" s="2">
+      <c r="M93" s="1">
         <v>46368</v>
       </c>
       <c r="N93" t="s">
@@ -14589,7 +14563,7 @@
       <c r="L94" t="s">
         <v>680</v>
       </c>
-      <c r="M94" s="2">
+      <c r="M94" s="1">
         <v>46368</v>
       </c>
       <c r="N94" t="s">
@@ -14633,7 +14607,7 @@
       <c r="L95" t="s">
         <v>680</v>
       </c>
-      <c r="M95" s="2">
+      <c r="M95" s="1">
         <v>46368</v>
       </c>
       <c r="N95" t="s">
@@ -14677,7 +14651,7 @@
       <c r="L96" t="s">
         <v>680</v>
       </c>
-      <c r="M96" s="2">
+      <c r="M96" s="1">
         <v>46368</v>
       </c>
       <c r="N96" t="s">
@@ -14721,7 +14695,7 @@
       <c r="L97" t="s">
         <v>680</v>
       </c>
-      <c r="M97" s="2">
+      <c r="M97" s="1">
         <v>46368</v>
       </c>
       <c r="N97" t="s">
@@ -14765,7 +14739,7 @@
       <c r="L98" t="s">
         <v>680</v>
       </c>
-      <c r="M98" s="2">
+      <c r="M98" s="1">
         <v>46368</v>
       </c>
       <c r="N98" t="s">
@@ -14809,7 +14783,7 @@
       <c r="L99" t="s">
         <v>680</v>
       </c>
-      <c r="M99" s="2">
+      <c r="M99" s="1">
         <v>46368</v>
       </c>
       <c r="N99" t="s">
@@ -14853,7 +14827,7 @@
       <c r="L100" t="s">
         <v>680</v>
       </c>
-      <c r="M100" s="2">
+      <c r="M100" s="1">
         <v>46368</v>
       </c>
       <c r="N100" t="s">
@@ -14897,7 +14871,7 @@
       <c r="L101" t="s">
         <v>680</v>
       </c>
-      <c r="M101" s="2">
+      <c r="M101" s="1">
         <v>46368</v>
       </c>
       <c r="N101" t="s">
@@ -14941,7 +14915,7 @@
       <c r="L102" t="s">
         <v>680</v>
       </c>
-      <c r="M102" s="2">
+      <c r="M102" s="1">
         <v>46368</v>
       </c>
       <c r="N102" t="s">
@@ -14985,7 +14959,7 @@
       <c r="L103" t="s">
         <v>680</v>
       </c>
-      <c r="M103" s="2">
+      <c r="M103" s="1">
         <v>46368</v>
       </c>
       <c r="N103" t="s">
@@ -15029,7 +15003,7 @@
       <c r="L104" t="s">
         <v>680</v>
       </c>
-      <c r="M104" s="2">
+      <c r="M104" s="1">
         <v>46368</v>
       </c>
       <c r="N104" t="s">
@@ -15073,7 +15047,7 @@
       <c r="L105" t="s">
         <v>680</v>
       </c>
-      <c r="M105" s="2">
+      <c r="M105" s="1">
         <v>46368</v>
       </c>
       <c r="N105" t="s">
@@ -15117,7 +15091,7 @@
       <c r="L106" t="s">
         <v>680</v>
       </c>
-      <c r="M106" s="2">
+      <c r="M106" s="1">
         <v>46368</v>
       </c>
       <c r="N106" t="s">
@@ -15161,7 +15135,7 @@
       <c r="L107" t="s">
         <v>680</v>
       </c>
-      <c r="M107" s="2">
+      <c r="M107" s="1">
         <v>46368</v>
       </c>
       <c r="N107" t="s">
@@ -15205,7 +15179,7 @@
       <c r="L108" t="s">
         <v>680</v>
       </c>
-      <c r="M108" s="2">
+      <c r="M108" s="1">
         <v>46368</v>
       </c>
       <c r="N108" t="s">
@@ -15249,7 +15223,7 @@
       <c r="L109" t="s">
         <v>680</v>
       </c>
-      <c r="M109" s="2">
+      <c r="M109" s="1">
         <v>46368</v>
       </c>
       <c r="N109" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (29/09/2026 13:53)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2976" uniqueCount="683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3093" uniqueCount="719">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1424,6 +1424,12 @@
     <t>LST239001U8</t>
   </si>
   <si>
+    <t>LST240003U8</t>
+  </si>
+  <si>
+    <t>LST243001U8</t>
+  </si>
+  <si>
     <t>LST243004U8</t>
   </si>
   <si>
@@ -1559,6 +1565,36 @@
     <t>LST266003U8</t>
   </si>
   <si>
+    <t>LST266005U8</t>
+  </si>
+  <si>
+    <t>LST266006U8</t>
+  </si>
+  <si>
+    <t>LST266007U8</t>
+  </si>
+  <si>
+    <t>LST266008U8</t>
+  </si>
+  <si>
+    <t>LST266009U8</t>
+  </si>
+  <si>
+    <t>LST266010U8</t>
+  </si>
+  <si>
+    <t>LST266011U8</t>
+  </si>
+  <si>
+    <t>LST266012U8</t>
+  </si>
+  <si>
+    <t>LST267005U8</t>
+  </si>
+  <si>
+    <t>LST267011U8</t>
+  </si>
+  <si>
     <t>A-1636-32</t>
   </si>
   <si>
@@ -1721,6 +1757,12 @@
     <t>M81934/2-32C032</t>
   </si>
   <si>
+    <t>2601102-1</t>
+  </si>
+  <si>
+    <t>S3461-76</t>
+  </si>
+  <si>
     <t>3074154-01</t>
   </si>
   <si>
@@ -1823,6 +1865,36 @@
     <t>AT-RL1019</t>
   </si>
   <si>
+    <t>065-0030-00</t>
+  </si>
+  <si>
+    <t>S3100-526</t>
+  </si>
+  <si>
+    <t>2621008-202</t>
+  </si>
+  <si>
+    <t>066-3054-01</t>
+  </si>
+  <si>
+    <t>2606014-2</t>
+  </si>
+  <si>
+    <t>071-1242-06</t>
+  </si>
+  <si>
+    <t>030-18200</t>
+  </si>
+  <si>
+    <t>8210-002</t>
+  </si>
+  <si>
+    <t>060-0017-00</t>
+  </si>
+  <si>
+    <t>2651040-2</t>
+  </si>
+  <si>
     <t>BUSHING</t>
   </si>
   <si>
@@ -1964,6 +2036,12 @@
     <t>CAP</t>
   </si>
   <si>
+    <t>HINGE-ASSY-HOISTING</t>
+  </si>
+  <si>
+    <t>BOLT MPI</t>
+  </si>
+  <si>
     <t>GOVERNOR PROPELLER</t>
   </si>
   <si>
@@ -1979,7 +2057,7 @@
     <t>ROD END</t>
   </si>
   <si>
-    <t>FITTING-WING STRUT LWR</t>
+    <t>FITTING-WING STRUT LWR - Confirmation of the requested PN and condition of the material is required.</t>
   </si>
   <si>
     <t>KIT CAB-33-02</t>
@@ -2045,22 +2123,52 @@
     <t>PLATE - COVER</t>
   </si>
   <si>
+    <t>PLATE,MOUNTING</t>
+  </si>
+  <si>
+    <t>NAV STROBE LIGHT ASSEMBLY LEFT</t>
+  </si>
+  <si>
+    <t>FITTING-WING STRUT UPR</t>
+  </si>
+  <si>
+    <t>INDICATOR RADAR ALTIMETER - TYPE KI250</t>
+  </si>
+  <si>
+    <t>INDICATOR, PROPELLER, RPM</t>
+  </si>
+  <si>
+    <t>SLAVING ACCESS,SPEC</t>
+  </si>
+  <si>
+    <t>MAIN WHEEL BRAKE</t>
+  </si>
+  <si>
+    <t>GOVERNOR,CONSTANT SPEED DRIVE</t>
+  </si>
+  <si>
+    <t>FLIGHT DIR HOR</t>
+  </si>
+  <si>
+    <t>ENGINE MOUNT WELD ASSEMBLY</t>
+  </si>
+  <si>
     <t>Empenho Solicitado</t>
   </si>
   <si>
+    <t>Validada</t>
+  </si>
+  <si>
+    <t>Selecionada em Plano</t>
+  </si>
+  <si>
+    <t>Mapa Gerado</t>
+  </si>
+  <si>
     <t>Análise do Pedido</t>
   </si>
   <si>
-    <t>Selecionada em Plano</t>
-  </si>
-  <si>
     <t>Em Cotação</t>
-  </si>
-  <si>
-    <t>Validada</t>
-  </si>
-  <si>
-    <t>Em Discrepância</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10515,7 +10623,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q109"/>
+  <dimension ref="A1:Q121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -10597,7 +10705,7 @@
         <v>516.34</v>
       </c>
       <c r="I2" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J2" t="s">
         <v>388</v>
@@ -10638,7 +10746,7 @@
         <v>191.04</v>
       </c>
       <c r="I3" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J3" t="s">
         <v>388</v>
@@ -10664,7 +10772,7 @@
         <v>173</v>
       </c>
       <c r="D4" t="s">
-        <v>514</v>
+        <v>526</v>
       </c>
       <c r="E4" t="s">
         <v>297</v>
@@ -10679,7 +10787,7 @@
         <v>314.56</v>
       </c>
       <c r="I4" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J4" t="s">
         <v>388</v>
@@ -10705,10 +10813,10 @@
         <v>173</v>
       </c>
       <c r="D5" t="s">
-        <v>515</v>
+        <v>527</v>
       </c>
       <c r="E5" t="s">
-        <v>602</v>
+        <v>626</v>
       </c>
       <c r="F5">
         <v>7</v>
@@ -10720,7 +10828,7 @@
         <v>1859.13</v>
       </c>
       <c r="I5" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J5" t="s">
         <v>388</v>
@@ -10761,7 +10869,7 @@
         <v>1572.48</v>
       </c>
       <c r="I6" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J6" t="s">
         <v>388</v>
@@ -10802,7 +10910,7 @@
         <v>1148.68</v>
       </c>
       <c r="I7" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J7" t="s">
         <v>388</v>
@@ -10869,7 +10977,7 @@
         <v>173</v>
       </c>
       <c r="D9" t="s">
-        <v>516</v>
+        <v>528</v>
       </c>
       <c r="E9" t="s">
         <v>298</v>
@@ -10884,7 +10992,7 @@
         <v>174</v>
       </c>
       <c r="I9" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J9" t="s">
         <v>388</v>
@@ -10910,10 +11018,10 @@
         <v>173</v>
       </c>
       <c r="D10" t="s">
-        <v>517</v>
+        <v>529</v>
       </c>
       <c r="E10" t="s">
-        <v>603</v>
+        <v>627</v>
       </c>
       <c r="F10">
         <v>4</v>
@@ -10925,22 +11033,22 @@
         <v>588.8</v>
       </c>
       <c r="I10" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="J10" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="K10" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="L10" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="M10" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N10" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10954,7 +11062,7 @@
         <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>518</v>
+        <v>530</v>
       </c>
       <c r="E11" t="s">
         <v>341</v>
@@ -10969,22 +11077,22 @@
         <v>862.6799999999999</v>
       </c>
       <c r="I11" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="J11" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="K11" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="L11" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="M11" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N11" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10998,10 +11106,10 @@
         <v>173</v>
       </c>
       <c r="D12" t="s">
-        <v>519</v>
+        <v>531</v>
       </c>
       <c r="E12" t="s">
-        <v>604</v>
+        <v>628</v>
       </c>
       <c r="F12">
         <v>2</v>
@@ -11054,7 +11162,7 @@
         <v>2292.34</v>
       </c>
       <c r="I13" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J13" t="s">
         <v>387</v>
@@ -11080,10 +11188,10 @@
         <v>173</v>
       </c>
       <c r="D14" t="s">
-        <v>520</v>
+        <v>532</v>
       </c>
       <c r="E14" t="s">
-        <v>605</v>
+        <v>629</v>
       </c>
       <c r="F14">
         <v>21</v>
@@ -11095,7 +11203,7 @@
         <v>10768.59</v>
       </c>
       <c r="I14" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J14" t="s">
         <v>387</v>
@@ -11121,10 +11229,10 @@
         <v>173</v>
       </c>
       <c r="D15" t="s">
-        <v>521</v>
+        <v>533</v>
       </c>
       <c r="E15" t="s">
-        <v>606</v>
+        <v>630</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -11136,7 +11244,7 @@
         <v>11325.54</v>
       </c>
       <c r="I15" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J15" t="s">
         <v>380</v>
@@ -11162,10 +11270,10 @@
         <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>522</v>
+        <v>534</v>
       </c>
       <c r="E16" t="s">
-        <v>607</v>
+        <v>631</v>
       </c>
       <c r="F16">
         <v>3</v>
@@ -11177,22 +11285,22 @@
         <v>140.58</v>
       </c>
       <c r="I16" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="J16" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="K16" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="L16" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="M16" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N16" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -11206,10 +11314,10 @@
         <v>173</v>
       </c>
       <c r="D17" t="s">
-        <v>523</v>
+        <v>535</v>
       </c>
       <c r="E17" t="s">
-        <v>608</v>
+        <v>632</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -11221,7 +11329,7 @@
         <v>1076.62</v>
       </c>
       <c r="I17" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J17" t="s">
         <v>380</v>
@@ -11247,10 +11355,10 @@
         <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>524</v>
+        <v>536</v>
       </c>
       <c r="E18" t="s">
-        <v>609</v>
+        <v>633</v>
       </c>
       <c r="F18">
         <v>2</v>
@@ -11262,22 +11370,22 @@
         <v>672.5599999999999</v>
       </c>
       <c r="I18" t="s">
-        <v>677</v>
+        <v>381</v>
       </c>
       <c r="J18" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="K18" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="L18" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="M18" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N18" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -11291,10 +11399,10 @@
         <v>173</v>
       </c>
       <c r="D19" t="s">
-        <v>525</v>
+        <v>537</v>
       </c>
       <c r="E19" t="s">
-        <v>610</v>
+        <v>634</v>
       </c>
       <c r="F19">
         <v>10</v>
@@ -11306,22 +11414,22 @@
         <v>1323.9</v>
       </c>
       <c r="I19" t="s">
-        <v>678</v>
+        <v>714</v>
       </c>
       <c r="J19" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K19" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L19" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M19" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N19" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11335,10 +11443,10 @@
         <v>173</v>
       </c>
       <c r="D20" t="s">
-        <v>526</v>
+        <v>538</v>
       </c>
       <c r="E20" t="s">
-        <v>611</v>
+        <v>635</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -11350,22 +11458,22 @@
         <v>340.73</v>
       </c>
       <c r="I20" t="s">
-        <v>677</v>
+        <v>714</v>
       </c>
       <c r="J20" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="K20" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="L20" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="M20" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N20" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11379,10 +11487,10 @@
         <v>173</v>
       </c>
       <c r="D21" t="s">
-        <v>527</v>
+        <v>539</v>
       </c>
       <c r="E21" t="s">
-        <v>612</v>
+        <v>636</v>
       </c>
       <c r="F21">
         <v>5</v>
@@ -11397,19 +11505,19 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K21" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L21" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M21" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N21" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11423,10 +11531,10 @@
         <v>173</v>
       </c>
       <c r="D22" t="s">
-        <v>528</v>
+        <v>540</v>
       </c>
       <c r="E22" t="s">
-        <v>613</v>
+        <v>637</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -11438,7 +11546,7 @@
         <v>285.3</v>
       </c>
       <c r="I22" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J22" t="s">
         <v>388</v>
@@ -11464,10 +11572,10 @@
         <v>173</v>
       </c>
       <c r="D23" t="s">
-        <v>529</v>
+        <v>541</v>
       </c>
       <c r="E23" t="s">
-        <v>614</v>
+        <v>638</v>
       </c>
       <c r="F23">
         <v>3</v>
@@ -11479,7 +11587,7 @@
         <v>274.86</v>
       </c>
       <c r="I23" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J23" t="s">
         <v>388</v>
@@ -11505,7 +11613,7 @@
         <v>173</v>
       </c>
       <c r="D24" t="s">
-        <v>530</v>
+        <v>542</v>
       </c>
       <c r="E24" t="s">
         <v>307</v>
@@ -11520,7 +11628,7 @@
         <v>245.6</v>
       </c>
       <c r="I24" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J24" t="s">
         <v>388</v>
@@ -11546,10 +11654,10 @@
         <v>173</v>
       </c>
       <c r="D25" t="s">
-        <v>531</v>
+        <v>543</v>
       </c>
       <c r="E25" t="s">
-        <v>615</v>
+        <v>639</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -11561,22 +11669,22 @@
         <v>21612.9</v>
       </c>
       <c r="I25" t="s">
-        <v>678</v>
+        <v>714</v>
       </c>
       <c r="J25" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K25" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L25" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M25" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N25" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11590,10 +11698,10 @@
         <v>173</v>
       </c>
       <c r="D26" t="s">
-        <v>532</v>
+        <v>544</v>
       </c>
       <c r="E26" t="s">
-        <v>616</v>
+        <v>640</v>
       </c>
       <c r="F26">
         <v>8</v>
@@ -11605,7 +11713,7 @@
         <v>8029.04</v>
       </c>
       <c r="I26" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J26" t="s">
         <v>388</v>
@@ -11631,10 +11739,10 @@
         <v>173</v>
       </c>
       <c r="D27" t="s">
-        <v>533</v>
+        <v>545</v>
       </c>
       <c r="E27" t="s">
-        <v>617</v>
+        <v>641</v>
       </c>
       <c r="F27">
         <v>7</v>
@@ -11646,7 +11754,7 @@
         <v>9269.4</v>
       </c>
       <c r="I27" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J27" t="s">
         <v>380</v>
@@ -11672,10 +11780,10 @@
         <v>173</v>
       </c>
       <c r="D28" t="s">
-        <v>534</v>
+        <v>546</v>
       </c>
       <c r="E28" t="s">
-        <v>618</v>
+        <v>642</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -11690,19 +11798,19 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K28" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L28" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M28" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N28" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11716,10 +11824,10 @@
         <v>173</v>
       </c>
       <c r="D29" t="s">
-        <v>535</v>
+        <v>547</v>
       </c>
       <c r="E29" t="s">
-        <v>619</v>
+        <v>643</v>
       </c>
       <c r="F29">
         <v>20</v>
@@ -11731,22 +11839,22 @@
         <v>24038.4</v>
       </c>
       <c r="I29" t="s">
-        <v>679</v>
+        <v>715</v>
       </c>
       <c r="J29" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="K29" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="L29" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="M29" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N29" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11760,10 +11868,10 @@
         <v>173</v>
       </c>
       <c r="D30" t="s">
-        <v>536</v>
+        <v>548</v>
       </c>
       <c r="E30" t="s">
-        <v>620</v>
+        <v>644</v>
       </c>
       <c r="F30">
         <v>2</v>
@@ -11778,19 +11886,19 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K30" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L30" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M30" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N30" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11804,10 +11912,10 @@
         <v>173</v>
       </c>
       <c r="D31" t="s">
-        <v>537</v>
+        <v>549</v>
       </c>
       <c r="E31" t="s">
-        <v>621</v>
+        <v>645</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -11819,22 +11927,22 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
-        <v>679</v>
+        <v>715</v>
       </c>
       <c r="J31" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="K31" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="L31" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="M31" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N31" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11848,10 +11956,10 @@
         <v>173</v>
       </c>
       <c r="D32" t="s">
-        <v>538</v>
+        <v>550</v>
       </c>
       <c r="E32" t="s">
-        <v>622</v>
+        <v>646</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -11863,7 +11971,7 @@
         <v>15090</v>
       </c>
       <c r="I32" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J32" t="s">
         <v>380</v>
@@ -11889,10 +11997,10 @@
         <v>173</v>
       </c>
       <c r="D33" t="s">
-        <v>539</v>
+        <v>551</v>
       </c>
       <c r="E33" t="s">
-        <v>623</v>
+        <v>647</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -11904,7 +12012,7 @@
         <v>1527.63</v>
       </c>
       <c r="I33" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J33" t="s">
         <v>380</v>
@@ -11930,10 +12038,10 @@
         <v>173</v>
       </c>
       <c r="D34" t="s">
-        <v>540</v>
+        <v>552</v>
       </c>
       <c r="E34" t="s">
-        <v>624</v>
+        <v>648</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -11945,7 +12053,7 @@
         <v>5078.8</v>
       </c>
       <c r="I34" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J34" t="s">
         <v>380</v>
@@ -11971,10 +12079,10 @@
         <v>173</v>
       </c>
       <c r="D35" t="s">
-        <v>541</v>
+        <v>553</v>
       </c>
       <c r="E35" t="s">
-        <v>625</v>
+        <v>649</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -11986,7 +12094,7 @@
         <v>828.12</v>
       </c>
       <c r="I35" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J35" t="s">
         <v>380</v>
@@ -12012,10 +12120,10 @@
         <v>173</v>
       </c>
       <c r="D36" t="s">
-        <v>542</v>
+        <v>554</v>
       </c>
       <c r="E36" t="s">
-        <v>626</v>
+        <v>650</v>
       </c>
       <c r="F36">
         <v>36</v>
@@ -12027,7 +12135,7 @@
         <v>4016.16</v>
       </c>
       <c r="I36" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J36" t="s">
         <v>380</v>
@@ -12053,10 +12161,10 @@
         <v>173</v>
       </c>
       <c r="D37" t="s">
-        <v>543</v>
+        <v>555</v>
       </c>
       <c r="E37" t="s">
-        <v>627</v>
+        <v>651</v>
       </c>
       <c r="F37">
         <v>2</v>
@@ -12068,7 +12176,7 @@
         <v>2270.92</v>
       </c>
       <c r="I37" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J37" t="s">
         <v>380</v>
@@ -12094,10 +12202,10 @@
         <v>173</v>
       </c>
       <c r="D38" t="s">
-        <v>544</v>
+        <v>556</v>
       </c>
       <c r="E38" t="s">
-        <v>628</v>
+        <v>652</v>
       </c>
       <c r="F38">
         <v>5</v>
@@ -12109,7 +12217,7 @@
         <v>3100.05</v>
       </c>
       <c r="I38" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J38" t="s">
         <v>380</v>
@@ -12135,10 +12243,10 @@
         <v>173</v>
       </c>
       <c r="D39" t="s">
-        <v>545</v>
+        <v>557</v>
       </c>
       <c r="E39" t="s">
-        <v>629</v>
+        <v>653</v>
       </c>
       <c r="F39">
         <v>4</v>
@@ -12176,10 +12284,10 @@
         <v>173</v>
       </c>
       <c r="D40" t="s">
-        <v>546</v>
+        <v>558</v>
       </c>
       <c r="E40" t="s">
-        <v>630</v>
+        <v>654</v>
       </c>
       <c r="F40">
         <v>2</v>
@@ -12191,7 +12299,7 @@
         <v>15180.86</v>
       </c>
       <c r="I40" t="s">
-        <v>380</v>
+        <v>712</v>
       </c>
       <c r="J40" t="s">
         <v>380</v>
@@ -12217,10 +12325,10 @@
         <v>173</v>
       </c>
       <c r="D41" t="s">
-        <v>547</v>
+        <v>559</v>
       </c>
       <c r="E41" t="s">
-        <v>631</v>
+        <v>655</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -12235,19 +12343,19 @@
         <v>382</v>
       </c>
       <c r="J41" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K41" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L41" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M41" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N41" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -12276,7 +12384,7 @@
         <v>210381.85</v>
       </c>
       <c r="I42" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J42" t="s">
         <v>380</v>
@@ -12302,10 +12410,10 @@
         <v>173</v>
       </c>
       <c r="D43" t="s">
-        <v>548</v>
+        <v>560</v>
       </c>
       <c r="E43" t="s">
-        <v>632</v>
+        <v>656</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -12317,22 +12425,22 @@
         <v>7890.58</v>
       </c>
       <c r="I43" t="s">
-        <v>678</v>
+        <v>714</v>
       </c>
       <c r="J43" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K43" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L43" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M43" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N43" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12346,7 +12454,7 @@
         <v>173</v>
       </c>
       <c r="D44" t="s">
-        <v>549</v>
+        <v>561</v>
       </c>
       <c r="E44" t="s">
         <v>296</v>
@@ -12361,22 +12469,22 @@
         <v>352.52</v>
       </c>
       <c r="I44" t="s">
-        <v>678</v>
+        <v>714</v>
       </c>
       <c r="J44" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K44" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L44" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M44" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N44" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12390,10 +12498,10 @@
         <v>173</v>
       </c>
       <c r="D45" t="s">
-        <v>550</v>
+        <v>562</v>
       </c>
       <c r="E45" t="s">
-        <v>633</v>
+        <v>657</v>
       </c>
       <c r="F45">
         <v>2</v>
@@ -12405,22 +12513,22 @@
         <v>376.62</v>
       </c>
       <c r="I45" t="s">
-        <v>678</v>
+        <v>714</v>
       </c>
       <c r="J45" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K45" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L45" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M45" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N45" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12434,10 +12542,10 @@
         <v>173</v>
       </c>
       <c r="D46" t="s">
-        <v>551</v>
+        <v>563</v>
       </c>
       <c r="E46" t="s">
-        <v>634</v>
+        <v>658</v>
       </c>
       <c r="F46">
         <v>2</v>
@@ -12449,7 +12557,7 @@
         <v>1721.52</v>
       </c>
       <c r="I46" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J46" t="s">
         <v>380</v>
@@ -12475,10 +12583,10 @@
         <v>173</v>
       </c>
       <c r="D47" t="s">
-        <v>552</v>
+        <v>564</v>
       </c>
       <c r="E47" t="s">
-        <v>635</v>
+        <v>659</v>
       </c>
       <c r="F47">
         <v>2</v>
@@ -12490,7 +12598,7 @@
         <v>2577.94</v>
       </c>
       <c r="I47" t="s">
-        <v>676</v>
+        <v>712</v>
       </c>
       <c r="J47" t="s">
         <v>380</v>
@@ -12516,10 +12624,10 @@
         <v>173</v>
       </c>
       <c r="D48" t="s">
-        <v>553</v>
+        <v>565</v>
       </c>
       <c r="E48" t="s">
-        <v>635</v>
+        <v>659</v>
       </c>
       <c r="F48">
         <v>2</v>
@@ -12531,22 +12639,22 @@
         <v>3459.72</v>
       </c>
       <c r="I48" t="s">
-        <v>678</v>
+        <v>714</v>
       </c>
       <c r="J48" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K48" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L48" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M48" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N48" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12560,10 +12668,10 @@
         <v>173</v>
       </c>
       <c r="D49" t="s">
-        <v>554</v>
+        <v>566</v>
       </c>
       <c r="E49" t="s">
-        <v>636</v>
+        <v>660</v>
       </c>
       <c r="F49">
         <v>9</v>
@@ -12575,22 +12683,22 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
-        <v>679</v>
+        <v>715</v>
       </c>
       <c r="J49" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="K49" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="L49" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="M49" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N49" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12604,10 +12712,10 @@
         <v>173</v>
       </c>
       <c r="D50" t="s">
-        <v>555</v>
+        <v>567</v>
       </c>
       <c r="E50" t="s">
-        <v>637</v>
+        <v>661</v>
       </c>
       <c r="F50">
         <v>1</v>
@@ -12619,22 +12727,22 @@
         <v>4208.01</v>
       </c>
       <c r="I50" t="s">
-        <v>679</v>
+        <v>715</v>
       </c>
       <c r="J50" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="K50" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="L50" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="M50" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N50" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12648,10 +12756,10 @@
         <v>173</v>
       </c>
       <c r="D51" t="s">
-        <v>556</v>
+        <v>568</v>
       </c>
       <c r="E51" t="s">
-        <v>638</v>
+        <v>662</v>
       </c>
       <c r="F51">
         <v>4</v>
@@ -12666,19 +12774,19 @@
         <v>382</v>
       </c>
       <c r="J51" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K51" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L51" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M51" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N51" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12692,10 +12800,10 @@
         <v>173</v>
       </c>
       <c r="D52" t="s">
-        <v>557</v>
+        <v>569</v>
       </c>
       <c r="E52" t="s">
-        <v>639</v>
+        <v>663</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -12710,19 +12818,19 @@
         <v>382</v>
       </c>
       <c r="J52" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K52" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L52" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M52" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N52" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12736,10 +12844,10 @@
         <v>173</v>
       </c>
       <c r="D53" t="s">
-        <v>558</v>
+        <v>570</v>
       </c>
       <c r="E53" t="s">
-        <v>640</v>
+        <v>664</v>
       </c>
       <c r="F53">
         <v>2</v>
@@ -12754,19 +12862,19 @@
         <v>382</v>
       </c>
       <c r="J53" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K53" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L53" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M53" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N53" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12780,10 +12888,10 @@
         <v>173</v>
       </c>
       <c r="D54" t="s">
-        <v>559</v>
+        <v>571</v>
       </c>
       <c r="E54" t="s">
-        <v>641</v>
+        <v>665</v>
       </c>
       <c r="F54">
         <v>4</v>
@@ -12795,22 +12903,22 @@
         <v>3875.24</v>
       </c>
       <c r="I54" t="s">
-        <v>678</v>
+        <v>714</v>
       </c>
       <c r="J54" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K54" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L54" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M54" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N54" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12824,37 +12932,37 @@
         <v>173</v>
       </c>
       <c r="D55" t="s">
-        <v>560</v>
+        <v>572</v>
       </c>
       <c r="E55" t="s">
-        <v>642</v>
+        <v>666</v>
       </c>
       <c r="F55">
         <v>1</v>
       </c>
       <c r="G55">
-        <v>78000</v>
+        <v>84382.42999999999</v>
       </c>
       <c r="H55">
-        <v>78000</v>
+        <v>84382.42999999999</v>
       </c>
       <c r="I55" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J55" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K55" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L55" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M55" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N55" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -12868,10 +12976,10 @@
         <v>173</v>
       </c>
       <c r="D56" t="s">
-        <v>561</v>
+        <v>573</v>
       </c>
       <c r="E56" t="s">
-        <v>643</v>
+        <v>667</v>
       </c>
       <c r="F56">
         <v>1</v>
@@ -12883,22 +12991,22 @@
         <v>3576.55</v>
       </c>
       <c r="I56" t="s">
-        <v>679</v>
+        <v>715</v>
       </c>
       <c r="J56" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="K56" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="L56" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="M56" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N56" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -12912,10 +13020,10 @@
         <v>173</v>
       </c>
       <c r="D57" t="s">
-        <v>562</v>
+        <v>574</v>
       </c>
       <c r="E57" t="s">
-        <v>644</v>
+        <v>668</v>
       </c>
       <c r="F57">
         <v>1</v>
@@ -12927,22 +13035,22 @@
         <v>908.11</v>
       </c>
       <c r="I57" t="s">
-        <v>679</v>
+        <v>715</v>
       </c>
       <c r="J57" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="K57" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="L57" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="M57" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N57" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -12956,10 +13064,10 @@
         <v>173</v>
       </c>
       <c r="D58" t="s">
-        <v>563</v>
+        <v>575</v>
       </c>
       <c r="E58" t="s">
-        <v>645</v>
+        <v>669</v>
       </c>
       <c r="F58">
         <v>4</v>
@@ -12971,22 +13079,22 @@
         <v>1500.8</v>
       </c>
       <c r="I58" t="s">
-        <v>679</v>
+        <v>715</v>
       </c>
       <c r="J58" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="K58" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="L58" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="M58" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N58" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -13015,22 +13123,22 @@
         <v>869.98</v>
       </c>
       <c r="I59" t="s">
-        <v>678</v>
+        <v>714</v>
       </c>
       <c r="J59" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K59" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L59" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M59" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N59" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -13044,10 +13152,10 @@
         <v>173</v>
       </c>
       <c r="D60" t="s">
-        <v>564</v>
+        <v>576</v>
       </c>
       <c r="E60" t="s">
-        <v>646</v>
+        <v>670</v>
       </c>
       <c r="F60">
         <v>3</v>
@@ -13059,22 +13167,22 @@
         <v>1379.52</v>
       </c>
       <c r="I60" t="s">
-        <v>679</v>
+        <v>715</v>
       </c>
       <c r="J60" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="K60" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="L60" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="M60" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N60" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="61" spans="1:14">
@@ -13088,10 +13196,10 @@
         <v>173</v>
       </c>
       <c r="D61" t="s">
-        <v>565</v>
+        <v>577</v>
       </c>
       <c r="E61" t="s">
-        <v>647</v>
+        <v>671</v>
       </c>
       <c r="F61">
         <v>5</v>
@@ -13103,22 +13211,22 @@
         <v>5645.05</v>
       </c>
       <c r="I61" t="s">
-        <v>679</v>
+        <v>715</v>
       </c>
       <c r="J61" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="K61" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="L61" t="s">
-        <v>679</v>
+        <v>717</v>
       </c>
       <c r="M61" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N61" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="62" spans="1:14">
@@ -13132,10 +13240,10 @@
         <v>173</v>
       </c>
       <c r="D62" t="s">
-        <v>566</v>
+        <v>578</v>
       </c>
       <c r="E62" t="s">
-        <v>648</v>
+        <v>672</v>
       </c>
       <c r="F62">
         <v>21</v>
@@ -13147,22 +13255,22 @@
         <v>204.96</v>
       </c>
       <c r="I62" t="s">
-        <v>680</v>
+        <v>714</v>
       </c>
       <c r="J62" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K62" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L62" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M62" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N62" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="63" spans="1:14">
@@ -13191,22 +13299,22 @@
         <v>421</v>
       </c>
       <c r="I63" t="s">
-        <v>680</v>
+        <v>714</v>
       </c>
       <c r="J63" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K63" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L63" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M63" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N63" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="64" spans="1:14">
@@ -13220,7 +13328,7 @@
         <v>173</v>
       </c>
       <c r="D64" t="s">
-        <v>567</v>
+        <v>579</v>
       </c>
       <c r="E64" t="s">
         <v>308</v>
@@ -13235,22 +13343,22 @@
         <v>1999.52</v>
       </c>
       <c r="I64" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="J64" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K64" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L64" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M64" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N64" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="65" spans="1:14">
@@ -13264,37 +13372,37 @@
         <v>173</v>
       </c>
       <c r="D65" t="s">
-        <v>568</v>
+        <v>580</v>
       </c>
       <c r="E65" t="s">
-        <v>649</v>
+        <v>673</v>
       </c>
       <c r="F65">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G65">
-        <v>27326.55</v>
+        <v>4424.23</v>
       </c>
       <c r="H65">
-        <v>27326.55</v>
+        <v>8848.459999999999</v>
       </c>
       <c r="I65" t="s">
-        <v>680</v>
+        <v>714</v>
       </c>
       <c r="J65" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K65" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L65" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M65" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N65" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="66" spans="1:14">
@@ -13308,37 +13416,37 @@
         <v>173</v>
       </c>
       <c r="D66" t="s">
-        <v>569</v>
+        <v>581</v>
       </c>
       <c r="E66" t="s">
-        <v>298</v>
+        <v>674</v>
       </c>
       <c r="F66">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G66">
-        <v>50.39</v>
+        <v>148.96</v>
       </c>
       <c r="H66">
-        <v>806.24</v>
+        <v>297.92</v>
       </c>
       <c r="I66" t="s">
-        <v>680</v>
+        <v>714</v>
       </c>
       <c r="J66" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K66" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L66" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M66" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N66" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="67" spans="1:14">
@@ -13352,37 +13460,37 @@
         <v>173</v>
       </c>
       <c r="D67" t="s">
-        <v>570</v>
+        <v>582</v>
       </c>
       <c r="E67" t="s">
-        <v>650</v>
+        <v>675</v>
       </c>
       <c r="F67">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G67">
-        <v>1390.6</v>
+        <v>27326.55</v>
       </c>
       <c r="H67">
-        <v>11124.8</v>
+        <v>27326.55</v>
       </c>
       <c r="I67" t="s">
-        <v>678</v>
+        <v>714</v>
       </c>
       <c r="J67" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K67" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L67" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M67" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N67" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="68" spans="1:14">
@@ -13396,37 +13504,37 @@
         <v>173</v>
       </c>
       <c r="D68" t="s">
-        <v>212</v>
+        <v>583</v>
       </c>
       <c r="E68" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="F68">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="G68">
-        <v>63.78</v>
+        <v>50.39</v>
       </c>
       <c r="H68">
-        <v>1658.28</v>
+        <v>806.24</v>
       </c>
       <c r="I68" t="s">
-        <v>678</v>
+        <v>714</v>
       </c>
       <c r="J68" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K68" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L68" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M68" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N68" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="69" spans="1:14">
@@ -13440,37 +13548,37 @@
         <v>173</v>
       </c>
       <c r="D69" t="s">
-        <v>286</v>
+        <v>584</v>
       </c>
       <c r="E69" t="s">
-        <v>378</v>
+        <v>676</v>
       </c>
       <c r="F69">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G69">
-        <v>1984.24</v>
+        <v>1390.6</v>
       </c>
       <c r="H69">
-        <v>3968.48</v>
+        <v>11124.8</v>
       </c>
       <c r="I69" t="s">
-        <v>680</v>
+        <v>714</v>
       </c>
       <c r="J69" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K69" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L69" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M69" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N69" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="70" spans="1:14">
@@ -13484,37 +13592,37 @@
         <v>173</v>
       </c>
       <c r="D70" t="s">
-        <v>571</v>
+        <v>212</v>
       </c>
       <c r="E70" t="s">
-        <v>294</v>
+        <v>305</v>
       </c>
       <c r="F70">
-        <v>100</v>
+        <v>26</v>
       </c>
       <c r="G70">
-        <v>4</v>
+        <v>63.78</v>
       </c>
       <c r="H70">
-        <v>400</v>
+        <v>1658.28</v>
       </c>
       <c r="I70" t="s">
-        <v>680</v>
+        <v>714</v>
       </c>
       <c r="J70" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K70" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L70" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M70" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N70" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="71" spans="1:14">
@@ -13528,37 +13636,37 @@
         <v>173</v>
       </c>
       <c r="D71" t="s">
-        <v>572</v>
+        <v>286</v>
       </c>
       <c r="E71" t="s">
-        <v>651</v>
+        <v>378</v>
       </c>
       <c r="F71">
         <v>2</v>
       </c>
       <c r="G71">
-        <v>1521.88</v>
+        <v>1984.24</v>
       </c>
       <c r="H71">
-        <v>3043.76</v>
+        <v>3968.48</v>
       </c>
       <c r="I71" t="s">
-        <v>680</v>
+        <v>714</v>
       </c>
       <c r="J71" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K71" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L71" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M71" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N71" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="72" spans="1:14">
@@ -13572,37 +13680,37 @@
         <v>173</v>
       </c>
       <c r="D72" t="s">
-        <v>573</v>
+        <v>585</v>
       </c>
       <c r="E72" t="s">
-        <v>652</v>
+        <v>294</v>
       </c>
       <c r="F72">
+        <v>100</v>
+      </c>
+      <c r="G72">
         <v>4</v>
       </c>
-      <c r="G72">
-        <v>512.08</v>
-      </c>
       <c r="H72">
-        <v>2048.32</v>
+        <v>400</v>
       </c>
       <c r="I72" t="s">
-        <v>680</v>
+        <v>714</v>
       </c>
       <c r="J72" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K72" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L72" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M72" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N72" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="73" spans="1:14">
@@ -13616,37 +13724,37 @@
         <v>173</v>
       </c>
       <c r="D73" t="s">
-        <v>574</v>
+        <v>586</v>
       </c>
       <c r="E73" t="s">
-        <v>653</v>
+        <v>677</v>
       </c>
       <c r="F73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G73">
-        <v>916.62</v>
+        <v>1521.88</v>
       </c>
       <c r="H73">
-        <v>916.62</v>
+        <v>3043.76</v>
       </c>
       <c r="I73" t="s">
-        <v>677</v>
+        <v>714</v>
       </c>
       <c r="J73" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="K73" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="L73" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="M73" s="1">
-        <v>46383</v>
+        <v>46369</v>
       </c>
       <c r="N73" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="74" spans="1:14">
@@ -13660,37 +13768,37 @@
         <v>173</v>
       </c>
       <c r="D74" t="s">
-        <v>268</v>
+        <v>587</v>
       </c>
       <c r="E74" t="s">
-        <v>364</v>
+        <v>678</v>
       </c>
       <c r="F74">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G74">
-        <v>41118.26</v>
+        <v>512.08</v>
       </c>
       <c r="H74">
-        <v>205591.3</v>
+        <v>2048.32</v>
       </c>
       <c r="I74" t="s">
-        <v>382</v>
+        <v>714</v>
       </c>
       <c r="J74" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K74" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L74" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M74" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N74" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="75" spans="1:14">
@@ -13704,37 +13812,37 @@
         <v>173</v>
       </c>
       <c r="D75" t="s">
-        <v>575</v>
+        <v>588</v>
       </c>
       <c r="E75" t="s">
-        <v>654</v>
+        <v>679</v>
       </c>
       <c r="F75">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G75">
-        <v>2197.5</v>
+        <v>1001.2</v>
       </c>
       <c r="H75">
-        <v>6592.5</v>
+        <v>1001.2</v>
       </c>
       <c r="I75" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="J75" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K75" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L75" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M75" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N75" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="76" spans="1:14">
@@ -13748,34 +13856,34 @@
         <v>173</v>
       </c>
       <c r="D76" t="s">
-        <v>523</v>
+        <v>268</v>
       </c>
       <c r="E76" t="s">
-        <v>608</v>
+        <v>364</v>
       </c>
       <c r="F76">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G76">
-        <v>567.61</v>
+        <v>39255.96</v>
       </c>
       <c r="H76">
-        <v>4540.88</v>
+        <v>196279.8</v>
       </c>
       <c r="I76" t="s">
-        <v>681</v>
-      </c>
-      <c r="J76" t="s">
-        <v>681</v>
+        <v>716</v>
       </c>
       <c r="K76" t="s">
-        <v>681</v>
+        <v>716</v>
       </c>
       <c r="L76" t="s">
-        <v>681</v>
+        <v>716</v>
+      </c>
+      <c r="M76" s="1">
+        <v>46384</v>
       </c>
       <c r="N76" t="s">
-        <v>395</v>
+        <v>718</v>
       </c>
     </row>
     <row r="77" spans="1:14">
@@ -13789,37 +13897,34 @@
         <v>173</v>
       </c>
       <c r="D77" t="s">
-        <v>278</v>
+        <v>589</v>
       </c>
       <c r="E77" t="s">
-        <v>305</v>
+        <v>680</v>
       </c>
       <c r="F77">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="G77">
-        <v>121</v>
+        <v>2197.5</v>
       </c>
       <c r="H77">
-        <v>2057</v>
+        <v>6592.5</v>
       </c>
       <c r="I77" t="s">
-        <v>677</v>
-      </c>
-      <c r="J77" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="K77" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="L77" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="M77" s="1">
-        <v>46383</v>
+        <v>46369</v>
       </c>
       <c r="N77" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="78" spans="1:14">
@@ -13833,37 +13938,37 @@
         <v>173</v>
       </c>
       <c r="D78" t="s">
-        <v>576</v>
+        <v>535</v>
       </c>
       <c r="E78" t="s">
-        <v>655</v>
+        <v>632</v>
       </c>
       <c r="F78">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G78">
-        <v>4972.78</v>
+        <v>580.22</v>
       </c>
       <c r="H78">
-        <v>9945.559999999999</v>
+        <v>4641.76</v>
       </c>
       <c r="I78" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="J78" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K78" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L78" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M78" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N78" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="79" spans="1:14">
@@ -13877,37 +13982,37 @@
         <v>173</v>
       </c>
       <c r="D79" t="s">
-        <v>177</v>
+        <v>278</v>
       </c>
       <c r="E79" t="s">
-        <v>291</v>
+        <v>305</v>
       </c>
       <c r="F79">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="G79">
-        <v>265.47</v>
+        <v>121</v>
       </c>
       <c r="H79">
-        <v>1592.82</v>
+        <v>2057</v>
       </c>
       <c r="I79" t="s">
-        <v>382</v>
+        <v>713</v>
       </c>
       <c r="J79" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K79" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L79" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M79" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N79" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="80" spans="1:14">
@@ -13921,37 +14026,37 @@
         <v>173</v>
       </c>
       <c r="D80" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="E80" t="s">
-        <v>656</v>
+        <v>681</v>
       </c>
       <c r="F80">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G80">
-        <v>359.34</v>
+        <v>4972.78</v>
       </c>
       <c r="H80">
-        <v>1437.36</v>
+        <v>9945.559999999999</v>
       </c>
       <c r="I80" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="J80" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="K80" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="L80" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="M80" s="1">
-        <v>46383</v>
+        <v>46369</v>
       </c>
       <c r="N80" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="81" spans="1:14">
@@ -13965,37 +14070,37 @@
         <v>173</v>
       </c>
       <c r="D81" t="s">
-        <v>578</v>
+        <v>177</v>
       </c>
       <c r="E81" t="s">
-        <v>657</v>
+        <v>291</v>
       </c>
       <c r="F81">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G81">
-        <v>2822.4</v>
+        <v>265.47</v>
       </c>
       <c r="H81">
-        <v>2822.4</v>
+        <v>1592.82</v>
       </c>
       <c r="I81" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="J81" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="K81" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="L81" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="M81" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N81" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="82" spans="1:14">
@@ -14009,37 +14114,37 @@
         <v>173</v>
       </c>
       <c r="D82" t="s">
-        <v>579</v>
+        <v>591</v>
       </c>
       <c r="E82" t="s">
-        <v>658</v>
+        <v>682</v>
       </c>
       <c r="F82">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G82">
-        <v>2865.92</v>
+        <v>359.34</v>
       </c>
       <c r="H82">
-        <v>20061.44</v>
+        <v>1437.36</v>
       </c>
       <c r="I82" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="J82" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="K82" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="L82" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="M82" s="1">
-        <v>46383</v>
+        <v>46369</v>
       </c>
       <c r="N82" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="83" spans="1:14">
@@ -14053,37 +14158,37 @@
         <v>173</v>
       </c>
       <c r="D83" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="E83" t="s">
-        <v>659</v>
+        <v>683</v>
       </c>
       <c r="F83">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G83">
-        <v>3000.85</v>
+        <v>2822.4</v>
       </c>
       <c r="H83">
-        <v>21005.95</v>
+        <v>2822.4</v>
       </c>
       <c r="I83" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="J83" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="K83" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="L83" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="M83" s="1">
-        <v>46383</v>
+        <v>46369</v>
       </c>
       <c r="N83" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="84" spans="1:14">
@@ -14097,37 +14202,37 @@
         <v>173</v>
       </c>
       <c r="D84" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="E84" t="s">
-        <v>660</v>
+        <v>684</v>
       </c>
       <c r="F84">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G84">
-        <v>3409.92</v>
+        <v>2865.92</v>
       </c>
       <c r="H84">
-        <v>13639.68</v>
+        <v>20061.44</v>
       </c>
       <c r="I84" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="J84" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="K84" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="L84" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="M84" s="1">
-        <v>46383</v>
+        <v>46369</v>
       </c>
       <c r="N84" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="85" spans="1:14">
@@ -14141,37 +14246,37 @@
         <v>173</v>
       </c>
       <c r="D85" t="s">
-        <v>582</v>
+        <v>594</v>
       </c>
       <c r="E85" t="s">
-        <v>308</v>
+        <v>685</v>
       </c>
       <c r="F85">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G85">
-        <v>55.58</v>
+        <v>3000.85</v>
       </c>
       <c r="H85">
-        <v>500.22</v>
+        <v>21005.95</v>
       </c>
       <c r="I85" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="J85" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K85" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L85" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M85" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N85" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="86" spans="1:14">
@@ -14185,37 +14290,37 @@
         <v>173</v>
       </c>
       <c r="D86" t="s">
-        <v>220</v>
+        <v>595</v>
       </c>
       <c r="E86" t="s">
-        <v>325</v>
+        <v>686</v>
       </c>
       <c r="F86">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="G86">
-        <v>47.2</v>
+        <v>3409.92</v>
       </c>
       <c r="H86">
-        <v>2360</v>
+        <v>13639.68</v>
       </c>
       <c r="I86" t="s">
-        <v>382</v>
+        <v>713</v>
       </c>
       <c r="J86" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K86" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L86" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M86" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N86" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="87" spans="1:14">
@@ -14229,37 +14334,37 @@
         <v>173</v>
       </c>
       <c r="D87" t="s">
-        <v>583</v>
+        <v>596</v>
       </c>
       <c r="E87" t="s">
-        <v>661</v>
+        <v>308</v>
       </c>
       <c r="F87">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G87">
-        <v>424.32</v>
+        <v>55.58</v>
       </c>
       <c r="H87">
-        <v>3394.56</v>
+        <v>500.22</v>
       </c>
       <c r="I87" t="s">
-        <v>677</v>
+        <v>713</v>
       </c>
       <c r="J87" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K87" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L87" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M87" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N87" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="88" spans="1:14">
@@ -14273,37 +14378,37 @@
         <v>173</v>
       </c>
       <c r="D88" t="s">
-        <v>584</v>
+        <v>220</v>
       </c>
       <c r="E88" t="s">
-        <v>311</v>
+        <v>325</v>
       </c>
       <c r="F88">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G88">
-        <v>2.7</v>
+        <v>47.2</v>
       </c>
       <c r="H88">
-        <v>270</v>
+        <v>2360</v>
       </c>
       <c r="I88" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J88" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K88" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L88" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M88" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N88" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="89" spans="1:14">
@@ -14317,37 +14422,37 @@
         <v>173</v>
       </c>
       <c r="D89" t="s">
-        <v>258</v>
+        <v>597</v>
       </c>
       <c r="E89" t="s">
-        <v>356</v>
+        <v>687</v>
       </c>
       <c r="F89">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="G89">
-        <v>7.61</v>
+        <v>424.32</v>
       </c>
       <c r="H89">
-        <v>761</v>
+        <v>3394.56</v>
       </c>
       <c r="I89" t="s">
-        <v>382</v>
+        <v>713</v>
       </c>
       <c r="J89" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K89" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L89" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M89" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N89" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="90" spans="1:14">
@@ -14361,37 +14466,37 @@
         <v>173</v>
       </c>
       <c r="D90" t="s">
-        <v>585</v>
+        <v>598</v>
       </c>
       <c r="E90" t="s">
-        <v>662</v>
+        <v>311</v>
       </c>
       <c r="F90">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="G90">
-        <v>130.19</v>
+        <v>2.65</v>
       </c>
       <c r="H90">
-        <v>520.76</v>
+        <v>265</v>
       </c>
       <c r="I90" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J90" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K90" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L90" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M90" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N90" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="91" spans="1:14">
@@ -14405,37 +14510,37 @@
         <v>173</v>
       </c>
       <c r="D91" t="s">
-        <v>586</v>
+        <v>258</v>
       </c>
       <c r="E91" t="s">
-        <v>663</v>
+        <v>356</v>
       </c>
       <c r="F91">
-        <v>11</v>
+        <v>100</v>
       </c>
       <c r="G91">
-        <v>70.08</v>
+        <v>7.94</v>
       </c>
       <c r="H91">
-        <v>770.88</v>
+        <v>794</v>
       </c>
       <c r="I91" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J91" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K91" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L91" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M91" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N91" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="92" spans="1:14">
@@ -14449,37 +14554,37 @@
         <v>173</v>
       </c>
       <c r="D92" t="s">
-        <v>587</v>
+        <v>599</v>
       </c>
       <c r="E92" t="s">
-        <v>664</v>
+        <v>688</v>
       </c>
       <c r="F92">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G92">
-        <v>7431.24</v>
+        <v>138.07</v>
       </c>
       <c r="H92">
-        <v>7431.24</v>
+        <v>552.28</v>
       </c>
       <c r="I92" t="s">
-        <v>382</v>
+        <v>713</v>
       </c>
       <c r="J92" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K92" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L92" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M92" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N92" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="93" spans="1:14">
@@ -14493,37 +14598,37 @@
         <v>173</v>
       </c>
       <c r="D93" t="s">
-        <v>588</v>
+        <v>600</v>
       </c>
       <c r="E93" t="s">
-        <v>665</v>
+        <v>689</v>
       </c>
       <c r="F93">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G93">
-        <v>9782.57</v>
+        <v>66.89</v>
       </c>
       <c r="H93">
-        <v>48912.85</v>
+        <v>735.79</v>
       </c>
       <c r="I93" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J93" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K93" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L93" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M93" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N93" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="94" spans="1:14">
@@ -14537,37 +14642,37 @@
         <v>173</v>
       </c>
       <c r="D94" t="s">
-        <v>589</v>
+        <v>601</v>
       </c>
       <c r="E94" t="s">
-        <v>666</v>
+        <v>690</v>
       </c>
       <c r="F94">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G94">
-        <v>811.5599999999999</v>
+        <v>7431.24</v>
       </c>
       <c r="H94">
-        <v>8115.6</v>
+        <v>7431.24</v>
       </c>
       <c r="I94" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J94" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K94" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L94" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M94" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N94" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="95" spans="1:14">
@@ -14581,37 +14686,37 @@
         <v>173</v>
       </c>
       <c r="D95" t="s">
-        <v>590</v>
+        <v>602</v>
       </c>
       <c r="E95" t="s">
-        <v>667</v>
+        <v>691</v>
       </c>
       <c r="F95">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G95">
-        <v>15390.97</v>
+        <v>9249.639999999999</v>
       </c>
       <c r="H95">
-        <v>30781.94</v>
+        <v>46248.2</v>
       </c>
       <c r="I95" t="s">
-        <v>677</v>
+        <v>716</v>
       </c>
       <c r="J95" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K95" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L95" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M95" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N95" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="96" spans="1:14">
@@ -14625,37 +14730,37 @@
         <v>173</v>
       </c>
       <c r="D96" t="s">
-        <v>591</v>
+        <v>603</v>
       </c>
       <c r="E96" t="s">
-        <v>612</v>
+        <v>692</v>
       </c>
       <c r="F96">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G96">
-        <v>171.76</v>
+        <v>811.5599999999999</v>
       </c>
       <c r="H96">
-        <v>343.52</v>
+        <v>8115.6</v>
       </c>
       <c r="I96" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J96" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K96" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L96" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M96" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N96" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="97" spans="1:14">
@@ -14669,37 +14774,37 @@
         <v>173</v>
       </c>
       <c r="D97" t="s">
-        <v>592</v>
+        <v>604</v>
       </c>
       <c r="E97" t="s">
-        <v>342</v>
+        <v>693</v>
       </c>
       <c r="F97">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="G97">
-        <v>7.03</v>
+        <v>15390.97</v>
       </c>
       <c r="H97">
-        <v>224.96</v>
+        <v>30781.94</v>
       </c>
       <c r="I97" t="s">
-        <v>382</v>
+        <v>713</v>
       </c>
       <c r="J97" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K97" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L97" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M97" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N97" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="98" spans="1:14">
@@ -14713,37 +14818,37 @@
         <v>173</v>
       </c>
       <c r="D98" t="s">
-        <v>593</v>
+        <v>605</v>
       </c>
       <c r="E98" t="s">
-        <v>668</v>
+        <v>636</v>
       </c>
       <c r="F98">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G98">
-        <v>562.25</v>
+        <v>171.77</v>
       </c>
       <c r="H98">
-        <v>1686.75</v>
+        <v>343.54</v>
       </c>
       <c r="I98" t="s">
-        <v>382</v>
+        <v>713</v>
       </c>
       <c r="J98" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K98" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L98" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M98" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N98" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="99" spans="1:14">
@@ -14757,37 +14862,37 @@
         <v>173</v>
       </c>
       <c r="D99" t="s">
-        <v>594</v>
+        <v>606</v>
       </c>
       <c r="E99" t="s">
-        <v>669</v>
+        <v>342</v>
       </c>
       <c r="F99">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="G99">
-        <v>630</v>
+        <v>7.03</v>
       </c>
       <c r="H99">
-        <v>630</v>
+        <v>224.96</v>
       </c>
       <c r="I99" t="s">
-        <v>382</v>
+        <v>713</v>
       </c>
       <c r="J99" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K99" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L99" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M99" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N99" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="100" spans="1:14">
@@ -14801,37 +14906,37 @@
         <v>173</v>
       </c>
       <c r="D100" t="s">
-        <v>595</v>
+        <v>607</v>
       </c>
       <c r="E100" t="s">
-        <v>670</v>
+        <v>694</v>
       </c>
       <c r="F100">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G100">
-        <v>512.98</v>
+        <v>589.47</v>
       </c>
       <c r="H100">
-        <v>512.98</v>
+        <v>1768.41</v>
       </c>
       <c r="I100" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J100" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K100" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L100" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M100" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N100" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="101" spans="1:14">
@@ -14845,37 +14950,37 @@
         <v>173</v>
       </c>
       <c r="D101" t="s">
-        <v>596</v>
+        <v>608</v>
       </c>
       <c r="E101" t="s">
-        <v>671</v>
+        <v>695</v>
       </c>
       <c r="F101">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G101">
-        <v>3508.01</v>
+        <v>630</v>
       </c>
       <c r="H101">
-        <v>7016.02</v>
+        <v>630</v>
       </c>
       <c r="I101" t="s">
-        <v>382</v>
+        <v>713</v>
       </c>
       <c r="J101" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K101" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L101" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M101" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N101" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="102" spans="1:14">
@@ -14889,37 +14994,37 @@
         <v>173</v>
       </c>
       <c r="D102" t="s">
-        <v>261</v>
+        <v>609</v>
       </c>
       <c r="E102" t="s">
-        <v>358</v>
+        <v>696</v>
       </c>
       <c r="F102">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G102">
-        <v>7381.62</v>
+        <v>512.98</v>
       </c>
       <c r="H102">
-        <v>29526.48</v>
+        <v>512.98</v>
       </c>
       <c r="I102" t="s">
-        <v>382</v>
+        <v>713</v>
       </c>
       <c r="J102" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K102" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L102" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M102" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N102" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="103" spans="1:14">
@@ -14933,37 +15038,37 @@
         <v>173</v>
       </c>
       <c r="D103" t="s">
-        <v>524</v>
+        <v>610</v>
       </c>
       <c r="E103" t="s">
-        <v>609</v>
+        <v>697</v>
       </c>
       <c r="F103">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G103">
-        <v>500.49</v>
+        <v>3687.68</v>
       </c>
       <c r="H103">
-        <v>1501.47</v>
+        <v>7375.36</v>
       </c>
       <c r="I103" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J103" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K103" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L103" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M103" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N103" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="104" spans="1:14">
@@ -14977,37 +15082,37 @@
         <v>173</v>
       </c>
       <c r="D104" t="s">
-        <v>532</v>
+        <v>261</v>
       </c>
       <c r="E104" t="s">
-        <v>616</v>
+        <v>358</v>
       </c>
       <c r="F104">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="G104">
-        <v>969</v>
+        <v>7381.62</v>
       </c>
       <c r="H104">
-        <v>17442</v>
+        <v>29526.48</v>
       </c>
       <c r="I104" t="s">
         <v>382</v>
       </c>
       <c r="J104" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K104" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L104" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M104" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N104" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="105" spans="1:14">
@@ -15021,37 +15126,37 @@
         <v>173</v>
       </c>
       <c r="D105" t="s">
-        <v>597</v>
+        <v>536</v>
       </c>
       <c r="E105" t="s">
-        <v>672</v>
+        <v>633</v>
       </c>
       <c r="F105">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G105">
-        <v>2958.25</v>
+        <v>526.21</v>
       </c>
       <c r="H105">
-        <v>2958.25</v>
+        <v>1578.63</v>
       </c>
       <c r="I105" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J105" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K105" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L105" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M105" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N105" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="106" spans="1:14">
@@ -15065,37 +15170,37 @@
         <v>173</v>
       </c>
       <c r="D106" t="s">
-        <v>598</v>
+        <v>544</v>
       </c>
       <c r="E106" t="s">
-        <v>673</v>
+        <v>640</v>
       </c>
       <c r="F106">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="G106">
-        <v>3864.72</v>
+        <v>969</v>
       </c>
       <c r="H106">
-        <v>23188.32</v>
+        <v>17442</v>
       </c>
       <c r="I106" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J106" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K106" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L106" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M106" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N106" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="107" spans="1:14">
@@ -15109,37 +15214,37 @@
         <v>173</v>
       </c>
       <c r="D107" t="s">
-        <v>599</v>
+        <v>611</v>
       </c>
       <c r="E107" t="s">
-        <v>298</v>
+        <v>698</v>
       </c>
       <c r="F107">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G107">
-        <v>67.89</v>
+        <v>3100.94</v>
       </c>
       <c r="H107">
-        <v>678.9</v>
+        <v>3100.94</v>
       </c>
       <c r="I107" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="J107" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="K107" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="L107" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="M107" s="1">
-        <v>46368</v>
+        <v>46384</v>
       </c>
       <c r="N107" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="108" spans="1:14">
@@ -15153,37 +15258,37 @@
         <v>173</v>
       </c>
       <c r="D108" t="s">
-        <v>600</v>
+        <v>612</v>
       </c>
       <c r="E108" t="s">
-        <v>674</v>
+        <v>699</v>
       </c>
       <c r="F108">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G108">
-        <v>41.41</v>
+        <v>3490.43</v>
       </c>
       <c r="H108">
-        <v>331.28</v>
+        <v>20942.58</v>
       </c>
       <c r="I108" t="s">
         <v>382</v>
       </c>
       <c r="J108" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K108" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L108" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M108" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N108" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
     </row>
     <row r="109" spans="1:14">
@@ -15197,37 +15302,562 @@
         <v>173</v>
       </c>
       <c r="D109" t="s">
-        <v>601</v>
+        <v>613</v>
       </c>
       <c r="E109" t="s">
-        <v>675</v>
+        <v>298</v>
       </c>
       <c r="F109">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G109">
-        <v>139.45</v>
+        <v>67.89</v>
       </c>
       <c r="H109">
-        <v>278.9</v>
+        <v>678.9</v>
       </c>
       <c r="I109" t="s">
         <v>382</v>
       </c>
       <c r="J109" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="K109" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="L109" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="M109" s="1">
-        <v>46368</v>
+        <v>46369</v>
       </c>
       <c r="N109" t="s">
-        <v>682</v>
+        <v>718</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14">
+      <c r="A110" t="s">
+        <v>514</v>
+      </c>
+      <c r="B110" t="s">
+        <v>172</v>
+      </c>
+      <c r="C110" t="s">
+        <v>173</v>
+      </c>
+      <c r="D110" t="s">
+        <v>614</v>
+      </c>
+      <c r="E110" t="s">
+        <v>700</v>
+      </c>
+      <c r="F110">
+        <v>8</v>
+      </c>
+      <c r="G110">
+        <v>41.41</v>
+      </c>
+      <c r="H110">
+        <v>331.28</v>
+      </c>
+      <c r="I110" t="s">
+        <v>713</v>
+      </c>
+      <c r="J110" t="s">
+        <v>713</v>
+      </c>
+      <c r="K110" t="s">
+        <v>713</v>
+      </c>
+      <c r="L110" t="s">
+        <v>713</v>
+      </c>
+      <c r="M110" s="1">
+        <v>46369</v>
+      </c>
+      <c r="N110" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14">
+      <c r="A111" t="s">
+        <v>515</v>
+      </c>
+      <c r="B111" t="s">
+        <v>172</v>
+      </c>
+      <c r="C111" t="s">
+        <v>173</v>
+      </c>
+      <c r="D111" t="s">
+        <v>615</v>
+      </c>
+      <c r="E111" t="s">
+        <v>701</v>
+      </c>
+      <c r="F111">
+        <v>2</v>
+      </c>
+      <c r="G111">
+        <v>146.21</v>
+      </c>
+      <c r="H111">
+        <v>292.42</v>
+      </c>
+      <c r="I111" t="s">
+        <v>713</v>
+      </c>
+      <c r="J111" t="s">
+        <v>713</v>
+      </c>
+      <c r="K111" t="s">
+        <v>713</v>
+      </c>
+      <c r="L111" t="s">
+        <v>713</v>
+      </c>
+      <c r="M111" s="1">
+        <v>46369</v>
+      </c>
+      <c r="N111" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14">
+      <c r="A112" t="s">
+        <v>516</v>
+      </c>
+      <c r="B112" t="s">
+        <v>172</v>
+      </c>
+      <c r="C112" t="s">
+        <v>173</v>
+      </c>
+      <c r="D112" t="s">
+        <v>616</v>
+      </c>
+      <c r="E112" t="s">
+        <v>702</v>
+      </c>
+      <c r="F112">
+        <v>5</v>
+      </c>
+      <c r="G112">
+        <v>1614.96</v>
+      </c>
+      <c r="H112">
+        <v>8074.8</v>
+      </c>
+      <c r="I112" t="s">
+        <v>713</v>
+      </c>
+      <c r="J112" t="s">
+        <v>713</v>
+      </c>
+      <c r="K112" t="s">
+        <v>713</v>
+      </c>
+      <c r="L112" t="s">
+        <v>713</v>
+      </c>
+      <c r="M112" s="1">
+        <v>46369</v>
+      </c>
+      <c r="N112" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="113" spans="1:14">
+      <c r="A113" t="s">
+        <v>517</v>
+      </c>
+      <c r="B113" t="s">
+        <v>172</v>
+      </c>
+      <c r="C113" t="s">
+        <v>173</v>
+      </c>
+      <c r="D113" t="s">
+        <v>617</v>
+      </c>
+      <c r="E113" t="s">
+        <v>703</v>
+      </c>
+      <c r="F113">
+        <v>2</v>
+      </c>
+      <c r="G113">
+        <v>1153.78</v>
+      </c>
+      <c r="H113">
+        <v>2307.56</v>
+      </c>
+      <c r="I113" t="s">
+        <v>713</v>
+      </c>
+      <c r="J113" t="s">
+        <v>713</v>
+      </c>
+      <c r="K113" t="s">
+        <v>713</v>
+      </c>
+      <c r="L113" t="s">
+        <v>713</v>
+      </c>
+      <c r="M113" s="1">
+        <v>46369</v>
+      </c>
+      <c r="N113" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="114" spans="1:14">
+      <c r="A114" t="s">
+        <v>518</v>
+      </c>
+      <c r="B114" t="s">
+        <v>172</v>
+      </c>
+      <c r="C114" t="s">
+        <v>173</v>
+      </c>
+      <c r="D114" t="s">
+        <v>618</v>
+      </c>
+      <c r="E114" t="s">
+        <v>704</v>
+      </c>
+      <c r="F114">
+        <v>3</v>
+      </c>
+      <c r="G114">
+        <v>2492.21</v>
+      </c>
+      <c r="H114">
+        <v>7476.63</v>
+      </c>
+      <c r="I114" t="s">
+        <v>713</v>
+      </c>
+      <c r="J114" t="s">
+        <v>713</v>
+      </c>
+      <c r="K114" t="s">
+        <v>713</v>
+      </c>
+      <c r="L114" t="s">
+        <v>713</v>
+      </c>
+      <c r="M114" s="1">
+        <v>46369</v>
+      </c>
+      <c r="N114" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="115" spans="1:14">
+      <c r="A115" t="s">
+        <v>519</v>
+      </c>
+      <c r="B115" t="s">
+        <v>172</v>
+      </c>
+      <c r="C115" t="s">
+        <v>173</v>
+      </c>
+      <c r="D115" t="s">
+        <v>619</v>
+      </c>
+      <c r="E115" t="s">
+        <v>705</v>
+      </c>
+      <c r="F115">
+        <v>4</v>
+      </c>
+      <c r="G115">
+        <v>4191.72</v>
+      </c>
+      <c r="H115">
+        <v>16766.88</v>
+      </c>
+      <c r="I115" t="s">
+        <v>713</v>
+      </c>
+      <c r="J115" t="s">
+        <v>713</v>
+      </c>
+      <c r="K115" t="s">
+        <v>713</v>
+      </c>
+      <c r="L115" t="s">
+        <v>713</v>
+      </c>
+      <c r="M115" s="1">
+        <v>46369</v>
+      </c>
+      <c r="N115" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="116" spans="1:14">
+      <c r="A116" t="s">
+        <v>520</v>
+      </c>
+      <c r="B116" t="s">
+        <v>172</v>
+      </c>
+      <c r="C116" t="s">
+        <v>173</v>
+      </c>
+      <c r="D116" t="s">
+        <v>620</v>
+      </c>
+      <c r="E116" t="s">
+        <v>706</v>
+      </c>
+      <c r="F116">
+        <v>1</v>
+      </c>
+      <c r="G116">
+        <v>6320.46</v>
+      </c>
+      <c r="H116">
+        <v>6320.46</v>
+      </c>
+      <c r="I116" t="s">
+        <v>713</v>
+      </c>
+      <c r="J116" t="s">
+        <v>713</v>
+      </c>
+      <c r="K116" t="s">
+        <v>713</v>
+      </c>
+      <c r="L116" t="s">
+        <v>713</v>
+      </c>
+      <c r="M116" s="1">
+        <v>46369</v>
+      </c>
+      <c r="N116" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="117" spans="1:14">
+      <c r="A117" t="s">
+        <v>521</v>
+      </c>
+      <c r="B117" t="s">
+        <v>172</v>
+      </c>
+      <c r="C117" t="s">
+        <v>173</v>
+      </c>
+      <c r="D117" t="s">
+        <v>621</v>
+      </c>
+      <c r="E117" t="s">
+        <v>707</v>
+      </c>
+      <c r="F117">
+        <v>5</v>
+      </c>
+      <c r="G117">
+        <v>2084.06</v>
+      </c>
+      <c r="H117">
+        <v>10420.3</v>
+      </c>
+      <c r="I117" t="s">
+        <v>713</v>
+      </c>
+      <c r="J117" t="s">
+        <v>713</v>
+      </c>
+      <c r="K117" t="s">
+        <v>713</v>
+      </c>
+      <c r="L117" t="s">
+        <v>713</v>
+      </c>
+      <c r="M117" s="1">
+        <v>46369</v>
+      </c>
+      <c r="N117" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="118" spans="1:14">
+      <c r="A118" t="s">
+        <v>522</v>
+      </c>
+      <c r="B118" t="s">
+        <v>172</v>
+      </c>
+      <c r="C118" t="s">
+        <v>173</v>
+      </c>
+      <c r="D118" t="s">
+        <v>622</v>
+      </c>
+      <c r="E118" t="s">
+        <v>708</v>
+      </c>
+      <c r="F118">
+        <v>5</v>
+      </c>
+      <c r="G118">
+        <v>3202.46</v>
+      </c>
+      <c r="H118">
+        <v>16012.3</v>
+      </c>
+      <c r="I118" t="s">
+        <v>713</v>
+      </c>
+      <c r="J118" t="s">
+        <v>713</v>
+      </c>
+      <c r="K118" t="s">
+        <v>713</v>
+      </c>
+      <c r="L118" t="s">
+        <v>713</v>
+      </c>
+      <c r="M118" s="1">
+        <v>46369</v>
+      </c>
+      <c r="N118" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="119" spans="1:14">
+      <c r="A119" t="s">
+        <v>523</v>
+      </c>
+      <c r="B119" t="s">
+        <v>172</v>
+      </c>
+      <c r="C119" t="s">
+        <v>173</v>
+      </c>
+      <c r="D119" t="s">
+        <v>623</v>
+      </c>
+      <c r="E119" t="s">
+        <v>709</v>
+      </c>
+      <c r="F119">
+        <v>1</v>
+      </c>
+      <c r="G119">
+        <v>16427.97</v>
+      </c>
+      <c r="H119">
+        <v>16427.97</v>
+      </c>
+      <c r="I119" t="s">
+        <v>382</v>
+      </c>
+      <c r="J119" t="s">
+        <v>713</v>
+      </c>
+      <c r="K119" t="s">
+        <v>713</v>
+      </c>
+      <c r="L119" t="s">
+        <v>713</v>
+      </c>
+      <c r="M119" s="1">
+        <v>46369</v>
+      </c>
+      <c r="N119" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="120" spans="1:14">
+      <c r="A120" t="s">
+        <v>524</v>
+      </c>
+      <c r="B120" t="s">
+        <v>172</v>
+      </c>
+      <c r="C120" t="s">
+        <v>173</v>
+      </c>
+      <c r="D120" t="s">
+        <v>624</v>
+      </c>
+      <c r="E120" t="s">
+        <v>710</v>
+      </c>
+      <c r="F120">
+        <v>2</v>
+      </c>
+      <c r="G120">
+        <v>12325.12</v>
+      </c>
+      <c r="H120">
+        <v>24650.24</v>
+      </c>
+      <c r="I120" t="s">
+        <v>713</v>
+      </c>
+      <c r="J120" t="s">
+        <v>713</v>
+      </c>
+      <c r="K120" t="s">
+        <v>713</v>
+      </c>
+      <c r="L120" t="s">
+        <v>713</v>
+      </c>
+      <c r="M120" s="1">
+        <v>46369</v>
+      </c>
+      <c r="N120" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="121" spans="1:14">
+      <c r="A121" t="s">
+        <v>525</v>
+      </c>
+      <c r="B121" t="s">
+        <v>172</v>
+      </c>
+      <c r="C121" t="s">
+        <v>173</v>
+      </c>
+      <c r="D121" t="s">
+        <v>625</v>
+      </c>
+      <c r="E121" t="s">
+        <v>711</v>
+      </c>
+      <c r="F121">
+        <v>11</v>
+      </c>
+      <c r="G121">
+        <v>15038</v>
+      </c>
+      <c r="H121">
+        <v>165418</v>
+      </c>
+      <c r="I121" t="s">
+        <v>382</v>
+      </c>
+      <c r="K121" t="s">
+        <v>382</v>
+      </c>
+      <c r="L121" t="s">
+        <v>382</v>
+      </c>
+      <c r="M121" s="1">
+        <v>46374</v>
+      </c>
+      <c r="N121" t="s">
+        <v>718</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (29/09/2026 19:54)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2181,8 +2181,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2198,7 +2206,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2206,12 +2214,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2511,55 +2537,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2603,7 +2629,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2647,7 +2673,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2691,7 +2717,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2817,7 +2843,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2861,7 +2887,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2905,7 +2931,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2952,7 +2978,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3075,7 +3101,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -3119,7 +3145,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3163,7 +3189,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3207,7 +3233,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3254,7 +3280,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3298,7 +3324,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3424,7 +3450,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3468,7 +3494,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3553,7 +3579,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3600,7 +3626,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3647,7 +3673,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3691,7 +3717,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3735,7 +3761,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3820,7 +3846,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3905,7 +3931,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3952,7 +3978,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3996,7 +4022,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4040,7 +4066,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4125,7 +4151,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4169,7 +4195,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4213,7 +4239,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4298,7 +4324,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4342,7 +4368,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4386,7 +4412,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4430,7 +4456,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4597,7 +4623,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4641,7 +4667,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4685,7 +4711,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4729,7 +4755,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4776,7 +4802,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4820,7 +4846,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4902,7 +4928,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4946,7 +4972,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5034,7 +5060,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5078,7 +5104,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5125,7 +5151,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5169,7 +5195,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -5213,7 +5239,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5257,7 +5283,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5301,7 +5327,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5348,7 +5374,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5392,7 +5418,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5439,7 +5465,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5483,7 +5509,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5530,7 +5556,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5618,7 +5644,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5662,7 +5688,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5706,7 +5732,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5750,7 +5776,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5794,7 +5820,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5838,7 +5864,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5923,7 +5949,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5967,7 +5993,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -6011,7 +6037,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -6055,7 +6081,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -6099,7 +6125,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -6143,7 +6169,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6187,7 +6213,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6231,7 +6257,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6278,7 +6304,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6322,7 +6348,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6366,7 +6392,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6410,7 +6436,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6454,7 +6480,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6498,7 +6524,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6542,7 +6568,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6586,7 +6612,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6630,7 +6656,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6718,7 +6744,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6762,7 +6788,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6888,7 +6914,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6932,7 +6958,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6976,7 +7002,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7020,7 +7046,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7102,7 +7128,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7146,7 +7172,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7193,7 +7219,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7237,7 +7263,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7363,7 +7389,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7407,7 +7433,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7492,7 +7518,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7536,7 +7562,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7580,7 +7606,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7624,7 +7650,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7668,7 +7694,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7712,7 +7738,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7756,7 +7782,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7800,7 +7826,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7885,7 +7911,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8052,7 +8078,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8096,7 +8122,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8140,7 +8166,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8184,7 +8210,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8228,7 +8254,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8272,7 +8298,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8316,7 +8342,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8401,7 +8427,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8445,7 +8471,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8530,7 +8556,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8656,7 +8682,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8700,7 +8726,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8785,7 +8811,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8829,7 +8855,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8873,7 +8899,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8917,7 +8943,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8961,7 +8987,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -9005,7 +9031,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9049,7 +9075,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9093,7 +9119,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9178,7 +9204,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9345,7 +9371,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9389,7 +9415,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9433,7 +9459,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9477,7 +9503,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9562,7 +9588,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9606,7 +9632,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9650,7 +9676,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9694,7 +9720,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9738,7 +9764,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9782,7 +9808,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9826,7 +9852,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9870,7 +9896,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9914,7 +9940,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9958,7 +9984,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10002,7 +10028,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -10046,7 +10072,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10090,7 +10116,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10134,7 +10160,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -10178,7 +10204,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10222,7 +10248,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10266,7 +10292,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10310,7 +10336,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10354,7 +10380,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10398,7 +10424,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10442,7 +10468,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10527,7 +10553,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10612,7 +10638,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10627,55 +10653,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11044,7 +11070,7 @@
       <c r="L10" t="s">
         <v>716</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46384</v>
       </c>
       <c r="N10" t="s">
@@ -11088,7 +11114,7 @@
       <c r="L11" t="s">
         <v>716</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46384</v>
       </c>
       <c r="N11" t="s">
@@ -11296,7 +11322,7 @@
       <c r="L16" t="s">
         <v>716</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46384</v>
       </c>
       <c r="N16" t="s">
@@ -11381,7 +11407,7 @@
       <c r="L18" t="s">
         <v>716</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>46384</v>
       </c>
       <c r="N18" t="s">
@@ -11425,7 +11451,7 @@
       <c r="L19" t="s">
         <v>713</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46369</v>
       </c>
       <c r="N19" t="s">
@@ -11469,7 +11495,7 @@
       <c r="L20" t="s">
         <v>716</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46384</v>
       </c>
       <c r="N20" t="s">
@@ -11513,7 +11539,7 @@
       <c r="L21" t="s">
         <v>713</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46369</v>
       </c>
       <c r="N21" t="s">
@@ -11680,7 +11706,7 @@
       <c r="L25" t="s">
         <v>713</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46369</v>
       </c>
       <c r="N25" t="s">
@@ -11806,7 +11832,7 @@
       <c r="L28" t="s">
         <v>713</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46369</v>
       </c>
       <c r="N28" t="s">
@@ -11850,7 +11876,7 @@
       <c r="L29" t="s">
         <v>717</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="2">
         <v>46324</v>
       </c>
       <c r="N29" t="s">
@@ -11894,7 +11920,7 @@
       <c r="L30" t="s">
         <v>713</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46369</v>
       </c>
       <c r="N30" t="s">
@@ -11938,7 +11964,7 @@
       <c r="L31" t="s">
         <v>717</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="2">
         <v>46324</v>
       </c>
       <c r="N31" t="s">
@@ -12351,7 +12377,7 @@
       <c r="L41" t="s">
         <v>713</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46369</v>
       </c>
       <c r="N41" t="s">
@@ -12436,7 +12462,7 @@
       <c r="L43" t="s">
         <v>713</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46369</v>
       </c>
       <c r="N43" t="s">
@@ -12480,7 +12506,7 @@
       <c r="L44" t="s">
         <v>713</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46369</v>
       </c>
       <c r="N44" t="s">
@@ -12524,7 +12550,7 @@
       <c r="L45" t="s">
         <v>713</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46369</v>
       </c>
       <c r="N45" t="s">
@@ -12650,7 +12676,7 @@
       <c r="L48" t="s">
         <v>713</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46369</v>
       </c>
       <c r="N48" t="s">
@@ -12694,7 +12720,7 @@
       <c r="L49" t="s">
         <v>717</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46324</v>
       </c>
       <c r="N49" t="s">
@@ -12738,7 +12764,7 @@
       <c r="L50" t="s">
         <v>717</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46324</v>
       </c>
       <c r="N50" t="s">
@@ -12782,7 +12808,7 @@
       <c r="L51" t="s">
         <v>713</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46369</v>
       </c>
       <c r="N51" t="s">
@@ -12826,7 +12852,7 @@
       <c r="L52" t="s">
         <v>713</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46369</v>
       </c>
       <c r="N52" t="s">
@@ -12870,7 +12896,7 @@
       <c r="L53" t="s">
         <v>713</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46369</v>
       </c>
       <c r="N53" t="s">
@@ -12914,7 +12940,7 @@
       <c r="L54" t="s">
         <v>713</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46369</v>
       </c>
       <c r="N54" t="s">
@@ -12958,7 +12984,7 @@
       <c r="L55" t="s">
         <v>713</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46369</v>
       </c>
       <c r="N55" t="s">
@@ -13002,7 +13028,7 @@
       <c r="L56" t="s">
         <v>717</v>
       </c>
-      <c r="M56" s="1">
+      <c r="M56" s="2">
         <v>46324</v>
       </c>
       <c r="N56" t="s">
@@ -13046,7 +13072,7 @@
       <c r="L57" t="s">
         <v>717</v>
       </c>
-      <c r="M57" s="1">
+      <c r="M57" s="2">
         <v>46324</v>
       </c>
       <c r="N57" t="s">
@@ -13090,7 +13116,7 @@
       <c r="L58" t="s">
         <v>717</v>
       </c>
-      <c r="M58" s="1">
+      <c r="M58" s="2">
         <v>46324</v>
       </c>
       <c r="N58" t="s">
@@ -13134,7 +13160,7 @@
       <c r="L59" t="s">
         <v>713</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46369</v>
       </c>
       <c r="N59" t="s">
@@ -13178,7 +13204,7 @@
       <c r="L60" t="s">
         <v>717</v>
       </c>
-      <c r="M60" s="1">
+      <c r="M60" s="2">
         <v>46324</v>
       </c>
       <c r="N60" t="s">
@@ -13222,7 +13248,7 @@
       <c r="L61" t="s">
         <v>717</v>
       </c>
-      <c r="M61" s="1">
+      <c r="M61" s="2">
         <v>46324</v>
       </c>
       <c r="N61" t="s">
@@ -13266,7 +13292,7 @@
       <c r="L62" t="s">
         <v>713</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46369</v>
       </c>
       <c r="N62" t="s">
@@ -13310,7 +13336,7 @@
       <c r="L63" t="s">
         <v>713</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46369</v>
       </c>
       <c r="N63" t="s">
@@ -13354,7 +13380,7 @@
       <c r="L64" t="s">
         <v>713</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46369</v>
       </c>
       <c r="N64" t="s">
@@ -13398,7 +13424,7 @@
       <c r="L65" t="s">
         <v>713</v>
       </c>
-      <c r="M65" s="1">
+      <c r="M65" s="2">
         <v>46369</v>
       </c>
       <c r="N65" t="s">
@@ -13442,7 +13468,7 @@
       <c r="L66" t="s">
         <v>713</v>
       </c>
-      <c r="M66" s="1">
+      <c r="M66" s="2">
         <v>46369</v>
       </c>
       <c r="N66" t="s">
@@ -13486,7 +13512,7 @@
       <c r="L67" t="s">
         <v>713</v>
       </c>
-      <c r="M67" s="1">
+      <c r="M67" s="2">
         <v>46369</v>
       </c>
       <c r="N67" t="s">
@@ -13530,7 +13556,7 @@
       <c r="L68" t="s">
         <v>713</v>
       </c>
-      <c r="M68" s="1">
+      <c r="M68" s="2">
         <v>46369</v>
       </c>
       <c r="N68" t="s">
@@ -13574,7 +13600,7 @@
       <c r="L69" t="s">
         <v>713</v>
       </c>
-      <c r="M69" s="1">
+      <c r="M69" s="2">
         <v>46369</v>
       </c>
       <c r="N69" t="s">
@@ -13618,7 +13644,7 @@
       <c r="L70" t="s">
         <v>713</v>
       </c>
-      <c r="M70" s="1">
+      <c r="M70" s="2">
         <v>46369</v>
       </c>
       <c r="N70" t="s">
@@ -13662,7 +13688,7 @@
       <c r="L71" t="s">
         <v>713</v>
       </c>
-      <c r="M71" s="1">
+      <c r="M71" s="2">
         <v>46369</v>
       </c>
       <c r="N71" t="s">
@@ -13706,7 +13732,7 @@
       <c r="L72" t="s">
         <v>713</v>
       </c>
-      <c r="M72" s="1">
+      <c r="M72" s="2">
         <v>46369</v>
       </c>
       <c r="N72" t="s">
@@ -13750,7 +13776,7 @@
       <c r="L73" t="s">
         <v>713</v>
       </c>
-      <c r="M73" s="1">
+      <c r="M73" s="2">
         <v>46369</v>
       </c>
       <c r="N73" t="s">
@@ -13794,7 +13820,7 @@
       <c r="L74" t="s">
         <v>713</v>
       </c>
-      <c r="M74" s="1">
+      <c r="M74" s="2">
         <v>46369</v>
       </c>
       <c r="N74" t="s">
@@ -13838,7 +13864,7 @@
       <c r="L75" t="s">
         <v>713</v>
       </c>
-      <c r="M75" s="1">
+      <c r="M75" s="2">
         <v>46369</v>
       </c>
       <c r="N75" t="s">
@@ -13879,7 +13905,7 @@
       <c r="L76" t="s">
         <v>716</v>
       </c>
-      <c r="M76" s="1">
+      <c r="M76" s="2">
         <v>46384</v>
       </c>
       <c r="N76" t="s">
@@ -13920,7 +13946,7 @@
       <c r="L77" t="s">
         <v>713</v>
       </c>
-      <c r="M77" s="1">
+      <c r="M77" s="2">
         <v>46369</v>
       </c>
       <c r="N77" t="s">
@@ -13964,7 +13990,7 @@
       <c r="L78" t="s">
         <v>713</v>
       </c>
-      <c r="M78" s="1">
+      <c r="M78" s="2">
         <v>46369</v>
       </c>
       <c r="N78" t="s">
@@ -14008,7 +14034,7 @@
       <c r="L79" t="s">
         <v>713</v>
       </c>
-      <c r="M79" s="1">
+      <c r="M79" s="2">
         <v>46369</v>
       </c>
       <c r="N79" t="s">
@@ -14052,7 +14078,7 @@
       <c r="L80" t="s">
         <v>713</v>
       </c>
-      <c r="M80" s="1">
+      <c r="M80" s="2">
         <v>46369</v>
       </c>
       <c r="N80" t="s">
@@ -14096,7 +14122,7 @@
       <c r="L81" t="s">
         <v>716</v>
       </c>
-      <c r="M81" s="1">
+      <c r="M81" s="2">
         <v>46384</v>
       </c>
       <c r="N81" t="s">
@@ -14140,7 +14166,7 @@
       <c r="L82" t="s">
         <v>713</v>
       </c>
-      <c r="M82" s="1">
+      <c r="M82" s="2">
         <v>46369</v>
       </c>
       <c r="N82" t="s">
@@ -14184,7 +14210,7 @@
       <c r="L83" t="s">
         <v>713</v>
       </c>
-      <c r="M83" s="1">
+      <c r="M83" s="2">
         <v>46369</v>
       </c>
       <c r="N83" t="s">
@@ -14228,7 +14254,7 @@
       <c r="L84" t="s">
         <v>713</v>
       </c>
-      <c r="M84" s="1">
+      <c r="M84" s="2">
         <v>46369</v>
       </c>
       <c r="N84" t="s">
@@ -14272,7 +14298,7 @@
       <c r="L85" t="s">
         <v>713</v>
       </c>
-      <c r="M85" s="1">
+      <c r="M85" s="2">
         <v>46369</v>
       </c>
       <c r="N85" t="s">
@@ -14316,7 +14342,7 @@
       <c r="L86" t="s">
         <v>713</v>
       </c>
-      <c r="M86" s="1">
+      <c r="M86" s="2">
         <v>46369</v>
       </c>
       <c r="N86" t="s">
@@ -14360,7 +14386,7 @@
       <c r="L87" t="s">
         <v>713</v>
       </c>
-      <c r="M87" s="1">
+      <c r="M87" s="2">
         <v>46369</v>
       </c>
       <c r="N87" t="s">
@@ -14404,7 +14430,7 @@
       <c r="L88" t="s">
         <v>716</v>
       </c>
-      <c r="M88" s="1">
+      <c r="M88" s="2">
         <v>46384</v>
       </c>
       <c r="N88" t="s">
@@ -14448,7 +14474,7 @@
       <c r="L89" t="s">
         <v>713</v>
       </c>
-      <c r="M89" s="1">
+      <c r="M89" s="2">
         <v>46369</v>
       </c>
       <c r="N89" t="s">
@@ -14492,7 +14518,7 @@
       <c r="L90" t="s">
         <v>716</v>
       </c>
-      <c r="M90" s="1">
+      <c r="M90" s="2">
         <v>46384</v>
       </c>
       <c r="N90" t="s">
@@ -14536,7 +14562,7 @@
       <c r="L91" t="s">
         <v>716</v>
       </c>
-      <c r="M91" s="1">
+      <c r="M91" s="2">
         <v>46384</v>
       </c>
       <c r="N91" t="s">
@@ -14580,7 +14606,7 @@
       <c r="L92" t="s">
         <v>713</v>
       </c>
-      <c r="M92" s="1">
+      <c r="M92" s="2">
         <v>46369</v>
       </c>
       <c r="N92" t="s">
@@ -14624,7 +14650,7 @@
       <c r="L93" t="s">
         <v>716</v>
       </c>
-      <c r="M93" s="1">
+      <c r="M93" s="2">
         <v>46384</v>
       </c>
       <c r="N93" t="s">
@@ -14668,7 +14694,7 @@
       <c r="L94" t="s">
         <v>716</v>
       </c>
-      <c r="M94" s="1">
+      <c r="M94" s="2">
         <v>46384</v>
       </c>
       <c r="N94" t="s">
@@ -14712,7 +14738,7 @@
       <c r="L95" t="s">
         <v>716</v>
       </c>
-      <c r="M95" s="1">
+      <c r="M95" s="2">
         <v>46384</v>
       </c>
       <c r="N95" t="s">
@@ -14756,7 +14782,7 @@
       <c r="L96" t="s">
         <v>716</v>
       </c>
-      <c r="M96" s="1">
+      <c r="M96" s="2">
         <v>46384</v>
       </c>
       <c r="N96" t="s">
@@ -14800,7 +14826,7 @@
       <c r="L97" t="s">
         <v>713</v>
       </c>
-      <c r="M97" s="1">
+      <c r="M97" s="2">
         <v>46369</v>
       </c>
       <c r="N97" t="s">
@@ -14844,7 +14870,7 @@
       <c r="L98" t="s">
         <v>713</v>
       </c>
-      <c r="M98" s="1">
+      <c r="M98" s="2">
         <v>46369</v>
       </c>
       <c r="N98" t="s">
@@ -14888,7 +14914,7 @@
       <c r="L99" t="s">
         <v>713</v>
       </c>
-      <c r="M99" s="1">
+      <c r="M99" s="2">
         <v>46369</v>
       </c>
       <c r="N99" t="s">
@@ -14932,7 +14958,7 @@
       <c r="L100" t="s">
         <v>716</v>
       </c>
-      <c r="M100" s="1">
+      <c r="M100" s="2">
         <v>46384</v>
       </c>
       <c r="N100" t="s">
@@ -14976,7 +15002,7 @@
       <c r="L101" t="s">
         <v>713</v>
       </c>
-      <c r="M101" s="1">
+      <c r="M101" s="2">
         <v>46369</v>
       </c>
       <c r="N101" t="s">
@@ -15020,7 +15046,7 @@
       <c r="L102" t="s">
         <v>713</v>
       </c>
-      <c r="M102" s="1">
+      <c r="M102" s="2">
         <v>46369</v>
       </c>
       <c r="N102" t="s">
@@ -15064,7 +15090,7 @@
       <c r="L103" t="s">
         <v>716</v>
       </c>
-      <c r="M103" s="1">
+      <c r="M103" s="2">
         <v>46384</v>
       </c>
       <c r="N103" t="s">
@@ -15108,7 +15134,7 @@
       <c r="L104" t="s">
         <v>713</v>
       </c>
-      <c r="M104" s="1">
+      <c r="M104" s="2">
         <v>46369</v>
       </c>
       <c r="N104" t="s">
@@ -15152,7 +15178,7 @@
       <c r="L105" t="s">
         <v>716</v>
       </c>
-      <c r="M105" s="1">
+      <c r="M105" s="2">
         <v>46384</v>
       </c>
       <c r="N105" t="s">
@@ -15196,7 +15222,7 @@
       <c r="L106" t="s">
         <v>716</v>
       </c>
-      <c r="M106" s="1">
+      <c r="M106" s="2">
         <v>46384</v>
       </c>
       <c r="N106" t="s">
@@ -15240,7 +15266,7 @@
       <c r="L107" t="s">
         <v>716</v>
       </c>
-      <c r="M107" s="1">
+      <c r="M107" s="2">
         <v>46384</v>
       </c>
       <c r="N107" t="s">
@@ -15284,7 +15310,7 @@
       <c r="L108" t="s">
         <v>713</v>
       </c>
-      <c r="M108" s="1">
+      <c r="M108" s="2">
         <v>46369</v>
       </c>
       <c r="N108" t="s">
@@ -15328,7 +15354,7 @@
       <c r="L109" t="s">
         <v>713</v>
       </c>
-      <c r="M109" s="1">
+      <c r="M109" s="2">
         <v>46369</v>
       </c>
       <c r="N109" t="s">
@@ -15372,7 +15398,7 @@
       <c r="L110" t="s">
         <v>713</v>
       </c>
-      <c r="M110" s="1">
+      <c r="M110" s="2">
         <v>46369</v>
       </c>
       <c r="N110" t="s">
@@ -15416,7 +15442,7 @@
       <c r="L111" t="s">
         <v>713</v>
       </c>
-      <c r="M111" s="1">
+      <c r="M111" s="2">
         <v>46369</v>
       </c>
       <c r="N111" t="s">
@@ -15460,7 +15486,7 @@
       <c r="L112" t="s">
         <v>713</v>
       </c>
-      <c r="M112" s="1">
+      <c r="M112" s="2">
         <v>46369</v>
       </c>
       <c r="N112" t="s">
@@ -15504,7 +15530,7 @@
       <c r="L113" t="s">
         <v>713</v>
       </c>
-      <c r="M113" s="1">
+      <c r="M113" s="2">
         <v>46369</v>
       </c>
       <c r="N113" t="s">
@@ -15548,7 +15574,7 @@
       <c r="L114" t="s">
         <v>713</v>
       </c>
-      <c r="M114" s="1">
+      <c r="M114" s="2">
         <v>46369</v>
       </c>
       <c r="N114" t="s">
@@ -15592,7 +15618,7 @@
       <c r="L115" t="s">
         <v>713</v>
       </c>
-      <c r="M115" s="1">
+      <c r="M115" s="2">
         <v>46369</v>
       </c>
       <c r="N115" t="s">
@@ -15636,7 +15662,7 @@
       <c r="L116" t="s">
         <v>713</v>
       </c>
-      <c r="M116" s="1">
+      <c r="M116" s="2">
         <v>46369</v>
       </c>
       <c r="N116" t="s">
@@ -15680,7 +15706,7 @@
       <c r="L117" t="s">
         <v>713</v>
       </c>
-      <c r="M117" s="1">
+      <c r="M117" s="2">
         <v>46369</v>
       </c>
       <c r="N117" t="s">
@@ -15724,7 +15750,7 @@
       <c r="L118" t="s">
         <v>713</v>
       </c>
-      <c r="M118" s="1">
+      <c r="M118" s="2">
         <v>46369</v>
       </c>
       <c r="N118" t="s">
@@ -15768,7 +15794,7 @@
       <c r="L119" t="s">
         <v>713</v>
       </c>
-      <c r="M119" s="1">
+      <c r="M119" s="2">
         <v>46369</v>
       </c>
       <c r="N119" t="s">
@@ -15812,7 +15838,7 @@
       <c r="L120" t="s">
         <v>713</v>
       </c>
-      <c r="M120" s="1">
+      <c r="M120" s="2">
         <v>46369</v>
       </c>
       <c r="N120" t="s">
@@ -15853,7 +15879,7 @@
       <c r="L121" t="s">
         <v>382</v>
       </c>
-      <c r="M121" s="1">
+      <c r="M121" s="2">
         <v>46374</v>
       </c>
       <c r="N121" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (30/09/2026 13:49)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2181,16 +2181,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2206,7 +2198,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2214,30 +2206,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2537,55 +2511,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2629,7 +2603,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2673,7 +2647,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2717,7 +2691,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2843,7 +2817,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2887,7 +2861,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2931,7 +2905,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2978,7 +2952,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3101,7 +3075,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -3145,7 +3119,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3189,7 +3163,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3233,7 +3207,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3280,7 +3254,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3324,7 +3298,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3450,7 +3424,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3494,7 +3468,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3579,7 +3553,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3626,7 +3600,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3673,7 +3647,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3717,7 +3691,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3761,7 +3735,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3846,7 +3820,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3931,7 +3905,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3978,7 +3952,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4022,7 +3996,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4066,7 +4040,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4151,7 +4125,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4195,7 +4169,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4239,7 +4213,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4324,7 +4298,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4368,7 +4342,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4412,7 +4386,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4456,7 +4430,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4623,7 +4597,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4667,7 +4641,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4711,7 +4685,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4755,7 +4729,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4802,7 +4776,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4846,7 +4820,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4928,7 +4902,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4972,7 +4946,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5060,7 +5034,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5104,7 +5078,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5151,7 +5125,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5195,7 +5169,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -5239,7 +5213,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5283,7 +5257,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5327,7 +5301,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5374,7 +5348,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5418,7 +5392,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5465,7 +5439,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5509,7 +5483,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5556,7 +5530,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5644,7 +5618,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5688,7 +5662,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5732,7 +5706,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5776,7 +5750,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5820,7 +5794,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5864,7 +5838,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5949,7 +5923,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5993,7 +5967,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -6037,7 +6011,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -6081,7 +6055,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -6125,7 +6099,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -6169,7 +6143,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6213,7 +6187,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6257,7 +6231,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6304,7 +6278,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6348,7 +6322,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6392,7 +6366,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6436,7 +6410,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6480,7 +6454,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6524,7 +6498,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6568,7 +6542,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6612,7 +6586,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6656,7 +6630,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6744,7 +6718,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6788,7 +6762,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6914,7 +6888,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6958,7 +6932,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7002,7 +6976,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7046,7 +7020,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7128,7 +7102,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7172,7 +7146,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7219,7 +7193,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7263,7 +7237,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7389,7 +7363,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7433,7 +7407,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7518,7 +7492,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7562,7 +7536,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7606,7 +7580,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7650,7 +7624,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7694,7 +7668,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7738,7 +7712,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7782,7 +7756,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7826,7 +7800,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7911,7 +7885,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8078,7 +8052,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8122,7 +8096,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8166,7 +8140,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8210,7 +8184,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8254,7 +8228,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8298,7 +8272,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8342,7 +8316,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8427,7 +8401,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8471,7 +8445,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8556,7 +8530,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8682,7 +8656,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8726,7 +8700,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8811,7 +8785,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8855,7 +8829,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8899,7 +8873,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8943,7 +8917,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8987,7 +8961,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -9031,7 +9005,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9075,7 +9049,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9119,7 +9093,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9204,7 +9178,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9371,7 +9345,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9415,7 +9389,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9459,7 +9433,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9503,7 +9477,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9588,7 +9562,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9632,7 +9606,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9676,7 +9650,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9720,7 +9694,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9764,7 +9738,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9808,7 +9782,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9852,7 +9826,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9896,7 +9870,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9940,7 +9914,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9984,7 +9958,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10028,7 +10002,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -10072,7 +10046,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10116,7 +10090,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10160,7 +10134,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -10204,7 +10178,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10248,7 +10222,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10292,7 +10266,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10336,7 +10310,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10380,7 +10354,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10424,7 +10398,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10468,7 +10442,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10553,7 +10527,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10638,7 +10612,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10653,55 +10627,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11070,8 +11044,8 @@
       <c r="L10" t="s">
         <v>716</v>
       </c>
-      <c r="M10" s="2">
-        <v>46384</v>
+      <c r="M10" s="1">
+        <v>46385</v>
       </c>
       <c r="N10" t="s">
         <v>718</v>
@@ -11114,8 +11088,8 @@
       <c r="L11" t="s">
         <v>716</v>
       </c>
-      <c r="M11" s="2">
-        <v>46384</v>
+      <c r="M11" s="1">
+        <v>46385</v>
       </c>
       <c r="N11" t="s">
         <v>718</v>
@@ -11322,8 +11296,8 @@
       <c r="L16" t="s">
         <v>716</v>
       </c>
-      <c r="M16" s="2">
-        <v>46384</v>
+      <c r="M16" s="1">
+        <v>46385</v>
       </c>
       <c r="N16" t="s">
         <v>718</v>
@@ -11407,8 +11381,8 @@
       <c r="L18" t="s">
         <v>716</v>
       </c>
-      <c r="M18" s="2">
-        <v>46384</v>
+      <c r="M18" s="1">
+        <v>46385</v>
       </c>
       <c r="N18" t="s">
         <v>718</v>
@@ -11451,8 +11425,8 @@
       <c r="L19" t="s">
         <v>713</v>
       </c>
-      <c r="M19" s="2">
-        <v>46369</v>
+      <c r="M19" s="1">
+        <v>46370</v>
       </c>
       <c r="N19" t="s">
         <v>718</v>
@@ -11495,8 +11469,8 @@
       <c r="L20" t="s">
         <v>716</v>
       </c>
-      <c r="M20" s="2">
-        <v>46384</v>
+      <c r="M20" s="1">
+        <v>46385</v>
       </c>
       <c r="N20" t="s">
         <v>718</v>
@@ -11539,8 +11513,8 @@
       <c r="L21" t="s">
         <v>713</v>
       </c>
-      <c r="M21" s="2">
-        <v>46369</v>
+      <c r="M21" s="1">
+        <v>46370</v>
       </c>
       <c r="N21" t="s">
         <v>718</v>
@@ -11706,8 +11680,8 @@
       <c r="L25" t="s">
         <v>713</v>
       </c>
-      <c r="M25" s="2">
-        <v>46369</v>
+      <c r="M25" s="1">
+        <v>46370</v>
       </c>
       <c r="N25" t="s">
         <v>718</v>
@@ -11832,8 +11806,8 @@
       <c r="L28" t="s">
         <v>713</v>
       </c>
-      <c r="M28" s="2">
-        <v>46369</v>
+      <c r="M28" s="1">
+        <v>46370</v>
       </c>
       <c r="N28" t="s">
         <v>718</v>
@@ -11876,8 +11850,8 @@
       <c r="L29" t="s">
         <v>717</v>
       </c>
-      <c r="M29" s="2">
-        <v>46324</v>
+      <c r="M29" s="1">
+        <v>46325</v>
       </c>
       <c r="N29" t="s">
         <v>718</v>
@@ -11920,8 +11894,8 @@
       <c r="L30" t="s">
         <v>713</v>
       </c>
-      <c r="M30" s="2">
-        <v>46369</v>
+      <c r="M30" s="1">
+        <v>46370</v>
       </c>
       <c r="N30" t="s">
         <v>718</v>
@@ -11964,8 +11938,8 @@
       <c r="L31" t="s">
         <v>717</v>
       </c>
-      <c r="M31" s="2">
-        <v>46324</v>
+      <c r="M31" s="1">
+        <v>46325</v>
       </c>
       <c r="N31" t="s">
         <v>718</v>
@@ -12377,8 +12351,8 @@
       <c r="L41" t="s">
         <v>713</v>
       </c>
-      <c r="M41" s="2">
-        <v>46369</v>
+      <c r="M41" s="1">
+        <v>46370</v>
       </c>
       <c r="N41" t="s">
         <v>718</v>
@@ -12462,8 +12436,8 @@
       <c r="L43" t="s">
         <v>713</v>
       </c>
-      <c r="M43" s="2">
-        <v>46369</v>
+      <c r="M43" s="1">
+        <v>46370</v>
       </c>
       <c r="N43" t="s">
         <v>718</v>
@@ -12506,8 +12480,8 @@
       <c r="L44" t="s">
         <v>713</v>
       </c>
-      <c r="M44" s="2">
-        <v>46369</v>
+      <c r="M44" s="1">
+        <v>46370</v>
       </c>
       <c r="N44" t="s">
         <v>718</v>
@@ -12550,8 +12524,8 @@
       <c r="L45" t="s">
         <v>713</v>
       </c>
-      <c r="M45" s="2">
-        <v>46369</v>
+      <c r="M45" s="1">
+        <v>46370</v>
       </c>
       <c r="N45" t="s">
         <v>718</v>
@@ -12676,8 +12650,8 @@
       <c r="L48" t="s">
         <v>713</v>
       </c>
-      <c r="M48" s="2">
-        <v>46369</v>
+      <c r="M48" s="1">
+        <v>46370</v>
       </c>
       <c r="N48" t="s">
         <v>718</v>
@@ -12720,8 +12694,8 @@
       <c r="L49" t="s">
         <v>717</v>
       </c>
-      <c r="M49" s="2">
-        <v>46324</v>
+      <c r="M49" s="1">
+        <v>46325</v>
       </c>
       <c r="N49" t="s">
         <v>718</v>
@@ -12764,8 +12738,8 @@
       <c r="L50" t="s">
         <v>717</v>
       </c>
-      <c r="M50" s="2">
-        <v>46324</v>
+      <c r="M50" s="1">
+        <v>46325</v>
       </c>
       <c r="N50" t="s">
         <v>718</v>
@@ -12808,8 +12782,8 @@
       <c r="L51" t="s">
         <v>713</v>
       </c>
-      <c r="M51" s="2">
-        <v>46369</v>
+      <c r="M51" s="1">
+        <v>46370</v>
       </c>
       <c r="N51" t="s">
         <v>718</v>
@@ -12852,8 +12826,8 @@
       <c r="L52" t="s">
         <v>713</v>
       </c>
-      <c r="M52" s="2">
-        <v>46369</v>
+      <c r="M52" s="1">
+        <v>46370</v>
       </c>
       <c r="N52" t="s">
         <v>718</v>
@@ -12896,8 +12870,8 @@
       <c r="L53" t="s">
         <v>713</v>
       </c>
-      <c r="M53" s="2">
-        <v>46369</v>
+      <c r="M53" s="1">
+        <v>46370</v>
       </c>
       <c r="N53" t="s">
         <v>718</v>
@@ -12940,8 +12914,8 @@
       <c r="L54" t="s">
         <v>713</v>
       </c>
-      <c r="M54" s="2">
-        <v>46369</v>
+      <c r="M54" s="1">
+        <v>46370</v>
       </c>
       <c r="N54" t="s">
         <v>718</v>
@@ -12984,8 +12958,8 @@
       <c r="L55" t="s">
         <v>713</v>
       </c>
-      <c r="M55" s="2">
-        <v>46369</v>
+      <c r="M55" s="1">
+        <v>46370</v>
       </c>
       <c r="N55" t="s">
         <v>718</v>
@@ -13028,8 +13002,8 @@
       <c r="L56" t="s">
         <v>717</v>
       </c>
-      <c r="M56" s="2">
-        <v>46324</v>
+      <c r="M56" s="1">
+        <v>46325</v>
       </c>
       <c r="N56" t="s">
         <v>718</v>
@@ -13072,8 +13046,8 @@
       <c r="L57" t="s">
         <v>717</v>
       </c>
-      <c r="M57" s="2">
-        <v>46324</v>
+      <c r="M57" s="1">
+        <v>46325</v>
       </c>
       <c r="N57" t="s">
         <v>718</v>
@@ -13116,8 +13090,8 @@
       <c r="L58" t="s">
         <v>717</v>
       </c>
-      <c r="M58" s="2">
-        <v>46324</v>
+      <c r="M58" s="1">
+        <v>46325</v>
       </c>
       <c r="N58" t="s">
         <v>718</v>
@@ -13160,8 +13134,8 @@
       <c r="L59" t="s">
         <v>713</v>
       </c>
-      <c r="M59" s="2">
-        <v>46369</v>
+      <c r="M59" s="1">
+        <v>46370</v>
       </c>
       <c r="N59" t="s">
         <v>718</v>
@@ -13204,8 +13178,8 @@
       <c r="L60" t="s">
         <v>717</v>
       </c>
-      <c r="M60" s="2">
-        <v>46324</v>
+      <c r="M60" s="1">
+        <v>46325</v>
       </c>
       <c r="N60" t="s">
         <v>718</v>
@@ -13248,8 +13222,8 @@
       <c r="L61" t="s">
         <v>717</v>
       </c>
-      <c r="M61" s="2">
-        <v>46324</v>
+      <c r="M61" s="1">
+        <v>46325</v>
       </c>
       <c r="N61" t="s">
         <v>718</v>
@@ -13292,8 +13266,8 @@
       <c r="L62" t="s">
         <v>713</v>
       </c>
-      <c r="M62" s="2">
-        <v>46369</v>
+      <c r="M62" s="1">
+        <v>46370</v>
       </c>
       <c r="N62" t="s">
         <v>718</v>
@@ -13336,8 +13310,8 @@
       <c r="L63" t="s">
         <v>713</v>
       </c>
-      <c r="M63" s="2">
-        <v>46369</v>
+      <c r="M63" s="1">
+        <v>46370</v>
       </c>
       <c r="N63" t="s">
         <v>718</v>
@@ -13380,8 +13354,8 @@
       <c r="L64" t="s">
         <v>713</v>
       </c>
-      <c r="M64" s="2">
-        <v>46369</v>
+      <c r="M64" s="1">
+        <v>46370</v>
       </c>
       <c r="N64" t="s">
         <v>718</v>
@@ -13424,8 +13398,8 @@
       <c r="L65" t="s">
         <v>713</v>
       </c>
-      <c r="M65" s="2">
-        <v>46369</v>
+      <c r="M65" s="1">
+        <v>46370</v>
       </c>
       <c r="N65" t="s">
         <v>718</v>
@@ -13468,8 +13442,8 @@
       <c r="L66" t="s">
         <v>713</v>
       </c>
-      <c r="M66" s="2">
-        <v>46369</v>
+      <c r="M66" s="1">
+        <v>46370</v>
       </c>
       <c r="N66" t="s">
         <v>718</v>
@@ -13512,8 +13486,8 @@
       <c r="L67" t="s">
         <v>713</v>
       </c>
-      <c r="M67" s="2">
-        <v>46369</v>
+      <c r="M67" s="1">
+        <v>46370</v>
       </c>
       <c r="N67" t="s">
         <v>718</v>
@@ -13556,8 +13530,8 @@
       <c r="L68" t="s">
         <v>713</v>
       </c>
-      <c r="M68" s="2">
-        <v>46369</v>
+      <c r="M68" s="1">
+        <v>46370</v>
       </c>
       <c r="N68" t="s">
         <v>718</v>
@@ -13600,8 +13574,8 @@
       <c r="L69" t="s">
         <v>713</v>
       </c>
-      <c r="M69" s="2">
-        <v>46369</v>
+      <c r="M69" s="1">
+        <v>46370</v>
       </c>
       <c r="N69" t="s">
         <v>718</v>
@@ -13644,8 +13618,8 @@
       <c r="L70" t="s">
         <v>713</v>
       </c>
-      <c r="M70" s="2">
-        <v>46369</v>
+      <c r="M70" s="1">
+        <v>46370</v>
       </c>
       <c r="N70" t="s">
         <v>718</v>
@@ -13688,8 +13662,8 @@
       <c r="L71" t="s">
         <v>713</v>
       </c>
-      <c r="M71" s="2">
-        <v>46369</v>
+      <c r="M71" s="1">
+        <v>46370</v>
       </c>
       <c r="N71" t="s">
         <v>718</v>
@@ -13732,8 +13706,8 @@
       <c r="L72" t="s">
         <v>713</v>
       </c>
-      <c r="M72" s="2">
-        <v>46369</v>
+      <c r="M72" s="1">
+        <v>46370</v>
       </c>
       <c r="N72" t="s">
         <v>718</v>
@@ -13776,8 +13750,8 @@
       <c r="L73" t="s">
         <v>713</v>
       </c>
-      <c r="M73" s="2">
-        <v>46369</v>
+      <c r="M73" s="1">
+        <v>46370</v>
       </c>
       <c r="N73" t="s">
         <v>718</v>
@@ -13820,8 +13794,8 @@
       <c r="L74" t="s">
         <v>713</v>
       </c>
-      <c r="M74" s="2">
-        <v>46369</v>
+      <c r="M74" s="1">
+        <v>46370</v>
       </c>
       <c r="N74" t="s">
         <v>718</v>
@@ -13864,8 +13838,8 @@
       <c r="L75" t="s">
         <v>713</v>
       </c>
-      <c r="M75" s="2">
-        <v>46369</v>
+      <c r="M75" s="1">
+        <v>46370</v>
       </c>
       <c r="N75" t="s">
         <v>718</v>
@@ -13905,8 +13879,8 @@
       <c r="L76" t="s">
         <v>716</v>
       </c>
-      <c r="M76" s="2">
-        <v>46384</v>
+      <c r="M76" s="1">
+        <v>46385</v>
       </c>
       <c r="N76" t="s">
         <v>718</v>
@@ -13946,8 +13920,8 @@
       <c r="L77" t="s">
         <v>713</v>
       </c>
-      <c r="M77" s="2">
-        <v>46369</v>
+      <c r="M77" s="1">
+        <v>46370</v>
       </c>
       <c r="N77" t="s">
         <v>718</v>
@@ -13990,8 +13964,8 @@
       <c r="L78" t="s">
         <v>713</v>
       </c>
-      <c r="M78" s="2">
-        <v>46369</v>
+      <c r="M78" s="1">
+        <v>46370</v>
       </c>
       <c r="N78" t="s">
         <v>718</v>
@@ -14034,8 +14008,8 @@
       <c r="L79" t="s">
         <v>713</v>
       </c>
-      <c r="M79" s="2">
-        <v>46369</v>
+      <c r="M79" s="1">
+        <v>46370</v>
       </c>
       <c r="N79" t="s">
         <v>718</v>
@@ -14078,8 +14052,8 @@
       <c r="L80" t="s">
         <v>713</v>
       </c>
-      <c r="M80" s="2">
-        <v>46369</v>
+      <c r="M80" s="1">
+        <v>46370</v>
       </c>
       <c r="N80" t="s">
         <v>718</v>
@@ -14122,8 +14096,8 @@
       <c r="L81" t="s">
         <v>716</v>
       </c>
-      <c r="M81" s="2">
-        <v>46384</v>
+      <c r="M81" s="1">
+        <v>46385</v>
       </c>
       <c r="N81" t="s">
         <v>718</v>
@@ -14166,8 +14140,8 @@
       <c r="L82" t="s">
         <v>713</v>
       </c>
-      <c r="M82" s="2">
-        <v>46369</v>
+      <c r="M82" s="1">
+        <v>46370</v>
       </c>
       <c r="N82" t="s">
         <v>718</v>
@@ -14210,8 +14184,8 @@
       <c r="L83" t="s">
         <v>713</v>
       </c>
-      <c r="M83" s="2">
-        <v>46369</v>
+      <c r="M83" s="1">
+        <v>46370</v>
       </c>
       <c r="N83" t="s">
         <v>718</v>
@@ -14254,8 +14228,8 @@
       <c r="L84" t="s">
         <v>713</v>
       </c>
-      <c r="M84" s="2">
-        <v>46369</v>
+      <c r="M84" s="1">
+        <v>46370</v>
       </c>
       <c r="N84" t="s">
         <v>718</v>
@@ -14298,8 +14272,8 @@
       <c r="L85" t="s">
         <v>713</v>
       </c>
-      <c r="M85" s="2">
-        <v>46369</v>
+      <c r="M85" s="1">
+        <v>46370</v>
       </c>
       <c r="N85" t="s">
         <v>718</v>
@@ -14342,8 +14316,8 @@
       <c r="L86" t="s">
         <v>713</v>
       </c>
-      <c r="M86" s="2">
-        <v>46369</v>
+      <c r="M86" s="1">
+        <v>46370</v>
       </c>
       <c r="N86" t="s">
         <v>718</v>
@@ -14386,8 +14360,8 @@
       <c r="L87" t="s">
         <v>713</v>
       </c>
-      <c r="M87" s="2">
-        <v>46369</v>
+      <c r="M87" s="1">
+        <v>46370</v>
       </c>
       <c r="N87" t="s">
         <v>718</v>
@@ -14430,8 +14404,8 @@
       <c r="L88" t="s">
         <v>716</v>
       </c>
-      <c r="M88" s="2">
-        <v>46384</v>
+      <c r="M88" s="1">
+        <v>46385</v>
       </c>
       <c r="N88" t="s">
         <v>718</v>
@@ -14474,8 +14448,8 @@
       <c r="L89" t="s">
         <v>713</v>
       </c>
-      <c r="M89" s="2">
-        <v>46369</v>
+      <c r="M89" s="1">
+        <v>46370</v>
       </c>
       <c r="N89" t="s">
         <v>718</v>
@@ -14518,8 +14492,8 @@
       <c r="L90" t="s">
         <v>716</v>
       </c>
-      <c r="M90" s="2">
-        <v>46384</v>
+      <c r="M90" s="1">
+        <v>46385</v>
       </c>
       <c r="N90" t="s">
         <v>718</v>
@@ -14562,8 +14536,8 @@
       <c r="L91" t="s">
         <v>716</v>
       </c>
-      <c r="M91" s="2">
-        <v>46384</v>
+      <c r="M91" s="1">
+        <v>46385</v>
       </c>
       <c r="N91" t="s">
         <v>718</v>
@@ -14606,8 +14580,8 @@
       <c r="L92" t="s">
         <v>713</v>
       </c>
-      <c r="M92" s="2">
-        <v>46369</v>
+      <c r="M92" s="1">
+        <v>46370</v>
       </c>
       <c r="N92" t="s">
         <v>718</v>
@@ -14650,8 +14624,8 @@
       <c r="L93" t="s">
         <v>716</v>
       </c>
-      <c r="M93" s="2">
-        <v>46384</v>
+      <c r="M93" s="1">
+        <v>46385</v>
       </c>
       <c r="N93" t="s">
         <v>718</v>
@@ -14694,8 +14668,8 @@
       <c r="L94" t="s">
         <v>716</v>
       </c>
-      <c r="M94" s="2">
-        <v>46384</v>
+      <c r="M94" s="1">
+        <v>46385</v>
       </c>
       <c r="N94" t="s">
         <v>718</v>
@@ -14738,8 +14712,8 @@
       <c r="L95" t="s">
         <v>716</v>
       </c>
-      <c r="M95" s="2">
-        <v>46384</v>
+      <c r="M95" s="1">
+        <v>46385</v>
       </c>
       <c r="N95" t="s">
         <v>718</v>
@@ -14782,8 +14756,8 @@
       <c r="L96" t="s">
         <v>716</v>
       </c>
-      <c r="M96" s="2">
-        <v>46384</v>
+      <c r="M96" s="1">
+        <v>46385</v>
       </c>
       <c r="N96" t="s">
         <v>718</v>
@@ -14826,8 +14800,8 @@
       <c r="L97" t="s">
         <v>713</v>
       </c>
-      <c r="M97" s="2">
-        <v>46369</v>
+      <c r="M97" s="1">
+        <v>46370</v>
       </c>
       <c r="N97" t="s">
         <v>718</v>
@@ -14870,8 +14844,8 @@
       <c r="L98" t="s">
         <v>713</v>
       </c>
-      <c r="M98" s="2">
-        <v>46369</v>
+      <c r="M98" s="1">
+        <v>46370</v>
       </c>
       <c r="N98" t="s">
         <v>718</v>
@@ -14914,8 +14888,8 @@
       <c r="L99" t="s">
         <v>713</v>
       </c>
-      <c r="M99" s="2">
-        <v>46369</v>
+      <c r="M99" s="1">
+        <v>46370</v>
       </c>
       <c r="N99" t="s">
         <v>718</v>
@@ -14958,8 +14932,8 @@
       <c r="L100" t="s">
         <v>716</v>
       </c>
-      <c r="M100" s="2">
-        <v>46384</v>
+      <c r="M100" s="1">
+        <v>46385</v>
       </c>
       <c r="N100" t="s">
         <v>718</v>
@@ -15002,8 +14976,8 @@
       <c r="L101" t="s">
         <v>713</v>
       </c>
-      <c r="M101" s="2">
-        <v>46369</v>
+      <c r="M101" s="1">
+        <v>46370</v>
       </c>
       <c r="N101" t="s">
         <v>718</v>
@@ -15046,8 +15020,8 @@
       <c r="L102" t="s">
         <v>713</v>
       </c>
-      <c r="M102" s="2">
-        <v>46369</v>
+      <c r="M102" s="1">
+        <v>46370</v>
       </c>
       <c r="N102" t="s">
         <v>718</v>
@@ -15090,8 +15064,8 @@
       <c r="L103" t="s">
         <v>716</v>
       </c>
-      <c r="M103" s="2">
-        <v>46384</v>
+      <c r="M103" s="1">
+        <v>46385</v>
       </c>
       <c r="N103" t="s">
         <v>718</v>
@@ -15134,8 +15108,8 @@
       <c r="L104" t="s">
         <v>713</v>
       </c>
-      <c r="M104" s="2">
-        <v>46369</v>
+      <c r="M104" s="1">
+        <v>46370</v>
       </c>
       <c r="N104" t="s">
         <v>718</v>
@@ -15178,8 +15152,8 @@
       <c r="L105" t="s">
         <v>716</v>
       </c>
-      <c r="M105" s="2">
-        <v>46384</v>
+      <c r="M105" s="1">
+        <v>46385</v>
       </c>
       <c r="N105" t="s">
         <v>718</v>
@@ -15222,8 +15196,8 @@
       <c r="L106" t="s">
         <v>716</v>
       </c>
-      <c r="M106" s="2">
-        <v>46384</v>
+      <c r="M106" s="1">
+        <v>46385</v>
       </c>
       <c r="N106" t="s">
         <v>718</v>
@@ -15266,8 +15240,8 @@
       <c r="L107" t="s">
         <v>716</v>
       </c>
-      <c r="M107" s="2">
-        <v>46384</v>
+      <c r="M107" s="1">
+        <v>46385</v>
       </c>
       <c r="N107" t="s">
         <v>718</v>
@@ -15310,8 +15284,8 @@
       <c r="L108" t="s">
         <v>713</v>
       </c>
-      <c r="M108" s="2">
-        <v>46369</v>
+      <c r="M108" s="1">
+        <v>46370</v>
       </c>
       <c r="N108" t="s">
         <v>718</v>
@@ -15354,8 +15328,8 @@
       <c r="L109" t="s">
         <v>713</v>
       </c>
-      <c r="M109" s="2">
-        <v>46369</v>
+      <c r="M109" s="1">
+        <v>46370</v>
       </c>
       <c r="N109" t="s">
         <v>718</v>
@@ -15398,8 +15372,8 @@
       <c r="L110" t="s">
         <v>713</v>
       </c>
-      <c r="M110" s="2">
-        <v>46369</v>
+      <c r="M110" s="1">
+        <v>46370</v>
       </c>
       <c r="N110" t="s">
         <v>718</v>
@@ -15442,8 +15416,8 @@
       <c r="L111" t="s">
         <v>713</v>
       </c>
-      <c r="M111" s="2">
-        <v>46369</v>
+      <c r="M111" s="1">
+        <v>46370</v>
       </c>
       <c r="N111" t="s">
         <v>718</v>
@@ -15486,8 +15460,8 @@
       <c r="L112" t="s">
         <v>713</v>
       </c>
-      <c r="M112" s="2">
-        <v>46369</v>
+      <c r="M112" s="1">
+        <v>46370</v>
       </c>
       <c r="N112" t="s">
         <v>718</v>
@@ -15530,8 +15504,8 @@
       <c r="L113" t="s">
         <v>713</v>
       </c>
-      <c r="M113" s="2">
-        <v>46369</v>
+      <c r="M113" s="1">
+        <v>46370</v>
       </c>
       <c r="N113" t="s">
         <v>718</v>
@@ -15574,8 +15548,8 @@
       <c r="L114" t="s">
         <v>713</v>
       </c>
-      <c r="M114" s="2">
-        <v>46369</v>
+      <c r="M114" s="1">
+        <v>46370</v>
       </c>
       <c r="N114" t="s">
         <v>718</v>
@@ -15618,8 +15592,8 @@
       <c r="L115" t="s">
         <v>713</v>
       </c>
-      <c r="M115" s="2">
-        <v>46369</v>
+      <c r="M115" s="1">
+        <v>46370</v>
       </c>
       <c r="N115" t="s">
         <v>718</v>
@@ -15662,8 +15636,8 @@
       <c r="L116" t="s">
         <v>713</v>
       </c>
-      <c r="M116" s="2">
-        <v>46369</v>
+      <c r="M116" s="1">
+        <v>46370</v>
       </c>
       <c r="N116" t="s">
         <v>718</v>
@@ -15706,8 +15680,8 @@
       <c r="L117" t="s">
         <v>713</v>
       </c>
-      <c r="M117" s="2">
-        <v>46369</v>
+      <c r="M117" s="1">
+        <v>46370</v>
       </c>
       <c r="N117" t="s">
         <v>718</v>
@@ -15750,8 +15724,8 @@
       <c r="L118" t="s">
         <v>713</v>
       </c>
-      <c r="M118" s="2">
-        <v>46369</v>
+      <c r="M118" s="1">
+        <v>46370</v>
       </c>
       <c r="N118" t="s">
         <v>718</v>
@@ -15794,8 +15768,8 @@
       <c r="L119" t="s">
         <v>713</v>
       </c>
-      <c r="M119" s="2">
-        <v>46369</v>
+      <c r="M119" s="1">
+        <v>46370</v>
       </c>
       <c r="N119" t="s">
         <v>718</v>
@@ -15838,8 +15812,8 @@
       <c r="L120" t="s">
         <v>713</v>
       </c>
-      <c r="M120" s="2">
-        <v>46369</v>
+      <c r="M120" s="1">
+        <v>46370</v>
       </c>
       <c r="N120" t="s">
         <v>718</v>
@@ -15879,8 +15853,8 @@
       <c r="L121" t="s">
         <v>382</v>
       </c>
-      <c r="M121" s="2">
-        <v>46374</v>
+      <c r="M121" s="1">
+        <v>46375</v>
       </c>
       <c r="N121" t="s">
         <v>718</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (01/10/2026 14:22)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -11045,7 +11045,7 @@
         <v>716</v>
       </c>
       <c r="M10" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N10" t="s">
         <v>718</v>
@@ -11089,7 +11089,7 @@
         <v>716</v>
       </c>
       <c r="M11" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N11" t="s">
         <v>718</v>
@@ -11297,7 +11297,7 @@
         <v>716</v>
       </c>
       <c r="M16" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N16" t="s">
         <v>718</v>
@@ -11382,7 +11382,7 @@
         <v>716</v>
       </c>
       <c r="M18" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N18" t="s">
         <v>718</v>
@@ -11426,7 +11426,7 @@
         <v>713</v>
       </c>
       <c r="M19" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N19" t="s">
         <v>718</v>
@@ -11470,7 +11470,7 @@
         <v>716</v>
       </c>
       <c r="M20" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N20" t="s">
         <v>718</v>
@@ -11514,7 +11514,7 @@
         <v>713</v>
       </c>
       <c r="M21" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N21" t="s">
         <v>718</v>
@@ -11681,7 +11681,7 @@
         <v>713</v>
       </c>
       <c r="M25" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N25" t="s">
         <v>718</v>
@@ -11807,7 +11807,7 @@
         <v>713</v>
       </c>
       <c r="M28" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N28" t="s">
         <v>718</v>
@@ -11851,7 +11851,7 @@
         <v>717</v>
       </c>
       <c r="M29" s="1">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="N29" t="s">
         <v>718</v>
@@ -11895,7 +11895,7 @@
         <v>713</v>
       </c>
       <c r="M30" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N30" t="s">
         <v>718</v>
@@ -11939,7 +11939,7 @@
         <v>717</v>
       </c>
       <c r="M31" s="1">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="N31" t="s">
         <v>718</v>
@@ -12352,7 +12352,7 @@
         <v>713</v>
       </c>
       <c r="M41" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N41" t="s">
         <v>718</v>
@@ -12437,7 +12437,7 @@
         <v>713</v>
       </c>
       <c r="M43" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N43" t="s">
         <v>718</v>
@@ -12481,7 +12481,7 @@
         <v>713</v>
       </c>
       <c r="M44" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N44" t="s">
         <v>718</v>
@@ -12525,7 +12525,7 @@
         <v>713</v>
       </c>
       <c r="M45" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N45" t="s">
         <v>718</v>
@@ -12651,7 +12651,7 @@
         <v>713</v>
       </c>
       <c r="M48" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N48" t="s">
         <v>718</v>
@@ -12695,7 +12695,7 @@
         <v>717</v>
       </c>
       <c r="M49" s="1">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="N49" t="s">
         <v>718</v>
@@ -12739,7 +12739,7 @@
         <v>717</v>
       </c>
       <c r="M50" s="1">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="N50" t="s">
         <v>718</v>
@@ -12783,7 +12783,7 @@
         <v>713</v>
       </c>
       <c r="M51" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N51" t="s">
         <v>718</v>
@@ -12827,7 +12827,7 @@
         <v>713</v>
       </c>
       <c r="M52" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N52" t="s">
         <v>718</v>
@@ -12871,7 +12871,7 @@
         <v>713</v>
       </c>
       <c r="M53" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N53" t="s">
         <v>718</v>
@@ -12915,7 +12915,7 @@
         <v>713</v>
       </c>
       <c r="M54" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N54" t="s">
         <v>718</v>
@@ -12959,7 +12959,7 @@
         <v>713</v>
       </c>
       <c r="M55" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N55" t="s">
         <v>718</v>
@@ -13003,7 +13003,7 @@
         <v>717</v>
       </c>
       <c r="M56" s="1">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="N56" t="s">
         <v>718</v>
@@ -13047,7 +13047,7 @@
         <v>717</v>
       </c>
       <c r="M57" s="1">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="N57" t="s">
         <v>718</v>
@@ -13091,7 +13091,7 @@
         <v>717</v>
       </c>
       <c r="M58" s="1">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="N58" t="s">
         <v>718</v>
@@ -13135,7 +13135,7 @@
         <v>713</v>
       </c>
       <c r="M59" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N59" t="s">
         <v>718</v>
@@ -13179,7 +13179,7 @@
         <v>717</v>
       </c>
       <c r="M60" s="1">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="N60" t="s">
         <v>718</v>
@@ -13223,7 +13223,7 @@
         <v>717</v>
       </c>
       <c r="M61" s="1">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="N61" t="s">
         <v>718</v>
@@ -13267,7 +13267,7 @@
         <v>713</v>
       </c>
       <c r="M62" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N62" t="s">
         <v>718</v>
@@ -13311,7 +13311,7 @@
         <v>713</v>
       </c>
       <c r="M63" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N63" t="s">
         <v>718</v>
@@ -13355,7 +13355,7 @@
         <v>713</v>
       </c>
       <c r="M64" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N64" t="s">
         <v>718</v>
@@ -13399,7 +13399,7 @@
         <v>713</v>
       </c>
       <c r="M65" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N65" t="s">
         <v>718</v>
@@ -13443,7 +13443,7 @@
         <v>713</v>
       </c>
       <c r="M66" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N66" t="s">
         <v>718</v>
@@ -13487,7 +13487,7 @@
         <v>713</v>
       </c>
       <c r="M67" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N67" t="s">
         <v>718</v>
@@ -13531,7 +13531,7 @@
         <v>713</v>
       </c>
       <c r="M68" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N68" t="s">
         <v>718</v>
@@ -13575,7 +13575,7 @@
         <v>713</v>
       </c>
       <c r="M69" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N69" t="s">
         <v>718</v>
@@ -13619,7 +13619,7 @@
         <v>713</v>
       </c>
       <c r="M70" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N70" t="s">
         <v>718</v>
@@ -13663,7 +13663,7 @@
         <v>713</v>
       </c>
       <c r="M71" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N71" t="s">
         <v>718</v>
@@ -13707,7 +13707,7 @@
         <v>713</v>
       </c>
       <c r="M72" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N72" t="s">
         <v>718</v>
@@ -13751,7 +13751,7 @@
         <v>713</v>
       </c>
       <c r="M73" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N73" t="s">
         <v>718</v>
@@ -13795,7 +13795,7 @@
         <v>713</v>
       </c>
       <c r="M74" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N74" t="s">
         <v>718</v>
@@ -13839,7 +13839,7 @@
         <v>713</v>
       </c>
       <c r="M75" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N75" t="s">
         <v>718</v>
@@ -13880,7 +13880,7 @@
         <v>716</v>
       </c>
       <c r="M76" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N76" t="s">
         <v>718</v>
@@ -13921,7 +13921,7 @@
         <v>713</v>
       </c>
       <c r="M77" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N77" t="s">
         <v>718</v>
@@ -13965,7 +13965,7 @@
         <v>713</v>
       </c>
       <c r="M78" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N78" t="s">
         <v>718</v>
@@ -14009,7 +14009,7 @@
         <v>713</v>
       </c>
       <c r="M79" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N79" t="s">
         <v>718</v>
@@ -14053,7 +14053,7 @@
         <v>713</v>
       </c>
       <c r="M80" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N80" t="s">
         <v>718</v>
@@ -14097,7 +14097,7 @@
         <v>716</v>
       </c>
       <c r="M81" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N81" t="s">
         <v>718</v>
@@ -14141,7 +14141,7 @@
         <v>713</v>
       </c>
       <c r="M82" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N82" t="s">
         <v>718</v>
@@ -14185,7 +14185,7 @@
         <v>713</v>
       </c>
       <c r="M83" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N83" t="s">
         <v>718</v>
@@ -14229,7 +14229,7 @@
         <v>713</v>
       </c>
       <c r="M84" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N84" t="s">
         <v>718</v>
@@ -14273,7 +14273,7 @@
         <v>713</v>
       </c>
       <c r="M85" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N85" t="s">
         <v>718</v>
@@ -14317,7 +14317,7 @@
         <v>713</v>
       </c>
       <c r="M86" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N86" t="s">
         <v>718</v>
@@ -14361,7 +14361,7 @@
         <v>713</v>
       </c>
       <c r="M87" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N87" t="s">
         <v>718</v>
@@ -14405,7 +14405,7 @@
         <v>716</v>
       </c>
       <c r="M88" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N88" t="s">
         <v>718</v>
@@ -14449,7 +14449,7 @@
         <v>713</v>
       </c>
       <c r="M89" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N89" t="s">
         <v>718</v>
@@ -14493,7 +14493,7 @@
         <v>716</v>
       </c>
       <c r="M90" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N90" t="s">
         <v>718</v>
@@ -14537,7 +14537,7 @@
         <v>716</v>
       </c>
       <c r="M91" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N91" t="s">
         <v>718</v>
@@ -14581,7 +14581,7 @@
         <v>713</v>
       </c>
       <c r="M92" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N92" t="s">
         <v>718</v>
@@ -14625,7 +14625,7 @@
         <v>716</v>
       </c>
       <c r="M93" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N93" t="s">
         <v>718</v>
@@ -14669,7 +14669,7 @@
         <v>716</v>
       </c>
       <c r="M94" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N94" t="s">
         <v>718</v>
@@ -14713,7 +14713,7 @@
         <v>716</v>
       </c>
       <c r="M95" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N95" t="s">
         <v>718</v>
@@ -14757,7 +14757,7 @@
         <v>716</v>
       </c>
       <c r="M96" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N96" t="s">
         <v>718</v>
@@ -14801,7 +14801,7 @@
         <v>713</v>
       </c>
       <c r="M97" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N97" t="s">
         <v>718</v>
@@ -14845,7 +14845,7 @@
         <v>713</v>
       </c>
       <c r="M98" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N98" t="s">
         <v>718</v>
@@ -14889,7 +14889,7 @@
         <v>713</v>
       </c>
       <c r="M99" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N99" t="s">
         <v>718</v>
@@ -14933,7 +14933,7 @@
         <v>716</v>
       </c>
       <c r="M100" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N100" t="s">
         <v>718</v>
@@ -14977,7 +14977,7 @@
         <v>713</v>
       </c>
       <c r="M101" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N101" t="s">
         <v>718</v>
@@ -15021,7 +15021,7 @@
         <v>713</v>
       </c>
       <c r="M102" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N102" t="s">
         <v>718</v>
@@ -15065,7 +15065,7 @@
         <v>716</v>
       </c>
       <c r="M103" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N103" t="s">
         <v>718</v>
@@ -15109,7 +15109,7 @@
         <v>713</v>
       </c>
       <c r="M104" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N104" t="s">
         <v>718</v>
@@ -15153,7 +15153,7 @@
         <v>716</v>
       </c>
       <c r="M105" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N105" t="s">
         <v>718</v>
@@ -15197,7 +15197,7 @@
         <v>716</v>
       </c>
       <c r="M106" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N106" t="s">
         <v>718</v>
@@ -15241,7 +15241,7 @@
         <v>716</v>
       </c>
       <c r="M107" s="1">
-        <v>46385</v>
+        <v>46386</v>
       </c>
       <c r="N107" t="s">
         <v>718</v>
@@ -15285,7 +15285,7 @@
         <v>713</v>
       </c>
       <c r="M108" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N108" t="s">
         <v>718</v>
@@ -15329,7 +15329,7 @@
         <v>713</v>
       </c>
       <c r="M109" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N109" t="s">
         <v>718</v>
@@ -15373,7 +15373,7 @@
         <v>713</v>
       </c>
       <c r="M110" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N110" t="s">
         <v>718</v>
@@ -15417,7 +15417,7 @@
         <v>713</v>
       </c>
       <c r="M111" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N111" t="s">
         <v>718</v>
@@ -15461,7 +15461,7 @@
         <v>713</v>
       </c>
       <c r="M112" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N112" t="s">
         <v>718</v>
@@ -15505,7 +15505,7 @@
         <v>713</v>
       </c>
       <c r="M113" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N113" t="s">
         <v>718</v>
@@ -15549,7 +15549,7 @@
         <v>713</v>
       </c>
       <c r="M114" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N114" t="s">
         <v>718</v>
@@ -15593,7 +15593,7 @@
         <v>713</v>
       </c>
       <c r="M115" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N115" t="s">
         <v>718</v>
@@ -15637,7 +15637,7 @@
         <v>713</v>
       </c>
       <c r="M116" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N116" t="s">
         <v>718</v>
@@ -15681,7 +15681,7 @@
         <v>713</v>
       </c>
       <c r="M117" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N117" t="s">
         <v>718</v>
@@ -15725,7 +15725,7 @@
         <v>713</v>
       </c>
       <c r="M118" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N118" t="s">
         <v>718</v>
@@ -15769,7 +15769,7 @@
         <v>713</v>
       </c>
       <c r="M119" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N119" t="s">
         <v>718</v>
@@ -15813,7 +15813,7 @@
         <v>713</v>
       </c>
       <c r="M120" s="1">
-        <v>46370</v>
+        <v>46371</v>
       </c>
       <c r="N120" t="s">
         <v>718</v>
@@ -15854,7 +15854,7 @@
         <v>382</v>
       </c>
       <c r="M121" s="1">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N121" t="s">
         <v>718</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (02/10/2026 09:57)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3093" uniqueCount="719">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3096" uniqueCount="718">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -2057,7 +2057,7 @@
     <t>ROD END</t>
   </si>
   <si>
-    <t>FITTING-WING STRUT LWR - Confirmation of the requested PN and condition of the material is required.</t>
+    <t>FITTING-WING STRUT LWR</t>
   </si>
   <si>
     <t>KIT CAB-33-02</t>
@@ -2166,9 +2166,6 @@
   </si>
   <si>
     <t>Análise do Pedido</t>
-  </si>
-  <si>
-    <t>Em Cotação</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -2181,8 +2178,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2198,7 +2203,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2206,12 +2211,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2511,55 +2534,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2603,7 +2626,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2647,7 +2670,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2691,7 +2714,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2817,7 +2840,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2861,7 +2884,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2905,7 +2928,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2952,7 +2975,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3075,7 +3098,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -3119,7 +3142,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3163,7 +3186,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3207,7 +3230,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3254,7 +3277,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3298,7 +3321,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3424,7 +3447,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3468,7 +3491,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3553,7 +3576,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3600,7 +3623,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3647,7 +3670,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3691,7 +3714,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3735,7 +3758,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3820,7 +3843,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3905,7 +3928,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3952,7 +3975,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3996,7 +4019,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4040,7 +4063,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4125,7 +4148,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4169,7 +4192,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4213,7 +4236,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4298,7 +4321,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4342,7 +4365,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4386,7 +4409,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4430,7 +4453,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4597,7 +4620,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4641,7 +4664,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4685,7 +4708,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4729,7 +4752,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4776,7 +4799,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4820,7 +4843,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4902,7 +4925,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4946,7 +4969,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5034,7 +5057,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5078,7 +5101,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5125,7 +5148,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5169,7 +5192,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -5213,7 +5236,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5257,7 +5280,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5301,7 +5324,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5348,7 +5371,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5392,7 +5415,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5439,7 +5462,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5483,7 +5506,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5530,7 +5553,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5618,7 +5641,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5662,7 +5685,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5706,7 +5729,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5750,7 +5773,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5794,7 +5817,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5838,7 +5861,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5923,7 +5946,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5967,7 +5990,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -6011,7 +6034,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -6055,7 +6078,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -6099,7 +6122,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -6143,7 +6166,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6187,7 +6210,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6231,7 +6254,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6278,7 +6301,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6322,7 +6345,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6366,7 +6389,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6410,7 +6433,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6454,7 +6477,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6498,7 +6521,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6542,7 +6565,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6586,7 +6609,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6630,7 +6653,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6718,7 +6741,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6762,7 +6785,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6888,7 +6911,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6932,7 +6955,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6976,7 +6999,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7020,7 +7043,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7102,7 +7125,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7146,7 +7169,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7193,7 +7216,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7237,7 +7260,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7363,7 +7386,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7407,7 +7430,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7492,7 +7515,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7536,7 +7559,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7580,7 +7603,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7624,7 +7647,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7668,7 +7691,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7712,7 +7735,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7756,7 +7779,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7800,7 +7823,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7885,7 +7908,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8052,7 +8075,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8096,7 +8119,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8140,7 +8163,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8184,7 +8207,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8228,7 +8251,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8272,7 +8295,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8316,7 +8339,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8401,7 +8424,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8445,7 +8468,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8530,7 +8553,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8656,7 +8679,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8700,7 +8723,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8785,7 +8808,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8829,7 +8852,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8873,7 +8896,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8917,7 +8940,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8961,7 +8984,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -9005,7 +9028,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9049,7 +9072,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9093,7 +9116,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9178,7 +9201,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9345,7 +9368,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9389,7 +9412,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9433,7 +9456,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9477,7 +9500,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9562,7 +9585,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9606,7 +9629,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9650,7 +9673,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9694,7 +9717,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9738,7 +9761,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9782,7 +9805,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9826,7 +9849,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9870,7 +9893,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9914,7 +9937,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9958,7 +9981,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10002,7 +10025,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -10046,7 +10069,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10090,7 +10113,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10134,7 +10157,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -10178,7 +10201,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10222,7 +10245,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10266,7 +10289,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10310,7 +10333,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10354,7 +10377,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10398,7 +10421,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10442,7 +10465,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10527,7 +10550,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10612,7 +10635,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10627,55 +10650,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11036,19 +11059,19 @@
         <v>713</v>
       </c>
       <c r="J10" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="K10" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="L10" t="s">
-        <v>716</v>
-      </c>
-      <c r="M10" s="1">
-        <v>46386</v>
+        <v>713</v>
+      </c>
+      <c r="M10" s="2">
+        <v>46372</v>
       </c>
       <c r="N10" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -11080,19 +11103,19 @@
         <v>713</v>
       </c>
       <c r="J11" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="K11" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="L11" t="s">
-        <v>716</v>
-      </c>
-      <c r="M11" s="1">
-        <v>46386</v>
+        <v>713</v>
+      </c>
+      <c r="M11" s="2">
+        <v>46372</v>
       </c>
       <c r="N11" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -11247,13 +11270,13 @@
         <v>712</v>
       </c>
       <c r="J15" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="K15" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="L15" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="N15" t="s">
         <v>395</v>
@@ -11288,19 +11311,19 @@
         <v>713</v>
       </c>
       <c r="J16" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="K16" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="L16" t="s">
-        <v>716</v>
-      </c>
-      <c r="M16" s="1">
-        <v>46386</v>
+        <v>713</v>
+      </c>
+      <c r="M16" s="2">
+        <v>46372</v>
       </c>
       <c r="N16" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -11373,19 +11396,16 @@
         <v>381</v>
       </c>
       <c r="J18" t="s">
-        <v>716</v>
+        <v>381</v>
       </c>
       <c r="K18" t="s">
-        <v>716</v>
+        <v>381</v>
       </c>
       <c r="L18" t="s">
-        <v>716</v>
-      </c>
-      <c r="M18" s="1">
-        <v>46386</v>
+        <v>394</v>
       </c>
       <c r="N18" t="s">
-        <v>718</v>
+        <v>394</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -11425,11 +11445,11 @@
       <c r="L19" t="s">
         <v>713</v>
       </c>
-      <c r="M19" s="1">
-        <v>46371</v>
+      <c r="M19" s="2">
+        <v>46372</v>
       </c>
       <c r="N19" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11461,19 +11481,19 @@
         <v>714</v>
       </c>
       <c r="J20" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="K20" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="L20" t="s">
-        <v>716</v>
-      </c>
-      <c r="M20" s="1">
-        <v>46386</v>
+        <v>713</v>
+      </c>
+      <c r="M20" s="2">
+        <v>46372</v>
       </c>
       <c r="N20" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11513,11 +11533,11 @@
       <c r="L21" t="s">
         <v>713</v>
       </c>
-      <c r="M21" s="1">
-        <v>46371</v>
+      <c r="M21" s="2">
+        <v>46372</v>
       </c>
       <c r="N21" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11680,11 +11700,11 @@
       <c r="L25" t="s">
         <v>713</v>
       </c>
-      <c r="M25" s="1">
-        <v>46371</v>
+      <c r="M25" s="2">
+        <v>46372</v>
       </c>
       <c r="N25" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11806,11 +11826,11 @@
       <c r="L28" t="s">
         <v>713</v>
       </c>
-      <c r="M28" s="1">
-        <v>46371</v>
+      <c r="M28" s="2">
+        <v>46372</v>
       </c>
       <c r="N28" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11842,19 +11862,19 @@
         <v>715</v>
       </c>
       <c r="J29" t="s">
+        <v>715</v>
+      </c>
+      <c r="K29" t="s">
+        <v>715</v>
+      </c>
+      <c r="L29" t="s">
+        <v>715</v>
+      </c>
+      <c r="M29" s="2">
+        <v>46307</v>
+      </c>
+      <c r="N29" t="s">
         <v>717</v>
-      </c>
-      <c r="K29" t="s">
-        <v>717</v>
-      </c>
-      <c r="L29" t="s">
-        <v>717</v>
-      </c>
-      <c r="M29" s="1">
-        <v>46326</v>
-      </c>
-      <c r="N29" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11894,11 +11914,11 @@
       <c r="L30" t="s">
         <v>713</v>
       </c>
-      <c r="M30" s="1">
-        <v>46371</v>
+      <c r="M30" s="2">
+        <v>46372</v>
       </c>
       <c r="N30" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11930,19 +11950,19 @@
         <v>715</v>
       </c>
       <c r="J31" t="s">
+        <v>715</v>
+      </c>
+      <c r="K31" t="s">
+        <v>715</v>
+      </c>
+      <c r="L31" t="s">
+        <v>715</v>
+      </c>
+      <c r="M31" s="2">
+        <v>46307</v>
+      </c>
+      <c r="N31" t="s">
         <v>717</v>
-      </c>
-      <c r="K31" t="s">
-        <v>717</v>
-      </c>
-      <c r="L31" t="s">
-        <v>717</v>
-      </c>
-      <c r="M31" s="1">
-        <v>46326</v>
-      </c>
-      <c r="N31" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -12179,13 +12199,13 @@
         <v>712</v>
       </c>
       <c r="J37" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="K37" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="L37" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="N37" t="s">
         <v>395</v>
@@ -12351,11 +12371,11 @@
       <c r="L41" t="s">
         <v>713</v>
       </c>
-      <c r="M41" s="1">
-        <v>46371</v>
+      <c r="M41" s="2">
+        <v>46372</v>
       </c>
       <c r="N41" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -12387,13 +12407,13 @@
         <v>712</v>
       </c>
       <c r="J42" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="K42" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="L42" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="N42" t="s">
         <v>395</v>
@@ -12436,11 +12456,11 @@
       <c r="L43" t="s">
         <v>713</v>
       </c>
-      <c r="M43" s="1">
-        <v>46371</v>
+      <c r="M43" s="2">
+        <v>46372</v>
       </c>
       <c r="N43" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12480,11 +12500,11 @@
       <c r="L44" t="s">
         <v>713</v>
       </c>
-      <c r="M44" s="1">
-        <v>46371</v>
+      <c r="M44" s="2">
+        <v>46372</v>
       </c>
       <c r="N44" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12524,11 +12544,11 @@
       <c r="L45" t="s">
         <v>713</v>
       </c>
-      <c r="M45" s="1">
-        <v>46371</v>
+      <c r="M45" s="2">
+        <v>46372</v>
       </c>
       <c r="N45" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12650,11 +12670,11 @@
       <c r="L48" t="s">
         <v>713</v>
       </c>
-      <c r="M48" s="1">
-        <v>46371</v>
+      <c r="M48" s="2">
+        <v>46372</v>
       </c>
       <c r="N48" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12686,19 +12706,19 @@
         <v>715</v>
       </c>
       <c r="J49" t="s">
+        <v>715</v>
+      </c>
+      <c r="K49" t="s">
+        <v>715</v>
+      </c>
+      <c r="L49" t="s">
+        <v>715</v>
+      </c>
+      <c r="M49" s="2">
+        <v>46307</v>
+      </c>
+      <c r="N49" t="s">
         <v>717</v>
-      </c>
-      <c r="K49" t="s">
-        <v>717</v>
-      </c>
-      <c r="L49" t="s">
-        <v>717</v>
-      </c>
-      <c r="M49" s="1">
-        <v>46326</v>
-      </c>
-      <c r="N49" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12730,19 +12750,19 @@
         <v>715</v>
       </c>
       <c r="J50" t="s">
+        <v>715</v>
+      </c>
+      <c r="K50" t="s">
+        <v>715</v>
+      </c>
+      <c r="L50" t="s">
+        <v>715</v>
+      </c>
+      <c r="M50" s="2">
+        <v>46307</v>
+      </c>
+      <c r="N50" t="s">
         <v>717</v>
-      </c>
-      <c r="K50" t="s">
-        <v>717</v>
-      </c>
-      <c r="L50" t="s">
-        <v>717</v>
-      </c>
-      <c r="M50" s="1">
-        <v>46326</v>
-      </c>
-      <c r="N50" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12782,11 +12802,11 @@
       <c r="L51" t="s">
         <v>713</v>
       </c>
-      <c r="M51" s="1">
-        <v>46371</v>
+      <c r="M51" s="2">
+        <v>46372</v>
       </c>
       <c r="N51" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12826,11 +12846,11 @@
       <c r="L52" t="s">
         <v>713</v>
       </c>
-      <c r="M52" s="1">
-        <v>46371</v>
+      <c r="M52" s="2">
+        <v>46372</v>
       </c>
       <c r="N52" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12870,11 +12890,11 @@
       <c r="L53" t="s">
         <v>713</v>
       </c>
-      <c r="M53" s="1">
-        <v>46371</v>
+      <c r="M53" s="2">
+        <v>46372</v>
       </c>
       <c r="N53" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12914,11 +12934,11 @@
       <c r="L54" t="s">
         <v>713</v>
       </c>
-      <c r="M54" s="1">
-        <v>46371</v>
+      <c r="M54" s="2">
+        <v>46372</v>
       </c>
       <c r="N54" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12950,19 +12970,19 @@
         <v>716</v>
       </c>
       <c r="J55" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="K55" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="L55" t="s">
-        <v>713</v>
-      </c>
-      <c r="M55" s="1">
-        <v>46371</v>
+        <v>716</v>
+      </c>
+      <c r="M55" s="2">
+        <v>46387</v>
       </c>
       <c r="N55" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -12994,19 +13014,19 @@
         <v>715</v>
       </c>
       <c r="J56" t="s">
+        <v>715</v>
+      </c>
+      <c r="K56" t="s">
+        <v>715</v>
+      </c>
+      <c r="L56" t="s">
+        <v>715</v>
+      </c>
+      <c r="M56" s="2">
+        <v>46307</v>
+      </c>
+      <c r="N56" t="s">
         <v>717</v>
-      </c>
-      <c r="K56" t="s">
-        <v>717</v>
-      </c>
-      <c r="L56" t="s">
-        <v>717</v>
-      </c>
-      <c r="M56" s="1">
-        <v>46326</v>
-      </c>
-      <c r="N56" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -13038,19 +13058,19 @@
         <v>715</v>
       </c>
       <c r="J57" t="s">
+        <v>715</v>
+      </c>
+      <c r="K57" t="s">
+        <v>715</v>
+      </c>
+      <c r="L57" t="s">
+        <v>715</v>
+      </c>
+      <c r="M57" s="2">
+        <v>46307</v>
+      </c>
+      <c r="N57" t="s">
         <v>717</v>
-      </c>
-      <c r="K57" t="s">
-        <v>717</v>
-      </c>
-      <c r="L57" t="s">
-        <v>717</v>
-      </c>
-      <c r="M57" s="1">
-        <v>46326</v>
-      </c>
-      <c r="N57" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -13082,19 +13102,19 @@
         <v>715</v>
       </c>
       <c r="J58" t="s">
+        <v>715</v>
+      </c>
+      <c r="K58" t="s">
+        <v>715</v>
+      </c>
+      <c r="L58" t="s">
+        <v>715</v>
+      </c>
+      <c r="M58" s="2">
+        <v>46307</v>
+      </c>
+      <c r="N58" t="s">
         <v>717</v>
-      </c>
-      <c r="K58" t="s">
-        <v>717</v>
-      </c>
-      <c r="L58" t="s">
-        <v>717</v>
-      </c>
-      <c r="M58" s="1">
-        <v>46326</v>
-      </c>
-      <c r="N58" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -13134,11 +13154,11 @@
       <c r="L59" t="s">
         <v>713</v>
       </c>
-      <c r="M59" s="1">
-        <v>46371</v>
+      <c r="M59" s="2">
+        <v>46372</v>
       </c>
       <c r="N59" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -13170,19 +13190,19 @@
         <v>715</v>
       </c>
       <c r="J60" t="s">
+        <v>715</v>
+      </c>
+      <c r="K60" t="s">
+        <v>715</v>
+      </c>
+      <c r="L60" t="s">
+        <v>715</v>
+      </c>
+      <c r="M60" s="2">
+        <v>46307</v>
+      </c>
+      <c r="N60" t="s">
         <v>717</v>
-      </c>
-      <c r="K60" t="s">
-        <v>717</v>
-      </c>
-      <c r="L60" t="s">
-        <v>717</v>
-      </c>
-      <c r="M60" s="1">
-        <v>46326</v>
-      </c>
-      <c r="N60" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="61" spans="1:14">
@@ -13214,19 +13234,19 @@
         <v>715</v>
       </c>
       <c r="J61" t="s">
+        <v>715</v>
+      </c>
+      <c r="K61" t="s">
+        <v>715</v>
+      </c>
+      <c r="L61" t="s">
+        <v>715</v>
+      </c>
+      <c r="M61" s="2">
+        <v>46307</v>
+      </c>
+      <c r="N61" t="s">
         <v>717</v>
-      </c>
-      <c r="K61" t="s">
-        <v>717</v>
-      </c>
-      <c r="L61" t="s">
-        <v>717</v>
-      </c>
-      <c r="M61" s="1">
-        <v>46326</v>
-      </c>
-      <c r="N61" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="62" spans="1:14">
@@ -13266,11 +13286,11 @@
       <c r="L62" t="s">
         <v>713</v>
       </c>
-      <c r="M62" s="1">
-        <v>46371</v>
+      <c r="M62" s="2">
+        <v>46372</v>
       </c>
       <c r="N62" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="63" spans="1:14">
@@ -13310,11 +13330,11 @@
       <c r="L63" t="s">
         <v>713</v>
       </c>
-      <c r="M63" s="1">
-        <v>46371</v>
+      <c r="M63" s="2">
+        <v>46372</v>
       </c>
       <c r="N63" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="64" spans="1:14">
@@ -13354,11 +13374,11 @@
       <c r="L64" t="s">
         <v>713</v>
       </c>
-      <c r="M64" s="1">
-        <v>46371</v>
+      <c r="M64" s="2">
+        <v>46372</v>
       </c>
       <c r="N64" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="65" spans="1:14">
@@ -13398,11 +13418,11 @@
       <c r="L65" t="s">
         <v>713</v>
       </c>
-      <c r="M65" s="1">
-        <v>46371</v>
+      <c r="M65" s="2">
+        <v>46372</v>
       </c>
       <c r="N65" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="66" spans="1:14">
@@ -13442,11 +13462,11 @@
       <c r="L66" t="s">
         <v>713</v>
       </c>
-      <c r="M66" s="1">
-        <v>46371</v>
+      <c r="M66" s="2">
+        <v>46372</v>
       </c>
       <c r="N66" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="67" spans="1:14">
@@ -13486,11 +13506,11 @@
       <c r="L67" t="s">
         <v>713</v>
       </c>
-      <c r="M67" s="1">
-        <v>46371</v>
+      <c r="M67" s="2">
+        <v>46372</v>
       </c>
       <c r="N67" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="68" spans="1:14">
@@ -13530,11 +13550,11 @@
       <c r="L68" t="s">
         <v>713</v>
       </c>
-      <c r="M68" s="1">
-        <v>46371</v>
+      <c r="M68" s="2">
+        <v>46372</v>
       </c>
       <c r="N68" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="69" spans="1:14">
@@ -13574,11 +13594,11 @@
       <c r="L69" t="s">
         <v>713</v>
       </c>
-      <c r="M69" s="1">
-        <v>46371</v>
+      <c r="M69" s="2">
+        <v>46372</v>
       </c>
       <c r="N69" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="70" spans="1:14">
@@ -13618,11 +13638,11 @@
       <c r="L70" t="s">
         <v>713</v>
       </c>
-      <c r="M70" s="1">
-        <v>46371</v>
+      <c r="M70" s="2">
+        <v>46372</v>
       </c>
       <c r="N70" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="71" spans="1:14">
@@ -13662,11 +13682,11 @@
       <c r="L71" t="s">
         <v>713</v>
       </c>
-      <c r="M71" s="1">
-        <v>46371</v>
+      <c r="M71" s="2">
+        <v>46372</v>
       </c>
       <c r="N71" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="72" spans="1:14">
@@ -13706,11 +13726,11 @@
       <c r="L72" t="s">
         <v>713</v>
       </c>
-      <c r="M72" s="1">
-        <v>46371</v>
+      <c r="M72" s="2">
+        <v>46372</v>
       </c>
       <c r="N72" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="73" spans="1:14">
@@ -13750,11 +13770,11 @@
       <c r="L73" t="s">
         <v>713</v>
       </c>
-      <c r="M73" s="1">
-        <v>46371</v>
+      <c r="M73" s="2">
+        <v>46372</v>
       </c>
       <c r="N73" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="74" spans="1:14">
@@ -13794,11 +13814,11 @@
       <c r="L74" t="s">
         <v>713</v>
       </c>
-      <c r="M74" s="1">
-        <v>46371</v>
+      <c r="M74" s="2">
+        <v>46372</v>
       </c>
       <c r="N74" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="75" spans="1:14">
@@ -13830,19 +13850,19 @@
         <v>716</v>
       </c>
       <c r="J75" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="K75" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="L75" t="s">
-        <v>713</v>
-      </c>
-      <c r="M75" s="1">
-        <v>46371</v>
+        <v>716</v>
+      </c>
+      <c r="M75" s="2">
+        <v>46387</v>
       </c>
       <c r="N75" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="76" spans="1:14">
@@ -13873,17 +13893,20 @@
       <c r="I76" t="s">
         <v>716</v>
       </c>
+      <c r="J76" t="s">
+        <v>716</v>
+      </c>
       <c r="K76" t="s">
         <v>716</v>
       </c>
       <c r="L76" t="s">
         <v>716</v>
       </c>
-      <c r="M76" s="1">
-        <v>46386</v>
+      <c r="M76" s="2">
+        <v>46387</v>
       </c>
       <c r="N76" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="77" spans="1:14">
@@ -13914,17 +13937,20 @@
       <c r="I77" t="s">
         <v>713</v>
       </c>
+      <c r="J77" t="s">
+        <v>713</v>
+      </c>
       <c r="K77" t="s">
         <v>713</v>
       </c>
       <c r="L77" t="s">
         <v>713</v>
       </c>
-      <c r="M77" s="1">
-        <v>46371</v>
+      <c r="M77" s="2">
+        <v>46372</v>
       </c>
       <c r="N77" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="78" spans="1:14">
@@ -13964,11 +13990,11 @@
       <c r="L78" t="s">
         <v>713</v>
       </c>
-      <c r="M78" s="1">
-        <v>46371</v>
+      <c r="M78" s="2">
+        <v>46372</v>
       </c>
       <c r="N78" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="79" spans="1:14">
@@ -14008,11 +14034,11 @@
       <c r="L79" t="s">
         <v>713</v>
       </c>
-      <c r="M79" s="1">
-        <v>46371</v>
+      <c r="M79" s="2">
+        <v>46372</v>
       </c>
       <c r="N79" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="80" spans="1:14">
@@ -14052,11 +14078,11 @@
       <c r="L80" t="s">
         <v>713</v>
       </c>
-      <c r="M80" s="1">
-        <v>46371</v>
+      <c r="M80" s="2">
+        <v>46372</v>
       </c>
       <c r="N80" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="81" spans="1:14">
@@ -14096,11 +14122,11 @@
       <c r="L81" t="s">
         <v>716</v>
       </c>
-      <c r="M81" s="1">
-        <v>46386</v>
+      <c r="M81" s="2">
+        <v>46387</v>
       </c>
       <c r="N81" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="82" spans="1:14">
@@ -14140,11 +14166,11 @@
       <c r="L82" t="s">
         <v>713</v>
       </c>
-      <c r="M82" s="1">
-        <v>46371</v>
+      <c r="M82" s="2">
+        <v>46372</v>
       </c>
       <c r="N82" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="83" spans="1:14">
@@ -14184,11 +14210,11 @@
       <c r="L83" t="s">
         <v>713</v>
       </c>
-      <c r="M83" s="1">
-        <v>46371</v>
+      <c r="M83" s="2">
+        <v>46372</v>
       </c>
       <c r="N83" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="84" spans="1:14">
@@ -14228,11 +14254,11 @@
       <c r="L84" t="s">
         <v>713</v>
       </c>
-      <c r="M84" s="1">
-        <v>46371</v>
+      <c r="M84" s="2">
+        <v>46372</v>
       </c>
       <c r="N84" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="85" spans="1:14">
@@ -14272,11 +14298,11 @@
       <c r="L85" t="s">
         <v>713</v>
       </c>
-      <c r="M85" s="1">
-        <v>46371</v>
+      <c r="M85" s="2">
+        <v>46372</v>
       </c>
       <c r="N85" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="86" spans="1:14">
@@ -14316,11 +14342,11 @@
       <c r="L86" t="s">
         <v>713</v>
       </c>
-      <c r="M86" s="1">
-        <v>46371</v>
+      <c r="M86" s="2">
+        <v>46372</v>
       </c>
       <c r="N86" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="87" spans="1:14">
@@ -14360,11 +14386,11 @@
       <c r="L87" t="s">
         <v>713</v>
       </c>
-      <c r="M87" s="1">
-        <v>46371</v>
+      <c r="M87" s="2">
+        <v>46372</v>
       </c>
       <c r="N87" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="88" spans="1:14">
@@ -14404,11 +14430,11 @@
       <c r="L88" t="s">
         <v>716</v>
       </c>
-      <c r="M88" s="1">
-        <v>46386</v>
+      <c r="M88" s="2">
+        <v>46387</v>
       </c>
       <c r="N88" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="89" spans="1:14">
@@ -14448,11 +14474,11 @@
       <c r="L89" t="s">
         <v>713</v>
       </c>
-      <c r="M89" s="1">
-        <v>46371</v>
+      <c r="M89" s="2">
+        <v>46372</v>
       </c>
       <c r="N89" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="90" spans="1:14">
@@ -14492,11 +14518,11 @@
       <c r="L90" t="s">
         <v>716</v>
       </c>
-      <c r="M90" s="1">
-        <v>46386</v>
+      <c r="M90" s="2">
+        <v>46387</v>
       </c>
       <c r="N90" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="91" spans="1:14">
@@ -14536,11 +14562,11 @@
       <c r="L91" t="s">
         <v>716</v>
       </c>
-      <c r="M91" s="1">
-        <v>46386</v>
+      <c r="M91" s="2">
+        <v>46387</v>
       </c>
       <c r="N91" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="92" spans="1:14">
@@ -14580,11 +14606,11 @@
       <c r="L92" t="s">
         <v>713</v>
       </c>
-      <c r="M92" s="1">
-        <v>46371</v>
+      <c r="M92" s="2">
+        <v>46372</v>
       </c>
       <c r="N92" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="93" spans="1:14">
@@ -14624,11 +14650,11 @@
       <c r="L93" t="s">
         <v>716</v>
       </c>
-      <c r="M93" s="1">
-        <v>46386</v>
+      <c r="M93" s="2">
+        <v>46387</v>
       </c>
       <c r="N93" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="94" spans="1:14">
@@ -14668,11 +14694,11 @@
       <c r="L94" t="s">
         <v>716</v>
       </c>
-      <c r="M94" s="1">
-        <v>46386</v>
+      <c r="M94" s="2">
+        <v>46387</v>
       </c>
       <c r="N94" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="95" spans="1:14">
@@ -14712,11 +14738,11 @@
       <c r="L95" t="s">
         <v>716</v>
       </c>
-      <c r="M95" s="1">
-        <v>46386</v>
+      <c r="M95" s="2">
+        <v>46387</v>
       </c>
       <c r="N95" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="96" spans="1:14">
@@ -14756,11 +14782,11 @@
       <c r="L96" t="s">
         <v>716</v>
       </c>
-      <c r="M96" s="1">
-        <v>46386</v>
+      <c r="M96" s="2">
+        <v>46387</v>
       </c>
       <c r="N96" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="97" spans="1:14">
@@ -14800,11 +14826,11 @@
       <c r="L97" t="s">
         <v>713</v>
       </c>
-      <c r="M97" s="1">
-        <v>46371</v>
+      <c r="M97" s="2">
+        <v>46372</v>
       </c>
       <c r="N97" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="98" spans="1:14">
@@ -14844,11 +14870,11 @@
       <c r="L98" t="s">
         <v>713</v>
       </c>
-      <c r="M98" s="1">
-        <v>46371</v>
+      <c r="M98" s="2">
+        <v>46372</v>
       </c>
       <c r="N98" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="99" spans="1:14">
@@ -14888,11 +14914,11 @@
       <c r="L99" t="s">
         <v>713</v>
       </c>
-      <c r="M99" s="1">
-        <v>46371</v>
+      <c r="M99" s="2">
+        <v>46372</v>
       </c>
       <c r="N99" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="100" spans="1:14">
@@ -14924,19 +14950,19 @@
         <v>716</v>
       </c>
       <c r="J100" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="K100" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="L100" t="s">
-        <v>716</v>
-      </c>
-      <c r="M100" s="1">
-        <v>46386</v>
+        <v>713</v>
+      </c>
+      <c r="M100" s="2">
+        <v>46372</v>
       </c>
       <c r="N100" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="101" spans="1:14">
@@ -14976,11 +15002,11 @@
       <c r="L101" t="s">
         <v>713</v>
       </c>
-      <c r="M101" s="1">
-        <v>46371</v>
+      <c r="M101" s="2">
+        <v>46372</v>
       </c>
       <c r="N101" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="102" spans="1:14">
@@ -15020,11 +15046,11 @@
       <c r="L102" t="s">
         <v>713</v>
       </c>
-      <c r="M102" s="1">
-        <v>46371</v>
+      <c r="M102" s="2">
+        <v>46372</v>
       </c>
       <c r="N102" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="103" spans="1:14">
@@ -15056,19 +15082,19 @@
         <v>716</v>
       </c>
       <c r="J103" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="K103" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="L103" t="s">
-        <v>716</v>
-      </c>
-      <c r="M103" s="1">
-        <v>46386</v>
+        <v>713</v>
+      </c>
+      <c r="M103" s="2">
+        <v>46372</v>
       </c>
       <c r="N103" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="104" spans="1:14">
@@ -15108,11 +15134,11 @@
       <c r="L104" t="s">
         <v>713</v>
       </c>
-      <c r="M104" s="1">
-        <v>46371</v>
+      <c r="M104" s="2">
+        <v>46372</v>
       </c>
       <c r="N104" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="105" spans="1:14">
@@ -15144,19 +15170,19 @@
         <v>716</v>
       </c>
       <c r="J105" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="K105" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="L105" t="s">
-        <v>716</v>
-      </c>
-      <c r="M105" s="1">
-        <v>46386</v>
+        <v>713</v>
+      </c>
+      <c r="M105" s="2">
+        <v>46372</v>
       </c>
       <c r="N105" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="106" spans="1:14">
@@ -15196,11 +15222,11 @@
       <c r="L106" t="s">
         <v>716</v>
       </c>
-      <c r="M106" s="1">
-        <v>46386</v>
+      <c r="M106" s="2">
+        <v>46387</v>
       </c>
       <c r="N106" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="107" spans="1:14">
@@ -15232,19 +15258,19 @@
         <v>716</v>
       </c>
       <c r="J107" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="K107" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="L107" t="s">
-        <v>716</v>
-      </c>
-      <c r="M107" s="1">
-        <v>46386</v>
+        <v>713</v>
+      </c>
+      <c r="M107" s="2">
+        <v>46372</v>
       </c>
       <c r="N107" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="108" spans="1:14">
@@ -15284,11 +15310,11 @@
       <c r="L108" t="s">
         <v>713</v>
       </c>
-      <c r="M108" s="1">
-        <v>46371</v>
+      <c r="M108" s="2">
+        <v>46372</v>
       </c>
       <c r="N108" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="109" spans="1:14">
@@ -15328,11 +15354,11 @@
       <c r="L109" t="s">
         <v>713</v>
       </c>
-      <c r="M109" s="1">
-        <v>46371</v>
+      <c r="M109" s="2">
+        <v>46372</v>
       </c>
       <c r="N109" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="110" spans="1:14">
@@ -15372,11 +15398,11 @@
       <c r="L110" t="s">
         <v>713</v>
       </c>
-      <c r="M110" s="1">
-        <v>46371</v>
+      <c r="M110" s="2">
+        <v>46372</v>
       </c>
       <c r="N110" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="111" spans="1:14">
@@ -15416,11 +15442,11 @@
       <c r="L111" t="s">
         <v>713</v>
       </c>
-      <c r="M111" s="1">
-        <v>46371</v>
+      <c r="M111" s="2">
+        <v>46372</v>
       </c>
       <c r="N111" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="112" spans="1:14">
@@ -15460,11 +15486,11 @@
       <c r="L112" t="s">
         <v>713</v>
       </c>
-      <c r="M112" s="1">
-        <v>46371</v>
+      <c r="M112" s="2">
+        <v>46372</v>
       </c>
       <c r="N112" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="113" spans="1:14">
@@ -15504,11 +15530,11 @@
       <c r="L113" t="s">
         <v>713</v>
       </c>
-      <c r="M113" s="1">
-        <v>46371</v>
+      <c r="M113" s="2">
+        <v>46372</v>
       </c>
       <c r="N113" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="114" spans="1:14">
@@ -15548,11 +15574,11 @@
       <c r="L114" t="s">
         <v>713</v>
       </c>
-      <c r="M114" s="1">
-        <v>46371</v>
+      <c r="M114" s="2">
+        <v>46372</v>
       </c>
       <c r="N114" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="115" spans="1:14">
@@ -15592,11 +15618,11 @@
       <c r="L115" t="s">
         <v>713</v>
       </c>
-      <c r="M115" s="1">
-        <v>46371</v>
+      <c r="M115" s="2">
+        <v>46372</v>
       </c>
       <c r="N115" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="116" spans="1:14">
@@ -15636,11 +15662,11 @@
       <c r="L116" t="s">
         <v>713</v>
       </c>
-      <c r="M116" s="1">
-        <v>46371</v>
+      <c r="M116" s="2">
+        <v>46372</v>
       </c>
       <c r="N116" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="117" spans="1:14">
@@ -15680,11 +15706,11 @@
       <c r="L117" t="s">
         <v>713</v>
       </c>
-      <c r="M117" s="1">
-        <v>46371</v>
+      <c r="M117" s="2">
+        <v>46372</v>
       </c>
       <c r="N117" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="118" spans="1:14">
@@ -15724,11 +15750,11 @@
       <c r="L118" t="s">
         <v>713</v>
       </c>
-      <c r="M118" s="1">
-        <v>46371</v>
+      <c r="M118" s="2">
+        <v>46372</v>
       </c>
       <c r="N118" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="119" spans="1:14">
@@ -15768,11 +15794,11 @@
       <c r="L119" t="s">
         <v>713</v>
       </c>
-      <c r="M119" s="1">
-        <v>46371</v>
+      <c r="M119" s="2">
+        <v>46372</v>
       </c>
       <c r="N119" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="120" spans="1:14">
@@ -15812,11 +15838,11 @@
       <c r="L120" t="s">
         <v>713</v>
       </c>
-      <c r="M120" s="1">
-        <v>46371</v>
+      <c r="M120" s="2">
+        <v>46372</v>
       </c>
       <c r="N120" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="121" spans="1:14">
@@ -15847,17 +15873,20 @@
       <c r="I121" t="s">
         <v>382</v>
       </c>
+      <c r="J121" t="s">
+        <v>716</v>
+      </c>
       <c r="K121" t="s">
-        <v>382</v>
+        <v>716</v>
       </c>
       <c r="L121" t="s">
-        <v>382</v>
-      </c>
-      <c r="M121" s="1">
-        <v>46376</v>
+        <v>716</v>
+      </c>
+      <c r="M121" s="2">
+        <v>46387</v>
       </c>
       <c r="N121" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (02/10/2026 13:37)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2178,16 +2178,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2203,7 +2195,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2211,30 +2203,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2534,55 +2508,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2626,7 +2600,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2670,7 +2644,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2714,7 +2688,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2840,7 +2814,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2884,7 +2858,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2928,7 +2902,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2975,7 +2949,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3098,7 +3072,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -3142,7 +3116,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3186,7 +3160,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3230,7 +3204,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3277,7 +3251,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3321,7 +3295,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3447,7 +3421,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3491,7 +3465,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3576,7 +3550,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3623,7 +3597,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3670,7 +3644,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3714,7 +3688,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3758,7 +3732,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3843,7 +3817,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3928,7 +3902,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3975,7 +3949,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4019,7 +3993,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4063,7 +4037,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4148,7 +4122,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4192,7 +4166,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4236,7 +4210,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4321,7 +4295,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4365,7 +4339,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4409,7 +4383,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4453,7 +4427,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4620,7 +4594,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4664,7 +4638,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4708,7 +4682,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4752,7 +4726,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4799,7 +4773,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4843,7 +4817,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4925,7 +4899,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4969,7 +4943,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5057,7 +5031,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5101,7 +5075,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5148,7 +5122,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5192,7 +5166,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -5236,7 +5210,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5280,7 +5254,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5324,7 +5298,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5371,7 +5345,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5415,7 +5389,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5462,7 +5436,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5506,7 +5480,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5553,7 +5527,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5641,7 +5615,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5685,7 +5659,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5729,7 +5703,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5773,7 +5747,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5817,7 +5791,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5861,7 +5835,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5946,7 +5920,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5990,7 +5964,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -6034,7 +6008,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -6078,7 +6052,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -6122,7 +6096,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -6166,7 +6140,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6210,7 +6184,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6254,7 +6228,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6301,7 +6275,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6345,7 +6319,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6389,7 +6363,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6433,7 +6407,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6477,7 +6451,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6521,7 +6495,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6565,7 +6539,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6609,7 +6583,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6653,7 +6627,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6741,7 +6715,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6785,7 +6759,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6911,7 +6885,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6955,7 +6929,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6999,7 +6973,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7043,7 +7017,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7125,7 +7099,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7169,7 +7143,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7216,7 +7190,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7260,7 +7234,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7386,7 +7360,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7430,7 +7404,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7515,7 +7489,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7559,7 +7533,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7603,7 +7577,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7647,7 +7621,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7691,7 +7665,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7735,7 +7709,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7779,7 +7753,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7823,7 +7797,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7908,7 +7882,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8075,7 +8049,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8119,7 +8093,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8163,7 +8137,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8207,7 +8181,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8251,7 +8225,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8295,7 +8269,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8339,7 +8313,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8424,7 +8398,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8468,7 +8442,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8553,7 +8527,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8679,7 +8653,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8723,7 +8697,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8808,7 +8782,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8852,7 +8826,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8896,7 +8870,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8940,7 +8914,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8984,7 +8958,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -9028,7 +9002,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9072,7 +9046,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9116,7 +9090,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9201,7 +9175,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9368,7 +9342,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9412,7 +9386,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9456,7 +9430,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9500,7 +9474,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9585,7 +9559,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9629,7 +9603,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9673,7 +9647,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9717,7 +9691,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9761,7 +9735,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9805,7 +9779,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9849,7 +9823,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9893,7 +9867,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9937,7 +9911,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9981,7 +9955,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10025,7 +9999,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -10069,7 +10043,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10113,7 +10087,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10157,7 +10131,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -10201,7 +10175,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10245,7 +10219,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10289,7 +10263,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10333,7 +10307,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10377,7 +10351,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10421,7 +10395,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10465,7 +10439,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10550,7 +10524,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10635,7 +10609,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10650,55 +10624,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11067,7 +11041,7 @@
       <c r="L10" t="s">
         <v>713</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46372</v>
       </c>
       <c r="N10" t="s">
@@ -11111,7 +11085,7 @@
       <c r="L11" t="s">
         <v>713</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46372</v>
       </c>
       <c r="N11" t="s">
@@ -11319,7 +11293,7 @@
       <c r="L16" t="s">
         <v>713</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46372</v>
       </c>
       <c r="N16" t="s">
@@ -11445,7 +11419,7 @@
       <c r="L19" t="s">
         <v>713</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46372</v>
       </c>
       <c r="N19" t="s">
@@ -11489,7 +11463,7 @@
       <c r="L20" t="s">
         <v>713</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46372</v>
       </c>
       <c r="N20" t="s">
@@ -11533,7 +11507,7 @@
       <c r="L21" t="s">
         <v>713</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46372</v>
       </c>
       <c r="N21" t="s">
@@ -11700,7 +11674,7 @@
       <c r="L25" t="s">
         <v>713</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46372</v>
       </c>
       <c r="N25" t="s">
@@ -11826,7 +11800,7 @@
       <c r="L28" t="s">
         <v>713</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46372</v>
       </c>
       <c r="N28" t="s">
@@ -11870,7 +11844,7 @@
       <c r="L29" t="s">
         <v>715</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46307</v>
       </c>
       <c r="N29" t="s">
@@ -11914,7 +11888,7 @@
       <c r="L30" t="s">
         <v>713</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46372</v>
       </c>
       <c r="N30" t="s">
@@ -11958,7 +11932,7 @@
       <c r="L31" t="s">
         <v>715</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46307</v>
       </c>
       <c r="N31" t="s">
@@ -12371,7 +12345,7 @@
       <c r="L41" t="s">
         <v>713</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46372</v>
       </c>
       <c r="N41" t="s">
@@ -12456,7 +12430,7 @@
       <c r="L43" t="s">
         <v>713</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46372</v>
       </c>
       <c r="N43" t="s">
@@ -12500,7 +12474,7 @@
       <c r="L44" t="s">
         <v>713</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46372</v>
       </c>
       <c r="N44" t="s">
@@ -12544,7 +12518,7 @@
       <c r="L45" t="s">
         <v>713</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46372</v>
       </c>
       <c r="N45" t="s">
@@ -12670,7 +12644,7 @@
       <c r="L48" t="s">
         <v>713</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46372</v>
       </c>
       <c r="N48" t="s">
@@ -12714,7 +12688,7 @@
       <c r="L49" t="s">
         <v>715</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46307</v>
       </c>
       <c r="N49" t="s">
@@ -12758,7 +12732,7 @@
       <c r="L50" t="s">
         <v>715</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46307</v>
       </c>
       <c r="N50" t="s">
@@ -12802,7 +12776,7 @@
       <c r="L51" t="s">
         <v>713</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46372</v>
       </c>
       <c r="N51" t="s">
@@ -12846,7 +12820,7 @@
       <c r="L52" t="s">
         <v>713</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46372</v>
       </c>
       <c r="N52" t="s">
@@ -12890,7 +12864,7 @@
       <c r="L53" t="s">
         <v>713</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46372</v>
       </c>
       <c r="N53" t="s">
@@ -12934,7 +12908,7 @@
       <c r="L54" t="s">
         <v>713</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46372</v>
       </c>
       <c r="N54" t="s">
@@ -12978,7 +12952,7 @@
       <c r="L55" t="s">
         <v>716</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46387</v>
       </c>
       <c r="N55" t="s">
@@ -13022,7 +12996,7 @@
       <c r="L56" t="s">
         <v>715</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46307</v>
       </c>
       <c r="N56" t="s">
@@ -13066,7 +13040,7 @@
       <c r="L57" t="s">
         <v>715</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46307</v>
       </c>
       <c r="N57" t="s">
@@ -13110,7 +13084,7 @@
       <c r="L58" t="s">
         <v>715</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46307</v>
       </c>
       <c r="N58" t="s">
@@ -13154,7 +13128,7 @@
       <c r="L59" t="s">
         <v>713</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46372</v>
       </c>
       <c r="N59" t="s">
@@ -13198,7 +13172,7 @@
       <c r="L60" t="s">
         <v>715</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46307</v>
       </c>
       <c r="N60" t="s">
@@ -13242,7 +13216,7 @@
       <c r="L61" t="s">
         <v>715</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46307</v>
       </c>
       <c r="N61" t="s">
@@ -13286,7 +13260,7 @@
       <c r="L62" t="s">
         <v>713</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46372</v>
       </c>
       <c r="N62" t="s">
@@ -13330,7 +13304,7 @@
       <c r="L63" t="s">
         <v>713</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46372</v>
       </c>
       <c r="N63" t="s">
@@ -13374,7 +13348,7 @@
       <c r="L64" t="s">
         <v>713</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46372</v>
       </c>
       <c r="N64" t="s">
@@ -13418,7 +13392,7 @@
       <c r="L65" t="s">
         <v>713</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="1">
         <v>46372</v>
       </c>
       <c r="N65" t="s">
@@ -13462,7 +13436,7 @@
       <c r="L66" t="s">
         <v>713</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="1">
         <v>46372</v>
       </c>
       <c r="N66" t="s">
@@ -13506,7 +13480,7 @@
       <c r="L67" t="s">
         <v>713</v>
       </c>
-      <c r="M67" s="2">
+      <c r="M67" s="1">
         <v>46372</v>
       </c>
       <c r="N67" t="s">
@@ -13550,7 +13524,7 @@
       <c r="L68" t="s">
         <v>713</v>
       </c>
-      <c r="M68" s="2">
+      <c r="M68" s="1">
         <v>46372</v>
       </c>
       <c r="N68" t="s">
@@ -13594,7 +13568,7 @@
       <c r="L69" t="s">
         <v>713</v>
       </c>
-      <c r="M69" s="2">
+      <c r="M69" s="1">
         <v>46372</v>
       </c>
       <c r="N69" t="s">
@@ -13638,7 +13612,7 @@
       <c r="L70" t="s">
         <v>713</v>
       </c>
-      <c r="M70" s="2">
+      <c r="M70" s="1">
         <v>46372</v>
       </c>
       <c r="N70" t="s">
@@ -13682,7 +13656,7 @@
       <c r="L71" t="s">
         <v>713</v>
       </c>
-      <c r="M71" s="2">
+      <c r="M71" s="1">
         <v>46372</v>
       </c>
       <c r="N71" t="s">
@@ -13726,7 +13700,7 @@
       <c r="L72" t="s">
         <v>713</v>
       </c>
-      <c r="M72" s="2">
+      <c r="M72" s="1">
         <v>46372</v>
       </c>
       <c r="N72" t="s">
@@ -13770,7 +13744,7 @@
       <c r="L73" t="s">
         <v>713</v>
       </c>
-      <c r="M73" s="2">
+      <c r="M73" s="1">
         <v>46372</v>
       </c>
       <c r="N73" t="s">
@@ -13814,7 +13788,7 @@
       <c r="L74" t="s">
         <v>713</v>
       </c>
-      <c r="M74" s="2">
+      <c r="M74" s="1">
         <v>46372</v>
       </c>
       <c r="N74" t="s">
@@ -13858,7 +13832,7 @@
       <c r="L75" t="s">
         <v>716</v>
       </c>
-      <c r="M75" s="2">
+      <c r="M75" s="1">
         <v>46387</v>
       </c>
       <c r="N75" t="s">
@@ -13902,7 +13876,7 @@
       <c r="L76" t="s">
         <v>716</v>
       </c>
-      <c r="M76" s="2">
+      <c r="M76" s="1">
         <v>46387</v>
       </c>
       <c r="N76" t="s">
@@ -13946,7 +13920,7 @@
       <c r="L77" t="s">
         <v>713</v>
       </c>
-      <c r="M77" s="2">
+      <c r="M77" s="1">
         <v>46372</v>
       </c>
       <c r="N77" t="s">
@@ -13990,7 +13964,7 @@
       <c r="L78" t="s">
         <v>713</v>
       </c>
-      <c r="M78" s="2">
+      <c r="M78" s="1">
         <v>46372</v>
       </c>
       <c r="N78" t="s">
@@ -14034,7 +14008,7 @@
       <c r="L79" t="s">
         <v>713</v>
       </c>
-      <c r="M79" s="2">
+      <c r="M79" s="1">
         <v>46372</v>
       </c>
       <c r="N79" t="s">
@@ -14078,7 +14052,7 @@
       <c r="L80" t="s">
         <v>713</v>
       </c>
-      <c r="M80" s="2">
+      <c r="M80" s="1">
         <v>46372</v>
       </c>
       <c r="N80" t="s">
@@ -14122,7 +14096,7 @@
       <c r="L81" t="s">
         <v>716</v>
       </c>
-      <c r="M81" s="2">
+      <c r="M81" s="1">
         <v>46387</v>
       </c>
       <c r="N81" t="s">
@@ -14166,7 +14140,7 @@
       <c r="L82" t="s">
         <v>713</v>
       </c>
-      <c r="M82" s="2">
+      <c r="M82" s="1">
         <v>46372</v>
       </c>
       <c r="N82" t="s">
@@ -14210,7 +14184,7 @@
       <c r="L83" t="s">
         <v>713</v>
       </c>
-      <c r="M83" s="2">
+      <c r="M83" s="1">
         <v>46372</v>
       </c>
       <c r="N83" t="s">
@@ -14254,7 +14228,7 @@
       <c r="L84" t="s">
         <v>713</v>
       </c>
-      <c r="M84" s="2">
+      <c r="M84" s="1">
         <v>46372</v>
       </c>
       <c r="N84" t="s">
@@ -14298,7 +14272,7 @@
       <c r="L85" t="s">
         <v>713</v>
       </c>
-      <c r="M85" s="2">
+      <c r="M85" s="1">
         <v>46372</v>
       </c>
       <c r="N85" t="s">
@@ -14342,7 +14316,7 @@
       <c r="L86" t="s">
         <v>713</v>
       </c>
-      <c r="M86" s="2">
+      <c r="M86" s="1">
         <v>46372</v>
       </c>
       <c r="N86" t="s">
@@ -14386,7 +14360,7 @@
       <c r="L87" t="s">
         <v>713</v>
       </c>
-      <c r="M87" s="2">
+      <c r="M87" s="1">
         <v>46372</v>
       </c>
       <c r="N87" t="s">
@@ -14430,7 +14404,7 @@
       <c r="L88" t="s">
         <v>716</v>
       </c>
-      <c r="M88" s="2">
+      <c r="M88" s="1">
         <v>46387</v>
       </c>
       <c r="N88" t="s">
@@ -14474,7 +14448,7 @@
       <c r="L89" t="s">
         <v>713</v>
       </c>
-      <c r="M89" s="2">
+      <c r="M89" s="1">
         <v>46372</v>
       </c>
       <c r="N89" t="s">
@@ -14518,7 +14492,7 @@
       <c r="L90" t="s">
         <v>716</v>
       </c>
-      <c r="M90" s="2">
+      <c r="M90" s="1">
         <v>46387</v>
       </c>
       <c r="N90" t="s">
@@ -14562,7 +14536,7 @@
       <c r="L91" t="s">
         <v>716</v>
       </c>
-      <c r="M91" s="2">
+      <c r="M91" s="1">
         <v>46387</v>
       </c>
       <c r="N91" t="s">
@@ -14606,7 +14580,7 @@
       <c r="L92" t="s">
         <v>713</v>
       </c>
-      <c r="M92" s="2">
+      <c r="M92" s="1">
         <v>46372</v>
       </c>
       <c r="N92" t="s">
@@ -14650,7 +14624,7 @@
       <c r="L93" t="s">
         <v>716</v>
       </c>
-      <c r="M93" s="2">
+      <c r="M93" s="1">
         <v>46387</v>
       </c>
       <c r="N93" t="s">
@@ -14694,7 +14668,7 @@
       <c r="L94" t="s">
         <v>716</v>
       </c>
-      <c r="M94" s="2">
+      <c r="M94" s="1">
         <v>46387</v>
       </c>
       <c r="N94" t="s">
@@ -14738,7 +14712,7 @@
       <c r="L95" t="s">
         <v>716</v>
       </c>
-      <c r="M95" s="2">
+      <c r="M95" s="1">
         <v>46387</v>
       </c>
       <c r="N95" t="s">
@@ -14782,7 +14756,7 @@
       <c r="L96" t="s">
         <v>716</v>
       </c>
-      <c r="M96" s="2">
+      <c r="M96" s="1">
         <v>46387</v>
       </c>
       <c r="N96" t="s">
@@ -14826,7 +14800,7 @@
       <c r="L97" t="s">
         <v>713</v>
       </c>
-      <c r="M97" s="2">
+      <c r="M97" s="1">
         <v>46372</v>
       </c>
       <c r="N97" t="s">
@@ -14870,7 +14844,7 @@
       <c r="L98" t="s">
         <v>713</v>
       </c>
-      <c r="M98" s="2">
+      <c r="M98" s="1">
         <v>46372</v>
       </c>
       <c r="N98" t="s">
@@ -14914,7 +14888,7 @@
       <c r="L99" t="s">
         <v>713</v>
       </c>
-      <c r="M99" s="2">
+      <c r="M99" s="1">
         <v>46372</v>
       </c>
       <c r="N99" t="s">
@@ -14958,7 +14932,7 @@
       <c r="L100" t="s">
         <v>713</v>
       </c>
-      <c r="M100" s="2">
+      <c r="M100" s="1">
         <v>46372</v>
       </c>
       <c r="N100" t="s">
@@ -15002,7 +14976,7 @@
       <c r="L101" t="s">
         <v>713</v>
       </c>
-      <c r="M101" s="2">
+      <c r="M101" s="1">
         <v>46372</v>
       </c>
       <c r="N101" t="s">
@@ -15046,7 +15020,7 @@
       <c r="L102" t="s">
         <v>713</v>
       </c>
-      <c r="M102" s="2">
+      <c r="M102" s="1">
         <v>46372</v>
       </c>
       <c r="N102" t="s">
@@ -15090,7 +15064,7 @@
       <c r="L103" t="s">
         <v>713</v>
       </c>
-      <c r="M103" s="2">
+      <c r="M103" s="1">
         <v>46372</v>
       </c>
       <c r="N103" t="s">
@@ -15134,7 +15108,7 @@
       <c r="L104" t="s">
         <v>713</v>
       </c>
-      <c r="M104" s="2">
+      <c r="M104" s="1">
         <v>46372</v>
       </c>
       <c r="N104" t="s">
@@ -15178,7 +15152,7 @@
       <c r="L105" t="s">
         <v>713</v>
       </c>
-      <c r="M105" s="2">
+      <c r="M105" s="1">
         <v>46372</v>
       </c>
       <c r="N105" t="s">
@@ -15222,7 +15196,7 @@
       <c r="L106" t="s">
         <v>716</v>
       </c>
-      <c r="M106" s="2">
+      <c r="M106" s="1">
         <v>46387</v>
       </c>
       <c r="N106" t="s">
@@ -15266,7 +15240,7 @@
       <c r="L107" t="s">
         <v>713</v>
       </c>
-      <c r="M107" s="2">
+      <c r="M107" s="1">
         <v>46372</v>
       </c>
       <c r="N107" t="s">
@@ -15310,7 +15284,7 @@
       <c r="L108" t="s">
         <v>713</v>
       </c>
-      <c r="M108" s="2">
+      <c r="M108" s="1">
         <v>46372</v>
       </c>
       <c r="N108" t="s">
@@ -15354,7 +15328,7 @@
       <c r="L109" t="s">
         <v>713</v>
       </c>
-      <c r="M109" s="2">
+      <c r="M109" s="1">
         <v>46372</v>
       </c>
       <c r="N109" t="s">
@@ -15398,7 +15372,7 @@
       <c r="L110" t="s">
         <v>713</v>
       </c>
-      <c r="M110" s="2">
+      <c r="M110" s="1">
         <v>46372</v>
       </c>
       <c r="N110" t="s">
@@ -15442,7 +15416,7 @@
       <c r="L111" t="s">
         <v>713</v>
       </c>
-      <c r="M111" s="2">
+      <c r="M111" s="1">
         <v>46372</v>
       </c>
       <c r="N111" t="s">
@@ -15486,7 +15460,7 @@
       <c r="L112" t="s">
         <v>713</v>
       </c>
-      <c r="M112" s="2">
+      <c r="M112" s="1">
         <v>46372</v>
       </c>
       <c r="N112" t="s">
@@ -15530,7 +15504,7 @@
       <c r="L113" t="s">
         <v>713</v>
       </c>
-      <c r="M113" s="2">
+      <c r="M113" s="1">
         <v>46372</v>
       </c>
       <c r="N113" t="s">
@@ -15574,7 +15548,7 @@
       <c r="L114" t="s">
         <v>713</v>
       </c>
-      <c r="M114" s="2">
+      <c r="M114" s="1">
         <v>46372</v>
       </c>
       <c r="N114" t="s">
@@ -15618,7 +15592,7 @@
       <c r="L115" t="s">
         <v>713</v>
       </c>
-      <c r="M115" s="2">
+      <c r="M115" s="1">
         <v>46372</v>
       </c>
       <c r="N115" t="s">
@@ -15662,7 +15636,7 @@
       <c r="L116" t="s">
         <v>713</v>
       </c>
-      <c r="M116" s="2">
+      <c r="M116" s="1">
         <v>46372</v>
       </c>
       <c r="N116" t="s">
@@ -15706,7 +15680,7 @@
       <c r="L117" t="s">
         <v>713</v>
       </c>
-      <c r="M117" s="2">
+      <c r="M117" s="1">
         <v>46372</v>
       </c>
       <c r="N117" t="s">
@@ -15750,7 +15724,7 @@
       <c r="L118" t="s">
         <v>713</v>
       </c>
-      <c r="M118" s="2">
+      <c r="M118" s="1">
         <v>46372</v>
       </c>
       <c r="N118" t="s">
@@ -15794,7 +15768,7 @@
       <c r="L119" t="s">
         <v>713</v>
       </c>
-      <c r="M119" s="2">
+      <c r="M119" s="1">
         <v>46372</v>
       </c>
       <c r="N119" t="s">
@@ -15838,7 +15812,7 @@
       <c r="L120" t="s">
         <v>713</v>
       </c>
-      <c r="M120" s="2">
+      <c r="M120" s="1">
         <v>46372</v>
       </c>
       <c r="N120" t="s">
@@ -15882,7 +15856,7 @@
       <c r="L121" t="s">
         <v>716</v>
       </c>
-      <c r="M121" s="2">
+      <c r="M121" s="1">
         <v>46387</v>
       </c>
       <c r="N121" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (05/10/2026 08:41)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2178,8 +2178,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2195,7 +2203,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2203,12 +2211,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2508,55 +2534,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2600,7 +2626,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2644,7 +2670,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2688,7 +2714,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2814,7 +2840,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2858,7 +2884,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2902,7 +2928,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2949,7 +2975,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3072,7 +3098,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -3116,7 +3142,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3160,7 +3186,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3204,7 +3230,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3251,7 +3277,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3295,7 +3321,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3421,7 +3447,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3465,7 +3491,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3550,7 +3576,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3597,7 +3623,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3644,7 +3670,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3688,7 +3714,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3732,7 +3758,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3817,7 +3843,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3902,7 +3928,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3949,7 +3975,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3993,7 +4019,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4037,7 +4063,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4122,7 +4148,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4166,7 +4192,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4210,7 +4236,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4295,7 +4321,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4339,7 +4365,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4383,7 +4409,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4427,7 +4453,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4594,7 +4620,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4638,7 +4664,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4682,7 +4708,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4726,7 +4752,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4773,7 +4799,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4817,7 +4843,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4899,7 +4925,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4943,7 +4969,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5031,7 +5057,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5075,7 +5101,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5122,7 +5148,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5166,7 +5192,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -5210,7 +5236,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5254,7 +5280,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5298,7 +5324,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5345,7 +5371,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5389,7 +5415,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5436,7 +5462,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5480,7 +5506,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5527,7 +5553,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5615,7 +5641,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5659,7 +5685,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5703,7 +5729,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5747,7 +5773,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5791,7 +5817,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5835,7 +5861,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5920,7 +5946,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5964,7 +5990,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -6008,7 +6034,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -6052,7 +6078,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -6096,7 +6122,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -6140,7 +6166,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6184,7 +6210,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6228,7 +6254,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6275,7 +6301,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6319,7 +6345,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6363,7 +6389,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6407,7 +6433,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6451,7 +6477,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6495,7 +6521,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6539,7 +6565,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6583,7 +6609,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6627,7 +6653,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6715,7 +6741,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6759,7 +6785,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6885,7 +6911,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6929,7 +6955,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6973,7 +6999,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7017,7 +7043,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7099,7 +7125,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7143,7 +7169,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7190,7 +7216,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7234,7 +7260,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7360,7 +7386,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7404,7 +7430,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7489,7 +7515,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7533,7 +7559,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7577,7 +7603,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7621,7 +7647,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7665,7 +7691,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7709,7 +7735,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7753,7 +7779,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7797,7 +7823,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7882,7 +7908,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8049,7 +8075,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8093,7 +8119,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8137,7 +8163,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8181,7 +8207,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8225,7 +8251,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8269,7 +8295,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8313,7 +8339,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8398,7 +8424,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8442,7 +8468,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8527,7 +8553,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8653,7 +8679,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8697,7 +8723,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8782,7 +8808,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8826,7 +8852,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8870,7 +8896,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8914,7 +8940,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8958,7 +8984,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -9002,7 +9028,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9046,7 +9072,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9090,7 +9116,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9175,7 +9201,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9342,7 +9368,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9386,7 +9412,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9430,7 +9456,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9474,7 +9500,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9559,7 +9585,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9603,7 +9629,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9647,7 +9673,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9691,7 +9717,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9735,7 +9761,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9779,7 +9805,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9823,7 +9849,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9867,7 +9893,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9911,7 +9937,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9955,7 +9981,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9999,7 +10025,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -10043,7 +10069,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10087,7 +10113,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10131,7 +10157,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -10175,7 +10201,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10219,7 +10245,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10263,7 +10289,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10307,7 +10333,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10351,7 +10377,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10395,7 +10421,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10439,7 +10465,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10524,7 +10550,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10609,7 +10635,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10624,55 +10650,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11041,8 +11067,8 @@
       <c r="L10" t="s">
         <v>713</v>
       </c>
-      <c r="M10" s="1">
-        <v>46372</v>
+      <c r="M10" s="2">
+        <v>46375</v>
       </c>
       <c r="N10" t="s">
         <v>717</v>
@@ -11085,8 +11111,8 @@
       <c r="L11" t="s">
         <v>713</v>
       </c>
-      <c r="M11" s="1">
-        <v>46372</v>
+      <c r="M11" s="2">
+        <v>46375</v>
       </c>
       <c r="N11" t="s">
         <v>717</v>
@@ -11293,8 +11319,8 @@
       <c r="L16" t="s">
         <v>713</v>
       </c>
-      <c r="M16" s="1">
-        <v>46372</v>
+      <c r="M16" s="2">
+        <v>46375</v>
       </c>
       <c r="N16" t="s">
         <v>717</v>
@@ -11419,8 +11445,8 @@
       <c r="L19" t="s">
         <v>713</v>
       </c>
-      <c r="M19" s="1">
-        <v>46372</v>
+      <c r="M19" s="2">
+        <v>46375</v>
       </c>
       <c r="N19" t="s">
         <v>717</v>
@@ -11463,8 +11489,8 @@
       <c r="L20" t="s">
         <v>713</v>
       </c>
-      <c r="M20" s="1">
-        <v>46372</v>
+      <c r="M20" s="2">
+        <v>46375</v>
       </c>
       <c r="N20" t="s">
         <v>717</v>
@@ -11507,8 +11533,8 @@
       <c r="L21" t="s">
         <v>713</v>
       </c>
-      <c r="M21" s="1">
-        <v>46372</v>
+      <c r="M21" s="2">
+        <v>46375</v>
       </c>
       <c r="N21" t="s">
         <v>717</v>
@@ -11674,8 +11700,8 @@
       <c r="L25" t="s">
         <v>713</v>
       </c>
-      <c r="M25" s="1">
-        <v>46372</v>
+      <c r="M25" s="2">
+        <v>46375</v>
       </c>
       <c r="N25" t="s">
         <v>717</v>
@@ -11800,8 +11826,8 @@
       <c r="L28" t="s">
         <v>713</v>
       </c>
-      <c r="M28" s="1">
-        <v>46372</v>
+      <c r="M28" s="2">
+        <v>46375</v>
       </c>
       <c r="N28" t="s">
         <v>717</v>
@@ -11844,8 +11870,8 @@
       <c r="L29" t="s">
         <v>715</v>
       </c>
-      <c r="M29" s="1">
-        <v>46307</v>
+      <c r="M29" s="2">
+        <v>46310</v>
       </c>
       <c r="N29" t="s">
         <v>717</v>
@@ -11888,8 +11914,8 @@
       <c r="L30" t="s">
         <v>713</v>
       </c>
-      <c r="M30" s="1">
-        <v>46372</v>
+      <c r="M30" s="2">
+        <v>46375</v>
       </c>
       <c r="N30" t="s">
         <v>717</v>
@@ -11932,8 +11958,8 @@
       <c r="L31" t="s">
         <v>715</v>
       </c>
-      <c r="M31" s="1">
-        <v>46307</v>
+      <c r="M31" s="2">
+        <v>46310</v>
       </c>
       <c r="N31" t="s">
         <v>717</v>
@@ -12345,8 +12371,8 @@
       <c r="L41" t="s">
         <v>713</v>
       </c>
-      <c r="M41" s="1">
-        <v>46372</v>
+      <c r="M41" s="2">
+        <v>46375</v>
       </c>
       <c r="N41" t="s">
         <v>717</v>
@@ -12430,8 +12456,8 @@
       <c r="L43" t="s">
         <v>713</v>
       </c>
-      <c r="M43" s="1">
-        <v>46372</v>
+      <c r="M43" s="2">
+        <v>46375</v>
       </c>
       <c r="N43" t="s">
         <v>717</v>
@@ -12474,8 +12500,8 @@
       <c r="L44" t="s">
         <v>713</v>
       </c>
-      <c r="M44" s="1">
-        <v>46372</v>
+      <c r="M44" s="2">
+        <v>46375</v>
       </c>
       <c r="N44" t="s">
         <v>717</v>
@@ -12518,8 +12544,8 @@
       <c r="L45" t="s">
         <v>713</v>
       </c>
-      <c r="M45" s="1">
-        <v>46372</v>
+      <c r="M45" s="2">
+        <v>46375</v>
       </c>
       <c r="N45" t="s">
         <v>717</v>
@@ -12644,8 +12670,8 @@
       <c r="L48" t="s">
         <v>713</v>
       </c>
-      <c r="M48" s="1">
-        <v>46372</v>
+      <c r="M48" s="2">
+        <v>46375</v>
       </c>
       <c r="N48" t="s">
         <v>717</v>
@@ -12688,8 +12714,8 @@
       <c r="L49" t="s">
         <v>715</v>
       </c>
-      <c r="M49" s="1">
-        <v>46307</v>
+      <c r="M49" s="2">
+        <v>46310</v>
       </c>
       <c r="N49" t="s">
         <v>717</v>
@@ -12732,8 +12758,8 @@
       <c r="L50" t="s">
         <v>715</v>
       </c>
-      <c r="M50" s="1">
-        <v>46307</v>
+      <c r="M50" s="2">
+        <v>46310</v>
       </c>
       <c r="N50" t="s">
         <v>717</v>
@@ -12776,8 +12802,8 @@
       <c r="L51" t="s">
         <v>713</v>
       </c>
-      <c r="M51" s="1">
-        <v>46372</v>
+      <c r="M51" s="2">
+        <v>46375</v>
       </c>
       <c r="N51" t="s">
         <v>717</v>
@@ -12820,8 +12846,8 @@
       <c r="L52" t="s">
         <v>713</v>
       </c>
-      <c r="M52" s="1">
-        <v>46372</v>
+      <c r="M52" s="2">
+        <v>46375</v>
       </c>
       <c r="N52" t="s">
         <v>717</v>
@@ -12864,8 +12890,8 @@
       <c r="L53" t="s">
         <v>713</v>
       </c>
-      <c r="M53" s="1">
-        <v>46372</v>
+      <c r="M53" s="2">
+        <v>46375</v>
       </c>
       <c r="N53" t="s">
         <v>717</v>
@@ -12908,8 +12934,8 @@
       <c r="L54" t="s">
         <v>713</v>
       </c>
-      <c r="M54" s="1">
-        <v>46372</v>
+      <c r="M54" s="2">
+        <v>46375</v>
       </c>
       <c r="N54" t="s">
         <v>717</v>
@@ -12952,8 +12978,8 @@
       <c r="L55" t="s">
         <v>716</v>
       </c>
-      <c r="M55" s="1">
-        <v>46387</v>
+      <c r="M55" s="2">
+        <v>46390</v>
       </c>
       <c r="N55" t="s">
         <v>717</v>
@@ -12996,8 +13022,8 @@
       <c r="L56" t="s">
         <v>715</v>
       </c>
-      <c r="M56" s="1">
-        <v>46307</v>
+      <c r="M56" s="2">
+        <v>46310</v>
       </c>
       <c r="N56" t="s">
         <v>717</v>
@@ -13040,8 +13066,8 @@
       <c r="L57" t="s">
         <v>715</v>
       </c>
-      <c r="M57" s="1">
-        <v>46307</v>
+      <c r="M57" s="2">
+        <v>46310</v>
       </c>
       <c r="N57" t="s">
         <v>717</v>
@@ -13084,8 +13110,8 @@
       <c r="L58" t="s">
         <v>715</v>
       </c>
-      <c r="M58" s="1">
-        <v>46307</v>
+      <c r="M58" s="2">
+        <v>46310</v>
       </c>
       <c r="N58" t="s">
         <v>717</v>
@@ -13128,8 +13154,8 @@
       <c r="L59" t="s">
         <v>713</v>
       </c>
-      <c r="M59" s="1">
-        <v>46372</v>
+      <c r="M59" s="2">
+        <v>46375</v>
       </c>
       <c r="N59" t="s">
         <v>717</v>
@@ -13172,8 +13198,8 @@
       <c r="L60" t="s">
         <v>715</v>
       </c>
-      <c r="M60" s="1">
-        <v>46307</v>
+      <c r="M60" s="2">
+        <v>46310</v>
       </c>
       <c r="N60" t="s">
         <v>717</v>
@@ -13216,8 +13242,8 @@
       <c r="L61" t="s">
         <v>715</v>
       </c>
-      <c r="M61" s="1">
-        <v>46307</v>
+      <c r="M61" s="2">
+        <v>46310</v>
       </c>
       <c r="N61" t="s">
         <v>717</v>
@@ -13260,8 +13286,8 @@
       <c r="L62" t="s">
         <v>713</v>
       </c>
-      <c r="M62" s="1">
-        <v>46372</v>
+      <c r="M62" s="2">
+        <v>46375</v>
       </c>
       <c r="N62" t="s">
         <v>717</v>
@@ -13304,8 +13330,8 @@
       <c r="L63" t="s">
         <v>713</v>
       </c>
-      <c r="M63" s="1">
-        <v>46372</v>
+      <c r="M63" s="2">
+        <v>46375</v>
       </c>
       <c r="N63" t="s">
         <v>717</v>
@@ -13348,8 +13374,8 @@
       <c r="L64" t="s">
         <v>713</v>
       </c>
-      <c r="M64" s="1">
-        <v>46372</v>
+      <c r="M64" s="2">
+        <v>46375</v>
       </c>
       <c r="N64" t="s">
         <v>717</v>
@@ -13392,8 +13418,8 @@
       <c r="L65" t="s">
         <v>713</v>
       </c>
-      <c r="M65" s="1">
-        <v>46372</v>
+      <c r="M65" s="2">
+        <v>46375</v>
       </c>
       <c r="N65" t="s">
         <v>717</v>
@@ -13436,8 +13462,8 @@
       <c r="L66" t="s">
         <v>713</v>
       </c>
-      <c r="M66" s="1">
-        <v>46372</v>
+      <c r="M66" s="2">
+        <v>46375</v>
       </c>
       <c r="N66" t="s">
         <v>717</v>
@@ -13480,8 +13506,8 @@
       <c r="L67" t="s">
         <v>713</v>
       </c>
-      <c r="M67" s="1">
-        <v>46372</v>
+      <c r="M67" s="2">
+        <v>46375</v>
       </c>
       <c r="N67" t="s">
         <v>717</v>
@@ -13524,8 +13550,8 @@
       <c r="L68" t="s">
         <v>713</v>
       </c>
-      <c r="M68" s="1">
-        <v>46372</v>
+      <c r="M68" s="2">
+        <v>46375</v>
       </c>
       <c r="N68" t="s">
         <v>717</v>
@@ -13568,8 +13594,8 @@
       <c r="L69" t="s">
         <v>713</v>
       </c>
-      <c r="M69" s="1">
-        <v>46372</v>
+      <c r="M69" s="2">
+        <v>46375</v>
       </c>
       <c r="N69" t="s">
         <v>717</v>
@@ -13612,8 +13638,8 @@
       <c r="L70" t="s">
         <v>713</v>
       </c>
-      <c r="M70" s="1">
-        <v>46372</v>
+      <c r="M70" s="2">
+        <v>46375</v>
       </c>
       <c r="N70" t="s">
         <v>717</v>
@@ -13656,8 +13682,8 @@
       <c r="L71" t="s">
         <v>713</v>
       </c>
-      <c r="M71" s="1">
-        <v>46372</v>
+      <c r="M71" s="2">
+        <v>46375</v>
       </c>
       <c r="N71" t="s">
         <v>717</v>
@@ -13700,8 +13726,8 @@
       <c r="L72" t="s">
         <v>713</v>
       </c>
-      <c r="M72" s="1">
-        <v>46372</v>
+      <c r="M72" s="2">
+        <v>46375</v>
       </c>
       <c r="N72" t="s">
         <v>717</v>
@@ -13744,8 +13770,8 @@
       <c r="L73" t="s">
         <v>713</v>
       </c>
-      <c r="M73" s="1">
-        <v>46372</v>
+      <c r="M73" s="2">
+        <v>46375</v>
       </c>
       <c r="N73" t="s">
         <v>717</v>
@@ -13788,8 +13814,8 @@
       <c r="L74" t="s">
         <v>713</v>
       </c>
-      <c r="M74" s="1">
-        <v>46372</v>
+      <c r="M74" s="2">
+        <v>46375</v>
       </c>
       <c r="N74" t="s">
         <v>717</v>
@@ -13832,8 +13858,8 @@
       <c r="L75" t="s">
         <v>716</v>
       </c>
-      <c r="M75" s="1">
-        <v>46387</v>
+      <c r="M75" s="2">
+        <v>46390</v>
       </c>
       <c r="N75" t="s">
         <v>717</v>
@@ -13876,8 +13902,8 @@
       <c r="L76" t="s">
         <v>716</v>
       </c>
-      <c r="M76" s="1">
-        <v>46387</v>
+      <c r="M76" s="2">
+        <v>46390</v>
       </c>
       <c r="N76" t="s">
         <v>717</v>
@@ -13920,8 +13946,8 @@
       <c r="L77" t="s">
         <v>713</v>
       </c>
-      <c r="M77" s="1">
-        <v>46372</v>
+      <c r="M77" s="2">
+        <v>46375</v>
       </c>
       <c r="N77" t="s">
         <v>717</v>
@@ -13964,8 +13990,8 @@
       <c r="L78" t="s">
         <v>713</v>
       </c>
-      <c r="M78" s="1">
-        <v>46372</v>
+      <c r="M78" s="2">
+        <v>46375</v>
       </c>
       <c r="N78" t="s">
         <v>717</v>
@@ -14008,8 +14034,8 @@
       <c r="L79" t="s">
         <v>713</v>
       </c>
-      <c r="M79" s="1">
-        <v>46372</v>
+      <c r="M79" s="2">
+        <v>46375</v>
       </c>
       <c r="N79" t="s">
         <v>717</v>
@@ -14052,8 +14078,8 @@
       <c r="L80" t="s">
         <v>713</v>
       </c>
-      <c r="M80" s="1">
-        <v>46372</v>
+      <c r="M80" s="2">
+        <v>46375</v>
       </c>
       <c r="N80" t="s">
         <v>717</v>
@@ -14096,8 +14122,8 @@
       <c r="L81" t="s">
         <v>716</v>
       </c>
-      <c r="M81" s="1">
-        <v>46387</v>
+      <c r="M81" s="2">
+        <v>46390</v>
       </c>
       <c r="N81" t="s">
         <v>717</v>
@@ -14140,8 +14166,8 @@
       <c r="L82" t="s">
         <v>713</v>
       </c>
-      <c r="M82" s="1">
-        <v>46372</v>
+      <c r="M82" s="2">
+        <v>46375</v>
       </c>
       <c r="N82" t="s">
         <v>717</v>
@@ -14184,8 +14210,8 @@
       <c r="L83" t="s">
         <v>713</v>
       </c>
-      <c r="M83" s="1">
-        <v>46372</v>
+      <c r="M83" s="2">
+        <v>46375</v>
       </c>
       <c r="N83" t="s">
         <v>717</v>
@@ -14228,8 +14254,8 @@
       <c r="L84" t="s">
         <v>713</v>
       </c>
-      <c r="M84" s="1">
-        <v>46372</v>
+      <c r="M84" s="2">
+        <v>46375</v>
       </c>
       <c r="N84" t="s">
         <v>717</v>
@@ -14272,8 +14298,8 @@
       <c r="L85" t="s">
         <v>713</v>
       </c>
-      <c r="M85" s="1">
-        <v>46372</v>
+      <c r="M85" s="2">
+        <v>46375</v>
       </c>
       <c r="N85" t="s">
         <v>717</v>
@@ -14316,8 +14342,8 @@
       <c r="L86" t="s">
         <v>713</v>
       </c>
-      <c r="M86" s="1">
-        <v>46372</v>
+      <c r="M86" s="2">
+        <v>46375</v>
       </c>
       <c r="N86" t="s">
         <v>717</v>
@@ -14360,8 +14386,8 @@
       <c r="L87" t="s">
         <v>713</v>
       </c>
-      <c r="M87" s="1">
-        <v>46372</v>
+      <c r="M87" s="2">
+        <v>46375</v>
       </c>
       <c r="N87" t="s">
         <v>717</v>
@@ -14404,8 +14430,8 @@
       <c r="L88" t="s">
         <v>716</v>
       </c>
-      <c r="M88" s="1">
-        <v>46387</v>
+      <c r="M88" s="2">
+        <v>46390</v>
       </c>
       <c r="N88" t="s">
         <v>717</v>
@@ -14448,8 +14474,8 @@
       <c r="L89" t="s">
         <v>713</v>
       </c>
-      <c r="M89" s="1">
-        <v>46372</v>
+      <c r="M89" s="2">
+        <v>46375</v>
       </c>
       <c r="N89" t="s">
         <v>717</v>
@@ -14492,8 +14518,8 @@
       <c r="L90" t="s">
         <v>716</v>
       </c>
-      <c r="M90" s="1">
-        <v>46387</v>
+      <c r="M90" s="2">
+        <v>46390</v>
       </c>
       <c r="N90" t="s">
         <v>717</v>
@@ -14536,8 +14562,8 @@
       <c r="L91" t="s">
         <v>716</v>
       </c>
-      <c r="M91" s="1">
-        <v>46387</v>
+      <c r="M91" s="2">
+        <v>46390</v>
       </c>
       <c r="N91" t="s">
         <v>717</v>
@@ -14580,8 +14606,8 @@
       <c r="L92" t="s">
         <v>713</v>
       </c>
-      <c r="M92" s="1">
-        <v>46372</v>
+      <c r="M92" s="2">
+        <v>46375</v>
       </c>
       <c r="N92" t="s">
         <v>717</v>
@@ -14624,8 +14650,8 @@
       <c r="L93" t="s">
         <v>716</v>
       </c>
-      <c r="M93" s="1">
-        <v>46387</v>
+      <c r="M93" s="2">
+        <v>46390</v>
       </c>
       <c r="N93" t="s">
         <v>717</v>
@@ -14668,8 +14694,8 @@
       <c r="L94" t="s">
         <v>716</v>
       </c>
-      <c r="M94" s="1">
-        <v>46387</v>
+      <c r="M94" s="2">
+        <v>46390</v>
       </c>
       <c r="N94" t="s">
         <v>717</v>
@@ -14712,8 +14738,8 @@
       <c r="L95" t="s">
         <v>716</v>
       </c>
-      <c r="M95" s="1">
-        <v>46387</v>
+      <c r="M95" s="2">
+        <v>46390</v>
       </c>
       <c r="N95" t="s">
         <v>717</v>
@@ -14756,8 +14782,8 @@
       <c r="L96" t="s">
         <v>716</v>
       </c>
-      <c r="M96" s="1">
-        <v>46387</v>
+      <c r="M96" s="2">
+        <v>46390</v>
       </c>
       <c r="N96" t="s">
         <v>717</v>
@@ -14800,8 +14826,8 @@
       <c r="L97" t="s">
         <v>713</v>
       </c>
-      <c r="M97" s="1">
-        <v>46372</v>
+      <c r="M97" s="2">
+        <v>46375</v>
       </c>
       <c r="N97" t="s">
         <v>717</v>
@@ -14844,8 +14870,8 @@
       <c r="L98" t="s">
         <v>713</v>
       </c>
-      <c r="M98" s="1">
-        <v>46372</v>
+      <c r="M98" s="2">
+        <v>46375</v>
       </c>
       <c r="N98" t="s">
         <v>717</v>
@@ -14888,8 +14914,8 @@
       <c r="L99" t="s">
         <v>713</v>
       </c>
-      <c r="M99" s="1">
-        <v>46372</v>
+      <c r="M99" s="2">
+        <v>46375</v>
       </c>
       <c r="N99" t="s">
         <v>717</v>
@@ -14932,8 +14958,8 @@
       <c r="L100" t="s">
         <v>713</v>
       </c>
-      <c r="M100" s="1">
-        <v>46372</v>
+      <c r="M100" s="2">
+        <v>46375</v>
       </c>
       <c r="N100" t="s">
         <v>717</v>
@@ -14976,8 +15002,8 @@
       <c r="L101" t="s">
         <v>713</v>
       </c>
-      <c r="M101" s="1">
-        <v>46372</v>
+      <c r="M101" s="2">
+        <v>46375</v>
       </c>
       <c r="N101" t="s">
         <v>717</v>
@@ -15020,8 +15046,8 @@
       <c r="L102" t="s">
         <v>713</v>
       </c>
-      <c r="M102" s="1">
-        <v>46372</v>
+      <c r="M102" s="2">
+        <v>46375</v>
       </c>
       <c r="N102" t="s">
         <v>717</v>
@@ -15064,8 +15090,8 @@
       <c r="L103" t="s">
         <v>713</v>
       </c>
-      <c r="M103" s="1">
-        <v>46372</v>
+      <c r="M103" s="2">
+        <v>46375</v>
       </c>
       <c r="N103" t="s">
         <v>717</v>
@@ -15108,8 +15134,8 @@
       <c r="L104" t="s">
         <v>713</v>
       </c>
-      <c r="M104" s="1">
-        <v>46372</v>
+      <c r="M104" s="2">
+        <v>46375</v>
       </c>
       <c r="N104" t="s">
         <v>717</v>
@@ -15152,8 +15178,8 @@
       <c r="L105" t="s">
         <v>713</v>
       </c>
-      <c r="M105" s="1">
-        <v>46372</v>
+      <c r="M105" s="2">
+        <v>46375</v>
       </c>
       <c r="N105" t="s">
         <v>717</v>
@@ -15196,8 +15222,8 @@
       <c r="L106" t="s">
         <v>716</v>
       </c>
-      <c r="M106" s="1">
-        <v>46387</v>
+      <c r="M106" s="2">
+        <v>46390</v>
       </c>
       <c r="N106" t="s">
         <v>717</v>
@@ -15240,8 +15266,8 @@
       <c r="L107" t="s">
         <v>713</v>
       </c>
-      <c r="M107" s="1">
-        <v>46372</v>
+      <c r="M107" s="2">
+        <v>46375</v>
       </c>
       <c r="N107" t="s">
         <v>717</v>
@@ -15284,8 +15310,8 @@
       <c r="L108" t="s">
         <v>713</v>
       </c>
-      <c r="M108" s="1">
-        <v>46372</v>
+      <c r="M108" s="2">
+        <v>46375</v>
       </c>
       <c r="N108" t="s">
         <v>717</v>
@@ -15328,8 +15354,8 @@
       <c r="L109" t="s">
         <v>713</v>
       </c>
-      <c r="M109" s="1">
-        <v>46372</v>
+      <c r="M109" s="2">
+        <v>46375</v>
       </c>
       <c r="N109" t="s">
         <v>717</v>
@@ -15372,8 +15398,8 @@
       <c r="L110" t="s">
         <v>713</v>
       </c>
-      <c r="M110" s="1">
-        <v>46372</v>
+      <c r="M110" s="2">
+        <v>46375</v>
       </c>
       <c r="N110" t="s">
         <v>717</v>
@@ -15416,8 +15442,8 @@
       <c r="L111" t="s">
         <v>713</v>
       </c>
-      <c r="M111" s="1">
-        <v>46372</v>
+      <c r="M111" s="2">
+        <v>46375</v>
       </c>
       <c r="N111" t="s">
         <v>717</v>
@@ -15460,8 +15486,8 @@
       <c r="L112" t="s">
         <v>713</v>
       </c>
-      <c r="M112" s="1">
-        <v>46372</v>
+      <c r="M112" s="2">
+        <v>46375</v>
       </c>
       <c r="N112" t="s">
         <v>717</v>
@@ -15504,8 +15530,8 @@
       <c r="L113" t="s">
         <v>713</v>
       </c>
-      <c r="M113" s="1">
-        <v>46372</v>
+      <c r="M113" s="2">
+        <v>46375</v>
       </c>
       <c r="N113" t="s">
         <v>717</v>
@@ -15548,8 +15574,8 @@
       <c r="L114" t="s">
         <v>713</v>
       </c>
-      <c r="M114" s="1">
-        <v>46372</v>
+      <c r="M114" s="2">
+        <v>46375</v>
       </c>
       <c r="N114" t="s">
         <v>717</v>
@@ -15592,8 +15618,8 @@
       <c r="L115" t="s">
         <v>713</v>
       </c>
-      <c r="M115" s="1">
-        <v>46372</v>
+      <c r="M115" s="2">
+        <v>46375</v>
       </c>
       <c r="N115" t="s">
         <v>717</v>
@@ -15636,8 +15662,8 @@
       <c r="L116" t="s">
         <v>713</v>
       </c>
-      <c r="M116" s="1">
-        <v>46372</v>
+      <c r="M116" s="2">
+        <v>46375</v>
       </c>
       <c r="N116" t="s">
         <v>717</v>
@@ -15680,8 +15706,8 @@
       <c r="L117" t="s">
         <v>713</v>
       </c>
-      <c r="M117" s="1">
-        <v>46372</v>
+      <c r="M117" s="2">
+        <v>46375</v>
       </c>
       <c r="N117" t="s">
         <v>717</v>
@@ -15724,8 +15750,8 @@
       <c r="L118" t="s">
         <v>713</v>
       </c>
-      <c r="M118" s="1">
-        <v>46372</v>
+      <c r="M118" s="2">
+        <v>46375</v>
       </c>
       <c r="N118" t="s">
         <v>717</v>
@@ -15768,8 +15794,8 @@
       <c r="L119" t="s">
         <v>713</v>
       </c>
-      <c r="M119" s="1">
-        <v>46372</v>
+      <c r="M119" s="2">
+        <v>46375</v>
       </c>
       <c r="N119" t="s">
         <v>717</v>
@@ -15812,8 +15838,8 @@
       <c r="L120" t="s">
         <v>713</v>
       </c>
-      <c r="M120" s="1">
-        <v>46372</v>
+      <c r="M120" s="2">
+        <v>46375</v>
       </c>
       <c r="N120" t="s">
         <v>717</v>
@@ -15856,8 +15882,8 @@
       <c r="L121" t="s">
         <v>716</v>
       </c>
-      <c r="M121" s="1">
-        <v>46387</v>
+      <c r="M121" s="2">
+        <v>46390</v>
       </c>
       <c r="N121" t="s">
         <v>717</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (06/10/2026 13:46)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3096" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3116" uniqueCount="723">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1595,6 +1595,12 @@
     <t>LST267011U8</t>
   </si>
   <si>
+    <t>LST274003U8</t>
+  </si>
+  <si>
+    <t>LST274005U8</t>
+  </si>
+  <si>
     <t>A-1636-32</t>
   </si>
   <si>
@@ -1895,6 +1901,12 @@
     <t>2651040-2</t>
   </si>
   <si>
+    <t>011-00868-10</t>
+  </si>
+  <si>
+    <t>MS20365-1032</t>
+  </si>
+  <si>
     <t>BUSHING</t>
   </si>
   <si>
@@ -2153,19 +2165,22 @@
     <t>ENGINE MOUNT WELD ASSEMBLY</t>
   </si>
   <si>
+    <t>UNIT-AHRS</t>
+  </si>
+  <si>
     <t>Empenho Solicitado</t>
   </si>
   <si>
+    <t>Selecionada em Plano</t>
+  </si>
+  <si>
+    <t>Mapa Gerado</t>
+  </si>
+  <si>
+    <t>Análise do Pedido</t>
+  </si>
+  <si>
     <t>Validada</t>
-  </si>
-  <si>
-    <t>Selecionada em Plano</t>
-  </si>
-  <si>
-    <t>Mapa Gerado</t>
-  </si>
-  <si>
-    <t>Análise do Pedido</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10646,7 +10661,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q121"/>
+  <dimension ref="A1:Q123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -10728,7 +10743,7 @@
         <v>516.34</v>
       </c>
       <c r="I2" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J2" t="s">
         <v>388</v>
@@ -10769,7 +10784,7 @@
         <v>191.04</v>
       </c>
       <c r="I3" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J3" t="s">
         <v>388</v>
@@ -10795,7 +10810,7 @@
         <v>173</v>
       </c>
       <c r="D4" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E4" t="s">
         <v>297</v>
@@ -10810,7 +10825,7 @@
         <v>314.56</v>
       </c>
       <c r="I4" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J4" t="s">
         <v>388</v>
@@ -10836,10 +10851,10 @@
         <v>173</v>
       </c>
       <c r="D5" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="E5" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="F5">
         <v>7</v>
@@ -10851,7 +10866,7 @@
         <v>1859.13</v>
       </c>
       <c r="I5" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J5" t="s">
         <v>388</v>
@@ -10892,7 +10907,7 @@
         <v>1572.48</v>
       </c>
       <c r="I6" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J6" t="s">
         <v>388</v>
@@ -10933,7 +10948,7 @@
         <v>1148.68</v>
       </c>
       <c r="I7" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J7" t="s">
         <v>388</v>
@@ -11000,7 +11015,7 @@
         <v>173</v>
       </c>
       <c r="D9" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="E9" t="s">
         <v>298</v>
@@ -11015,7 +11030,7 @@
         <v>174</v>
       </c>
       <c r="I9" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J9" t="s">
         <v>388</v>
@@ -11041,10 +11056,10 @@
         <v>173</v>
       </c>
       <c r="D10" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="E10" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="F10">
         <v>4</v>
@@ -11056,22 +11071,22 @@
         <v>588.8</v>
       </c>
       <c r="I10" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J10" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K10" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L10" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M10" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N10" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -11085,7 +11100,7 @@
         <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="E11" t="s">
         <v>341</v>
@@ -11100,22 +11115,22 @@
         <v>862.6799999999999</v>
       </c>
       <c r="I11" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J11" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K11" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L11" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M11" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N11" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -11129,10 +11144,10 @@
         <v>173</v>
       </c>
       <c r="D12" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E12" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="F12">
         <v>2</v>
@@ -11185,7 +11200,7 @@
         <v>2292.34</v>
       </c>
       <c r="I13" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J13" t="s">
         <v>387</v>
@@ -11211,10 +11226,10 @@
         <v>173</v>
       </c>
       <c r="D14" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="E14" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="F14">
         <v>21</v>
@@ -11226,7 +11241,7 @@
         <v>10768.59</v>
       </c>
       <c r="I14" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J14" t="s">
         <v>387</v>
@@ -11252,10 +11267,10 @@
         <v>173</v>
       </c>
       <c r="D15" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="E15" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -11267,7 +11282,7 @@
         <v>11325.54</v>
       </c>
       <c r="I15" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J15" t="s">
         <v>387</v>
@@ -11293,10 +11308,10 @@
         <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="E16" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="F16">
         <v>3</v>
@@ -11308,22 +11323,22 @@
         <v>140.58</v>
       </c>
       <c r="I16" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J16" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K16" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L16" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M16" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N16" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -11337,10 +11352,10 @@
         <v>173</v>
       </c>
       <c r="D17" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="E17" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -11352,7 +11367,7 @@
         <v>1076.62</v>
       </c>
       <c r="I17" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J17" t="s">
         <v>380</v>
@@ -11378,10 +11393,10 @@
         <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="E18" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="F18">
         <v>2</v>
@@ -11419,10 +11434,10 @@
         <v>173</v>
       </c>
       <c r="D19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="E19" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="F19">
         <v>10</v>
@@ -11434,22 +11449,22 @@
         <v>1323.9</v>
       </c>
       <c r="I19" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J19" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K19" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L19" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M19" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N19" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11463,10 +11478,10 @@
         <v>173</v>
       </c>
       <c r="D20" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="E20" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -11478,22 +11493,22 @@
         <v>340.73</v>
       </c>
       <c r="I20" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J20" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K20" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L20" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M20" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N20" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11507,10 +11522,10 @@
         <v>173</v>
       </c>
       <c r="D21" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="E21" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="F21">
         <v>5</v>
@@ -11525,19 +11540,19 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K21" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L21" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M21" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N21" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11551,10 +11566,10 @@
         <v>173</v>
       </c>
       <c r="D22" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="E22" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -11566,7 +11581,7 @@
         <v>285.3</v>
       </c>
       <c r="I22" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J22" t="s">
         <v>388</v>
@@ -11592,10 +11607,10 @@
         <v>173</v>
       </c>
       <c r="D23" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="E23" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="F23">
         <v>3</v>
@@ -11607,7 +11622,7 @@
         <v>274.86</v>
       </c>
       <c r="I23" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J23" t="s">
         <v>388</v>
@@ -11633,7 +11648,7 @@
         <v>173</v>
       </c>
       <c r="D24" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="E24" t="s">
         <v>307</v>
@@ -11648,7 +11663,7 @@
         <v>245.6</v>
       </c>
       <c r="I24" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J24" t="s">
         <v>388</v>
@@ -11674,10 +11689,10 @@
         <v>173</v>
       </c>
       <c r="D25" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="E25" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -11689,22 +11704,22 @@
         <v>21612.9</v>
       </c>
       <c r="I25" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J25" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K25" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L25" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M25" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N25" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11718,10 +11733,10 @@
         <v>173</v>
       </c>
       <c r="D26" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="E26" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="F26">
         <v>8</v>
@@ -11733,7 +11748,7 @@
         <v>8029.04</v>
       </c>
       <c r="I26" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J26" t="s">
         <v>388</v>
@@ -11759,10 +11774,10 @@
         <v>173</v>
       </c>
       <c r="D27" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="E27" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="F27">
         <v>7</v>
@@ -11774,7 +11789,7 @@
         <v>9269.4</v>
       </c>
       <c r="I27" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J27" t="s">
         <v>380</v>
@@ -11800,10 +11815,10 @@
         <v>173</v>
       </c>
       <c r="D28" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="E28" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -11818,19 +11833,19 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K28" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L28" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M28" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N28" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11844,10 +11859,10 @@
         <v>173</v>
       </c>
       <c r="D29" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="E29" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="F29">
         <v>20</v>
@@ -11859,22 +11874,22 @@
         <v>24038.4</v>
       </c>
       <c r="I29" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="J29" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="K29" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="L29" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="M29" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="N29" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11888,10 +11903,10 @@
         <v>173</v>
       </c>
       <c r="D30" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E30" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="F30">
         <v>2</v>
@@ -11906,19 +11921,19 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K30" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L30" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M30" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N30" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11932,10 +11947,10 @@
         <v>173</v>
       </c>
       <c r="D31" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="E31" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -11947,22 +11962,22 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="J31" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="K31" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="L31" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="M31" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="N31" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11976,10 +11991,10 @@
         <v>173</v>
       </c>
       <c r="D32" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="E32" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -11991,7 +12006,7 @@
         <v>15090</v>
       </c>
       <c r="I32" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J32" t="s">
         <v>380</v>
@@ -12017,10 +12032,10 @@
         <v>173</v>
       </c>
       <c r="D33" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="E33" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -12032,7 +12047,7 @@
         <v>1527.63</v>
       </c>
       <c r="I33" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J33" t="s">
         <v>380</v>
@@ -12058,10 +12073,10 @@
         <v>173</v>
       </c>
       <c r="D34" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E34" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -12073,7 +12088,7 @@
         <v>5078.8</v>
       </c>
       <c r="I34" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J34" t="s">
         <v>380</v>
@@ -12099,10 +12114,10 @@
         <v>173</v>
       </c>
       <c r="D35" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="E35" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -12114,7 +12129,7 @@
         <v>828.12</v>
       </c>
       <c r="I35" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J35" t="s">
         <v>380</v>
@@ -12140,10 +12155,10 @@
         <v>173</v>
       </c>
       <c r="D36" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="E36" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="F36">
         <v>36</v>
@@ -12155,7 +12170,7 @@
         <v>4016.16</v>
       </c>
       <c r="I36" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J36" t="s">
         <v>380</v>
@@ -12181,10 +12196,10 @@
         <v>173</v>
       </c>
       <c r="D37" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="E37" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="F37">
         <v>2</v>
@@ -12196,7 +12211,7 @@
         <v>2270.92</v>
       </c>
       <c r="I37" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J37" t="s">
         <v>387</v>
@@ -12222,10 +12237,10 @@
         <v>173</v>
       </c>
       <c r="D38" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="E38" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="F38">
         <v>5</v>
@@ -12237,7 +12252,7 @@
         <v>3100.05</v>
       </c>
       <c r="I38" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J38" t="s">
         <v>380</v>
@@ -12263,10 +12278,10 @@
         <v>173</v>
       </c>
       <c r="D39" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="E39" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="F39">
         <v>4</v>
@@ -12304,10 +12319,10 @@
         <v>173</v>
       </c>
       <c r="D40" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="E40" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="F40">
         <v>2</v>
@@ -12319,7 +12334,7 @@
         <v>15180.86</v>
       </c>
       <c r="I40" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J40" t="s">
         <v>380</v>
@@ -12345,10 +12360,10 @@
         <v>173</v>
       </c>
       <c r="D41" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="E41" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -12363,19 +12378,19 @@
         <v>382</v>
       </c>
       <c r="J41" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K41" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L41" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M41" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N41" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -12404,7 +12419,7 @@
         <v>210381.85</v>
       </c>
       <c r="I42" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J42" t="s">
         <v>387</v>
@@ -12430,10 +12445,10 @@
         <v>173</v>
       </c>
       <c r="D43" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="E43" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -12445,22 +12460,22 @@
         <v>7890.58</v>
       </c>
       <c r="I43" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J43" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K43" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L43" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M43" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N43" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12474,7 +12489,7 @@
         <v>173</v>
       </c>
       <c r="D44" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="E44" t="s">
         <v>296</v>
@@ -12489,22 +12504,22 @@
         <v>352.52</v>
       </c>
       <c r="I44" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J44" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K44" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L44" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M44" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N44" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12518,10 +12533,10 @@
         <v>173</v>
       </c>
       <c r="D45" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="E45" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="F45">
         <v>2</v>
@@ -12533,22 +12548,22 @@
         <v>376.62</v>
       </c>
       <c r="I45" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J45" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K45" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L45" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M45" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N45" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12562,10 +12577,10 @@
         <v>173</v>
       </c>
       <c r="D46" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="E46" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="F46">
         <v>2</v>
@@ -12577,7 +12592,7 @@
         <v>1721.52</v>
       </c>
       <c r="I46" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J46" t="s">
         <v>380</v>
@@ -12603,10 +12618,10 @@
         <v>173</v>
       </c>
       <c r="D47" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="E47" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="F47">
         <v>2</v>
@@ -12618,7 +12633,7 @@
         <v>2577.94</v>
       </c>
       <c r="I47" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="J47" t="s">
         <v>380</v>
@@ -12644,10 +12659,10 @@
         <v>173</v>
       </c>
       <c r="D48" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="E48" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="F48">
         <v>2</v>
@@ -12659,22 +12674,22 @@
         <v>3459.72</v>
       </c>
       <c r="I48" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J48" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K48" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L48" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M48" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N48" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12688,10 +12703,10 @@
         <v>173</v>
       </c>
       <c r="D49" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E49" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="F49">
         <v>9</v>
@@ -12703,22 +12718,22 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="J49" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="K49" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="L49" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="M49" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="N49" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12732,10 +12747,10 @@
         <v>173</v>
       </c>
       <c r="D50" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="E50" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="F50">
         <v>1</v>
@@ -12747,22 +12762,22 @@
         <v>4208.01</v>
       </c>
       <c r="I50" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="J50" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="K50" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="L50" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="M50" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="N50" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12776,10 +12791,10 @@
         <v>173</v>
       </c>
       <c r="D51" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="E51" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="F51">
         <v>4</v>
@@ -12794,19 +12809,19 @@
         <v>382</v>
       </c>
       <c r="J51" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K51" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L51" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M51" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N51" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12820,10 +12835,10 @@
         <v>173</v>
       </c>
       <c r="D52" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E52" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -12838,19 +12853,19 @@
         <v>382</v>
       </c>
       <c r="J52" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K52" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L52" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M52" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N52" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12864,10 +12879,10 @@
         <v>173</v>
       </c>
       <c r="D53" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="E53" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="F53">
         <v>2</v>
@@ -12882,19 +12897,19 @@
         <v>382</v>
       </c>
       <c r="J53" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K53" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L53" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M53" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N53" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12908,10 +12923,10 @@
         <v>173</v>
       </c>
       <c r="D54" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="E54" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="F54">
         <v>4</v>
@@ -12923,22 +12938,22 @@
         <v>3875.24</v>
       </c>
       <c r="I54" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J54" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K54" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L54" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M54" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N54" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12952,10 +12967,10 @@
         <v>173</v>
       </c>
       <c r="D55" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="E55" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="F55">
         <v>1</v>
@@ -12967,22 +12982,22 @@
         <v>84382.42999999999</v>
       </c>
       <c r="I55" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J55" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K55" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L55" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M55" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N55" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -12996,10 +13011,10 @@
         <v>173</v>
       </c>
       <c r="D56" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="E56" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="F56">
         <v>1</v>
@@ -13011,22 +13026,22 @@
         <v>3576.55</v>
       </c>
       <c r="I56" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="J56" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="K56" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="L56" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="M56" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="N56" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -13040,10 +13055,10 @@
         <v>173</v>
       </c>
       <c r="D57" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="E57" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="F57">
         <v>1</v>
@@ -13055,22 +13070,22 @@
         <v>908.11</v>
       </c>
       <c r="I57" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="J57" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="K57" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="L57" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="M57" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="N57" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -13084,10 +13099,10 @@
         <v>173</v>
       </c>
       <c r="D58" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="E58" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="F58">
         <v>4</v>
@@ -13099,22 +13114,22 @@
         <v>1500.8</v>
       </c>
       <c r="I58" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="J58" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="K58" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="L58" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="M58" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="N58" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -13143,22 +13158,22 @@
         <v>869.98</v>
       </c>
       <c r="I59" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J59" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K59" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L59" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M59" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N59" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -13172,10 +13187,10 @@
         <v>173</v>
       </c>
       <c r="D60" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="E60" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="F60">
         <v>3</v>
@@ -13187,22 +13202,22 @@
         <v>1379.52</v>
       </c>
       <c r="I60" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="J60" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="K60" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="L60" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="M60" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="N60" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="61" spans="1:14">
@@ -13216,10 +13231,10 @@
         <v>173</v>
       </c>
       <c r="D61" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E61" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="F61">
         <v>5</v>
@@ -13231,22 +13246,22 @@
         <v>5645.05</v>
       </c>
       <c r="I61" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="J61" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="K61" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="L61" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="M61" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="N61" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="62" spans="1:14">
@@ -13260,10 +13275,10 @@
         <v>173</v>
       </c>
       <c r="D62" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="E62" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="F62">
         <v>21</v>
@@ -13275,22 +13290,22 @@
         <v>204.96</v>
       </c>
       <c r="I62" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J62" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K62" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L62" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M62" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N62" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="63" spans="1:14">
@@ -13319,22 +13334,22 @@
         <v>421</v>
       </c>
       <c r="I63" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J63" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K63" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L63" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M63" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N63" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="64" spans="1:14">
@@ -13348,7 +13363,7 @@
         <v>173</v>
       </c>
       <c r="D64" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E64" t="s">
         <v>308</v>
@@ -13363,22 +13378,22 @@
         <v>1999.52</v>
       </c>
       <c r="I64" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J64" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K64" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L64" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M64" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N64" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="65" spans="1:14">
@@ -13392,10 +13407,10 @@
         <v>173</v>
       </c>
       <c r="D65" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="E65" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="F65">
         <v>2</v>
@@ -13407,22 +13422,22 @@
         <v>8848.459999999999</v>
       </c>
       <c r="I65" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J65" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K65" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L65" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M65" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N65" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="66" spans="1:14">
@@ -13436,10 +13451,10 @@
         <v>173</v>
       </c>
       <c r="D66" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E66" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="F66">
         <v>2</v>
@@ -13451,22 +13466,22 @@
         <v>297.92</v>
       </c>
       <c r="I66" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J66" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K66" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L66" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M66" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N66" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="67" spans="1:14">
@@ -13480,10 +13495,10 @@
         <v>173</v>
       </c>
       <c r="D67" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="E67" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="F67">
         <v>1</v>
@@ -13495,22 +13510,22 @@
         <v>27326.55</v>
       </c>
       <c r="I67" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J67" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K67" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L67" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M67" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N67" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="68" spans="1:14">
@@ -13524,7 +13539,7 @@
         <v>173</v>
       </c>
       <c r="D68" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="E68" t="s">
         <v>298</v>
@@ -13539,22 +13554,22 @@
         <v>806.24</v>
       </c>
       <c r="I68" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J68" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K68" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L68" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M68" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N68" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="69" spans="1:14">
@@ -13568,10 +13583,10 @@
         <v>173</v>
       </c>
       <c r="D69" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="E69" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="F69">
         <v>8</v>
@@ -13583,22 +13598,22 @@
         <v>11124.8</v>
       </c>
       <c r="I69" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J69" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K69" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L69" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M69" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N69" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="70" spans="1:14">
@@ -13627,22 +13642,22 @@
         <v>1658.28</v>
       </c>
       <c r="I70" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J70" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K70" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L70" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M70" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N70" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="71" spans="1:14">
@@ -13671,22 +13686,22 @@
         <v>3968.48</v>
       </c>
       <c r="I71" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J71" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K71" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L71" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M71" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N71" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="72" spans="1:14">
@@ -13700,7 +13715,7 @@
         <v>173</v>
       </c>
       <c r="D72" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="E72" t="s">
         <v>294</v>
@@ -13715,22 +13730,22 @@
         <v>400</v>
       </c>
       <c r="I72" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J72" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K72" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L72" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M72" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N72" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="73" spans="1:14">
@@ -13744,10 +13759,10 @@
         <v>173</v>
       </c>
       <c r="D73" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="E73" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="F73">
         <v>2</v>
@@ -13759,22 +13774,22 @@
         <v>3043.76</v>
       </c>
       <c r="I73" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J73" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K73" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L73" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M73" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N73" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="74" spans="1:14">
@@ -13788,10 +13803,10 @@
         <v>173</v>
       </c>
       <c r="D74" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="E74" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="F74">
         <v>4</v>
@@ -13803,22 +13818,22 @@
         <v>2048.32</v>
       </c>
       <c r="I74" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="J74" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K74" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L74" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M74" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N74" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="75" spans="1:14">
@@ -13832,10 +13847,10 @@
         <v>173</v>
       </c>
       <c r="D75" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E75" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="F75">
         <v>1</v>
@@ -13847,22 +13862,22 @@
         <v>1001.2</v>
       </c>
       <c r="I75" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J75" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K75" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L75" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M75" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N75" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="76" spans="1:14">
@@ -13891,22 +13906,22 @@
         <v>196279.8</v>
       </c>
       <c r="I76" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J76" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K76" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L76" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M76" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N76" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="77" spans="1:14">
@@ -13920,10 +13935,10 @@
         <v>173</v>
       </c>
       <c r="D77" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="E77" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="F77">
         <v>3</v>
@@ -13935,22 +13950,22 @@
         <v>6592.5</v>
       </c>
       <c r="I77" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J77" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K77" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L77" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M77" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N77" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="78" spans="1:14">
@@ -13964,10 +13979,10 @@
         <v>173</v>
       </c>
       <c r="D78" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="E78" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="F78">
         <v>8</v>
@@ -13979,22 +13994,22 @@
         <v>4641.76</v>
       </c>
       <c r="I78" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J78" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K78" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L78" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M78" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N78" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="79" spans="1:14">
@@ -14023,22 +14038,22 @@
         <v>2057</v>
       </c>
       <c r="I79" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J79" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K79" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L79" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M79" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N79" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="80" spans="1:14">
@@ -14052,10 +14067,10 @@
         <v>173</v>
       </c>
       <c r="D80" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="E80" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="F80">
         <v>2</v>
@@ -14067,22 +14082,22 @@
         <v>9945.559999999999</v>
       </c>
       <c r="I80" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J80" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K80" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L80" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M80" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N80" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="81" spans="1:14">
@@ -14111,22 +14126,22 @@
         <v>1592.82</v>
       </c>
       <c r="I81" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J81" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K81" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L81" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M81" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N81" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="82" spans="1:14">
@@ -14140,10 +14155,10 @@
         <v>173</v>
       </c>
       <c r="D82" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E82" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="F82">
         <v>4</v>
@@ -14155,22 +14170,22 @@
         <v>1437.36</v>
       </c>
       <c r="I82" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J82" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K82" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L82" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M82" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N82" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="83" spans="1:14">
@@ -14184,10 +14199,10 @@
         <v>173</v>
       </c>
       <c r="D83" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="E83" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="F83">
         <v>1</v>
@@ -14199,22 +14214,22 @@
         <v>2822.4</v>
       </c>
       <c r="I83" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J83" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K83" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L83" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M83" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N83" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="84" spans="1:14">
@@ -14228,10 +14243,10 @@
         <v>173</v>
       </c>
       <c r="D84" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="E84" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="F84">
         <v>7</v>
@@ -14243,22 +14258,22 @@
         <v>20061.44</v>
       </c>
       <c r="I84" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J84" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K84" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L84" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M84" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N84" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="85" spans="1:14">
@@ -14272,10 +14287,10 @@
         <v>173</v>
       </c>
       <c r="D85" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="E85" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="F85">
         <v>7</v>
@@ -14287,22 +14302,22 @@
         <v>21005.95</v>
       </c>
       <c r="I85" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J85" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K85" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L85" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M85" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N85" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="86" spans="1:14">
@@ -14316,10 +14331,10 @@
         <v>173</v>
       </c>
       <c r="D86" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="E86" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="F86">
         <v>4</v>
@@ -14331,22 +14346,22 @@
         <v>13639.68</v>
       </c>
       <c r="I86" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J86" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K86" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L86" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M86" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N86" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="87" spans="1:14">
@@ -14360,7 +14375,7 @@
         <v>173</v>
       </c>
       <c r="D87" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="E87" t="s">
         <v>308</v>
@@ -14375,22 +14390,22 @@
         <v>500.22</v>
       </c>
       <c r="I87" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J87" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K87" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L87" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M87" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N87" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="88" spans="1:14">
@@ -14419,22 +14434,22 @@
         <v>2360</v>
       </c>
       <c r="I88" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J88" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K88" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L88" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M88" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N88" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="89" spans="1:14">
@@ -14448,10 +14463,10 @@
         <v>173</v>
       </c>
       <c r="D89" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="E89" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="F89">
         <v>8</v>
@@ -14463,22 +14478,22 @@
         <v>3394.56</v>
       </c>
       <c r="I89" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J89" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K89" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L89" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M89" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N89" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="90" spans="1:14">
@@ -14492,7 +14507,7 @@
         <v>173</v>
       </c>
       <c r="D90" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="E90" t="s">
         <v>311</v>
@@ -14507,22 +14522,22 @@
         <v>265</v>
       </c>
       <c r="I90" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J90" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K90" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L90" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M90" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N90" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="91" spans="1:14">
@@ -14551,22 +14566,22 @@
         <v>794</v>
       </c>
       <c r="I91" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J91" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K91" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L91" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M91" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N91" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="92" spans="1:14">
@@ -14580,10 +14595,10 @@
         <v>173</v>
       </c>
       <c r="D92" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="E92" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="F92">
         <v>4</v>
@@ -14595,22 +14610,22 @@
         <v>552.28</v>
       </c>
       <c r="I92" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J92" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K92" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L92" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M92" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N92" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="93" spans="1:14">
@@ -14624,10 +14639,10 @@
         <v>173</v>
       </c>
       <c r="D93" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="E93" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="F93">
         <v>11</v>
@@ -14639,22 +14654,22 @@
         <v>735.79</v>
       </c>
       <c r="I93" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J93" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K93" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L93" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M93" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N93" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="94" spans="1:14">
@@ -14668,10 +14683,10 @@
         <v>173</v>
       </c>
       <c r="D94" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E94" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="F94">
         <v>1</v>
@@ -14683,22 +14698,22 @@
         <v>7431.24</v>
       </c>
       <c r="I94" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J94" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K94" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L94" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M94" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N94" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="95" spans="1:14">
@@ -14712,10 +14727,10 @@
         <v>173</v>
       </c>
       <c r="D95" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="E95" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="F95">
         <v>5</v>
@@ -14727,22 +14742,22 @@
         <v>46248.2</v>
       </c>
       <c r="I95" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J95" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K95" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L95" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M95" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N95" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="96" spans="1:14">
@@ -14756,10 +14771,10 @@
         <v>173</v>
       </c>
       <c r="D96" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="E96" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="F96">
         <v>10</v>
@@ -14771,22 +14786,22 @@
         <v>8115.6</v>
       </c>
       <c r="I96" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J96" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K96" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L96" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M96" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N96" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="97" spans="1:14">
@@ -14800,10 +14815,10 @@
         <v>173</v>
       </c>
       <c r="D97" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="E97" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="F97">
         <v>2</v>
@@ -14815,22 +14830,22 @@
         <v>30781.94</v>
       </c>
       <c r="I97" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J97" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K97" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L97" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M97" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N97" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="98" spans="1:14">
@@ -14844,10 +14859,10 @@
         <v>173</v>
       </c>
       <c r="D98" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="E98" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="F98">
         <v>2</v>
@@ -14859,22 +14874,22 @@
         <v>343.54</v>
       </c>
       <c r="I98" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J98" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K98" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L98" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M98" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N98" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="99" spans="1:14">
@@ -14888,7 +14903,7 @@
         <v>173</v>
       </c>
       <c r="D99" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="E99" t="s">
         <v>342</v>
@@ -14903,22 +14918,22 @@
         <v>224.96</v>
       </c>
       <c r="I99" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J99" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K99" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L99" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M99" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N99" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="100" spans="1:14">
@@ -14932,10 +14947,10 @@
         <v>173</v>
       </c>
       <c r="D100" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="E100" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="F100">
         <v>3</v>
@@ -14947,22 +14962,22 @@
         <v>1768.41</v>
       </c>
       <c r="I100" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="J100" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K100" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L100" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M100" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N100" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="101" spans="1:14">
@@ -14976,10 +14991,10 @@
         <v>173</v>
       </c>
       <c r="D101" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="E101" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="F101">
         <v>1</v>
@@ -14991,22 +15006,22 @@
         <v>630</v>
       </c>
       <c r="I101" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J101" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K101" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L101" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M101" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N101" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="102" spans="1:14">
@@ -15020,10 +15035,10 @@
         <v>173</v>
       </c>
       <c r="D102" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E102" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="F102">
         <v>1</v>
@@ -15035,22 +15050,22 @@
         <v>512.98</v>
       </c>
       <c r="I102" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J102" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K102" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L102" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M102" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N102" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="103" spans="1:14">
@@ -15064,10 +15079,10 @@
         <v>173</v>
       </c>
       <c r="D103" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="E103" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="F103">
         <v>2</v>
@@ -15079,22 +15094,22 @@
         <v>7375.36</v>
       </c>
       <c r="I103" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="J103" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K103" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L103" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M103" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N103" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="104" spans="1:14">
@@ -15126,19 +15141,19 @@
         <v>382</v>
       </c>
       <c r="J104" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K104" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L104" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M104" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N104" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="105" spans="1:14">
@@ -15152,10 +15167,10 @@
         <v>173</v>
       </c>
       <c r="D105" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="E105" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="F105">
         <v>3</v>
@@ -15167,22 +15182,22 @@
         <v>1578.63</v>
       </c>
       <c r="I105" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="J105" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K105" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L105" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M105" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N105" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="106" spans="1:14">
@@ -15196,10 +15211,10 @@
         <v>173</v>
       </c>
       <c r="D106" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="E106" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="F106">
         <v>18</v>
@@ -15211,22 +15226,22 @@
         <v>17442</v>
       </c>
       <c r="I106" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="J106" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="K106" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="L106" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M106" s="2">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N106" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="107" spans="1:14">
@@ -15240,10 +15255,10 @@
         <v>173</v>
       </c>
       <c r="D107" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="E107" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="F107">
         <v>1</v>
@@ -15255,22 +15270,22 @@
         <v>3100.94</v>
       </c>
       <c r="I107" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="J107" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K107" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L107" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M107" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N107" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="108" spans="1:14">
@@ -15284,10 +15299,10 @@
         <v>173</v>
       </c>
       <c r="D108" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="E108" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="F108">
         <v>6</v>
@@ -15302,19 +15317,19 @@
         <v>382</v>
       </c>
       <c r="J108" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K108" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L108" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M108" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N108" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="109" spans="1:14">
@@ -15328,7 +15343,7 @@
         <v>173</v>
       </c>
       <c r="D109" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="E109" t="s">
         <v>298</v>
@@ -15337,28 +15352,28 @@
         <v>10</v>
       </c>
       <c r="G109">
-        <v>67.89</v>
+        <v>230</v>
       </c>
       <c r="H109">
-        <v>678.9</v>
+        <v>2300</v>
       </c>
       <c r="I109" t="s">
         <v>382</v>
       </c>
       <c r="J109" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K109" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L109" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M109" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N109" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="110" spans="1:14">
@@ -15372,10 +15387,10 @@
         <v>173</v>
       </c>
       <c r="D110" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="E110" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="F110">
         <v>8</v>
@@ -15387,22 +15402,22 @@
         <v>331.28</v>
       </c>
       <c r="I110" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J110" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K110" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L110" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M110" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N110" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="111" spans="1:14">
@@ -15416,10 +15431,10 @@
         <v>173</v>
       </c>
       <c r="D111" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="E111" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="F111">
         <v>2</v>
@@ -15431,22 +15446,22 @@
         <v>292.42</v>
       </c>
       <c r="I111" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J111" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K111" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L111" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M111" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N111" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="112" spans="1:14">
@@ -15460,10 +15475,10 @@
         <v>173</v>
       </c>
       <c r="D112" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="E112" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="F112">
         <v>5</v>
@@ -15475,22 +15490,22 @@
         <v>8074.8</v>
       </c>
       <c r="I112" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J112" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K112" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L112" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M112" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N112" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="113" spans="1:14">
@@ -15504,10 +15519,10 @@
         <v>173</v>
       </c>
       <c r="D113" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="E113" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="F113">
         <v>2</v>
@@ -15519,22 +15534,22 @@
         <v>2307.56</v>
       </c>
       <c r="I113" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J113" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K113" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L113" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M113" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N113" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="114" spans="1:14">
@@ -15548,10 +15563,10 @@
         <v>173</v>
       </c>
       <c r="D114" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="E114" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="F114">
         <v>3</v>
@@ -15563,22 +15578,22 @@
         <v>7476.63</v>
       </c>
       <c r="I114" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J114" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K114" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L114" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M114" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N114" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="115" spans="1:14">
@@ -15592,10 +15607,10 @@
         <v>173</v>
       </c>
       <c r="D115" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="E115" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="F115">
         <v>4</v>
@@ -15607,22 +15622,22 @@
         <v>16766.88</v>
       </c>
       <c r="I115" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J115" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K115" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L115" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M115" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N115" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="116" spans="1:14">
@@ -15636,10 +15651,10 @@
         <v>173</v>
       </c>
       <c r="D116" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E116" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="F116">
         <v>1</v>
@@ -15651,22 +15666,22 @@
         <v>6320.46</v>
       </c>
       <c r="I116" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J116" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K116" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L116" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M116" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N116" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="117" spans="1:14">
@@ -15680,10 +15695,10 @@
         <v>173</v>
       </c>
       <c r="D117" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="E117" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="F117">
         <v>5</v>
@@ -15695,22 +15710,22 @@
         <v>10420.3</v>
       </c>
       <c r="I117" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J117" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K117" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L117" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M117" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N117" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="118" spans="1:14">
@@ -15724,10 +15739,10 @@
         <v>173</v>
       </c>
       <c r="D118" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E118" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="F118">
         <v>5</v>
@@ -15739,22 +15754,22 @@
         <v>16012.3</v>
       </c>
       <c r="I118" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J118" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K118" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L118" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M118" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N118" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="119" spans="1:14">
@@ -15768,10 +15783,10 @@
         <v>173</v>
       </c>
       <c r="D119" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="E119" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="F119">
         <v>1</v>
@@ -15786,19 +15801,19 @@
         <v>382</v>
       </c>
       <c r="J119" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K119" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L119" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M119" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N119" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="120" spans="1:14">
@@ -15812,10 +15827,10 @@
         <v>173</v>
       </c>
       <c r="D120" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="E120" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="F120">
         <v>2</v>
@@ -15827,22 +15842,22 @@
         <v>24650.24</v>
       </c>
       <c r="I120" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="J120" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="K120" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="L120" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="M120" s="2">
-        <v>46375</v>
+        <v>46376</v>
       </c>
       <c r="N120" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
     </row>
     <row r="121" spans="1:14">
@@ -15856,37 +15871,125 @@
         <v>173</v>
       </c>
       <c r="D121" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="E121" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="F121">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G121">
-        <v>15038</v>
+        <v>17614.88</v>
       </c>
       <c r="H121">
-        <v>165418</v>
+        <v>105689.28</v>
       </c>
       <c r="I121" t="s">
+        <v>720</v>
+      </c>
+      <c r="J121" t="s">
+        <v>720</v>
+      </c>
+      <c r="K121" t="s">
+        <v>720</v>
+      </c>
+      <c r="L121" t="s">
+        <v>720</v>
+      </c>
+      <c r="M121" s="2">
+        <v>46391</v>
+      </c>
+      <c r="N121" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="122" spans="1:14">
+      <c r="A122" t="s">
+        <v>526</v>
+      </c>
+      <c r="B122" t="s">
+        <v>172</v>
+      </c>
+      <c r="C122" t="s">
+        <v>173</v>
+      </c>
+      <c r="D122" t="s">
+        <v>628</v>
+      </c>
+      <c r="E122" t="s">
+        <v>716</v>
+      </c>
+      <c r="F122">
+        <v>2</v>
+      </c>
+      <c r="G122">
+        <v>7466.64</v>
+      </c>
+      <c r="H122">
+        <v>14933.28</v>
+      </c>
+      <c r="I122" t="s">
         <v>382</v>
       </c>
-      <c r="J121" t="s">
-        <v>716</v>
-      </c>
-      <c r="K121" t="s">
-        <v>716</v>
-      </c>
-      <c r="L121" t="s">
-        <v>716</v>
-      </c>
-      <c r="M121" s="2">
-        <v>46390</v>
-      </c>
-      <c r="N121" t="s">
-        <v>717</v>
+      <c r="J122" t="s">
+        <v>721</v>
+      </c>
+      <c r="K122" t="s">
+        <v>721</v>
+      </c>
+      <c r="L122" t="s">
+        <v>721</v>
+      </c>
+      <c r="M122" s="2">
+        <v>46376</v>
+      </c>
+      <c r="N122" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="123" spans="1:14">
+      <c r="A123" t="s">
+        <v>527</v>
+      </c>
+      <c r="B123" t="s">
+        <v>172</v>
+      </c>
+      <c r="C123" t="s">
+        <v>173</v>
+      </c>
+      <c r="D123" t="s">
+        <v>629</v>
+      </c>
+      <c r="E123" t="s">
+        <v>368</v>
+      </c>
+      <c r="F123">
+        <v>1000</v>
+      </c>
+      <c r="G123">
+        <v>0.71</v>
+      </c>
+      <c r="H123">
+        <v>710</v>
+      </c>
+      <c r="I123" t="s">
+        <v>382</v>
+      </c>
+      <c r="J123" t="s">
+        <v>721</v>
+      </c>
+      <c r="K123" t="s">
+        <v>721</v>
+      </c>
+      <c r="L123" t="s">
+        <v>721</v>
+      </c>
+      <c r="M123" s="2">
+        <v>46376</v>
+      </c>
+      <c r="N123" t="s">
+        <v>722</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (06/10/2026 14:10)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2193,16 +2193,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2218,7 +2210,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2226,30 +2218,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2549,55 +2523,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2641,7 +2615,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2685,7 +2659,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2729,7 +2703,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2855,7 +2829,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2899,7 +2873,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2943,7 +2917,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2990,7 +2964,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3113,7 +3087,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -3157,7 +3131,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3201,7 +3175,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3245,7 +3219,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3292,7 +3266,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3336,7 +3310,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3462,7 +3436,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3506,7 +3480,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3591,7 +3565,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3638,7 +3612,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3685,7 +3659,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3729,7 +3703,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3773,7 +3747,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3858,7 +3832,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3943,7 +3917,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3990,7 +3964,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4034,7 +4008,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4078,7 +4052,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4163,7 +4137,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4207,7 +4181,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4251,7 +4225,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4336,7 +4310,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4380,7 +4354,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4424,7 +4398,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4468,7 +4442,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4635,7 +4609,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4679,7 +4653,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4723,7 +4697,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4767,7 +4741,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4814,7 +4788,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4858,7 +4832,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4940,7 +4914,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4984,7 +4958,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5072,7 +5046,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5116,7 +5090,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5163,7 +5137,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5207,7 +5181,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -5251,7 +5225,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5295,7 +5269,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5339,7 +5313,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5386,7 +5360,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5430,7 +5404,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5477,7 +5451,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5521,7 +5495,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5568,7 +5542,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5656,7 +5630,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5700,7 +5674,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5744,7 +5718,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5788,7 +5762,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5832,7 +5806,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5876,7 +5850,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5961,7 +5935,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6005,7 +5979,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -6049,7 +6023,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -6093,7 +6067,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -6137,7 +6111,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -6181,7 +6155,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6225,7 +6199,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6269,7 +6243,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6316,7 +6290,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6360,7 +6334,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6404,7 +6378,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6448,7 +6422,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6492,7 +6466,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6536,7 +6510,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6580,7 +6554,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6624,7 +6598,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6668,7 +6642,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6756,7 +6730,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6800,7 +6774,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6926,7 +6900,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6970,7 +6944,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7014,7 +6988,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7058,7 +7032,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7140,7 +7114,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7184,7 +7158,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7231,7 +7205,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7275,7 +7249,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7401,7 +7375,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7445,7 +7419,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7530,7 +7504,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7574,7 +7548,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7618,7 +7592,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7662,7 +7636,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7706,7 +7680,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7750,7 +7724,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7794,7 +7768,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7838,7 +7812,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7923,7 +7897,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8090,7 +8064,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8134,7 +8108,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8178,7 +8152,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8222,7 +8196,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8266,7 +8240,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8310,7 +8284,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8354,7 +8328,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8439,7 +8413,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8483,7 +8457,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8568,7 +8542,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8694,7 +8668,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8738,7 +8712,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8823,7 +8797,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8867,7 +8841,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8911,7 +8885,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8955,7 +8929,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8999,7 +8973,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -9043,7 +9017,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9087,7 +9061,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9131,7 +9105,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9216,7 +9190,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9383,7 +9357,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9427,7 +9401,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9471,7 +9445,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9515,7 +9489,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9600,7 +9574,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9644,7 +9618,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9688,7 +9662,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9732,7 +9706,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9776,7 +9750,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9820,7 +9794,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9864,7 +9838,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9908,7 +9882,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9952,7 +9926,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9996,7 +9970,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10040,7 +10014,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -10084,7 +10058,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10128,7 +10102,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10172,7 +10146,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -10216,7 +10190,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10260,7 +10234,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10304,7 +10278,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10348,7 +10322,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10392,7 +10366,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10436,7 +10410,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10480,7 +10454,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10565,7 +10539,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10650,7 +10624,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10665,55 +10639,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11082,7 +11056,7 @@
       <c r="L10" t="s">
         <v>721</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46376</v>
       </c>
       <c r="N10" t="s">
@@ -11126,7 +11100,7 @@
       <c r="L11" t="s">
         <v>721</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46376</v>
       </c>
       <c r="N11" t="s">
@@ -11334,7 +11308,7 @@
       <c r="L16" t="s">
         <v>721</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46376</v>
       </c>
       <c r="N16" t="s">
@@ -11460,7 +11434,7 @@
       <c r="L19" t="s">
         <v>721</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46376</v>
       </c>
       <c r="N19" t="s">
@@ -11504,7 +11478,7 @@
       <c r="L20" t="s">
         <v>721</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46376</v>
       </c>
       <c r="N20" t="s">
@@ -11548,7 +11522,7 @@
       <c r="L21" t="s">
         <v>721</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46376</v>
       </c>
       <c r="N21" t="s">
@@ -11715,7 +11689,7 @@
       <c r="L25" t="s">
         <v>721</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46376</v>
       </c>
       <c r="N25" t="s">
@@ -11841,7 +11815,7 @@
       <c r="L28" t="s">
         <v>721</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46376</v>
       </c>
       <c r="N28" t="s">
@@ -11885,7 +11859,7 @@
       <c r="L29" t="s">
         <v>719</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46311</v>
       </c>
       <c r="N29" t="s">
@@ -11929,7 +11903,7 @@
       <c r="L30" t="s">
         <v>721</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46376</v>
       </c>
       <c r="N30" t="s">
@@ -11973,7 +11947,7 @@
       <c r="L31" t="s">
         <v>719</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46311</v>
       </c>
       <c r="N31" t="s">
@@ -12386,7 +12360,7 @@
       <c r="L41" t="s">
         <v>721</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46376</v>
       </c>
       <c r="N41" t="s">
@@ -12471,7 +12445,7 @@
       <c r="L43" t="s">
         <v>721</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46376</v>
       </c>
       <c r="N43" t="s">
@@ -12515,7 +12489,7 @@
       <c r="L44" t="s">
         <v>721</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46376</v>
       </c>
       <c r="N44" t="s">
@@ -12559,7 +12533,7 @@
       <c r="L45" t="s">
         <v>721</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46376</v>
       </c>
       <c r="N45" t="s">
@@ -12685,7 +12659,7 @@
       <c r="L48" t="s">
         <v>721</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46376</v>
       </c>
       <c r="N48" t="s">
@@ -12729,7 +12703,7 @@
       <c r="L49" t="s">
         <v>719</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46311</v>
       </c>
       <c r="N49" t="s">
@@ -12773,7 +12747,7 @@
       <c r="L50" t="s">
         <v>719</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46311</v>
       </c>
       <c r="N50" t="s">
@@ -12817,7 +12791,7 @@
       <c r="L51" t="s">
         <v>721</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46376</v>
       </c>
       <c r="N51" t="s">
@@ -12861,7 +12835,7 @@
       <c r="L52" t="s">
         <v>721</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46376</v>
       </c>
       <c r="N52" t="s">
@@ -12905,7 +12879,7 @@
       <c r="L53" t="s">
         <v>721</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46376</v>
       </c>
       <c r="N53" t="s">
@@ -12949,7 +12923,7 @@
       <c r="L54" t="s">
         <v>721</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46376</v>
       </c>
       <c r="N54" t="s">
@@ -12993,7 +12967,7 @@
       <c r="L55" t="s">
         <v>720</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46391</v>
       </c>
       <c r="N55" t="s">
@@ -13037,7 +13011,7 @@
       <c r="L56" t="s">
         <v>719</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46311</v>
       </c>
       <c r="N56" t="s">
@@ -13081,7 +13055,7 @@
       <c r="L57" t="s">
         <v>719</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46311</v>
       </c>
       <c r="N57" t="s">
@@ -13125,7 +13099,7 @@
       <c r="L58" t="s">
         <v>719</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46311</v>
       </c>
       <c r="N58" t="s">
@@ -13169,7 +13143,7 @@
       <c r="L59" t="s">
         <v>721</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46376</v>
       </c>
       <c r="N59" t="s">
@@ -13213,7 +13187,7 @@
       <c r="L60" t="s">
         <v>719</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46311</v>
       </c>
       <c r="N60" t="s">
@@ -13257,7 +13231,7 @@
       <c r="L61" t="s">
         <v>719</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46311</v>
       </c>
       <c r="N61" t="s">
@@ -13301,7 +13275,7 @@
       <c r="L62" t="s">
         <v>721</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46376</v>
       </c>
       <c r="N62" t="s">
@@ -13345,7 +13319,7 @@
       <c r="L63" t="s">
         <v>721</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46376</v>
       </c>
       <c r="N63" t="s">
@@ -13389,7 +13363,7 @@
       <c r="L64" t="s">
         <v>721</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46376</v>
       </c>
       <c r="N64" t="s">
@@ -13433,7 +13407,7 @@
       <c r="L65" t="s">
         <v>721</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="1">
         <v>46376</v>
       </c>
       <c r="N65" t="s">
@@ -13477,7 +13451,7 @@
       <c r="L66" t="s">
         <v>721</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="1">
         <v>46376</v>
       </c>
       <c r="N66" t="s">
@@ -13521,7 +13495,7 @@
       <c r="L67" t="s">
         <v>721</v>
       </c>
-      <c r="M67" s="2">
+      <c r="M67" s="1">
         <v>46376</v>
       </c>
       <c r="N67" t="s">
@@ -13565,7 +13539,7 @@
       <c r="L68" t="s">
         <v>721</v>
       </c>
-      <c r="M68" s="2">
+      <c r="M68" s="1">
         <v>46376</v>
       </c>
       <c r="N68" t="s">
@@ -13609,7 +13583,7 @@
       <c r="L69" t="s">
         <v>721</v>
       </c>
-      <c r="M69" s="2">
+      <c r="M69" s="1">
         <v>46376</v>
       </c>
       <c r="N69" t="s">
@@ -13653,7 +13627,7 @@
       <c r="L70" t="s">
         <v>721</v>
       </c>
-      <c r="M70" s="2">
+      <c r="M70" s="1">
         <v>46376</v>
       </c>
       <c r="N70" t="s">
@@ -13697,7 +13671,7 @@
       <c r="L71" t="s">
         <v>721</v>
       </c>
-      <c r="M71" s="2">
+      <c r="M71" s="1">
         <v>46376</v>
       </c>
       <c r="N71" t="s">
@@ -13741,7 +13715,7 @@
       <c r="L72" t="s">
         <v>721</v>
       </c>
-      <c r="M72" s="2">
+      <c r="M72" s="1">
         <v>46376</v>
       </c>
       <c r="N72" t="s">
@@ -13785,7 +13759,7 @@
       <c r="L73" t="s">
         <v>721</v>
       </c>
-      <c r="M73" s="2">
+      <c r="M73" s="1">
         <v>46376</v>
       </c>
       <c r="N73" t="s">
@@ -13829,7 +13803,7 @@
       <c r="L74" t="s">
         <v>721</v>
       </c>
-      <c r="M74" s="2">
+      <c r="M74" s="1">
         <v>46376</v>
       </c>
       <c r="N74" t="s">
@@ -13873,7 +13847,7 @@
       <c r="L75" t="s">
         <v>720</v>
       </c>
-      <c r="M75" s="2">
+      <c r="M75" s="1">
         <v>46391</v>
       </c>
       <c r="N75" t="s">
@@ -13917,7 +13891,7 @@
       <c r="L76" t="s">
         <v>720</v>
       </c>
-      <c r="M76" s="2">
+      <c r="M76" s="1">
         <v>46391</v>
       </c>
       <c r="N76" t="s">
@@ -13961,7 +13935,7 @@
       <c r="L77" t="s">
         <v>721</v>
       </c>
-      <c r="M77" s="2">
+      <c r="M77" s="1">
         <v>46376</v>
       </c>
       <c r="N77" t="s">
@@ -14005,7 +13979,7 @@
       <c r="L78" t="s">
         <v>721</v>
       </c>
-      <c r="M78" s="2">
+      <c r="M78" s="1">
         <v>46376</v>
       </c>
       <c r="N78" t="s">
@@ -14049,7 +14023,7 @@
       <c r="L79" t="s">
         <v>721</v>
       </c>
-      <c r="M79" s="2">
+      <c r="M79" s="1">
         <v>46376</v>
       </c>
       <c r="N79" t="s">
@@ -14093,7 +14067,7 @@
       <c r="L80" t="s">
         <v>721</v>
       </c>
-      <c r="M80" s="2">
+      <c r="M80" s="1">
         <v>46376</v>
       </c>
       <c r="N80" t="s">
@@ -14137,7 +14111,7 @@
       <c r="L81" t="s">
         <v>720</v>
       </c>
-      <c r="M81" s="2">
+      <c r="M81" s="1">
         <v>46391</v>
       </c>
       <c r="N81" t="s">
@@ -14181,7 +14155,7 @@
       <c r="L82" t="s">
         <v>721</v>
       </c>
-      <c r="M82" s="2">
+      <c r="M82" s="1">
         <v>46376</v>
       </c>
       <c r="N82" t="s">
@@ -14225,7 +14199,7 @@
       <c r="L83" t="s">
         <v>721</v>
       </c>
-      <c r="M83" s="2">
+      <c r="M83" s="1">
         <v>46376</v>
       </c>
       <c r="N83" t="s">
@@ -14269,7 +14243,7 @@
       <c r="L84" t="s">
         <v>721</v>
       </c>
-      <c r="M84" s="2">
+      <c r="M84" s="1">
         <v>46376</v>
       </c>
       <c r="N84" t="s">
@@ -14313,7 +14287,7 @@
       <c r="L85" t="s">
         <v>721</v>
       </c>
-      <c r="M85" s="2">
+      <c r="M85" s="1">
         <v>46376</v>
       </c>
       <c r="N85" t="s">
@@ -14357,7 +14331,7 @@
       <c r="L86" t="s">
         <v>721</v>
       </c>
-      <c r="M86" s="2">
+      <c r="M86" s="1">
         <v>46376</v>
       </c>
       <c r="N86" t="s">
@@ -14401,7 +14375,7 @@
       <c r="L87" t="s">
         <v>721</v>
       </c>
-      <c r="M87" s="2">
+      <c r="M87" s="1">
         <v>46376</v>
       </c>
       <c r="N87" t="s">
@@ -14445,7 +14419,7 @@
       <c r="L88" t="s">
         <v>720</v>
       </c>
-      <c r="M88" s="2">
+      <c r="M88" s="1">
         <v>46391</v>
       </c>
       <c r="N88" t="s">
@@ -14489,7 +14463,7 @@
       <c r="L89" t="s">
         <v>721</v>
       </c>
-      <c r="M89" s="2">
+      <c r="M89" s="1">
         <v>46376</v>
       </c>
       <c r="N89" t="s">
@@ -14533,7 +14507,7 @@
       <c r="L90" t="s">
         <v>720</v>
       </c>
-      <c r="M90" s="2">
+      <c r="M90" s="1">
         <v>46391</v>
       </c>
       <c r="N90" t="s">
@@ -14577,7 +14551,7 @@
       <c r="L91" t="s">
         <v>720</v>
       </c>
-      <c r="M91" s="2">
+      <c r="M91" s="1">
         <v>46391</v>
       </c>
       <c r="N91" t="s">
@@ -14621,7 +14595,7 @@
       <c r="L92" t="s">
         <v>721</v>
       </c>
-      <c r="M92" s="2">
+      <c r="M92" s="1">
         <v>46376</v>
       </c>
       <c r="N92" t="s">
@@ -14665,7 +14639,7 @@
       <c r="L93" t="s">
         <v>720</v>
       </c>
-      <c r="M93" s="2">
+      <c r="M93" s="1">
         <v>46391</v>
       </c>
       <c r="N93" t="s">
@@ -14709,7 +14683,7 @@
       <c r="L94" t="s">
         <v>720</v>
       </c>
-      <c r="M94" s="2">
+      <c r="M94" s="1">
         <v>46391</v>
       </c>
       <c r="N94" t="s">
@@ -14753,7 +14727,7 @@
       <c r="L95" t="s">
         <v>720</v>
       </c>
-      <c r="M95" s="2">
+      <c r="M95" s="1">
         <v>46391</v>
       </c>
       <c r="N95" t="s">
@@ -14797,7 +14771,7 @@
       <c r="L96" t="s">
         <v>720</v>
       </c>
-      <c r="M96" s="2">
+      <c r="M96" s="1">
         <v>46391</v>
       </c>
       <c r="N96" t="s">
@@ -14841,7 +14815,7 @@
       <c r="L97" t="s">
         <v>721</v>
       </c>
-      <c r="M97" s="2">
+      <c r="M97" s="1">
         <v>46376</v>
       </c>
       <c r="N97" t="s">
@@ -14885,7 +14859,7 @@
       <c r="L98" t="s">
         <v>721</v>
       </c>
-      <c r="M98" s="2">
+      <c r="M98" s="1">
         <v>46376</v>
       </c>
       <c r="N98" t="s">
@@ -14929,7 +14903,7 @@
       <c r="L99" t="s">
         <v>721</v>
       </c>
-      <c r="M99" s="2">
+      <c r="M99" s="1">
         <v>46376</v>
       </c>
       <c r="N99" t="s">
@@ -14973,7 +14947,7 @@
       <c r="L100" t="s">
         <v>721</v>
       </c>
-      <c r="M100" s="2">
+      <c r="M100" s="1">
         <v>46376</v>
       </c>
       <c r="N100" t="s">
@@ -15017,7 +14991,7 @@
       <c r="L101" t="s">
         <v>721</v>
       </c>
-      <c r="M101" s="2">
+      <c r="M101" s="1">
         <v>46376</v>
       </c>
       <c r="N101" t="s">
@@ -15061,7 +15035,7 @@
       <c r="L102" t="s">
         <v>721</v>
       </c>
-      <c r="M102" s="2">
+      <c r="M102" s="1">
         <v>46376</v>
       </c>
       <c r="N102" t="s">
@@ -15105,7 +15079,7 @@
       <c r="L103" t="s">
         <v>721</v>
       </c>
-      <c r="M103" s="2">
+      <c r="M103" s="1">
         <v>46376</v>
       </c>
       <c r="N103" t="s">
@@ -15149,7 +15123,7 @@
       <c r="L104" t="s">
         <v>721</v>
       </c>
-      <c r="M104" s="2">
+      <c r="M104" s="1">
         <v>46376</v>
       </c>
       <c r="N104" t="s">
@@ -15193,7 +15167,7 @@
       <c r="L105" t="s">
         <v>721</v>
       </c>
-      <c r="M105" s="2">
+      <c r="M105" s="1">
         <v>46376</v>
       </c>
       <c r="N105" t="s">
@@ -15237,7 +15211,7 @@
       <c r="L106" t="s">
         <v>720</v>
       </c>
-      <c r="M106" s="2">
+      <c r="M106" s="1">
         <v>46391</v>
       </c>
       <c r="N106" t="s">
@@ -15281,7 +15255,7 @@
       <c r="L107" t="s">
         <v>721</v>
       </c>
-      <c r="M107" s="2">
+      <c r="M107" s="1">
         <v>46376</v>
       </c>
       <c r="N107" t="s">
@@ -15325,7 +15299,7 @@
       <c r="L108" t="s">
         <v>721</v>
       </c>
-      <c r="M108" s="2">
+      <c r="M108" s="1">
         <v>46376</v>
       </c>
       <c r="N108" t="s">
@@ -15369,7 +15343,7 @@
       <c r="L109" t="s">
         <v>721</v>
       </c>
-      <c r="M109" s="2">
+      <c r="M109" s="1">
         <v>46376</v>
       </c>
       <c r="N109" t="s">
@@ -15413,7 +15387,7 @@
       <c r="L110" t="s">
         <v>721</v>
       </c>
-      <c r="M110" s="2">
+      <c r="M110" s="1">
         <v>46376</v>
       </c>
       <c r="N110" t="s">
@@ -15457,7 +15431,7 @@
       <c r="L111" t="s">
         <v>721</v>
       </c>
-      <c r="M111" s="2">
+      <c r="M111" s="1">
         <v>46376</v>
       </c>
       <c r="N111" t="s">
@@ -15501,7 +15475,7 @@
       <c r="L112" t="s">
         <v>721</v>
       </c>
-      <c r="M112" s="2">
+      <c r="M112" s="1">
         <v>46376</v>
       </c>
       <c r="N112" t="s">
@@ -15545,7 +15519,7 @@
       <c r="L113" t="s">
         <v>721</v>
       </c>
-      <c r="M113" s="2">
+      <c r="M113" s="1">
         <v>46376</v>
       </c>
       <c r="N113" t="s">
@@ -15589,7 +15563,7 @@
       <c r="L114" t="s">
         <v>721</v>
       </c>
-      <c r="M114" s="2">
+      <c r="M114" s="1">
         <v>46376</v>
       </c>
       <c r="N114" t="s">
@@ -15633,7 +15607,7 @@
       <c r="L115" t="s">
         <v>721</v>
       </c>
-      <c r="M115" s="2">
+      <c r="M115" s="1">
         <v>46376</v>
       </c>
       <c r="N115" t="s">
@@ -15677,7 +15651,7 @@
       <c r="L116" t="s">
         <v>721</v>
       </c>
-      <c r="M116" s="2">
+      <c r="M116" s="1">
         <v>46376</v>
       </c>
       <c r="N116" t="s">
@@ -15721,7 +15695,7 @@
       <c r="L117" t="s">
         <v>721</v>
       </c>
-      <c r="M117" s="2">
+      <c r="M117" s="1">
         <v>46376</v>
       </c>
       <c r="N117" t="s">
@@ -15765,7 +15739,7 @@
       <c r="L118" t="s">
         <v>721</v>
       </c>
-      <c r="M118" s="2">
+      <c r="M118" s="1">
         <v>46376</v>
       </c>
       <c r="N118" t="s">
@@ -15809,7 +15783,7 @@
       <c r="L119" t="s">
         <v>721</v>
       </c>
-      <c r="M119" s="2">
+      <c r="M119" s="1">
         <v>46376</v>
       </c>
       <c r="N119" t="s">
@@ -15853,7 +15827,7 @@
       <c r="L120" t="s">
         <v>721</v>
       </c>
-      <c r="M120" s="2">
+      <c r="M120" s="1">
         <v>46376</v>
       </c>
       <c r="N120" t="s">
@@ -15897,7 +15871,7 @@
       <c r="L121" t="s">
         <v>720</v>
       </c>
-      <c r="M121" s="2">
+      <c r="M121" s="1">
         <v>46391</v>
       </c>
       <c r="N121" t="s">
@@ -15941,7 +15915,7 @@
       <c r="L122" t="s">
         <v>721</v>
       </c>
-      <c r="M122" s="2">
+      <c r="M122" s="1">
         <v>46376</v>
       </c>
       <c r="N122" t="s">
@@ -15985,7 +15959,7 @@
       <c r="L123" t="s">
         <v>721</v>
       </c>
-      <c r="M123" s="2">
+      <c r="M123" s="1">
         <v>46376</v>
       </c>
       <c r="N123" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (07/10/2026 11:11)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2193,8 +2193,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2210,7 +2218,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2218,12 +2226,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2523,55 +2549,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2615,7 +2641,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2659,7 +2685,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2703,7 +2729,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2829,7 +2855,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2873,7 +2899,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2917,7 +2943,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2964,7 +2990,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3087,7 +3113,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -3131,7 +3157,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3175,7 +3201,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3219,7 +3245,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3266,7 +3292,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3310,7 +3336,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3436,7 +3462,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3480,7 +3506,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3565,7 +3591,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3612,7 +3638,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3659,7 +3685,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3703,7 +3729,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3747,7 +3773,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3832,7 +3858,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3917,7 +3943,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3964,7 +3990,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4008,7 +4034,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4052,7 +4078,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4137,7 +4163,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4181,7 +4207,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4225,7 +4251,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4310,7 +4336,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4354,7 +4380,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4398,7 +4424,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4442,7 +4468,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4609,7 +4635,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4653,7 +4679,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4697,7 +4723,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4741,7 +4767,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4788,7 +4814,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4832,7 +4858,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4914,7 +4940,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4958,7 +4984,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5046,7 +5072,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5090,7 +5116,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5137,7 +5163,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5181,7 +5207,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -5225,7 +5251,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5269,7 +5295,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5313,7 +5339,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5360,7 +5386,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5404,7 +5430,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5451,7 +5477,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5495,7 +5521,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5542,7 +5568,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5630,7 +5656,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5674,7 +5700,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5718,7 +5744,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5762,7 +5788,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5806,7 +5832,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5850,7 +5876,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5935,7 +5961,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5979,7 +6005,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -6023,7 +6049,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -6067,7 +6093,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -6111,7 +6137,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -6155,7 +6181,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6199,7 +6225,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6243,7 +6269,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6290,7 +6316,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6334,7 +6360,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6378,7 +6404,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6422,7 +6448,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6466,7 +6492,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6510,7 +6536,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6554,7 +6580,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6598,7 +6624,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6642,7 +6668,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6730,7 +6756,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6774,7 +6800,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6900,7 +6926,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6944,7 +6970,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6988,7 +7014,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7032,7 +7058,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7114,7 +7140,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7158,7 +7184,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7205,7 +7231,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7249,7 +7275,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7375,7 +7401,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7419,7 +7445,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7504,7 +7530,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7548,7 +7574,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7592,7 +7618,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7636,7 +7662,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7680,7 +7706,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7724,7 +7750,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7768,7 +7794,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7812,7 +7838,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7897,7 +7923,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8064,7 +8090,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8108,7 +8134,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8152,7 +8178,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8196,7 +8222,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8240,7 +8266,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8284,7 +8310,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8328,7 +8354,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8413,7 +8439,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8457,7 +8483,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8542,7 +8568,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8668,7 +8694,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8712,7 +8738,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8797,7 +8823,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8841,7 +8867,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8885,7 +8911,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8929,7 +8955,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8973,7 +8999,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -9017,7 +9043,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9061,7 +9087,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9105,7 +9131,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9190,7 +9216,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9357,7 +9383,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9401,7 +9427,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9445,7 +9471,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9489,7 +9515,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9574,7 +9600,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9618,7 +9644,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9662,7 +9688,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9706,7 +9732,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9750,7 +9776,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9794,7 +9820,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9838,7 +9864,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9882,7 +9908,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9926,7 +9952,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9970,7 +9996,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10014,7 +10040,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -10058,7 +10084,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10102,7 +10128,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10146,7 +10172,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -10190,7 +10216,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10234,7 +10260,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10278,7 +10304,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10322,7 +10348,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10366,7 +10392,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10410,7 +10436,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10454,7 +10480,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10539,7 +10565,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10624,7 +10650,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10639,55 +10665,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11056,8 +11082,8 @@
       <c r="L10" t="s">
         <v>721</v>
       </c>
-      <c r="M10" s="1">
-        <v>46376</v>
+      <c r="M10" s="2">
+        <v>46377</v>
       </c>
       <c r="N10" t="s">
         <v>722</v>
@@ -11100,8 +11126,8 @@
       <c r="L11" t="s">
         <v>721</v>
       </c>
-      <c r="M11" s="1">
-        <v>46376</v>
+      <c r="M11" s="2">
+        <v>46377</v>
       </c>
       <c r="N11" t="s">
         <v>722</v>
@@ -11308,8 +11334,8 @@
       <c r="L16" t="s">
         <v>721</v>
       </c>
-      <c r="M16" s="1">
-        <v>46376</v>
+      <c r="M16" s="2">
+        <v>46377</v>
       </c>
       <c r="N16" t="s">
         <v>722</v>
@@ -11434,8 +11460,8 @@
       <c r="L19" t="s">
         <v>721</v>
       </c>
-      <c r="M19" s="1">
-        <v>46376</v>
+      <c r="M19" s="2">
+        <v>46377</v>
       </c>
       <c r="N19" t="s">
         <v>722</v>
@@ -11478,8 +11504,8 @@
       <c r="L20" t="s">
         <v>721</v>
       </c>
-      <c r="M20" s="1">
-        <v>46376</v>
+      <c r="M20" s="2">
+        <v>46377</v>
       </c>
       <c r="N20" t="s">
         <v>722</v>
@@ -11522,8 +11548,8 @@
       <c r="L21" t="s">
         <v>721</v>
       </c>
-      <c r="M21" s="1">
-        <v>46376</v>
+      <c r="M21" s="2">
+        <v>46377</v>
       </c>
       <c r="N21" t="s">
         <v>722</v>
@@ -11689,8 +11715,8 @@
       <c r="L25" t="s">
         <v>721</v>
       </c>
-      <c r="M25" s="1">
-        <v>46376</v>
+      <c r="M25" s="2">
+        <v>46377</v>
       </c>
       <c r="N25" t="s">
         <v>722</v>
@@ -11815,8 +11841,8 @@
       <c r="L28" t="s">
         <v>721</v>
       </c>
-      <c r="M28" s="1">
-        <v>46376</v>
+      <c r="M28" s="2">
+        <v>46377</v>
       </c>
       <c r="N28" t="s">
         <v>722</v>
@@ -11859,8 +11885,8 @@
       <c r="L29" t="s">
         <v>719</v>
       </c>
-      <c r="M29" s="1">
-        <v>46311</v>
+      <c r="M29" s="2">
+        <v>46312</v>
       </c>
       <c r="N29" t="s">
         <v>722</v>
@@ -11903,8 +11929,8 @@
       <c r="L30" t="s">
         <v>721</v>
       </c>
-      <c r="M30" s="1">
-        <v>46376</v>
+      <c r="M30" s="2">
+        <v>46377</v>
       </c>
       <c r="N30" t="s">
         <v>722</v>
@@ -11947,8 +11973,8 @@
       <c r="L31" t="s">
         <v>719</v>
       </c>
-      <c r="M31" s="1">
-        <v>46311</v>
+      <c r="M31" s="2">
+        <v>46312</v>
       </c>
       <c r="N31" t="s">
         <v>722</v>
@@ -12360,8 +12386,8 @@
       <c r="L41" t="s">
         <v>721</v>
       </c>
-      <c r="M41" s="1">
-        <v>46376</v>
+      <c r="M41" s="2">
+        <v>46377</v>
       </c>
       <c r="N41" t="s">
         <v>722</v>
@@ -12445,8 +12471,8 @@
       <c r="L43" t="s">
         <v>721</v>
       </c>
-      <c r="M43" s="1">
-        <v>46376</v>
+      <c r="M43" s="2">
+        <v>46377</v>
       </c>
       <c r="N43" t="s">
         <v>722</v>
@@ -12489,8 +12515,8 @@
       <c r="L44" t="s">
         <v>721</v>
       </c>
-      <c r="M44" s="1">
-        <v>46376</v>
+      <c r="M44" s="2">
+        <v>46377</v>
       </c>
       <c r="N44" t="s">
         <v>722</v>
@@ -12533,8 +12559,8 @@
       <c r="L45" t="s">
         <v>721</v>
       </c>
-      <c r="M45" s="1">
-        <v>46376</v>
+      <c r="M45" s="2">
+        <v>46377</v>
       </c>
       <c r="N45" t="s">
         <v>722</v>
@@ -12659,8 +12685,8 @@
       <c r="L48" t="s">
         <v>721</v>
       </c>
-      <c r="M48" s="1">
-        <v>46376</v>
+      <c r="M48" s="2">
+        <v>46377</v>
       </c>
       <c r="N48" t="s">
         <v>722</v>
@@ -12703,8 +12729,8 @@
       <c r="L49" t="s">
         <v>719</v>
       </c>
-      <c r="M49" s="1">
-        <v>46311</v>
+      <c r="M49" s="2">
+        <v>46312</v>
       </c>
       <c r="N49" t="s">
         <v>722</v>
@@ -12747,8 +12773,8 @@
       <c r="L50" t="s">
         <v>719</v>
       </c>
-      <c r="M50" s="1">
-        <v>46311</v>
+      <c r="M50" s="2">
+        <v>46312</v>
       </c>
       <c r="N50" t="s">
         <v>722</v>
@@ -12791,8 +12817,8 @@
       <c r="L51" t="s">
         <v>721</v>
       </c>
-      <c r="M51" s="1">
-        <v>46376</v>
+      <c r="M51" s="2">
+        <v>46377</v>
       </c>
       <c r="N51" t="s">
         <v>722</v>
@@ -12835,8 +12861,8 @@
       <c r="L52" t="s">
         <v>721</v>
       </c>
-      <c r="M52" s="1">
-        <v>46376</v>
+      <c r="M52" s="2">
+        <v>46377</v>
       </c>
       <c r="N52" t="s">
         <v>722</v>
@@ -12879,8 +12905,8 @@
       <c r="L53" t="s">
         <v>721</v>
       </c>
-      <c r="M53" s="1">
-        <v>46376</v>
+      <c r="M53" s="2">
+        <v>46377</v>
       </c>
       <c r="N53" t="s">
         <v>722</v>
@@ -12923,8 +12949,8 @@
       <c r="L54" t="s">
         <v>721</v>
       </c>
-      <c r="M54" s="1">
-        <v>46376</v>
+      <c r="M54" s="2">
+        <v>46377</v>
       </c>
       <c r="N54" t="s">
         <v>722</v>
@@ -12967,8 +12993,8 @@
       <c r="L55" t="s">
         <v>720</v>
       </c>
-      <c r="M55" s="1">
-        <v>46391</v>
+      <c r="M55" s="2">
+        <v>46392</v>
       </c>
       <c r="N55" t="s">
         <v>722</v>
@@ -13011,8 +13037,8 @@
       <c r="L56" t="s">
         <v>719</v>
       </c>
-      <c r="M56" s="1">
-        <v>46311</v>
+      <c r="M56" s="2">
+        <v>46312</v>
       </c>
       <c r="N56" t="s">
         <v>722</v>
@@ -13055,8 +13081,8 @@
       <c r="L57" t="s">
         <v>719</v>
       </c>
-      <c r="M57" s="1">
-        <v>46311</v>
+      <c r="M57" s="2">
+        <v>46312</v>
       </c>
       <c r="N57" t="s">
         <v>722</v>
@@ -13099,8 +13125,8 @@
       <c r="L58" t="s">
         <v>719</v>
       </c>
-      <c r="M58" s="1">
-        <v>46311</v>
+      <c r="M58" s="2">
+        <v>46312</v>
       </c>
       <c r="N58" t="s">
         <v>722</v>
@@ -13143,8 +13169,8 @@
       <c r="L59" t="s">
         <v>721</v>
       </c>
-      <c r="M59" s="1">
-        <v>46376</v>
+      <c r="M59" s="2">
+        <v>46377</v>
       </c>
       <c r="N59" t="s">
         <v>722</v>
@@ -13187,8 +13213,8 @@
       <c r="L60" t="s">
         <v>719</v>
       </c>
-      <c r="M60" s="1">
-        <v>46311</v>
+      <c r="M60" s="2">
+        <v>46312</v>
       </c>
       <c r="N60" t="s">
         <v>722</v>
@@ -13231,8 +13257,8 @@
       <c r="L61" t="s">
         <v>719</v>
       </c>
-      <c r="M61" s="1">
-        <v>46311</v>
+      <c r="M61" s="2">
+        <v>46312</v>
       </c>
       <c r="N61" t="s">
         <v>722</v>
@@ -13275,8 +13301,8 @@
       <c r="L62" t="s">
         <v>721</v>
       </c>
-      <c r="M62" s="1">
-        <v>46376</v>
+      <c r="M62" s="2">
+        <v>46377</v>
       </c>
       <c r="N62" t="s">
         <v>722</v>
@@ -13319,8 +13345,8 @@
       <c r="L63" t="s">
         <v>721</v>
       </c>
-      <c r="M63" s="1">
-        <v>46376</v>
+      <c r="M63" s="2">
+        <v>46377</v>
       </c>
       <c r="N63" t="s">
         <v>722</v>
@@ -13363,8 +13389,8 @@
       <c r="L64" t="s">
         <v>721</v>
       </c>
-      <c r="M64" s="1">
-        <v>46376</v>
+      <c r="M64" s="2">
+        <v>46377</v>
       </c>
       <c r="N64" t="s">
         <v>722</v>
@@ -13407,8 +13433,8 @@
       <c r="L65" t="s">
         <v>721</v>
       </c>
-      <c r="M65" s="1">
-        <v>46376</v>
+      <c r="M65" s="2">
+        <v>46377</v>
       </c>
       <c r="N65" t="s">
         <v>722</v>
@@ -13451,8 +13477,8 @@
       <c r="L66" t="s">
         <v>721</v>
       </c>
-      <c r="M66" s="1">
-        <v>46376</v>
+      <c r="M66" s="2">
+        <v>46377</v>
       </c>
       <c r="N66" t="s">
         <v>722</v>
@@ -13495,8 +13521,8 @@
       <c r="L67" t="s">
         <v>721</v>
       </c>
-      <c r="M67" s="1">
-        <v>46376</v>
+      <c r="M67" s="2">
+        <v>46377</v>
       </c>
       <c r="N67" t="s">
         <v>722</v>
@@ -13539,8 +13565,8 @@
       <c r="L68" t="s">
         <v>721</v>
       </c>
-      <c r="M68" s="1">
-        <v>46376</v>
+      <c r="M68" s="2">
+        <v>46377</v>
       </c>
       <c r="N68" t="s">
         <v>722</v>
@@ -13583,8 +13609,8 @@
       <c r="L69" t="s">
         <v>721</v>
       </c>
-      <c r="M69" s="1">
-        <v>46376</v>
+      <c r="M69" s="2">
+        <v>46377</v>
       </c>
       <c r="N69" t="s">
         <v>722</v>
@@ -13627,8 +13653,8 @@
       <c r="L70" t="s">
         <v>721</v>
       </c>
-      <c r="M70" s="1">
-        <v>46376</v>
+      <c r="M70" s="2">
+        <v>46377</v>
       </c>
       <c r="N70" t="s">
         <v>722</v>
@@ -13671,8 +13697,8 @@
       <c r="L71" t="s">
         <v>721</v>
       </c>
-      <c r="M71" s="1">
-        <v>46376</v>
+      <c r="M71" s="2">
+        <v>46377</v>
       </c>
       <c r="N71" t="s">
         <v>722</v>
@@ -13715,8 +13741,8 @@
       <c r="L72" t="s">
         <v>721</v>
       </c>
-      <c r="M72" s="1">
-        <v>46376</v>
+      <c r="M72" s="2">
+        <v>46377</v>
       </c>
       <c r="N72" t="s">
         <v>722</v>
@@ -13759,8 +13785,8 @@
       <c r="L73" t="s">
         <v>721</v>
       </c>
-      <c r="M73" s="1">
-        <v>46376</v>
+      <c r="M73" s="2">
+        <v>46377</v>
       </c>
       <c r="N73" t="s">
         <v>722</v>
@@ -13803,8 +13829,8 @@
       <c r="L74" t="s">
         <v>721</v>
       </c>
-      <c r="M74" s="1">
-        <v>46376</v>
+      <c r="M74" s="2">
+        <v>46377</v>
       </c>
       <c r="N74" t="s">
         <v>722</v>
@@ -13847,8 +13873,8 @@
       <c r="L75" t="s">
         <v>720</v>
       </c>
-      <c r="M75" s="1">
-        <v>46391</v>
+      <c r="M75" s="2">
+        <v>46392</v>
       </c>
       <c r="N75" t="s">
         <v>722</v>
@@ -13891,8 +13917,8 @@
       <c r="L76" t="s">
         <v>720</v>
       </c>
-      <c r="M76" s="1">
-        <v>46391</v>
+      <c r="M76" s="2">
+        <v>46392</v>
       </c>
       <c r="N76" t="s">
         <v>722</v>
@@ -13935,8 +13961,8 @@
       <c r="L77" t="s">
         <v>721</v>
       </c>
-      <c r="M77" s="1">
-        <v>46376</v>
+      <c r="M77" s="2">
+        <v>46377</v>
       </c>
       <c r="N77" t="s">
         <v>722</v>
@@ -13979,8 +14005,8 @@
       <c r="L78" t="s">
         <v>721</v>
       </c>
-      <c r="M78" s="1">
-        <v>46376</v>
+      <c r="M78" s="2">
+        <v>46377</v>
       </c>
       <c r="N78" t="s">
         <v>722</v>
@@ -14023,8 +14049,8 @@
       <c r="L79" t="s">
         <v>721</v>
       </c>
-      <c r="M79" s="1">
-        <v>46376</v>
+      <c r="M79" s="2">
+        <v>46377</v>
       </c>
       <c r="N79" t="s">
         <v>722</v>
@@ -14067,8 +14093,8 @@
       <c r="L80" t="s">
         <v>721</v>
       </c>
-      <c r="M80" s="1">
-        <v>46376</v>
+      <c r="M80" s="2">
+        <v>46377</v>
       </c>
       <c r="N80" t="s">
         <v>722</v>
@@ -14111,8 +14137,8 @@
       <c r="L81" t="s">
         <v>720</v>
       </c>
-      <c r="M81" s="1">
-        <v>46391</v>
+      <c r="M81" s="2">
+        <v>46392</v>
       </c>
       <c r="N81" t="s">
         <v>722</v>
@@ -14155,8 +14181,8 @@
       <c r="L82" t="s">
         <v>721</v>
       </c>
-      <c r="M82" s="1">
-        <v>46376</v>
+      <c r="M82" s="2">
+        <v>46377</v>
       </c>
       <c r="N82" t="s">
         <v>722</v>
@@ -14199,8 +14225,8 @@
       <c r="L83" t="s">
         <v>721</v>
       </c>
-      <c r="M83" s="1">
-        <v>46376</v>
+      <c r="M83" s="2">
+        <v>46377</v>
       </c>
       <c r="N83" t="s">
         <v>722</v>
@@ -14243,8 +14269,8 @@
       <c r="L84" t="s">
         <v>721</v>
       </c>
-      <c r="M84" s="1">
-        <v>46376</v>
+      <c r="M84" s="2">
+        <v>46377</v>
       </c>
       <c r="N84" t="s">
         <v>722</v>
@@ -14287,8 +14313,8 @@
       <c r="L85" t="s">
         <v>721</v>
       </c>
-      <c r="M85" s="1">
-        <v>46376</v>
+      <c r="M85" s="2">
+        <v>46377</v>
       </c>
       <c r="N85" t="s">
         <v>722</v>
@@ -14331,8 +14357,8 @@
       <c r="L86" t="s">
         <v>721</v>
       </c>
-      <c r="M86" s="1">
-        <v>46376</v>
+      <c r="M86" s="2">
+        <v>46377</v>
       </c>
       <c r="N86" t="s">
         <v>722</v>
@@ -14375,8 +14401,8 @@
       <c r="L87" t="s">
         <v>721</v>
       </c>
-      <c r="M87" s="1">
-        <v>46376</v>
+      <c r="M87" s="2">
+        <v>46377</v>
       </c>
       <c r="N87" t="s">
         <v>722</v>
@@ -14419,8 +14445,8 @@
       <c r="L88" t="s">
         <v>720</v>
       </c>
-      <c r="M88" s="1">
-        <v>46391</v>
+      <c r="M88" s="2">
+        <v>46392</v>
       </c>
       <c r="N88" t="s">
         <v>722</v>
@@ -14463,8 +14489,8 @@
       <c r="L89" t="s">
         <v>721</v>
       </c>
-      <c r="M89" s="1">
-        <v>46376</v>
+      <c r="M89" s="2">
+        <v>46377</v>
       </c>
       <c r="N89" t="s">
         <v>722</v>
@@ -14507,8 +14533,8 @@
       <c r="L90" t="s">
         <v>720</v>
       </c>
-      <c r="M90" s="1">
-        <v>46391</v>
+      <c r="M90" s="2">
+        <v>46392</v>
       </c>
       <c r="N90" t="s">
         <v>722</v>
@@ -14551,8 +14577,8 @@
       <c r="L91" t="s">
         <v>720</v>
       </c>
-      <c r="M91" s="1">
-        <v>46391</v>
+      <c r="M91" s="2">
+        <v>46392</v>
       </c>
       <c r="N91" t="s">
         <v>722</v>
@@ -14595,8 +14621,8 @@
       <c r="L92" t="s">
         <v>721</v>
       </c>
-      <c r="M92" s="1">
-        <v>46376</v>
+      <c r="M92" s="2">
+        <v>46377</v>
       </c>
       <c r="N92" t="s">
         <v>722</v>
@@ -14639,8 +14665,8 @@
       <c r="L93" t="s">
         <v>720</v>
       </c>
-      <c r="M93" s="1">
-        <v>46391</v>
+      <c r="M93" s="2">
+        <v>46392</v>
       </c>
       <c r="N93" t="s">
         <v>722</v>
@@ -14683,8 +14709,8 @@
       <c r="L94" t="s">
         <v>720</v>
       </c>
-      <c r="M94" s="1">
-        <v>46391</v>
+      <c r="M94" s="2">
+        <v>46392</v>
       </c>
       <c r="N94" t="s">
         <v>722</v>
@@ -14727,8 +14753,8 @@
       <c r="L95" t="s">
         <v>720</v>
       </c>
-      <c r="M95" s="1">
-        <v>46391</v>
+      <c r="M95" s="2">
+        <v>46392</v>
       </c>
       <c r="N95" t="s">
         <v>722</v>
@@ -14771,8 +14797,8 @@
       <c r="L96" t="s">
         <v>720</v>
       </c>
-      <c r="M96" s="1">
-        <v>46391</v>
+      <c r="M96" s="2">
+        <v>46392</v>
       </c>
       <c r="N96" t="s">
         <v>722</v>
@@ -14815,8 +14841,8 @@
       <c r="L97" t="s">
         <v>721</v>
       </c>
-      <c r="M97" s="1">
-        <v>46376</v>
+      <c r="M97" s="2">
+        <v>46377</v>
       </c>
       <c r="N97" t="s">
         <v>722</v>
@@ -14859,8 +14885,8 @@
       <c r="L98" t="s">
         <v>721</v>
       </c>
-      <c r="M98" s="1">
-        <v>46376</v>
+      <c r="M98" s="2">
+        <v>46377</v>
       </c>
       <c r="N98" t="s">
         <v>722</v>
@@ -14903,8 +14929,8 @@
       <c r="L99" t="s">
         <v>721</v>
       </c>
-      <c r="M99" s="1">
-        <v>46376</v>
+      <c r="M99" s="2">
+        <v>46377</v>
       </c>
       <c r="N99" t="s">
         <v>722</v>
@@ -14947,8 +14973,8 @@
       <c r="L100" t="s">
         <v>721</v>
       </c>
-      <c r="M100" s="1">
-        <v>46376</v>
+      <c r="M100" s="2">
+        <v>46377</v>
       </c>
       <c r="N100" t="s">
         <v>722</v>
@@ -14991,8 +15017,8 @@
       <c r="L101" t="s">
         <v>721</v>
       </c>
-      <c r="M101" s="1">
-        <v>46376</v>
+      <c r="M101" s="2">
+        <v>46377</v>
       </c>
       <c r="N101" t="s">
         <v>722</v>
@@ -15035,8 +15061,8 @@
       <c r="L102" t="s">
         <v>721</v>
       </c>
-      <c r="M102" s="1">
-        <v>46376</v>
+      <c r="M102" s="2">
+        <v>46377</v>
       </c>
       <c r="N102" t="s">
         <v>722</v>
@@ -15079,8 +15105,8 @@
       <c r="L103" t="s">
         <v>721</v>
       </c>
-      <c r="M103" s="1">
-        <v>46376</v>
+      <c r="M103" s="2">
+        <v>46377</v>
       </c>
       <c r="N103" t="s">
         <v>722</v>
@@ -15123,8 +15149,8 @@
       <c r="L104" t="s">
         <v>721</v>
       </c>
-      <c r="M104" s="1">
-        <v>46376</v>
+      <c r="M104" s="2">
+        <v>46377</v>
       </c>
       <c r="N104" t="s">
         <v>722</v>
@@ -15167,8 +15193,8 @@
       <c r="L105" t="s">
         <v>721</v>
       </c>
-      <c r="M105" s="1">
-        <v>46376</v>
+      <c r="M105" s="2">
+        <v>46377</v>
       </c>
       <c r="N105" t="s">
         <v>722</v>
@@ -15211,8 +15237,8 @@
       <c r="L106" t="s">
         <v>720</v>
       </c>
-      <c r="M106" s="1">
-        <v>46391</v>
+      <c r="M106" s="2">
+        <v>46392</v>
       </c>
       <c r="N106" t="s">
         <v>722</v>
@@ -15255,8 +15281,8 @@
       <c r="L107" t="s">
         <v>721</v>
       </c>
-      <c r="M107" s="1">
-        <v>46376</v>
+      <c r="M107" s="2">
+        <v>46377</v>
       </c>
       <c r="N107" t="s">
         <v>722</v>
@@ -15299,8 +15325,8 @@
       <c r="L108" t="s">
         <v>721</v>
       </c>
-      <c r="M108" s="1">
-        <v>46376</v>
+      <c r="M108" s="2">
+        <v>46377</v>
       </c>
       <c r="N108" t="s">
         <v>722</v>
@@ -15343,8 +15369,8 @@
       <c r="L109" t="s">
         <v>721</v>
       </c>
-      <c r="M109" s="1">
-        <v>46376</v>
+      <c r="M109" s="2">
+        <v>46377</v>
       </c>
       <c r="N109" t="s">
         <v>722</v>
@@ -15387,8 +15413,8 @@
       <c r="L110" t="s">
         <v>721</v>
       </c>
-      <c r="M110" s="1">
-        <v>46376</v>
+      <c r="M110" s="2">
+        <v>46377</v>
       </c>
       <c r="N110" t="s">
         <v>722</v>
@@ -15431,8 +15457,8 @@
       <c r="L111" t="s">
         <v>721</v>
       </c>
-      <c r="M111" s="1">
-        <v>46376</v>
+      <c r="M111" s="2">
+        <v>46377</v>
       </c>
       <c r="N111" t="s">
         <v>722</v>
@@ -15475,8 +15501,8 @@
       <c r="L112" t="s">
         <v>721</v>
       </c>
-      <c r="M112" s="1">
-        <v>46376</v>
+      <c r="M112" s="2">
+        <v>46377</v>
       </c>
       <c r="N112" t="s">
         <v>722</v>
@@ -15519,8 +15545,8 @@
       <c r="L113" t="s">
         <v>721</v>
       </c>
-      <c r="M113" s="1">
-        <v>46376</v>
+      <c r="M113" s="2">
+        <v>46377</v>
       </c>
       <c r="N113" t="s">
         <v>722</v>
@@ -15563,8 +15589,8 @@
       <c r="L114" t="s">
         <v>721</v>
       </c>
-      <c r="M114" s="1">
-        <v>46376</v>
+      <c r="M114" s="2">
+        <v>46377</v>
       </c>
       <c r="N114" t="s">
         <v>722</v>
@@ -15607,8 +15633,8 @@
       <c r="L115" t="s">
         <v>721</v>
       </c>
-      <c r="M115" s="1">
-        <v>46376</v>
+      <c r="M115" s="2">
+        <v>46377</v>
       </c>
       <c r="N115" t="s">
         <v>722</v>
@@ -15651,8 +15677,8 @@
       <c r="L116" t="s">
         <v>721</v>
       </c>
-      <c r="M116" s="1">
-        <v>46376</v>
+      <c r="M116" s="2">
+        <v>46377</v>
       </c>
       <c r="N116" t="s">
         <v>722</v>
@@ -15695,8 +15721,8 @@
       <c r="L117" t="s">
         <v>721</v>
       </c>
-      <c r="M117" s="1">
-        <v>46376</v>
+      <c r="M117" s="2">
+        <v>46377</v>
       </c>
       <c r="N117" t="s">
         <v>722</v>
@@ -15739,8 +15765,8 @@
       <c r="L118" t="s">
         <v>721</v>
       </c>
-      <c r="M118" s="1">
-        <v>46376</v>
+      <c r="M118" s="2">
+        <v>46377</v>
       </c>
       <c r="N118" t="s">
         <v>722</v>
@@ -15783,8 +15809,8 @@
       <c r="L119" t="s">
         <v>721</v>
       </c>
-      <c r="M119" s="1">
-        <v>46376</v>
+      <c r="M119" s="2">
+        <v>46377</v>
       </c>
       <c r="N119" t="s">
         <v>722</v>
@@ -15827,8 +15853,8 @@
       <c r="L120" t="s">
         <v>721</v>
       </c>
-      <c r="M120" s="1">
-        <v>46376</v>
+      <c r="M120" s="2">
+        <v>46377</v>
       </c>
       <c r="N120" t="s">
         <v>722</v>
@@ -15871,8 +15897,8 @@
       <c r="L121" t="s">
         <v>720</v>
       </c>
-      <c r="M121" s="1">
-        <v>46391</v>
+      <c r="M121" s="2">
+        <v>46392</v>
       </c>
       <c r="N121" t="s">
         <v>722</v>
@@ -15915,8 +15941,8 @@
       <c r="L122" t="s">
         <v>721</v>
       </c>
-      <c r="M122" s="1">
-        <v>46376</v>
+      <c r="M122" s="2">
+        <v>46377</v>
       </c>
       <c r="N122" t="s">
         <v>722</v>
@@ -15959,8 +15985,8 @@
       <c r="L123" t="s">
         <v>721</v>
       </c>
-      <c r="M123" s="1">
-        <v>46376</v>
+      <c r="M123" s="2">
+        <v>46377</v>
       </c>
       <c r="N123" t="s">
         <v>722</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (07/10/2026 14:47)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2193,16 +2193,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2218,7 +2210,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2226,30 +2218,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2549,55 +2523,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2641,7 +2615,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2685,7 +2659,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2729,7 +2703,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2855,7 +2829,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2899,7 +2873,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2943,7 +2917,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2990,7 +2964,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3113,7 +3087,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -3157,7 +3131,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3201,7 +3175,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3245,7 +3219,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3292,7 +3266,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3336,7 +3310,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3462,7 +3436,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3506,7 +3480,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3591,7 +3565,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3638,7 +3612,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3685,7 +3659,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3729,7 +3703,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3773,7 +3747,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3858,7 +3832,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3943,7 +3917,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3990,7 +3964,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4034,7 +4008,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4078,7 +4052,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4163,7 +4137,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4207,7 +4181,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4251,7 +4225,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4336,7 +4310,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4380,7 +4354,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4424,7 +4398,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4468,7 +4442,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4635,7 +4609,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4679,7 +4653,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4723,7 +4697,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4767,7 +4741,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4814,7 +4788,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4858,7 +4832,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4940,7 +4914,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4984,7 +4958,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5072,7 +5046,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5116,7 +5090,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5163,7 +5137,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5207,7 +5181,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -5251,7 +5225,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5295,7 +5269,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5339,7 +5313,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5386,7 +5360,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5430,7 +5404,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5477,7 +5451,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5521,7 +5495,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5568,7 +5542,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5656,7 +5630,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5700,7 +5674,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5744,7 +5718,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5788,7 +5762,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5832,7 +5806,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5876,7 +5850,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5961,7 +5935,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6005,7 +5979,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -6049,7 +6023,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -6093,7 +6067,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -6137,7 +6111,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -6181,7 +6155,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6225,7 +6199,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6269,7 +6243,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6316,7 +6290,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6360,7 +6334,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6404,7 +6378,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6448,7 +6422,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6492,7 +6466,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6536,7 +6510,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6580,7 +6554,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6624,7 +6598,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6668,7 +6642,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6756,7 +6730,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6800,7 +6774,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6926,7 +6900,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6970,7 +6944,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7014,7 +6988,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7058,7 +7032,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7140,7 +7114,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7184,7 +7158,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7231,7 +7205,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7275,7 +7249,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7401,7 +7375,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7445,7 +7419,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7530,7 +7504,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7574,7 +7548,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7618,7 +7592,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7662,7 +7636,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7706,7 +7680,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7750,7 +7724,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7794,7 +7768,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7838,7 +7812,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7923,7 +7897,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8090,7 +8064,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8134,7 +8108,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8178,7 +8152,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8222,7 +8196,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8266,7 +8240,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8310,7 +8284,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8354,7 +8328,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8439,7 +8413,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8483,7 +8457,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8568,7 +8542,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8694,7 +8668,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8738,7 +8712,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8823,7 +8797,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8867,7 +8841,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8911,7 +8885,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8955,7 +8929,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8999,7 +8973,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -9043,7 +9017,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9087,7 +9061,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9131,7 +9105,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9216,7 +9190,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9383,7 +9357,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9427,7 +9401,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9471,7 +9445,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9515,7 +9489,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9600,7 +9574,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9644,7 +9618,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9688,7 +9662,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9732,7 +9706,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9776,7 +9750,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9820,7 +9794,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9864,7 +9838,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9908,7 +9882,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9952,7 +9926,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9996,7 +9970,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10040,7 +10014,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -10084,7 +10058,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10128,7 +10102,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10172,7 +10146,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -10216,7 +10190,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10260,7 +10234,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10304,7 +10278,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10348,7 +10322,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10392,7 +10366,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10436,7 +10410,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10480,7 +10454,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10565,7 +10539,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10650,7 +10624,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10665,55 +10639,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11082,7 +11056,7 @@
       <c r="L10" t="s">
         <v>721</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46377</v>
       </c>
       <c r="N10" t="s">
@@ -11126,7 +11100,7 @@
       <c r="L11" t="s">
         <v>721</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46377</v>
       </c>
       <c r="N11" t="s">
@@ -11334,7 +11308,7 @@
       <c r="L16" t="s">
         <v>721</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46377</v>
       </c>
       <c r="N16" t="s">
@@ -11460,7 +11434,7 @@
       <c r="L19" t="s">
         <v>721</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46377</v>
       </c>
       <c r="N19" t="s">
@@ -11504,7 +11478,7 @@
       <c r="L20" t="s">
         <v>721</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46377</v>
       </c>
       <c r="N20" t="s">
@@ -11548,7 +11522,7 @@
       <c r="L21" t="s">
         <v>721</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46377</v>
       </c>
       <c r="N21" t="s">
@@ -11715,7 +11689,7 @@
       <c r="L25" t="s">
         <v>721</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46377</v>
       </c>
       <c r="N25" t="s">
@@ -11841,7 +11815,7 @@
       <c r="L28" t="s">
         <v>721</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46377</v>
       </c>
       <c r="N28" t="s">
@@ -11885,7 +11859,7 @@
       <c r="L29" t="s">
         <v>719</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46312</v>
       </c>
       <c r="N29" t="s">
@@ -11929,7 +11903,7 @@
       <c r="L30" t="s">
         <v>721</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46377</v>
       </c>
       <c r="N30" t="s">
@@ -11973,7 +11947,7 @@
       <c r="L31" t="s">
         <v>719</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46312</v>
       </c>
       <c r="N31" t="s">
@@ -12386,7 +12360,7 @@
       <c r="L41" t="s">
         <v>721</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46377</v>
       </c>
       <c r="N41" t="s">
@@ -12471,7 +12445,7 @@
       <c r="L43" t="s">
         <v>721</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46377</v>
       </c>
       <c r="N43" t="s">
@@ -12515,7 +12489,7 @@
       <c r="L44" t="s">
         <v>721</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46377</v>
       </c>
       <c r="N44" t="s">
@@ -12559,7 +12533,7 @@
       <c r="L45" t="s">
         <v>721</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46377</v>
       </c>
       <c r="N45" t="s">
@@ -12685,7 +12659,7 @@
       <c r="L48" t="s">
         <v>721</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46377</v>
       </c>
       <c r="N48" t="s">
@@ -12729,7 +12703,7 @@
       <c r="L49" t="s">
         <v>719</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46312</v>
       </c>
       <c r="N49" t="s">
@@ -12773,7 +12747,7 @@
       <c r="L50" t="s">
         <v>719</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46312</v>
       </c>
       <c r="N50" t="s">
@@ -12817,7 +12791,7 @@
       <c r="L51" t="s">
         <v>721</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46377</v>
       </c>
       <c r="N51" t="s">
@@ -12861,7 +12835,7 @@
       <c r="L52" t="s">
         <v>721</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46377</v>
       </c>
       <c r="N52" t="s">
@@ -12905,7 +12879,7 @@
       <c r="L53" t="s">
         <v>721</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46377</v>
       </c>
       <c r="N53" t="s">
@@ -12949,7 +12923,7 @@
       <c r="L54" t="s">
         <v>721</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46377</v>
       </c>
       <c r="N54" t="s">
@@ -12993,7 +12967,7 @@
       <c r="L55" t="s">
         <v>720</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46392</v>
       </c>
       <c r="N55" t="s">
@@ -13037,7 +13011,7 @@
       <c r="L56" t="s">
         <v>719</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46312</v>
       </c>
       <c r="N56" t="s">
@@ -13081,7 +13055,7 @@
       <c r="L57" t="s">
         <v>719</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46312</v>
       </c>
       <c r="N57" t="s">
@@ -13125,7 +13099,7 @@
       <c r="L58" t="s">
         <v>719</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46312</v>
       </c>
       <c r="N58" t="s">
@@ -13169,7 +13143,7 @@
       <c r="L59" t="s">
         <v>721</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46377</v>
       </c>
       <c r="N59" t="s">
@@ -13213,7 +13187,7 @@
       <c r="L60" t="s">
         <v>719</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46312</v>
       </c>
       <c r="N60" t="s">
@@ -13257,7 +13231,7 @@
       <c r="L61" t="s">
         <v>719</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46312</v>
       </c>
       <c r="N61" t="s">
@@ -13301,7 +13275,7 @@
       <c r="L62" t="s">
         <v>721</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46377</v>
       </c>
       <c r="N62" t="s">
@@ -13345,7 +13319,7 @@
       <c r="L63" t="s">
         <v>721</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46377</v>
       </c>
       <c r="N63" t="s">
@@ -13389,7 +13363,7 @@
       <c r="L64" t="s">
         <v>721</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46377</v>
       </c>
       <c r="N64" t="s">
@@ -13433,7 +13407,7 @@
       <c r="L65" t="s">
         <v>721</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="1">
         <v>46377</v>
       </c>
       <c r="N65" t="s">
@@ -13477,7 +13451,7 @@
       <c r="L66" t="s">
         <v>721</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="1">
         <v>46377</v>
       </c>
       <c r="N66" t="s">
@@ -13521,7 +13495,7 @@
       <c r="L67" t="s">
         <v>721</v>
       </c>
-      <c r="M67" s="2">
+      <c r="M67" s="1">
         <v>46377</v>
       </c>
       <c r="N67" t="s">
@@ -13565,7 +13539,7 @@
       <c r="L68" t="s">
         <v>721</v>
       </c>
-      <c r="M68" s="2">
+      <c r="M68" s="1">
         <v>46377</v>
       </c>
       <c r="N68" t="s">
@@ -13609,7 +13583,7 @@
       <c r="L69" t="s">
         <v>721</v>
       </c>
-      <c r="M69" s="2">
+      <c r="M69" s="1">
         <v>46377</v>
       </c>
       <c r="N69" t="s">
@@ -13653,7 +13627,7 @@
       <c r="L70" t="s">
         <v>721</v>
       </c>
-      <c r="M70" s="2">
+      <c r="M70" s="1">
         <v>46377</v>
       </c>
       <c r="N70" t="s">
@@ -13697,7 +13671,7 @@
       <c r="L71" t="s">
         <v>721</v>
       </c>
-      <c r="M71" s="2">
+      <c r="M71" s="1">
         <v>46377</v>
       </c>
       <c r="N71" t="s">
@@ -13741,7 +13715,7 @@
       <c r="L72" t="s">
         <v>721</v>
       </c>
-      <c r="M72" s="2">
+      <c r="M72" s="1">
         <v>46377</v>
       </c>
       <c r="N72" t="s">
@@ -13785,7 +13759,7 @@
       <c r="L73" t="s">
         <v>721</v>
       </c>
-      <c r="M73" s="2">
+      <c r="M73" s="1">
         <v>46377</v>
       </c>
       <c r="N73" t="s">
@@ -13829,7 +13803,7 @@
       <c r="L74" t="s">
         <v>721</v>
       </c>
-      <c r="M74" s="2">
+      <c r="M74" s="1">
         <v>46377</v>
       </c>
       <c r="N74" t="s">
@@ -13873,7 +13847,7 @@
       <c r="L75" t="s">
         <v>720</v>
       </c>
-      <c r="M75" s="2">
+      <c r="M75" s="1">
         <v>46392</v>
       </c>
       <c r="N75" t="s">
@@ -13917,7 +13891,7 @@
       <c r="L76" t="s">
         <v>720</v>
       </c>
-      <c r="M76" s="2">
+      <c r="M76" s="1">
         <v>46392</v>
       </c>
       <c r="N76" t="s">
@@ -13961,7 +13935,7 @@
       <c r="L77" t="s">
         <v>721</v>
       </c>
-      <c r="M77" s="2">
+      <c r="M77" s="1">
         <v>46377</v>
       </c>
       <c r="N77" t="s">
@@ -14005,7 +13979,7 @@
       <c r="L78" t="s">
         <v>721</v>
       </c>
-      <c r="M78" s="2">
+      <c r="M78" s="1">
         <v>46377</v>
       </c>
       <c r="N78" t="s">
@@ -14049,7 +14023,7 @@
       <c r="L79" t="s">
         <v>721</v>
       </c>
-      <c r="M79" s="2">
+      <c r="M79" s="1">
         <v>46377</v>
       </c>
       <c r="N79" t="s">
@@ -14093,7 +14067,7 @@
       <c r="L80" t="s">
         <v>721</v>
       </c>
-      <c r="M80" s="2">
+      <c r="M80" s="1">
         <v>46377</v>
       </c>
       <c r="N80" t="s">
@@ -14137,7 +14111,7 @@
       <c r="L81" t="s">
         <v>720</v>
       </c>
-      <c r="M81" s="2">
+      <c r="M81" s="1">
         <v>46392</v>
       </c>
       <c r="N81" t="s">
@@ -14181,7 +14155,7 @@
       <c r="L82" t="s">
         <v>721</v>
       </c>
-      <c r="M82" s="2">
+      <c r="M82" s="1">
         <v>46377</v>
       </c>
       <c r="N82" t="s">
@@ -14225,7 +14199,7 @@
       <c r="L83" t="s">
         <v>721</v>
       </c>
-      <c r="M83" s="2">
+      <c r="M83" s="1">
         <v>46377</v>
       </c>
       <c r="N83" t="s">
@@ -14269,7 +14243,7 @@
       <c r="L84" t="s">
         <v>721</v>
       </c>
-      <c r="M84" s="2">
+      <c r="M84" s="1">
         <v>46377</v>
       </c>
       <c r="N84" t="s">
@@ -14313,7 +14287,7 @@
       <c r="L85" t="s">
         <v>721</v>
       </c>
-      <c r="M85" s="2">
+      <c r="M85" s="1">
         <v>46377</v>
       </c>
       <c r="N85" t="s">
@@ -14357,7 +14331,7 @@
       <c r="L86" t="s">
         <v>721</v>
       </c>
-      <c r="M86" s="2">
+      <c r="M86" s="1">
         <v>46377</v>
       </c>
       <c r="N86" t="s">
@@ -14401,7 +14375,7 @@
       <c r="L87" t="s">
         <v>721</v>
       </c>
-      <c r="M87" s="2">
+      <c r="M87" s="1">
         <v>46377</v>
       </c>
       <c r="N87" t="s">
@@ -14445,7 +14419,7 @@
       <c r="L88" t="s">
         <v>720</v>
       </c>
-      <c r="M88" s="2">
+      <c r="M88" s="1">
         <v>46392</v>
       </c>
       <c r="N88" t="s">
@@ -14489,7 +14463,7 @@
       <c r="L89" t="s">
         <v>721</v>
       </c>
-      <c r="M89" s="2">
+      <c r="M89" s="1">
         <v>46377</v>
       </c>
       <c r="N89" t="s">
@@ -14533,7 +14507,7 @@
       <c r="L90" t="s">
         <v>720</v>
       </c>
-      <c r="M90" s="2">
+      <c r="M90" s="1">
         <v>46392</v>
       </c>
       <c r="N90" t="s">
@@ -14577,7 +14551,7 @@
       <c r="L91" t="s">
         <v>720</v>
       </c>
-      <c r="M91" s="2">
+      <c r="M91" s="1">
         <v>46392</v>
       </c>
       <c r="N91" t="s">
@@ -14621,7 +14595,7 @@
       <c r="L92" t="s">
         <v>721</v>
       </c>
-      <c r="M92" s="2">
+      <c r="M92" s="1">
         <v>46377</v>
       </c>
       <c r="N92" t="s">
@@ -14665,7 +14639,7 @@
       <c r="L93" t="s">
         <v>720</v>
       </c>
-      <c r="M93" s="2">
+      <c r="M93" s="1">
         <v>46392</v>
       </c>
       <c r="N93" t="s">
@@ -14709,7 +14683,7 @@
       <c r="L94" t="s">
         <v>720</v>
       </c>
-      <c r="M94" s="2">
+      <c r="M94" s="1">
         <v>46392</v>
       </c>
       <c r="N94" t="s">
@@ -14753,7 +14727,7 @@
       <c r="L95" t="s">
         <v>720</v>
       </c>
-      <c r="M95" s="2">
+      <c r="M95" s="1">
         <v>46392</v>
       </c>
       <c r="N95" t="s">
@@ -14797,7 +14771,7 @@
       <c r="L96" t="s">
         <v>720</v>
       </c>
-      <c r="M96" s="2">
+      <c r="M96" s="1">
         <v>46392</v>
       </c>
       <c r="N96" t="s">
@@ -14841,7 +14815,7 @@
       <c r="L97" t="s">
         <v>721</v>
       </c>
-      <c r="M97" s="2">
+      <c r="M97" s="1">
         <v>46377</v>
       </c>
       <c r="N97" t="s">
@@ -14885,7 +14859,7 @@
       <c r="L98" t="s">
         <v>721</v>
       </c>
-      <c r="M98" s="2">
+      <c r="M98" s="1">
         <v>46377</v>
       </c>
       <c r="N98" t="s">
@@ -14929,7 +14903,7 @@
       <c r="L99" t="s">
         <v>721</v>
       </c>
-      <c r="M99" s="2">
+      <c r="M99" s="1">
         <v>46377</v>
       </c>
       <c r="N99" t="s">
@@ -14973,7 +14947,7 @@
       <c r="L100" t="s">
         <v>721</v>
       </c>
-      <c r="M100" s="2">
+      <c r="M100" s="1">
         <v>46377</v>
       </c>
       <c r="N100" t="s">
@@ -15017,7 +14991,7 @@
       <c r="L101" t="s">
         <v>721</v>
       </c>
-      <c r="M101" s="2">
+      <c r="M101" s="1">
         <v>46377</v>
       </c>
       <c r="N101" t="s">
@@ -15061,7 +15035,7 @@
       <c r="L102" t="s">
         <v>721</v>
       </c>
-      <c r="M102" s="2">
+      <c r="M102" s="1">
         <v>46377</v>
       </c>
       <c r="N102" t="s">
@@ -15105,7 +15079,7 @@
       <c r="L103" t="s">
         <v>721</v>
       </c>
-      <c r="M103" s="2">
+      <c r="M103" s="1">
         <v>46377</v>
       </c>
       <c r="N103" t="s">
@@ -15149,7 +15123,7 @@
       <c r="L104" t="s">
         <v>721</v>
       </c>
-      <c r="M104" s="2">
+      <c r="M104" s="1">
         <v>46377</v>
       </c>
       <c r="N104" t="s">
@@ -15193,7 +15167,7 @@
       <c r="L105" t="s">
         <v>721</v>
       </c>
-      <c r="M105" s="2">
+      <c r="M105" s="1">
         <v>46377</v>
       </c>
       <c r="N105" t="s">
@@ -15237,7 +15211,7 @@
       <c r="L106" t="s">
         <v>720</v>
       </c>
-      <c r="M106" s="2">
+      <c r="M106" s="1">
         <v>46392</v>
       </c>
       <c r="N106" t="s">
@@ -15281,7 +15255,7 @@
       <c r="L107" t="s">
         <v>721</v>
       </c>
-      <c r="M107" s="2">
+      <c r="M107" s="1">
         <v>46377</v>
       </c>
       <c r="N107" t="s">
@@ -15325,7 +15299,7 @@
       <c r="L108" t="s">
         <v>721</v>
       </c>
-      <c r="M108" s="2">
+      <c r="M108" s="1">
         <v>46377</v>
       </c>
       <c r="N108" t="s">
@@ -15369,7 +15343,7 @@
       <c r="L109" t="s">
         <v>721</v>
       </c>
-      <c r="M109" s="2">
+      <c r="M109" s="1">
         <v>46377</v>
       </c>
       <c r="N109" t="s">
@@ -15413,7 +15387,7 @@
       <c r="L110" t="s">
         <v>721</v>
       </c>
-      <c r="M110" s="2">
+      <c r="M110" s="1">
         <v>46377</v>
       </c>
       <c r="N110" t="s">
@@ -15457,7 +15431,7 @@
       <c r="L111" t="s">
         <v>721</v>
       </c>
-      <c r="M111" s="2">
+      <c r="M111" s="1">
         <v>46377</v>
       </c>
       <c r="N111" t="s">
@@ -15501,7 +15475,7 @@
       <c r="L112" t="s">
         <v>721</v>
       </c>
-      <c r="M112" s="2">
+      <c r="M112" s="1">
         <v>46377</v>
       </c>
       <c r="N112" t="s">
@@ -15545,7 +15519,7 @@
       <c r="L113" t="s">
         <v>721</v>
       </c>
-      <c r="M113" s="2">
+      <c r="M113" s="1">
         <v>46377</v>
       </c>
       <c r="N113" t="s">
@@ -15589,7 +15563,7 @@
       <c r="L114" t="s">
         <v>721</v>
       </c>
-      <c r="M114" s="2">
+      <c r="M114" s="1">
         <v>46377</v>
       </c>
       <c r="N114" t="s">
@@ -15633,7 +15607,7 @@
       <c r="L115" t="s">
         <v>721</v>
       </c>
-      <c r="M115" s="2">
+      <c r="M115" s="1">
         <v>46377</v>
       </c>
       <c r="N115" t="s">
@@ -15677,7 +15651,7 @@
       <c r="L116" t="s">
         <v>721</v>
       </c>
-      <c r="M116" s="2">
+      <c r="M116" s="1">
         <v>46377</v>
       </c>
       <c r="N116" t="s">
@@ -15721,7 +15695,7 @@
       <c r="L117" t="s">
         <v>721</v>
       </c>
-      <c r="M117" s="2">
+      <c r="M117" s="1">
         <v>46377</v>
       </c>
       <c r="N117" t="s">
@@ -15765,7 +15739,7 @@
       <c r="L118" t="s">
         <v>721</v>
       </c>
-      <c r="M118" s="2">
+      <c r="M118" s="1">
         <v>46377</v>
       </c>
       <c r="N118" t="s">
@@ -15809,7 +15783,7 @@
       <c r="L119" t="s">
         <v>721</v>
       </c>
-      <c r="M119" s="2">
+      <c r="M119" s="1">
         <v>46377</v>
       </c>
       <c r="N119" t="s">
@@ -15853,7 +15827,7 @@
       <c r="L120" t="s">
         <v>721</v>
       </c>
-      <c r="M120" s="2">
+      <c r="M120" s="1">
         <v>46377</v>
       </c>
       <c r="N120" t="s">
@@ -15897,7 +15871,7 @@
       <c r="L121" t="s">
         <v>720</v>
       </c>
-      <c r="M121" s="2">
+      <c r="M121" s="1">
         <v>46392</v>
       </c>
       <c r="N121" t="s">
@@ -15941,7 +15915,7 @@
       <c r="L122" t="s">
         <v>721</v>
       </c>
-      <c r="M122" s="2">
+      <c r="M122" s="1">
         <v>46377</v>
       </c>
       <c r="N122" t="s">
@@ -15985,7 +15959,7 @@
       <c r="L123" t="s">
         <v>721</v>
       </c>
-      <c r="M123" s="2">
+      <c r="M123" s="1">
         <v>46377</v>
       </c>
       <c r="N123" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (08/10/2026 14:51)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -11057,7 +11057,7 @@
         <v>721</v>
       </c>
       <c r="M10" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N10" t="s">
         <v>722</v>
@@ -11101,7 +11101,7 @@
         <v>721</v>
       </c>
       <c r="M11" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N11" t="s">
         <v>722</v>
@@ -11309,7 +11309,7 @@
         <v>721</v>
       </c>
       <c r="M16" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N16" t="s">
         <v>722</v>
@@ -11435,7 +11435,7 @@
         <v>721</v>
       </c>
       <c r="M19" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N19" t="s">
         <v>722</v>
@@ -11479,7 +11479,7 @@
         <v>721</v>
       </c>
       <c r="M20" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N20" t="s">
         <v>722</v>
@@ -11523,7 +11523,7 @@
         <v>721</v>
       </c>
       <c r="M21" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N21" t="s">
         <v>722</v>
@@ -11690,7 +11690,7 @@
         <v>721</v>
       </c>
       <c r="M25" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N25" t="s">
         <v>722</v>
@@ -11816,7 +11816,7 @@
         <v>721</v>
       </c>
       <c r="M28" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N28" t="s">
         <v>722</v>
@@ -11860,7 +11860,7 @@
         <v>719</v>
       </c>
       <c r="M29" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N29" t="s">
         <v>722</v>
@@ -11904,7 +11904,7 @@
         <v>721</v>
       </c>
       <c r="M30" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N30" t="s">
         <v>722</v>
@@ -11948,7 +11948,7 @@
         <v>719</v>
       </c>
       <c r="M31" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N31" t="s">
         <v>722</v>
@@ -12361,7 +12361,7 @@
         <v>721</v>
       </c>
       <c r="M41" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N41" t="s">
         <v>722</v>
@@ -12446,7 +12446,7 @@
         <v>721</v>
       </c>
       <c r="M43" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N43" t="s">
         <v>722</v>
@@ -12490,7 +12490,7 @@
         <v>721</v>
       </c>
       <c r="M44" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N44" t="s">
         <v>722</v>
@@ -12534,7 +12534,7 @@
         <v>721</v>
       </c>
       <c r="M45" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N45" t="s">
         <v>722</v>
@@ -12660,7 +12660,7 @@
         <v>721</v>
       </c>
       <c r="M48" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N48" t="s">
         <v>722</v>
@@ -12704,7 +12704,7 @@
         <v>719</v>
       </c>
       <c r="M49" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N49" t="s">
         <v>722</v>
@@ -12748,7 +12748,7 @@
         <v>719</v>
       </c>
       <c r="M50" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N50" t="s">
         <v>722</v>
@@ -12792,7 +12792,7 @@
         <v>721</v>
       </c>
       <c r="M51" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N51" t="s">
         <v>722</v>
@@ -12836,7 +12836,7 @@
         <v>721</v>
       </c>
       <c r="M52" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N52" t="s">
         <v>722</v>
@@ -12880,7 +12880,7 @@
         <v>721</v>
       </c>
       <c r="M53" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N53" t="s">
         <v>722</v>
@@ -12924,7 +12924,7 @@
         <v>721</v>
       </c>
       <c r="M54" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N54" t="s">
         <v>722</v>
@@ -12968,7 +12968,7 @@
         <v>720</v>
       </c>
       <c r="M55" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N55" t="s">
         <v>722</v>
@@ -13012,7 +13012,7 @@
         <v>719</v>
       </c>
       <c r="M56" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N56" t="s">
         <v>722</v>
@@ -13056,7 +13056,7 @@
         <v>719</v>
       </c>
       <c r="M57" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N57" t="s">
         <v>722</v>
@@ -13100,7 +13100,7 @@
         <v>719</v>
       </c>
       <c r="M58" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N58" t="s">
         <v>722</v>
@@ -13144,7 +13144,7 @@
         <v>721</v>
       </c>
       <c r="M59" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N59" t="s">
         <v>722</v>
@@ -13188,7 +13188,7 @@
         <v>719</v>
       </c>
       <c r="M60" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N60" t="s">
         <v>722</v>
@@ -13232,7 +13232,7 @@
         <v>719</v>
       </c>
       <c r="M61" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N61" t="s">
         <v>722</v>
@@ -13276,7 +13276,7 @@
         <v>721</v>
       </c>
       <c r="M62" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N62" t="s">
         <v>722</v>
@@ -13320,7 +13320,7 @@
         <v>721</v>
       </c>
       <c r="M63" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N63" t="s">
         <v>722</v>
@@ -13364,7 +13364,7 @@
         <v>721</v>
       </c>
       <c r="M64" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N64" t="s">
         <v>722</v>
@@ -13408,7 +13408,7 @@
         <v>721</v>
       </c>
       <c r="M65" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N65" t="s">
         <v>722</v>
@@ -13452,7 +13452,7 @@
         <v>721</v>
       </c>
       <c r="M66" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N66" t="s">
         <v>722</v>
@@ -13496,7 +13496,7 @@
         <v>721</v>
       </c>
       <c r="M67" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N67" t="s">
         <v>722</v>
@@ -13540,7 +13540,7 @@
         <v>721</v>
       </c>
       <c r="M68" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N68" t="s">
         <v>722</v>
@@ -13584,7 +13584,7 @@
         <v>721</v>
       </c>
       <c r="M69" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N69" t="s">
         <v>722</v>
@@ -13628,7 +13628,7 @@
         <v>721</v>
       </c>
       <c r="M70" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N70" t="s">
         <v>722</v>
@@ -13672,7 +13672,7 @@
         <v>721</v>
       </c>
       <c r="M71" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N71" t="s">
         <v>722</v>
@@ -13716,7 +13716,7 @@
         <v>721</v>
       </c>
       <c r="M72" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N72" t="s">
         <v>722</v>
@@ -13760,7 +13760,7 @@
         <v>721</v>
       </c>
       <c r="M73" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N73" t="s">
         <v>722</v>
@@ -13804,7 +13804,7 @@
         <v>721</v>
       </c>
       <c r="M74" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N74" t="s">
         <v>722</v>
@@ -13848,7 +13848,7 @@
         <v>720</v>
       </c>
       <c r="M75" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N75" t="s">
         <v>722</v>
@@ -13892,7 +13892,7 @@
         <v>720</v>
       </c>
       <c r="M76" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N76" t="s">
         <v>722</v>
@@ -13936,7 +13936,7 @@
         <v>721</v>
       </c>
       <c r="M77" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N77" t="s">
         <v>722</v>
@@ -13980,7 +13980,7 @@
         <v>721</v>
       </c>
       <c r="M78" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N78" t="s">
         <v>722</v>
@@ -14024,7 +14024,7 @@
         <v>721</v>
       </c>
       <c r="M79" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N79" t="s">
         <v>722</v>
@@ -14068,7 +14068,7 @@
         <v>721</v>
       </c>
       <c r="M80" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N80" t="s">
         <v>722</v>
@@ -14112,7 +14112,7 @@
         <v>720</v>
       </c>
       <c r="M81" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N81" t="s">
         <v>722</v>
@@ -14156,7 +14156,7 @@
         <v>721</v>
       </c>
       <c r="M82" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N82" t="s">
         <v>722</v>
@@ -14200,7 +14200,7 @@
         <v>721</v>
       </c>
       <c r="M83" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N83" t="s">
         <v>722</v>
@@ -14244,7 +14244,7 @@
         <v>721</v>
       </c>
       <c r="M84" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N84" t="s">
         <v>722</v>
@@ -14288,7 +14288,7 @@
         <v>721</v>
       </c>
       <c r="M85" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N85" t="s">
         <v>722</v>
@@ -14332,7 +14332,7 @@
         <v>721</v>
       </c>
       <c r="M86" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N86" t="s">
         <v>722</v>
@@ -14376,7 +14376,7 @@
         <v>721</v>
       </c>
       <c r="M87" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N87" t="s">
         <v>722</v>
@@ -14420,7 +14420,7 @@
         <v>720</v>
       </c>
       <c r="M88" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N88" t="s">
         <v>722</v>
@@ -14464,7 +14464,7 @@
         <v>721</v>
       </c>
       <c r="M89" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N89" t="s">
         <v>722</v>
@@ -14508,7 +14508,7 @@
         <v>720</v>
       </c>
       <c r="M90" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N90" t="s">
         <v>722</v>
@@ -14552,7 +14552,7 @@
         <v>720</v>
       </c>
       <c r="M91" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N91" t="s">
         <v>722</v>
@@ -14596,7 +14596,7 @@
         <v>721</v>
       </c>
       <c r="M92" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N92" t="s">
         <v>722</v>
@@ -14640,7 +14640,7 @@
         <v>720</v>
       </c>
       <c r="M93" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N93" t="s">
         <v>722</v>
@@ -14684,7 +14684,7 @@
         <v>720</v>
       </c>
       <c r="M94" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N94" t="s">
         <v>722</v>
@@ -14728,7 +14728,7 @@
         <v>720</v>
       </c>
       <c r="M95" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N95" t="s">
         <v>722</v>
@@ -14772,7 +14772,7 @@
         <v>720</v>
       </c>
       <c r="M96" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N96" t="s">
         <v>722</v>
@@ -14816,7 +14816,7 @@
         <v>721</v>
       </c>
       <c r="M97" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N97" t="s">
         <v>722</v>
@@ -14860,7 +14860,7 @@
         <v>721</v>
       </c>
       <c r="M98" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N98" t="s">
         <v>722</v>
@@ -14904,7 +14904,7 @@
         <v>721</v>
       </c>
       <c r="M99" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N99" t="s">
         <v>722</v>
@@ -14948,7 +14948,7 @@
         <v>721</v>
       </c>
       <c r="M100" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N100" t="s">
         <v>722</v>
@@ -14992,7 +14992,7 @@
         <v>721</v>
       </c>
       <c r="M101" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N101" t="s">
         <v>722</v>
@@ -15036,7 +15036,7 @@
         <v>721</v>
       </c>
       <c r="M102" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N102" t="s">
         <v>722</v>
@@ -15080,7 +15080,7 @@
         <v>721</v>
       </c>
       <c r="M103" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N103" t="s">
         <v>722</v>
@@ -15124,7 +15124,7 @@
         <v>721</v>
       </c>
       <c r="M104" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N104" t="s">
         <v>722</v>
@@ -15168,7 +15168,7 @@
         <v>721</v>
       </c>
       <c r="M105" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N105" t="s">
         <v>722</v>
@@ -15212,7 +15212,7 @@
         <v>720</v>
       </c>
       <c r="M106" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N106" t="s">
         <v>722</v>
@@ -15256,7 +15256,7 @@
         <v>721</v>
       </c>
       <c r="M107" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N107" t="s">
         <v>722</v>
@@ -15300,7 +15300,7 @@
         <v>721</v>
       </c>
       <c r="M108" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N108" t="s">
         <v>722</v>
@@ -15344,7 +15344,7 @@
         <v>721</v>
       </c>
       <c r="M109" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N109" t="s">
         <v>722</v>
@@ -15388,7 +15388,7 @@
         <v>721</v>
       </c>
       <c r="M110" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N110" t="s">
         <v>722</v>
@@ -15432,7 +15432,7 @@
         <v>721</v>
       </c>
       <c r="M111" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N111" t="s">
         <v>722</v>
@@ -15476,7 +15476,7 @@
         <v>721</v>
       </c>
       <c r="M112" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N112" t="s">
         <v>722</v>
@@ -15520,7 +15520,7 @@
         <v>721</v>
       </c>
       <c r="M113" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N113" t="s">
         <v>722</v>
@@ -15564,7 +15564,7 @@
         <v>721</v>
       </c>
       <c r="M114" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N114" t="s">
         <v>722</v>
@@ -15608,7 +15608,7 @@
         <v>721</v>
       </c>
       <c r="M115" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N115" t="s">
         <v>722</v>
@@ -15652,7 +15652,7 @@
         <v>721</v>
       </c>
       <c r="M116" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N116" t="s">
         <v>722</v>
@@ -15696,7 +15696,7 @@
         <v>721</v>
       </c>
       <c r="M117" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N117" t="s">
         <v>722</v>
@@ -15740,7 +15740,7 @@
         <v>721</v>
       </c>
       <c r="M118" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N118" t="s">
         <v>722</v>
@@ -15784,7 +15784,7 @@
         <v>721</v>
       </c>
       <c r="M119" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N119" t="s">
         <v>722</v>
@@ -15828,7 +15828,7 @@
         <v>721</v>
       </c>
       <c r="M120" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N120" t="s">
         <v>722</v>
@@ -15872,7 +15872,7 @@
         <v>720</v>
       </c>
       <c r="M121" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N121" t="s">
         <v>722</v>
@@ -15916,7 +15916,7 @@
         <v>721</v>
       </c>
       <c r="M122" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N122" t="s">
         <v>722</v>
@@ -15960,7 +15960,7 @@
         <v>721</v>
       </c>
       <c r="M123" s="1">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="N123" t="s">
         <v>722</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (09/10/2026 14:26)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3116" uniqueCount="723">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3116" uniqueCount="724">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -2181,6 +2181,9 @@
   </si>
   <si>
     <t>Validada</t>
+  </si>
+  <si>
+    <t>Em Discrepância</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10720,13 +10723,13 @@
         <v>717</v>
       </c>
       <c r="J2" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K2" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="L2" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="N2" t="s">
         <v>395</v>
@@ -10761,13 +10764,13 @@
         <v>717</v>
       </c>
       <c r="J3" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K3" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="L3" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="N3" t="s">
         <v>395</v>
@@ -10802,13 +10805,13 @@
         <v>717</v>
       </c>
       <c r="J4" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K4" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="L4" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="N4" t="s">
         <v>395</v>
@@ -10884,13 +10887,13 @@
         <v>717</v>
       </c>
       <c r="J6" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K6" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="L6" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="N6" t="s">
         <v>395</v>
@@ -10925,13 +10928,13 @@
         <v>717</v>
       </c>
       <c r="J7" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K7" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="L7" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="N7" t="s">
         <v>395</v>
@@ -11007,13 +11010,13 @@
         <v>717</v>
       </c>
       <c r="J9" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K9" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="L9" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="N9" t="s">
         <v>395</v>
@@ -11057,10 +11060,10 @@
         <v>721</v>
       </c>
       <c r="M10" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N10" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -11101,10 +11104,10 @@
         <v>721</v>
       </c>
       <c r="M11" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N11" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -11309,10 +11312,10 @@
         <v>721</v>
       </c>
       <c r="M16" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N16" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -11435,10 +11438,10 @@
         <v>721</v>
       </c>
       <c r="M19" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N19" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11479,10 +11482,10 @@
         <v>721</v>
       </c>
       <c r="M20" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N20" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11514,19 +11517,19 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K21" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L21" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M21" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N21" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11558,13 +11561,13 @@
         <v>717</v>
       </c>
       <c r="J22" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K22" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="L22" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="N22" t="s">
         <v>395</v>
@@ -11599,13 +11602,13 @@
         <v>717</v>
       </c>
       <c r="J23" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K23" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="L23" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="N23" t="s">
         <v>395</v>
@@ -11640,13 +11643,13 @@
         <v>717</v>
       </c>
       <c r="J24" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K24" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="L24" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="N24" t="s">
         <v>395</v>
@@ -11690,10 +11693,10 @@
         <v>721</v>
       </c>
       <c r="M25" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N25" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11725,13 +11728,13 @@
         <v>717</v>
       </c>
       <c r="J26" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K26" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="L26" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="N26" t="s">
         <v>395</v>
@@ -11816,10 +11819,10 @@
         <v>721</v>
       </c>
       <c r="M28" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N28" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11860,10 +11863,10 @@
         <v>719</v>
       </c>
       <c r="M29" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N29" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11895,19 +11898,19 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K30" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L30" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M30" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N30" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11948,10 +11951,10 @@
         <v>719</v>
       </c>
       <c r="M31" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N31" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -12352,19 +12355,19 @@
         <v>382</v>
       </c>
       <c r="J41" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K41" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L41" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M41" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N41" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -12446,10 +12449,10 @@
         <v>721</v>
       </c>
       <c r="M43" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N43" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12490,10 +12493,10 @@
         <v>721</v>
       </c>
       <c r="M44" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N44" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12534,10 +12537,10 @@
         <v>721</v>
       </c>
       <c r="M45" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N45" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12660,10 +12663,10 @@
         <v>721</v>
       </c>
       <c r="M48" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N48" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12704,10 +12707,10 @@
         <v>719</v>
       </c>
       <c r="M49" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N49" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12748,10 +12751,10 @@
         <v>719</v>
       </c>
       <c r="M50" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N50" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12783,19 +12786,19 @@
         <v>382</v>
       </c>
       <c r="J51" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K51" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L51" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M51" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N51" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12827,19 +12830,19 @@
         <v>382</v>
       </c>
       <c r="J52" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K52" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L52" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M52" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N52" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12871,19 +12874,19 @@
         <v>382</v>
       </c>
       <c r="J53" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K53" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L53" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M53" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N53" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12924,10 +12927,10 @@
         <v>721</v>
       </c>
       <c r="M54" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N54" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12959,19 +12962,19 @@
         <v>720</v>
       </c>
       <c r="J55" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="K55" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="L55" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="M55" s="1">
-        <v>46393</v>
+        <v>46379</v>
       </c>
       <c r="N55" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -13012,10 +13015,10 @@
         <v>719</v>
       </c>
       <c r="M56" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N56" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -13047,19 +13050,16 @@
         <v>719</v>
       </c>
       <c r="J57" t="s">
-        <v>719</v>
+        <v>391</v>
       </c>
       <c r="K57" t="s">
-        <v>719</v>
+        <v>391</v>
       </c>
       <c r="L57" t="s">
-        <v>719</v>
-      </c>
-      <c r="M57" s="1">
-        <v>46313</v>
+        <v>391</v>
       </c>
       <c r="N57" t="s">
-        <v>722</v>
+        <v>395</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -13091,19 +13091,16 @@
         <v>719</v>
       </c>
       <c r="J58" t="s">
-        <v>719</v>
+        <v>391</v>
       </c>
       <c r="K58" t="s">
-        <v>719</v>
+        <v>391</v>
       </c>
       <c r="L58" t="s">
-        <v>719</v>
-      </c>
-      <c r="M58" s="1">
-        <v>46313</v>
+        <v>391</v>
       </c>
       <c r="N58" t="s">
-        <v>722</v>
+        <v>395</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -13144,10 +13141,10 @@
         <v>721</v>
       </c>
       <c r="M59" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N59" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -13179,19 +13176,16 @@
         <v>719</v>
       </c>
       <c r="J60" t="s">
-        <v>719</v>
+        <v>391</v>
       </c>
       <c r="K60" t="s">
-        <v>719</v>
+        <v>391</v>
       </c>
       <c r="L60" t="s">
-        <v>719</v>
-      </c>
-      <c r="M60" s="1">
-        <v>46313</v>
+        <v>391</v>
       </c>
       <c r="N60" t="s">
-        <v>722</v>
+        <v>395</v>
       </c>
     </row>
     <row r="61" spans="1:14">
@@ -13223,19 +13217,16 @@
         <v>719</v>
       </c>
       <c r="J61" t="s">
-        <v>719</v>
+        <v>391</v>
       </c>
       <c r="K61" t="s">
-        <v>719</v>
+        <v>391</v>
       </c>
       <c r="L61" t="s">
-        <v>719</v>
-      </c>
-      <c r="M61" s="1">
-        <v>46313</v>
+        <v>391</v>
       </c>
       <c r="N61" t="s">
-        <v>722</v>
+        <v>395</v>
       </c>
     </row>
     <row r="62" spans="1:14">
@@ -13276,10 +13267,10 @@
         <v>721</v>
       </c>
       <c r="M62" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N62" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="63" spans="1:14">
@@ -13320,10 +13311,10 @@
         <v>721</v>
       </c>
       <c r="M63" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N63" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="64" spans="1:14">
@@ -13364,10 +13355,10 @@
         <v>721</v>
       </c>
       <c r="M64" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N64" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="65" spans="1:14">
@@ -13408,10 +13399,10 @@
         <v>721</v>
       </c>
       <c r="M65" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N65" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="66" spans="1:14">
@@ -13452,10 +13443,10 @@
         <v>721</v>
       </c>
       <c r="M66" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N66" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="67" spans="1:14">
@@ -13496,10 +13487,10 @@
         <v>721</v>
       </c>
       <c r="M67" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N67" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="68" spans="1:14">
@@ -13540,10 +13531,10 @@
         <v>721</v>
       </c>
       <c r="M68" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N68" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="69" spans="1:14">
@@ -13584,10 +13575,10 @@
         <v>721</v>
       </c>
       <c r="M69" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N69" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="70" spans="1:14">
@@ -13628,10 +13619,10 @@
         <v>721</v>
       </c>
       <c r="M70" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N70" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="71" spans="1:14">
@@ -13672,10 +13663,10 @@
         <v>721</v>
       </c>
       <c r="M71" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N71" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="72" spans="1:14">
@@ -13716,10 +13707,10 @@
         <v>721</v>
       </c>
       <c r="M72" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N72" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="73" spans="1:14">
@@ -13760,10 +13751,10 @@
         <v>721</v>
       </c>
       <c r="M73" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N73" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="74" spans="1:14">
@@ -13804,10 +13795,10 @@
         <v>721</v>
       </c>
       <c r="M74" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N74" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="75" spans="1:14">
@@ -13848,10 +13839,10 @@
         <v>720</v>
       </c>
       <c r="M75" s="1">
-        <v>46393</v>
+        <v>46394</v>
       </c>
       <c r="N75" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="76" spans="1:14">
@@ -13892,10 +13883,10 @@
         <v>720</v>
       </c>
       <c r="M76" s="1">
-        <v>46393</v>
+        <v>46394</v>
       </c>
       <c r="N76" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="77" spans="1:14">
@@ -13936,10 +13927,10 @@
         <v>721</v>
       </c>
       <c r="M77" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N77" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="78" spans="1:14">
@@ -13980,10 +13971,10 @@
         <v>721</v>
       </c>
       <c r="M78" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N78" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="79" spans="1:14">
@@ -14024,10 +14015,10 @@
         <v>721</v>
       </c>
       <c r="M79" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N79" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="80" spans="1:14">
@@ -14068,10 +14059,10 @@
         <v>721</v>
       </c>
       <c r="M80" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N80" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="81" spans="1:14">
@@ -14103,19 +14094,19 @@
         <v>720</v>
       </c>
       <c r="J81" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="K81" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="L81" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="M81" s="1">
-        <v>46393</v>
+        <v>46379</v>
       </c>
       <c r="N81" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="82" spans="1:14">
@@ -14156,10 +14147,10 @@
         <v>721</v>
       </c>
       <c r="M82" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N82" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="83" spans="1:14">
@@ -14200,10 +14191,10 @@
         <v>721</v>
       </c>
       <c r="M83" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N83" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="84" spans="1:14">
@@ -14244,10 +14235,10 @@
         <v>721</v>
       </c>
       <c r="M84" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N84" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="85" spans="1:14">
@@ -14288,10 +14279,10 @@
         <v>721</v>
       </c>
       <c r="M85" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N85" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="86" spans="1:14">
@@ -14332,10 +14323,10 @@
         <v>721</v>
       </c>
       <c r="M86" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N86" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="87" spans="1:14">
@@ -14376,10 +14367,10 @@
         <v>721</v>
       </c>
       <c r="M87" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N87" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="88" spans="1:14">
@@ -14411,19 +14402,19 @@
         <v>720</v>
       </c>
       <c r="J88" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="K88" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="L88" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="M88" s="1">
-        <v>46393</v>
+        <v>46379</v>
       </c>
       <c r="N88" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="89" spans="1:14">
@@ -14464,10 +14455,10 @@
         <v>721</v>
       </c>
       <c r="M89" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N89" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="90" spans="1:14">
@@ -14499,19 +14490,19 @@
         <v>720</v>
       </c>
       <c r="J90" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="K90" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="L90" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="M90" s="1">
-        <v>46393</v>
+        <v>46379</v>
       </c>
       <c r="N90" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="91" spans="1:14">
@@ -14543,19 +14534,16 @@
         <v>720</v>
       </c>
       <c r="J91" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="K91" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="L91" t="s">
-        <v>720</v>
-      </c>
-      <c r="M91" s="1">
-        <v>46393</v>
+        <v>722</v>
       </c>
       <c r="N91" t="s">
-        <v>722</v>
+        <v>395</v>
       </c>
     </row>
     <row r="92" spans="1:14">
@@ -14596,10 +14584,10 @@
         <v>721</v>
       </c>
       <c r="M92" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N92" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="93" spans="1:14">
@@ -14631,19 +14619,19 @@
         <v>720</v>
       </c>
       <c r="J93" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="K93" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="L93" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="M93" s="1">
-        <v>46393</v>
+        <v>46379</v>
       </c>
       <c r="N93" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="94" spans="1:14">
@@ -14675,19 +14663,19 @@
         <v>720</v>
       </c>
       <c r="J94" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="K94" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="L94" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="M94" s="1">
-        <v>46393</v>
+        <v>46379</v>
       </c>
       <c r="N94" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="95" spans="1:14">
@@ -14728,10 +14716,10 @@
         <v>720</v>
       </c>
       <c r="M95" s="1">
-        <v>46393</v>
+        <v>46394</v>
       </c>
       <c r="N95" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="96" spans="1:14">
@@ -14772,10 +14760,10 @@
         <v>720</v>
       </c>
       <c r="M96" s="1">
-        <v>46393</v>
+        <v>46394</v>
       </c>
       <c r="N96" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="97" spans="1:14">
@@ -14816,10 +14804,10 @@
         <v>721</v>
       </c>
       <c r="M97" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N97" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="98" spans="1:14">
@@ -14860,10 +14848,10 @@
         <v>721</v>
       </c>
       <c r="M98" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N98" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="99" spans="1:14">
@@ -14904,10 +14892,10 @@
         <v>721</v>
       </c>
       <c r="M99" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N99" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="100" spans="1:14">
@@ -14948,10 +14936,10 @@
         <v>721</v>
       </c>
       <c r="M100" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N100" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="101" spans="1:14">
@@ -14992,10 +14980,10 @@
         <v>721</v>
       </c>
       <c r="M101" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N101" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="102" spans="1:14">
@@ -15036,10 +15024,10 @@
         <v>721</v>
       </c>
       <c r="M102" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N102" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="103" spans="1:14">
@@ -15080,10 +15068,10 @@
         <v>721</v>
       </c>
       <c r="M103" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N103" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="104" spans="1:14">
@@ -15115,19 +15103,19 @@
         <v>382</v>
       </c>
       <c r="J104" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K104" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L104" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M104" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N104" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="105" spans="1:14">
@@ -15168,10 +15156,10 @@
         <v>721</v>
       </c>
       <c r="M105" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N105" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="106" spans="1:14">
@@ -15212,10 +15200,10 @@
         <v>720</v>
       </c>
       <c r="M106" s="1">
-        <v>46393</v>
+        <v>46394</v>
       </c>
       <c r="N106" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="107" spans="1:14">
@@ -15256,10 +15244,10 @@
         <v>721</v>
       </c>
       <c r="M107" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N107" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="108" spans="1:14">
@@ -15291,19 +15279,19 @@
         <v>382</v>
       </c>
       <c r="J108" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K108" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L108" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M108" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N108" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="109" spans="1:14">
@@ -15335,19 +15323,19 @@
         <v>382</v>
       </c>
       <c r="J109" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K109" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L109" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M109" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N109" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="110" spans="1:14">
@@ -15388,10 +15376,10 @@
         <v>721</v>
       </c>
       <c r="M110" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N110" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="111" spans="1:14">
@@ -15432,10 +15420,10 @@
         <v>721</v>
       </c>
       <c r="M111" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N111" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="112" spans="1:14">
@@ -15476,10 +15464,10 @@
         <v>721</v>
       </c>
       <c r="M112" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N112" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="113" spans="1:14">
@@ -15520,10 +15508,10 @@
         <v>721</v>
       </c>
       <c r="M113" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N113" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="114" spans="1:14">
@@ -15564,10 +15552,10 @@
         <v>721</v>
       </c>
       <c r="M114" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N114" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="115" spans="1:14">
@@ -15608,10 +15596,10 @@
         <v>721</v>
       </c>
       <c r="M115" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N115" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="116" spans="1:14">
@@ -15652,10 +15640,10 @@
         <v>721</v>
       </c>
       <c r="M116" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N116" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="117" spans="1:14">
@@ -15696,10 +15684,10 @@
         <v>721</v>
       </c>
       <c r="M117" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N117" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="118" spans="1:14">
@@ -15740,10 +15728,10 @@
         <v>721</v>
       </c>
       <c r="M118" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N118" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="119" spans="1:14">
@@ -15775,19 +15763,19 @@
         <v>382</v>
       </c>
       <c r="J119" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K119" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L119" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M119" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N119" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="120" spans="1:14">
@@ -15828,10 +15816,10 @@
         <v>721</v>
       </c>
       <c r="M120" s="1">
-        <v>46378</v>
+        <v>46379</v>
       </c>
       <c r="N120" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="121" spans="1:14">
@@ -15872,10 +15860,10 @@
         <v>720</v>
       </c>
       <c r="M121" s="1">
-        <v>46393</v>
+        <v>46394</v>
       </c>
       <c r="N121" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="122" spans="1:14">
@@ -15907,19 +15895,19 @@
         <v>382</v>
       </c>
       <c r="J122" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K122" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L122" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M122" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N122" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="123" spans="1:14">
@@ -15951,19 +15939,19 @@
         <v>382</v>
       </c>
       <c r="J123" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K123" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="L123" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M123" s="1">
-        <v>46378</v>
+        <v>46394</v>
       </c>
       <c r="N123" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (12/10/2026 17:16)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -11060,7 +11060,7 @@
         <v>721</v>
       </c>
       <c r="M10" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N10" t="s">
         <v>723</v>
@@ -11104,7 +11104,7 @@
         <v>721</v>
       </c>
       <c r="M11" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N11" t="s">
         <v>723</v>
@@ -11312,7 +11312,7 @@
         <v>721</v>
       </c>
       <c r="M16" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N16" t="s">
         <v>723</v>
@@ -11438,7 +11438,7 @@
         <v>721</v>
       </c>
       <c r="M19" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N19" t="s">
         <v>723</v>
@@ -11482,7 +11482,7 @@
         <v>721</v>
       </c>
       <c r="M20" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N20" t="s">
         <v>723</v>
@@ -11526,7 +11526,7 @@
         <v>720</v>
       </c>
       <c r="M21" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N21" t="s">
         <v>723</v>
@@ -11693,7 +11693,7 @@
         <v>721</v>
       </c>
       <c r="M25" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N25" t="s">
         <v>723</v>
@@ -11819,7 +11819,7 @@
         <v>721</v>
       </c>
       <c r="M28" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N28" t="s">
         <v>723</v>
@@ -11863,7 +11863,7 @@
         <v>719</v>
       </c>
       <c r="M29" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N29" t="s">
         <v>723</v>
@@ -11907,7 +11907,7 @@
         <v>720</v>
       </c>
       <c r="M30" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N30" t="s">
         <v>723</v>
@@ -11951,7 +11951,7 @@
         <v>719</v>
       </c>
       <c r="M31" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N31" t="s">
         <v>723</v>
@@ -12364,7 +12364,7 @@
         <v>720</v>
       </c>
       <c r="M41" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N41" t="s">
         <v>723</v>
@@ -12449,7 +12449,7 @@
         <v>721</v>
       </c>
       <c r="M43" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N43" t="s">
         <v>723</v>
@@ -12493,7 +12493,7 @@
         <v>721</v>
       </c>
       <c r="M44" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N44" t="s">
         <v>723</v>
@@ -12537,7 +12537,7 @@
         <v>721</v>
       </c>
       <c r="M45" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N45" t="s">
         <v>723</v>
@@ -12663,7 +12663,7 @@
         <v>721</v>
       </c>
       <c r="M48" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N48" t="s">
         <v>723</v>
@@ -12707,7 +12707,7 @@
         <v>719</v>
       </c>
       <c r="M49" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N49" t="s">
         <v>723</v>
@@ -12751,7 +12751,7 @@
         <v>719</v>
       </c>
       <c r="M50" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N50" t="s">
         <v>723</v>
@@ -12795,7 +12795,7 @@
         <v>720</v>
       </c>
       <c r="M51" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N51" t="s">
         <v>723</v>
@@ -12839,7 +12839,7 @@
         <v>720</v>
       </c>
       <c r="M52" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N52" t="s">
         <v>723</v>
@@ -12883,7 +12883,7 @@
         <v>720</v>
       </c>
       <c r="M53" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N53" t="s">
         <v>723</v>
@@ -12927,7 +12927,7 @@
         <v>721</v>
       </c>
       <c r="M54" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N54" t="s">
         <v>723</v>
@@ -12971,7 +12971,7 @@
         <v>721</v>
       </c>
       <c r="M55" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N55" t="s">
         <v>723</v>
@@ -13015,7 +13015,7 @@
         <v>719</v>
       </c>
       <c r="M56" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N56" t="s">
         <v>723</v>
@@ -13141,7 +13141,7 @@
         <v>721</v>
       </c>
       <c r="M59" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N59" t="s">
         <v>723</v>
@@ -13267,7 +13267,7 @@
         <v>721</v>
       </c>
       <c r="M62" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N62" t="s">
         <v>723</v>
@@ -13311,7 +13311,7 @@
         <v>721</v>
       </c>
       <c r="M63" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N63" t="s">
         <v>723</v>
@@ -13355,7 +13355,7 @@
         <v>721</v>
       </c>
       <c r="M64" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N64" t="s">
         <v>723</v>
@@ -13399,7 +13399,7 @@
         <v>721</v>
       </c>
       <c r="M65" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N65" t="s">
         <v>723</v>
@@ -13443,7 +13443,7 @@
         <v>721</v>
       </c>
       <c r="M66" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N66" t="s">
         <v>723</v>
@@ -13487,7 +13487,7 @@
         <v>721</v>
       </c>
       <c r="M67" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N67" t="s">
         <v>723</v>
@@ -13531,7 +13531,7 @@
         <v>721</v>
       </c>
       <c r="M68" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N68" t="s">
         <v>723</v>
@@ -13575,7 +13575,7 @@
         <v>721</v>
       </c>
       <c r="M69" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N69" t="s">
         <v>723</v>
@@ -13619,7 +13619,7 @@
         <v>721</v>
       </c>
       <c r="M70" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N70" t="s">
         <v>723</v>
@@ -13663,7 +13663,7 @@
         <v>721</v>
       </c>
       <c r="M71" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N71" t="s">
         <v>723</v>
@@ -13707,7 +13707,7 @@
         <v>721</v>
       </c>
       <c r="M72" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N72" t="s">
         <v>723</v>
@@ -13751,7 +13751,7 @@
         <v>721</v>
       </c>
       <c r="M73" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N73" t="s">
         <v>723</v>
@@ -13795,7 +13795,7 @@
         <v>721</v>
       </c>
       <c r="M74" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N74" t="s">
         <v>723</v>
@@ -13839,7 +13839,7 @@
         <v>720</v>
       </c>
       <c r="M75" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N75" t="s">
         <v>723</v>
@@ -13883,7 +13883,7 @@
         <v>720</v>
       </c>
       <c r="M76" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N76" t="s">
         <v>723</v>
@@ -13927,7 +13927,7 @@
         <v>721</v>
       </c>
       <c r="M77" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N77" t="s">
         <v>723</v>
@@ -13971,7 +13971,7 @@
         <v>721</v>
       </c>
       <c r="M78" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N78" t="s">
         <v>723</v>
@@ -14015,7 +14015,7 @@
         <v>721</v>
       </c>
       <c r="M79" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N79" t="s">
         <v>723</v>
@@ -14059,7 +14059,7 @@
         <v>721</v>
       </c>
       <c r="M80" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N80" t="s">
         <v>723</v>
@@ -14103,7 +14103,7 @@
         <v>721</v>
       </c>
       <c r="M81" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N81" t="s">
         <v>723</v>
@@ -14147,7 +14147,7 @@
         <v>721</v>
       </c>
       <c r="M82" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N82" t="s">
         <v>723</v>
@@ -14191,7 +14191,7 @@
         <v>721</v>
       </c>
       <c r="M83" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N83" t="s">
         <v>723</v>
@@ -14235,7 +14235,7 @@
         <v>721</v>
       </c>
       <c r="M84" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N84" t="s">
         <v>723</v>
@@ -14279,7 +14279,7 @@
         <v>721</v>
       </c>
       <c r="M85" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N85" t="s">
         <v>723</v>
@@ -14323,7 +14323,7 @@
         <v>721</v>
       </c>
       <c r="M86" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N86" t="s">
         <v>723</v>
@@ -14367,7 +14367,7 @@
         <v>721</v>
       </c>
       <c r="M87" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N87" t="s">
         <v>723</v>
@@ -14411,7 +14411,7 @@
         <v>721</v>
       </c>
       <c r="M88" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N88" t="s">
         <v>723</v>
@@ -14455,7 +14455,7 @@
         <v>721</v>
       </c>
       <c r="M89" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N89" t="s">
         <v>723</v>
@@ -14499,7 +14499,7 @@
         <v>721</v>
       </c>
       <c r="M90" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N90" t="s">
         <v>723</v>
@@ -14584,7 +14584,7 @@
         <v>721</v>
       </c>
       <c r="M92" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N92" t="s">
         <v>723</v>
@@ -14628,7 +14628,7 @@
         <v>721</v>
       </c>
       <c r="M93" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N93" t="s">
         <v>723</v>
@@ -14672,7 +14672,7 @@
         <v>721</v>
       </c>
       <c r="M94" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N94" t="s">
         <v>723</v>
@@ -14716,7 +14716,7 @@
         <v>720</v>
       </c>
       <c r="M95" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N95" t="s">
         <v>723</v>
@@ -14760,7 +14760,7 @@
         <v>720</v>
       </c>
       <c r="M96" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N96" t="s">
         <v>723</v>
@@ -14804,7 +14804,7 @@
         <v>721</v>
       </c>
       <c r="M97" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N97" t="s">
         <v>723</v>
@@ -14848,7 +14848,7 @@
         <v>721</v>
       </c>
       <c r="M98" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N98" t="s">
         <v>723</v>
@@ -14892,7 +14892,7 @@
         <v>721</v>
       </c>
       <c r="M99" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N99" t="s">
         <v>723</v>
@@ -14936,7 +14936,7 @@
         <v>721</v>
       </c>
       <c r="M100" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N100" t="s">
         <v>723</v>
@@ -14980,7 +14980,7 @@
         <v>721</v>
       </c>
       <c r="M101" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N101" t="s">
         <v>723</v>
@@ -15024,7 +15024,7 @@
         <v>721</v>
       </c>
       <c r="M102" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N102" t="s">
         <v>723</v>
@@ -15068,7 +15068,7 @@
         <v>721</v>
       </c>
       <c r="M103" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N103" t="s">
         <v>723</v>
@@ -15112,7 +15112,7 @@
         <v>720</v>
       </c>
       <c r="M104" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N104" t="s">
         <v>723</v>
@@ -15156,7 +15156,7 @@
         <v>721</v>
       </c>
       <c r="M105" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N105" t="s">
         <v>723</v>
@@ -15200,7 +15200,7 @@
         <v>720</v>
       </c>
       <c r="M106" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N106" t="s">
         <v>723</v>
@@ -15244,7 +15244,7 @@
         <v>721</v>
       </c>
       <c r="M107" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N107" t="s">
         <v>723</v>
@@ -15288,7 +15288,7 @@
         <v>720</v>
       </c>
       <c r="M108" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N108" t="s">
         <v>723</v>
@@ -15332,7 +15332,7 @@
         <v>720</v>
       </c>
       <c r="M109" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N109" t="s">
         <v>723</v>
@@ -15376,7 +15376,7 @@
         <v>721</v>
       </c>
       <c r="M110" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N110" t="s">
         <v>723</v>
@@ -15420,7 +15420,7 @@
         <v>721</v>
       </c>
       <c r="M111" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N111" t="s">
         <v>723</v>
@@ -15464,7 +15464,7 @@
         <v>721</v>
       </c>
       <c r="M112" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N112" t="s">
         <v>723</v>
@@ -15508,7 +15508,7 @@
         <v>721</v>
       </c>
       <c r="M113" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N113" t="s">
         <v>723</v>
@@ -15552,7 +15552,7 @@
         <v>721</v>
       </c>
       <c r="M114" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N114" t="s">
         <v>723</v>
@@ -15596,7 +15596,7 @@
         <v>721</v>
       </c>
       <c r="M115" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N115" t="s">
         <v>723</v>
@@ -15640,7 +15640,7 @@
         <v>721</v>
       </c>
       <c r="M116" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N116" t="s">
         <v>723</v>
@@ -15684,7 +15684,7 @@
         <v>721</v>
       </c>
       <c r="M117" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N117" t="s">
         <v>723</v>
@@ -15728,7 +15728,7 @@
         <v>721</v>
       </c>
       <c r="M118" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N118" t="s">
         <v>723</v>
@@ -15772,7 +15772,7 @@
         <v>720</v>
       </c>
       <c r="M119" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N119" t="s">
         <v>723</v>
@@ -15816,7 +15816,7 @@
         <v>721</v>
       </c>
       <c r="M120" s="1">
-        <v>46379</v>
+        <v>46382</v>
       </c>
       <c r="N120" t="s">
         <v>723</v>
@@ -15860,7 +15860,7 @@
         <v>720</v>
       </c>
       <c r="M121" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N121" t="s">
         <v>723</v>
@@ -15904,7 +15904,7 @@
         <v>720</v>
       </c>
       <c r="M122" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N122" t="s">
         <v>723</v>
@@ -15948,7 +15948,7 @@
         <v>720</v>
       </c>
       <c r="M123" s="1">
-        <v>46394</v>
+        <v>46397</v>
       </c>
       <c r="N123" t="s">
         <v>723</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (13/10/2026 10:14)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2196,8 +2196,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2213,7 +2221,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2221,12 +2229,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2526,55 +2552,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2618,7 +2644,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2662,7 +2688,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2706,7 +2732,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2832,7 +2858,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2876,7 +2902,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2920,7 +2946,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2967,7 +2993,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3090,7 +3116,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -3134,7 +3160,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3178,7 +3204,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3222,7 +3248,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3269,7 +3295,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3313,7 +3339,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3439,7 +3465,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3483,7 +3509,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3568,7 +3594,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3615,7 +3641,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3662,7 +3688,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3706,7 +3732,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3750,7 +3776,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3835,7 +3861,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3920,7 +3946,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3967,7 +3993,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4011,7 +4037,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4055,7 +4081,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4140,7 +4166,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4184,7 +4210,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4228,7 +4254,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4313,7 +4339,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4357,7 +4383,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4401,7 +4427,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4445,7 +4471,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4612,7 +4638,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4656,7 +4682,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4700,7 +4726,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4744,7 +4770,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4791,7 +4817,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4835,7 +4861,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4917,7 +4943,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4961,7 +4987,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5049,7 +5075,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5093,7 +5119,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5140,7 +5166,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5184,7 +5210,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -5228,7 +5254,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5272,7 +5298,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5316,7 +5342,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5363,7 +5389,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5407,7 +5433,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5454,7 +5480,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5498,7 +5524,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5545,7 +5571,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5633,7 +5659,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5677,7 +5703,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5721,7 +5747,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5765,7 +5791,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5809,7 +5835,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5853,7 +5879,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5938,7 +5964,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5982,7 +6008,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -6026,7 +6052,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -6070,7 +6096,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -6114,7 +6140,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -6158,7 +6184,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6202,7 +6228,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6246,7 +6272,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6293,7 +6319,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6337,7 +6363,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6381,7 +6407,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6425,7 +6451,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6469,7 +6495,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6513,7 +6539,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6557,7 +6583,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6601,7 +6627,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6645,7 +6671,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6733,7 +6759,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6777,7 +6803,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6903,7 +6929,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6947,7 +6973,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6991,7 +7017,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7035,7 +7061,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7117,7 +7143,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7161,7 +7187,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7208,7 +7234,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7252,7 +7278,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7378,7 +7404,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7422,7 +7448,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7507,7 +7533,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7551,7 +7577,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7595,7 +7621,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7639,7 +7665,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7683,7 +7709,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7727,7 +7753,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7771,7 +7797,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7815,7 +7841,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7900,7 +7926,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8067,7 +8093,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8111,7 +8137,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8155,7 +8181,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8199,7 +8225,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8243,7 +8269,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8287,7 +8313,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8331,7 +8357,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8416,7 +8442,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8460,7 +8486,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8545,7 +8571,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8671,7 +8697,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8715,7 +8741,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8800,7 +8826,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8844,7 +8870,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8888,7 +8914,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8932,7 +8958,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8976,7 +9002,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -9020,7 +9046,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9064,7 +9090,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9108,7 +9134,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9193,7 +9219,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9360,7 +9386,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9404,7 +9430,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9448,7 +9474,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9492,7 +9518,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9577,7 +9603,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9621,7 +9647,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9665,7 +9691,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9709,7 +9735,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9753,7 +9779,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9797,7 +9823,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9841,7 +9867,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9885,7 +9911,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9929,7 +9955,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9973,7 +9999,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10017,7 +10043,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -10061,7 +10087,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10105,7 +10131,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10149,7 +10175,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -10193,7 +10219,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10237,7 +10263,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10281,7 +10307,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10325,7 +10351,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10369,7 +10395,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10413,7 +10439,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10457,7 +10483,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10542,7 +10568,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10627,7 +10653,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10642,55 +10668,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11059,8 +11085,8 @@
       <c r="L10" t="s">
         <v>721</v>
       </c>
-      <c r="M10" s="1">
-        <v>46382</v>
+      <c r="M10" s="2">
+        <v>46383</v>
       </c>
       <c r="N10" t="s">
         <v>723</v>
@@ -11103,8 +11129,8 @@
       <c r="L11" t="s">
         <v>721</v>
       </c>
-      <c r="M11" s="1">
-        <v>46382</v>
+      <c r="M11" s="2">
+        <v>46383</v>
       </c>
       <c r="N11" t="s">
         <v>723</v>
@@ -11311,8 +11337,8 @@
       <c r="L16" t="s">
         <v>721</v>
       </c>
-      <c r="M16" s="1">
-        <v>46382</v>
+      <c r="M16" s="2">
+        <v>46383</v>
       </c>
       <c r="N16" t="s">
         <v>723</v>
@@ -11437,8 +11463,8 @@
       <c r="L19" t="s">
         <v>721</v>
       </c>
-      <c r="M19" s="1">
-        <v>46382</v>
+      <c r="M19" s="2">
+        <v>46383</v>
       </c>
       <c r="N19" t="s">
         <v>723</v>
@@ -11481,8 +11507,8 @@
       <c r="L20" t="s">
         <v>721</v>
       </c>
-      <c r="M20" s="1">
-        <v>46382</v>
+      <c r="M20" s="2">
+        <v>46383</v>
       </c>
       <c r="N20" t="s">
         <v>723</v>
@@ -11525,8 +11551,8 @@
       <c r="L21" t="s">
         <v>720</v>
       </c>
-      <c r="M21" s="1">
-        <v>46397</v>
+      <c r="M21" s="2">
+        <v>46398</v>
       </c>
       <c r="N21" t="s">
         <v>723</v>
@@ -11692,8 +11718,8 @@
       <c r="L25" t="s">
         <v>721</v>
       </c>
-      <c r="M25" s="1">
-        <v>46382</v>
+      <c r="M25" s="2">
+        <v>46383</v>
       </c>
       <c r="N25" t="s">
         <v>723</v>
@@ -11818,8 +11844,8 @@
       <c r="L28" t="s">
         <v>721</v>
       </c>
-      <c r="M28" s="1">
-        <v>46382</v>
+      <c r="M28" s="2">
+        <v>46383</v>
       </c>
       <c r="N28" t="s">
         <v>723</v>
@@ -11862,8 +11888,8 @@
       <c r="L29" t="s">
         <v>719</v>
       </c>
-      <c r="M29" s="1">
-        <v>46317</v>
+      <c r="M29" s="2">
+        <v>46318</v>
       </c>
       <c r="N29" t="s">
         <v>723</v>
@@ -11906,8 +11932,8 @@
       <c r="L30" t="s">
         <v>720</v>
       </c>
-      <c r="M30" s="1">
-        <v>46397</v>
+      <c r="M30" s="2">
+        <v>46398</v>
       </c>
       <c r="N30" t="s">
         <v>723</v>
@@ -11950,8 +11976,8 @@
       <c r="L31" t="s">
         <v>719</v>
       </c>
-      <c r="M31" s="1">
-        <v>46317</v>
+      <c r="M31" s="2">
+        <v>46318</v>
       </c>
       <c r="N31" t="s">
         <v>723</v>
@@ -12363,8 +12389,8 @@
       <c r="L41" t="s">
         <v>720</v>
       </c>
-      <c r="M41" s="1">
-        <v>46397</v>
+      <c r="M41" s="2">
+        <v>46398</v>
       </c>
       <c r="N41" t="s">
         <v>723</v>
@@ -12448,8 +12474,8 @@
       <c r="L43" t="s">
         <v>721</v>
       </c>
-      <c r="M43" s="1">
-        <v>46382</v>
+      <c r="M43" s="2">
+        <v>46383</v>
       </c>
       <c r="N43" t="s">
         <v>723</v>
@@ -12492,8 +12518,8 @@
       <c r="L44" t="s">
         <v>721</v>
       </c>
-      <c r="M44" s="1">
-        <v>46382</v>
+      <c r="M44" s="2">
+        <v>46383</v>
       </c>
       <c r="N44" t="s">
         <v>723</v>
@@ -12536,8 +12562,8 @@
       <c r="L45" t="s">
         <v>721</v>
       </c>
-      <c r="M45" s="1">
-        <v>46382</v>
+      <c r="M45" s="2">
+        <v>46383</v>
       </c>
       <c r="N45" t="s">
         <v>723</v>
@@ -12662,8 +12688,8 @@
       <c r="L48" t="s">
         <v>721</v>
       </c>
-      <c r="M48" s="1">
-        <v>46382</v>
+      <c r="M48" s="2">
+        <v>46383</v>
       </c>
       <c r="N48" t="s">
         <v>723</v>
@@ -12706,8 +12732,8 @@
       <c r="L49" t="s">
         <v>719</v>
       </c>
-      <c r="M49" s="1">
-        <v>46317</v>
+      <c r="M49" s="2">
+        <v>46318</v>
       </c>
       <c r="N49" t="s">
         <v>723</v>
@@ -12750,8 +12776,8 @@
       <c r="L50" t="s">
         <v>719</v>
       </c>
-      <c r="M50" s="1">
-        <v>46317</v>
+      <c r="M50" s="2">
+        <v>46318</v>
       </c>
       <c r="N50" t="s">
         <v>723</v>
@@ -12794,8 +12820,8 @@
       <c r="L51" t="s">
         <v>720</v>
       </c>
-      <c r="M51" s="1">
-        <v>46397</v>
+      <c r="M51" s="2">
+        <v>46398</v>
       </c>
       <c r="N51" t="s">
         <v>723</v>
@@ -12838,8 +12864,8 @@
       <c r="L52" t="s">
         <v>720</v>
       </c>
-      <c r="M52" s="1">
-        <v>46397</v>
+      <c r="M52" s="2">
+        <v>46398</v>
       </c>
       <c r="N52" t="s">
         <v>723</v>
@@ -12882,8 +12908,8 @@
       <c r="L53" t="s">
         <v>720</v>
       </c>
-      <c r="M53" s="1">
-        <v>46397</v>
+      <c r="M53" s="2">
+        <v>46398</v>
       </c>
       <c r="N53" t="s">
         <v>723</v>
@@ -12926,8 +12952,8 @@
       <c r="L54" t="s">
         <v>721</v>
       </c>
-      <c r="M54" s="1">
-        <v>46382</v>
+      <c r="M54" s="2">
+        <v>46383</v>
       </c>
       <c r="N54" t="s">
         <v>723</v>
@@ -12970,8 +12996,8 @@
       <c r="L55" t="s">
         <v>721</v>
       </c>
-      <c r="M55" s="1">
-        <v>46382</v>
+      <c r="M55" s="2">
+        <v>46383</v>
       </c>
       <c r="N55" t="s">
         <v>723</v>
@@ -13014,8 +13040,8 @@
       <c r="L56" t="s">
         <v>719</v>
       </c>
-      <c r="M56" s="1">
-        <v>46317</v>
+      <c r="M56" s="2">
+        <v>46318</v>
       </c>
       <c r="N56" t="s">
         <v>723</v>
@@ -13140,8 +13166,8 @@
       <c r="L59" t="s">
         <v>721</v>
       </c>
-      <c r="M59" s="1">
-        <v>46382</v>
+      <c r="M59" s="2">
+        <v>46383</v>
       </c>
       <c r="N59" t="s">
         <v>723</v>
@@ -13266,8 +13292,8 @@
       <c r="L62" t="s">
         <v>721</v>
       </c>
-      <c r="M62" s="1">
-        <v>46382</v>
+      <c r="M62" s="2">
+        <v>46383</v>
       </c>
       <c r="N62" t="s">
         <v>723</v>
@@ -13310,8 +13336,8 @@
       <c r="L63" t="s">
         <v>721</v>
       </c>
-      <c r="M63" s="1">
-        <v>46382</v>
+      <c r="M63" s="2">
+        <v>46383</v>
       </c>
       <c r="N63" t="s">
         <v>723</v>
@@ -13354,8 +13380,8 @@
       <c r="L64" t="s">
         <v>721</v>
       </c>
-      <c r="M64" s="1">
-        <v>46382</v>
+      <c r="M64" s="2">
+        <v>46383</v>
       </c>
       <c r="N64" t="s">
         <v>723</v>
@@ -13398,8 +13424,8 @@
       <c r="L65" t="s">
         <v>721</v>
       </c>
-      <c r="M65" s="1">
-        <v>46382</v>
+      <c r="M65" s="2">
+        <v>46383</v>
       </c>
       <c r="N65" t="s">
         <v>723</v>
@@ -13442,8 +13468,8 @@
       <c r="L66" t="s">
         <v>721</v>
       </c>
-      <c r="M66" s="1">
-        <v>46382</v>
+      <c r="M66" s="2">
+        <v>46383</v>
       </c>
       <c r="N66" t="s">
         <v>723</v>
@@ -13486,8 +13512,8 @@
       <c r="L67" t="s">
         <v>721</v>
       </c>
-      <c r="M67" s="1">
-        <v>46382</v>
+      <c r="M67" s="2">
+        <v>46383</v>
       </c>
       <c r="N67" t="s">
         <v>723</v>
@@ -13530,8 +13556,8 @@
       <c r="L68" t="s">
         <v>721</v>
       </c>
-      <c r="M68" s="1">
-        <v>46382</v>
+      <c r="M68" s="2">
+        <v>46383</v>
       </c>
       <c r="N68" t="s">
         <v>723</v>
@@ -13574,8 +13600,8 @@
       <c r="L69" t="s">
         <v>721</v>
       </c>
-      <c r="M69" s="1">
-        <v>46382</v>
+      <c r="M69" s="2">
+        <v>46383</v>
       </c>
       <c r="N69" t="s">
         <v>723</v>
@@ -13618,8 +13644,8 @@
       <c r="L70" t="s">
         <v>721</v>
       </c>
-      <c r="M70" s="1">
-        <v>46382</v>
+      <c r="M70" s="2">
+        <v>46383</v>
       </c>
       <c r="N70" t="s">
         <v>723</v>
@@ -13662,8 +13688,8 @@
       <c r="L71" t="s">
         <v>721</v>
       </c>
-      <c r="M71" s="1">
-        <v>46382</v>
+      <c r="M71" s="2">
+        <v>46383</v>
       </c>
       <c r="N71" t="s">
         <v>723</v>
@@ -13706,8 +13732,8 @@
       <c r="L72" t="s">
         <v>721</v>
       </c>
-      <c r="M72" s="1">
-        <v>46382</v>
+      <c r="M72" s="2">
+        <v>46383</v>
       </c>
       <c r="N72" t="s">
         <v>723</v>
@@ -13750,8 +13776,8 @@
       <c r="L73" t="s">
         <v>721</v>
       </c>
-      <c r="M73" s="1">
-        <v>46382</v>
+      <c r="M73" s="2">
+        <v>46383</v>
       </c>
       <c r="N73" t="s">
         <v>723</v>
@@ -13794,8 +13820,8 @@
       <c r="L74" t="s">
         <v>721</v>
       </c>
-      <c r="M74" s="1">
-        <v>46382</v>
+      <c r="M74" s="2">
+        <v>46383</v>
       </c>
       <c r="N74" t="s">
         <v>723</v>
@@ -13838,8 +13864,8 @@
       <c r="L75" t="s">
         <v>720</v>
       </c>
-      <c r="M75" s="1">
-        <v>46397</v>
+      <c r="M75" s="2">
+        <v>46398</v>
       </c>
       <c r="N75" t="s">
         <v>723</v>
@@ -13882,8 +13908,8 @@
       <c r="L76" t="s">
         <v>720</v>
       </c>
-      <c r="M76" s="1">
-        <v>46397</v>
+      <c r="M76" s="2">
+        <v>46398</v>
       </c>
       <c r="N76" t="s">
         <v>723</v>
@@ -13926,8 +13952,8 @@
       <c r="L77" t="s">
         <v>721</v>
       </c>
-      <c r="M77" s="1">
-        <v>46382</v>
+      <c r="M77" s="2">
+        <v>46383</v>
       </c>
       <c r="N77" t="s">
         <v>723</v>
@@ -13970,8 +13996,8 @@
       <c r="L78" t="s">
         <v>721</v>
       </c>
-      <c r="M78" s="1">
-        <v>46382</v>
+      <c r="M78" s="2">
+        <v>46383</v>
       </c>
       <c r="N78" t="s">
         <v>723</v>
@@ -14014,8 +14040,8 @@
       <c r="L79" t="s">
         <v>721</v>
       </c>
-      <c r="M79" s="1">
-        <v>46382</v>
+      <c r="M79" s="2">
+        <v>46383</v>
       </c>
       <c r="N79" t="s">
         <v>723</v>
@@ -14058,8 +14084,8 @@
       <c r="L80" t="s">
         <v>721</v>
       </c>
-      <c r="M80" s="1">
-        <v>46382</v>
+      <c r="M80" s="2">
+        <v>46383</v>
       </c>
       <c r="N80" t="s">
         <v>723</v>
@@ -14102,8 +14128,8 @@
       <c r="L81" t="s">
         <v>721</v>
       </c>
-      <c r="M81" s="1">
-        <v>46382</v>
+      <c r="M81" s="2">
+        <v>46383</v>
       </c>
       <c r="N81" t="s">
         <v>723</v>
@@ -14146,8 +14172,8 @@
       <c r="L82" t="s">
         <v>721</v>
       </c>
-      <c r="M82" s="1">
-        <v>46382</v>
+      <c r="M82" s="2">
+        <v>46383</v>
       </c>
       <c r="N82" t="s">
         <v>723</v>
@@ -14190,8 +14216,8 @@
       <c r="L83" t="s">
         <v>721</v>
       </c>
-      <c r="M83" s="1">
-        <v>46382</v>
+      <c r="M83" s="2">
+        <v>46383</v>
       </c>
       <c r="N83" t="s">
         <v>723</v>
@@ -14234,8 +14260,8 @@
       <c r="L84" t="s">
         <v>721</v>
       </c>
-      <c r="M84" s="1">
-        <v>46382</v>
+      <c r="M84" s="2">
+        <v>46383</v>
       </c>
       <c r="N84" t="s">
         <v>723</v>
@@ -14278,8 +14304,8 @@
       <c r="L85" t="s">
         <v>721</v>
       </c>
-      <c r="M85" s="1">
-        <v>46382</v>
+      <c r="M85" s="2">
+        <v>46383</v>
       </c>
       <c r="N85" t="s">
         <v>723</v>
@@ -14322,8 +14348,8 @@
       <c r="L86" t="s">
         <v>721</v>
       </c>
-      <c r="M86" s="1">
-        <v>46382</v>
+      <c r="M86" s="2">
+        <v>46383</v>
       </c>
       <c r="N86" t="s">
         <v>723</v>
@@ -14366,8 +14392,8 @@
       <c r="L87" t="s">
         <v>721</v>
       </c>
-      <c r="M87" s="1">
-        <v>46382</v>
+      <c r="M87" s="2">
+        <v>46383</v>
       </c>
       <c r="N87" t="s">
         <v>723</v>
@@ -14410,8 +14436,8 @@
       <c r="L88" t="s">
         <v>721</v>
       </c>
-      <c r="M88" s="1">
-        <v>46382</v>
+      <c r="M88" s="2">
+        <v>46383</v>
       </c>
       <c r="N88" t="s">
         <v>723</v>
@@ -14454,8 +14480,8 @@
       <c r="L89" t="s">
         <v>721</v>
       </c>
-      <c r="M89" s="1">
-        <v>46382</v>
+      <c r="M89" s="2">
+        <v>46383</v>
       </c>
       <c r="N89" t="s">
         <v>723</v>
@@ -14498,8 +14524,8 @@
       <c r="L90" t="s">
         <v>721</v>
       </c>
-      <c r="M90" s="1">
-        <v>46382</v>
+      <c r="M90" s="2">
+        <v>46383</v>
       </c>
       <c r="N90" t="s">
         <v>723</v>
@@ -14583,8 +14609,8 @@
       <c r="L92" t="s">
         <v>721</v>
       </c>
-      <c r="M92" s="1">
-        <v>46382</v>
+      <c r="M92" s="2">
+        <v>46383</v>
       </c>
       <c r="N92" t="s">
         <v>723</v>
@@ -14627,8 +14653,8 @@
       <c r="L93" t="s">
         <v>721</v>
       </c>
-      <c r="M93" s="1">
-        <v>46382</v>
+      <c r="M93" s="2">
+        <v>46383</v>
       </c>
       <c r="N93" t="s">
         <v>723</v>
@@ -14671,8 +14697,8 @@
       <c r="L94" t="s">
         <v>721</v>
       </c>
-      <c r="M94" s="1">
-        <v>46382</v>
+      <c r="M94" s="2">
+        <v>46383</v>
       </c>
       <c r="N94" t="s">
         <v>723</v>
@@ -14715,8 +14741,8 @@
       <c r="L95" t="s">
         <v>720</v>
       </c>
-      <c r="M95" s="1">
-        <v>46397</v>
+      <c r="M95" s="2">
+        <v>46398</v>
       </c>
       <c r="N95" t="s">
         <v>723</v>
@@ -14759,8 +14785,8 @@
       <c r="L96" t="s">
         <v>720</v>
       </c>
-      <c r="M96" s="1">
-        <v>46397</v>
+      <c r="M96" s="2">
+        <v>46398</v>
       </c>
       <c r="N96" t="s">
         <v>723</v>
@@ -14803,8 +14829,8 @@
       <c r="L97" t="s">
         <v>721</v>
       </c>
-      <c r="M97" s="1">
-        <v>46382</v>
+      <c r="M97" s="2">
+        <v>46383</v>
       </c>
       <c r="N97" t="s">
         <v>723</v>
@@ -14847,8 +14873,8 @@
       <c r="L98" t="s">
         <v>721</v>
       </c>
-      <c r="M98" s="1">
-        <v>46382</v>
+      <c r="M98" s="2">
+        <v>46383</v>
       </c>
       <c r="N98" t="s">
         <v>723</v>
@@ -14891,8 +14917,8 @@
       <c r="L99" t="s">
         <v>721</v>
       </c>
-      <c r="M99" s="1">
-        <v>46382</v>
+      <c r="M99" s="2">
+        <v>46383</v>
       </c>
       <c r="N99" t="s">
         <v>723</v>
@@ -14935,8 +14961,8 @@
       <c r="L100" t="s">
         <v>721</v>
       </c>
-      <c r="M100" s="1">
-        <v>46382</v>
+      <c r="M100" s="2">
+        <v>46383</v>
       </c>
       <c r="N100" t="s">
         <v>723</v>
@@ -14979,8 +15005,8 @@
       <c r="L101" t="s">
         <v>721</v>
       </c>
-      <c r="M101" s="1">
-        <v>46382</v>
+      <c r="M101" s="2">
+        <v>46383</v>
       </c>
       <c r="N101" t="s">
         <v>723</v>
@@ -15023,8 +15049,8 @@
       <c r="L102" t="s">
         <v>721</v>
       </c>
-      <c r="M102" s="1">
-        <v>46382</v>
+      <c r="M102" s="2">
+        <v>46383</v>
       </c>
       <c r="N102" t="s">
         <v>723</v>
@@ -15067,8 +15093,8 @@
       <c r="L103" t="s">
         <v>721</v>
       </c>
-      <c r="M103" s="1">
-        <v>46382</v>
+      <c r="M103" s="2">
+        <v>46383</v>
       </c>
       <c r="N103" t="s">
         <v>723</v>
@@ -15111,8 +15137,8 @@
       <c r="L104" t="s">
         <v>720</v>
       </c>
-      <c r="M104" s="1">
-        <v>46397</v>
+      <c r="M104" s="2">
+        <v>46398</v>
       </c>
       <c r="N104" t="s">
         <v>723</v>
@@ -15155,8 +15181,8 @@
       <c r="L105" t="s">
         <v>721</v>
       </c>
-      <c r="M105" s="1">
-        <v>46382</v>
+      <c r="M105" s="2">
+        <v>46383</v>
       </c>
       <c r="N105" t="s">
         <v>723</v>
@@ -15199,8 +15225,8 @@
       <c r="L106" t="s">
         <v>720</v>
       </c>
-      <c r="M106" s="1">
-        <v>46397</v>
+      <c r="M106" s="2">
+        <v>46398</v>
       </c>
       <c r="N106" t="s">
         <v>723</v>
@@ -15243,8 +15269,8 @@
       <c r="L107" t="s">
         <v>721</v>
       </c>
-      <c r="M107" s="1">
-        <v>46382</v>
+      <c r="M107" s="2">
+        <v>46383</v>
       </c>
       <c r="N107" t="s">
         <v>723</v>
@@ -15287,8 +15313,8 @@
       <c r="L108" t="s">
         <v>720</v>
       </c>
-      <c r="M108" s="1">
-        <v>46397</v>
+      <c r="M108" s="2">
+        <v>46398</v>
       </c>
       <c r="N108" t="s">
         <v>723</v>
@@ -15331,8 +15357,8 @@
       <c r="L109" t="s">
         <v>720</v>
       </c>
-      <c r="M109" s="1">
-        <v>46397</v>
+      <c r="M109" s="2">
+        <v>46398</v>
       </c>
       <c r="N109" t="s">
         <v>723</v>
@@ -15375,8 +15401,8 @@
       <c r="L110" t="s">
         <v>721</v>
       </c>
-      <c r="M110" s="1">
-        <v>46382</v>
+      <c r="M110" s="2">
+        <v>46383</v>
       </c>
       <c r="N110" t="s">
         <v>723</v>
@@ -15419,8 +15445,8 @@
       <c r="L111" t="s">
         <v>721</v>
       </c>
-      <c r="M111" s="1">
-        <v>46382</v>
+      <c r="M111" s="2">
+        <v>46383</v>
       </c>
       <c r="N111" t="s">
         <v>723</v>
@@ -15463,8 +15489,8 @@
       <c r="L112" t="s">
         <v>721</v>
       </c>
-      <c r="M112" s="1">
-        <v>46382</v>
+      <c r="M112" s="2">
+        <v>46383</v>
       </c>
       <c r="N112" t="s">
         <v>723</v>
@@ -15507,8 +15533,8 @@
       <c r="L113" t="s">
         <v>721</v>
       </c>
-      <c r="M113" s="1">
-        <v>46382</v>
+      <c r="M113" s="2">
+        <v>46383</v>
       </c>
       <c r="N113" t="s">
         <v>723</v>
@@ -15551,8 +15577,8 @@
       <c r="L114" t="s">
         <v>721</v>
       </c>
-      <c r="M114" s="1">
-        <v>46382</v>
+      <c r="M114" s="2">
+        <v>46383</v>
       </c>
       <c r="N114" t="s">
         <v>723</v>
@@ -15595,8 +15621,8 @@
       <c r="L115" t="s">
         <v>721</v>
       </c>
-      <c r="M115" s="1">
-        <v>46382</v>
+      <c r="M115" s="2">
+        <v>46383</v>
       </c>
       <c r="N115" t="s">
         <v>723</v>
@@ -15639,8 +15665,8 @@
       <c r="L116" t="s">
         <v>721</v>
       </c>
-      <c r="M116" s="1">
-        <v>46382</v>
+      <c r="M116" s="2">
+        <v>46383</v>
       </c>
       <c r="N116" t="s">
         <v>723</v>
@@ -15683,8 +15709,8 @@
       <c r="L117" t="s">
         <v>721</v>
       </c>
-      <c r="M117" s="1">
-        <v>46382</v>
+      <c r="M117" s="2">
+        <v>46383</v>
       </c>
       <c r="N117" t="s">
         <v>723</v>
@@ -15727,8 +15753,8 @@
       <c r="L118" t="s">
         <v>721</v>
       </c>
-      <c r="M118" s="1">
-        <v>46382</v>
+      <c r="M118" s="2">
+        <v>46383</v>
       </c>
       <c r="N118" t="s">
         <v>723</v>
@@ -15771,8 +15797,8 @@
       <c r="L119" t="s">
         <v>720</v>
       </c>
-      <c r="M119" s="1">
-        <v>46397</v>
+      <c r="M119" s="2">
+        <v>46398</v>
       </c>
       <c r="N119" t="s">
         <v>723</v>
@@ -15815,8 +15841,8 @@
       <c r="L120" t="s">
         <v>721</v>
       </c>
-      <c r="M120" s="1">
-        <v>46382</v>
+      <c r="M120" s="2">
+        <v>46383</v>
       </c>
       <c r="N120" t="s">
         <v>723</v>
@@ -15859,8 +15885,8 @@
       <c r="L121" t="s">
         <v>720</v>
       </c>
-      <c r="M121" s="1">
-        <v>46397</v>
+      <c r="M121" s="2">
+        <v>46398</v>
       </c>
       <c r="N121" t="s">
         <v>723</v>
@@ -15903,8 +15929,8 @@
       <c r="L122" t="s">
         <v>720</v>
       </c>
-      <c r="M122" s="1">
-        <v>46397</v>
+      <c r="M122" s="2">
+        <v>46398</v>
       </c>
       <c r="N122" t="s">
         <v>723</v>
@@ -15947,8 +15973,8 @@
       <c r="L123" t="s">
         <v>720</v>
       </c>
-      <c r="M123" s="1">
-        <v>46397</v>
+      <c r="M123" s="2">
+        <v>46398</v>
       </c>
       <c r="N123" t="s">
         <v>723</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (14/10/2026 12:49)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -11069,7 +11069,7 @@
         <v>724</v>
       </c>
       <c r="M10" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N10" t="s">
         <v>726</v>
@@ -11113,7 +11113,7 @@
         <v>724</v>
       </c>
       <c r="M11" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N11" t="s">
         <v>726</v>
@@ -11321,7 +11321,7 @@
         <v>724</v>
       </c>
       <c r="M16" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N16" t="s">
         <v>726</v>
@@ -11447,7 +11447,7 @@
         <v>724</v>
       </c>
       <c r="M19" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N19" t="s">
         <v>726</v>
@@ -11491,7 +11491,7 @@
         <v>724</v>
       </c>
       <c r="M20" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N20" t="s">
         <v>726</v>
@@ -11535,7 +11535,7 @@
         <v>722</v>
       </c>
       <c r="M21" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N21" t="s">
         <v>726</v>
@@ -11702,7 +11702,7 @@
         <v>724</v>
       </c>
       <c r="M25" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N25" t="s">
         <v>726</v>
@@ -11828,7 +11828,7 @@
         <v>722</v>
       </c>
       <c r="M28" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N28" t="s">
         <v>726</v>
@@ -11913,7 +11913,7 @@
         <v>722</v>
       </c>
       <c r="M30" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N30" t="s">
         <v>726</v>
@@ -12367,7 +12367,7 @@
         <v>722</v>
       </c>
       <c r="M41" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N41" t="s">
         <v>726</v>
@@ -12452,7 +12452,7 @@
         <v>724</v>
       </c>
       <c r="M43" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N43" t="s">
         <v>726</v>
@@ -12496,7 +12496,7 @@
         <v>724</v>
       </c>
       <c r="M44" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N44" t="s">
         <v>726</v>
@@ -12540,7 +12540,7 @@
         <v>724</v>
       </c>
       <c r="M45" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N45" t="s">
         <v>726</v>
@@ -12666,7 +12666,7 @@
         <v>724</v>
       </c>
       <c r="M48" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N48" t="s">
         <v>726</v>
@@ -12710,7 +12710,7 @@
         <v>723</v>
       </c>
       <c r="M49" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N49" t="s">
         <v>726</v>
@@ -12754,7 +12754,7 @@
         <v>723</v>
       </c>
       <c r="M50" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N50" t="s">
         <v>726</v>
@@ -12798,7 +12798,7 @@
         <v>722</v>
       </c>
       <c r="M51" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N51" t="s">
         <v>726</v>
@@ -12842,7 +12842,7 @@
         <v>722</v>
       </c>
       <c r="M52" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N52" t="s">
         <v>726</v>
@@ -12886,7 +12886,7 @@
         <v>722</v>
       </c>
       <c r="M53" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N53" t="s">
         <v>726</v>
@@ -12930,7 +12930,7 @@
         <v>724</v>
       </c>
       <c r="M54" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N54" t="s">
         <v>726</v>
@@ -12974,7 +12974,7 @@
         <v>724</v>
       </c>
       <c r="M55" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N55" t="s">
         <v>726</v>
@@ -13141,7 +13141,7 @@
         <v>724</v>
       </c>
       <c r="M59" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N59" t="s">
         <v>726</v>
@@ -13267,7 +13267,7 @@
         <v>724</v>
       </c>
       <c r="M62" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N62" t="s">
         <v>726</v>
@@ -13311,7 +13311,7 @@
         <v>724</v>
       </c>
       <c r="M63" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N63" t="s">
         <v>726</v>
@@ -13355,7 +13355,7 @@
         <v>724</v>
       </c>
       <c r="M64" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N64" t="s">
         <v>726</v>
@@ -13399,7 +13399,7 @@
         <v>724</v>
       </c>
       <c r="M65" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N65" t="s">
         <v>726</v>
@@ -13443,7 +13443,7 @@
         <v>724</v>
       </c>
       <c r="M66" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N66" t="s">
         <v>726</v>
@@ -13487,7 +13487,7 @@
         <v>724</v>
       </c>
       <c r="M67" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N67" t="s">
         <v>726</v>
@@ -13531,7 +13531,7 @@
         <v>724</v>
       </c>
       <c r="M68" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N68" t="s">
         <v>726</v>
@@ -13575,7 +13575,7 @@
         <v>724</v>
       </c>
       <c r="M69" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N69" t="s">
         <v>726</v>
@@ -13619,7 +13619,7 @@
         <v>724</v>
       </c>
       <c r="M70" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N70" t="s">
         <v>726</v>
@@ -13663,7 +13663,7 @@
         <v>724</v>
       </c>
       <c r="M71" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N71" t="s">
         <v>726</v>
@@ -13707,7 +13707,7 @@
         <v>724</v>
       </c>
       <c r="M72" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N72" t="s">
         <v>726</v>
@@ -13751,7 +13751,7 @@
         <v>724</v>
       </c>
       <c r="M73" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N73" t="s">
         <v>726</v>
@@ -13795,7 +13795,7 @@
         <v>724</v>
       </c>
       <c r="M74" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N74" t="s">
         <v>726</v>
@@ -13839,7 +13839,7 @@
         <v>722</v>
       </c>
       <c r="M75" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N75" t="s">
         <v>726</v>
@@ -13883,7 +13883,7 @@
         <v>722</v>
       </c>
       <c r="M76" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N76" t="s">
         <v>726</v>
@@ -13927,7 +13927,7 @@
         <v>724</v>
       </c>
       <c r="M77" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N77" t="s">
         <v>726</v>
@@ -13971,7 +13971,7 @@
         <v>724</v>
       </c>
       <c r="M78" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N78" t="s">
         <v>726</v>
@@ -14015,7 +14015,7 @@
         <v>724</v>
       </c>
       <c r="M79" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N79" t="s">
         <v>726</v>
@@ -14059,7 +14059,7 @@
         <v>724</v>
       </c>
       <c r="M80" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N80" t="s">
         <v>726</v>
@@ -14103,7 +14103,7 @@
         <v>724</v>
       </c>
       <c r="M81" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N81" t="s">
         <v>726</v>
@@ -14147,7 +14147,7 @@
         <v>724</v>
       </c>
       <c r="M82" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N82" t="s">
         <v>726</v>
@@ -14191,7 +14191,7 @@
         <v>724</v>
       </c>
       <c r="M83" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N83" t="s">
         <v>726</v>
@@ -14235,7 +14235,7 @@
         <v>724</v>
       </c>
       <c r="M84" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N84" t="s">
         <v>726</v>
@@ -14279,7 +14279,7 @@
         <v>724</v>
       </c>
       <c r="M85" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N85" t="s">
         <v>726</v>
@@ -14323,7 +14323,7 @@
         <v>724</v>
       </c>
       <c r="M86" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N86" t="s">
         <v>726</v>
@@ -14367,7 +14367,7 @@
         <v>724</v>
       </c>
       <c r="M87" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N87" t="s">
         <v>726</v>
@@ -14411,7 +14411,7 @@
         <v>724</v>
       </c>
       <c r="M88" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N88" t="s">
         <v>726</v>
@@ -14455,7 +14455,7 @@
         <v>724</v>
       </c>
       <c r="M89" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N89" t="s">
         <v>726</v>
@@ -14499,7 +14499,7 @@
         <v>724</v>
       </c>
       <c r="M90" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N90" t="s">
         <v>726</v>
@@ -14584,7 +14584,7 @@
         <v>724</v>
       </c>
       <c r="M92" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N92" t="s">
         <v>726</v>
@@ -14628,7 +14628,7 @@
         <v>724</v>
       </c>
       <c r="M93" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N93" t="s">
         <v>726</v>
@@ -14672,7 +14672,7 @@
         <v>724</v>
       </c>
       <c r="M94" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N94" t="s">
         <v>726</v>
@@ -14716,7 +14716,7 @@
         <v>722</v>
       </c>
       <c r="M95" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N95" t="s">
         <v>726</v>
@@ -14760,7 +14760,7 @@
         <v>722</v>
       </c>
       <c r="M96" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N96" t="s">
         <v>726</v>
@@ -14804,7 +14804,7 @@
         <v>724</v>
       </c>
       <c r="M97" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N97" t="s">
         <v>726</v>
@@ -14848,7 +14848,7 @@
         <v>724</v>
       </c>
       <c r="M98" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N98" t="s">
         <v>726</v>
@@ -14892,7 +14892,7 @@
         <v>724</v>
       </c>
       <c r="M99" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N99" t="s">
         <v>726</v>
@@ -14936,7 +14936,7 @@
         <v>724</v>
       </c>
       <c r="M100" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N100" t="s">
         <v>726</v>
@@ -14980,7 +14980,7 @@
         <v>724</v>
       </c>
       <c r="M101" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N101" t="s">
         <v>726</v>
@@ -15024,7 +15024,7 @@
         <v>724</v>
       </c>
       <c r="M102" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N102" t="s">
         <v>726</v>
@@ -15068,7 +15068,7 @@
         <v>724</v>
       </c>
       <c r="M103" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N103" t="s">
         <v>726</v>
@@ -15112,7 +15112,7 @@
         <v>722</v>
       </c>
       <c r="M104" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N104" t="s">
         <v>726</v>
@@ -15156,7 +15156,7 @@
         <v>724</v>
       </c>
       <c r="M105" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N105" t="s">
         <v>726</v>
@@ -15200,7 +15200,7 @@
         <v>722</v>
       </c>
       <c r="M106" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N106" t="s">
         <v>726</v>
@@ -15244,7 +15244,7 @@
         <v>724</v>
       </c>
       <c r="M107" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N107" t="s">
         <v>726</v>
@@ -15288,7 +15288,7 @@
         <v>722</v>
       </c>
       <c r="M108" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N108" t="s">
         <v>726</v>
@@ -15332,7 +15332,7 @@
         <v>722</v>
       </c>
       <c r="M109" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N109" t="s">
         <v>726</v>
@@ -15376,7 +15376,7 @@
         <v>724</v>
       </c>
       <c r="M110" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N110" t="s">
         <v>726</v>
@@ -15420,7 +15420,7 @@
         <v>724</v>
       </c>
       <c r="M111" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N111" t="s">
         <v>726</v>
@@ -15464,7 +15464,7 @@
         <v>724</v>
       </c>
       <c r="M112" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N112" t="s">
         <v>726</v>
@@ -15508,7 +15508,7 @@
         <v>724</v>
       </c>
       <c r="M113" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N113" t="s">
         <v>726</v>
@@ -15552,7 +15552,7 @@
         <v>724</v>
       </c>
       <c r="M114" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N114" t="s">
         <v>726</v>
@@ -15596,7 +15596,7 @@
         <v>724</v>
       </c>
       <c r="M115" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N115" t="s">
         <v>726</v>
@@ -15640,7 +15640,7 @@
         <v>724</v>
       </c>
       <c r="M116" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N116" t="s">
         <v>726</v>
@@ -15684,7 +15684,7 @@
         <v>724</v>
       </c>
       <c r="M117" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N117" t="s">
         <v>726</v>
@@ -15728,7 +15728,7 @@
         <v>724</v>
       </c>
       <c r="M118" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N118" t="s">
         <v>726</v>
@@ -15772,7 +15772,7 @@
         <v>722</v>
       </c>
       <c r="M119" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N119" t="s">
         <v>726</v>
@@ -15816,7 +15816,7 @@
         <v>724</v>
       </c>
       <c r="M120" s="1">
-        <v>46383</v>
+        <v>46384</v>
       </c>
       <c r="N120" t="s">
         <v>726</v>
@@ -15860,7 +15860,7 @@
         <v>722</v>
       </c>
       <c r="M121" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N121" t="s">
         <v>726</v>
@@ -15904,7 +15904,7 @@
         <v>722</v>
       </c>
       <c r="M122" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N122" t="s">
         <v>726</v>
@@ -15948,7 +15948,7 @@
         <v>722</v>
       </c>
       <c r="M123" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N123" t="s">
         <v>726</v>
@@ -15992,7 +15992,7 @@
         <v>722</v>
       </c>
       <c r="M124" s="1">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="N124" t="s">
         <v>726</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (14/10/2026 13:34)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2205,8 +2205,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2222,7 +2230,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2230,12 +2238,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2535,55 +2561,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2627,7 +2653,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2671,7 +2697,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2715,7 +2741,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2885,7 +2911,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2929,7 +2955,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2976,7 +3002,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3099,7 +3125,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -3143,7 +3169,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3187,7 +3213,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3231,7 +3257,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3278,7 +3304,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3322,7 +3348,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3448,7 +3474,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3492,7 +3518,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3577,7 +3603,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3624,7 +3650,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3671,7 +3697,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3715,7 +3741,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3759,7 +3785,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3844,7 +3870,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3929,7 +3955,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3976,7 +4002,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4020,7 +4046,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4064,7 +4090,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4149,7 +4175,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4193,7 +4219,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4237,7 +4263,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4322,7 +4348,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4366,7 +4392,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4410,7 +4436,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4454,7 +4480,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4621,7 +4647,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4665,7 +4691,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4709,7 +4735,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4753,7 +4779,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4800,7 +4826,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4844,7 +4870,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4926,7 +4952,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4970,7 +4996,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5058,7 +5084,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5102,7 +5128,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5149,7 +5175,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5193,7 +5219,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -5237,7 +5263,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5281,7 +5307,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5325,7 +5351,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5372,7 +5398,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5416,7 +5442,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5463,7 +5489,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5507,7 +5533,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5554,7 +5580,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5642,7 +5668,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5686,7 +5712,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5730,7 +5756,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5774,7 +5800,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5818,7 +5844,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5862,7 +5888,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5947,7 +5973,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5991,7 +6017,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -6035,7 +6061,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -6079,7 +6105,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -6123,7 +6149,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -6167,7 +6193,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6211,7 +6237,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6255,7 +6281,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6302,7 +6328,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6346,7 +6372,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6390,7 +6416,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6434,7 +6460,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6478,7 +6504,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6566,7 +6592,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6610,7 +6636,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6654,7 +6680,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6742,7 +6768,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6786,7 +6812,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6912,7 +6938,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6956,7 +6982,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7000,7 +7026,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7044,7 +7070,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7126,7 +7152,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7170,7 +7196,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7217,7 +7243,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7261,7 +7287,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7387,7 +7413,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7431,7 +7457,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7516,7 +7542,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7560,7 +7586,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7604,7 +7630,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7648,7 +7674,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7692,7 +7718,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7736,7 +7762,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7780,7 +7806,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7824,7 +7850,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7909,7 +7935,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8076,7 +8102,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8120,7 +8146,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8164,7 +8190,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8208,7 +8234,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8252,7 +8278,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8296,7 +8322,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8340,7 +8366,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8425,7 +8451,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8469,7 +8495,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8554,7 +8580,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8680,7 +8706,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8724,7 +8750,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8809,7 +8835,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8853,7 +8879,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8897,7 +8923,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8941,7 +8967,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8985,7 +9011,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -9029,7 +9055,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9073,7 +9099,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9117,7 +9143,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9202,7 +9228,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9369,7 +9395,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9413,7 +9439,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9457,7 +9483,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9501,7 +9527,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9586,7 +9612,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9630,7 +9656,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9674,7 +9700,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9718,7 +9744,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9762,7 +9788,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9806,7 +9832,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9850,7 +9876,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9894,7 +9920,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9938,7 +9964,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9982,7 +10008,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10026,7 +10052,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -10070,7 +10096,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10114,7 +10140,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10158,7 +10184,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -10202,7 +10228,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10246,7 +10272,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10290,7 +10316,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10334,7 +10360,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10378,7 +10404,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10422,7 +10448,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10466,7 +10492,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10551,7 +10577,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10636,7 +10662,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10651,55 +10677,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11068,7 +11094,7 @@
       <c r="L10" t="s">
         <v>724</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46384</v>
       </c>
       <c r="N10" t="s">
@@ -11112,7 +11138,7 @@
       <c r="L11" t="s">
         <v>724</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46384</v>
       </c>
       <c r="N11" t="s">
@@ -11320,7 +11346,7 @@
       <c r="L16" t="s">
         <v>724</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46384</v>
       </c>
       <c r="N16" t="s">
@@ -11446,7 +11472,7 @@
       <c r="L19" t="s">
         <v>724</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46384</v>
       </c>
       <c r="N19" t="s">
@@ -11490,7 +11516,7 @@
       <c r="L20" t="s">
         <v>724</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46384</v>
       </c>
       <c r="N20" t="s">
@@ -11534,7 +11560,7 @@
       <c r="L21" t="s">
         <v>722</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46399</v>
       </c>
       <c r="N21" t="s">
@@ -11701,7 +11727,7 @@
       <c r="L25" t="s">
         <v>724</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46384</v>
       </c>
       <c r="N25" t="s">
@@ -11827,7 +11853,7 @@
       <c r="L28" t="s">
         <v>722</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46399</v>
       </c>
       <c r="N28" t="s">
@@ -11912,7 +11938,7 @@
       <c r="L30" t="s">
         <v>722</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46399</v>
       </c>
       <c r="N30" t="s">
@@ -12366,7 +12392,7 @@
       <c r="L41" t="s">
         <v>722</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46399</v>
       </c>
       <c r="N41" t="s">
@@ -12451,7 +12477,7 @@
       <c r="L43" t="s">
         <v>724</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46384</v>
       </c>
       <c r="N43" t="s">
@@ -12495,7 +12521,7 @@
       <c r="L44" t="s">
         <v>724</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46384</v>
       </c>
       <c r="N44" t="s">
@@ -12539,7 +12565,7 @@
       <c r="L45" t="s">
         <v>724</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46384</v>
       </c>
       <c r="N45" t="s">
@@ -12665,7 +12691,7 @@
       <c r="L48" t="s">
         <v>724</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46384</v>
       </c>
       <c r="N48" t="s">
@@ -12709,7 +12735,7 @@
       <c r="L49" t="s">
         <v>723</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46319</v>
       </c>
       <c r="N49" t="s">
@@ -12753,7 +12779,7 @@
       <c r="L50" t="s">
         <v>723</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46319</v>
       </c>
       <c r="N50" t="s">
@@ -12797,7 +12823,7 @@
       <c r="L51" t="s">
         <v>722</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46399</v>
       </c>
       <c r="N51" t="s">
@@ -12841,7 +12867,7 @@
       <c r="L52" t="s">
         <v>722</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46399</v>
       </c>
       <c r="N52" t="s">
@@ -12885,7 +12911,7 @@
       <c r="L53" t="s">
         <v>722</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46399</v>
       </c>
       <c r="N53" t="s">
@@ -12929,7 +12955,7 @@
       <c r="L54" t="s">
         <v>724</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46384</v>
       </c>
       <c r="N54" t="s">
@@ -12973,7 +12999,7 @@
       <c r="L55" t="s">
         <v>724</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46384</v>
       </c>
       <c r="N55" t="s">
@@ -13140,7 +13166,7 @@
       <c r="L59" t="s">
         <v>724</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46384</v>
       </c>
       <c r="N59" t="s">
@@ -13266,7 +13292,7 @@
       <c r="L62" t="s">
         <v>724</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46384</v>
       </c>
       <c r="N62" t="s">
@@ -13310,7 +13336,7 @@
       <c r="L63" t="s">
         <v>724</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46384</v>
       </c>
       <c r="N63" t="s">
@@ -13354,7 +13380,7 @@
       <c r="L64" t="s">
         <v>724</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46384</v>
       </c>
       <c r="N64" t="s">
@@ -13398,7 +13424,7 @@
       <c r="L65" t="s">
         <v>724</v>
       </c>
-      <c r="M65" s="1">
+      <c r="M65" s="2">
         <v>46384</v>
       </c>
       <c r="N65" t="s">
@@ -13442,7 +13468,7 @@
       <c r="L66" t="s">
         <v>724</v>
       </c>
-      <c r="M66" s="1">
+      <c r="M66" s="2">
         <v>46384</v>
       </c>
       <c r="N66" t="s">
@@ -13486,7 +13512,7 @@
       <c r="L67" t="s">
         <v>724</v>
       </c>
-      <c r="M67" s="1">
+      <c r="M67" s="2">
         <v>46384</v>
       </c>
       <c r="N67" t="s">
@@ -13530,7 +13556,7 @@
       <c r="L68" t="s">
         <v>724</v>
       </c>
-      <c r="M68" s="1">
+      <c r="M68" s="2">
         <v>46384</v>
       </c>
       <c r="N68" t="s">
@@ -13574,7 +13600,7 @@
       <c r="L69" t="s">
         <v>724</v>
       </c>
-      <c r="M69" s="1">
+      <c r="M69" s="2">
         <v>46384</v>
       </c>
       <c r="N69" t="s">
@@ -13618,7 +13644,7 @@
       <c r="L70" t="s">
         <v>724</v>
       </c>
-      <c r="M70" s="1">
+      <c r="M70" s="2">
         <v>46384</v>
       </c>
       <c r="N70" t="s">
@@ -13662,7 +13688,7 @@
       <c r="L71" t="s">
         <v>724</v>
       </c>
-      <c r="M71" s="1">
+      <c r="M71" s="2">
         <v>46384</v>
       </c>
       <c r="N71" t="s">
@@ -13706,7 +13732,7 @@
       <c r="L72" t="s">
         <v>724</v>
       </c>
-      <c r="M72" s="1">
+      <c r="M72" s="2">
         <v>46384</v>
       </c>
       <c r="N72" t="s">
@@ -13750,7 +13776,7 @@
       <c r="L73" t="s">
         <v>724</v>
       </c>
-      <c r="M73" s="1">
+      <c r="M73" s="2">
         <v>46384</v>
       </c>
       <c r="N73" t="s">
@@ -13794,7 +13820,7 @@
       <c r="L74" t="s">
         <v>724</v>
       </c>
-      <c r="M74" s="1">
+      <c r="M74" s="2">
         <v>46384</v>
       </c>
       <c r="N74" t="s">
@@ -13838,7 +13864,7 @@
       <c r="L75" t="s">
         <v>722</v>
       </c>
-      <c r="M75" s="1">
+      <c r="M75" s="2">
         <v>46399</v>
       </c>
       <c r="N75" t="s">
@@ -13882,7 +13908,7 @@
       <c r="L76" t="s">
         <v>722</v>
       </c>
-      <c r="M76" s="1">
+      <c r="M76" s="2">
         <v>46399</v>
       </c>
       <c r="N76" t="s">
@@ -13926,7 +13952,7 @@
       <c r="L77" t="s">
         <v>724</v>
       </c>
-      <c r="M77" s="1">
+      <c r="M77" s="2">
         <v>46384</v>
       </c>
       <c r="N77" t="s">
@@ -13970,7 +13996,7 @@
       <c r="L78" t="s">
         <v>724</v>
       </c>
-      <c r="M78" s="1">
+      <c r="M78" s="2">
         <v>46384</v>
       </c>
       <c r="N78" t="s">
@@ -14014,7 +14040,7 @@
       <c r="L79" t="s">
         <v>724</v>
       </c>
-      <c r="M79" s="1">
+      <c r="M79" s="2">
         <v>46384</v>
       </c>
       <c r="N79" t="s">
@@ -14058,7 +14084,7 @@
       <c r="L80" t="s">
         <v>724</v>
       </c>
-      <c r="M80" s="1">
+      <c r="M80" s="2">
         <v>46384</v>
       </c>
       <c r="N80" t="s">
@@ -14102,7 +14128,7 @@
       <c r="L81" t="s">
         <v>724</v>
       </c>
-      <c r="M81" s="1">
+      <c r="M81" s="2">
         <v>46384</v>
       </c>
       <c r="N81" t="s">
@@ -14146,7 +14172,7 @@
       <c r="L82" t="s">
         <v>724</v>
       </c>
-      <c r="M82" s="1">
+      <c r="M82" s="2">
         <v>46384</v>
       </c>
       <c r="N82" t="s">
@@ -14190,7 +14216,7 @@
       <c r="L83" t="s">
         <v>724</v>
       </c>
-      <c r="M83" s="1">
+      <c r="M83" s="2">
         <v>46384</v>
       </c>
       <c r="N83" t="s">
@@ -14234,7 +14260,7 @@
       <c r="L84" t="s">
         <v>724</v>
       </c>
-      <c r="M84" s="1">
+      <c r="M84" s="2">
         <v>46384</v>
       </c>
       <c r="N84" t="s">
@@ -14278,7 +14304,7 @@
       <c r="L85" t="s">
         <v>724</v>
       </c>
-      <c r="M85" s="1">
+      <c r="M85" s="2">
         <v>46384</v>
       </c>
       <c r="N85" t="s">
@@ -14322,7 +14348,7 @@
       <c r="L86" t="s">
         <v>724</v>
       </c>
-      <c r="M86" s="1">
+      <c r="M86" s="2">
         <v>46384</v>
       </c>
       <c r="N86" t="s">
@@ -14366,7 +14392,7 @@
       <c r="L87" t="s">
         <v>724</v>
       </c>
-      <c r="M87" s="1">
+      <c r="M87" s="2">
         <v>46384</v>
       </c>
       <c r="N87" t="s">
@@ -14410,7 +14436,7 @@
       <c r="L88" t="s">
         <v>724</v>
       </c>
-      <c r="M88" s="1">
+      <c r="M88" s="2">
         <v>46384</v>
       </c>
       <c r="N88" t="s">
@@ -14454,7 +14480,7 @@
       <c r="L89" t="s">
         <v>724</v>
       </c>
-      <c r="M89" s="1">
+      <c r="M89" s="2">
         <v>46384</v>
       </c>
       <c r="N89" t="s">
@@ -14498,7 +14524,7 @@
       <c r="L90" t="s">
         <v>724</v>
       </c>
-      <c r="M90" s="1">
+      <c r="M90" s="2">
         <v>46384</v>
       </c>
       <c r="N90" t="s">
@@ -14583,7 +14609,7 @@
       <c r="L92" t="s">
         <v>724</v>
       </c>
-      <c r="M92" s="1">
+      <c r="M92" s="2">
         <v>46384</v>
       </c>
       <c r="N92" t="s">
@@ -14627,7 +14653,7 @@
       <c r="L93" t="s">
         <v>724</v>
       </c>
-      <c r="M93" s="1">
+      <c r="M93" s="2">
         <v>46384</v>
       </c>
       <c r="N93" t="s">
@@ -14671,7 +14697,7 @@
       <c r="L94" t="s">
         <v>724</v>
       </c>
-      <c r="M94" s="1">
+      <c r="M94" s="2">
         <v>46384</v>
       </c>
       <c r="N94" t="s">
@@ -14715,7 +14741,7 @@
       <c r="L95" t="s">
         <v>722</v>
       </c>
-      <c r="M95" s="1">
+      <c r="M95" s="2">
         <v>46399</v>
       </c>
       <c r="N95" t="s">
@@ -14759,7 +14785,7 @@
       <c r="L96" t="s">
         <v>722</v>
       </c>
-      <c r="M96" s="1">
+      <c r="M96" s="2">
         <v>46399</v>
       </c>
       <c r="N96" t="s">
@@ -14803,7 +14829,7 @@
       <c r="L97" t="s">
         <v>724</v>
       </c>
-      <c r="M97" s="1">
+      <c r="M97" s="2">
         <v>46384</v>
       </c>
       <c r="N97" t="s">
@@ -14847,7 +14873,7 @@
       <c r="L98" t="s">
         <v>724</v>
       </c>
-      <c r="M98" s="1">
+      <c r="M98" s="2">
         <v>46384</v>
       </c>
       <c r="N98" t="s">
@@ -14891,7 +14917,7 @@
       <c r="L99" t="s">
         <v>724</v>
       </c>
-      <c r="M99" s="1">
+      <c r="M99" s="2">
         <v>46384</v>
       </c>
       <c r="N99" t="s">
@@ -14935,7 +14961,7 @@
       <c r="L100" t="s">
         <v>724</v>
       </c>
-      <c r="M100" s="1">
+      <c r="M100" s="2">
         <v>46384</v>
       </c>
       <c r="N100" t="s">
@@ -14979,7 +15005,7 @@
       <c r="L101" t="s">
         <v>724</v>
       </c>
-      <c r="M101" s="1">
+      <c r="M101" s="2">
         <v>46384</v>
       </c>
       <c r="N101" t="s">
@@ -15023,7 +15049,7 @@
       <c r="L102" t="s">
         <v>724</v>
       </c>
-      <c r="M102" s="1">
+      <c r="M102" s="2">
         <v>46384</v>
       </c>
       <c r="N102" t="s">
@@ -15067,7 +15093,7 @@
       <c r="L103" t="s">
         <v>724</v>
       </c>
-      <c r="M103" s="1">
+      <c r="M103" s="2">
         <v>46384</v>
       </c>
       <c r="N103" t="s">
@@ -15111,7 +15137,7 @@
       <c r="L104" t="s">
         <v>722</v>
       </c>
-      <c r="M104" s="1">
+      <c r="M104" s="2">
         <v>46399</v>
       </c>
       <c r="N104" t="s">
@@ -15155,7 +15181,7 @@
       <c r="L105" t="s">
         <v>724</v>
       </c>
-      <c r="M105" s="1">
+      <c r="M105" s="2">
         <v>46384</v>
       </c>
       <c r="N105" t="s">
@@ -15199,7 +15225,7 @@
       <c r="L106" t="s">
         <v>722</v>
       </c>
-      <c r="M106" s="1">
+      <c r="M106" s="2">
         <v>46399</v>
       </c>
       <c r="N106" t="s">
@@ -15243,7 +15269,7 @@
       <c r="L107" t="s">
         <v>724</v>
       </c>
-      <c r="M107" s="1">
+      <c r="M107" s="2">
         <v>46384</v>
       </c>
       <c r="N107" t="s">
@@ -15287,7 +15313,7 @@
       <c r="L108" t="s">
         <v>722</v>
       </c>
-      <c r="M108" s="1">
+      <c r="M108" s="2">
         <v>46399</v>
       </c>
       <c r="N108" t="s">
@@ -15331,7 +15357,7 @@
       <c r="L109" t="s">
         <v>722</v>
       </c>
-      <c r="M109" s="1">
+      <c r="M109" s="2">
         <v>46399</v>
       </c>
       <c r="N109" t="s">
@@ -15375,7 +15401,7 @@
       <c r="L110" t="s">
         <v>724</v>
       </c>
-      <c r="M110" s="1">
+      <c r="M110" s="2">
         <v>46384</v>
       </c>
       <c r="N110" t="s">
@@ -15419,7 +15445,7 @@
       <c r="L111" t="s">
         <v>724</v>
       </c>
-      <c r="M111" s="1">
+      <c r="M111" s="2">
         <v>46384</v>
       </c>
       <c r="N111" t="s">
@@ -15463,7 +15489,7 @@
       <c r="L112" t="s">
         <v>724</v>
       </c>
-      <c r="M112" s="1">
+      <c r="M112" s="2">
         <v>46384</v>
       </c>
       <c r="N112" t="s">
@@ -15507,7 +15533,7 @@
       <c r="L113" t="s">
         <v>724</v>
       </c>
-      <c r="M113" s="1">
+      <c r="M113" s="2">
         <v>46384</v>
       </c>
       <c r="N113" t="s">
@@ -15551,7 +15577,7 @@
       <c r="L114" t="s">
         <v>724</v>
       </c>
-      <c r="M114" s="1">
+      <c r="M114" s="2">
         <v>46384</v>
       </c>
       <c r="N114" t="s">
@@ -15595,7 +15621,7 @@
       <c r="L115" t="s">
         <v>724</v>
       </c>
-      <c r="M115" s="1">
+      <c r="M115" s="2">
         <v>46384</v>
       </c>
       <c r="N115" t="s">
@@ -15639,7 +15665,7 @@
       <c r="L116" t="s">
         <v>724</v>
       </c>
-      <c r="M116" s="1">
+      <c r="M116" s="2">
         <v>46384</v>
       </c>
       <c r="N116" t="s">
@@ -15683,7 +15709,7 @@
       <c r="L117" t="s">
         <v>724</v>
       </c>
-      <c r="M117" s="1">
+      <c r="M117" s="2">
         <v>46384</v>
       </c>
       <c r="N117" t="s">
@@ -15727,7 +15753,7 @@
       <c r="L118" t="s">
         <v>724</v>
       </c>
-      <c r="M118" s="1">
+      <c r="M118" s="2">
         <v>46384</v>
       </c>
       <c r="N118" t="s">
@@ -15771,7 +15797,7 @@
       <c r="L119" t="s">
         <v>722</v>
       </c>
-      <c r="M119" s="1">
+      <c r="M119" s="2">
         <v>46399</v>
       </c>
       <c r="N119" t="s">
@@ -15815,7 +15841,7 @@
       <c r="L120" t="s">
         <v>724</v>
       </c>
-      <c r="M120" s="1">
+      <c r="M120" s="2">
         <v>46384</v>
       </c>
       <c r="N120" t="s">
@@ -15859,7 +15885,7 @@
       <c r="L121" t="s">
         <v>722</v>
       </c>
-      <c r="M121" s="1">
+      <c r="M121" s="2">
         <v>46399</v>
       </c>
       <c r="N121" t="s">
@@ -15903,7 +15929,7 @@
       <c r="L122" t="s">
         <v>722</v>
       </c>
-      <c r="M122" s="1">
+      <c r="M122" s="2">
         <v>46399</v>
       </c>
       <c r="N122" t="s">
@@ -15947,7 +15973,7 @@
       <c r="L123" t="s">
         <v>722</v>
       </c>
-      <c r="M123" s="1">
+      <c r="M123" s="2">
         <v>46399</v>
       </c>
       <c r="N123" t="s">
@@ -15991,7 +16017,7 @@
       <c r="L124" t="s">
         <v>722</v>
       </c>
-      <c r="M124" s="1">
+      <c r="M124" s="2">
         <v>46399</v>
       </c>
       <c r="N124" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (15/10/2026 12:35)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3126" uniqueCount="727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3126" uniqueCount="726">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -2183,13 +2183,10 @@
     <t>Selecionada em Plano</t>
   </si>
   <si>
-    <t>Análise do Pedido</t>
+    <t>Validada</t>
   </si>
   <si>
     <t>Mapa Gerado</t>
-  </si>
-  <si>
-    <t>Validada</t>
   </si>
   <si>
     <t>Em Discrepância</t>
@@ -2205,16 +2202,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2230,7 +2219,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2238,30 +2227,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2561,55 +2532,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2653,7 +2624,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2697,7 +2668,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2741,7 +2712,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2867,7 +2838,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2911,7 +2882,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2955,7 +2926,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -3002,7 +2973,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3125,7 +3096,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -3169,7 +3140,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3213,7 +3184,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3257,7 +3228,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3304,7 +3275,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3348,7 +3319,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3474,7 +3445,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3518,7 +3489,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3603,7 +3574,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3650,7 +3621,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3697,7 +3668,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3741,7 +3712,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3785,7 +3756,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3870,7 +3841,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3955,7 +3926,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -4002,7 +3973,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4046,7 +4017,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4090,7 +4061,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4175,7 +4146,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4219,7 +4190,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4263,7 +4234,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4348,7 +4319,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4392,7 +4363,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4436,7 +4407,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4480,7 +4451,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4647,7 +4618,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4691,7 +4662,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4735,7 +4706,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4779,7 +4750,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4826,7 +4797,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4870,7 +4841,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4952,7 +4923,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4996,7 +4967,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5084,7 +5055,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5128,7 +5099,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5175,7 +5146,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5219,7 +5190,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -5263,7 +5234,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5307,7 +5278,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5351,7 +5322,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5398,7 +5369,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5442,7 +5413,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5489,7 +5460,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5533,7 +5504,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5580,7 +5551,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5668,7 +5639,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5712,7 +5683,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5756,7 +5727,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5800,7 +5771,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5844,7 +5815,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5888,7 +5859,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5973,7 +5944,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6017,7 +5988,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -6061,7 +6032,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -6105,7 +6076,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -6149,7 +6120,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -6193,7 +6164,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6237,7 +6208,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6281,7 +6252,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6328,7 +6299,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6372,7 +6343,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6416,7 +6387,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6460,7 +6431,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6504,7 +6475,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6548,7 +6519,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6592,7 +6563,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6636,7 +6607,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6680,7 +6651,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6768,7 +6739,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6812,7 +6783,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6938,7 +6909,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6982,7 +6953,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7026,7 +6997,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7070,7 +7041,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7152,7 +7123,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7196,7 +7167,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7243,7 +7214,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7287,7 +7258,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7413,7 +7384,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7457,7 +7428,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7542,7 +7513,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7586,7 +7557,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7630,7 +7601,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7674,7 +7645,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7718,7 +7689,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7762,7 +7733,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7806,7 +7777,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7850,7 +7821,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7935,7 +7906,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8102,7 +8073,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8146,7 +8117,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8190,7 +8161,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8234,7 +8205,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8278,7 +8249,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8322,7 +8293,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8366,7 +8337,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8451,7 +8422,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8495,7 +8466,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8580,7 +8551,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8706,7 +8677,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8750,7 +8721,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8835,7 +8806,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8879,7 +8850,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8923,7 +8894,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8967,7 +8938,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -9011,7 +8982,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -9055,7 +9026,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9099,7 +9070,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9143,7 +9114,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9228,7 +9199,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9395,7 +9366,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9439,7 +9410,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9483,7 +9454,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9527,7 +9498,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9612,7 +9583,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9656,7 +9627,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9700,7 +9671,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9744,7 +9715,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9788,7 +9759,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9832,7 +9803,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9876,7 +9847,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9920,7 +9891,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9964,7 +9935,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10008,7 +9979,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10052,7 +10023,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -10096,7 +10067,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10140,7 +10111,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10184,7 +10155,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -10228,7 +10199,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10272,7 +10243,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10316,7 +10287,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10360,7 +10331,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10404,7 +10375,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10448,7 +10419,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10492,7 +10463,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10577,7 +10548,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10662,7 +10633,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10677,55 +10648,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11086,19 +11057,19 @@
         <v>721</v>
       </c>
       <c r="J10" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K10" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L10" t="s">
-        <v>724</v>
-      </c>
-      <c r="M10" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M10" s="1">
+        <v>46385</v>
       </c>
       <c r="N10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -11130,19 +11101,19 @@
         <v>721</v>
       </c>
       <c r="J11" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K11" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L11" t="s">
-        <v>724</v>
-      </c>
-      <c r="M11" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M11" s="1">
+        <v>46385</v>
       </c>
       <c r="N11" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -11338,19 +11309,19 @@
         <v>721</v>
       </c>
       <c r="J16" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K16" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L16" t="s">
-        <v>724</v>
-      </c>
-      <c r="M16" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M16" s="1">
+        <v>46385</v>
       </c>
       <c r="N16" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -11464,19 +11435,19 @@
         <v>721</v>
       </c>
       <c r="J19" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K19" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L19" t="s">
-        <v>724</v>
-      </c>
-      <c r="M19" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M19" s="1">
+        <v>46385</v>
       </c>
       <c r="N19" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11508,19 +11479,19 @@
         <v>721</v>
       </c>
       <c r="J20" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K20" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L20" t="s">
-        <v>724</v>
-      </c>
-      <c r="M20" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M20" s="1">
+        <v>46385</v>
       </c>
       <c r="N20" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11560,11 +11531,11 @@
       <c r="L21" t="s">
         <v>722</v>
       </c>
-      <c r="M21" s="2">
-        <v>46399</v>
+      <c r="M21" s="1">
+        <v>46385</v>
       </c>
       <c r="N21" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11719,19 +11690,19 @@
         <v>721</v>
       </c>
       <c r="J25" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K25" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L25" t="s">
-        <v>724</v>
-      </c>
-      <c r="M25" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M25" s="1">
+        <v>46385</v>
       </c>
       <c r="N25" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11853,11 +11824,11 @@
       <c r="L28" t="s">
         <v>722</v>
       </c>
-      <c r="M28" s="2">
-        <v>46399</v>
+      <c r="M28" s="1">
+        <v>46385</v>
       </c>
       <c r="N28" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11938,11 +11909,11 @@
       <c r="L30" t="s">
         <v>722</v>
       </c>
-      <c r="M30" s="2">
-        <v>46399</v>
+      <c r="M30" s="1">
+        <v>46385</v>
       </c>
       <c r="N30" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -12392,11 +12363,11 @@
       <c r="L41" t="s">
         <v>722</v>
       </c>
-      <c r="M41" s="2">
-        <v>46399</v>
+      <c r="M41" s="1">
+        <v>46385</v>
       </c>
       <c r="N41" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -12469,19 +12440,19 @@
         <v>721</v>
       </c>
       <c r="J43" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K43" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L43" t="s">
-        <v>724</v>
-      </c>
-      <c r="M43" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M43" s="1">
+        <v>46385</v>
       </c>
       <c r="N43" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12513,19 +12484,19 @@
         <v>721</v>
       </c>
       <c r="J44" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K44" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L44" t="s">
-        <v>724</v>
-      </c>
-      <c r="M44" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M44" s="1">
+        <v>46385</v>
       </c>
       <c r="N44" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12557,19 +12528,19 @@
         <v>721</v>
       </c>
       <c r="J45" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K45" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L45" t="s">
-        <v>724</v>
-      </c>
-      <c r="M45" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M45" s="1">
+        <v>46385</v>
       </c>
       <c r="N45" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12683,19 +12654,19 @@
         <v>721</v>
       </c>
       <c r="J48" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K48" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L48" t="s">
-        <v>724</v>
-      </c>
-      <c r="M48" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M48" s="1">
+        <v>46385</v>
       </c>
       <c r="N48" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12735,11 +12706,11 @@
       <c r="L49" t="s">
         <v>723</v>
       </c>
-      <c r="M49" s="2">
-        <v>46319</v>
+      <c r="M49" s="1">
+        <v>46320</v>
       </c>
       <c r="N49" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12779,11 +12750,11 @@
       <c r="L50" t="s">
         <v>723</v>
       </c>
-      <c r="M50" s="2">
-        <v>46319</v>
+      <c r="M50" s="1">
+        <v>46320</v>
       </c>
       <c r="N50" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12823,11 +12794,11 @@
       <c r="L51" t="s">
         <v>722</v>
       </c>
-      <c r="M51" s="2">
-        <v>46399</v>
+      <c r="M51" s="1">
+        <v>46385</v>
       </c>
       <c r="N51" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12867,11 +12838,11 @@
       <c r="L52" t="s">
         <v>722</v>
       </c>
-      <c r="M52" s="2">
-        <v>46399</v>
+      <c r="M52" s="1">
+        <v>46385</v>
       </c>
       <c r="N52" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12911,11 +12882,11 @@
       <c r="L53" t="s">
         <v>722</v>
       </c>
-      <c r="M53" s="2">
-        <v>46399</v>
+      <c r="M53" s="1">
+        <v>46385</v>
       </c>
       <c r="N53" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12947,19 +12918,19 @@
         <v>721</v>
       </c>
       <c r="J54" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K54" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L54" t="s">
-        <v>724</v>
-      </c>
-      <c r="M54" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M54" s="1">
+        <v>46385</v>
       </c>
       <c r="N54" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12988,22 +12959,22 @@
         <v>84382.42999999999</v>
       </c>
       <c r="I55" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="J55" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K55" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L55" t="s">
-        <v>724</v>
-      </c>
-      <c r="M55" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M55" s="1">
+        <v>46385</v>
       </c>
       <c r="N55" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -13158,19 +13129,19 @@
         <v>721</v>
       </c>
       <c r="J59" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K59" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L59" t="s">
-        <v>724</v>
-      </c>
-      <c r="M59" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M59" s="1">
+        <v>46385</v>
       </c>
       <c r="N59" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -13284,19 +13255,19 @@
         <v>721</v>
       </c>
       <c r="J62" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K62" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L62" t="s">
-        <v>724</v>
-      </c>
-      <c r="M62" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M62" s="1">
+        <v>46385</v>
       </c>
       <c r="N62" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="63" spans="1:14">
@@ -13328,19 +13299,19 @@
         <v>721</v>
       </c>
       <c r="J63" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K63" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L63" t="s">
-        <v>724</v>
-      </c>
-      <c r="M63" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M63" s="1">
+        <v>46385</v>
       </c>
       <c r="N63" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="64" spans="1:14">
@@ -13372,19 +13343,19 @@
         <v>721</v>
       </c>
       <c r="J64" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K64" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L64" t="s">
-        <v>724</v>
-      </c>
-      <c r="M64" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M64" s="1">
+        <v>46385</v>
       </c>
       <c r="N64" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="65" spans="1:14">
@@ -13416,19 +13387,19 @@
         <v>721</v>
       </c>
       <c r="J65" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K65" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L65" t="s">
-        <v>724</v>
-      </c>
-      <c r="M65" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M65" s="1">
+        <v>46385</v>
       </c>
       <c r="N65" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="66" spans="1:14">
@@ -13460,19 +13431,19 @@
         <v>721</v>
       </c>
       <c r="J66" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K66" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L66" t="s">
-        <v>724</v>
-      </c>
-      <c r="M66" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M66" s="1">
+        <v>46385</v>
       </c>
       <c r="N66" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="67" spans="1:14">
@@ -13504,19 +13475,19 @@
         <v>721</v>
       </c>
       <c r="J67" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K67" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L67" t="s">
-        <v>724</v>
-      </c>
-      <c r="M67" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M67" s="1">
+        <v>46385</v>
       </c>
       <c r="N67" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="68" spans="1:14">
@@ -13548,19 +13519,19 @@
         <v>721</v>
       </c>
       <c r="J68" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K68" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L68" t="s">
-        <v>724</v>
-      </c>
-      <c r="M68" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M68" s="1">
+        <v>46385</v>
       </c>
       <c r="N68" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="69" spans="1:14">
@@ -13592,19 +13563,19 @@
         <v>721</v>
       </c>
       <c r="J69" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K69" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L69" t="s">
-        <v>724</v>
-      </c>
-      <c r="M69" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M69" s="1">
+        <v>46385</v>
       </c>
       <c r="N69" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="70" spans="1:14">
@@ -13636,19 +13607,19 @@
         <v>721</v>
       </c>
       <c r="J70" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K70" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L70" t="s">
-        <v>724</v>
-      </c>
-      <c r="M70" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M70" s="1">
+        <v>46385</v>
       </c>
       <c r="N70" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="71" spans="1:14">
@@ -13680,19 +13651,19 @@
         <v>721</v>
       </c>
       <c r="J71" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K71" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L71" t="s">
-        <v>724</v>
-      </c>
-      <c r="M71" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M71" s="1">
+        <v>46385</v>
       </c>
       <c r="N71" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="72" spans="1:14">
@@ -13724,19 +13695,19 @@
         <v>721</v>
       </c>
       <c r="J72" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K72" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L72" t="s">
-        <v>724</v>
-      </c>
-      <c r="M72" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M72" s="1">
+        <v>46385</v>
       </c>
       <c r="N72" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="73" spans="1:14">
@@ -13768,19 +13739,19 @@
         <v>721</v>
       </c>
       <c r="J73" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K73" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L73" t="s">
-        <v>724</v>
-      </c>
-      <c r="M73" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M73" s="1">
+        <v>46385</v>
       </c>
       <c r="N73" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="74" spans="1:14">
@@ -13812,19 +13783,19 @@
         <v>721</v>
       </c>
       <c r="J74" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K74" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L74" t="s">
-        <v>724</v>
-      </c>
-      <c r="M74" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M74" s="1">
+        <v>46385</v>
       </c>
       <c r="N74" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="75" spans="1:14">
@@ -13864,11 +13835,11 @@
       <c r="L75" t="s">
         <v>722</v>
       </c>
-      <c r="M75" s="2">
-        <v>46399</v>
+      <c r="M75" s="1">
+        <v>46385</v>
       </c>
       <c r="N75" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="76" spans="1:14">
@@ -13908,11 +13879,11 @@
       <c r="L76" t="s">
         <v>722</v>
       </c>
-      <c r="M76" s="2">
-        <v>46399</v>
+      <c r="M76" s="1">
+        <v>46385</v>
       </c>
       <c r="N76" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="77" spans="1:14">
@@ -13944,19 +13915,19 @@
         <v>721</v>
       </c>
       <c r="J77" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K77" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L77" t="s">
-        <v>724</v>
-      </c>
-      <c r="M77" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M77" s="1">
+        <v>46385</v>
       </c>
       <c r="N77" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="78" spans="1:14">
@@ -13988,19 +13959,19 @@
         <v>721</v>
       </c>
       <c r="J78" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K78" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L78" t="s">
-        <v>724</v>
-      </c>
-      <c r="M78" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M78" s="1">
+        <v>46385</v>
       </c>
       <c r="N78" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="79" spans="1:14">
@@ -14032,19 +14003,19 @@
         <v>721</v>
       </c>
       <c r="J79" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K79" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L79" t="s">
-        <v>724</v>
-      </c>
-      <c r="M79" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M79" s="1">
+        <v>46385</v>
       </c>
       <c r="N79" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="80" spans="1:14">
@@ -14076,19 +14047,19 @@
         <v>721</v>
       </c>
       <c r="J80" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K80" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L80" t="s">
-        <v>724</v>
-      </c>
-      <c r="M80" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M80" s="1">
+        <v>46385</v>
       </c>
       <c r="N80" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="81" spans="1:14">
@@ -14117,22 +14088,22 @@
         <v>1592.82</v>
       </c>
       <c r="I81" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="J81" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K81" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L81" t="s">
-        <v>724</v>
-      </c>
-      <c r="M81" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M81" s="1">
+        <v>46385</v>
       </c>
       <c r="N81" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="82" spans="1:14">
@@ -14164,19 +14135,19 @@
         <v>721</v>
       </c>
       <c r="J82" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K82" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L82" t="s">
-        <v>724</v>
-      </c>
-      <c r="M82" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M82" s="1">
+        <v>46385</v>
       </c>
       <c r="N82" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="83" spans="1:14">
@@ -14208,19 +14179,19 @@
         <v>721</v>
       </c>
       <c r="J83" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K83" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L83" t="s">
-        <v>724</v>
-      </c>
-      <c r="M83" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M83" s="1">
+        <v>46385</v>
       </c>
       <c r="N83" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="84" spans="1:14">
@@ -14252,19 +14223,19 @@
         <v>721</v>
       </c>
       <c r="J84" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K84" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L84" t="s">
-        <v>724</v>
-      </c>
-      <c r="M84" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M84" s="1">
+        <v>46385</v>
       </c>
       <c r="N84" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="85" spans="1:14">
@@ -14296,19 +14267,19 @@
         <v>721</v>
       </c>
       <c r="J85" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K85" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L85" t="s">
-        <v>724</v>
-      </c>
-      <c r="M85" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M85" s="1">
+        <v>46385</v>
       </c>
       <c r="N85" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="86" spans="1:14">
@@ -14340,19 +14311,19 @@
         <v>721</v>
       </c>
       <c r="J86" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K86" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L86" t="s">
-        <v>724</v>
-      </c>
-      <c r="M86" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M86" s="1">
+        <v>46385</v>
       </c>
       <c r="N86" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="87" spans="1:14">
@@ -14384,19 +14355,19 @@
         <v>721</v>
       </c>
       <c r="J87" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K87" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L87" t="s">
-        <v>724</v>
-      </c>
-      <c r="M87" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M87" s="1">
+        <v>46385</v>
       </c>
       <c r="N87" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="88" spans="1:14">
@@ -14425,22 +14396,22 @@
         <v>2360</v>
       </c>
       <c r="I88" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="J88" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K88" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L88" t="s">
-        <v>724</v>
-      </c>
-      <c r="M88" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M88" s="1">
+        <v>46385</v>
       </c>
       <c r="N88" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="89" spans="1:14">
@@ -14472,19 +14443,19 @@
         <v>721</v>
       </c>
       <c r="J89" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K89" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L89" t="s">
-        <v>724</v>
-      </c>
-      <c r="M89" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M89" s="1">
+        <v>46385</v>
       </c>
       <c r="N89" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="90" spans="1:14">
@@ -14513,22 +14484,22 @@
         <v>265</v>
       </c>
       <c r="I90" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="J90" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K90" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L90" t="s">
-        <v>724</v>
-      </c>
-      <c r="M90" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M90" s="1">
+        <v>46385</v>
       </c>
       <c r="N90" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="91" spans="1:14">
@@ -14557,16 +14528,16 @@
         <v>794</v>
       </c>
       <c r="I91" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="J91" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K91" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L91" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="N91" t="s">
         <v>395</v>
@@ -14601,19 +14572,19 @@
         <v>721</v>
       </c>
       <c r="J92" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K92" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L92" t="s">
-        <v>724</v>
-      </c>
-      <c r="M92" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M92" s="1">
+        <v>46385</v>
       </c>
       <c r="N92" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="93" spans="1:14">
@@ -14642,22 +14613,22 @@
         <v>735.79</v>
       </c>
       <c r="I93" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="J93" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K93" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L93" t="s">
-        <v>724</v>
-      </c>
-      <c r="M93" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M93" s="1">
+        <v>46385</v>
       </c>
       <c r="N93" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="94" spans="1:14">
@@ -14686,22 +14657,22 @@
         <v>7431.24</v>
       </c>
       <c r="I94" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="J94" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K94" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L94" t="s">
-        <v>724</v>
-      </c>
-      <c r="M94" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M94" s="1">
+        <v>46385</v>
       </c>
       <c r="N94" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="95" spans="1:14">
@@ -14741,11 +14712,11 @@
       <c r="L95" t="s">
         <v>722</v>
       </c>
-      <c r="M95" s="2">
-        <v>46399</v>
+      <c r="M95" s="1">
+        <v>46385</v>
       </c>
       <c r="N95" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="96" spans="1:14">
@@ -14785,11 +14756,11 @@
       <c r="L96" t="s">
         <v>722</v>
       </c>
-      <c r="M96" s="2">
-        <v>46399</v>
+      <c r="M96" s="1">
+        <v>46385</v>
       </c>
       <c r="N96" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="97" spans="1:14">
@@ -14821,19 +14792,19 @@
         <v>721</v>
       </c>
       <c r="J97" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K97" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L97" t="s">
-        <v>724</v>
-      </c>
-      <c r="M97" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M97" s="1">
+        <v>46385</v>
       </c>
       <c r="N97" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="98" spans="1:14">
@@ -14865,19 +14836,19 @@
         <v>721</v>
       </c>
       <c r="J98" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K98" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L98" t="s">
-        <v>724</v>
-      </c>
-      <c r="M98" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M98" s="1">
+        <v>46385</v>
       </c>
       <c r="N98" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="99" spans="1:14">
@@ -14909,19 +14880,19 @@
         <v>721</v>
       </c>
       <c r="J99" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K99" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L99" t="s">
-        <v>724</v>
-      </c>
-      <c r="M99" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M99" s="1">
+        <v>46385</v>
       </c>
       <c r="N99" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="100" spans="1:14">
@@ -14950,22 +14921,22 @@
         <v>1768.41</v>
       </c>
       <c r="I100" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="J100" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K100" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L100" t="s">
-        <v>724</v>
-      </c>
-      <c r="M100" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M100" s="1">
+        <v>46385</v>
       </c>
       <c r="N100" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="101" spans="1:14">
@@ -14997,19 +14968,19 @@
         <v>721</v>
       </c>
       <c r="J101" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K101" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L101" t="s">
-        <v>724</v>
-      </c>
-      <c r="M101" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M101" s="1">
+        <v>46385</v>
       </c>
       <c r="N101" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="102" spans="1:14">
@@ -15041,19 +15012,19 @@
         <v>721</v>
       </c>
       <c r="J102" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K102" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L102" t="s">
-        <v>724</v>
-      </c>
-      <c r="M102" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M102" s="1">
+        <v>46385</v>
       </c>
       <c r="N102" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="103" spans="1:14">
@@ -15082,22 +15053,22 @@
         <v>7375.36</v>
       </c>
       <c r="I103" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="J103" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K103" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L103" t="s">
-        <v>724</v>
-      </c>
-      <c r="M103" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M103" s="1">
+        <v>46385</v>
       </c>
       <c r="N103" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="104" spans="1:14">
@@ -15137,11 +15108,11 @@
       <c r="L104" t="s">
         <v>722</v>
       </c>
-      <c r="M104" s="2">
-        <v>46399</v>
+      <c r="M104" s="1">
+        <v>46385</v>
       </c>
       <c r="N104" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="105" spans="1:14">
@@ -15170,22 +15141,22 @@
         <v>1578.63</v>
       </c>
       <c r="I105" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="J105" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K105" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L105" t="s">
-        <v>724</v>
-      </c>
-      <c r="M105" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M105" s="1">
+        <v>46385</v>
       </c>
       <c r="N105" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="106" spans="1:14">
@@ -15225,11 +15196,11 @@
       <c r="L106" t="s">
         <v>722</v>
       </c>
-      <c r="M106" s="2">
-        <v>46399</v>
+      <c r="M106" s="1">
+        <v>46385</v>
       </c>
       <c r="N106" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="107" spans="1:14">
@@ -15258,22 +15229,22 @@
         <v>3100.94</v>
       </c>
       <c r="I107" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="J107" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K107" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L107" t="s">
-        <v>724</v>
-      </c>
-      <c r="M107" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M107" s="1">
+        <v>46385</v>
       </c>
       <c r="N107" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="108" spans="1:14">
@@ -15313,11 +15284,11 @@
       <c r="L108" t="s">
         <v>722</v>
       </c>
-      <c r="M108" s="2">
-        <v>46399</v>
+      <c r="M108" s="1">
+        <v>46385</v>
       </c>
       <c r="N108" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="109" spans="1:14">
@@ -15357,11 +15328,11 @@
       <c r="L109" t="s">
         <v>722</v>
       </c>
-      <c r="M109" s="2">
-        <v>46399</v>
+      <c r="M109" s="1">
+        <v>46385</v>
       </c>
       <c r="N109" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="110" spans="1:14">
@@ -15393,19 +15364,19 @@
         <v>721</v>
       </c>
       <c r="J110" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K110" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L110" t="s">
-        <v>724</v>
-      </c>
-      <c r="M110" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M110" s="1">
+        <v>46385</v>
       </c>
       <c r="N110" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="111" spans="1:14">
@@ -15437,19 +15408,19 @@
         <v>721</v>
       </c>
       <c r="J111" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K111" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L111" t="s">
-        <v>724</v>
-      </c>
-      <c r="M111" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M111" s="1">
+        <v>46385</v>
       </c>
       <c r="N111" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="112" spans="1:14">
@@ -15481,19 +15452,19 @@
         <v>721</v>
       </c>
       <c r="J112" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K112" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L112" t="s">
-        <v>724</v>
-      </c>
-      <c r="M112" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M112" s="1">
+        <v>46385</v>
       </c>
       <c r="N112" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="113" spans="1:14">
@@ -15525,19 +15496,19 @@
         <v>721</v>
       </c>
       <c r="J113" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K113" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L113" t="s">
-        <v>724</v>
-      </c>
-      <c r="M113" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M113" s="1">
+        <v>46385</v>
       </c>
       <c r="N113" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="114" spans="1:14">
@@ -15569,19 +15540,19 @@
         <v>721</v>
       </c>
       <c r="J114" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K114" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L114" t="s">
-        <v>724</v>
-      </c>
-      <c r="M114" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M114" s="1">
+        <v>46385</v>
       </c>
       <c r="N114" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="115" spans="1:14">
@@ -15613,19 +15584,19 @@
         <v>721</v>
       </c>
       <c r="J115" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K115" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L115" t="s">
-        <v>724</v>
-      </c>
-      <c r="M115" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M115" s="1">
+        <v>46385</v>
       </c>
       <c r="N115" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="116" spans="1:14">
@@ -15657,19 +15628,19 @@
         <v>721</v>
       </c>
       <c r="J116" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K116" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L116" t="s">
-        <v>724</v>
-      </c>
-      <c r="M116" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M116" s="1">
+        <v>46385</v>
       </c>
       <c r="N116" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="117" spans="1:14">
@@ -15701,19 +15672,19 @@
         <v>721</v>
       </c>
       <c r="J117" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K117" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L117" t="s">
-        <v>724</v>
-      </c>
-      <c r="M117" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M117" s="1">
+        <v>46385</v>
       </c>
       <c r="N117" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="118" spans="1:14">
@@ -15745,19 +15716,19 @@
         <v>721</v>
       </c>
       <c r="J118" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K118" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L118" t="s">
-        <v>724</v>
-      </c>
-      <c r="M118" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M118" s="1">
+        <v>46385</v>
       </c>
       <c r="N118" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="119" spans="1:14">
@@ -15797,11 +15768,11 @@
       <c r="L119" t="s">
         <v>722</v>
       </c>
-      <c r="M119" s="2">
-        <v>46399</v>
+      <c r="M119" s="1">
+        <v>46385</v>
       </c>
       <c r="N119" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="120" spans="1:14">
@@ -15833,19 +15804,19 @@
         <v>721</v>
       </c>
       <c r="J120" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K120" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="L120" t="s">
-        <v>724</v>
-      </c>
-      <c r="M120" s="2">
-        <v>46384</v>
+        <v>722</v>
+      </c>
+      <c r="M120" s="1">
+        <v>46385</v>
       </c>
       <c r="N120" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="121" spans="1:14">
@@ -15885,11 +15856,11 @@
       <c r="L121" t="s">
         <v>722</v>
       </c>
-      <c r="M121" s="2">
-        <v>46399</v>
+      <c r="M121" s="1">
+        <v>46385</v>
       </c>
       <c r="N121" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="122" spans="1:14">
@@ -15929,11 +15900,11 @@
       <c r="L122" t="s">
         <v>722</v>
       </c>
-      <c r="M122" s="2">
-        <v>46399</v>
+      <c r="M122" s="1">
+        <v>46385</v>
       </c>
       <c r="N122" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="123" spans="1:14">
@@ -15973,11 +15944,11 @@
       <c r="L123" t="s">
         <v>722</v>
       </c>
-      <c r="M123" s="2">
-        <v>46399</v>
+      <c r="M123" s="1">
+        <v>46385</v>
       </c>
       <c r="N123" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="124" spans="1:14">
@@ -16017,11 +15988,11 @@
       <c r="L124" t="s">
         <v>722</v>
       </c>
-      <c r="M124" s="2">
-        <v>46399</v>
+      <c r="M124" s="1">
+        <v>46385</v>
       </c>
       <c r="N124" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (16/10/2026 12:03)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2202,8 +2202,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2219,7 +2227,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2227,12 +2235,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2532,55 +2558,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2624,7 +2650,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2668,7 +2694,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2712,7 +2738,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2838,7 +2864,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2882,7 +2908,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2926,7 +2952,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2973,7 +2999,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3096,7 +3122,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -3140,7 +3166,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3184,7 +3210,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3228,7 +3254,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3275,7 +3301,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3319,7 +3345,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3445,7 +3471,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3489,7 +3515,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3574,7 +3600,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3621,7 +3647,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3668,7 +3694,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3712,7 +3738,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3756,7 +3782,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3841,7 +3867,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3926,7 +3952,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3973,7 +3999,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4017,7 +4043,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4061,7 +4087,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4146,7 +4172,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4190,7 +4216,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4234,7 +4260,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4319,7 +4345,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4363,7 +4389,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4407,7 +4433,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4451,7 +4477,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4618,7 +4644,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4662,7 +4688,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4706,7 +4732,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4750,7 +4776,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4797,7 +4823,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4841,7 +4867,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4923,7 +4949,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4967,7 +4993,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5055,7 +5081,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5099,7 +5125,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5146,7 +5172,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5190,7 +5216,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -5234,7 +5260,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5278,7 +5304,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5322,7 +5348,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5369,7 +5395,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5413,7 +5439,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5460,7 +5486,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5504,7 +5530,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5551,7 +5577,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5639,7 +5665,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5683,7 +5709,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5727,7 +5753,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5771,7 +5797,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5815,7 +5841,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5859,7 +5885,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5944,7 +5970,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5988,7 +6014,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -6032,7 +6058,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -6076,7 +6102,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -6120,7 +6146,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -6164,7 +6190,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6208,7 +6234,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6252,7 +6278,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6299,7 +6325,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6343,7 +6369,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6387,7 +6413,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6431,7 +6457,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6475,7 +6501,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6519,7 +6545,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6563,7 +6589,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6607,7 +6633,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6651,7 +6677,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6739,7 +6765,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6783,7 +6809,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6909,7 +6935,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6953,7 +6979,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6997,7 +7023,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7041,7 +7067,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7123,7 +7149,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7167,7 +7193,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7214,7 +7240,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7258,7 +7284,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7384,7 +7410,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7428,7 +7454,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7513,7 +7539,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7557,7 +7583,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7601,7 +7627,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7645,7 +7671,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7689,7 +7715,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7733,7 +7759,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7777,7 +7803,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7821,7 +7847,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7906,7 +7932,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8073,7 +8099,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8117,7 +8143,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8161,7 +8187,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8205,7 +8231,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8249,7 +8275,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8293,7 +8319,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8337,7 +8363,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8422,7 +8448,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8466,7 +8492,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8551,7 +8577,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8677,7 +8703,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8721,7 +8747,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8806,7 +8832,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8850,7 +8876,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8894,7 +8920,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8938,7 +8964,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8982,7 +9008,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -9026,7 +9052,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9070,7 +9096,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9114,7 +9140,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9199,7 +9225,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9366,7 +9392,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9410,7 +9436,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9454,7 +9480,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9498,7 +9524,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9583,7 +9609,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9627,7 +9653,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9671,7 +9697,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9715,7 +9741,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9759,7 +9785,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9803,7 +9829,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9847,7 +9873,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9891,7 +9917,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9935,7 +9961,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9979,7 +10005,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10023,7 +10049,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -10067,7 +10093,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10111,7 +10137,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10155,7 +10181,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -10199,7 +10225,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10243,7 +10269,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10287,7 +10313,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10331,7 +10357,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10375,7 +10401,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10419,7 +10445,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10463,7 +10489,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10548,7 +10574,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10633,7 +10659,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10648,55 +10674,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11065,8 +11091,8 @@
       <c r="L10" t="s">
         <v>722</v>
       </c>
-      <c r="M10" s="1">
-        <v>46385</v>
+      <c r="M10" s="2">
+        <v>46386</v>
       </c>
       <c r="N10" t="s">
         <v>725</v>
@@ -11109,8 +11135,8 @@
       <c r="L11" t="s">
         <v>722</v>
       </c>
-      <c r="M11" s="1">
-        <v>46385</v>
+      <c r="M11" s="2">
+        <v>46386</v>
       </c>
       <c r="N11" t="s">
         <v>725</v>
@@ -11317,8 +11343,8 @@
       <c r="L16" t="s">
         <v>722</v>
       </c>
-      <c r="M16" s="1">
-        <v>46385</v>
+      <c r="M16" s="2">
+        <v>46386</v>
       </c>
       <c r="N16" t="s">
         <v>725</v>
@@ -11443,8 +11469,8 @@
       <c r="L19" t="s">
         <v>722</v>
       </c>
-      <c r="M19" s="1">
-        <v>46385</v>
+      <c r="M19" s="2">
+        <v>46386</v>
       </c>
       <c r="N19" t="s">
         <v>725</v>
@@ -11487,8 +11513,8 @@
       <c r="L20" t="s">
         <v>722</v>
       </c>
-      <c r="M20" s="1">
-        <v>46385</v>
+      <c r="M20" s="2">
+        <v>46386</v>
       </c>
       <c r="N20" t="s">
         <v>725</v>
@@ -11531,8 +11557,8 @@
       <c r="L21" t="s">
         <v>722</v>
       </c>
-      <c r="M21" s="1">
-        <v>46385</v>
+      <c r="M21" s="2">
+        <v>46386</v>
       </c>
       <c r="N21" t="s">
         <v>725</v>
@@ -11698,8 +11724,8 @@
       <c r="L25" t="s">
         <v>722</v>
       </c>
-      <c r="M25" s="1">
-        <v>46385</v>
+      <c r="M25" s="2">
+        <v>46386</v>
       </c>
       <c r="N25" t="s">
         <v>725</v>
@@ -11824,8 +11850,8 @@
       <c r="L28" t="s">
         <v>722</v>
       </c>
-      <c r="M28" s="1">
-        <v>46385</v>
+      <c r="M28" s="2">
+        <v>46386</v>
       </c>
       <c r="N28" t="s">
         <v>725</v>
@@ -11909,8 +11935,8 @@
       <c r="L30" t="s">
         <v>722</v>
       </c>
-      <c r="M30" s="1">
-        <v>46385</v>
+      <c r="M30" s="2">
+        <v>46386</v>
       </c>
       <c r="N30" t="s">
         <v>725</v>
@@ -12363,8 +12389,8 @@
       <c r="L41" t="s">
         <v>722</v>
       </c>
-      <c r="M41" s="1">
-        <v>46385</v>
+      <c r="M41" s="2">
+        <v>46386</v>
       </c>
       <c r="N41" t="s">
         <v>725</v>
@@ -12448,8 +12474,8 @@
       <c r="L43" t="s">
         <v>722</v>
       </c>
-      <c r="M43" s="1">
-        <v>46385</v>
+      <c r="M43" s="2">
+        <v>46386</v>
       </c>
       <c r="N43" t="s">
         <v>725</v>
@@ -12492,8 +12518,8 @@
       <c r="L44" t="s">
         <v>722</v>
       </c>
-      <c r="M44" s="1">
-        <v>46385</v>
+      <c r="M44" s="2">
+        <v>46386</v>
       </c>
       <c r="N44" t="s">
         <v>725</v>
@@ -12536,8 +12562,8 @@
       <c r="L45" t="s">
         <v>722</v>
       </c>
-      <c r="M45" s="1">
-        <v>46385</v>
+      <c r="M45" s="2">
+        <v>46386</v>
       </c>
       <c r="N45" t="s">
         <v>725</v>
@@ -12662,8 +12688,8 @@
       <c r="L48" t="s">
         <v>722</v>
       </c>
-      <c r="M48" s="1">
-        <v>46385</v>
+      <c r="M48" s="2">
+        <v>46386</v>
       </c>
       <c r="N48" t="s">
         <v>725</v>
@@ -12706,8 +12732,8 @@
       <c r="L49" t="s">
         <v>723</v>
       </c>
-      <c r="M49" s="1">
-        <v>46320</v>
+      <c r="M49" s="2">
+        <v>46321</v>
       </c>
       <c r="N49" t="s">
         <v>725</v>
@@ -12750,8 +12776,8 @@
       <c r="L50" t="s">
         <v>723</v>
       </c>
-      <c r="M50" s="1">
-        <v>46320</v>
+      <c r="M50" s="2">
+        <v>46321</v>
       </c>
       <c r="N50" t="s">
         <v>725</v>
@@ -12794,8 +12820,8 @@
       <c r="L51" t="s">
         <v>722</v>
       </c>
-      <c r="M51" s="1">
-        <v>46385</v>
+      <c r="M51" s="2">
+        <v>46386</v>
       </c>
       <c r="N51" t="s">
         <v>725</v>
@@ -12838,8 +12864,8 @@
       <c r="L52" t="s">
         <v>722</v>
       </c>
-      <c r="M52" s="1">
-        <v>46385</v>
+      <c r="M52" s="2">
+        <v>46386</v>
       </c>
       <c r="N52" t="s">
         <v>725</v>
@@ -12882,8 +12908,8 @@
       <c r="L53" t="s">
         <v>722</v>
       </c>
-      <c r="M53" s="1">
-        <v>46385</v>
+      <c r="M53" s="2">
+        <v>46386</v>
       </c>
       <c r="N53" t="s">
         <v>725</v>
@@ -12926,8 +12952,8 @@
       <c r="L54" t="s">
         <v>722</v>
       </c>
-      <c r="M54" s="1">
-        <v>46385</v>
+      <c r="M54" s="2">
+        <v>46386</v>
       </c>
       <c r="N54" t="s">
         <v>725</v>
@@ -12970,8 +12996,8 @@
       <c r="L55" t="s">
         <v>722</v>
       </c>
-      <c r="M55" s="1">
-        <v>46385</v>
+      <c r="M55" s="2">
+        <v>46386</v>
       </c>
       <c r="N55" t="s">
         <v>725</v>
@@ -13137,8 +13163,8 @@
       <c r="L59" t="s">
         <v>722</v>
       </c>
-      <c r="M59" s="1">
-        <v>46385</v>
+      <c r="M59" s="2">
+        <v>46386</v>
       </c>
       <c r="N59" t="s">
         <v>725</v>
@@ -13263,8 +13289,8 @@
       <c r="L62" t="s">
         <v>722</v>
       </c>
-      <c r="M62" s="1">
-        <v>46385</v>
+      <c r="M62" s="2">
+        <v>46386</v>
       </c>
       <c r="N62" t="s">
         <v>725</v>
@@ -13307,8 +13333,8 @@
       <c r="L63" t="s">
         <v>722</v>
       </c>
-      <c r="M63" s="1">
-        <v>46385</v>
+      <c r="M63" s="2">
+        <v>46386</v>
       </c>
       <c r="N63" t="s">
         <v>725</v>
@@ -13351,8 +13377,8 @@
       <c r="L64" t="s">
         <v>722</v>
       </c>
-      <c r="M64" s="1">
-        <v>46385</v>
+      <c r="M64" s="2">
+        <v>46386</v>
       </c>
       <c r="N64" t="s">
         <v>725</v>
@@ -13395,8 +13421,8 @@
       <c r="L65" t="s">
         <v>722</v>
       </c>
-      <c r="M65" s="1">
-        <v>46385</v>
+      <c r="M65" s="2">
+        <v>46386</v>
       </c>
       <c r="N65" t="s">
         <v>725</v>
@@ -13439,8 +13465,8 @@
       <c r="L66" t="s">
         <v>722</v>
       </c>
-      <c r="M66" s="1">
-        <v>46385</v>
+      <c r="M66" s="2">
+        <v>46386</v>
       </c>
       <c r="N66" t="s">
         <v>725</v>
@@ -13483,8 +13509,8 @@
       <c r="L67" t="s">
         <v>722</v>
       </c>
-      <c r="M67" s="1">
-        <v>46385</v>
+      <c r="M67" s="2">
+        <v>46386</v>
       </c>
       <c r="N67" t="s">
         <v>725</v>
@@ -13527,8 +13553,8 @@
       <c r="L68" t="s">
         <v>722</v>
       </c>
-      <c r="M68" s="1">
-        <v>46385</v>
+      <c r="M68" s="2">
+        <v>46386</v>
       </c>
       <c r="N68" t="s">
         <v>725</v>
@@ -13571,8 +13597,8 @@
       <c r="L69" t="s">
         <v>722</v>
       </c>
-      <c r="M69" s="1">
-        <v>46385</v>
+      <c r="M69" s="2">
+        <v>46386</v>
       </c>
       <c r="N69" t="s">
         <v>725</v>
@@ -13615,8 +13641,8 @@
       <c r="L70" t="s">
         <v>722</v>
       </c>
-      <c r="M70" s="1">
-        <v>46385</v>
+      <c r="M70" s="2">
+        <v>46386</v>
       </c>
       <c r="N70" t="s">
         <v>725</v>
@@ -13659,8 +13685,8 @@
       <c r="L71" t="s">
         <v>722</v>
       </c>
-      <c r="M71" s="1">
-        <v>46385</v>
+      <c r="M71" s="2">
+        <v>46386</v>
       </c>
       <c r="N71" t="s">
         <v>725</v>
@@ -13703,8 +13729,8 @@
       <c r="L72" t="s">
         <v>722</v>
       </c>
-      <c r="M72" s="1">
-        <v>46385</v>
+      <c r="M72" s="2">
+        <v>46386</v>
       </c>
       <c r="N72" t="s">
         <v>725</v>
@@ -13747,8 +13773,8 @@
       <c r="L73" t="s">
         <v>722</v>
       </c>
-      <c r="M73" s="1">
-        <v>46385</v>
+      <c r="M73" s="2">
+        <v>46386</v>
       </c>
       <c r="N73" t="s">
         <v>725</v>
@@ -13791,8 +13817,8 @@
       <c r="L74" t="s">
         <v>722</v>
       </c>
-      <c r="M74" s="1">
-        <v>46385</v>
+      <c r="M74" s="2">
+        <v>46386</v>
       </c>
       <c r="N74" t="s">
         <v>725</v>
@@ -13835,8 +13861,8 @@
       <c r="L75" t="s">
         <v>722</v>
       </c>
-      <c r="M75" s="1">
-        <v>46385</v>
+      <c r="M75" s="2">
+        <v>46386</v>
       </c>
       <c r="N75" t="s">
         <v>725</v>
@@ -13879,8 +13905,8 @@
       <c r="L76" t="s">
         <v>722</v>
       </c>
-      <c r="M76" s="1">
-        <v>46385</v>
+      <c r="M76" s="2">
+        <v>46386</v>
       </c>
       <c r="N76" t="s">
         <v>725</v>
@@ -13923,8 +13949,8 @@
       <c r="L77" t="s">
         <v>722</v>
       </c>
-      <c r="M77" s="1">
-        <v>46385</v>
+      <c r="M77" s="2">
+        <v>46386</v>
       </c>
       <c r="N77" t="s">
         <v>725</v>
@@ -13967,8 +13993,8 @@
       <c r="L78" t="s">
         <v>722</v>
       </c>
-      <c r="M78" s="1">
-        <v>46385</v>
+      <c r="M78" s="2">
+        <v>46386</v>
       </c>
       <c r="N78" t="s">
         <v>725</v>
@@ -14011,8 +14037,8 @@
       <c r="L79" t="s">
         <v>722</v>
       </c>
-      <c r="M79" s="1">
-        <v>46385</v>
+      <c r="M79" s="2">
+        <v>46386</v>
       </c>
       <c r="N79" t="s">
         <v>725</v>
@@ -14055,8 +14081,8 @@
       <c r="L80" t="s">
         <v>722</v>
       </c>
-      <c r="M80" s="1">
-        <v>46385</v>
+      <c r="M80" s="2">
+        <v>46386</v>
       </c>
       <c r="N80" t="s">
         <v>725</v>
@@ -14099,8 +14125,8 @@
       <c r="L81" t="s">
         <v>722</v>
       </c>
-      <c r="M81" s="1">
-        <v>46385</v>
+      <c r="M81" s="2">
+        <v>46386</v>
       </c>
       <c r="N81" t="s">
         <v>725</v>
@@ -14143,8 +14169,8 @@
       <c r="L82" t="s">
         <v>722</v>
       </c>
-      <c r="M82" s="1">
-        <v>46385</v>
+      <c r="M82" s="2">
+        <v>46386</v>
       </c>
       <c r="N82" t="s">
         <v>725</v>
@@ -14187,8 +14213,8 @@
       <c r="L83" t="s">
         <v>722</v>
       </c>
-      <c r="M83" s="1">
-        <v>46385</v>
+      <c r="M83" s="2">
+        <v>46386</v>
       </c>
       <c r="N83" t="s">
         <v>725</v>
@@ -14231,8 +14257,8 @@
       <c r="L84" t="s">
         <v>722</v>
       </c>
-      <c r="M84" s="1">
-        <v>46385</v>
+      <c r="M84" s="2">
+        <v>46386</v>
       </c>
       <c r="N84" t="s">
         <v>725</v>
@@ -14275,8 +14301,8 @@
       <c r="L85" t="s">
         <v>722</v>
       </c>
-      <c r="M85" s="1">
-        <v>46385</v>
+      <c r="M85" s="2">
+        <v>46386</v>
       </c>
       <c r="N85" t="s">
         <v>725</v>
@@ -14319,8 +14345,8 @@
       <c r="L86" t="s">
         <v>722</v>
       </c>
-      <c r="M86" s="1">
-        <v>46385</v>
+      <c r="M86" s="2">
+        <v>46386</v>
       </c>
       <c r="N86" t="s">
         <v>725</v>
@@ -14363,8 +14389,8 @@
       <c r="L87" t="s">
         <v>722</v>
       </c>
-      <c r="M87" s="1">
-        <v>46385</v>
+      <c r="M87" s="2">
+        <v>46386</v>
       </c>
       <c r="N87" t="s">
         <v>725</v>
@@ -14407,8 +14433,8 @@
       <c r="L88" t="s">
         <v>722</v>
       </c>
-      <c r="M88" s="1">
-        <v>46385</v>
+      <c r="M88" s="2">
+        <v>46386</v>
       </c>
       <c r="N88" t="s">
         <v>725</v>
@@ -14451,8 +14477,8 @@
       <c r="L89" t="s">
         <v>722</v>
       </c>
-      <c r="M89" s="1">
-        <v>46385</v>
+      <c r="M89" s="2">
+        <v>46386</v>
       </c>
       <c r="N89" t="s">
         <v>725</v>
@@ -14495,8 +14521,8 @@
       <c r="L90" t="s">
         <v>722</v>
       </c>
-      <c r="M90" s="1">
-        <v>46385</v>
+      <c r="M90" s="2">
+        <v>46386</v>
       </c>
       <c r="N90" t="s">
         <v>725</v>
@@ -14580,8 +14606,8 @@
       <c r="L92" t="s">
         <v>722</v>
       </c>
-      <c r="M92" s="1">
-        <v>46385</v>
+      <c r="M92" s="2">
+        <v>46386</v>
       </c>
       <c r="N92" t="s">
         <v>725</v>
@@ -14624,8 +14650,8 @@
       <c r="L93" t="s">
         <v>722</v>
       </c>
-      <c r="M93" s="1">
-        <v>46385</v>
+      <c r="M93" s="2">
+        <v>46386</v>
       </c>
       <c r="N93" t="s">
         <v>725</v>
@@ -14668,8 +14694,8 @@
       <c r="L94" t="s">
         <v>722</v>
       </c>
-      <c r="M94" s="1">
-        <v>46385</v>
+      <c r="M94" s="2">
+        <v>46386</v>
       </c>
       <c r="N94" t="s">
         <v>725</v>
@@ -14712,8 +14738,8 @@
       <c r="L95" t="s">
         <v>722</v>
       </c>
-      <c r="M95" s="1">
-        <v>46385</v>
+      <c r="M95" s="2">
+        <v>46386</v>
       </c>
       <c r="N95" t="s">
         <v>725</v>
@@ -14756,8 +14782,8 @@
       <c r="L96" t="s">
         <v>722</v>
       </c>
-      <c r="M96" s="1">
-        <v>46385</v>
+      <c r="M96" s="2">
+        <v>46386</v>
       </c>
       <c r="N96" t="s">
         <v>725</v>
@@ -14800,8 +14826,8 @@
       <c r="L97" t="s">
         <v>722</v>
       </c>
-      <c r="M97" s="1">
-        <v>46385</v>
+      <c r="M97" s="2">
+        <v>46386</v>
       </c>
       <c r="N97" t="s">
         <v>725</v>
@@ -14844,8 +14870,8 @@
       <c r="L98" t="s">
         <v>722</v>
       </c>
-      <c r="M98" s="1">
-        <v>46385</v>
+      <c r="M98" s="2">
+        <v>46386</v>
       </c>
       <c r="N98" t="s">
         <v>725</v>
@@ -14888,8 +14914,8 @@
       <c r="L99" t="s">
         <v>722</v>
       </c>
-      <c r="M99" s="1">
-        <v>46385</v>
+      <c r="M99" s="2">
+        <v>46386</v>
       </c>
       <c r="N99" t="s">
         <v>725</v>
@@ -14932,8 +14958,8 @@
       <c r="L100" t="s">
         <v>722</v>
       </c>
-      <c r="M100" s="1">
-        <v>46385</v>
+      <c r="M100" s="2">
+        <v>46386</v>
       </c>
       <c r="N100" t="s">
         <v>725</v>
@@ -14976,8 +15002,8 @@
       <c r="L101" t="s">
         <v>722</v>
       </c>
-      <c r="M101" s="1">
-        <v>46385</v>
+      <c r="M101" s="2">
+        <v>46386</v>
       </c>
       <c r="N101" t="s">
         <v>725</v>
@@ -15020,8 +15046,8 @@
       <c r="L102" t="s">
         <v>722</v>
       </c>
-      <c r="M102" s="1">
-        <v>46385</v>
+      <c r="M102" s="2">
+        <v>46386</v>
       </c>
       <c r="N102" t="s">
         <v>725</v>
@@ -15064,8 +15090,8 @@
       <c r="L103" t="s">
         <v>722</v>
       </c>
-      <c r="M103" s="1">
-        <v>46385</v>
+      <c r="M103" s="2">
+        <v>46386</v>
       </c>
       <c r="N103" t="s">
         <v>725</v>
@@ -15108,8 +15134,8 @@
       <c r="L104" t="s">
         <v>722</v>
       </c>
-      <c r="M104" s="1">
-        <v>46385</v>
+      <c r="M104" s="2">
+        <v>46386</v>
       </c>
       <c r="N104" t="s">
         <v>725</v>
@@ -15152,8 +15178,8 @@
       <c r="L105" t="s">
         <v>722</v>
       </c>
-      <c r="M105" s="1">
-        <v>46385</v>
+      <c r="M105" s="2">
+        <v>46386</v>
       </c>
       <c r="N105" t="s">
         <v>725</v>
@@ -15196,8 +15222,8 @@
       <c r="L106" t="s">
         <v>722</v>
       </c>
-      <c r="M106" s="1">
-        <v>46385</v>
+      <c r="M106" s="2">
+        <v>46386</v>
       </c>
       <c r="N106" t="s">
         <v>725</v>
@@ -15240,8 +15266,8 @@
       <c r="L107" t="s">
         <v>722</v>
       </c>
-      <c r="M107" s="1">
-        <v>46385</v>
+      <c r="M107" s="2">
+        <v>46386</v>
       </c>
       <c r="N107" t="s">
         <v>725</v>
@@ -15284,8 +15310,8 @@
       <c r="L108" t="s">
         <v>722</v>
       </c>
-      <c r="M108" s="1">
-        <v>46385</v>
+      <c r="M108" s="2">
+        <v>46386</v>
       </c>
       <c r="N108" t="s">
         <v>725</v>
@@ -15328,8 +15354,8 @@
       <c r="L109" t="s">
         <v>722</v>
       </c>
-      <c r="M109" s="1">
-        <v>46385</v>
+      <c r="M109" s="2">
+        <v>46386</v>
       </c>
       <c r="N109" t="s">
         <v>725</v>
@@ -15372,8 +15398,8 @@
       <c r="L110" t="s">
         <v>722</v>
       </c>
-      <c r="M110" s="1">
-        <v>46385</v>
+      <c r="M110" s="2">
+        <v>46386</v>
       </c>
       <c r="N110" t="s">
         <v>725</v>
@@ -15416,8 +15442,8 @@
       <c r="L111" t="s">
         <v>722</v>
       </c>
-      <c r="M111" s="1">
-        <v>46385</v>
+      <c r="M111" s="2">
+        <v>46386</v>
       </c>
       <c r="N111" t="s">
         <v>725</v>
@@ -15460,8 +15486,8 @@
       <c r="L112" t="s">
         <v>722</v>
       </c>
-      <c r="M112" s="1">
-        <v>46385</v>
+      <c r="M112" s="2">
+        <v>46386</v>
       </c>
       <c r="N112" t="s">
         <v>725</v>
@@ -15504,8 +15530,8 @@
       <c r="L113" t="s">
         <v>722</v>
       </c>
-      <c r="M113" s="1">
-        <v>46385</v>
+      <c r="M113" s="2">
+        <v>46386</v>
       </c>
       <c r="N113" t="s">
         <v>725</v>
@@ -15548,8 +15574,8 @@
       <c r="L114" t="s">
         <v>722</v>
       </c>
-      <c r="M114" s="1">
-        <v>46385</v>
+      <c r="M114" s="2">
+        <v>46386</v>
       </c>
       <c r="N114" t="s">
         <v>725</v>
@@ -15592,8 +15618,8 @@
       <c r="L115" t="s">
         <v>722</v>
       </c>
-      <c r="M115" s="1">
-        <v>46385</v>
+      <c r="M115" s="2">
+        <v>46386</v>
       </c>
       <c r="N115" t="s">
         <v>725</v>
@@ -15636,8 +15662,8 @@
       <c r="L116" t="s">
         <v>722</v>
       </c>
-      <c r="M116" s="1">
-        <v>46385</v>
+      <c r="M116" s="2">
+        <v>46386</v>
       </c>
       <c r="N116" t="s">
         <v>725</v>
@@ -15680,8 +15706,8 @@
       <c r="L117" t="s">
         <v>722</v>
       </c>
-      <c r="M117" s="1">
-        <v>46385</v>
+      <c r="M117" s="2">
+        <v>46386</v>
       </c>
       <c r="N117" t="s">
         <v>725</v>
@@ -15724,8 +15750,8 @@
       <c r="L118" t="s">
         <v>722</v>
       </c>
-      <c r="M118" s="1">
-        <v>46385</v>
+      <c r="M118" s="2">
+        <v>46386</v>
       </c>
       <c r="N118" t="s">
         <v>725</v>
@@ -15768,8 +15794,8 @@
       <c r="L119" t="s">
         <v>722</v>
       </c>
-      <c r="M119" s="1">
-        <v>46385</v>
+      <c r="M119" s="2">
+        <v>46386</v>
       </c>
       <c r="N119" t="s">
         <v>725</v>
@@ -15812,8 +15838,8 @@
       <c r="L120" t="s">
         <v>722</v>
       </c>
-      <c r="M120" s="1">
-        <v>46385</v>
+      <c r="M120" s="2">
+        <v>46386</v>
       </c>
       <c r="N120" t="s">
         <v>725</v>
@@ -15856,8 +15882,8 @@
       <c r="L121" t="s">
         <v>722</v>
       </c>
-      <c r="M121" s="1">
-        <v>46385</v>
+      <c r="M121" s="2">
+        <v>46386</v>
       </c>
       <c r="N121" t="s">
         <v>725</v>
@@ -15900,8 +15926,8 @@
       <c r="L122" t="s">
         <v>722</v>
       </c>
-      <c r="M122" s="1">
-        <v>46385</v>
+      <c r="M122" s="2">
+        <v>46386</v>
       </c>
       <c r="N122" t="s">
         <v>725</v>
@@ -15944,8 +15970,8 @@
       <c r="L123" t="s">
         <v>722</v>
       </c>
-      <c r="M123" s="1">
-        <v>46385</v>
+      <c r="M123" s="2">
+        <v>46386</v>
       </c>
       <c r="N123" t="s">
         <v>725</v>
@@ -15988,8 +16014,8 @@
       <c r="L124" t="s">
         <v>722</v>
       </c>
-      <c r="M124" s="1">
-        <v>46385</v>
+      <c r="M124" s="2">
+        <v>46386</v>
       </c>
       <c r="N124" t="s">
         <v>725</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (16/10/2026 12:22)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2202,16 +2202,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2227,7 +2219,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2235,30 +2227,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2558,55 +2532,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2650,7 +2624,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2694,7 +2668,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2738,7 +2712,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2864,7 +2838,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2908,7 +2882,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2952,7 +2926,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2999,7 +2973,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3122,7 +3096,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -3166,7 +3140,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3210,7 +3184,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3254,7 +3228,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3301,7 +3275,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3345,7 +3319,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3471,7 +3445,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3515,7 +3489,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3600,7 +3574,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3647,7 +3621,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3694,7 +3668,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3738,7 +3712,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3782,7 +3756,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3867,7 +3841,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3952,7 +3926,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3999,7 +3973,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4043,7 +4017,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4087,7 +4061,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4172,7 +4146,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4216,7 +4190,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4260,7 +4234,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4345,7 +4319,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4389,7 +4363,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4433,7 +4407,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4477,7 +4451,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4644,7 +4618,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4688,7 +4662,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4732,7 +4706,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4776,7 +4750,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4823,7 +4797,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4867,7 +4841,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4949,7 +4923,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4993,7 +4967,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5081,7 +5055,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5125,7 +5099,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5172,7 +5146,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5216,7 +5190,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -5260,7 +5234,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5304,7 +5278,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5348,7 +5322,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5395,7 +5369,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5439,7 +5413,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5486,7 +5460,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5530,7 +5504,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5577,7 +5551,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5665,7 +5639,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5709,7 +5683,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5753,7 +5727,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5797,7 +5771,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5841,7 +5815,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5885,7 +5859,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5970,7 +5944,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6014,7 +5988,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -6058,7 +6032,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -6102,7 +6076,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -6146,7 +6120,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -6190,7 +6164,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6234,7 +6208,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6278,7 +6252,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6325,7 +6299,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6369,7 +6343,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6413,7 +6387,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6457,7 +6431,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6501,7 +6475,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6545,7 +6519,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6589,7 +6563,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6633,7 +6607,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6677,7 +6651,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6765,7 +6739,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6809,7 +6783,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6935,7 +6909,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6979,7 +6953,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7023,7 +6997,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7067,7 +7041,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7149,7 +7123,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7193,7 +7167,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7240,7 +7214,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7284,7 +7258,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7410,7 +7384,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7454,7 +7428,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7539,7 +7513,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7583,7 +7557,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7627,7 +7601,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7671,7 +7645,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7715,7 +7689,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7759,7 +7733,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7803,7 +7777,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7847,7 +7821,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7932,7 +7906,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8099,7 +8073,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8143,7 +8117,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8187,7 +8161,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8231,7 +8205,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8275,7 +8249,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8319,7 +8293,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8363,7 +8337,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8448,7 +8422,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8492,7 +8466,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8577,7 +8551,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8703,7 +8677,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8747,7 +8721,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8832,7 +8806,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8876,7 +8850,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8920,7 +8894,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8964,7 +8938,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -9008,7 +8982,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -9052,7 +9026,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9096,7 +9070,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9140,7 +9114,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9225,7 +9199,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9392,7 +9366,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9436,7 +9410,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9480,7 +9454,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9524,7 +9498,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9609,7 +9583,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9653,7 +9627,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9697,7 +9671,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9741,7 +9715,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9785,7 +9759,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9829,7 +9803,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9873,7 +9847,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9917,7 +9891,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9961,7 +9935,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10005,7 +9979,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10049,7 +10023,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -10093,7 +10067,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10137,7 +10111,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10181,7 +10155,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -10225,7 +10199,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10269,7 +10243,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10313,7 +10287,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10357,7 +10331,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10401,7 +10375,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10445,7 +10419,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10489,7 +10463,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10574,7 +10548,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10659,7 +10633,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10674,55 +10648,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11091,7 +11065,7 @@
       <c r="L10" t="s">
         <v>722</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46386</v>
       </c>
       <c r="N10" t="s">
@@ -11135,7 +11109,7 @@
       <c r="L11" t="s">
         <v>722</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46386</v>
       </c>
       <c r="N11" t="s">
@@ -11343,7 +11317,7 @@
       <c r="L16" t="s">
         <v>722</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46386</v>
       </c>
       <c r="N16" t="s">
@@ -11469,7 +11443,7 @@
       <c r="L19" t="s">
         <v>722</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46386</v>
       </c>
       <c r="N19" t="s">
@@ -11513,7 +11487,7 @@
       <c r="L20" t="s">
         <v>722</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46386</v>
       </c>
       <c r="N20" t="s">
@@ -11557,7 +11531,7 @@
       <c r="L21" t="s">
         <v>722</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46386</v>
       </c>
       <c r="N21" t="s">
@@ -11724,7 +11698,7 @@
       <c r="L25" t="s">
         <v>722</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46386</v>
       </c>
       <c r="N25" t="s">
@@ -11850,7 +11824,7 @@
       <c r="L28" t="s">
         <v>722</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46386</v>
       </c>
       <c r="N28" t="s">
@@ -11935,7 +11909,7 @@
       <c r="L30" t="s">
         <v>722</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46386</v>
       </c>
       <c r="N30" t="s">
@@ -12389,7 +12363,7 @@
       <c r="L41" t="s">
         <v>722</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46386</v>
       </c>
       <c r="N41" t="s">
@@ -12474,7 +12448,7 @@
       <c r="L43" t="s">
         <v>722</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46386</v>
       </c>
       <c r="N43" t="s">
@@ -12518,7 +12492,7 @@
       <c r="L44" t="s">
         <v>722</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46386</v>
       </c>
       <c r="N44" t="s">
@@ -12562,7 +12536,7 @@
       <c r="L45" t="s">
         <v>722</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46386</v>
       </c>
       <c r="N45" t="s">
@@ -12688,7 +12662,7 @@
       <c r="L48" t="s">
         <v>722</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46386</v>
       </c>
       <c r="N48" t="s">
@@ -12732,7 +12706,7 @@
       <c r="L49" t="s">
         <v>723</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46321</v>
       </c>
       <c r="N49" t="s">
@@ -12776,7 +12750,7 @@
       <c r="L50" t="s">
         <v>723</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46321</v>
       </c>
       <c r="N50" t="s">
@@ -12820,7 +12794,7 @@
       <c r="L51" t="s">
         <v>722</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46386</v>
       </c>
       <c r="N51" t="s">
@@ -12864,7 +12838,7 @@
       <c r="L52" t="s">
         <v>722</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46386</v>
       </c>
       <c r="N52" t="s">
@@ -12908,7 +12882,7 @@
       <c r="L53" t="s">
         <v>722</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46386</v>
       </c>
       <c r="N53" t="s">
@@ -12952,7 +12926,7 @@
       <c r="L54" t="s">
         <v>722</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46386</v>
       </c>
       <c r="N54" t="s">
@@ -12996,7 +12970,7 @@
       <c r="L55" t="s">
         <v>722</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46386</v>
       </c>
       <c r="N55" t="s">
@@ -13163,7 +13137,7 @@
       <c r="L59" t="s">
         <v>722</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46386</v>
       </c>
       <c r="N59" t="s">
@@ -13289,7 +13263,7 @@
       <c r="L62" t="s">
         <v>722</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46386</v>
       </c>
       <c r="N62" t="s">
@@ -13333,7 +13307,7 @@
       <c r="L63" t="s">
         <v>722</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46386</v>
       </c>
       <c r="N63" t="s">
@@ -13377,7 +13351,7 @@
       <c r="L64" t="s">
         <v>722</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46386</v>
       </c>
       <c r="N64" t="s">
@@ -13421,7 +13395,7 @@
       <c r="L65" t="s">
         <v>722</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="1">
         <v>46386</v>
       </c>
       <c r="N65" t="s">
@@ -13465,7 +13439,7 @@
       <c r="L66" t="s">
         <v>722</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="1">
         <v>46386</v>
       </c>
       <c r="N66" t="s">
@@ -13509,7 +13483,7 @@
       <c r="L67" t="s">
         <v>722</v>
       </c>
-      <c r="M67" s="2">
+      <c r="M67" s="1">
         <v>46386</v>
       </c>
       <c r="N67" t="s">
@@ -13553,7 +13527,7 @@
       <c r="L68" t="s">
         <v>722</v>
       </c>
-      <c r="M68" s="2">
+      <c r="M68" s="1">
         <v>46386</v>
       </c>
       <c r="N68" t="s">
@@ -13597,7 +13571,7 @@
       <c r="L69" t="s">
         <v>722</v>
       </c>
-      <c r="M69" s="2">
+      <c r="M69" s="1">
         <v>46386</v>
       </c>
       <c r="N69" t="s">
@@ -13641,7 +13615,7 @@
       <c r="L70" t="s">
         <v>722</v>
       </c>
-      <c r="M70" s="2">
+      <c r="M70" s="1">
         <v>46386</v>
       </c>
       <c r="N70" t="s">
@@ -13685,7 +13659,7 @@
       <c r="L71" t="s">
         <v>722</v>
       </c>
-      <c r="M71" s="2">
+      <c r="M71" s="1">
         <v>46386</v>
       </c>
       <c r="N71" t="s">
@@ -13729,7 +13703,7 @@
       <c r="L72" t="s">
         <v>722</v>
       </c>
-      <c r="M72" s="2">
+      <c r="M72" s="1">
         <v>46386</v>
       </c>
       <c r="N72" t="s">
@@ -13773,7 +13747,7 @@
       <c r="L73" t="s">
         <v>722</v>
       </c>
-      <c r="M73" s="2">
+      <c r="M73" s="1">
         <v>46386</v>
       </c>
       <c r="N73" t="s">
@@ -13817,7 +13791,7 @@
       <c r="L74" t="s">
         <v>722</v>
       </c>
-      <c r="M74" s="2">
+      <c r="M74" s="1">
         <v>46386</v>
       </c>
       <c r="N74" t="s">
@@ -13861,7 +13835,7 @@
       <c r="L75" t="s">
         <v>722</v>
       </c>
-      <c r="M75" s="2">
+      <c r="M75" s="1">
         <v>46386</v>
       </c>
       <c r="N75" t="s">
@@ -13905,7 +13879,7 @@
       <c r="L76" t="s">
         <v>722</v>
       </c>
-      <c r="M76" s="2">
+      <c r="M76" s="1">
         <v>46386</v>
       </c>
       <c r="N76" t="s">
@@ -13949,7 +13923,7 @@
       <c r="L77" t="s">
         <v>722</v>
       </c>
-      <c r="M77" s="2">
+      <c r="M77" s="1">
         <v>46386</v>
       </c>
       <c r="N77" t="s">
@@ -13993,7 +13967,7 @@
       <c r="L78" t="s">
         <v>722</v>
       </c>
-      <c r="M78" s="2">
+      <c r="M78" s="1">
         <v>46386</v>
       </c>
       <c r="N78" t="s">
@@ -14037,7 +14011,7 @@
       <c r="L79" t="s">
         <v>722</v>
       </c>
-      <c r="M79" s="2">
+      <c r="M79" s="1">
         <v>46386</v>
       </c>
       <c r="N79" t="s">
@@ -14081,7 +14055,7 @@
       <c r="L80" t="s">
         <v>722</v>
       </c>
-      <c r="M80" s="2">
+      <c r="M80" s="1">
         <v>46386</v>
       </c>
       <c r="N80" t="s">
@@ -14125,7 +14099,7 @@
       <c r="L81" t="s">
         <v>722</v>
       </c>
-      <c r="M81" s="2">
+      <c r="M81" s="1">
         <v>46386</v>
       </c>
       <c r="N81" t="s">
@@ -14169,7 +14143,7 @@
       <c r="L82" t="s">
         <v>722</v>
       </c>
-      <c r="M82" s="2">
+      <c r="M82" s="1">
         <v>46386</v>
       </c>
       <c r="N82" t="s">
@@ -14213,7 +14187,7 @@
       <c r="L83" t="s">
         <v>722</v>
       </c>
-      <c r="M83" s="2">
+      <c r="M83" s="1">
         <v>46386</v>
       </c>
       <c r="N83" t="s">
@@ -14257,7 +14231,7 @@
       <c r="L84" t="s">
         <v>722</v>
       </c>
-      <c r="M84" s="2">
+      <c r="M84" s="1">
         <v>46386</v>
       </c>
       <c r="N84" t="s">
@@ -14301,7 +14275,7 @@
       <c r="L85" t="s">
         <v>722</v>
       </c>
-      <c r="M85" s="2">
+      <c r="M85" s="1">
         <v>46386</v>
       </c>
       <c r="N85" t="s">
@@ -14345,7 +14319,7 @@
       <c r="L86" t="s">
         <v>722</v>
       </c>
-      <c r="M86" s="2">
+      <c r="M86" s="1">
         <v>46386</v>
       </c>
       <c r="N86" t="s">
@@ -14389,7 +14363,7 @@
       <c r="L87" t="s">
         <v>722</v>
       </c>
-      <c r="M87" s="2">
+      <c r="M87" s="1">
         <v>46386</v>
       </c>
       <c r="N87" t="s">
@@ -14433,7 +14407,7 @@
       <c r="L88" t="s">
         <v>722</v>
       </c>
-      <c r="M88" s="2">
+      <c r="M88" s="1">
         <v>46386</v>
       </c>
       <c r="N88" t="s">
@@ -14477,7 +14451,7 @@
       <c r="L89" t="s">
         <v>722</v>
       </c>
-      <c r="M89" s="2">
+      <c r="M89" s="1">
         <v>46386</v>
       </c>
       <c r="N89" t="s">
@@ -14521,7 +14495,7 @@
       <c r="L90" t="s">
         <v>722</v>
       </c>
-      <c r="M90" s="2">
+      <c r="M90" s="1">
         <v>46386</v>
       </c>
       <c r="N90" t="s">
@@ -14606,7 +14580,7 @@
       <c r="L92" t="s">
         <v>722</v>
       </c>
-      <c r="M92" s="2">
+      <c r="M92" s="1">
         <v>46386</v>
       </c>
       <c r="N92" t="s">
@@ -14650,7 +14624,7 @@
       <c r="L93" t="s">
         <v>722</v>
       </c>
-      <c r="M93" s="2">
+      <c r="M93" s="1">
         <v>46386</v>
       </c>
       <c r="N93" t="s">
@@ -14694,7 +14668,7 @@
       <c r="L94" t="s">
         <v>722</v>
       </c>
-      <c r="M94" s="2">
+      <c r="M94" s="1">
         <v>46386</v>
       </c>
       <c r="N94" t="s">
@@ -14738,7 +14712,7 @@
       <c r="L95" t="s">
         <v>722</v>
       </c>
-      <c r="M95" s="2">
+      <c r="M95" s="1">
         <v>46386</v>
       </c>
       <c r="N95" t="s">
@@ -14782,7 +14756,7 @@
       <c r="L96" t="s">
         <v>722</v>
       </c>
-      <c r="M96" s="2">
+      <c r="M96" s="1">
         <v>46386</v>
       </c>
       <c r="N96" t="s">
@@ -14826,7 +14800,7 @@
       <c r="L97" t="s">
         <v>722</v>
       </c>
-      <c r="M97" s="2">
+      <c r="M97" s="1">
         <v>46386</v>
       </c>
       <c r="N97" t="s">
@@ -14870,7 +14844,7 @@
       <c r="L98" t="s">
         <v>722</v>
       </c>
-      <c r="M98" s="2">
+      <c r="M98" s="1">
         <v>46386</v>
       </c>
       <c r="N98" t="s">
@@ -14914,7 +14888,7 @@
       <c r="L99" t="s">
         <v>722</v>
       </c>
-      <c r="M99" s="2">
+      <c r="M99" s="1">
         <v>46386</v>
       </c>
       <c r="N99" t="s">
@@ -14958,7 +14932,7 @@
       <c r="L100" t="s">
         <v>722</v>
       </c>
-      <c r="M100" s="2">
+      <c r="M100" s="1">
         <v>46386</v>
       </c>
       <c r="N100" t="s">
@@ -15002,7 +14976,7 @@
       <c r="L101" t="s">
         <v>722</v>
       </c>
-      <c r="M101" s="2">
+      <c r="M101" s="1">
         <v>46386</v>
       </c>
       <c r="N101" t="s">
@@ -15046,7 +15020,7 @@
       <c r="L102" t="s">
         <v>722</v>
       </c>
-      <c r="M102" s="2">
+      <c r="M102" s="1">
         <v>46386</v>
       </c>
       <c r="N102" t="s">
@@ -15090,7 +15064,7 @@
       <c r="L103" t="s">
         <v>722</v>
       </c>
-      <c r="M103" s="2">
+      <c r="M103" s="1">
         <v>46386</v>
       </c>
       <c r="N103" t="s">
@@ -15134,7 +15108,7 @@
       <c r="L104" t="s">
         <v>722</v>
       </c>
-      <c r="M104" s="2">
+      <c r="M104" s="1">
         <v>46386</v>
       </c>
       <c r="N104" t="s">
@@ -15178,7 +15152,7 @@
       <c r="L105" t="s">
         <v>722</v>
       </c>
-      <c r="M105" s="2">
+      <c r="M105" s="1">
         <v>46386</v>
       </c>
       <c r="N105" t="s">
@@ -15222,7 +15196,7 @@
       <c r="L106" t="s">
         <v>722</v>
       </c>
-      <c r="M106" s="2">
+      <c r="M106" s="1">
         <v>46386</v>
       </c>
       <c r="N106" t="s">
@@ -15266,7 +15240,7 @@
       <c r="L107" t="s">
         <v>722</v>
       </c>
-      <c r="M107" s="2">
+      <c r="M107" s="1">
         <v>46386</v>
       </c>
       <c r="N107" t="s">
@@ -15310,7 +15284,7 @@
       <c r="L108" t="s">
         <v>722</v>
       </c>
-      <c r="M108" s="2">
+      <c r="M108" s="1">
         <v>46386</v>
       </c>
       <c r="N108" t="s">
@@ -15354,7 +15328,7 @@
       <c r="L109" t="s">
         <v>722</v>
       </c>
-      <c r="M109" s="2">
+      <c r="M109" s="1">
         <v>46386</v>
       </c>
       <c r="N109" t="s">
@@ -15398,7 +15372,7 @@
       <c r="L110" t="s">
         <v>722</v>
       </c>
-      <c r="M110" s="2">
+      <c r="M110" s="1">
         <v>46386</v>
       </c>
       <c r="N110" t="s">
@@ -15442,7 +15416,7 @@
       <c r="L111" t="s">
         <v>722</v>
       </c>
-      <c r="M111" s="2">
+      <c r="M111" s="1">
         <v>46386</v>
       </c>
       <c r="N111" t="s">
@@ -15486,7 +15460,7 @@
       <c r="L112" t="s">
         <v>722</v>
       </c>
-      <c r="M112" s="2">
+      <c r="M112" s="1">
         <v>46386</v>
       </c>
       <c r="N112" t="s">
@@ -15530,7 +15504,7 @@
       <c r="L113" t="s">
         <v>722</v>
       </c>
-      <c r="M113" s="2">
+      <c r="M113" s="1">
         <v>46386</v>
       </c>
       <c r="N113" t="s">
@@ -15574,7 +15548,7 @@
       <c r="L114" t="s">
         <v>722</v>
       </c>
-      <c r="M114" s="2">
+      <c r="M114" s="1">
         <v>46386</v>
       </c>
       <c r="N114" t="s">
@@ -15618,7 +15592,7 @@
       <c r="L115" t="s">
         <v>722</v>
       </c>
-      <c r="M115" s="2">
+      <c r="M115" s="1">
         <v>46386</v>
       </c>
       <c r="N115" t="s">
@@ -15662,7 +15636,7 @@
       <c r="L116" t="s">
         <v>722</v>
       </c>
-      <c r="M116" s="2">
+      <c r="M116" s="1">
         <v>46386</v>
       </c>
       <c r="N116" t="s">
@@ -15706,7 +15680,7 @@
       <c r="L117" t="s">
         <v>722</v>
       </c>
-      <c r="M117" s="2">
+      <c r="M117" s="1">
         <v>46386</v>
       </c>
       <c r="N117" t="s">
@@ -15750,7 +15724,7 @@
       <c r="L118" t="s">
         <v>722</v>
       </c>
-      <c r="M118" s="2">
+      <c r="M118" s="1">
         <v>46386</v>
       </c>
       <c r="N118" t="s">
@@ -15794,7 +15768,7 @@
       <c r="L119" t="s">
         <v>722</v>
       </c>
-      <c r="M119" s="2">
+      <c r="M119" s="1">
         <v>46386</v>
       </c>
       <c r="N119" t="s">
@@ -15838,7 +15812,7 @@
       <c r="L120" t="s">
         <v>722</v>
       </c>
-      <c r="M120" s="2">
+      <c r="M120" s="1">
         <v>46386</v>
       </c>
       <c r="N120" t="s">
@@ -15882,7 +15856,7 @@
       <c r="L121" t="s">
         <v>722</v>
       </c>
-      <c r="M121" s="2">
+      <c r="M121" s="1">
         <v>46386</v>
       </c>
       <c r="N121" t="s">
@@ -15926,7 +15900,7 @@
       <c r="L122" t="s">
         <v>722</v>
       </c>
-      <c r="M122" s="2">
+      <c r="M122" s="1">
         <v>46386</v>
       </c>
       <c r="N122" t="s">
@@ -15970,7 +15944,7 @@
       <c r="L123" t="s">
         <v>722</v>
       </c>
-      <c r="M123" s="2">
+      <c r="M123" s="1">
         <v>46386</v>
       </c>
       <c r="N123" t="s">
@@ -16014,7 +15988,7 @@
       <c r="L124" t="s">
         <v>722</v>
       </c>
-      <c r="M124" s="2">
+      <c r="M124" s="1">
         <v>46386</v>
       </c>
       <c r="N124" t="s">

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (19/10/2026 13:32)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2202,8 +2202,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2219,7 +2227,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2227,12 +2235,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2532,55 +2558,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2624,7 +2650,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2668,7 +2694,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2712,7 +2738,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2838,7 +2864,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2882,7 +2908,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2926,7 +2952,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2973,7 +2999,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3096,7 +3122,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -3140,7 +3166,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3184,7 +3210,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3228,7 +3254,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3275,7 +3301,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3319,7 +3345,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3445,7 +3471,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3489,7 +3515,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3574,7 +3600,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3621,7 +3647,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3668,7 +3694,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3712,7 +3738,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3756,7 +3782,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3841,7 +3867,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3926,7 +3952,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3973,7 +3999,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4017,7 +4043,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4061,7 +4087,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4146,7 +4172,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4190,7 +4216,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4234,7 +4260,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4319,7 +4345,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4363,7 +4389,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4407,7 +4433,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4451,7 +4477,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4618,7 +4644,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4662,7 +4688,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4706,7 +4732,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4750,7 +4776,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4797,7 +4823,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4841,7 +4867,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4923,7 +4949,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4967,7 +4993,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5055,7 +5081,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5099,7 +5125,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5146,7 +5172,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5190,7 +5216,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -5234,7 +5260,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5278,7 +5304,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5322,7 +5348,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5369,7 +5395,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5413,7 +5439,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5460,7 +5486,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5504,7 +5530,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5551,7 +5577,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5639,7 +5665,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5683,7 +5709,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5727,7 +5753,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5771,7 +5797,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5815,7 +5841,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5859,7 +5885,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5944,7 +5970,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5988,7 +6014,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -6032,7 +6058,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -6076,7 +6102,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -6120,7 +6146,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -6164,7 +6190,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6208,7 +6234,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6252,7 +6278,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6299,7 +6325,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6343,7 +6369,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6387,7 +6413,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6431,7 +6457,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6475,7 +6501,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6519,7 +6545,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6563,7 +6589,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6607,7 +6633,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6651,7 +6677,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6739,7 +6765,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6783,7 +6809,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6909,7 +6935,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6953,7 +6979,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6997,7 +7023,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7041,7 +7067,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7123,7 +7149,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7167,7 +7193,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7214,7 +7240,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7258,7 +7284,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7384,7 +7410,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7428,7 +7454,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7513,7 +7539,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7557,7 +7583,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7601,7 +7627,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7645,7 +7671,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7689,7 +7715,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7733,7 +7759,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7777,7 +7803,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7821,7 +7847,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7906,7 +7932,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8073,7 +8099,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8117,7 +8143,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8161,7 +8187,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8205,7 +8231,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8249,7 +8275,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8293,7 +8319,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8337,7 +8363,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8422,7 +8448,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8466,7 +8492,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8551,7 +8577,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8677,7 +8703,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8721,7 +8747,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8806,7 +8832,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8850,7 +8876,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8894,7 +8920,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8938,7 +8964,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8982,7 +9008,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -9026,7 +9052,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9070,7 +9096,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9114,7 +9140,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9199,7 +9225,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9366,7 +9392,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9410,7 +9436,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9454,7 +9480,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9498,7 +9524,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9583,7 +9609,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9627,7 +9653,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9671,7 +9697,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9715,7 +9741,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9759,7 +9785,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9803,7 +9829,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9847,7 +9873,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9891,7 +9917,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9935,7 +9961,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9979,7 +10005,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10023,7 +10049,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -10067,7 +10093,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10111,7 +10137,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10155,7 +10181,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -10199,7 +10225,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10243,7 +10269,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10287,7 +10313,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10331,7 +10357,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10375,7 +10401,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10419,7 +10445,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10463,7 +10489,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10548,7 +10574,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10633,7 +10659,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10648,55 +10674,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11065,7 +11091,7 @@
       <c r="L10" t="s">
         <v>722</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46386</v>
       </c>
       <c r="N10" t="s">
@@ -11109,7 +11135,7 @@
       <c r="L11" t="s">
         <v>722</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46386</v>
       </c>
       <c r="N11" t="s">
@@ -11317,7 +11343,7 @@
       <c r="L16" t="s">
         <v>722</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46386</v>
       </c>
       <c r="N16" t="s">
@@ -11443,7 +11469,7 @@
       <c r="L19" t="s">
         <v>722</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46386</v>
       </c>
       <c r="N19" t="s">
@@ -11487,7 +11513,7 @@
       <c r="L20" t="s">
         <v>722</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46386</v>
       </c>
       <c r="N20" t="s">
@@ -11531,7 +11557,7 @@
       <c r="L21" t="s">
         <v>722</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46386</v>
       </c>
       <c r="N21" t="s">
@@ -11698,7 +11724,7 @@
       <c r="L25" t="s">
         <v>722</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46386</v>
       </c>
       <c r="N25" t="s">
@@ -11824,7 +11850,7 @@
       <c r="L28" t="s">
         <v>722</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46386</v>
       </c>
       <c r="N28" t="s">
@@ -11909,7 +11935,7 @@
       <c r="L30" t="s">
         <v>722</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46386</v>
       </c>
       <c r="N30" t="s">
@@ -12363,7 +12389,7 @@
       <c r="L41" t="s">
         <v>722</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46386</v>
       </c>
       <c r="N41" t="s">
@@ -12448,7 +12474,7 @@
       <c r="L43" t="s">
         <v>722</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46386</v>
       </c>
       <c r="N43" t="s">
@@ -12492,7 +12518,7 @@
       <c r="L44" t="s">
         <v>722</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46386</v>
       </c>
       <c r="N44" t="s">
@@ -12536,7 +12562,7 @@
       <c r="L45" t="s">
         <v>722</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46386</v>
       </c>
       <c r="N45" t="s">
@@ -12662,7 +12688,7 @@
       <c r="L48" t="s">
         <v>722</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46386</v>
       </c>
       <c r="N48" t="s">
@@ -12706,7 +12732,7 @@
       <c r="L49" t="s">
         <v>723</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46321</v>
       </c>
       <c r="N49" t="s">
@@ -12750,7 +12776,7 @@
       <c r="L50" t="s">
         <v>723</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46321</v>
       </c>
       <c r="N50" t="s">
@@ -12794,7 +12820,7 @@
       <c r="L51" t="s">
         <v>722</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46386</v>
       </c>
       <c r="N51" t="s">
@@ -12838,7 +12864,7 @@
       <c r="L52" t="s">
         <v>722</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46386</v>
       </c>
       <c r="N52" t="s">
@@ -12882,7 +12908,7 @@
       <c r="L53" t="s">
         <v>722</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46386</v>
       </c>
       <c r="N53" t="s">
@@ -12926,7 +12952,7 @@
       <c r="L54" t="s">
         <v>722</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46386</v>
       </c>
       <c r="N54" t="s">
@@ -12970,7 +12996,7 @@
       <c r="L55" t="s">
         <v>722</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46386</v>
       </c>
       <c r="N55" t="s">
@@ -13137,7 +13163,7 @@
       <c r="L59" t="s">
         <v>722</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46386</v>
       </c>
       <c r="N59" t="s">
@@ -13263,7 +13289,7 @@
       <c r="L62" t="s">
         <v>722</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46386</v>
       </c>
       <c r="N62" t="s">
@@ -13307,7 +13333,7 @@
       <c r="L63" t="s">
         <v>722</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46386</v>
       </c>
       <c r="N63" t="s">
@@ -13351,7 +13377,7 @@
       <c r="L64" t="s">
         <v>722</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46386</v>
       </c>
       <c r="N64" t="s">
@@ -13395,7 +13421,7 @@
       <c r="L65" t="s">
         <v>722</v>
       </c>
-      <c r="M65" s="1">
+      <c r="M65" s="2">
         <v>46386</v>
       </c>
       <c r="N65" t="s">
@@ -13439,7 +13465,7 @@
       <c r="L66" t="s">
         <v>722</v>
       </c>
-      <c r="M66" s="1">
+      <c r="M66" s="2">
         <v>46386</v>
       </c>
       <c r="N66" t="s">
@@ -13483,7 +13509,7 @@
       <c r="L67" t="s">
         <v>722</v>
       </c>
-      <c r="M67" s="1">
+      <c r="M67" s="2">
         <v>46386</v>
       </c>
       <c r="N67" t="s">
@@ -13527,7 +13553,7 @@
       <c r="L68" t="s">
         <v>722</v>
       </c>
-      <c r="M68" s="1">
+      <c r="M68" s="2">
         <v>46386</v>
       </c>
       <c r="N68" t="s">
@@ -13571,7 +13597,7 @@
       <c r="L69" t="s">
         <v>722</v>
       </c>
-      <c r="M69" s="1">
+      <c r="M69" s="2">
         <v>46386</v>
       </c>
       <c r="N69" t="s">
@@ -13615,7 +13641,7 @@
       <c r="L70" t="s">
         <v>722</v>
       </c>
-      <c r="M70" s="1">
+      <c r="M70" s="2">
         <v>46386</v>
       </c>
       <c r="N70" t="s">
@@ -13659,7 +13685,7 @@
       <c r="L71" t="s">
         <v>722</v>
       </c>
-      <c r="M71" s="1">
+      <c r="M71" s="2">
         <v>46386</v>
       </c>
       <c r="N71" t="s">
@@ -13703,7 +13729,7 @@
       <c r="L72" t="s">
         <v>722</v>
       </c>
-      <c r="M72" s="1">
+      <c r="M72" s="2">
         <v>46386</v>
       </c>
       <c r="N72" t="s">
@@ -13747,7 +13773,7 @@
       <c r="L73" t="s">
         <v>722</v>
       </c>
-      <c r="M73" s="1">
+      <c r="M73" s="2">
         <v>46386</v>
       </c>
       <c r="N73" t="s">
@@ -13791,7 +13817,7 @@
       <c r="L74" t="s">
         <v>722</v>
       </c>
-      <c r="M74" s="1">
+      <c r="M74" s="2">
         <v>46386</v>
       </c>
       <c r="N74" t="s">
@@ -13835,7 +13861,7 @@
       <c r="L75" t="s">
         <v>722</v>
       </c>
-      <c r="M75" s="1">
+      <c r="M75" s="2">
         <v>46386</v>
       </c>
       <c r="N75" t="s">
@@ -13879,7 +13905,7 @@
       <c r="L76" t="s">
         <v>722</v>
       </c>
-      <c r="M76" s="1">
+      <c r="M76" s="2">
         <v>46386</v>
       </c>
       <c r="N76" t="s">
@@ -13923,7 +13949,7 @@
       <c r="L77" t="s">
         <v>722</v>
       </c>
-      <c r="M77" s="1">
+      <c r="M77" s="2">
         <v>46386</v>
       </c>
       <c r="N77" t="s">
@@ -13967,7 +13993,7 @@
       <c r="L78" t="s">
         <v>722</v>
       </c>
-      <c r="M78" s="1">
+      <c r="M78" s="2">
         <v>46386</v>
       </c>
       <c r="N78" t="s">
@@ -14011,7 +14037,7 @@
       <c r="L79" t="s">
         <v>722</v>
       </c>
-      <c r="M79" s="1">
+      <c r="M79" s="2">
         <v>46386</v>
       </c>
       <c r="N79" t="s">
@@ -14055,7 +14081,7 @@
       <c r="L80" t="s">
         <v>722</v>
       </c>
-      <c r="M80" s="1">
+      <c r="M80" s="2">
         <v>46386</v>
       </c>
       <c r="N80" t="s">
@@ -14099,7 +14125,7 @@
       <c r="L81" t="s">
         <v>722</v>
       </c>
-      <c r="M81" s="1">
+      <c r="M81" s="2">
         <v>46386</v>
       </c>
       <c r="N81" t="s">
@@ -14143,7 +14169,7 @@
       <c r="L82" t="s">
         <v>722</v>
       </c>
-      <c r="M82" s="1">
+      <c r="M82" s="2">
         <v>46386</v>
       </c>
       <c r="N82" t="s">
@@ -14187,7 +14213,7 @@
       <c r="L83" t="s">
         <v>722</v>
       </c>
-      <c r="M83" s="1">
+      <c r="M83" s="2">
         <v>46386</v>
       </c>
       <c r="N83" t="s">
@@ -14231,7 +14257,7 @@
       <c r="L84" t="s">
         <v>722</v>
       </c>
-      <c r="M84" s="1">
+      <c r="M84" s="2">
         <v>46386</v>
       </c>
       <c r="N84" t="s">
@@ -14275,7 +14301,7 @@
       <c r="L85" t="s">
         <v>722</v>
       </c>
-      <c r="M85" s="1">
+      <c r="M85" s="2">
         <v>46386</v>
       </c>
       <c r="N85" t="s">
@@ -14319,7 +14345,7 @@
       <c r="L86" t="s">
         <v>722</v>
       </c>
-      <c r="M86" s="1">
+      <c r="M86" s="2">
         <v>46386</v>
       </c>
       <c r="N86" t="s">
@@ -14363,7 +14389,7 @@
       <c r="L87" t="s">
         <v>722</v>
       </c>
-      <c r="M87" s="1">
+      <c r="M87" s="2">
         <v>46386</v>
       </c>
       <c r="N87" t="s">
@@ -14407,7 +14433,7 @@
       <c r="L88" t="s">
         <v>722</v>
       </c>
-      <c r="M88" s="1">
+      <c r="M88" s="2">
         <v>46386</v>
       </c>
       <c r="N88" t="s">
@@ -14451,7 +14477,7 @@
       <c r="L89" t="s">
         <v>722</v>
       </c>
-      <c r="M89" s="1">
+      <c r="M89" s="2">
         <v>46386</v>
       </c>
       <c r="N89" t="s">
@@ -14495,7 +14521,7 @@
       <c r="L90" t="s">
         <v>722</v>
       </c>
-      <c r="M90" s="1">
+      <c r="M90" s="2">
         <v>46386</v>
       </c>
       <c r="N90" t="s">
@@ -14580,7 +14606,7 @@
       <c r="L92" t="s">
         <v>722</v>
       </c>
-      <c r="M92" s="1">
+      <c r="M92" s="2">
         <v>46386</v>
       </c>
       <c r="N92" t="s">
@@ -14624,7 +14650,7 @@
       <c r="L93" t="s">
         <v>722</v>
       </c>
-      <c r="M93" s="1">
+      <c r="M93" s="2">
         <v>46386</v>
       </c>
       <c r="N93" t="s">
@@ -14668,7 +14694,7 @@
       <c r="L94" t="s">
         <v>722</v>
       </c>
-      <c r="M94" s="1">
+      <c r="M94" s="2">
         <v>46386</v>
       </c>
       <c r="N94" t="s">
@@ -14712,7 +14738,7 @@
       <c r="L95" t="s">
         <v>722</v>
       </c>
-      <c r="M95" s="1">
+      <c r="M95" s="2">
         <v>46386</v>
       </c>
       <c r="N95" t="s">
@@ -14756,7 +14782,7 @@
       <c r="L96" t="s">
         <v>722</v>
       </c>
-      <c r="M96" s="1">
+      <c r="M96" s="2">
         <v>46386</v>
       </c>
       <c r="N96" t="s">
@@ -14800,7 +14826,7 @@
       <c r="L97" t="s">
         <v>722</v>
       </c>
-      <c r="M97" s="1">
+      <c r="M97" s="2">
         <v>46386</v>
       </c>
       <c r="N97" t="s">
@@ -14844,7 +14870,7 @@
       <c r="L98" t="s">
         <v>722</v>
       </c>
-      <c r="M98" s="1">
+      <c r="M98" s="2">
         <v>46386</v>
       </c>
       <c r="N98" t="s">
@@ -14888,7 +14914,7 @@
       <c r="L99" t="s">
         <v>722</v>
       </c>
-      <c r="M99" s="1">
+      <c r="M99" s="2">
         <v>46386</v>
       </c>
       <c r="N99" t="s">
@@ -14932,7 +14958,7 @@
       <c r="L100" t="s">
         <v>722</v>
       </c>
-      <c r="M100" s="1">
+      <c r="M100" s="2">
         <v>46386</v>
       </c>
       <c r="N100" t="s">
@@ -14976,7 +15002,7 @@
       <c r="L101" t="s">
         <v>722</v>
       </c>
-      <c r="M101" s="1">
+      <c r="M101" s="2">
         <v>46386</v>
       </c>
       <c r="N101" t="s">
@@ -15020,7 +15046,7 @@
       <c r="L102" t="s">
         <v>722</v>
       </c>
-      <c r="M102" s="1">
+      <c r="M102" s="2">
         <v>46386</v>
       </c>
       <c r="N102" t="s">
@@ -15064,7 +15090,7 @@
       <c r="L103" t="s">
         <v>722</v>
       </c>
-      <c r="M103" s="1">
+      <c r="M103" s="2">
         <v>46386</v>
       </c>
       <c r="N103" t="s">
@@ -15108,7 +15134,7 @@
       <c r="L104" t="s">
         <v>722</v>
       </c>
-      <c r="M104" s="1">
+      <c r="M104" s="2">
         <v>46386</v>
       </c>
       <c r="N104" t="s">
@@ -15152,7 +15178,7 @@
       <c r="L105" t="s">
         <v>722</v>
       </c>
-      <c r="M105" s="1">
+      <c r="M105" s="2">
         <v>46386</v>
       </c>
       <c r="N105" t="s">
@@ -15196,7 +15222,7 @@
       <c r="L106" t="s">
         <v>722</v>
       </c>
-      <c r="M106" s="1">
+      <c r="M106" s="2">
         <v>46386</v>
       </c>
       <c r="N106" t="s">
@@ -15240,7 +15266,7 @@
       <c r="L107" t="s">
         <v>722</v>
       </c>
-      <c r="M107" s="1">
+      <c r="M107" s="2">
         <v>46386</v>
       </c>
       <c r="N107" t="s">
@@ -15284,7 +15310,7 @@
       <c r="L108" t="s">
         <v>722</v>
       </c>
-      <c r="M108" s="1">
+      <c r="M108" s="2">
         <v>46386</v>
       </c>
       <c r="N108" t="s">
@@ -15328,7 +15354,7 @@
       <c r="L109" t="s">
         <v>722</v>
       </c>
-      <c r="M109" s="1">
+      <c r="M109" s="2">
         <v>46386</v>
       </c>
       <c r="N109" t="s">
@@ -15372,7 +15398,7 @@
       <c r="L110" t="s">
         <v>722</v>
       </c>
-      <c r="M110" s="1">
+      <c r="M110" s="2">
         <v>46386</v>
       </c>
       <c r="N110" t="s">
@@ -15416,7 +15442,7 @@
       <c r="L111" t="s">
         <v>722</v>
       </c>
-      <c r="M111" s="1">
+      <c r="M111" s="2">
         <v>46386</v>
       </c>
       <c r="N111" t="s">
@@ -15460,7 +15486,7 @@
       <c r="L112" t="s">
         <v>722</v>
       </c>
-      <c r="M112" s="1">
+      <c r="M112" s="2">
         <v>46386</v>
       </c>
       <c r="N112" t="s">
@@ -15504,7 +15530,7 @@
       <c r="L113" t="s">
         <v>722</v>
       </c>
-      <c r="M113" s="1">
+      <c r="M113" s="2">
         <v>46386</v>
       </c>
       <c r="N113" t="s">
@@ -15548,7 +15574,7 @@
       <c r="L114" t="s">
         <v>722</v>
       </c>
-      <c r="M114" s="1">
+      <c r="M114" s="2">
         <v>46386</v>
       </c>
       <c r="N114" t="s">
@@ -15592,7 +15618,7 @@
       <c r="L115" t="s">
         <v>722</v>
       </c>
-      <c r="M115" s="1">
+      <c r="M115" s="2">
         <v>46386</v>
       </c>
       <c r="N115" t="s">
@@ -15636,7 +15662,7 @@
       <c r="L116" t="s">
         <v>722</v>
       </c>
-      <c r="M116" s="1">
+      <c r="M116" s="2">
         <v>46386</v>
       </c>
       <c r="N116" t="s">
@@ -15680,7 +15706,7 @@
       <c r="L117" t="s">
         <v>722</v>
       </c>
-      <c r="M117" s="1">
+      <c r="M117" s="2">
         <v>46386</v>
       </c>
       <c r="N117" t="s">
@@ -15724,7 +15750,7 @@
       <c r="L118" t="s">
         <v>722</v>
       </c>
-      <c r="M118" s="1">
+      <c r="M118" s="2">
         <v>46386</v>
       </c>
       <c r="N118" t="s">
@@ -15768,7 +15794,7 @@
       <c r="L119" t="s">
         <v>722</v>
       </c>
-      <c r="M119" s="1">
+      <c r="M119" s="2">
         <v>46386</v>
       </c>
       <c r="N119" t="s">
@@ -15812,7 +15838,7 @@
       <c r="L120" t="s">
         <v>722</v>
       </c>
-      <c r="M120" s="1">
+      <c r="M120" s="2">
         <v>46386</v>
       </c>
       <c r="N120" t="s">
@@ -15856,7 +15882,7 @@
       <c r="L121" t="s">
         <v>722</v>
       </c>
-      <c r="M121" s="1">
+      <c r="M121" s="2">
         <v>46386</v>
       </c>
       <c r="N121" t="s">
@@ -15900,7 +15926,7 @@
       <c r="L122" t="s">
         <v>722</v>
       </c>
-      <c r="M122" s="1">
+      <c r="M122" s="2">
         <v>46386</v>
       </c>
       <c r="N122" t="s">
@@ -15944,7 +15970,7 @@
       <c r="L123" t="s">
         <v>722</v>
       </c>
-      <c r="M123" s="1">
+      <c r="M123" s="2">
         <v>46386</v>
       </c>
       <c r="N123" t="s">
@@ -15988,7 +16014,7 @@
       <c r="L124" t="s">
         <v>722</v>
       </c>
-      <c r="M124" s="1">
+      <c r="M124" s="2">
         <v>46386</v>
       </c>
       <c r="N124" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (19/10/2026 13:34)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3126" uniqueCount="726">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3126" uniqueCount="727">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -2183,13 +2183,16 @@
     <t>Selecionada em Plano</t>
   </si>
   <si>
+    <t>Aguardando Intenção de Recurso</t>
+  </si>
+  <si>
+    <t>Mapa Gerado</t>
+  </si>
+  <si>
+    <t>Em Discrepância</t>
+  </si>
+  <si>
     <t>Validada</t>
-  </si>
-  <si>
-    <t>Mapa Gerado</t>
-  </si>
-  <si>
-    <t>Em Discrepância</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10878,13 +10881,13 @@
         <v>720</v>
       </c>
       <c r="J5" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K5" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="L5" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="N5" t="s">
         <v>395</v>
@@ -11083,19 +11086,19 @@
         <v>721</v>
       </c>
       <c r="J10" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K10" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L10" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M10" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N10" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -11127,19 +11130,19 @@
         <v>721</v>
       </c>
       <c r="J11" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K11" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L11" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M11" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N11" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -11335,19 +11338,19 @@
         <v>721</v>
       </c>
       <c r="J16" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K16" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L16" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M16" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N16" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -11461,19 +11464,19 @@
         <v>721</v>
       </c>
       <c r="J19" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K19" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L19" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M19" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N19" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11505,19 +11508,19 @@
         <v>721</v>
       </c>
       <c r="J20" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K20" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L20" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M20" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N20" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11546,22 +11549,22 @@
         <v>752.6</v>
       </c>
       <c r="I21" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J21" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K21" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L21" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M21" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N21" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11716,19 +11719,19 @@
         <v>721</v>
       </c>
       <c r="J25" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K25" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L25" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M25" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N25" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11839,22 +11842,22 @@
         <v>3991.71</v>
       </c>
       <c r="I28" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J28" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K28" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L28" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M28" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N28" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11924,22 +11927,22 @@
         <v>10666.22</v>
       </c>
       <c r="I30" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J30" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K30" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L30" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M30" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N30" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -12378,22 +12381,22 @@
         <v>9259.959999999999</v>
       </c>
       <c r="I41" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J41" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K41" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L41" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M41" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N41" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -12466,19 +12469,19 @@
         <v>721</v>
       </c>
       <c r="J43" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K43" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L43" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M43" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N43" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12510,19 +12513,19 @@
         <v>721</v>
       </c>
       <c r="J44" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K44" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L44" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M44" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N44" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12554,19 +12557,19 @@
         <v>721</v>
       </c>
       <c r="J45" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K45" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L45" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M45" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N45" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12680,19 +12683,19 @@
         <v>721</v>
       </c>
       <c r="J48" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K48" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L48" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M48" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N48" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12721,7 +12724,7 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="J49" t="s">
         <v>723</v>
@@ -12733,10 +12736,10 @@
         <v>723</v>
       </c>
       <c r="M49" s="2">
-        <v>46321</v>
+        <v>46324</v>
       </c>
       <c r="N49" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12777,10 +12780,10 @@
         <v>723</v>
       </c>
       <c r="M50" s="2">
-        <v>46321</v>
+        <v>46324</v>
       </c>
       <c r="N50" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12809,22 +12812,22 @@
         <v>1232.68</v>
       </c>
       <c r="I51" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J51" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K51" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L51" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M51" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N51" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12853,22 +12856,22 @@
         <v>802.84</v>
       </c>
       <c r="I52" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J52" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K52" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L52" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M52" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N52" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12897,22 +12900,22 @@
         <v>819.26</v>
       </c>
       <c r="I53" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J53" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K53" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L53" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M53" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N53" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12944,19 +12947,19 @@
         <v>721</v>
       </c>
       <c r="J54" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K54" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L54" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M54" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N54" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12985,22 +12988,22 @@
         <v>84382.42999999999</v>
       </c>
       <c r="I55" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J55" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K55" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L55" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M55" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N55" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -13155,19 +13158,19 @@
         <v>721</v>
       </c>
       <c r="J59" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K59" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L59" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M59" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N59" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -13281,19 +13284,19 @@
         <v>721</v>
       </c>
       <c r="J62" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K62" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L62" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M62" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N62" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="63" spans="1:14">
@@ -13325,19 +13328,19 @@
         <v>721</v>
       </c>
       <c r="J63" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K63" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L63" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M63" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N63" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="64" spans="1:14">
@@ -13369,19 +13372,19 @@
         <v>721</v>
       </c>
       <c r="J64" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K64" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L64" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M64" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N64" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="65" spans="1:14">
@@ -13413,19 +13416,19 @@
         <v>721</v>
       </c>
       <c r="J65" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K65" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L65" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M65" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N65" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="66" spans="1:14">
@@ -13457,19 +13460,19 @@
         <v>721</v>
       </c>
       <c r="J66" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K66" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L66" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M66" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N66" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="67" spans="1:14">
@@ -13501,19 +13504,19 @@
         <v>721</v>
       </c>
       <c r="J67" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K67" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L67" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M67" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N67" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="68" spans="1:14">
@@ -13545,19 +13548,19 @@
         <v>721</v>
       </c>
       <c r="J68" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K68" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L68" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M68" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N68" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="69" spans="1:14">
@@ -13589,19 +13592,19 @@
         <v>721</v>
       </c>
       <c r="J69" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K69" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L69" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M69" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N69" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="70" spans="1:14">
@@ -13633,19 +13636,19 @@
         <v>721</v>
       </c>
       <c r="J70" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K70" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L70" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M70" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N70" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="71" spans="1:14">
@@ -13677,19 +13680,19 @@
         <v>721</v>
       </c>
       <c r="J71" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K71" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L71" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M71" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N71" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="72" spans="1:14">
@@ -13721,19 +13724,19 @@
         <v>721</v>
       </c>
       <c r="J72" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K72" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L72" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M72" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N72" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="73" spans="1:14">
@@ -13765,19 +13768,19 @@
         <v>721</v>
       </c>
       <c r="J73" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K73" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L73" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M73" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N73" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="74" spans="1:14">
@@ -13809,19 +13812,19 @@
         <v>721</v>
       </c>
       <c r="J74" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K74" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L74" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M74" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N74" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="75" spans="1:14">
@@ -13850,22 +13853,22 @@
         <v>1001.2</v>
       </c>
       <c r="I75" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J75" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K75" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L75" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M75" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N75" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="76" spans="1:14">
@@ -13894,22 +13897,22 @@
         <v>205591.3</v>
       </c>
       <c r="I76" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J76" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K76" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L76" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M76" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N76" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="77" spans="1:14">
@@ -13941,19 +13944,19 @@
         <v>721</v>
       </c>
       <c r="J77" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K77" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L77" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M77" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N77" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="78" spans="1:14">
@@ -13985,19 +13988,19 @@
         <v>721</v>
       </c>
       <c r="J78" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K78" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L78" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M78" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N78" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="79" spans="1:14">
@@ -14029,19 +14032,19 @@
         <v>721</v>
       </c>
       <c r="J79" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K79" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L79" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M79" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N79" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="80" spans="1:14">
@@ -14073,19 +14076,19 @@
         <v>721</v>
       </c>
       <c r="J80" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K80" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L80" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M80" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N80" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="81" spans="1:14">
@@ -14114,22 +14117,22 @@
         <v>1592.82</v>
       </c>
       <c r="I81" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J81" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K81" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L81" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M81" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N81" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="82" spans="1:14">
@@ -14161,19 +14164,19 @@
         <v>721</v>
       </c>
       <c r="J82" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K82" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L82" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M82" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N82" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="83" spans="1:14">
@@ -14205,19 +14208,19 @@
         <v>721</v>
       </c>
       <c r="J83" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K83" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L83" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M83" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N83" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="84" spans="1:14">
@@ -14249,19 +14252,19 @@
         <v>721</v>
       </c>
       <c r="J84" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K84" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L84" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M84" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N84" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="85" spans="1:14">
@@ -14293,19 +14296,19 @@
         <v>721</v>
       </c>
       <c r="J85" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K85" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L85" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M85" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N85" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="86" spans="1:14">
@@ -14337,19 +14340,19 @@
         <v>721</v>
       </c>
       <c r="J86" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K86" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L86" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M86" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N86" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="87" spans="1:14">
@@ -14381,19 +14384,19 @@
         <v>721</v>
       </c>
       <c r="J87" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K87" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L87" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M87" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N87" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="88" spans="1:14">
@@ -14422,22 +14425,22 @@
         <v>2360</v>
       </c>
       <c r="I88" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J88" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K88" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L88" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M88" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N88" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="89" spans="1:14">
@@ -14469,19 +14472,19 @@
         <v>721</v>
       </c>
       <c r="J89" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K89" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L89" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M89" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N89" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="90" spans="1:14">
@@ -14510,22 +14513,22 @@
         <v>265</v>
       </c>
       <c r="I90" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J90" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K90" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L90" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M90" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N90" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="91" spans="1:14">
@@ -14598,19 +14601,19 @@
         <v>721</v>
       </c>
       <c r="J92" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K92" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L92" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M92" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N92" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="93" spans="1:14">
@@ -14639,22 +14642,22 @@
         <v>735.79</v>
       </c>
       <c r="I93" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J93" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K93" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L93" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M93" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N93" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="94" spans="1:14">
@@ -14683,22 +14686,22 @@
         <v>7431.24</v>
       </c>
       <c r="I94" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J94" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K94" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L94" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M94" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N94" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="95" spans="1:14">
@@ -14727,22 +14730,22 @@
         <v>48912.85</v>
       </c>
       <c r="I95" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J95" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K95" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L95" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M95" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N95" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="96" spans="1:14">
@@ -14771,22 +14774,22 @@
         <v>8115.6</v>
       </c>
       <c r="I96" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J96" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K96" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L96" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M96" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N96" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="97" spans="1:14">
@@ -14818,19 +14821,19 @@
         <v>721</v>
       </c>
       <c r="J97" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K97" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L97" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M97" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N97" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="98" spans="1:14">
@@ -14862,19 +14865,19 @@
         <v>721</v>
       </c>
       <c r="J98" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K98" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L98" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M98" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N98" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="99" spans="1:14">
@@ -14906,19 +14909,19 @@
         <v>721</v>
       </c>
       <c r="J99" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K99" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L99" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M99" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N99" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="100" spans="1:14">
@@ -14947,22 +14950,22 @@
         <v>1768.41</v>
       </c>
       <c r="I100" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J100" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K100" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L100" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M100" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N100" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="101" spans="1:14">
@@ -14994,19 +14997,19 @@
         <v>721</v>
       </c>
       <c r="J101" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K101" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L101" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M101" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N101" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="102" spans="1:14">
@@ -15038,19 +15041,19 @@
         <v>721</v>
       </c>
       <c r="J102" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K102" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L102" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M102" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N102" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="103" spans="1:14">
@@ -15079,22 +15082,22 @@
         <v>7375.36</v>
       </c>
       <c r="I103" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J103" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K103" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L103" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M103" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N103" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="104" spans="1:14">
@@ -15123,22 +15126,22 @@
         <v>29526.48</v>
       </c>
       <c r="I104" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J104" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K104" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L104" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M104" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N104" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="105" spans="1:14">
@@ -15167,22 +15170,22 @@
         <v>1578.63</v>
       </c>
       <c r="I105" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J105" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K105" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L105" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M105" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N105" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="106" spans="1:14">
@@ -15211,22 +15214,22 @@
         <v>17442</v>
       </c>
       <c r="I106" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J106" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K106" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L106" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M106" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N106" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="107" spans="1:14">
@@ -15255,22 +15258,22 @@
         <v>3100.94</v>
       </c>
       <c r="I107" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J107" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K107" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L107" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M107" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N107" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="108" spans="1:14">
@@ -15299,22 +15302,22 @@
         <v>20942.58</v>
       </c>
       <c r="I108" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J108" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K108" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L108" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M108" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N108" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="109" spans="1:14">
@@ -15343,22 +15346,22 @@
         <v>678.9</v>
       </c>
       <c r="I109" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J109" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K109" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L109" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M109" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N109" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="110" spans="1:14">
@@ -15390,19 +15393,19 @@
         <v>721</v>
       </c>
       <c r="J110" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K110" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L110" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M110" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N110" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="111" spans="1:14">
@@ -15434,19 +15437,19 @@
         <v>721</v>
       </c>
       <c r="J111" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K111" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L111" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M111" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N111" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="112" spans="1:14">
@@ -15478,19 +15481,19 @@
         <v>721</v>
       </c>
       <c r="J112" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K112" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L112" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M112" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N112" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="113" spans="1:14">
@@ -15522,19 +15525,19 @@
         <v>721</v>
       </c>
       <c r="J113" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K113" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L113" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M113" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N113" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="114" spans="1:14">
@@ -15566,19 +15569,19 @@
         <v>721</v>
       </c>
       <c r="J114" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K114" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L114" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M114" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N114" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="115" spans="1:14">
@@ -15610,19 +15613,19 @@
         <v>721</v>
       </c>
       <c r="J115" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K115" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L115" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M115" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N115" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="116" spans="1:14">
@@ -15654,19 +15657,19 @@
         <v>721</v>
       </c>
       <c r="J116" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K116" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L116" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M116" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N116" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="117" spans="1:14">
@@ -15698,19 +15701,19 @@
         <v>721</v>
       </c>
       <c r="J117" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K117" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L117" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M117" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N117" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="118" spans="1:14">
@@ -15742,19 +15745,19 @@
         <v>721</v>
       </c>
       <c r="J118" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K118" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L118" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M118" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N118" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="119" spans="1:14">
@@ -15783,22 +15786,22 @@
         <v>10935.84</v>
       </c>
       <c r="I119" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J119" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K119" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L119" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M119" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N119" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="120" spans="1:14">
@@ -15830,19 +15833,19 @@
         <v>721</v>
       </c>
       <c r="J120" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K120" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L120" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M120" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N120" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="121" spans="1:14">
@@ -15871,22 +15874,22 @@
         <v>105689.28</v>
       </c>
       <c r="I121" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J121" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K121" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L121" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M121" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N121" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="122" spans="1:14">
@@ -15915,22 +15918,22 @@
         <v>14929.78</v>
       </c>
       <c r="I122" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J122" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K122" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L122" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M122" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N122" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="123" spans="1:14">
@@ -15959,22 +15962,22 @@
         <v>710</v>
       </c>
       <c r="I123" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J123" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K123" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L123" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M123" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N123" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="124" spans="1:14">
@@ -16003,22 +16006,22 @@
         <v>7845.8</v>
       </c>
       <c r="I124" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J124" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="K124" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="L124" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="M124" s="2">
-        <v>46386</v>
+        <v>46389</v>
       </c>
       <c r="N124" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (19/10/2026 14:27)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2205,16 +2205,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2230,7 +2222,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2238,30 +2230,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2561,55 +2535,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2653,7 +2627,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2697,7 +2671,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2741,7 +2715,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2911,7 +2885,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2955,7 +2929,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -3002,7 +2976,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3125,7 +3099,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -3169,7 +3143,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3213,7 +3187,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3257,7 +3231,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3304,7 +3278,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3348,7 +3322,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3474,7 +3448,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3518,7 +3492,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3603,7 +3577,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3650,7 +3624,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3697,7 +3671,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3741,7 +3715,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3785,7 +3759,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3870,7 +3844,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3955,7 +3929,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -4002,7 +3976,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4046,7 +4020,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4090,7 +4064,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4175,7 +4149,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4219,7 +4193,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4263,7 +4237,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4348,7 +4322,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4392,7 +4366,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4436,7 +4410,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4480,7 +4454,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4647,7 +4621,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4691,7 +4665,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4735,7 +4709,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4779,7 +4753,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4826,7 +4800,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4870,7 +4844,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4952,7 +4926,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4996,7 +4970,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5084,7 +5058,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5128,7 +5102,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5175,7 +5149,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5219,7 +5193,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -5263,7 +5237,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5307,7 +5281,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5351,7 +5325,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5398,7 +5372,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5442,7 +5416,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5489,7 +5463,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5533,7 +5507,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5580,7 +5554,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5668,7 +5642,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5712,7 +5686,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5756,7 +5730,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5800,7 +5774,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5844,7 +5818,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5888,7 +5862,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5973,7 +5947,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6017,7 +5991,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -6061,7 +6035,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -6105,7 +6079,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -6149,7 +6123,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -6193,7 +6167,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6237,7 +6211,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6281,7 +6255,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6328,7 +6302,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6372,7 +6346,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6416,7 +6390,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6460,7 +6434,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6504,7 +6478,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6592,7 +6566,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6636,7 +6610,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6680,7 +6654,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6768,7 +6742,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6812,7 +6786,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6938,7 +6912,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6982,7 +6956,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7026,7 +7000,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7070,7 +7044,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7152,7 +7126,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7196,7 +7170,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7243,7 +7217,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7287,7 +7261,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7413,7 +7387,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7457,7 +7431,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7542,7 +7516,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7586,7 +7560,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7630,7 +7604,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7674,7 +7648,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7718,7 +7692,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7762,7 +7736,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7806,7 +7780,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7850,7 +7824,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7935,7 +7909,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8102,7 +8076,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8146,7 +8120,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8190,7 +8164,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8234,7 +8208,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8278,7 +8252,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8322,7 +8296,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8366,7 +8340,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8451,7 +8425,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8495,7 +8469,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8580,7 +8554,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8706,7 +8680,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8750,7 +8724,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8835,7 +8809,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8879,7 +8853,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8923,7 +8897,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8967,7 +8941,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -9011,7 +8985,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -9055,7 +9029,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9099,7 +9073,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9143,7 +9117,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9228,7 +9202,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9395,7 +9369,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9439,7 +9413,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9483,7 +9457,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9527,7 +9501,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9612,7 +9586,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9656,7 +9630,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9700,7 +9674,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9744,7 +9718,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9788,7 +9762,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9832,7 +9806,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9876,7 +9850,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9920,7 +9894,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9964,7 +9938,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10008,7 +9982,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10052,7 +10026,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -10096,7 +10070,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10140,7 +10114,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10184,7 +10158,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -10228,7 +10202,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10272,7 +10246,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10316,7 +10290,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10360,7 +10334,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10404,7 +10378,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10448,7 +10422,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10492,7 +10466,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10577,7 +10551,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10662,7 +10636,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10677,55 +10651,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11094,7 +11068,7 @@
       <c r="L10" t="s">
         <v>725</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46389</v>
       </c>
       <c r="N10" t="s">
@@ -11138,7 +11112,7 @@
       <c r="L11" t="s">
         <v>725</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46389</v>
       </c>
       <c r="N11" t="s">
@@ -11346,7 +11320,7 @@
       <c r="L16" t="s">
         <v>725</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46389</v>
       </c>
       <c r="N16" t="s">
@@ -11472,7 +11446,7 @@
       <c r="L19" t="s">
         <v>725</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46389</v>
       </c>
       <c r="N19" t="s">
@@ -11516,7 +11490,7 @@
       <c r="L20" t="s">
         <v>725</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46389</v>
       </c>
       <c r="N20" t="s">
@@ -11560,7 +11534,7 @@
       <c r="L21" t="s">
         <v>725</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46389</v>
       </c>
       <c r="N21" t="s">
@@ -11727,7 +11701,7 @@
       <c r="L25" t="s">
         <v>725</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46389</v>
       </c>
       <c r="N25" t="s">
@@ -11853,7 +11827,7 @@
       <c r="L28" t="s">
         <v>725</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46389</v>
       </c>
       <c r="N28" t="s">
@@ -11938,7 +11912,7 @@
       <c r="L30" t="s">
         <v>725</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46389</v>
       </c>
       <c r="N30" t="s">
@@ -12392,7 +12366,7 @@
       <c r="L41" t="s">
         <v>725</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46389</v>
       </c>
       <c r="N41" t="s">
@@ -12477,7 +12451,7 @@
       <c r="L43" t="s">
         <v>725</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46389</v>
       </c>
       <c r="N43" t="s">
@@ -12521,7 +12495,7 @@
       <c r="L44" t="s">
         <v>725</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46389</v>
       </c>
       <c r="N44" t="s">
@@ -12565,7 +12539,7 @@
       <c r="L45" t="s">
         <v>725</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46389</v>
       </c>
       <c r="N45" t="s">
@@ -12691,7 +12665,7 @@
       <c r="L48" t="s">
         <v>725</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46389</v>
       </c>
       <c r="N48" t="s">
@@ -12735,7 +12709,7 @@
       <c r="L49" t="s">
         <v>723</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46324</v>
       </c>
       <c r="N49" t="s">
@@ -12779,7 +12753,7 @@
       <c r="L50" t="s">
         <v>723</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46324</v>
       </c>
       <c r="N50" t="s">
@@ -12823,7 +12797,7 @@
       <c r="L51" t="s">
         <v>725</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46389</v>
       </c>
       <c r="N51" t="s">
@@ -12867,7 +12841,7 @@
       <c r="L52" t="s">
         <v>725</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46389</v>
       </c>
       <c r="N52" t="s">
@@ -12911,7 +12885,7 @@
       <c r="L53" t="s">
         <v>725</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46389</v>
       </c>
       <c r="N53" t="s">
@@ -12955,7 +12929,7 @@
       <c r="L54" t="s">
         <v>725</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46389</v>
       </c>
       <c r="N54" t="s">
@@ -12999,7 +12973,7 @@
       <c r="L55" t="s">
         <v>725</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46389</v>
       </c>
       <c r="N55" t="s">
@@ -13166,7 +13140,7 @@
       <c r="L59" t="s">
         <v>725</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46389</v>
       </c>
       <c r="N59" t="s">
@@ -13292,7 +13266,7 @@
       <c r="L62" t="s">
         <v>725</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46389</v>
       </c>
       <c r="N62" t="s">
@@ -13336,7 +13310,7 @@
       <c r="L63" t="s">
         <v>725</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46389</v>
       </c>
       <c r="N63" t="s">
@@ -13380,7 +13354,7 @@
       <c r="L64" t="s">
         <v>725</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46389</v>
       </c>
       <c r="N64" t="s">
@@ -13424,7 +13398,7 @@
       <c r="L65" t="s">
         <v>725</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="1">
         <v>46389</v>
       </c>
       <c r="N65" t="s">
@@ -13468,7 +13442,7 @@
       <c r="L66" t="s">
         <v>725</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="1">
         <v>46389</v>
       </c>
       <c r="N66" t="s">
@@ -13512,7 +13486,7 @@
       <c r="L67" t="s">
         <v>725</v>
       </c>
-      <c r="M67" s="2">
+      <c r="M67" s="1">
         <v>46389</v>
       </c>
       <c r="N67" t="s">
@@ -13556,7 +13530,7 @@
       <c r="L68" t="s">
         <v>725</v>
       </c>
-      <c r="M68" s="2">
+      <c r="M68" s="1">
         <v>46389</v>
       </c>
       <c r="N68" t="s">
@@ -13600,7 +13574,7 @@
       <c r="L69" t="s">
         <v>725</v>
       </c>
-      <c r="M69" s="2">
+      <c r="M69" s="1">
         <v>46389</v>
       </c>
       <c r="N69" t="s">
@@ -13644,7 +13618,7 @@
       <c r="L70" t="s">
         <v>725</v>
       </c>
-      <c r="M70" s="2">
+      <c r="M70" s="1">
         <v>46389</v>
       </c>
       <c r="N70" t="s">
@@ -13688,7 +13662,7 @@
       <c r="L71" t="s">
         <v>725</v>
       </c>
-      <c r="M71" s="2">
+      <c r="M71" s="1">
         <v>46389</v>
       </c>
       <c r="N71" t="s">
@@ -13732,7 +13706,7 @@
       <c r="L72" t="s">
         <v>725</v>
       </c>
-      <c r="M72" s="2">
+      <c r="M72" s="1">
         <v>46389</v>
       </c>
       <c r="N72" t="s">
@@ -13776,7 +13750,7 @@
       <c r="L73" t="s">
         <v>725</v>
       </c>
-      <c r="M73" s="2">
+      <c r="M73" s="1">
         <v>46389</v>
       </c>
       <c r="N73" t="s">
@@ -13820,7 +13794,7 @@
       <c r="L74" t="s">
         <v>725</v>
       </c>
-      <c r="M74" s="2">
+      <c r="M74" s="1">
         <v>46389</v>
       </c>
       <c r="N74" t="s">
@@ -13864,7 +13838,7 @@
       <c r="L75" t="s">
         <v>725</v>
       </c>
-      <c r="M75" s="2">
+      <c r="M75" s="1">
         <v>46389</v>
       </c>
       <c r="N75" t="s">
@@ -13908,7 +13882,7 @@
       <c r="L76" t="s">
         <v>725</v>
       </c>
-      <c r="M76" s="2">
+      <c r="M76" s="1">
         <v>46389</v>
       </c>
       <c r="N76" t="s">
@@ -13952,7 +13926,7 @@
       <c r="L77" t="s">
         <v>725</v>
       </c>
-      <c r="M77" s="2">
+      <c r="M77" s="1">
         <v>46389</v>
       </c>
       <c r="N77" t="s">
@@ -13996,7 +13970,7 @@
       <c r="L78" t="s">
         <v>725</v>
       </c>
-      <c r="M78" s="2">
+      <c r="M78" s="1">
         <v>46389</v>
       </c>
       <c r="N78" t="s">
@@ -14040,7 +14014,7 @@
       <c r="L79" t="s">
         <v>725</v>
       </c>
-      <c r="M79" s="2">
+      <c r="M79" s="1">
         <v>46389</v>
       </c>
       <c r="N79" t="s">
@@ -14084,7 +14058,7 @@
       <c r="L80" t="s">
         <v>725</v>
       </c>
-      <c r="M80" s="2">
+      <c r="M80" s="1">
         <v>46389</v>
       </c>
       <c r="N80" t="s">
@@ -14128,7 +14102,7 @@
       <c r="L81" t="s">
         <v>725</v>
       </c>
-      <c r="M81" s="2">
+      <c r="M81" s="1">
         <v>46389</v>
       </c>
       <c r="N81" t="s">
@@ -14172,7 +14146,7 @@
       <c r="L82" t="s">
         <v>725</v>
       </c>
-      <c r="M82" s="2">
+      <c r="M82" s="1">
         <v>46389</v>
       </c>
       <c r="N82" t="s">
@@ -14216,7 +14190,7 @@
       <c r="L83" t="s">
         <v>725</v>
       </c>
-      <c r="M83" s="2">
+      <c r="M83" s="1">
         <v>46389</v>
       </c>
       <c r="N83" t="s">
@@ -14260,7 +14234,7 @@
       <c r="L84" t="s">
         <v>725</v>
       </c>
-      <c r="M84" s="2">
+      <c r="M84" s="1">
         <v>46389</v>
       </c>
       <c r="N84" t="s">
@@ -14304,7 +14278,7 @@
       <c r="L85" t="s">
         <v>725</v>
       </c>
-      <c r="M85" s="2">
+      <c r="M85" s="1">
         <v>46389</v>
       </c>
       <c r="N85" t="s">
@@ -14348,7 +14322,7 @@
       <c r="L86" t="s">
         <v>725</v>
       </c>
-      <c r="M86" s="2">
+      <c r="M86" s="1">
         <v>46389</v>
       </c>
       <c r="N86" t="s">
@@ -14392,7 +14366,7 @@
       <c r="L87" t="s">
         <v>725</v>
       </c>
-      <c r="M87" s="2">
+      <c r="M87" s="1">
         <v>46389</v>
       </c>
       <c r="N87" t="s">
@@ -14436,7 +14410,7 @@
       <c r="L88" t="s">
         <v>725</v>
       </c>
-      <c r="M88" s="2">
+      <c r="M88" s="1">
         <v>46389</v>
       </c>
       <c r="N88" t="s">
@@ -14480,7 +14454,7 @@
       <c r="L89" t="s">
         <v>725</v>
       </c>
-      <c r="M89" s="2">
+      <c r="M89" s="1">
         <v>46389</v>
       </c>
       <c r="N89" t="s">
@@ -14524,7 +14498,7 @@
       <c r="L90" t="s">
         <v>725</v>
       </c>
-      <c r="M90" s="2">
+      <c r="M90" s="1">
         <v>46389</v>
       </c>
       <c r="N90" t="s">
@@ -14609,7 +14583,7 @@
       <c r="L92" t="s">
         <v>725</v>
       </c>
-      <c r="M92" s="2">
+      <c r="M92" s="1">
         <v>46389</v>
       </c>
       <c r="N92" t="s">
@@ -14653,7 +14627,7 @@
       <c r="L93" t="s">
         <v>725</v>
       </c>
-      <c r="M93" s="2">
+      <c r="M93" s="1">
         <v>46389</v>
       </c>
       <c r="N93" t="s">
@@ -14697,7 +14671,7 @@
       <c r="L94" t="s">
         <v>725</v>
       </c>
-      <c r="M94" s="2">
+      <c r="M94" s="1">
         <v>46389</v>
       </c>
       <c r="N94" t="s">
@@ -14741,7 +14715,7 @@
       <c r="L95" t="s">
         <v>725</v>
       </c>
-      <c r="M95" s="2">
+      <c r="M95" s="1">
         <v>46389</v>
       </c>
       <c r="N95" t="s">
@@ -14785,7 +14759,7 @@
       <c r="L96" t="s">
         <v>725</v>
       </c>
-      <c r="M96" s="2">
+      <c r="M96" s="1">
         <v>46389</v>
       </c>
       <c r="N96" t="s">
@@ -14829,7 +14803,7 @@
       <c r="L97" t="s">
         <v>725</v>
       </c>
-      <c r="M97" s="2">
+      <c r="M97" s="1">
         <v>46389</v>
       </c>
       <c r="N97" t="s">
@@ -14873,7 +14847,7 @@
       <c r="L98" t="s">
         <v>725</v>
       </c>
-      <c r="M98" s="2">
+      <c r="M98" s="1">
         <v>46389</v>
       </c>
       <c r="N98" t="s">
@@ -14917,7 +14891,7 @@
       <c r="L99" t="s">
         <v>725</v>
       </c>
-      <c r="M99" s="2">
+      <c r="M99" s="1">
         <v>46389</v>
       </c>
       <c r="N99" t="s">
@@ -14961,7 +14935,7 @@
       <c r="L100" t="s">
         <v>725</v>
       </c>
-      <c r="M100" s="2">
+      <c r="M100" s="1">
         <v>46389</v>
       </c>
       <c r="N100" t="s">
@@ -15005,7 +14979,7 @@
       <c r="L101" t="s">
         <v>725</v>
       </c>
-      <c r="M101" s="2">
+      <c r="M101" s="1">
         <v>46389</v>
       </c>
       <c r="N101" t="s">
@@ -15049,7 +15023,7 @@
       <c r="L102" t="s">
         <v>725</v>
       </c>
-      <c r="M102" s="2">
+      <c r="M102" s="1">
         <v>46389</v>
       </c>
       <c r="N102" t="s">
@@ -15093,7 +15067,7 @@
       <c r="L103" t="s">
         <v>725</v>
       </c>
-      <c r="M103" s="2">
+      <c r="M103" s="1">
         <v>46389</v>
       </c>
       <c r="N103" t="s">
@@ -15137,7 +15111,7 @@
       <c r="L104" t="s">
         <v>725</v>
       </c>
-      <c r="M104" s="2">
+      <c r="M104" s="1">
         <v>46389</v>
       </c>
       <c r="N104" t="s">
@@ -15181,7 +15155,7 @@
       <c r="L105" t="s">
         <v>725</v>
       </c>
-      <c r="M105" s="2">
+      <c r="M105" s="1">
         <v>46389</v>
       </c>
       <c r="N105" t="s">
@@ -15225,7 +15199,7 @@
       <c r="L106" t="s">
         <v>725</v>
       </c>
-      <c r="M106" s="2">
+      <c r="M106" s="1">
         <v>46389</v>
       </c>
       <c r="N106" t="s">
@@ -15269,7 +15243,7 @@
       <c r="L107" t="s">
         <v>725</v>
       </c>
-      <c r="M107" s="2">
+      <c r="M107" s="1">
         <v>46389</v>
       </c>
       <c r="N107" t="s">
@@ -15313,7 +15287,7 @@
       <c r="L108" t="s">
         <v>725</v>
       </c>
-      <c r="M108" s="2">
+      <c r="M108" s="1">
         <v>46389</v>
       </c>
       <c r="N108" t="s">
@@ -15357,7 +15331,7 @@
       <c r="L109" t="s">
         <v>725</v>
       </c>
-      <c r="M109" s="2">
+      <c r="M109" s="1">
         <v>46389</v>
       </c>
       <c r="N109" t="s">
@@ -15401,7 +15375,7 @@
       <c r="L110" t="s">
         <v>725</v>
       </c>
-      <c r="M110" s="2">
+      <c r="M110" s="1">
         <v>46389</v>
       </c>
       <c r="N110" t="s">
@@ -15445,7 +15419,7 @@
       <c r="L111" t="s">
         <v>725</v>
       </c>
-      <c r="M111" s="2">
+      <c r="M111" s="1">
         <v>46389</v>
       </c>
       <c r="N111" t="s">
@@ -15489,7 +15463,7 @@
       <c r="L112" t="s">
         <v>725</v>
       </c>
-      <c r="M112" s="2">
+      <c r="M112" s="1">
         <v>46389</v>
       </c>
       <c r="N112" t="s">
@@ -15533,7 +15507,7 @@
       <c r="L113" t="s">
         <v>725</v>
       </c>
-      <c r="M113" s="2">
+      <c r="M113" s="1">
         <v>46389</v>
       </c>
       <c r="N113" t="s">
@@ -15577,7 +15551,7 @@
       <c r="L114" t="s">
         <v>725</v>
       </c>
-      <c r="M114" s="2">
+      <c r="M114" s="1">
         <v>46389</v>
       </c>
       <c r="N114" t="s">
@@ -15621,7 +15595,7 @@
       <c r="L115" t="s">
         <v>725</v>
       </c>
-      <c r="M115" s="2">
+      <c r="M115" s="1">
         <v>46389</v>
       </c>
       <c r="N115" t="s">
@@ -15665,7 +15639,7 @@
       <c r="L116" t="s">
         <v>725</v>
       </c>
-      <c r="M116" s="2">
+      <c r="M116" s="1">
         <v>46389</v>
       </c>
       <c r="N116" t="s">
@@ -15709,7 +15683,7 @@
       <c r="L117" t="s">
         <v>725</v>
       </c>
-      <c r="M117" s="2">
+      <c r="M117" s="1">
         <v>46389</v>
       </c>
       <c r="N117" t="s">
@@ -15753,7 +15727,7 @@
       <c r="L118" t="s">
         <v>725</v>
       </c>
-      <c r="M118" s="2">
+      <c r="M118" s="1">
         <v>46389</v>
       </c>
       <c r="N118" t="s">
@@ -15797,7 +15771,7 @@
       <c r="L119" t="s">
         <v>725</v>
       </c>
-      <c r="M119" s="2">
+      <c r="M119" s="1">
         <v>46389</v>
       </c>
       <c r="N119" t="s">
@@ -15841,7 +15815,7 @@
       <c r="L120" t="s">
         <v>725</v>
       </c>
-      <c r="M120" s="2">
+      <c r="M120" s="1">
         <v>46389</v>
       </c>
       <c r="N120" t="s">
@@ -15885,7 +15859,7 @@
       <c r="L121" t="s">
         <v>725</v>
       </c>
-      <c r="M121" s="2">
+      <c r="M121" s="1">
         <v>46389</v>
       </c>
       <c r="N121" t="s">
@@ -15929,7 +15903,7 @@
       <c r="L122" t="s">
         <v>725</v>
       </c>
-      <c r="M122" s="2">
+      <c r="M122" s="1">
         <v>46389</v>
       </c>
       <c r="N122" t="s">
@@ -15973,7 +15947,7 @@
       <c r="L123" t="s">
         <v>725</v>
       </c>
-      <c r="M123" s="2">
+      <c r="M123" s="1">
         <v>46389</v>
       </c>
       <c r="N123" t="s">
@@ -16017,7 +15991,7 @@
       <c r="L124" t="s">
         <v>725</v>
       </c>
-      <c r="M124" s="2">
+      <c r="M124" s="1">
         <v>46389</v>
       </c>
       <c r="N124" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (20/10/2026 12:39)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -11069,7 +11069,7 @@
         <v>725</v>
       </c>
       <c r="M10" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N10" t="s">
         <v>726</v>
@@ -11113,7 +11113,7 @@
         <v>725</v>
       </c>
       <c r="M11" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N11" t="s">
         <v>726</v>
@@ -11321,7 +11321,7 @@
         <v>725</v>
       </c>
       <c r="M16" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N16" t="s">
         <v>726</v>
@@ -11447,7 +11447,7 @@
         <v>725</v>
       </c>
       <c r="M19" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N19" t="s">
         <v>726</v>
@@ -11491,7 +11491,7 @@
         <v>725</v>
       </c>
       <c r="M20" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N20" t="s">
         <v>726</v>
@@ -11535,7 +11535,7 @@
         <v>725</v>
       </c>
       <c r="M21" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N21" t="s">
         <v>726</v>
@@ -11702,7 +11702,7 @@
         <v>725</v>
       </c>
       <c r="M25" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N25" t="s">
         <v>726</v>
@@ -11828,7 +11828,7 @@
         <v>725</v>
       </c>
       <c r="M28" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N28" t="s">
         <v>726</v>
@@ -11913,7 +11913,7 @@
         <v>725</v>
       </c>
       <c r="M30" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N30" t="s">
         <v>726</v>
@@ -12367,7 +12367,7 @@
         <v>725</v>
       </c>
       <c r="M41" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N41" t="s">
         <v>726</v>
@@ -12452,7 +12452,7 @@
         <v>725</v>
       </c>
       <c r="M43" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N43" t="s">
         <v>726</v>
@@ -12496,7 +12496,7 @@
         <v>725</v>
       </c>
       <c r="M44" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N44" t="s">
         <v>726</v>
@@ -12540,7 +12540,7 @@
         <v>725</v>
       </c>
       <c r="M45" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N45" t="s">
         <v>726</v>
@@ -12666,7 +12666,7 @@
         <v>725</v>
       </c>
       <c r="M48" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N48" t="s">
         <v>726</v>
@@ -12710,7 +12710,7 @@
         <v>723</v>
       </c>
       <c r="M49" s="1">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="N49" t="s">
         <v>726</v>
@@ -12754,7 +12754,7 @@
         <v>723</v>
       </c>
       <c r="M50" s="1">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="N50" t="s">
         <v>726</v>
@@ -12798,7 +12798,7 @@
         <v>725</v>
       </c>
       <c r="M51" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N51" t="s">
         <v>726</v>
@@ -12842,7 +12842,7 @@
         <v>725</v>
       </c>
       <c r="M52" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N52" t="s">
         <v>726</v>
@@ -12886,7 +12886,7 @@
         <v>725</v>
       </c>
       <c r="M53" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N53" t="s">
         <v>726</v>
@@ -12930,7 +12930,7 @@
         <v>725</v>
       </c>
       <c r="M54" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N54" t="s">
         <v>726</v>
@@ -12974,7 +12974,7 @@
         <v>725</v>
       </c>
       <c r="M55" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N55" t="s">
         <v>726</v>
@@ -13141,7 +13141,7 @@
         <v>725</v>
       </c>
       <c r="M59" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N59" t="s">
         <v>726</v>
@@ -13267,7 +13267,7 @@
         <v>725</v>
       </c>
       <c r="M62" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N62" t="s">
         <v>726</v>
@@ -13311,7 +13311,7 @@
         <v>725</v>
       </c>
       <c r="M63" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N63" t="s">
         <v>726</v>
@@ -13355,7 +13355,7 @@
         <v>725</v>
       </c>
       <c r="M64" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N64" t="s">
         <v>726</v>
@@ -13399,7 +13399,7 @@
         <v>725</v>
       </c>
       <c r="M65" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N65" t="s">
         <v>726</v>
@@ -13443,7 +13443,7 @@
         <v>725</v>
       </c>
       <c r="M66" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N66" t="s">
         <v>726</v>
@@ -13487,7 +13487,7 @@
         <v>725</v>
       </c>
       <c r="M67" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N67" t="s">
         <v>726</v>
@@ -13531,7 +13531,7 @@
         <v>725</v>
       </c>
       <c r="M68" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N68" t="s">
         <v>726</v>
@@ -13575,7 +13575,7 @@
         <v>725</v>
       </c>
       <c r="M69" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N69" t="s">
         <v>726</v>
@@ -13619,7 +13619,7 @@
         <v>725</v>
       </c>
       <c r="M70" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N70" t="s">
         <v>726</v>
@@ -13663,7 +13663,7 @@
         <v>725</v>
       </c>
       <c r="M71" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N71" t="s">
         <v>726</v>
@@ -13707,7 +13707,7 @@
         <v>725</v>
       </c>
       <c r="M72" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N72" t="s">
         <v>726</v>
@@ -13751,7 +13751,7 @@
         <v>725</v>
       </c>
       <c r="M73" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N73" t="s">
         <v>726</v>
@@ -13795,7 +13795,7 @@
         <v>725</v>
       </c>
       <c r="M74" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N74" t="s">
         <v>726</v>
@@ -13839,7 +13839,7 @@
         <v>725</v>
       </c>
       <c r="M75" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N75" t="s">
         <v>726</v>
@@ -13883,7 +13883,7 @@
         <v>725</v>
       </c>
       <c r="M76" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N76" t="s">
         <v>726</v>
@@ -13927,7 +13927,7 @@
         <v>725</v>
       </c>
       <c r="M77" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N77" t="s">
         <v>726</v>
@@ -13971,7 +13971,7 @@
         <v>725</v>
       </c>
       <c r="M78" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N78" t="s">
         <v>726</v>
@@ -14015,7 +14015,7 @@
         <v>725</v>
       </c>
       <c r="M79" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N79" t="s">
         <v>726</v>
@@ -14059,7 +14059,7 @@
         <v>725</v>
       </c>
       <c r="M80" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N80" t="s">
         <v>726</v>
@@ -14103,7 +14103,7 @@
         <v>725</v>
       </c>
       <c r="M81" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N81" t="s">
         <v>726</v>
@@ -14147,7 +14147,7 @@
         <v>725</v>
       </c>
       <c r="M82" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N82" t="s">
         <v>726</v>
@@ -14191,7 +14191,7 @@
         <v>725</v>
       </c>
       <c r="M83" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N83" t="s">
         <v>726</v>
@@ -14235,7 +14235,7 @@
         <v>725</v>
       </c>
       <c r="M84" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N84" t="s">
         <v>726</v>
@@ -14279,7 +14279,7 @@
         <v>725</v>
       </c>
       <c r="M85" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N85" t="s">
         <v>726</v>
@@ -14323,7 +14323,7 @@
         <v>725</v>
       </c>
       <c r="M86" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N86" t="s">
         <v>726</v>
@@ -14367,7 +14367,7 @@
         <v>725</v>
       </c>
       <c r="M87" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N87" t="s">
         <v>726</v>
@@ -14411,7 +14411,7 @@
         <v>725</v>
       </c>
       <c r="M88" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N88" t="s">
         <v>726</v>
@@ -14455,7 +14455,7 @@
         <v>725</v>
       </c>
       <c r="M89" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N89" t="s">
         <v>726</v>
@@ -14499,7 +14499,7 @@
         <v>725</v>
       </c>
       <c r="M90" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N90" t="s">
         <v>726</v>
@@ -14584,7 +14584,7 @@
         <v>725</v>
       </c>
       <c r="M92" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N92" t="s">
         <v>726</v>
@@ -14628,7 +14628,7 @@
         <v>725</v>
       </c>
       <c r="M93" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N93" t="s">
         <v>726</v>
@@ -14672,7 +14672,7 @@
         <v>725</v>
       </c>
       <c r="M94" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N94" t="s">
         <v>726</v>
@@ -14716,7 +14716,7 @@
         <v>725</v>
       </c>
       <c r="M95" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N95" t="s">
         <v>726</v>
@@ -14760,7 +14760,7 @@
         <v>725</v>
       </c>
       <c r="M96" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N96" t="s">
         <v>726</v>
@@ -14804,7 +14804,7 @@
         <v>725</v>
       </c>
       <c r="M97" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N97" t="s">
         <v>726</v>
@@ -14848,7 +14848,7 @@
         <v>725</v>
       </c>
       <c r="M98" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N98" t="s">
         <v>726</v>
@@ -14892,7 +14892,7 @@
         <v>725</v>
       </c>
       <c r="M99" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N99" t="s">
         <v>726</v>
@@ -14936,7 +14936,7 @@
         <v>725</v>
       </c>
       <c r="M100" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N100" t="s">
         <v>726</v>
@@ -14980,7 +14980,7 @@
         <v>725</v>
       </c>
       <c r="M101" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N101" t="s">
         <v>726</v>
@@ -15024,7 +15024,7 @@
         <v>725</v>
       </c>
       <c r="M102" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N102" t="s">
         <v>726</v>
@@ -15068,7 +15068,7 @@
         <v>725</v>
       </c>
       <c r="M103" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N103" t="s">
         <v>726</v>
@@ -15112,7 +15112,7 @@
         <v>725</v>
       </c>
       <c r="M104" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N104" t="s">
         <v>726</v>
@@ -15156,7 +15156,7 @@
         <v>725</v>
       </c>
       <c r="M105" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N105" t="s">
         <v>726</v>
@@ -15200,7 +15200,7 @@
         <v>725</v>
       </c>
       <c r="M106" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N106" t="s">
         <v>726</v>
@@ -15244,7 +15244,7 @@
         <v>725</v>
       </c>
       <c r="M107" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N107" t="s">
         <v>726</v>
@@ -15288,7 +15288,7 @@
         <v>725</v>
       </c>
       <c r="M108" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N108" t="s">
         <v>726</v>
@@ -15332,7 +15332,7 @@
         <v>725</v>
       </c>
       <c r="M109" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N109" t="s">
         <v>726</v>
@@ -15376,7 +15376,7 @@
         <v>725</v>
       </c>
       <c r="M110" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N110" t="s">
         <v>726</v>
@@ -15420,7 +15420,7 @@
         <v>725</v>
       </c>
       <c r="M111" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N111" t="s">
         <v>726</v>
@@ -15464,7 +15464,7 @@
         <v>725</v>
       </c>
       <c r="M112" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N112" t="s">
         <v>726</v>
@@ -15508,7 +15508,7 @@
         <v>725</v>
       </c>
       <c r="M113" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N113" t="s">
         <v>726</v>
@@ -15552,7 +15552,7 @@
         <v>725</v>
       </c>
       <c r="M114" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N114" t="s">
         <v>726</v>
@@ -15596,7 +15596,7 @@
         <v>725</v>
       </c>
       <c r="M115" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N115" t="s">
         <v>726</v>
@@ -15640,7 +15640,7 @@
         <v>725</v>
       </c>
       <c r="M116" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N116" t="s">
         <v>726</v>
@@ -15684,7 +15684,7 @@
         <v>725</v>
       </c>
       <c r="M117" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N117" t="s">
         <v>726</v>
@@ -15728,7 +15728,7 @@
         <v>725</v>
       </c>
       <c r="M118" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N118" t="s">
         <v>726</v>
@@ -15772,7 +15772,7 @@
         <v>725</v>
       </c>
       <c r="M119" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N119" t="s">
         <v>726</v>
@@ -15816,7 +15816,7 @@
         <v>725</v>
       </c>
       <c r="M120" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N120" t="s">
         <v>726</v>
@@ -15860,7 +15860,7 @@
         <v>725</v>
       </c>
       <c r="M121" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N121" t="s">
         <v>726</v>
@@ -15904,7 +15904,7 @@
         <v>725</v>
       </c>
       <c r="M122" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N122" t="s">
         <v>726</v>
@@ -15948,7 +15948,7 @@
         <v>725</v>
       </c>
       <c r="M123" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N123" t="s">
         <v>726</v>
@@ -15992,7 +15992,7 @@
         <v>725</v>
       </c>
       <c r="M124" s="1">
-        <v>46389</v>
+        <v>46390</v>
       </c>
       <c r="N124" t="s">
         <v>726</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (21/10/2026 12:56)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -11069,7 +11069,7 @@
         <v>725</v>
       </c>
       <c r="M10" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N10" t="s">
         <v>726</v>
@@ -11113,7 +11113,7 @@
         <v>725</v>
       </c>
       <c r="M11" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N11" t="s">
         <v>726</v>
@@ -11321,7 +11321,7 @@
         <v>725</v>
       </c>
       <c r="M16" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N16" t="s">
         <v>726</v>
@@ -11447,7 +11447,7 @@
         <v>725</v>
       </c>
       <c r="M19" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N19" t="s">
         <v>726</v>
@@ -11491,7 +11491,7 @@
         <v>725</v>
       </c>
       <c r="M20" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N20" t="s">
         <v>726</v>
@@ -11535,7 +11535,7 @@
         <v>725</v>
       </c>
       <c r="M21" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N21" t="s">
         <v>726</v>
@@ -11702,7 +11702,7 @@
         <v>725</v>
       </c>
       <c r="M25" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N25" t="s">
         <v>726</v>
@@ -11828,7 +11828,7 @@
         <v>725</v>
       </c>
       <c r="M28" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N28" t="s">
         <v>726</v>
@@ -11913,7 +11913,7 @@
         <v>725</v>
       </c>
       <c r="M30" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N30" t="s">
         <v>726</v>
@@ -12367,7 +12367,7 @@
         <v>725</v>
       </c>
       <c r="M41" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N41" t="s">
         <v>726</v>
@@ -12452,7 +12452,7 @@
         <v>725</v>
       </c>
       <c r="M43" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N43" t="s">
         <v>726</v>
@@ -12496,7 +12496,7 @@
         <v>725</v>
       </c>
       <c r="M44" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N44" t="s">
         <v>726</v>
@@ -12540,7 +12540,7 @@
         <v>725</v>
       </c>
       <c r="M45" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N45" t="s">
         <v>726</v>
@@ -12666,7 +12666,7 @@
         <v>725</v>
       </c>
       <c r="M48" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N48" t="s">
         <v>726</v>
@@ -12710,7 +12710,7 @@
         <v>723</v>
       </c>
       <c r="M49" s="1">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="N49" t="s">
         <v>726</v>
@@ -12754,7 +12754,7 @@
         <v>723</v>
       </c>
       <c r="M50" s="1">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="N50" t="s">
         <v>726</v>
@@ -12798,7 +12798,7 @@
         <v>725</v>
       </c>
       <c r="M51" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N51" t="s">
         <v>726</v>
@@ -12842,7 +12842,7 @@
         <v>725</v>
       </c>
       <c r="M52" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N52" t="s">
         <v>726</v>
@@ -12886,7 +12886,7 @@
         <v>725</v>
       </c>
       <c r="M53" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N53" t="s">
         <v>726</v>
@@ -12930,7 +12930,7 @@
         <v>725</v>
       </c>
       <c r="M54" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N54" t="s">
         <v>726</v>
@@ -12974,7 +12974,7 @@
         <v>725</v>
       </c>
       <c r="M55" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N55" t="s">
         <v>726</v>
@@ -13141,7 +13141,7 @@
         <v>725</v>
       </c>
       <c r="M59" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N59" t="s">
         <v>726</v>
@@ -13267,7 +13267,7 @@
         <v>725</v>
       </c>
       <c r="M62" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N62" t="s">
         <v>726</v>
@@ -13311,7 +13311,7 @@
         <v>725</v>
       </c>
       <c r="M63" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N63" t="s">
         <v>726</v>
@@ -13355,7 +13355,7 @@
         <v>725</v>
       </c>
       <c r="M64" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N64" t="s">
         <v>726</v>
@@ -13399,7 +13399,7 @@
         <v>725</v>
       </c>
       <c r="M65" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N65" t="s">
         <v>726</v>
@@ -13443,7 +13443,7 @@
         <v>725</v>
       </c>
       <c r="M66" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N66" t="s">
         <v>726</v>
@@ -13487,7 +13487,7 @@
         <v>725</v>
       </c>
       <c r="M67" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N67" t="s">
         <v>726</v>
@@ -13531,7 +13531,7 @@
         <v>725</v>
       </c>
       <c r="M68" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N68" t="s">
         <v>726</v>
@@ -13575,7 +13575,7 @@
         <v>725</v>
       </c>
       <c r="M69" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N69" t="s">
         <v>726</v>
@@ -13619,7 +13619,7 @@
         <v>725</v>
       </c>
       <c r="M70" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N70" t="s">
         <v>726</v>
@@ -13663,7 +13663,7 @@
         <v>725</v>
       </c>
       <c r="M71" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N71" t="s">
         <v>726</v>
@@ -13707,7 +13707,7 @@
         <v>725</v>
       </c>
       <c r="M72" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N72" t="s">
         <v>726</v>
@@ -13751,7 +13751,7 @@
         <v>725</v>
       </c>
       <c r="M73" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N73" t="s">
         <v>726</v>
@@ -13795,7 +13795,7 @@
         <v>725</v>
       </c>
       <c r="M74" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N74" t="s">
         <v>726</v>
@@ -13839,7 +13839,7 @@
         <v>725</v>
       </c>
       <c r="M75" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N75" t="s">
         <v>726</v>
@@ -13883,7 +13883,7 @@
         <v>725</v>
       </c>
       <c r="M76" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N76" t="s">
         <v>726</v>
@@ -13927,7 +13927,7 @@
         <v>725</v>
       </c>
       <c r="M77" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N77" t="s">
         <v>726</v>
@@ -13971,7 +13971,7 @@
         <v>725</v>
       </c>
       <c r="M78" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N78" t="s">
         <v>726</v>
@@ -14015,7 +14015,7 @@
         <v>725</v>
       </c>
       <c r="M79" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N79" t="s">
         <v>726</v>
@@ -14059,7 +14059,7 @@
         <v>725</v>
       </c>
       <c r="M80" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N80" t="s">
         <v>726</v>
@@ -14103,7 +14103,7 @@
         <v>725</v>
       </c>
       <c r="M81" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N81" t="s">
         <v>726</v>
@@ -14147,7 +14147,7 @@
         <v>725</v>
       </c>
       <c r="M82" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N82" t="s">
         <v>726</v>
@@ -14191,7 +14191,7 @@
         <v>725</v>
       </c>
       <c r="M83" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N83" t="s">
         <v>726</v>
@@ -14235,7 +14235,7 @@
         <v>725</v>
       </c>
       <c r="M84" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N84" t="s">
         <v>726</v>
@@ -14279,7 +14279,7 @@
         <v>725</v>
       </c>
       <c r="M85" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N85" t="s">
         <v>726</v>
@@ -14323,7 +14323,7 @@
         <v>725</v>
       </c>
       <c r="M86" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N86" t="s">
         <v>726</v>
@@ -14367,7 +14367,7 @@
         <v>725</v>
       </c>
       <c r="M87" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N87" t="s">
         <v>726</v>
@@ -14411,7 +14411,7 @@
         <v>725</v>
       </c>
       <c r="M88" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N88" t="s">
         <v>726</v>
@@ -14455,7 +14455,7 @@
         <v>725</v>
       </c>
       <c r="M89" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N89" t="s">
         <v>726</v>
@@ -14499,7 +14499,7 @@
         <v>725</v>
       </c>
       <c r="M90" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N90" t="s">
         <v>726</v>
@@ -14584,7 +14584,7 @@
         <v>725</v>
       </c>
       <c r="M92" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N92" t="s">
         <v>726</v>
@@ -14628,7 +14628,7 @@
         <v>725</v>
       </c>
       <c r="M93" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N93" t="s">
         <v>726</v>
@@ -14672,7 +14672,7 @@
         <v>725</v>
       </c>
       <c r="M94" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N94" t="s">
         <v>726</v>
@@ -14716,7 +14716,7 @@
         <v>725</v>
       </c>
       <c r="M95" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N95" t="s">
         <v>726</v>
@@ -14760,7 +14760,7 @@
         <v>725</v>
       </c>
       <c r="M96" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N96" t="s">
         <v>726</v>
@@ -14804,7 +14804,7 @@
         <v>725</v>
       </c>
       <c r="M97" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N97" t="s">
         <v>726</v>
@@ -14848,7 +14848,7 @@
         <v>725</v>
       </c>
       <c r="M98" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N98" t="s">
         <v>726</v>
@@ -14892,7 +14892,7 @@
         <v>725</v>
       </c>
       <c r="M99" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N99" t="s">
         <v>726</v>
@@ -14936,7 +14936,7 @@
         <v>725</v>
       </c>
       <c r="M100" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N100" t="s">
         <v>726</v>
@@ -14980,7 +14980,7 @@
         <v>725</v>
       </c>
       <c r="M101" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N101" t="s">
         <v>726</v>
@@ -15024,7 +15024,7 @@
         <v>725</v>
       </c>
       <c r="M102" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N102" t="s">
         <v>726</v>
@@ -15068,7 +15068,7 @@
         <v>725</v>
       </c>
       <c r="M103" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N103" t="s">
         <v>726</v>
@@ -15112,7 +15112,7 @@
         <v>725</v>
       </c>
       <c r="M104" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N104" t="s">
         <v>726</v>
@@ -15156,7 +15156,7 @@
         <v>725</v>
       </c>
       <c r="M105" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N105" t="s">
         <v>726</v>
@@ -15200,7 +15200,7 @@
         <v>725</v>
       </c>
       <c r="M106" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N106" t="s">
         <v>726</v>
@@ -15244,7 +15244,7 @@
         <v>725</v>
       </c>
       <c r="M107" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N107" t="s">
         <v>726</v>
@@ -15288,7 +15288,7 @@
         <v>725</v>
       </c>
       <c r="M108" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N108" t="s">
         <v>726</v>
@@ -15332,7 +15332,7 @@
         <v>725</v>
       </c>
       <c r="M109" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N109" t="s">
         <v>726</v>
@@ -15376,7 +15376,7 @@
         <v>725</v>
       </c>
       <c r="M110" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N110" t="s">
         <v>726</v>
@@ -15420,7 +15420,7 @@
         <v>725</v>
       </c>
       <c r="M111" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N111" t="s">
         <v>726</v>
@@ -15464,7 +15464,7 @@
         <v>725</v>
       </c>
       <c r="M112" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N112" t="s">
         <v>726</v>
@@ -15508,7 +15508,7 @@
         <v>725</v>
       </c>
       <c r="M113" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N113" t="s">
         <v>726</v>
@@ -15552,7 +15552,7 @@
         <v>725</v>
       </c>
       <c r="M114" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N114" t="s">
         <v>726</v>
@@ -15596,7 +15596,7 @@
         <v>725</v>
       </c>
       <c r="M115" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N115" t="s">
         <v>726</v>
@@ -15640,7 +15640,7 @@
         <v>725</v>
       </c>
       <c r="M116" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N116" t="s">
         <v>726</v>
@@ -15684,7 +15684,7 @@
         <v>725</v>
       </c>
       <c r="M117" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N117" t="s">
         <v>726</v>
@@ -15728,7 +15728,7 @@
         <v>725</v>
       </c>
       <c r="M118" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N118" t="s">
         <v>726</v>
@@ -15772,7 +15772,7 @@
         <v>725</v>
       </c>
       <c r="M119" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N119" t="s">
         <v>726</v>
@@ -15816,7 +15816,7 @@
         <v>725</v>
       </c>
       <c r="M120" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N120" t="s">
         <v>726</v>
@@ -15860,7 +15860,7 @@
         <v>725</v>
       </c>
       <c r="M121" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N121" t="s">
         <v>726</v>
@@ -15904,7 +15904,7 @@
         <v>725</v>
       </c>
       <c r="M122" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N122" t="s">
         <v>726</v>
@@ -15948,7 +15948,7 @@
         <v>725</v>
       </c>
       <c r="M123" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N123" t="s">
         <v>726</v>
@@ -15992,7 +15992,7 @@
         <v>725</v>
       </c>
       <c r="M124" s="1">
-        <v>46390</v>
+        <v>46391</v>
       </c>
       <c r="N124" t="s">
         <v>726</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (21/10/2026 14:22)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2205,8 +2205,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2222,7 +2230,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2230,12 +2238,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2535,55 +2561,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2627,7 +2653,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2671,7 +2697,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2715,7 +2741,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2885,7 +2911,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2929,7 +2955,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2976,7 +3002,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3099,7 +3125,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -3143,7 +3169,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3187,7 +3213,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3231,7 +3257,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3278,7 +3304,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3322,7 +3348,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3448,7 +3474,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3492,7 +3518,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3577,7 +3603,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3624,7 +3650,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3671,7 +3697,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3715,7 +3741,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3759,7 +3785,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3844,7 +3870,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3929,7 +3955,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3976,7 +4002,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4020,7 +4046,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4064,7 +4090,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4149,7 +4175,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4193,7 +4219,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4237,7 +4263,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4322,7 +4348,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4366,7 +4392,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4410,7 +4436,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4454,7 +4480,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4621,7 +4647,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4665,7 +4691,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4709,7 +4735,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4753,7 +4779,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4800,7 +4826,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4844,7 +4870,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4926,7 +4952,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4970,7 +4996,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5058,7 +5084,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5102,7 +5128,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5149,7 +5175,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5193,7 +5219,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -5237,7 +5263,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5281,7 +5307,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5325,7 +5351,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5372,7 +5398,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5416,7 +5442,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5463,7 +5489,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5507,7 +5533,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5554,7 +5580,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5642,7 +5668,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5686,7 +5712,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5730,7 +5756,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5774,7 +5800,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5818,7 +5844,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5862,7 +5888,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5947,7 +5973,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5991,7 +6017,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -6035,7 +6061,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -6079,7 +6105,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -6123,7 +6149,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -6167,7 +6193,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6211,7 +6237,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6255,7 +6281,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6302,7 +6328,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6346,7 +6372,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6390,7 +6416,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6434,7 +6460,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6478,7 +6504,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6566,7 +6592,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6610,7 +6636,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6654,7 +6680,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6742,7 +6768,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6786,7 +6812,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6912,7 +6938,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6956,7 +6982,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7000,7 +7026,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7044,7 +7070,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7126,7 +7152,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7170,7 +7196,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7217,7 +7243,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7261,7 +7287,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7387,7 +7413,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7431,7 +7457,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7516,7 +7542,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7560,7 +7586,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7604,7 +7630,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7648,7 +7674,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7692,7 +7718,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7736,7 +7762,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7780,7 +7806,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7824,7 +7850,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7909,7 +7935,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8076,7 +8102,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8120,7 +8146,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8164,7 +8190,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8208,7 +8234,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8252,7 +8278,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8296,7 +8322,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8340,7 +8366,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8425,7 +8451,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8469,7 +8495,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8554,7 +8580,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8680,7 +8706,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8724,7 +8750,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8809,7 +8835,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8853,7 +8879,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8897,7 +8923,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8941,7 +8967,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8985,7 +9011,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -9029,7 +9055,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9073,7 +9099,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9117,7 +9143,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9202,7 +9228,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9369,7 +9395,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9413,7 +9439,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9457,7 +9483,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9501,7 +9527,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9586,7 +9612,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9630,7 +9656,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9674,7 +9700,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9718,7 +9744,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9762,7 +9788,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9806,7 +9832,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9850,7 +9876,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9894,7 +9920,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9938,7 +9964,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9982,7 +10008,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10026,7 +10052,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -10070,7 +10096,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10114,7 +10140,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10158,7 +10184,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -10202,7 +10228,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10246,7 +10272,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10290,7 +10316,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10334,7 +10360,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10378,7 +10404,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10422,7 +10448,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10466,7 +10492,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10551,7 +10577,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10636,7 +10662,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10651,55 +10677,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11068,7 +11094,7 @@
       <c r="L10" t="s">
         <v>725</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46391</v>
       </c>
       <c r="N10" t="s">
@@ -11112,7 +11138,7 @@
       <c r="L11" t="s">
         <v>725</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46391</v>
       </c>
       <c r="N11" t="s">
@@ -11320,7 +11346,7 @@
       <c r="L16" t="s">
         <v>725</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46391</v>
       </c>
       <c r="N16" t="s">
@@ -11446,7 +11472,7 @@
       <c r="L19" t="s">
         <v>725</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46391</v>
       </c>
       <c r="N19" t="s">
@@ -11490,7 +11516,7 @@
       <c r="L20" t="s">
         <v>725</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46391</v>
       </c>
       <c r="N20" t="s">
@@ -11534,7 +11560,7 @@
       <c r="L21" t="s">
         <v>725</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46391</v>
       </c>
       <c r="N21" t="s">
@@ -11701,7 +11727,7 @@
       <c r="L25" t="s">
         <v>725</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46391</v>
       </c>
       <c r="N25" t="s">
@@ -11827,7 +11853,7 @@
       <c r="L28" t="s">
         <v>725</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46391</v>
       </c>
       <c r="N28" t="s">
@@ -11912,7 +11938,7 @@
       <c r="L30" t="s">
         <v>725</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46391</v>
       </c>
       <c r="N30" t="s">
@@ -12366,7 +12392,7 @@
       <c r="L41" t="s">
         <v>725</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46391</v>
       </c>
       <c r="N41" t="s">
@@ -12451,7 +12477,7 @@
       <c r="L43" t="s">
         <v>725</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46391</v>
       </c>
       <c r="N43" t="s">
@@ -12495,7 +12521,7 @@
       <c r="L44" t="s">
         <v>725</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46391</v>
       </c>
       <c r="N44" t="s">
@@ -12539,7 +12565,7 @@
       <c r="L45" t="s">
         <v>725</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46391</v>
       </c>
       <c r="N45" t="s">
@@ -12665,7 +12691,7 @@
       <c r="L48" t="s">
         <v>725</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46391</v>
       </c>
       <c r="N48" t="s">
@@ -12709,7 +12735,7 @@
       <c r="L49" t="s">
         <v>723</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46326</v>
       </c>
       <c r="N49" t="s">
@@ -12753,7 +12779,7 @@
       <c r="L50" t="s">
         <v>723</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46326</v>
       </c>
       <c r="N50" t="s">
@@ -12797,7 +12823,7 @@
       <c r="L51" t="s">
         <v>725</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46391</v>
       </c>
       <c r="N51" t="s">
@@ -12841,7 +12867,7 @@
       <c r="L52" t="s">
         <v>725</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46391</v>
       </c>
       <c r="N52" t="s">
@@ -12885,7 +12911,7 @@
       <c r="L53" t="s">
         <v>725</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46391</v>
       </c>
       <c r="N53" t="s">
@@ -12929,7 +12955,7 @@
       <c r="L54" t="s">
         <v>725</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46391</v>
       </c>
       <c r="N54" t="s">
@@ -12973,7 +12999,7 @@
       <c r="L55" t="s">
         <v>725</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46391</v>
       </c>
       <c r="N55" t="s">
@@ -13140,7 +13166,7 @@
       <c r="L59" t="s">
         <v>725</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46391</v>
       </c>
       <c r="N59" t="s">
@@ -13266,7 +13292,7 @@
       <c r="L62" t="s">
         <v>725</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46391</v>
       </c>
       <c r="N62" t="s">
@@ -13310,7 +13336,7 @@
       <c r="L63" t="s">
         <v>725</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46391</v>
       </c>
       <c r="N63" t="s">
@@ -13354,7 +13380,7 @@
       <c r="L64" t="s">
         <v>725</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46391</v>
       </c>
       <c r="N64" t="s">
@@ -13398,7 +13424,7 @@
       <c r="L65" t="s">
         <v>725</v>
       </c>
-      <c r="M65" s="1">
+      <c r="M65" s="2">
         <v>46391</v>
       </c>
       <c r="N65" t="s">
@@ -13442,7 +13468,7 @@
       <c r="L66" t="s">
         <v>725</v>
       </c>
-      <c r="M66" s="1">
+      <c r="M66" s="2">
         <v>46391</v>
       </c>
       <c r="N66" t="s">
@@ -13486,7 +13512,7 @@
       <c r="L67" t="s">
         <v>725</v>
       </c>
-      <c r="M67" s="1">
+      <c r="M67" s="2">
         <v>46391</v>
       </c>
       <c r="N67" t="s">
@@ -13530,7 +13556,7 @@
       <c r="L68" t="s">
         <v>725</v>
       </c>
-      <c r="M68" s="1">
+      <c r="M68" s="2">
         <v>46391</v>
       </c>
       <c r="N68" t="s">
@@ -13574,7 +13600,7 @@
       <c r="L69" t="s">
         <v>725</v>
       </c>
-      <c r="M69" s="1">
+      <c r="M69" s="2">
         <v>46391</v>
       </c>
       <c r="N69" t="s">
@@ -13618,7 +13644,7 @@
       <c r="L70" t="s">
         <v>725</v>
       </c>
-      <c r="M70" s="1">
+      <c r="M70" s="2">
         <v>46391</v>
       </c>
       <c r="N70" t="s">
@@ -13662,7 +13688,7 @@
       <c r="L71" t="s">
         <v>725</v>
       </c>
-      <c r="M71" s="1">
+      <c r="M71" s="2">
         <v>46391</v>
       </c>
       <c r="N71" t="s">
@@ -13706,7 +13732,7 @@
       <c r="L72" t="s">
         <v>725</v>
       </c>
-      <c r="M72" s="1">
+      <c r="M72" s="2">
         <v>46391</v>
       </c>
       <c r="N72" t="s">
@@ -13750,7 +13776,7 @@
       <c r="L73" t="s">
         <v>725</v>
       </c>
-      <c r="M73" s="1">
+      <c r="M73" s="2">
         <v>46391</v>
       </c>
       <c r="N73" t="s">
@@ -13794,7 +13820,7 @@
       <c r="L74" t="s">
         <v>725</v>
       </c>
-      <c r="M74" s="1">
+      <c r="M74" s="2">
         <v>46391</v>
       </c>
       <c r="N74" t="s">
@@ -13838,7 +13864,7 @@
       <c r="L75" t="s">
         <v>725</v>
       </c>
-      <c r="M75" s="1">
+      <c r="M75" s="2">
         <v>46391</v>
       </c>
       <c r="N75" t="s">
@@ -13882,7 +13908,7 @@
       <c r="L76" t="s">
         <v>725</v>
       </c>
-      <c r="M76" s="1">
+      <c r="M76" s="2">
         <v>46391</v>
       </c>
       <c r="N76" t="s">
@@ -13926,7 +13952,7 @@
       <c r="L77" t="s">
         <v>725</v>
       </c>
-      <c r="M77" s="1">
+      <c r="M77" s="2">
         <v>46391</v>
       </c>
       <c r="N77" t="s">
@@ -13970,7 +13996,7 @@
       <c r="L78" t="s">
         <v>725</v>
       </c>
-      <c r="M78" s="1">
+      <c r="M78" s="2">
         <v>46391</v>
       </c>
       <c r="N78" t="s">
@@ -14014,7 +14040,7 @@
       <c r="L79" t="s">
         <v>725</v>
       </c>
-      <c r="M79" s="1">
+      <c r="M79" s="2">
         <v>46391</v>
       </c>
       <c r="N79" t="s">
@@ -14058,7 +14084,7 @@
       <c r="L80" t="s">
         <v>725</v>
       </c>
-      <c r="M80" s="1">
+      <c r="M80" s="2">
         <v>46391</v>
       </c>
       <c r="N80" t="s">
@@ -14102,7 +14128,7 @@
       <c r="L81" t="s">
         <v>725</v>
       </c>
-      <c r="M81" s="1">
+      <c r="M81" s="2">
         <v>46391</v>
       </c>
       <c r="N81" t="s">
@@ -14146,7 +14172,7 @@
       <c r="L82" t="s">
         <v>725</v>
       </c>
-      <c r="M82" s="1">
+      <c r="M82" s="2">
         <v>46391</v>
       </c>
       <c r="N82" t="s">
@@ -14190,7 +14216,7 @@
       <c r="L83" t="s">
         <v>725</v>
       </c>
-      <c r="M83" s="1">
+      <c r="M83" s="2">
         <v>46391</v>
       </c>
       <c r="N83" t="s">
@@ -14234,7 +14260,7 @@
       <c r="L84" t="s">
         <v>725</v>
       </c>
-      <c r="M84" s="1">
+      <c r="M84" s="2">
         <v>46391</v>
       </c>
       <c r="N84" t="s">
@@ -14278,7 +14304,7 @@
       <c r="L85" t="s">
         <v>725</v>
       </c>
-      <c r="M85" s="1">
+      <c r="M85" s="2">
         <v>46391</v>
       </c>
       <c r="N85" t="s">
@@ -14322,7 +14348,7 @@
       <c r="L86" t="s">
         <v>725</v>
       </c>
-      <c r="M86" s="1">
+      <c r="M86" s="2">
         <v>46391</v>
       </c>
       <c r="N86" t="s">
@@ -14366,7 +14392,7 @@
       <c r="L87" t="s">
         <v>725</v>
       </c>
-      <c r="M87" s="1">
+      <c r="M87" s="2">
         <v>46391</v>
       </c>
       <c r="N87" t="s">
@@ -14410,7 +14436,7 @@
       <c r="L88" t="s">
         <v>725</v>
       </c>
-      <c r="M88" s="1">
+      <c r="M88" s="2">
         <v>46391</v>
       </c>
       <c r="N88" t="s">
@@ -14454,7 +14480,7 @@
       <c r="L89" t="s">
         <v>725</v>
       </c>
-      <c r="M89" s="1">
+      <c r="M89" s="2">
         <v>46391</v>
       </c>
       <c r="N89" t="s">
@@ -14498,7 +14524,7 @@
       <c r="L90" t="s">
         <v>725</v>
       </c>
-      <c r="M90" s="1">
+      <c r="M90" s="2">
         <v>46391</v>
       </c>
       <c r="N90" t="s">
@@ -14583,7 +14609,7 @@
       <c r="L92" t="s">
         <v>725</v>
       </c>
-      <c r="M92" s="1">
+      <c r="M92" s="2">
         <v>46391</v>
       </c>
       <c r="N92" t="s">
@@ -14627,7 +14653,7 @@
       <c r="L93" t="s">
         <v>725</v>
       </c>
-      <c r="M93" s="1">
+      <c r="M93" s="2">
         <v>46391</v>
       </c>
       <c r="N93" t="s">
@@ -14671,7 +14697,7 @@
       <c r="L94" t="s">
         <v>725</v>
       </c>
-      <c r="M94" s="1">
+      <c r="M94" s="2">
         <v>46391</v>
       </c>
       <c r="N94" t="s">
@@ -14715,7 +14741,7 @@
       <c r="L95" t="s">
         <v>725</v>
       </c>
-      <c r="M95" s="1">
+      <c r="M95" s="2">
         <v>46391</v>
       </c>
       <c r="N95" t="s">
@@ -14759,7 +14785,7 @@
       <c r="L96" t="s">
         <v>725</v>
       </c>
-      <c r="M96" s="1">
+      <c r="M96" s="2">
         <v>46391</v>
       </c>
       <c r="N96" t="s">
@@ -14803,7 +14829,7 @@
       <c r="L97" t="s">
         <v>725</v>
       </c>
-      <c r="M97" s="1">
+      <c r="M97" s="2">
         <v>46391</v>
       </c>
       <c r="N97" t="s">
@@ -14847,7 +14873,7 @@
       <c r="L98" t="s">
         <v>725</v>
       </c>
-      <c r="M98" s="1">
+      <c r="M98" s="2">
         <v>46391</v>
       </c>
       <c r="N98" t="s">
@@ -14891,7 +14917,7 @@
       <c r="L99" t="s">
         <v>725</v>
       </c>
-      <c r="M99" s="1">
+      <c r="M99" s="2">
         <v>46391</v>
       </c>
       <c r="N99" t="s">
@@ -14935,7 +14961,7 @@
       <c r="L100" t="s">
         <v>725</v>
       </c>
-      <c r="M100" s="1">
+      <c r="M100" s="2">
         <v>46391</v>
       </c>
       <c r="N100" t="s">
@@ -14979,7 +15005,7 @@
       <c r="L101" t="s">
         <v>725</v>
       </c>
-      <c r="M101" s="1">
+      <c r="M101" s="2">
         <v>46391</v>
       </c>
       <c r="N101" t="s">
@@ -15023,7 +15049,7 @@
       <c r="L102" t="s">
         <v>725</v>
       </c>
-      <c r="M102" s="1">
+      <c r="M102" s="2">
         <v>46391</v>
       </c>
       <c r="N102" t="s">
@@ -15067,7 +15093,7 @@
       <c r="L103" t="s">
         <v>725</v>
       </c>
-      <c r="M103" s="1">
+      <c r="M103" s="2">
         <v>46391</v>
       </c>
       <c r="N103" t="s">
@@ -15111,7 +15137,7 @@
       <c r="L104" t="s">
         <v>725</v>
       </c>
-      <c r="M104" s="1">
+      <c r="M104" s="2">
         <v>46391</v>
       </c>
       <c r="N104" t="s">
@@ -15155,7 +15181,7 @@
       <c r="L105" t="s">
         <v>725</v>
       </c>
-      <c r="M105" s="1">
+      <c r="M105" s="2">
         <v>46391</v>
       </c>
       <c r="N105" t="s">
@@ -15199,7 +15225,7 @@
       <c r="L106" t="s">
         <v>725</v>
       </c>
-      <c r="M106" s="1">
+      <c r="M106" s="2">
         <v>46391</v>
       </c>
       <c r="N106" t="s">
@@ -15243,7 +15269,7 @@
       <c r="L107" t="s">
         <v>725</v>
       </c>
-      <c r="M107" s="1">
+      <c r="M107" s="2">
         <v>46391</v>
       </c>
       <c r="N107" t="s">
@@ -15287,7 +15313,7 @@
       <c r="L108" t="s">
         <v>725</v>
       </c>
-      <c r="M108" s="1">
+      <c r="M108" s="2">
         <v>46391</v>
       </c>
       <c r="N108" t="s">
@@ -15331,7 +15357,7 @@
       <c r="L109" t="s">
         <v>725</v>
       </c>
-      <c r="M109" s="1">
+      <c r="M109" s="2">
         <v>46391</v>
       </c>
       <c r="N109" t="s">
@@ -15375,7 +15401,7 @@
       <c r="L110" t="s">
         <v>725</v>
       </c>
-      <c r="M110" s="1">
+      <c r="M110" s="2">
         <v>46391</v>
       </c>
       <c r="N110" t="s">
@@ -15419,7 +15445,7 @@
       <c r="L111" t="s">
         <v>725</v>
       </c>
-      <c r="M111" s="1">
+      <c r="M111" s="2">
         <v>46391</v>
       </c>
       <c r="N111" t="s">
@@ -15463,7 +15489,7 @@
       <c r="L112" t="s">
         <v>725</v>
       </c>
-      <c r="M112" s="1">
+      <c r="M112" s="2">
         <v>46391</v>
       </c>
       <c r="N112" t="s">
@@ -15507,7 +15533,7 @@
       <c r="L113" t="s">
         <v>725</v>
       </c>
-      <c r="M113" s="1">
+      <c r="M113" s="2">
         <v>46391</v>
       </c>
       <c r="N113" t="s">
@@ -15551,7 +15577,7 @@
       <c r="L114" t="s">
         <v>725</v>
       </c>
-      <c r="M114" s="1">
+      <c r="M114" s="2">
         <v>46391</v>
       </c>
       <c r="N114" t="s">
@@ -15595,7 +15621,7 @@
       <c r="L115" t="s">
         <v>725</v>
       </c>
-      <c r="M115" s="1">
+      <c r="M115" s="2">
         <v>46391</v>
       </c>
       <c r="N115" t="s">
@@ -15639,7 +15665,7 @@
       <c r="L116" t="s">
         <v>725</v>
       </c>
-      <c r="M116" s="1">
+      <c r="M116" s="2">
         <v>46391</v>
       </c>
       <c r="N116" t="s">
@@ -15683,7 +15709,7 @@
       <c r="L117" t="s">
         <v>725</v>
       </c>
-      <c r="M117" s="1">
+      <c r="M117" s="2">
         <v>46391</v>
       </c>
       <c r="N117" t="s">
@@ -15727,7 +15753,7 @@
       <c r="L118" t="s">
         <v>725</v>
       </c>
-      <c r="M118" s="1">
+      <c r="M118" s="2">
         <v>46391</v>
       </c>
       <c r="N118" t="s">
@@ -15771,7 +15797,7 @@
       <c r="L119" t="s">
         <v>725</v>
       </c>
-      <c r="M119" s="1">
+      <c r="M119" s="2">
         <v>46391</v>
       </c>
       <c r="N119" t="s">
@@ -15815,7 +15841,7 @@
       <c r="L120" t="s">
         <v>725</v>
       </c>
-      <c r="M120" s="1">
+      <c r="M120" s="2">
         <v>46391</v>
       </c>
       <c r="N120" t="s">
@@ -15859,7 +15885,7 @@
       <c r="L121" t="s">
         <v>725</v>
       </c>
-      <c r="M121" s="1">
+      <c r="M121" s="2">
         <v>46391</v>
       </c>
       <c r="N121" t="s">
@@ -15903,7 +15929,7 @@
       <c r="L122" t="s">
         <v>725</v>
       </c>
-      <c r="M122" s="1">
+      <c r="M122" s="2">
         <v>46391</v>
       </c>
       <c r="N122" t="s">
@@ -15947,7 +15973,7 @@
       <c r="L123" t="s">
         <v>725</v>
       </c>
-      <c r="M123" s="1">
+      <c r="M123" s="2">
         <v>46391</v>
       </c>
       <c r="N123" t="s">
@@ -15991,7 +16017,7 @@
       <c r="L124" t="s">
         <v>725</v>
       </c>
-      <c r="M124" s="1">
+      <c r="M124" s="2">
         <v>46391</v>
       </c>
       <c r="N124" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (22/10/2026 12:53)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2205,16 +2205,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2230,7 +2222,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2238,30 +2230,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2561,55 +2535,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2653,7 +2627,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2697,7 +2671,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2741,7 +2715,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2911,7 +2885,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2955,7 +2929,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -3002,7 +2976,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3125,7 +3099,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -3169,7 +3143,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3213,7 +3187,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3257,7 +3231,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3304,7 +3278,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3348,7 +3322,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3474,7 +3448,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3518,7 +3492,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3603,7 +3577,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3650,7 +3624,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3697,7 +3671,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3741,7 +3715,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3785,7 +3759,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3870,7 +3844,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3955,7 +3929,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -4002,7 +3976,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4046,7 +4020,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4090,7 +4064,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4175,7 +4149,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4219,7 +4193,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4263,7 +4237,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4348,7 +4322,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4392,7 +4366,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4436,7 +4410,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4480,7 +4454,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4647,7 +4621,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4691,7 +4665,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4735,7 +4709,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4779,7 +4753,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4826,7 +4800,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4870,7 +4844,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4952,7 +4926,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4996,7 +4970,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5084,7 +5058,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5128,7 +5102,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5175,7 +5149,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5219,7 +5193,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -5263,7 +5237,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5307,7 +5281,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5351,7 +5325,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5398,7 +5372,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5442,7 +5416,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5489,7 +5463,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5533,7 +5507,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5580,7 +5554,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5668,7 +5642,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5712,7 +5686,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5756,7 +5730,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5800,7 +5774,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5844,7 +5818,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5888,7 +5862,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5973,7 +5947,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6017,7 +5991,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -6061,7 +6035,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -6105,7 +6079,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -6149,7 +6123,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -6193,7 +6167,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6237,7 +6211,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6281,7 +6255,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6328,7 +6302,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6372,7 +6346,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6416,7 +6390,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6460,7 +6434,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6504,7 +6478,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6592,7 +6566,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6636,7 +6610,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6680,7 +6654,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6768,7 +6742,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6812,7 +6786,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6938,7 +6912,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6982,7 +6956,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7026,7 +7000,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7070,7 +7044,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7152,7 +7126,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7196,7 +7170,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7243,7 +7217,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7287,7 +7261,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7413,7 +7387,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7457,7 +7431,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7542,7 +7516,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7586,7 +7560,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7630,7 +7604,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7674,7 +7648,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7718,7 +7692,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7762,7 +7736,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7806,7 +7780,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7850,7 +7824,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7935,7 +7909,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8102,7 +8076,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8146,7 +8120,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8190,7 +8164,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8234,7 +8208,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8278,7 +8252,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8322,7 +8296,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8366,7 +8340,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8451,7 +8425,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8495,7 +8469,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8580,7 +8554,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8706,7 +8680,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8750,7 +8724,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8835,7 +8809,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8879,7 +8853,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8923,7 +8897,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8967,7 +8941,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -9011,7 +8985,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -9055,7 +9029,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9099,7 +9073,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9143,7 +9117,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -9228,7 +9202,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9395,7 +9369,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9439,7 +9413,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9483,7 +9457,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9527,7 +9501,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9612,7 +9586,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9656,7 +9630,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9700,7 +9674,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9744,7 +9718,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9788,7 +9762,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9832,7 +9806,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9876,7 +9850,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9920,7 +9894,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9964,7 +9938,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10008,7 +9982,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10052,7 +10026,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -10096,7 +10070,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10140,7 +10114,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10184,7 +10158,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -10228,7 +10202,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10272,7 +10246,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10316,7 +10290,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -10360,7 +10334,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -10404,7 +10378,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10448,7 +10422,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10492,7 +10466,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10577,7 +10551,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10662,7 +10636,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10677,55 +10651,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11094,8 +11068,8 @@
       <c r="L10" t="s">
         <v>725</v>
       </c>
-      <c r="M10" s="2">
-        <v>46391</v>
+      <c r="M10" s="1">
+        <v>46392</v>
       </c>
       <c r="N10" t="s">
         <v>726</v>
@@ -11138,8 +11112,8 @@
       <c r="L11" t="s">
         <v>725</v>
       </c>
-      <c r="M11" s="2">
-        <v>46391</v>
+      <c r="M11" s="1">
+        <v>46392</v>
       </c>
       <c r="N11" t="s">
         <v>726</v>
@@ -11346,8 +11320,8 @@
       <c r="L16" t="s">
         <v>725</v>
       </c>
-      <c r="M16" s="2">
-        <v>46391</v>
+      <c r="M16" s="1">
+        <v>46392</v>
       </c>
       <c r="N16" t="s">
         <v>726</v>
@@ -11472,8 +11446,8 @@
       <c r="L19" t="s">
         <v>725</v>
       </c>
-      <c r="M19" s="2">
-        <v>46391</v>
+      <c r="M19" s="1">
+        <v>46392</v>
       </c>
       <c r="N19" t="s">
         <v>726</v>
@@ -11516,8 +11490,8 @@
       <c r="L20" t="s">
         <v>725</v>
       </c>
-      <c r="M20" s="2">
-        <v>46391</v>
+      <c r="M20" s="1">
+        <v>46392</v>
       </c>
       <c r="N20" t="s">
         <v>726</v>
@@ -11560,8 +11534,8 @@
       <c r="L21" t="s">
         <v>725</v>
       </c>
-      <c r="M21" s="2">
-        <v>46391</v>
+      <c r="M21" s="1">
+        <v>46392</v>
       </c>
       <c r="N21" t="s">
         <v>726</v>
@@ -11727,8 +11701,8 @@
       <c r="L25" t="s">
         <v>725</v>
       </c>
-      <c r="M25" s="2">
-        <v>46391</v>
+      <c r="M25" s="1">
+        <v>46392</v>
       </c>
       <c r="N25" t="s">
         <v>726</v>
@@ -11853,8 +11827,8 @@
       <c r="L28" t="s">
         <v>725</v>
       </c>
-      <c r="M28" s="2">
-        <v>46391</v>
+      <c r="M28" s="1">
+        <v>46392</v>
       </c>
       <c r="N28" t="s">
         <v>726</v>
@@ -11938,8 +11912,8 @@
       <c r="L30" t="s">
         <v>725</v>
       </c>
-      <c r="M30" s="2">
-        <v>46391</v>
+      <c r="M30" s="1">
+        <v>46392</v>
       </c>
       <c r="N30" t="s">
         <v>726</v>
@@ -12392,8 +12366,8 @@
       <c r="L41" t="s">
         <v>725</v>
       </c>
-      <c r="M41" s="2">
-        <v>46391</v>
+      <c r="M41" s="1">
+        <v>46392</v>
       </c>
       <c r="N41" t="s">
         <v>726</v>
@@ -12477,8 +12451,8 @@
       <c r="L43" t="s">
         <v>725</v>
       </c>
-      <c r="M43" s="2">
-        <v>46391</v>
+      <c r="M43" s="1">
+        <v>46392</v>
       </c>
       <c r="N43" t="s">
         <v>726</v>
@@ -12521,8 +12495,8 @@
       <c r="L44" t="s">
         <v>725</v>
       </c>
-      <c r="M44" s="2">
-        <v>46391</v>
+      <c r="M44" s="1">
+        <v>46392</v>
       </c>
       <c r="N44" t="s">
         <v>726</v>
@@ -12565,8 +12539,8 @@
       <c r="L45" t="s">
         <v>725</v>
       </c>
-      <c r="M45" s="2">
-        <v>46391</v>
+      <c r="M45" s="1">
+        <v>46392</v>
       </c>
       <c r="N45" t="s">
         <v>726</v>
@@ -12691,8 +12665,8 @@
       <c r="L48" t="s">
         <v>725</v>
       </c>
-      <c r="M48" s="2">
-        <v>46391</v>
+      <c r="M48" s="1">
+        <v>46392</v>
       </c>
       <c r="N48" t="s">
         <v>726</v>
@@ -12735,8 +12709,8 @@
       <c r="L49" t="s">
         <v>723</v>
       </c>
-      <c r="M49" s="2">
-        <v>46326</v>
+      <c r="M49" s="1">
+        <v>46327</v>
       </c>
       <c r="N49" t="s">
         <v>726</v>
@@ -12779,8 +12753,8 @@
       <c r="L50" t="s">
         <v>723</v>
       </c>
-      <c r="M50" s="2">
-        <v>46326</v>
+      <c r="M50" s="1">
+        <v>46327</v>
       </c>
       <c r="N50" t="s">
         <v>726</v>
@@ -12823,8 +12797,8 @@
       <c r="L51" t="s">
         <v>725</v>
       </c>
-      <c r="M51" s="2">
-        <v>46391</v>
+      <c r="M51" s="1">
+        <v>46392</v>
       </c>
       <c r="N51" t="s">
         <v>726</v>
@@ -12867,8 +12841,8 @@
       <c r="L52" t="s">
         <v>725</v>
       </c>
-      <c r="M52" s="2">
-        <v>46391</v>
+      <c r="M52" s="1">
+        <v>46392</v>
       </c>
       <c r="N52" t="s">
         <v>726</v>
@@ -12911,8 +12885,8 @@
       <c r="L53" t="s">
         <v>725</v>
       </c>
-      <c r="M53" s="2">
-        <v>46391</v>
+      <c r="M53" s="1">
+        <v>46392</v>
       </c>
       <c r="N53" t="s">
         <v>726</v>
@@ -12955,8 +12929,8 @@
       <c r="L54" t="s">
         <v>725</v>
       </c>
-      <c r="M54" s="2">
-        <v>46391</v>
+      <c r="M54" s="1">
+        <v>46392</v>
       </c>
       <c r="N54" t="s">
         <v>726</v>
@@ -12999,8 +12973,8 @@
       <c r="L55" t="s">
         <v>725</v>
       </c>
-      <c r="M55" s="2">
-        <v>46391</v>
+      <c r="M55" s="1">
+        <v>46392</v>
       </c>
       <c r="N55" t="s">
         <v>726</v>
@@ -13166,8 +13140,8 @@
       <c r="L59" t="s">
         <v>725</v>
       </c>
-      <c r="M59" s="2">
-        <v>46391</v>
+      <c r="M59" s="1">
+        <v>46392</v>
       </c>
       <c r="N59" t="s">
         <v>726</v>
@@ -13292,8 +13266,8 @@
       <c r="L62" t="s">
         <v>725</v>
       </c>
-      <c r="M62" s="2">
-        <v>46391</v>
+      <c r="M62" s="1">
+        <v>46392</v>
       </c>
       <c r="N62" t="s">
         <v>726</v>
@@ -13336,8 +13310,8 @@
       <c r="L63" t="s">
         <v>725</v>
       </c>
-      <c r="M63" s="2">
-        <v>46391</v>
+      <c r="M63" s="1">
+        <v>46392</v>
       </c>
       <c r="N63" t="s">
         <v>726</v>
@@ -13380,8 +13354,8 @@
       <c r="L64" t="s">
         <v>725</v>
       </c>
-      <c r="M64" s="2">
-        <v>46391</v>
+      <c r="M64" s="1">
+        <v>46392</v>
       </c>
       <c r="N64" t="s">
         <v>726</v>
@@ -13424,8 +13398,8 @@
       <c r="L65" t="s">
         <v>725</v>
       </c>
-      <c r="M65" s="2">
-        <v>46391</v>
+      <c r="M65" s="1">
+        <v>46392</v>
       </c>
       <c r="N65" t="s">
         <v>726</v>
@@ -13468,8 +13442,8 @@
       <c r="L66" t="s">
         <v>725</v>
       </c>
-      <c r="M66" s="2">
-        <v>46391</v>
+      <c r="M66" s="1">
+        <v>46392</v>
       </c>
       <c r="N66" t="s">
         <v>726</v>
@@ -13512,8 +13486,8 @@
       <c r="L67" t="s">
         <v>725</v>
       </c>
-      <c r="M67" s="2">
-        <v>46391</v>
+      <c r="M67" s="1">
+        <v>46392</v>
       </c>
       <c r="N67" t="s">
         <v>726</v>
@@ -13556,8 +13530,8 @@
       <c r="L68" t="s">
         <v>725</v>
       </c>
-      <c r="M68" s="2">
-        <v>46391</v>
+      <c r="M68" s="1">
+        <v>46392</v>
       </c>
       <c r="N68" t="s">
         <v>726</v>
@@ -13600,8 +13574,8 @@
       <c r="L69" t="s">
         <v>725</v>
       </c>
-      <c r="M69" s="2">
-        <v>46391</v>
+      <c r="M69" s="1">
+        <v>46392</v>
       </c>
       <c r="N69" t="s">
         <v>726</v>
@@ -13644,8 +13618,8 @@
       <c r="L70" t="s">
         <v>725</v>
       </c>
-      <c r="M70" s="2">
-        <v>46391</v>
+      <c r="M70" s="1">
+        <v>46392</v>
       </c>
       <c r="N70" t="s">
         <v>726</v>
@@ -13688,8 +13662,8 @@
       <c r="L71" t="s">
         <v>725</v>
       </c>
-      <c r="M71" s="2">
-        <v>46391</v>
+      <c r="M71" s="1">
+        <v>46392</v>
       </c>
       <c r="N71" t="s">
         <v>726</v>
@@ -13732,8 +13706,8 @@
       <c r="L72" t="s">
         <v>725</v>
       </c>
-      <c r="M72" s="2">
-        <v>46391</v>
+      <c r="M72" s="1">
+        <v>46392</v>
       </c>
       <c r="N72" t="s">
         <v>726</v>
@@ -13776,8 +13750,8 @@
       <c r="L73" t="s">
         <v>725</v>
       </c>
-      <c r="M73" s="2">
-        <v>46391</v>
+      <c r="M73" s="1">
+        <v>46392</v>
       </c>
       <c r="N73" t="s">
         <v>726</v>
@@ -13820,8 +13794,8 @@
       <c r="L74" t="s">
         <v>725</v>
       </c>
-      <c r="M74" s="2">
-        <v>46391</v>
+      <c r="M74" s="1">
+        <v>46392</v>
       </c>
       <c r="N74" t="s">
         <v>726</v>
@@ -13864,8 +13838,8 @@
       <c r="L75" t="s">
         <v>725</v>
       </c>
-      <c r="M75" s="2">
-        <v>46391</v>
+      <c r="M75" s="1">
+        <v>46392</v>
       </c>
       <c r="N75" t="s">
         <v>726</v>
@@ -13908,8 +13882,8 @@
       <c r="L76" t="s">
         <v>725</v>
       </c>
-      <c r="M76" s="2">
-        <v>46391</v>
+      <c r="M76" s="1">
+        <v>46392</v>
       </c>
       <c r="N76" t="s">
         <v>726</v>
@@ -13952,8 +13926,8 @@
       <c r="L77" t="s">
         <v>725</v>
       </c>
-      <c r="M77" s="2">
-        <v>46391</v>
+      <c r="M77" s="1">
+        <v>46392</v>
       </c>
       <c r="N77" t="s">
         <v>726</v>
@@ -13996,8 +13970,8 @@
       <c r="L78" t="s">
         <v>725</v>
       </c>
-      <c r="M78" s="2">
-        <v>46391</v>
+      <c r="M78" s="1">
+        <v>46392</v>
       </c>
       <c r="N78" t="s">
         <v>726</v>
@@ -14040,8 +14014,8 @@
       <c r="L79" t="s">
         <v>725</v>
       </c>
-      <c r="M79" s="2">
-        <v>46391</v>
+      <c r="M79" s="1">
+        <v>46392</v>
       </c>
       <c r="N79" t="s">
         <v>726</v>
@@ -14084,8 +14058,8 @@
       <c r="L80" t="s">
         <v>725</v>
       </c>
-      <c r="M80" s="2">
-        <v>46391</v>
+      <c r="M80" s="1">
+        <v>46392</v>
       </c>
       <c r="N80" t="s">
         <v>726</v>
@@ -14128,8 +14102,8 @@
       <c r="L81" t="s">
         <v>725</v>
       </c>
-      <c r="M81" s="2">
-        <v>46391</v>
+      <c r="M81" s="1">
+        <v>46392</v>
       </c>
       <c r="N81" t="s">
         <v>726</v>
@@ -14172,8 +14146,8 @@
       <c r="L82" t="s">
         <v>725</v>
       </c>
-      <c r="M82" s="2">
-        <v>46391</v>
+      <c r="M82" s="1">
+        <v>46392</v>
       </c>
       <c r="N82" t="s">
         <v>726</v>
@@ -14216,8 +14190,8 @@
       <c r="L83" t="s">
         <v>725</v>
       </c>
-      <c r="M83" s="2">
-        <v>46391</v>
+      <c r="M83" s="1">
+        <v>46392</v>
       </c>
       <c r="N83" t="s">
         <v>726</v>
@@ -14260,8 +14234,8 @@
       <c r="L84" t="s">
         <v>725</v>
       </c>
-      <c r="M84" s="2">
-        <v>46391</v>
+      <c r="M84" s="1">
+        <v>46392</v>
       </c>
       <c r="N84" t="s">
         <v>726</v>
@@ -14304,8 +14278,8 @@
       <c r="L85" t="s">
         <v>725</v>
       </c>
-      <c r="M85" s="2">
-        <v>46391</v>
+      <c r="M85" s="1">
+        <v>46392</v>
       </c>
       <c r="N85" t="s">
         <v>726</v>
@@ -14348,8 +14322,8 @@
       <c r="L86" t="s">
         <v>725</v>
       </c>
-      <c r="M86" s="2">
-        <v>46391</v>
+      <c r="M86" s="1">
+        <v>46392</v>
       </c>
       <c r="N86" t="s">
         <v>726</v>
@@ -14392,8 +14366,8 @@
       <c r="L87" t="s">
         <v>725</v>
       </c>
-      <c r="M87" s="2">
-        <v>46391</v>
+      <c r="M87" s="1">
+        <v>46392</v>
       </c>
       <c r="N87" t="s">
         <v>726</v>
@@ -14436,8 +14410,8 @@
       <c r="L88" t="s">
         <v>725</v>
       </c>
-      <c r="M88" s="2">
-        <v>46391</v>
+      <c r="M88" s="1">
+        <v>46392</v>
       </c>
       <c r="N88" t="s">
         <v>726</v>
@@ -14480,8 +14454,8 @@
       <c r="L89" t="s">
         <v>725</v>
       </c>
-      <c r="M89" s="2">
-        <v>46391</v>
+      <c r="M89" s="1">
+        <v>46392</v>
       </c>
       <c r="N89" t="s">
         <v>726</v>
@@ -14524,8 +14498,8 @@
       <c r="L90" t="s">
         <v>725</v>
       </c>
-      <c r="M90" s="2">
-        <v>46391</v>
+      <c r="M90" s="1">
+        <v>46392</v>
       </c>
       <c r="N90" t="s">
         <v>726</v>
@@ -14609,8 +14583,8 @@
       <c r="L92" t="s">
         <v>725</v>
       </c>
-      <c r="M92" s="2">
-        <v>46391</v>
+      <c r="M92" s="1">
+        <v>46392</v>
       </c>
       <c r="N92" t="s">
         <v>726</v>
@@ -14653,8 +14627,8 @@
       <c r="L93" t="s">
         <v>725</v>
       </c>
-      <c r="M93" s="2">
-        <v>46391</v>
+      <c r="M93" s="1">
+        <v>46392</v>
       </c>
       <c r="N93" t="s">
         <v>726</v>
@@ -14697,8 +14671,8 @@
       <c r="L94" t="s">
         <v>725</v>
       </c>
-      <c r="M94" s="2">
-        <v>46391</v>
+      <c r="M94" s="1">
+        <v>46392</v>
       </c>
       <c r="N94" t="s">
         <v>726</v>
@@ -14741,8 +14715,8 @@
       <c r="L95" t="s">
         <v>725</v>
       </c>
-      <c r="M95" s="2">
-        <v>46391</v>
+      <c r="M95" s="1">
+        <v>46392</v>
       </c>
       <c r="N95" t="s">
         <v>726</v>
@@ -14785,8 +14759,8 @@
       <c r="L96" t="s">
         <v>725</v>
       </c>
-      <c r="M96" s="2">
-        <v>46391</v>
+      <c r="M96" s="1">
+        <v>46392</v>
       </c>
       <c r="N96" t="s">
         <v>726</v>
@@ -14829,8 +14803,8 @@
       <c r="L97" t="s">
         <v>725</v>
       </c>
-      <c r="M97" s="2">
-        <v>46391</v>
+      <c r="M97" s="1">
+        <v>46392</v>
       </c>
       <c r="N97" t="s">
         <v>726</v>
@@ -14873,8 +14847,8 @@
       <c r="L98" t="s">
         <v>725</v>
       </c>
-      <c r="M98" s="2">
-        <v>46391</v>
+      <c r="M98" s="1">
+        <v>46392</v>
       </c>
       <c r="N98" t="s">
         <v>726</v>
@@ -14917,8 +14891,8 @@
       <c r="L99" t="s">
         <v>725</v>
       </c>
-      <c r="M99" s="2">
-        <v>46391</v>
+      <c r="M99" s="1">
+        <v>46392</v>
       </c>
       <c r="N99" t="s">
         <v>726</v>
@@ -14961,8 +14935,8 @@
       <c r="L100" t="s">
         <v>725</v>
       </c>
-      <c r="M100" s="2">
-        <v>46391</v>
+      <c r="M100" s="1">
+        <v>46392</v>
       </c>
       <c r="N100" t="s">
         <v>726</v>
@@ -15005,8 +14979,8 @@
       <c r="L101" t="s">
         <v>725</v>
       </c>
-      <c r="M101" s="2">
-        <v>46391</v>
+      <c r="M101" s="1">
+        <v>46392</v>
       </c>
       <c r="N101" t="s">
         <v>726</v>
@@ -15049,8 +15023,8 @@
       <c r="L102" t="s">
         <v>725</v>
       </c>
-      <c r="M102" s="2">
-        <v>46391</v>
+      <c r="M102" s="1">
+        <v>46392</v>
       </c>
       <c r="N102" t="s">
         <v>726</v>
@@ -15093,8 +15067,8 @@
       <c r="L103" t="s">
         <v>725</v>
       </c>
-      <c r="M103" s="2">
-        <v>46391</v>
+      <c r="M103" s="1">
+        <v>46392</v>
       </c>
       <c r="N103" t="s">
         <v>726</v>
@@ -15137,8 +15111,8 @@
       <c r="L104" t="s">
         <v>725</v>
       </c>
-      <c r="M104" s="2">
-        <v>46391</v>
+      <c r="M104" s="1">
+        <v>46392</v>
       </c>
       <c r="N104" t="s">
         <v>726</v>
@@ -15181,8 +15155,8 @@
       <c r="L105" t="s">
         <v>725</v>
       </c>
-      <c r="M105" s="2">
-        <v>46391</v>
+      <c r="M105" s="1">
+        <v>46392</v>
       </c>
       <c r="N105" t="s">
         <v>726</v>
@@ -15225,8 +15199,8 @@
       <c r="L106" t="s">
         <v>725</v>
       </c>
-      <c r="M106" s="2">
-        <v>46391</v>
+      <c r="M106" s="1">
+        <v>46392</v>
       </c>
       <c r="N106" t="s">
         <v>726</v>
@@ -15269,8 +15243,8 @@
       <c r="L107" t="s">
         <v>725</v>
       </c>
-      <c r="M107" s="2">
-        <v>46391</v>
+      <c r="M107" s="1">
+        <v>46392</v>
       </c>
       <c r="N107" t="s">
         <v>726</v>
@@ -15313,8 +15287,8 @@
       <c r="L108" t="s">
         <v>725</v>
       </c>
-      <c r="M108" s="2">
-        <v>46391</v>
+      <c r="M108" s="1">
+        <v>46392</v>
       </c>
       <c r="N108" t="s">
         <v>726</v>
@@ -15357,8 +15331,8 @@
       <c r="L109" t="s">
         <v>725</v>
       </c>
-      <c r="M109" s="2">
-        <v>46391</v>
+      <c r="M109" s="1">
+        <v>46392</v>
       </c>
       <c r="N109" t="s">
         <v>726</v>
@@ -15401,8 +15375,8 @@
       <c r="L110" t="s">
         <v>725</v>
       </c>
-      <c r="M110" s="2">
-        <v>46391</v>
+      <c r="M110" s="1">
+        <v>46392</v>
       </c>
       <c r="N110" t="s">
         <v>726</v>
@@ -15445,8 +15419,8 @@
       <c r="L111" t="s">
         <v>725</v>
       </c>
-      <c r="M111" s="2">
-        <v>46391</v>
+      <c r="M111" s="1">
+        <v>46392</v>
       </c>
       <c r="N111" t="s">
         <v>726</v>
@@ -15489,8 +15463,8 @@
       <c r="L112" t="s">
         <v>725</v>
       </c>
-      <c r="M112" s="2">
-        <v>46391</v>
+      <c r="M112" s="1">
+        <v>46392</v>
       </c>
       <c r="N112" t="s">
         <v>726</v>
@@ -15533,8 +15507,8 @@
       <c r="L113" t="s">
         <v>725</v>
       </c>
-      <c r="M113" s="2">
-        <v>46391</v>
+      <c r="M113" s="1">
+        <v>46392</v>
       </c>
       <c r="N113" t="s">
         <v>726</v>
@@ -15577,8 +15551,8 @@
       <c r="L114" t="s">
         <v>725</v>
       </c>
-      <c r="M114" s="2">
-        <v>46391</v>
+      <c r="M114" s="1">
+        <v>46392</v>
       </c>
       <c r="N114" t="s">
         <v>726</v>
@@ -15621,8 +15595,8 @@
       <c r="L115" t="s">
         <v>725</v>
       </c>
-      <c r="M115" s="2">
-        <v>46391</v>
+      <c r="M115" s="1">
+        <v>46392</v>
       </c>
       <c r="N115" t="s">
         <v>726</v>
@@ -15665,8 +15639,8 @@
       <c r="L116" t="s">
         <v>725</v>
       </c>
-      <c r="M116" s="2">
-        <v>46391</v>
+      <c r="M116" s="1">
+        <v>46392</v>
       </c>
       <c r="N116" t="s">
         <v>726</v>
@@ -15709,8 +15683,8 @@
       <c r="L117" t="s">
         <v>725</v>
       </c>
-      <c r="M117" s="2">
-        <v>46391</v>
+      <c r="M117" s="1">
+        <v>46392</v>
       </c>
       <c r="N117" t="s">
         <v>726</v>
@@ -15753,8 +15727,8 @@
       <c r="L118" t="s">
         <v>725</v>
       </c>
-      <c r="M118" s="2">
-        <v>46391</v>
+      <c r="M118" s="1">
+        <v>46392</v>
       </c>
       <c r="N118" t="s">
         <v>726</v>
@@ -15797,8 +15771,8 @@
       <c r="L119" t="s">
         <v>725</v>
       </c>
-      <c r="M119" s="2">
-        <v>46391</v>
+      <c r="M119" s="1">
+        <v>46392</v>
       </c>
       <c r="N119" t="s">
         <v>726</v>
@@ -15841,8 +15815,8 @@
       <c r="L120" t="s">
         <v>725</v>
       </c>
-      <c r="M120" s="2">
-        <v>46391</v>
+      <c r="M120" s="1">
+        <v>46392</v>
       </c>
       <c r="N120" t="s">
         <v>726</v>
@@ -15885,8 +15859,8 @@
       <c r="L121" t="s">
         <v>725</v>
       </c>
-      <c r="M121" s="2">
-        <v>46391</v>
+      <c r="M121" s="1">
+        <v>46392</v>
       </c>
       <c r="N121" t="s">
         <v>726</v>
@@ -15929,8 +15903,8 @@
       <c r="L122" t="s">
         <v>725</v>
       </c>
-      <c r="M122" s="2">
-        <v>46391</v>
+      <c r="M122" s="1">
+        <v>46392</v>
       </c>
       <c r="N122" t="s">
         <v>726</v>
@@ -15973,8 +15947,8 @@
       <c r="L123" t="s">
         <v>725</v>
       </c>
-      <c r="M123" s="2">
-        <v>46391</v>
+      <c r="M123" s="1">
+        <v>46392</v>
       </c>
       <c r="N123" t="s">
         <v>726</v>
@@ -16017,8 +15991,8 @@
       <c r="L124" t="s">
         <v>725</v>
       </c>
-      <c r="M124" s="2">
-        <v>46391</v>
+      <c r="M124" s="1">
+        <v>46392</v>
       </c>
       <c r="N124" t="s">
         <v>726</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (23/10/2026 12:44)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2180,19 +2180,19 @@
     <t>Empenho Solicitado</t>
   </si>
   <si>
+    <t>Selecionada para Cotação</t>
+  </si>
+  <si>
     <t>Selecionada em Plano</t>
   </si>
   <si>
-    <t>Aguardando Intenção de Recurso</t>
-  </si>
-  <si>
     <t>Mapa Gerado</t>
   </si>
   <si>
+    <t>Validada</t>
+  </si>
+  <si>
     <t>Em Discrepância</t>
-  </si>
-  <si>
-    <t>Validada</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -11060,16 +11060,16 @@
         <v>721</v>
       </c>
       <c r="J10" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K10" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L10" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M10" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N10" t="s">
         <v>726</v>
@@ -11104,16 +11104,16 @@
         <v>721</v>
       </c>
       <c r="J11" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K11" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L11" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M11" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N11" t="s">
         <v>726</v>
@@ -11312,16 +11312,16 @@
         <v>721</v>
       </c>
       <c r="J16" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K16" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L16" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M16" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N16" t="s">
         <v>726</v>
@@ -11435,19 +11435,19 @@
         <v>1323.9</v>
       </c>
       <c r="I19" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J19" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K19" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L19" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M19" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N19" t="s">
         <v>726</v>
@@ -11479,19 +11479,19 @@
         <v>340.73</v>
       </c>
       <c r="I20" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J20" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K20" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L20" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M20" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N20" t="s">
         <v>726</v>
@@ -11526,16 +11526,16 @@
         <v>721</v>
       </c>
       <c r="J21" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K21" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L21" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M21" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N21" t="s">
         <v>726</v>
@@ -11690,19 +11690,19 @@
         <v>21612.9</v>
       </c>
       <c r="I25" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J25" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K25" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L25" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M25" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N25" t="s">
         <v>726</v>
@@ -11819,16 +11819,16 @@
         <v>721</v>
       </c>
       <c r="J28" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K28" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L28" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M28" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N28" t="s">
         <v>726</v>
@@ -11904,16 +11904,16 @@
         <v>721</v>
       </c>
       <c r="J30" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K30" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L30" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M30" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N30" t="s">
         <v>726</v>
@@ -12358,16 +12358,16 @@
         <v>721</v>
       </c>
       <c r="J41" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K41" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L41" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M41" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N41" t="s">
         <v>726</v>
@@ -12440,19 +12440,19 @@
         <v>7890.58</v>
       </c>
       <c r="I43" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J43" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K43" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L43" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M43" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N43" t="s">
         <v>726</v>
@@ -12484,19 +12484,19 @@
         <v>352.52</v>
       </c>
       <c r="I44" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J44" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K44" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L44" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M44" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N44" t="s">
         <v>726</v>
@@ -12528,19 +12528,19 @@
         <v>376.62</v>
       </c>
       <c r="I45" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J45" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K45" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L45" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M45" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N45" t="s">
         <v>726</v>
@@ -12654,19 +12654,19 @@
         <v>3459.72</v>
       </c>
       <c r="I48" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J48" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K48" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L48" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M48" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N48" t="s">
         <v>726</v>
@@ -12698,7 +12698,7 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
-        <v>722</v>
+        <v>385</v>
       </c>
       <c r="J49" t="s">
         <v>723</v>
@@ -12710,7 +12710,7 @@
         <v>723</v>
       </c>
       <c r="M49" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N49" t="s">
         <v>726</v>
@@ -12754,7 +12754,7 @@
         <v>723</v>
       </c>
       <c r="M50" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N50" t="s">
         <v>726</v>
@@ -12789,16 +12789,16 @@
         <v>721</v>
       </c>
       <c r="J51" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K51" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L51" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M51" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N51" t="s">
         <v>726</v>
@@ -12833,16 +12833,16 @@
         <v>721</v>
       </c>
       <c r="J52" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K52" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L52" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M52" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N52" t="s">
         <v>726</v>
@@ -12877,16 +12877,16 @@
         <v>721</v>
       </c>
       <c r="J53" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K53" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L53" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M53" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N53" t="s">
         <v>726</v>
@@ -12918,19 +12918,19 @@
         <v>3875.24</v>
       </c>
       <c r="I54" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J54" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K54" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L54" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M54" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N54" t="s">
         <v>726</v>
@@ -12965,16 +12965,16 @@
         <v>721</v>
       </c>
       <c r="J55" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K55" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L55" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M55" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N55" t="s">
         <v>726</v>
@@ -13129,19 +13129,19 @@
         <v>869.98</v>
       </c>
       <c r="I59" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J59" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K59" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L59" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M59" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N59" t="s">
         <v>726</v>
@@ -13255,19 +13255,19 @@
         <v>204.96</v>
       </c>
       <c r="I62" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J62" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K62" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L62" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M62" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N62" t="s">
         <v>726</v>
@@ -13299,19 +13299,19 @@
         <v>421</v>
       </c>
       <c r="I63" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J63" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K63" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L63" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M63" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N63" t="s">
         <v>726</v>
@@ -13346,16 +13346,16 @@
         <v>721</v>
       </c>
       <c r="J64" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K64" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L64" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M64" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N64" t="s">
         <v>726</v>
@@ -13387,19 +13387,19 @@
         <v>8848.459999999999</v>
       </c>
       <c r="I65" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J65" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K65" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L65" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M65" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N65" t="s">
         <v>726</v>
@@ -13431,19 +13431,19 @@
         <v>297.92</v>
       </c>
       <c r="I66" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J66" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K66" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L66" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M66" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N66" t="s">
         <v>726</v>
@@ -13475,19 +13475,19 @@
         <v>27326.55</v>
       </c>
       <c r="I67" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J67" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K67" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L67" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M67" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N67" t="s">
         <v>726</v>
@@ -13519,19 +13519,19 @@
         <v>806.24</v>
       </c>
       <c r="I68" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J68" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K68" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L68" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M68" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N68" t="s">
         <v>726</v>
@@ -13563,19 +13563,19 @@
         <v>11124.8</v>
       </c>
       <c r="I69" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J69" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K69" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L69" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M69" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N69" t="s">
         <v>726</v>
@@ -13607,19 +13607,19 @@
         <v>1658.28</v>
       </c>
       <c r="I70" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J70" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K70" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L70" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M70" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N70" t="s">
         <v>726</v>
@@ -13651,19 +13651,19 @@
         <v>3968.48</v>
       </c>
       <c r="I71" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J71" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K71" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L71" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M71" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N71" t="s">
         <v>726</v>
@@ -13695,19 +13695,19 @@
         <v>400</v>
       </c>
       <c r="I72" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J72" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K72" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L72" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M72" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N72" t="s">
         <v>726</v>
@@ -13739,19 +13739,19 @@
         <v>3043.76</v>
       </c>
       <c r="I73" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J73" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K73" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L73" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M73" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N73" t="s">
         <v>726</v>
@@ -13783,19 +13783,19 @@
         <v>2048.32</v>
       </c>
       <c r="I74" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J74" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K74" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L74" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M74" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N74" t="s">
         <v>726</v>
@@ -13830,16 +13830,16 @@
         <v>721</v>
       </c>
       <c r="J75" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K75" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L75" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M75" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N75" t="s">
         <v>726</v>
@@ -13874,16 +13874,16 @@
         <v>721</v>
       </c>
       <c r="J76" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K76" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L76" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M76" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N76" t="s">
         <v>726</v>
@@ -13918,16 +13918,16 @@
         <v>721</v>
       </c>
       <c r="J77" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K77" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L77" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M77" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N77" t="s">
         <v>726</v>
@@ -13962,16 +13962,16 @@
         <v>721</v>
       </c>
       <c r="J78" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K78" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L78" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M78" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N78" t="s">
         <v>726</v>
@@ -14006,16 +14006,16 @@
         <v>721</v>
       </c>
       <c r="J79" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K79" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L79" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M79" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N79" t="s">
         <v>726</v>
@@ -14050,16 +14050,16 @@
         <v>721</v>
       </c>
       <c r="J80" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K80" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L80" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M80" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N80" t="s">
         <v>726</v>
@@ -14094,16 +14094,16 @@
         <v>721</v>
       </c>
       <c r="J81" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K81" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L81" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M81" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N81" t="s">
         <v>726</v>
@@ -14138,16 +14138,16 @@
         <v>721</v>
       </c>
       <c r="J82" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K82" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L82" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M82" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N82" t="s">
         <v>726</v>
@@ -14182,16 +14182,16 @@
         <v>721</v>
       </c>
       <c r="J83" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K83" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L83" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M83" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N83" t="s">
         <v>726</v>
@@ -14226,16 +14226,16 @@
         <v>721</v>
       </c>
       <c r="J84" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K84" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L84" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M84" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N84" t="s">
         <v>726</v>
@@ -14270,16 +14270,16 @@
         <v>721</v>
       </c>
       <c r="J85" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K85" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L85" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M85" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N85" t="s">
         <v>726</v>
@@ -14314,16 +14314,16 @@
         <v>721</v>
       </c>
       <c r="J86" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K86" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L86" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M86" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N86" t="s">
         <v>726</v>
@@ -14358,16 +14358,16 @@
         <v>721</v>
       </c>
       <c r="J87" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K87" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L87" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M87" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N87" t="s">
         <v>726</v>
@@ -14402,16 +14402,16 @@
         <v>721</v>
       </c>
       <c r="J88" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K88" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L88" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M88" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N88" t="s">
         <v>726</v>
@@ -14446,16 +14446,16 @@
         <v>721</v>
       </c>
       <c r="J89" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K89" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L89" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M89" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N89" t="s">
         <v>726</v>
@@ -14490,16 +14490,16 @@
         <v>721</v>
       </c>
       <c r="J90" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K90" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L90" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M90" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N90" t="s">
         <v>726</v>
@@ -14534,13 +14534,13 @@
         <v>724</v>
       </c>
       <c r="J91" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="K91" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="L91" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="N91" t="s">
         <v>395</v>
@@ -14575,16 +14575,16 @@
         <v>721</v>
       </c>
       <c r="J92" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K92" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L92" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M92" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N92" t="s">
         <v>726</v>
@@ -14619,16 +14619,16 @@
         <v>721</v>
       </c>
       <c r="J93" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K93" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L93" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M93" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N93" t="s">
         <v>726</v>
@@ -14663,16 +14663,16 @@
         <v>721</v>
       </c>
       <c r="J94" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K94" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L94" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M94" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N94" t="s">
         <v>726</v>
@@ -14707,16 +14707,16 @@
         <v>721</v>
       </c>
       <c r="J95" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K95" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L95" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M95" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N95" t="s">
         <v>726</v>
@@ -14751,16 +14751,16 @@
         <v>721</v>
       </c>
       <c r="J96" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K96" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L96" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M96" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N96" t="s">
         <v>726</v>
@@ -14795,16 +14795,16 @@
         <v>721</v>
       </c>
       <c r="J97" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K97" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L97" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M97" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N97" t="s">
         <v>726</v>
@@ -14839,16 +14839,16 @@
         <v>721</v>
       </c>
       <c r="J98" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K98" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L98" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M98" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N98" t="s">
         <v>726</v>
@@ -14883,16 +14883,16 @@
         <v>721</v>
       </c>
       <c r="J99" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K99" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L99" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M99" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N99" t="s">
         <v>726</v>
@@ -14927,16 +14927,16 @@
         <v>721</v>
       </c>
       <c r="J100" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K100" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L100" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M100" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N100" t="s">
         <v>726</v>
@@ -14971,16 +14971,16 @@
         <v>721</v>
       </c>
       <c r="J101" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K101" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L101" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M101" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N101" t="s">
         <v>726</v>
@@ -15015,16 +15015,16 @@
         <v>721</v>
       </c>
       <c r="J102" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K102" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L102" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M102" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N102" t="s">
         <v>726</v>
@@ -15059,16 +15059,16 @@
         <v>721</v>
       </c>
       <c r="J103" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K103" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L103" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M103" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N103" t="s">
         <v>726</v>
@@ -15103,16 +15103,16 @@
         <v>721</v>
       </c>
       <c r="J104" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K104" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L104" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M104" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N104" t="s">
         <v>726</v>
@@ -15147,16 +15147,16 @@
         <v>721</v>
       </c>
       <c r="J105" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K105" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L105" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M105" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N105" t="s">
         <v>726</v>
@@ -15191,16 +15191,16 @@
         <v>721</v>
       </c>
       <c r="J106" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K106" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L106" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M106" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N106" t="s">
         <v>726</v>
@@ -15235,16 +15235,16 @@
         <v>721</v>
       </c>
       <c r="J107" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K107" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L107" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M107" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N107" t="s">
         <v>726</v>
@@ -15279,16 +15279,16 @@
         <v>721</v>
       </c>
       <c r="J108" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K108" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L108" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M108" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N108" t="s">
         <v>726</v>
@@ -15323,16 +15323,16 @@
         <v>721</v>
       </c>
       <c r="J109" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K109" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L109" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M109" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N109" t="s">
         <v>726</v>
@@ -15367,16 +15367,16 @@
         <v>721</v>
       </c>
       <c r="J110" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K110" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L110" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M110" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N110" t="s">
         <v>726</v>
@@ -15411,16 +15411,16 @@
         <v>721</v>
       </c>
       <c r="J111" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K111" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L111" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M111" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N111" t="s">
         <v>726</v>
@@ -15455,16 +15455,16 @@
         <v>721</v>
       </c>
       <c r="J112" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K112" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L112" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M112" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N112" t="s">
         <v>726</v>
@@ -15499,16 +15499,16 @@
         <v>721</v>
       </c>
       <c r="J113" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K113" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L113" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M113" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N113" t="s">
         <v>726</v>
@@ -15543,16 +15543,16 @@
         <v>721</v>
       </c>
       <c r="J114" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K114" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L114" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M114" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N114" t="s">
         <v>726</v>
@@ -15587,16 +15587,16 @@
         <v>721</v>
       </c>
       <c r="J115" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K115" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L115" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M115" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N115" t="s">
         <v>726</v>
@@ -15631,16 +15631,16 @@
         <v>721</v>
       </c>
       <c r="J116" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K116" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L116" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M116" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N116" t="s">
         <v>726</v>
@@ -15675,16 +15675,16 @@
         <v>721</v>
       </c>
       <c r="J117" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K117" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L117" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M117" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N117" t="s">
         <v>726</v>
@@ -15719,16 +15719,16 @@
         <v>721</v>
       </c>
       <c r="J118" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K118" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L118" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M118" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N118" t="s">
         <v>726</v>
@@ -15763,16 +15763,16 @@
         <v>721</v>
       </c>
       <c r="J119" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K119" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L119" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M119" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N119" t="s">
         <v>726</v>
@@ -15807,16 +15807,16 @@
         <v>721</v>
       </c>
       <c r="J120" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K120" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L120" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M120" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N120" t="s">
         <v>726</v>
@@ -15851,16 +15851,16 @@
         <v>721</v>
       </c>
       <c r="J121" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K121" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L121" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M121" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N121" t="s">
         <v>726</v>
@@ -15895,16 +15895,16 @@
         <v>721</v>
       </c>
       <c r="J122" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K122" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L122" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M122" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N122" t="s">
         <v>726</v>
@@ -15939,16 +15939,16 @@
         <v>721</v>
       </c>
       <c r="J123" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K123" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L123" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M123" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N123" t="s">
         <v>726</v>
@@ -15983,16 +15983,16 @@
         <v>721</v>
       </c>
       <c r="J124" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K124" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="L124" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="M124" s="1">
-        <v>46392</v>
+        <v>46393</v>
       </c>
       <c r="N124" t="s">
         <v>726</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (23/10/2026 14:22)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -2205,8 +2205,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2222,7 +2230,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2230,12 +2238,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2535,55 +2561,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2627,7 +2653,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2671,7 +2697,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2715,7 +2741,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2885,7 +2911,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2929,7 +2955,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2976,7 +3002,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3099,7 +3125,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -3143,7 +3169,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3187,7 +3213,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3231,7 +3257,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3278,7 +3304,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3322,7 +3348,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3448,7 +3474,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3492,7 +3518,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3577,7 +3603,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3624,7 +3650,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3671,7 +3697,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3715,7 +3741,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3759,7 +3785,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3844,7 +3870,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3929,7 +3955,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3976,7 +4002,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4020,7 +4046,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4064,7 +4090,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4149,7 +4175,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4193,7 +4219,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4237,7 +4263,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4322,7 +4348,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4366,7 +4392,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4410,7 +4436,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4454,7 +4480,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4621,7 +4647,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4665,7 +4691,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4709,7 +4735,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4753,7 +4779,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4800,7 +4826,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4844,7 +4870,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4926,7 +4952,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4970,7 +4996,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5058,7 +5084,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5102,7 +5128,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5149,7 +5175,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5193,7 +5219,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -5237,7 +5263,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -5281,7 +5307,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5325,7 +5351,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5372,7 +5398,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -5416,7 +5442,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5463,7 +5489,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5507,7 +5533,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5554,7 +5580,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5642,7 +5668,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5686,7 +5712,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5730,7 +5756,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5774,7 +5800,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5818,7 +5844,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5862,7 +5888,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5947,7 +5973,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5991,7 +6017,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -6035,7 +6061,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -6079,7 +6105,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -6123,7 +6149,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -6167,7 +6193,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6211,7 +6237,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6255,7 +6281,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6302,7 +6328,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6346,7 +6372,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6390,7 +6416,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6434,7 +6460,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6478,7 +6504,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6566,7 +6592,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6610,7 +6636,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6654,7 +6680,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6742,7 +6768,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6786,7 +6812,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6912,7 +6938,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6956,7 +6982,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7000,7 +7026,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7044,7 +7070,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -7126,7 +7152,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7170,7 +7196,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7217,7 +7243,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7261,7 +7287,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -7387,7 +7413,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -7431,7 +7457,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7516,7 +7542,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7560,7 +7586,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7604,7 +7630,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7648,7 +7674,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7692,7 +7718,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7736,7 +7762,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7780,7 +7806,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7824,7 +7850,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7909,7 +7935,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8076,7 +8102,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8120,7 +8146,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8164,7 +8190,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8208,7 +8234,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8252,7 +8278,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8296,7 +8322,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8340,7 +8366,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -8425,7 +8451,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8469,7 +8495,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8554,7 +8580,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8680,7 +8706,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8724,7 +8750,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8809,7 +8835,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8853,7 +8879,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8897,7 +8923,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8941,7 +8967,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8985,7 +9011,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -9029,7 +9055,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9073,7 +9099,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9117,7 +9143,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -9202,7 +9228,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9369,7 +9395,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -9413,7 +9439,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9457,7 +9483,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9501,7 +9527,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9586,7 +9612,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9630,7 +9656,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9674,7 +9700,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9718,7 +9744,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9762,7 +9788,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9806,7 +9832,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9850,7 +9876,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9894,7 +9920,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9938,7 +9964,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9982,7 +10008,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10026,7 +10052,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -10070,7 +10096,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10114,7 +10140,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10158,7 +10184,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -10202,7 +10228,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10246,7 +10272,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10290,7 +10316,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -10334,7 +10360,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -10378,7 +10404,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -10422,7 +10448,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10466,7 +10492,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10551,7 +10577,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10636,7 +10662,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10651,55 +10677,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -11068,7 +11094,7 @@
       <c r="L10" t="s">
         <v>724</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46393</v>
       </c>
       <c r="N10" t="s">
@@ -11112,7 +11138,7 @@
       <c r="L11" t="s">
         <v>724</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46393</v>
       </c>
       <c r="N11" t="s">
@@ -11320,7 +11346,7 @@
       <c r="L16" t="s">
         <v>724</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46393</v>
       </c>
       <c r="N16" t="s">
@@ -11446,7 +11472,7 @@
       <c r="L19" t="s">
         <v>724</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46393</v>
       </c>
       <c r="N19" t="s">
@@ -11490,7 +11516,7 @@
       <c r="L20" t="s">
         <v>724</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46393</v>
       </c>
       <c r="N20" t="s">
@@ -11534,7 +11560,7 @@
       <c r="L21" t="s">
         <v>724</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46393</v>
       </c>
       <c r="N21" t="s">
@@ -11701,7 +11727,7 @@
       <c r="L25" t="s">
         <v>724</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46393</v>
       </c>
       <c r="N25" t="s">
@@ -11827,7 +11853,7 @@
       <c r="L28" t="s">
         <v>724</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46393</v>
       </c>
       <c r="N28" t="s">
@@ -11912,7 +11938,7 @@
       <c r="L30" t="s">
         <v>724</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46393</v>
       </c>
       <c r="N30" t="s">
@@ -12366,7 +12392,7 @@
       <c r="L41" t="s">
         <v>724</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46393</v>
       </c>
       <c r="N41" t="s">
@@ -12451,7 +12477,7 @@
       <c r="L43" t="s">
         <v>724</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46393</v>
       </c>
       <c r="N43" t="s">
@@ -12495,7 +12521,7 @@
       <c r="L44" t="s">
         <v>724</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46393</v>
       </c>
       <c r="N44" t="s">
@@ -12539,7 +12565,7 @@
       <c r="L45" t="s">
         <v>724</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46393</v>
       </c>
       <c r="N45" t="s">
@@ -12665,7 +12691,7 @@
       <c r="L48" t="s">
         <v>724</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46393</v>
       </c>
       <c r="N48" t="s">
@@ -12709,7 +12735,7 @@
       <c r="L49" t="s">
         <v>723</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46328</v>
       </c>
       <c r="N49" t="s">
@@ -12753,7 +12779,7 @@
       <c r="L50" t="s">
         <v>723</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46328</v>
       </c>
       <c r="N50" t="s">
@@ -12797,7 +12823,7 @@
       <c r="L51" t="s">
         <v>724</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46393</v>
       </c>
       <c r="N51" t="s">
@@ -12841,7 +12867,7 @@
       <c r="L52" t="s">
         <v>724</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46393</v>
       </c>
       <c r="N52" t="s">
@@ -12885,7 +12911,7 @@
       <c r="L53" t="s">
         <v>724</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46393</v>
       </c>
       <c r="N53" t="s">
@@ -12929,7 +12955,7 @@
       <c r="L54" t="s">
         <v>724</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46393</v>
       </c>
       <c r="N54" t="s">
@@ -12973,7 +12999,7 @@
       <c r="L55" t="s">
         <v>724</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46393</v>
       </c>
       <c r="N55" t="s">
@@ -13140,7 +13166,7 @@
       <c r="L59" t="s">
         <v>724</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46393</v>
       </c>
       <c r="N59" t="s">
@@ -13266,7 +13292,7 @@
       <c r="L62" t="s">
         <v>724</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46393</v>
       </c>
       <c r="N62" t="s">
@@ -13310,7 +13336,7 @@
       <c r="L63" t="s">
         <v>724</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46393</v>
       </c>
       <c r="N63" t="s">
@@ -13354,7 +13380,7 @@
       <c r="L64" t="s">
         <v>724</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46393</v>
       </c>
       <c r="N64" t="s">
@@ -13398,7 +13424,7 @@
       <c r="L65" t="s">
         <v>724</v>
       </c>
-      <c r="M65" s="1">
+      <c r="M65" s="2">
         <v>46393</v>
       </c>
       <c r="N65" t="s">
@@ -13442,7 +13468,7 @@
       <c r="L66" t="s">
         <v>724</v>
       </c>
-      <c r="M66" s="1">
+      <c r="M66" s="2">
         <v>46393</v>
       </c>
       <c r="N66" t="s">
@@ -13486,7 +13512,7 @@
       <c r="L67" t="s">
         <v>724</v>
       </c>
-      <c r="M67" s="1">
+      <c r="M67" s="2">
         <v>46393</v>
       </c>
       <c r="N67" t="s">
@@ -13530,7 +13556,7 @@
       <c r="L68" t="s">
         <v>724</v>
       </c>
-      <c r="M68" s="1">
+      <c r="M68" s="2">
         <v>46393</v>
       </c>
       <c r="N68" t="s">
@@ -13574,7 +13600,7 @@
       <c r="L69" t="s">
         <v>724</v>
       </c>
-      <c r="M69" s="1">
+      <c r="M69" s="2">
         <v>46393</v>
       </c>
       <c r="N69" t="s">
@@ -13618,7 +13644,7 @@
       <c r="L70" t="s">
         <v>724</v>
       </c>
-      <c r="M70" s="1">
+      <c r="M70" s="2">
         <v>46393</v>
       </c>
       <c r="N70" t="s">
@@ -13662,7 +13688,7 @@
       <c r="L71" t="s">
         <v>724</v>
       </c>
-      <c r="M71" s="1">
+      <c r="M71" s="2">
         <v>46393</v>
       </c>
       <c r="N71" t="s">
@@ -13706,7 +13732,7 @@
       <c r="L72" t="s">
         <v>724</v>
       </c>
-      <c r="M72" s="1">
+      <c r="M72" s="2">
         <v>46393</v>
       </c>
       <c r="N72" t="s">
@@ -13750,7 +13776,7 @@
       <c r="L73" t="s">
         <v>724</v>
       </c>
-      <c r="M73" s="1">
+      <c r="M73" s="2">
         <v>46393</v>
       </c>
       <c r="N73" t="s">
@@ -13794,7 +13820,7 @@
       <c r="L74" t="s">
         <v>724</v>
       </c>
-      <c r="M74" s="1">
+      <c r="M74" s="2">
         <v>46393</v>
       </c>
       <c r="N74" t="s">
@@ -13838,7 +13864,7 @@
       <c r="L75" t="s">
         <v>724</v>
       </c>
-      <c r="M75" s="1">
+      <c r="M75" s="2">
         <v>46393</v>
       </c>
       <c r="N75" t="s">
@@ -13882,7 +13908,7 @@
       <c r="L76" t="s">
         <v>724</v>
       </c>
-      <c r="M76" s="1">
+      <c r="M76" s="2">
         <v>46393</v>
       </c>
       <c r="N76" t="s">
@@ -13926,7 +13952,7 @@
       <c r="L77" t="s">
         <v>724</v>
       </c>
-      <c r="M77" s="1">
+      <c r="M77" s="2">
         <v>46393</v>
       </c>
       <c r="N77" t="s">
@@ -13970,7 +13996,7 @@
       <c r="L78" t="s">
         <v>724</v>
       </c>
-      <c r="M78" s="1">
+      <c r="M78" s="2">
         <v>46393</v>
       </c>
       <c r="N78" t="s">
@@ -14014,7 +14040,7 @@
       <c r="L79" t="s">
         <v>724</v>
       </c>
-      <c r="M79" s="1">
+      <c r="M79" s="2">
         <v>46393</v>
       </c>
       <c r="N79" t="s">
@@ -14058,7 +14084,7 @@
       <c r="L80" t="s">
         <v>724</v>
       </c>
-      <c r="M80" s="1">
+      <c r="M80" s="2">
         <v>46393</v>
       </c>
       <c r="N80" t="s">
@@ -14102,7 +14128,7 @@
       <c r="L81" t="s">
         <v>724</v>
       </c>
-      <c r="M81" s="1">
+      <c r="M81" s="2">
         <v>46393</v>
       </c>
       <c r="N81" t="s">
@@ -14146,7 +14172,7 @@
       <c r="L82" t="s">
         <v>724</v>
       </c>
-      <c r="M82" s="1">
+      <c r="M82" s="2">
         <v>46393</v>
       </c>
       <c r="N82" t="s">
@@ -14190,7 +14216,7 @@
       <c r="L83" t="s">
         <v>724</v>
       </c>
-      <c r="M83" s="1">
+      <c r="M83" s="2">
         <v>46393</v>
       </c>
       <c r="N83" t="s">
@@ -14234,7 +14260,7 @@
       <c r="L84" t="s">
         <v>724</v>
       </c>
-      <c r="M84" s="1">
+      <c r="M84" s="2">
         <v>46393</v>
       </c>
       <c r="N84" t="s">
@@ -14278,7 +14304,7 @@
       <c r="L85" t="s">
         <v>724</v>
       </c>
-      <c r="M85" s="1">
+      <c r="M85" s="2">
         <v>46393</v>
       </c>
       <c r="N85" t="s">
@@ -14322,7 +14348,7 @@
       <c r="L86" t="s">
         <v>724</v>
       </c>
-      <c r="M86" s="1">
+      <c r="M86" s="2">
         <v>46393</v>
       </c>
       <c r="N86" t="s">
@@ -14366,7 +14392,7 @@
       <c r="L87" t="s">
         <v>724</v>
       </c>
-      <c r="M87" s="1">
+      <c r="M87" s="2">
         <v>46393</v>
       </c>
       <c r="N87" t="s">
@@ -14410,7 +14436,7 @@
       <c r="L88" t="s">
         <v>724</v>
       </c>
-      <c r="M88" s="1">
+      <c r="M88" s="2">
         <v>46393</v>
       </c>
       <c r="N88" t="s">
@@ -14454,7 +14480,7 @@
       <c r="L89" t="s">
         <v>724</v>
       </c>
-      <c r="M89" s="1">
+      <c r="M89" s="2">
         <v>46393</v>
       </c>
       <c r="N89" t="s">
@@ -14498,7 +14524,7 @@
       <c r="L90" t="s">
         <v>724</v>
       </c>
-      <c r="M90" s="1">
+      <c r="M90" s="2">
         <v>46393</v>
       </c>
       <c r="N90" t="s">
@@ -14583,7 +14609,7 @@
       <c r="L92" t="s">
         <v>724</v>
       </c>
-      <c r="M92" s="1">
+      <c r="M92" s="2">
         <v>46393</v>
       </c>
       <c r="N92" t="s">
@@ -14627,7 +14653,7 @@
       <c r="L93" t="s">
         <v>724</v>
       </c>
-      <c r="M93" s="1">
+      <c r="M93" s="2">
         <v>46393</v>
       </c>
       <c r="N93" t="s">
@@ -14671,7 +14697,7 @@
       <c r="L94" t="s">
         <v>724</v>
       </c>
-      <c r="M94" s="1">
+      <c r="M94" s="2">
         <v>46393</v>
       </c>
       <c r="N94" t="s">
@@ -14715,7 +14741,7 @@
       <c r="L95" t="s">
         <v>724</v>
       </c>
-      <c r="M95" s="1">
+      <c r="M95" s="2">
         <v>46393</v>
       </c>
       <c r="N95" t="s">
@@ -14759,7 +14785,7 @@
       <c r="L96" t="s">
         <v>724</v>
       </c>
-      <c r="M96" s="1">
+      <c r="M96" s="2">
         <v>46393</v>
       </c>
       <c r="N96" t="s">
@@ -14803,7 +14829,7 @@
       <c r="L97" t="s">
         <v>724</v>
       </c>
-      <c r="M97" s="1">
+      <c r="M97" s="2">
         <v>46393</v>
       </c>
       <c r="N97" t="s">
@@ -14847,7 +14873,7 @@
       <c r="L98" t="s">
         <v>724</v>
       </c>
-      <c r="M98" s="1">
+      <c r="M98" s="2">
         <v>46393</v>
       </c>
       <c r="N98" t="s">
@@ -14891,7 +14917,7 @@
       <c r="L99" t="s">
         <v>724</v>
       </c>
-      <c r="M99" s="1">
+      <c r="M99" s="2">
         <v>46393</v>
       </c>
       <c r="N99" t="s">
@@ -14935,7 +14961,7 @@
       <c r="L100" t="s">
         <v>724</v>
       </c>
-      <c r="M100" s="1">
+      <c r="M100" s="2">
         <v>46393</v>
       </c>
       <c r="N100" t="s">
@@ -14979,7 +15005,7 @@
       <c r="L101" t="s">
         <v>724</v>
       </c>
-      <c r="M101" s="1">
+      <c r="M101" s="2">
         <v>46393</v>
       </c>
       <c r="N101" t="s">
@@ -15023,7 +15049,7 @@
       <c r="L102" t="s">
         <v>724</v>
       </c>
-      <c r="M102" s="1">
+      <c r="M102" s="2">
         <v>46393</v>
       </c>
       <c r="N102" t="s">
@@ -15067,7 +15093,7 @@
       <c r="L103" t="s">
         <v>724</v>
       </c>
-      <c r="M103" s="1">
+      <c r="M103" s="2">
         <v>46393</v>
       </c>
       <c r="N103" t="s">
@@ -15111,7 +15137,7 @@
       <c r="L104" t="s">
         <v>724</v>
       </c>
-      <c r="M104" s="1">
+      <c r="M104" s="2">
         <v>46393</v>
       </c>
       <c r="N104" t="s">
@@ -15155,7 +15181,7 @@
       <c r="L105" t="s">
         <v>724</v>
       </c>
-      <c r="M105" s="1">
+      <c r="M105" s="2">
         <v>46393</v>
       </c>
       <c r="N105" t="s">
@@ -15199,7 +15225,7 @@
       <c r="L106" t="s">
         <v>724</v>
       </c>
-      <c r="M106" s="1">
+      <c r="M106" s="2">
         <v>46393</v>
       </c>
       <c r="N106" t="s">
@@ -15243,7 +15269,7 @@
       <c r="L107" t="s">
         <v>724</v>
       </c>
-      <c r="M107" s="1">
+      <c r="M107" s="2">
         <v>46393</v>
       </c>
       <c r="N107" t="s">
@@ -15287,7 +15313,7 @@
       <c r="L108" t="s">
         <v>724</v>
       </c>
-      <c r="M108" s="1">
+      <c r="M108" s="2">
         <v>46393</v>
       </c>
       <c r="N108" t="s">
@@ -15331,7 +15357,7 @@
       <c r="L109" t="s">
         <v>724</v>
       </c>
-      <c r="M109" s="1">
+      <c r="M109" s="2">
         <v>46393</v>
       </c>
       <c r="N109" t="s">
@@ -15375,7 +15401,7 @@
       <c r="L110" t="s">
         <v>724</v>
       </c>
-      <c r="M110" s="1">
+      <c r="M110" s="2">
         <v>46393</v>
       </c>
       <c r="N110" t="s">
@@ -15419,7 +15445,7 @@
       <c r="L111" t="s">
         <v>724</v>
       </c>
-      <c r="M111" s="1">
+      <c r="M111" s="2">
         <v>46393</v>
       </c>
       <c r="N111" t="s">
@@ -15463,7 +15489,7 @@
       <c r="L112" t="s">
         <v>724</v>
       </c>
-      <c r="M112" s="1">
+      <c r="M112" s="2">
         <v>46393</v>
       </c>
       <c r="N112" t="s">
@@ -15507,7 +15533,7 @@
       <c r="L113" t="s">
         <v>724</v>
       </c>
-      <c r="M113" s="1">
+      <c r="M113" s="2">
         <v>46393</v>
       </c>
       <c r="N113" t="s">
@@ -15551,7 +15577,7 @@
       <c r="L114" t="s">
         <v>724</v>
       </c>
-      <c r="M114" s="1">
+      <c r="M114" s="2">
         <v>46393</v>
       </c>
       <c r="N114" t="s">
@@ -15595,7 +15621,7 @@
       <c r="L115" t="s">
         <v>724</v>
       </c>
-      <c r="M115" s="1">
+      <c r="M115" s="2">
         <v>46393</v>
       </c>
       <c r="N115" t="s">
@@ -15639,7 +15665,7 @@
       <c r="L116" t="s">
         <v>724</v>
       </c>
-      <c r="M116" s="1">
+      <c r="M116" s="2">
         <v>46393</v>
       </c>
       <c r="N116" t="s">
@@ -15683,7 +15709,7 @@
       <c r="L117" t="s">
         <v>724</v>
       </c>
-      <c r="M117" s="1">
+      <c r="M117" s="2">
         <v>46393</v>
       </c>
       <c r="N117" t="s">
@@ -15727,7 +15753,7 @@
       <c r="L118" t="s">
         <v>724</v>
       </c>
-      <c r="M118" s="1">
+      <c r="M118" s="2">
         <v>46393</v>
       </c>
       <c r="N118" t="s">
@@ -15771,7 +15797,7 @@
       <c r="L119" t="s">
         <v>724</v>
       </c>
-      <c r="M119" s="1">
+      <c r="M119" s="2">
         <v>46393</v>
       </c>
       <c r="N119" t="s">
@@ -15815,7 +15841,7 @@
       <c r="L120" t="s">
         <v>724</v>
       </c>
-      <c r="M120" s="1">
+      <c r="M120" s="2">
         <v>46393</v>
       </c>
       <c r="N120" t="s">
@@ -15859,7 +15885,7 @@
       <c r="L121" t="s">
         <v>724</v>
       </c>
-      <c r="M121" s="1">
+      <c r="M121" s="2">
         <v>46393</v>
       </c>
       <c r="N121" t="s">
@@ -15903,7 +15929,7 @@
       <c r="L122" t="s">
         <v>724</v>
       </c>
-      <c r="M122" s="1">
+      <c r="M122" s="2">
         <v>46393</v>
       </c>
       <c r="N122" t="s">
@@ -15947,7 +15973,7 @@
       <c r="L123" t="s">
         <v>724</v>
       </c>
-      <c r="M123" s="1">
+      <c r="M123" s="2">
         <v>46393</v>
       </c>
       <c r="N123" t="s">
@@ -15991,7 +16017,7 @@
       <c r="L124" t="s">
         <v>724</v>
       </c>
-      <c r="M124" s="1">
+      <c r="M124" s="2">
         <v>46393</v>
       </c>
       <c r="N124" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (26/10/2026 14:18)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3126" uniqueCount="727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3126" uniqueCount="728">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -2189,10 +2189,13 @@
     <t>Mapa Gerado</t>
   </si>
   <si>
+    <t>Selecionada em PAM/S</t>
+  </si>
+  <si>
     <t>Validada</t>
   </si>
   <si>
-    <t>Em Discrepância</t>
+    <t>Selecionada para cotação</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -2205,16 +2208,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2230,7 +2225,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2238,30 +2233,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2561,55 +2538,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2653,7 +2630,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2697,7 +2674,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2741,7 +2718,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2867,7 +2844,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2911,7 +2888,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2955,7 +2932,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -3002,7 +2979,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3125,7 +3102,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -3169,7 +3146,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3213,7 +3190,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3257,7 +3234,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -3304,7 +3281,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3348,7 +3325,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3474,7 +3451,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3518,7 +3495,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3603,7 +3580,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3650,7 +3627,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3697,7 +3674,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3741,7 +3718,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3785,7 +3762,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3870,7 +3847,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3955,7 +3932,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -4002,7 +3979,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4046,7 +4023,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4090,7 +4067,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4175,7 +4152,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4219,7 +4196,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4263,7 +4240,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4348,7 +4325,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4392,7 +4369,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4436,7 +4413,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4480,7 +4457,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4647,7 +4624,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4691,7 +4668,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4735,7 +4712,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4779,7 +4756,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4826,7 +4803,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4870,7 +4847,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4952,7 +4929,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4996,7 +4973,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5084,7 +5061,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5128,7 +5105,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -5175,7 +5152,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5219,7 +5196,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -5263,7 +5240,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -5307,7 +5284,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5351,7 +5328,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -5398,7 +5375,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5442,7 +5419,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5489,7 +5466,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5533,7 +5510,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5580,7 +5557,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5668,7 +5645,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5712,7 +5689,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5756,7 +5733,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5800,7 +5777,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5844,7 +5821,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5888,7 +5865,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5973,7 +5950,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6017,7 +5994,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -6061,7 +6038,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -6105,7 +6082,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -6149,7 +6126,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -6193,7 +6170,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6237,7 +6214,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6281,7 +6258,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -6328,7 +6305,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6372,7 +6349,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6416,7 +6393,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6460,7 +6437,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6504,7 +6481,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6548,7 +6525,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6592,7 +6569,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6636,7 +6613,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6680,7 +6657,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6768,7 +6745,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6812,7 +6789,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6938,7 +6915,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6982,7 +6959,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7026,7 +7003,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7070,7 +7047,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -7152,7 +7129,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7196,7 +7173,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -7243,7 +7220,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7287,7 +7264,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -7413,7 +7390,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7457,7 +7434,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7542,7 +7519,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7586,7 +7563,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7630,7 +7607,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7674,7 +7651,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7718,7 +7695,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7762,7 +7739,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="